<commit_message>
update data Russia war case
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55D42ECD-15AC-45FA-9E70-C45F1348C0EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{624E3527-5A36-4AF9-AA42-EB73A45CE311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="95">
   <si>
     <t>Belgium</t>
   </si>
@@ -76,18 +76,9 @@
     <t>UK</t>
   </si>
   <si>
-    <t>Rest of EU</t>
-  </si>
-  <si>
-    <t>Rest of Europe</t>
-  </si>
-  <si>
     <t>LNG</t>
   </si>
   <si>
-    <t>Imports</t>
-  </si>
-  <si>
     <t>Share [2020]</t>
   </si>
   <si>
@@ -97,13 +88,250 @@
     <t>LNG Capacity Mrd m3 [2020]</t>
   </si>
   <si>
-    <t>node</t>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>BE</t>
+  </si>
+  <si>
+    <t>NL</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>AT</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>CH</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>HR</t>
+  </si>
+  <si>
+    <t>FR</t>
+  </si>
+  <si>
+    <t>DK</t>
+  </si>
+  <si>
+    <t>PL</t>
+  </si>
+  <si>
+    <t>CZ</t>
+  </si>
+  <si>
+    <t>SK</t>
+  </si>
+  <si>
+    <t>HU</t>
+  </si>
+  <si>
+    <t>RS</t>
+  </si>
+  <si>
+    <t>BG</t>
+  </si>
+  <si>
+    <t>GR</t>
+  </si>
+  <si>
+    <t>RO</t>
+  </si>
+  <si>
+    <t>LT</t>
+  </si>
+  <si>
+    <t>LV</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>PT</t>
+  </si>
+  <si>
+    <t>UA</t>
+  </si>
+  <si>
+    <t>MD</t>
+  </si>
+  <si>
+    <t>RU</t>
+  </si>
+  <si>
+    <t>AL</t>
+  </si>
+  <si>
+    <t>LU</t>
+  </si>
+  <si>
+    <t>IE</t>
+  </si>
+  <si>
+    <t>BA</t>
+  </si>
+  <si>
+    <t>MK</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>SM</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>DZ</t>
+  </si>
+  <si>
+    <t>TN</t>
+  </si>
+  <si>
+    <t>LY</t>
+  </si>
+  <si>
+    <t>BY</t>
+  </si>
+  <si>
+    <t>EE</t>
+  </si>
+  <si>
+    <t>FI</t>
+  </si>
+  <si>
+    <t>Long_name</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>Austria</t>
+  </si>
+  <si>
+    <t>Switzerland</t>
+  </si>
+  <si>
+    <t>Slovenia</t>
+  </si>
+  <si>
+    <t>Denmark</t>
+  </si>
+  <si>
+    <t>Czech Republic</t>
+  </si>
+  <si>
+    <t>Slovakia</t>
+  </si>
+  <si>
+    <t>Hungary</t>
+  </si>
+  <si>
+    <t>Bulgaria</t>
+  </si>
+  <si>
+    <t>Latvia</t>
+  </si>
+  <si>
+    <t>Estonia</t>
+  </si>
+  <si>
+    <t>Ukraine</t>
+  </si>
+  <si>
+    <t>Moldova</t>
+  </si>
+  <si>
+    <t>Russia</t>
+  </si>
+  <si>
+    <t>Luxemburg</t>
+  </si>
+  <si>
+    <t>Norway</t>
+  </si>
+  <si>
+    <t>Serbia</t>
+  </si>
+  <si>
+    <t>Albania</t>
+  </si>
+  <si>
+    <t>Irland</t>
+  </si>
+  <si>
+    <t>Bosnia and Herzegovina</t>
+  </si>
+  <si>
+    <t>North Macedonia</t>
+  </si>
+  <si>
+    <t>San Marino</t>
+  </si>
+  <si>
+    <t>Algeria</t>
+  </si>
+  <si>
+    <t>Tunisia</t>
+  </si>
+  <si>
+    <t>Libya</t>
+  </si>
+  <si>
+    <t>Belarus</t>
+  </si>
+  <si>
+    <t>SE</t>
+  </si>
+  <si>
+    <t>Sweden</t>
+  </si>
+  <si>
+    <t>https://www.bp.com/content/dam/bp/business-sites/en/global/corporate/pdfs/energy-economics/statistical-review/bp-stats-review-2021-full-report.pdf</t>
+  </si>
+  <si>
+    <t>Mrd m3 [2020]</t>
+  </si>
+  <si>
+    <t>Finland</t>
+  </si>
+  <si>
+    <t>Romania</t>
+  </si>
+  <si>
+    <t>SP</t>
+  </si>
+  <si>
+    <t>OE</t>
+  </si>
+  <si>
+    <t>Other Europe</t>
+  </si>
+  <si>
+    <t>https://www.ins.tn/sites/default/files/publication/pdf/bms%20octobre%202022.pdf</t>
+  </si>
+  <si>
+    <t>Imports [2020]</t>
+  </si>
+  <si>
+    <t>Malta</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="0.0"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -133,14 +361,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="168" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="0.0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -151,6 +387,36 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D12A1D17-871E-4E66-A144-F2ADD46C5E00}" name="Table2" displayName="Table2" ref="A1:C42" totalsRowShown="0">
+  <autoFilter ref="A1:C42" xr:uid="{D12A1D17-871E-4E66-A144-F2ADD46C5E00}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C41">
+    <sortCondition ref="B1:B41"/>
+  </sortState>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{D3465064-BCEE-4D04-A8E6-DEAE11BBDA92}" name="Country"/>
+    <tableColumn id="2" xr3:uid="{D66D54B4-4DED-47C6-BE50-755A236428ED}" name="Long_name"/>
+    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}" name="Table1" displayName="Table1" ref="A1:C39" totalsRowShown="0">
+  <autoFilter ref="A1:C39" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C39">
+    <sortCondition ref="B1:B39"/>
+  </sortState>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
+    <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -421,19 +687,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s">
         <v>14</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -441,14 +707,14 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>9</v>
+        <v>11.4</v>
       </c>
       <c r="C2">
         <v>5.0999999999999996</v>
       </c>
       <c r="D2" s="1">
         <f>C2/B2</f>
-        <v>0.56666666666666665</v>
+        <v>0.44736842105263153</v>
       </c>
       <c r="E2">
         <v>9</v>
@@ -477,14 +743,14 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="C4">
         <v>2.5</v>
       </c>
       <c r="D4" s="1">
         <f t="shared" si="0"/>
-        <v>0.33333333333333331</v>
+        <v>0.35714285714285715</v>
       </c>
       <c r="E4">
         <v>7.5</v>
@@ -495,14 +761,14 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>15.8</v>
+        <v>15.95</v>
       </c>
       <c r="C5">
         <v>12.1</v>
       </c>
       <c r="D5" s="1">
         <f t="shared" si="0"/>
-        <v>0.76582278481012656</v>
+        <v>0.75862068965517238</v>
       </c>
       <c r="E5">
         <v>15.8</v>
@@ -549,14 +815,14 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>12.5</v>
+        <v>12</v>
       </c>
       <c r="C8">
         <v>8.1999999999999993</v>
       </c>
       <c r="D8" s="1">
         <f t="shared" si="0"/>
-        <v>0.65599999999999992</v>
+        <v>0.68333333333333324</v>
       </c>
       <c r="E8">
         <v>12.5</v>
@@ -567,14 +833,14 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>7.5</v>
+        <v>6.2</v>
       </c>
       <c r="C9">
         <v>4.0999999999999996</v>
       </c>
       <c r="D9" s="1">
         <f t="shared" si="0"/>
-        <v>0.54666666666666663</v>
+        <v>0.66129032258064513</v>
       </c>
       <c r="E9">
         <v>5.8</v>
@@ -603,14 +869,14 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <v>67.099999999999994</v>
+        <v>60.1</v>
       </c>
       <c r="C11">
         <v>20.9</v>
       </c>
       <c r="D11" s="1">
         <f t="shared" si="0"/>
-        <v>0.31147540983606559</v>
+        <v>0.3477537437603993</v>
       </c>
       <c r="E11">
         <v>67.099999999999994</v>
@@ -621,14 +887,14 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>14.8</v>
+        <v>43.6</v>
       </c>
       <c r="C12">
         <v>14.8</v>
       </c>
       <c r="D12" s="1">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0.33944954128440369</v>
       </c>
       <c r="E12">
         <v>14.8</v>
@@ -639,14 +905,14 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>52.3</v>
+        <v>48.1</v>
       </c>
       <c r="C13">
         <v>18.600000000000001</v>
       </c>
       <c r="D13" s="1">
         <f t="shared" si="0"/>
-        <v>0.35564053537284901</v>
+        <v>0.38669438669438672</v>
       </c>
       <c r="E13">
         <v>52.3</v>
@@ -654,39 +920,18 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>94</v>
       </c>
       <c r="B14">
-        <v>1.3</v>
-      </c>
-      <c r="C14">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="D14" s="1">
         <f t="shared" si="0"/>
-        <v>0.61538461538461542</v>
-      </c>
-      <c r="E14">
-        <v>1.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15">
-        <v>1.3</v>
-      </c>
-      <c r="C15">
-        <v>0.1</v>
-      </c>
-      <c r="D15" s="1">
-        <f t="shared" si="0"/>
-        <v>7.6923076923076927E-2</v>
-      </c>
-      <c r="E15">
-        <v>1.3</v>
-      </c>
+      <c r="D15" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -695,24 +940,857 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF82F4-4954-4D06-9A30-AE8575CA18DE}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="2">
+        <v>81.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>19</v>
+      </c>
+      <c r="B16" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="2">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="2">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" t="s">
+        <v>81</v>
+      </c>
+      <c r="C22" s="2">
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="2"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="2"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" t="s">
+        <v>69</v>
+      </c>
+      <c r="C25" s="2"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" t="s">
+        <v>77</v>
+      </c>
+      <c r="C27" s="2"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" s="2">
+        <v>111.5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="2">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" s="2"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" s="2">
+        <v>8.6999999999999993</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>41</v>
+      </c>
+      <c r="B32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C32" s="2">
+        <v>638.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>48</v>
+      </c>
+      <c r="B33" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>73</v>
+      </c>
+      <c r="C34" s="2"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="2"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>23</v>
+      </c>
+      <c r="B36" t="s">
+        <v>60</v>
+      </c>
+      <c r="C36" s="2"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>22</v>
+      </c>
+      <c r="B37" t="s">
+        <v>59</v>
+      </c>
+      <c r="C37" s="2"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>51</v>
+      </c>
+      <c r="B38" t="s">
+        <v>80</v>
+      </c>
+      <c r="C38" s="2">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>47</v>
+      </c>
+      <c r="B39" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="2"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>11</v>
+      </c>
+      <c r="B40" t="s">
+        <v>11</v>
+      </c>
+      <c r="C40" s="2">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>39</v>
+      </c>
+      <c r="B41" t="s">
+        <v>68</v>
+      </c>
+      <c r="C41" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>90</v>
+      </c>
+      <c r="B42" t="s">
+        <v>91</v>
+      </c>
+      <c r="C42" s="2">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>80</v>
+      </c>
+      <c r="B49" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE55996C-4401-4161-B17D-CF2A8462856A}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="9.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="2">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="2">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C12" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13" s="2">
+        <v>40.700000000000003</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
+        <v>57</v>
+      </c>
+      <c r="C14" s="2">
+        <v>86.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="2">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="2">
+        <v>10.199999999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="2">
+        <v>67.7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" t="s">
+        <v>71</v>
+      </c>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="2">
+        <v>36.6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" t="s">
+        <v>77</v>
+      </c>
+      <c r="C24" s="2"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>90</v>
+      </c>
+      <c r="B26" t="s">
+        <v>91</v>
+      </c>
+      <c r="C26" s="2">
+        <v>29.6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" s="2">
+        <v>21.6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1</v>
+      </c>
+      <c r="C28" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>34</v>
+      </c>
+      <c r="B29" t="s">
+        <v>88</v>
+      </c>
+      <c r="C29" s="2">
+        <v>11.3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>48</v>
+      </c>
+      <c r="B30" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" s="2"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" t="s">
+        <v>73</v>
+      </c>
+      <c r="C31" s="2"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33" t="s">
+        <v>60</v>
+      </c>
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>89</v>
+      </c>
+      <c r="B34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="2">
+        <v>32.4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>83</v>
+      </c>
+      <c r="B35" t="s">
+        <v>84</v>
+      </c>
+      <c r="C35" s="2">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B36" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="2">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>47</v>
+      </c>
+      <c r="B37" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" s="2">
+        <v>46.4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38" t="s">
+        <v>11</v>
+      </c>
+      <c r="C38" s="2">
+        <v>72.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" t="s">
+        <v>68</v>
+      </c>
+      <c r="C39" s="2">
+        <v>29.3</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>85</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update input data with import capacity
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA12D333-4F34-42E8-8D78-D954B8B6924D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678E5D9E-05E8-4229-A41D-B29216D894B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10060" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
     <sheet name="nodes_gas_prod" sheetId="2" r:id="rId2"/>
     <sheet name="nodes_demand" sheetId="3" r:id="rId3"/>
     <sheet name="Connections" sheetId="4" r:id="rId4"/>
+    <sheet name="Import_Connections" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="107">
   <si>
     <t>Belgium</t>
   </si>
@@ -324,6 +325,42 @@
   </si>
   <si>
     <t>Malta</t>
+  </si>
+  <si>
+    <t>From</t>
+  </si>
+  <si>
+    <t>To</t>
+  </si>
+  <si>
+    <t>GWh/d</t>
+  </si>
+  <si>
+    <t>https://gasdashboard.entsog.eu/</t>
+  </si>
+  <si>
+    <t>AZ</t>
+  </si>
+  <si>
+    <t>TK</t>
+  </si>
+  <si>
+    <t>MA</t>
+  </si>
+  <si>
+    <t>IR</t>
+  </si>
+  <si>
+    <t>additional</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>_LNG</t>
+  </si>
+  <si>
+    <t>_Prod</t>
   </si>
 </sst>
 </file>
@@ -683,10 +720,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -702,8 +739,14 @@
       <c r="E1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="J1" t="s">
+        <v>95</v>
+      </c>
+      <c r="K1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -720,8 +763,22 @@
       <c r="E2">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
+        <v>105</v>
+      </c>
+      <c r="J2" t="str">
+        <f>_xlfn.CONCAT(G2,H2)</f>
+        <v>BE_LNG</v>
+      </c>
+      <c r="K2" t="str">
+        <f>G2</f>
+        <v>BE</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -738,8 +795,22 @@
       <c r="E3">
         <v>33</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J3" t="str">
+        <f t="shared" ref="J3:J13" si="1">_xlfn.CONCAT(G3,H3)</f>
+        <v>FR_LNG</v>
+      </c>
+      <c r="K3" t="str">
+        <f t="shared" ref="K3:K13" si="2">G3</f>
+        <v>FR</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -756,8 +827,22 @@
       <c r="E4">
         <v>7.5</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G4" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" t="s">
+        <v>105</v>
+      </c>
+      <c r="J4" t="str">
+        <f t="shared" si="1"/>
+        <v>GR_LNG</v>
+      </c>
+      <c r="K4" t="str">
+        <f t="shared" si="2"/>
+        <v>GR</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -774,8 +859,22 @@
       <c r="E5">
         <v>15.8</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" t="s">
+        <v>105</v>
+      </c>
+      <c r="J5" t="str">
+        <f t="shared" si="1"/>
+        <v>IT_LNG</v>
+      </c>
+      <c r="K5" t="str">
+        <f t="shared" si="2"/>
+        <v>IT</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -792,8 +891,22 @@
       <c r="E6">
         <v>2.6</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" t="s">
+        <v>105</v>
+      </c>
+      <c r="J6" t="str">
+        <f t="shared" si="1"/>
+        <v>HR_LNG</v>
+      </c>
+      <c r="K6" t="str">
+        <f t="shared" si="2"/>
+        <v>HR</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -810,8 +923,22 @@
       <c r="E7">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G7" t="s">
+        <v>35</v>
+      </c>
+      <c r="H7" t="s">
+        <v>105</v>
+      </c>
+      <c r="J7" t="str">
+        <f t="shared" si="1"/>
+        <v>LT_LNG</v>
+      </c>
+      <c r="K7" t="str">
+        <f t="shared" si="2"/>
+        <v>LT</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -828,8 +955,22 @@
       <c r="E8">
         <v>12.5</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H8" t="s">
+        <v>105</v>
+      </c>
+      <c r="J8" t="str">
+        <f t="shared" si="1"/>
+        <v>NL_LNG</v>
+      </c>
+      <c r="K8" t="str">
+        <f t="shared" si="2"/>
+        <v>NL</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -846,8 +987,22 @@
       <c r="E9">
         <v>5.8</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H9" t="s">
+        <v>105</v>
+      </c>
+      <c r="J9" t="str">
+        <f t="shared" si="1"/>
+        <v>PL_LNG</v>
+      </c>
+      <c r="K9" t="str">
+        <f t="shared" si="2"/>
+        <v>PL</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -864,8 +1019,22 @@
       <c r="E10">
         <v>7.3</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G10" t="s">
+        <v>38</v>
+      </c>
+      <c r="H10" t="s">
+        <v>105</v>
+      </c>
+      <c r="J10" t="str">
+        <f t="shared" si="1"/>
+        <v>PT_LNG</v>
+      </c>
+      <c r="K10" t="str">
+        <f t="shared" si="2"/>
+        <v>PT</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -882,8 +1051,22 @@
       <c r="E11">
         <v>67.099999999999994</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G11" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" t="s">
+        <v>105</v>
+      </c>
+      <c r="J11" t="str">
+        <f t="shared" si="1"/>
+        <v>ES_LNG</v>
+      </c>
+      <c r="K11" t="str">
+        <f t="shared" si="2"/>
+        <v>ES</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -900,8 +1083,22 @@
       <c r="E12">
         <v>14.8</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G12" t="s">
+        <v>47</v>
+      </c>
+      <c r="H12" t="s">
+        <v>105</v>
+      </c>
+      <c r="J12" t="str">
+        <f t="shared" si="1"/>
+        <v>TR_LNG</v>
+      </c>
+      <c r="K12" t="str">
+        <f t="shared" si="2"/>
+        <v>TR</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -918,8 +1115,22 @@
       <c r="E13">
         <v>52.3</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13" t="s">
+        <v>105</v>
+      </c>
+      <c r="J13" t="str">
+        <f t="shared" si="1"/>
+        <v>UK_LNG</v>
+      </c>
+      <c r="K13" t="str">
+        <f t="shared" si="2"/>
+        <v>UK</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>94</v>
       </c>
@@ -930,8 +1141,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G14" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="D15" s="1"/>
     </row>
   </sheetData>
@@ -941,7 +1155,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF82F4-4954-4D06-9A30-AE8575CA18DE}">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -949,7 +1163,7 @@
     <col min="3" max="3" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -959,8 +1173,14 @@
       <c r="C1" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H1" t="s">
+        <v>95</v>
+      </c>
+      <c r="I1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -968,8 +1188,19 @@
         <v>74</v>
       </c>
       <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="E2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H2" t="str">
+        <f>_xlfn.CONCAT(A2,$E$2)</f>
+        <v>AL_Prod</v>
+      </c>
+      <c r="I2" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>AL</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -979,8 +1210,16 @@
       <c r="C3" s="2">
         <v>81.5</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H3" t="str">
+        <f t="shared" ref="H3:H42" si="0">_xlfn.CONCAT(A3,$E$2)</f>
+        <v>DZ_Prod</v>
+      </c>
+      <c r="I3" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>DZ</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -988,8 +1227,16 @@
         <v>58</v>
       </c>
       <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H4" t="str">
+        <f t="shared" si="0"/>
+        <v>AT_Prod</v>
+      </c>
+      <c r="I4" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>AT</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -997,8 +1244,16 @@
         <v>82</v>
       </c>
       <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H5" t="str">
+        <f t="shared" si="0"/>
+        <v>BY_Prod</v>
+      </c>
+      <c r="I5" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>BY</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1006,8 +1261,16 @@
         <v>0</v>
       </c>
       <c r="C6" s="2"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H6" t="str">
+        <f t="shared" si="0"/>
+        <v>BE_Prod</v>
+      </c>
+      <c r="I6" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>BE</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>45</v>
       </c>
@@ -1015,8 +1278,16 @@
         <v>76</v>
       </c>
       <c r="C7" s="2"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H7" t="str">
+        <f t="shared" si="0"/>
+        <v>BA_Prod</v>
+      </c>
+      <c r="I7" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>BA</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1024,8 +1295,16 @@
         <v>65</v>
       </c>
       <c r="C8" s="2"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H8" t="str">
+        <f t="shared" si="0"/>
+        <v>BG_Prod</v>
+      </c>
+      <c r="I8" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>BG</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -1033,8 +1312,16 @@
         <v>5</v>
       </c>
       <c r="C9" s="2"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H9" t="str">
+        <f t="shared" si="0"/>
+        <v>HR_Prod</v>
+      </c>
+      <c r="I9" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>HR</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1042,8 +1329,16 @@
         <v>62</v>
       </c>
       <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H10" t="str">
+        <f t="shared" si="0"/>
+        <v>CZ_Prod</v>
+      </c>
+      <c r="I10" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>CZ</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -1053,8 +1348,16 @@
       <c r="C11" s="2">
         <v>1.4</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H11" t="str">
+        <f t="shared" si="0"/>
+        <v>DK_Prod</v>
+      </c>
+      <c r="I11" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>DK</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>37</v>
       </c>
@@ -1062,8 +1365,16 @@
         <v>67</v>
       </c>
       <c r="C12" s="2"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H12" t="str">
+        <f t="shared" si="0"/>
+        <v>ES_Prod</v>
+      </c>
+      <c r="I12" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>ES</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>54</v>
       </c>
@@ -1071,8 +1382,16 @@
         <v>67</v>
       </c>
       <c r="C13" s="2"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H13" t="str">
+        <f t="shared" si="0"/>
+        <v>EE_Prod</v>
+      </c>
+      <c r="I13" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>EE</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>55</v>
       </c>
@@ -1080,8 +1399,16 @@
         <v>87</v>
       </c>
       <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H14" t="str">
+        <f t="shared" si="0"/>
+        <v>FI_Prod</v>
+      </c>
+      <c r="I14" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>FI</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -1089,8 +1416,16 @@
         <v>2</v>
       </c>
       <c r="C15" s="2"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H15" t="str">
+        <f t="shared" si="0"/>
+        <v>FR_Prod</v>
+      </c>
+      <c r="I15" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>FR</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -1100,8 +1435,16 @@
       <c r="C16" s="2">
         <v>4.5</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H16" t="str">
+        <f t="shared" si="0"/>
+        <v>DE_Prod</v>
+      </c>
+      <c r="I16" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>DE</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -1109,8 +1452,16 @@
         <v>3</v>
       </c>
       <c r="C17" s="2"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H17" t="str">
+        <f t="shared" si="0"/>
+        <v>GR_Prod</v>
+      </c>
+      <c r="I17" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>GR</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1118,8 +1469,16 @@
         <v>64</v>
       </c>
       <c r="C18" s="2"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H18" t="str">
+        <f t="shared" si="0"/>
+        <v>HU_Prod</v>
+      </c>
+      <c r="I18" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>HU</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>44</v>
       </c>
@@ -1127,8 +1486,16 @@
         <v>75</v>
       </c>
       <c r="C19" s="2"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H19" t="str">
+        <f t="shared" si="0"/>
+        <v>IE_Prod</v>
+      </c>
+      <c r="I19" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>IE</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1138,8 +1505,16 @@
       <c r="C20" s="2">
         <v>3.9</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H20" t="str">
+        <f t="shared" si="0"/>
+        <v>IT_Prod</v>
+      </c>
+      <c r="I20" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>IT</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -1147,8 +1522,16 @@
         <v>66</v>
       </c>
       <c r="C21" s="2"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H21" t="str">
+        <f t="shared" si="0"/>
+        <v>LV_Prod</v>
+      </c>
+      <c r="I21" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>LV</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>52</v>
       </c>
@@ -1158,8 +1541,16 @@
       <c r="C22" s="2">
         <v>13.3</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H22" t="str">
+        <f t="shared" si="0"/>
+        <v>LY_Prod</v>
+      </c>
+      <c r="I22" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>LY</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>35</v>
       </c>
@@ -1167,8 +1558,16 @@
         <v>6</v>
       </c>
       <c r="C23" s="2"/>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H23" t="str">
+        <f t="shared" si="0"/>
+        <v>LT_Prod</v>
+      </c>
+      <c r="I23" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>LT</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -1176,8 +1575,16 @@
         <v>71</v>
       </c>
       <c r="C24" s="2"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H24" t="str">
+        <f t="shared" si="0"/>
+        <v>LU_Prod</v>
+      </c>
+      <c r="I24" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>LU</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>40</v>
       </c>
@@ -1185,8 +1592,16 @@
         <v>69</v>
       </c>
       <c r="C25" s="2"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H25" t="str">
+        <f t="shared" si="0"/>
+        <v>MD_Prod</v>
+      </c>
+      <c r="I25" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>MD</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -1196,8 +1611,16 @@
       <c r="C26" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H26" t="str">
+        <f t="shared" si="0"/>
+        <v>NL_Prod</v>
+      </c>
+      <c r="I26" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>NL</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>46</v>
       </c>
@@ -1205,8 +1628,16 @@
         <v>77</v>
       </c>
       <c r="C27" s="2"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H27" t="str">
+        <f t="shared" si="0"/>
+        <v>MK_Prod</v>
+      </c>
+      <c r="I27" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>MK</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>49</v>
       </c>
@@ -1216,8 +1647,16 @@
       <c r="C28" s="2">
         <v>111.5</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H28" t="str">
+        <f t="shared" si="0"/>
+        <v>NO_Prod</v>
+      </c>
+      <c r="I28" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>NO</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1227,8 +1666,16 @@
       <c r="C29" s="2">
         <v>3.9</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H29" t="str">
+        <f t="shared" si="0"/>
+        <v>PL_Prod</v>
+      </c>
+      <c r="I29" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>PL</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>38</v>
       </c>
@@ -1236,8 +1683,16 @@
         <v>1</v>
       </c>
       <c r="C30" s="2"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H30" t="str">
+        <f t="shared" si="0"/>
+        <v>PT_Prod</v>
+      </c>
+      <c r="I30" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>PT</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -1247,8 +1702,16 @@
       <c r="C31" s="2">
         <v>8.6999999999999993</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H31" t="str">
+        <f t="shared" si="0"/>
+        <v>RO_Prod</v>
+      </c>
+      <c r="I31" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>RO</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>41</v>
       </c>
@@ -1258,8 +1721,16 @@
       <c r="C32" s="2">
         <v>638.5</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H32" t="str">
+        <f t="shared" si="0"/>
+        <v>RU_Prod</v>
+      </c>
+      <c r="I32" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>RU</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>48</v>
       </c>
@@ -1267,8 +1738,16 @@
         <v>78</v>
       </c>
       <c r="C33" s="2"/>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H33" t="str">
+        <f t="shared" si="0"/>
+        <v>SM_Prod</v>
+      </c>
+      <c r="I33" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>SM</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>31</v>
       </c>
@@ -1276,8 +1755,16 @@
         <v>73</v>
       </c>
       <c r="C34" s="2"/>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H34" t="str">
+        <f t="shared" si="0"/>
+        <v>RS_Prod</v>
+      </c>
+      <c r="I34" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>RS</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>29</v>
       </c>
@@ -1285,8 +1772,16 @@
         <v>63</v>
       </c>
       <c r="C35" s="2"/>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H35" t="str">
+        <f t="shared" si="0"/>
+        <v>SK_Prod</v>
+      </c>
+      <c r="I35" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>SK</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -1294,8 +1789,16 @@
         <v>60</v>
       </c>
       <c r="C36" s="2"/>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H36" t="str">
+        <f t="shared" si="0"/>
+        <v>SI_Prod</v>
+      </c>
+      <c r="I36" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>SI</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -1303,8 +1806,16 @@
         <v>59</v>
       </c>
       <c r="C37" s="2"/>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H37" t="str">
+        <f t="shared" si="0"/>
+        <v>CH_Prod</v>
+      </c>
+      <c r="I37" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>CH</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>51</v>
       </c>
@@ -1314,8 +1825,16 @@
       <c r="C38" s="2">
         <v>1.9</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H38" t="str">
+        <f t="shared" si="0"/>
+        <v>TN_Prod</v>
+      </c>
+      <c r="I38" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>TN</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>47</v>
       </c>
@@ -1323,8 +1842,16 @@
         <v>10</v>
       </c>
       <c r="C39" s="2"/>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H39" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_Prod</v>
+      </c>
+      <c r="I39" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>TR</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>11</v>
       </c>
@@ -1334,8 +1861,16 @@
       <c r="C40" s="2">
         <v>39.5</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H40" t="str">
+        <f t="shared" si="0"/>
+        <v>UK_Prod</v>
+      </c>
+      <c r="I40" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>UK</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>39</v>
       </c>
@@ -1345,8 +1880,16 @@
       <c r="C41" s="2">
         <v>19</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="H41" t="str">
+        <f t="shared" si="0"/>
+        <v>UA_Prod</v>
+      </c>
+      <c r="I41" t="str">
+        <f>Table2[[#This Row],[Country]]</f>
+        <v>UA</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>90</v>
       </c>
@@ -1357,7 +1900,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>85</v>
       </c>
@@ -1798,18 +2341,18 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD7211D-DC17-4DD6-B657-CA08F8FBC20F}">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="B1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1">
-        <v>1455.1</v>
+        <v>96</v>
+      </c>
+      <c r="C1" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -1927,10 +2470,10 @@
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C12">
-        <v>669</v>
+        <v>344.24799999999993</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -1938,10 +2481,10 @@
         <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C13">
-        <v>344.24799999999993</v>
+        <v>328</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -1949,10 +2492,10 @@
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C14">
-        <v>328</v>
+        <v>613.71600000000001</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
@@ -1960,10 +2503,10 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C15">
-        <v>613.71600000000001</v>
+        <v>136.11199999999999</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
@@ -1971,10 +2514,10 @@
         <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C16">
-        <v>136.11199999999999</v>
+        <v>233.5</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
@@ -1982,10 +2525,10 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C17">
-        <v>233.5</v>
+        <v>1803.77</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
@@ -1993,21 +2536,21 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="C18">
-        <v>1803.77</v>
+        <v>26.71</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" t="s">
         <v>19</v>
       </c>
-      <c r="B19" t="s">
-        <v>43</v>
-      </c>
       <c r="C19">
-        <v>26.71</v>
+        <v>339.96799999999996</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
@@ -2015,10 +2558,10 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C20">
-        <v>339.96799999999996</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -2026,10 +2569,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C21">
-        <v>1150</v>
+        <v>112.5</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -2037,10 +2580,10 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C22">
-        <v>112.5</v>
+        <v>246.5</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -2048,21 +2591,21 @@
         <v>20</v>
       </c>
       <c r="B23" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C23">
-        <v>246.5</v>
+        <v>153.1</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" t="s">
         <v>20</v>
       </c>
-      <c r="B24" t="s">
-        <v>30</v>
-      </c>
       <c r="C24">
-        <v>153.1</v>
+        <v>193.5</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
@@ -2070,10 +2613,10 @@
         <v>21</v>
       </c>
       <c r="B25" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C25">
-        <v>193.5</v>
+        <v>431.4</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
@@ -2081,10 +2624,10 @@
         <v>21</v>
       </c>
       <c r="B26" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C26">
-        <v>431.4</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
@@ -2092,21 +2635,21 @@
         <v>21</v>
       </c>
       <c r="B27" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="C27">
-        <v>28.5</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="C28">
-        <v>4.3</v>
+        <v>172.8</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
@@ -2114,10 +2657,10 @@
         <v>22</v>
       </c>
       <c r="B29" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C29">
-        <v>172.8</v>
+        <v>640.4</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
@@ -2125,21 +2668,21 @@
         <v>22</v>
       </c>
       <c r="B30" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C30">
-        <v>640.4</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B31" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C31">
-        <v>100</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
@@ -2147,21 +2690,21 @@
         <v>23</v>
       </c>
       <c r="B32" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C32">
-        <v>21.5</v>
+        <v>53.7</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
+        <v>24</v>
+      </c>
+      <c r="B33" t="s">
         <v>23</v>
       </c>
-      <c r="B33" t="s">
-        <v>24</v>
-      </c>
       <c r="C33">
-        <v>53.7</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
@@ -2169,21 +2712,21 @@
         <v>24</v>
       </c>
       <c r="B34" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C34">
-        <v>7.7</v>
+        <v>48.57</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B35" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="C35">
-        <v>48.57</v>
+        <v>270</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
@@ -2191,10 +2734,10 @@
         <v>25</v>
       </c>
       <c r="B36" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C36">
-        <v>270</v>
+        <v>223</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
@@ -2202,43 +2745,43 @@
         <v>25</v>
       </c>
       <c r="B37" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="C37">
-        <v>223</v>
+        <v>164.572</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B38" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="C38">
-        <v>164.572</v>
+        <v>4.1189999999999998</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B39" t="s">
         <v>19</v>
       </c>
       <c r="C39">
-        <v>4.1189999999999998</v>
+        <v>931.6</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B40" t="s">
         <v>19</v>
       </c>
       <c r="C40">
-        <v>931.6</v>
+        <v>1231.759</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
@@ -2246,10 +2789,10 @@
         <v>28</v>
       </c>
       <c r="B41" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C41">
-        <v>1231.759</v>
+        <v>28</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
@@ -2257,21 +2800,21 @@
         <v>28</v>
       </c>
       <c r="B42" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C42">
-        <v>28</v>
+        <v>1246.4000000000001</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B43" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C43">
-        <v>1246.4000000000001</v>
+        <v>1570.4</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
@@ -2279,10 +2822,10 @@
         <v>29</v>
       </c>
       <c r="B44" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C44">
-        <v>1570.4</v>
+        <v>457.6</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
@@ -2290,10 +2833,10 @@
         <v>29</v>
       </c>
       <c r="B45" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C45">
-        <v>457.6</v>
+        <v>128.9</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
@@ -2301,21 +2844,21 @@
         <v>29</v>
       </c>
       <c r="B46" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C46">
-        <v>128.9</v>
+        <v>416</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B47" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="C47">
-        <v>416</v>
+        <v>77.400000000000006</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
@@ -2323,10 +2866,10 @@
         <v>30</v>
       </c>
       <c r="B48" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C48">
-        <v>77.400000000000006</v>
+        <v>50.883000000000003</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
@@ -2334,10 +2877,10 @@
         <v>30</v>
       </c>
       <c r="B49" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C49">
-        <v>50.883000000000003</v>
+        <v>142</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
@@ -2345,21 +2888,21 @@
         <v>30</v>
       </c>
       <c r="B50" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C50">
-        <v>142</v>
+        <v>77.5</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B51" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C51">
-        <v>77.5</v>
+        <v>335.26</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
@@ -2367,21 +2910,21 @@
         <v>31</v>
       </c>
       <c r="B52" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C52">
-        <v>335.26</v>
+        <v>17.98</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
+        <v>32</v>
+      </c>
+      <c r="B53" t="s">
         <v>31</v>
       </c>
-      <c r="B53" t="s">
-        <v>45</v>
-      </c>
       <c r="C53">
-        <v>17.98</v>
+        <v>398.13</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
@@ -2389,10 +2932,10 @@
         <v>32</v>
       </c>
       <c r="B54" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C54">
-        <v>398.13</v>
+        <v>117.8</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
@@ -2400,10 +2943,10 @@
         <v>32</v>
       </c>
       <c r="B55" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C55">
-        <v>117.8</v>
+        <v>148.15</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
@@ -2411,10 +2954,10 @@
         <v>32</v>
       </c>
       <c r="B56" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="C56">
-        <v>148.15</v>
+        <v>27.38</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
@@ -2422,21 +2965,21 @@
         <v>32</v>
       </c>
       <c r="B57" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C57">
-        <v>27.38</v>
+        <v>497.16</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
+        <v>33</v>
+      </c>
+      <c r="B58" t="s">
         <v>32</v>
       </c>
-      <c r="B58" t="s">
-        <v>47</v>
-      </c>
       <c r="C58">
-        <v>497.16</v>
+        <v>64.819999999999993</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
@@ -2444,21 +2987,21 @@
         <v>33</v>
       </c>
       <c r="B59" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C59">
-        <v>64.819999999999993</v>
+        <v>53.4</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B60" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C60">
-        <v>53.4</v>
+        <v>50.3</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
@@ -2466,10 +3009,10 @@
         <v>34</v>
       </c>
       <c r="B61" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C61">
-        <v>50.3</v>
+        <v>805.75000000000011</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
@@ -2477,10 +3020,10 @@
         <v>34</v>
       </c>
       <c r="B62" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="C62">
-        <v>805.75000000000011</v>
+        <v>122.2</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
@@ -2488,21 +3031,21 @@
         <v>34</v>
       </c>
       <c r="B63" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C63">
-        <v>122.2</v>
+        <v>16.100000000000001</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B64" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C64">
-        <v>16.100000000000001</v>
+        <v>67.599999999999994</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.35">
@@ -2510,21 +3053,21 @@
         <v>35</v>
       </c>
       <c r="B65" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="C65">
-        <v>67.599999999999994</v>
+        <v>114.2</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
+        <v>36</v>
+      </c>
+      <c r="B66" t="s">
         <v>35</v>
       </c>
-      <c r="B66" t="s">
-        <v>41</v>
-      </c>
       <c r="C66">
-        <v>114.2</v>
+        <v>65.099999999999994</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.35">
@@ -2532,21 +3075,21 @@
         <v>36</v>
       </c>
       <c r="B67" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C67">
-        <v>65.099999999999994</v>
+        <v>85</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B68" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="C68">
-        <v>85</v>
+        <v>224.4</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.35">
@@ -2554,32 +3097,32 @@
         <v>37</v>
       </c>
       <c r="B69" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="C69">
-        <v>224.4</v>
+        <v>144</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
+        <v>38</v>
+      </c>
+      <c r="B70" t="s">
         <v>37</v>
       </c>
-      <c r="B70" t="s">
-        <v>38</v>
-      </c>
       <c r="C70">
-        <v>144</v>
+        <v>80</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B71" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C71">
-        <v>80</v>
+        <v>135.6</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.35">
@@ -2587,10 +3130,10 @@
         <v>39</v>
       </c>
       <c r="B72" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C72">
-        <v>135.6</v>
+        <v>2277.6</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.35">
@@ -2598,10 +3141,10 @@
         <v>39</v>
       </c>
       <c r="B73" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C73">
-        <v>2277.6</v>
+        <v>515.6</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.35">
@@ -2609,32 +3152,32 @@
         <v>39</v>
       </c>
       <c r="B74" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C74">
-        <v>515.6</v>
+        <v>1163.4000000000001</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B75" t="s">
         <v>34</v>
       </c>
       <c r="C75">
-        <v>1163.4000000000001</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B76" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="C76">
-        <v>2.2000000000000002</v>
+        <v>1742</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.35">
@@ -2642,10 +3185,10 @@
         <v>41</v>
       </c>
       <c r="B77" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="C77">
-        <v>1742</v>
+        <v>168</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.35">
@@ -2653,32 +3196,32 @@
         <v>41</v>
       </c>
       <c r="B78" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="C78">
-        <v>168</v>
+        <v>220</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B79" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="C79">
-        <v>220</v>
+        <v>487.1</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B80" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="C80">
-        <v>487.1</v>
+        <v>576.03</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.35">
@@ -2686,21 +3229,21 @@
         <v>47</v>
       </c>
       <c r="B81" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C81">
-        <v>576.03</v>
+        <v>398.6</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B82" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="C82">
-        <v>398.6</v>
+        <v>1499.1</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.35">
@@ -2708,10 +3251,10 @@
         <v>49</v>
       </c>
       <c r="B83" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C83">
-        <v>1499.1</v>
+        <v>488</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.35">
@@ -2719,10 +3262,10 @@
         <v>49</v>
       </c>
       <c r="B84" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C84">
-        <v>488</v>
+        <v>2210.5639999999999</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.35">
@@ -2730,54 +3273,54 @@
         <v>49</v>
       </c>
       <c r="B85" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C85">
-        <v>2210.5639999999999</v>
+        <v>570</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B86" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="C86">
-        <v>570</v>
+        <v>731.7</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B87" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="C87">
-        <v>731.7</v>
+        <v>1138.0999999999999</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B88" t="s">
         <v>21</v>
       </c>
       <c r="C88">
-        <v>1138.0999999999999</v>
+        <v>475.8</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B89" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C89">
-        <v>475.8</v>
+        <v>1203.4999999999998</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.35">
@@ -2785,21 +3328,318 @@
         <v>53</v>
       </c>
       <c r="B90" t="s">
+        <v>35</v>
+      </c>
+      <c r="C90">
+        <v>325.39999999999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58F6DC53-AE01-4DBE-BF9B-43427CD51EF0}">
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2">
+        <v>1334</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" t="s">
         <v>27</v>
       </c>
-      <c r="C90">
-        <v>1203.4999999999998</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
-        <v>53</v>
-      </c>
-      <c r="B91" t="s">
-        <v>35</v>
-      </c>
-      <c r="C91">
-        <v>325.39999999999998</v>
+      <c r="C4">
+        <v>135.6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5">
+        <f>1799+436.8</f>
+        <v>2235.8000000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6">
+        <v>517.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7">
+        <v>245.8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8">
+        <v>467.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9">
+        <v>33.380000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10">
+        <v>701.8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13">
+        <v>493.7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15">
+        <v>337.1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16">
+        <v>442.8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17">
+        <v>1247</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18">
+        <v>963.6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19">
+        <v>459.6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20">
+        <v>568.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>49</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21">
+        <v>1406</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" t="s">
+        <v>102</v>
+      </c>
+      <c r="C22">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23">
+        <v>227.2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24">
+        <v>184.8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26">
+        <v>321.89999999999998</v>
+      </c>
+      <c r="E26" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27">
+        <v>321.89999999999998</v>
+      </c>
+      <c r="E27" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
improve Russian case script
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678E5D9E-05E8-4229-A41D-B29216D894B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93E6A5C2-2DEF-4F71-B2C6-17C7854374C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="10" windowWidth="19180" windowHeight="10060" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="112">
   <si>
     <t>Belgium</t>
   </si>
@@ -361,6 +361,21 @@
   </si>
   <si>
     <t>_Prod</t>
+  </si>
+  <si>
+    <t>Limitation</t>
+  </si>
+  <si>
+    <t>Limitation in TWh</t>
+  </si>
+  <si>
+    <t>TWh [2020]</t>
+  </si>
+  <si>
+    <t>GWh/a</t>
+  </si>
+  <si>
+    <t>TWh/a</t>
   </si>
 </sst>
 </file>
@@ -407,7 +422,13 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
@@ -428,30 +449,36 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D12A1D17-871E-4E66-A144-F2ADD46C5E00}" name="Table2" displayName="Table2" ref="A1:C42" totalsRowShown="0">
-  <autoFilter ref="A1:C42" xr:uid="{D12A1D17-871E-4E66-A144-F2ADD46C5E00}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D12A1D17-871E-4E66-A144-F2ADD46C5E00}" name="Table2" displayName="Table2" ref="A1:D42" totalsRowShown="0">
+  <autoFilter ref="A1:D42" xr:uid="{D12A1D17-871E-4E66-A144-F2ADD46C5E00}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C41">
     <sortCondition ref="B1:B41"/>
   </sortState>
-  <tableColumns count="3">
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{D3465064-BCEE-4D04-A8E6-DEAE11BBDA92}" name="Country"/>
     <tableColumn id="2" xr3:uid="{D66D54B4-4DED-47C6-BE50-755A236428ED}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="1">
+      <calculatedColumnFormula>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}" name="Table1" displayName="Table1" ref="A1:C39" totalsRowShown="0">
-  <autoFilter ref="A1:C39" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}" name="Table1" displayName="Table1" ref="A1:D39" totalsRowShown="0">
+  <autoFilter ref="A1:D39" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C39">
     <sortCondition ref="B1:B39"/>
   </sortState>
-  <tableColumns count="3">
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="0">
+      <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -720,10 +747,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -739,14 +766,20 @@
       <c r="E1" t="s">
         <v>14</v>
       </c>
-      <c r="J1" t="s">
+      <c r="F1" t="s">
+        <v>107</v>
+      </c>
+      <c r="G1" t="s">
+        <v>108</v>
+      </c>
+      <c r="L1" t="s">
         <v>95</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -763,22 +796,30 @@
       <c r="E2">
         <v>9</v>
       </c>
-      <c r="G2" t="s">
+      <c r="F2">
+        <f>IF(B2&gt;E2,B2,E2)</f>
+        <v>11.4</v>
+      </c>
+      <c r="G2">
+        <f>F2*9.77</f>
+        <v>111.378</v>
+      </c>
+      <c r="I2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>105</v>
       </c>
-      <c r="J2" t="str">
-        <f>_xlfn.CONCAT(G2,H2)</f>
+      <c r="L2" t="str">
+        <f>_xlfn.CONCAT(I2,J2)</f>
         <v>BE_LNG</v>
       </c>
-      <c r="K2" t="str">
-        <f>G2</f>
+      <c r="M2" t="str">
+        <f>I2</f>
         <v>BE</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -795,22 +836,30 @@
       <c r="E3">
         <v>33</v>
       </c>
-      <c r="G3" t="s">
+      <c r="F3">
+        <f t="shared" ref="F3:F14" si="1">IF(B3&gt;E3,B3,E3)</f>
+        <v>33</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G14" si="2">F3*9.77</f>
+        <v>322.40999999999997</v>
+      </c>
+      <c r="I3" t="s">
         <v>25</v>
       </c>
-      <c r="H3" t="s">
+      <c r="J3" t="s">
         <v>105</v>
       </c>
-      <c r="J3" t="str">
-        <f t="shared" ref="J3:J13" si="1">_xlfn.CONCAT(G3,H3)</f>
+      <c r="L3" t="str">
+        <f t="shared" ref="L3:L13" si="3">_xlfn.CONCAT(I3,J3)</f>
         <v>FR_LNG</v>
       </c>
-      <c r="K3" t="str">
-        <f t="shared" ref="K3:K13" si="2">G3</f>
+      <c r="M3" t="str">
+        <f t="shared" ref="M3:M13" si="4">I3</f>
         <v>FR</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -827,22 +876,30 @@
       <c r="E4">
         <v>7.5</v>
       </c>
-      <c r="G4" t="s">
+      <c r="F4">
+        <f t="shared" si="1"/>
+        <v>7.5</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="2"/>
+        <v>73.274999999999991</v>
+      </c>
+      <c r="I4" t="s">
         <v>33</v>
       </c>
-      <c r="H4" t="s">
+      <c r="J4" t="s">
         <v>105</v>
       </c>
-      <c r="J4" t="str">
-        <f t="shared" si="1"/>
+      <c r="L4" t="str">
+        <f t="shared" si="3"/>
         <v>GR_LNG</v>
       </c>
-      <c r="K4" t="str">
-        <f t="shared" si="2"/>
+      <c r="M4" t="str">
+        <f t="shared" si="4"/>
         <v>GR</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -859,22 +916,30 @@
       <c r="E5">
         <v>15.8</v>
       </c>
-      <c r="G5" t="s">
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>15.95</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="2"/>
+        <v>155.83149999999998</v>
+      </c>
+      <c r="I5" t="s">
         <v>21</v>
       </c>
-      <c r="H5" t="s">
+      <c r="J5" t="s">
         <v>105</v>
       </c>
-      <c r="J5" t="str">
-        <f t="shared" si="1"/>
+      <c r="L5" t="str">
+        <f t="shared" si="3"/>
         <v>IT_LNG</v>
       </c>
-      <c r="K5" t="str">
-        <f t="shared" si="2"/>
+      <c r="M5" t="str">
+        <f t="shared" si="4"/>
         <v>IT</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -891,22 +956,30 @@
       <c r="E6">
         <v>2.6</v>
       </c>
-      <c r="G6" t="s">
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>2.6</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="2"/>
+        <v>25.402000000000001</v>
+      </c>
+      <c r="I6" t="s">
         <v>24</v>
       </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>105</v>
       </c>
-      <c r="J6" t="str">
-        <f t="shared" si="1"/>
+      <c r="L6" t="str">
+        <f t="shared" si="3"/>
         <v>HR_LNG</v>
       </c>
-      <c r="K6" t="str">
-        <f t="shared" si="2"/>
+      <c r="M6" t="str">
+        <f t="shared" si="4"/>
         <v>HR</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -923,22 +996,30 @@
       <c r="E7">
         <v>4</v>
       </c>
-      <c r="G7" t="s">
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="2"/>
+        <v>39.08</v>
+      </c>
+      <c r="I7" t="s">
         <v>35</v>
       </c>
-      <c r="H7" t="s">
+      <c r="J7" t="s">
         <v>105</v>
       </c>
-      <c r="J7" t="str">
-        <f t="shared" si="1"/>
+      <c r="L7" t="str">
+        <f t="shared" si="3"/>
         <v>LT_LNG</v>
       </c>
-      <c r="K7" t="str">
-        <f t="shared" si="2"/>
+      <c r="M7" t="str">
+        <f t="shared" si="4"/>
         <v>LT</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -955,22 +1036,30 @@
       <c r="E8">
         <v>12.5</v>
       </c>
-      <c r="G8" t="s">
+      <c r="F8">
+        <f t="shared" si="1"/>
+        <v>12.5</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="2"/>
+        <v>122.125</v>
+      </c>
+      <c r="I8" t="s">
         <v>18</v>
       </c>
-      <c r="H8" t="s">
+      <c r="J8" t="s">
         <v>105</v>
       </c>
-      <c r="J8" t="str">
-        <f t="shared" si="1"/>
+      <c r="L8" t="str">
+        <f t="shared" si="3"/>
         <v>NL_LNG</v>
       </c>
-      <c r="K8" t="str">
-        <f t="shared" si="2"/>
+      <c r="M8" t="str">
+        <f t="shared" si="4"/>
         <v>NL</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -987,22 +1076,30 @@
       <c r="E9">
         <v>5.8</v>
       </c>
-      <c r="G9" t="s">
+      <c r="F9">
+        <f t="shared" si="1"/>
+        <v>6.2</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="2"/>
+        <v>60.573999999999998</v>
+      </c>
+      <c r="I9" t="s">
         <v>27</v>
       </c>
-      <c r="H9" t="s">
+      <c r="J9" t="s">
         <v>105</v>
       </c>
-      <c r="J9" t="str">
-        <f t="shared" si="1"/>
+      <c r="L9" t="str">
+        <f t="shared" si="3"/>
         <v>PL_LNG</v>
       </c>
-      <c r="K9" t="str">
-        <f t="shared" si="2"/>
+      <c r="M9" t="str">
+        <f t="shared" si="4"/>
         <v>PL</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -1019,22 +1116,30 @@
       <c r="E10">
         <v>7.3</v>
       </c>
-      <c r="G10" t="s">
+      <c r="F10">
+        <f t="shared" si="1"/>
+        <v>7.6</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="2"/>
+        <v>74.251999999999995</v>
+      </c>
+      <c r="I10" t="s">
         <v>38</v>
       </c>
-      <c r="H10" t="s">
+      <c r="J10" t="s">
         <v>105</v>
       </c>
-      <c r="J10" t="str">
-        <f t="shared" si="1"/>
+      <c r="L10" t="str">
+        <f t="shared" si="3"/>
         <v>PT_LNG</v>
       </c>
-      <c r="K10" t="str">
-        <f t="shared" si="2"/>
+      <c r="M10" t="str">
+        <f t="shared" si="4"/>
         <v>PT</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1051,22 +1156,30 @@
       <c r="E11">
         <v>67.099999999999994</v>
       </c>
-      <c r="G11" t="s">
+      <c r="F11">
+        <f t="shared" si="1"/>
+        <v>67.099999999999994</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="2"/>
+        <v>655.56699999999989</v>
+      </c>
+      <c r="I11" t="s">
         <v>37</v>
       </c>
-      <c r="H11" t="s">
+      <c r="J11" t="s">
         <v>105</v>
       </c>
-      <c r="J11" t="str">
-        <f t="shared" si="1"/>
+      <c r="L11" t="str">
+        <f t="shared" si="3"/>
         <v>ES_LNG</v>
       </c>
-      <c r="K11" t="str">
-        <f t="shared" si="2"/>
+      <c r="M11" t="str">
+        <f t="shared" si="4"/>
         <v>ES</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1083,22 +1196,30 @@
       <c r="E12">
         <v>14.8</v>
       </c>
-      <c r="G12" t="s">
+      <c r="F12">
+        <f t="shared" si="1"/>
+        <v>43.6</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="2"/>
+        <v>425.97199999999998</v>
+      </c>
+      <c r="I12" t="s">
         <v>47</v>
       </c>
-      <c r="H12" t="s">
+      <c r="J12" t="s">
         <v>105</v>
       </c>
-      <c r="J12" t="str">
-        <f t="shared" si="1"/>
+      <c r="L12" t="str">
+        <f t="shared" si="3"/>
         <v>TR_LNG</v>
       </c>
-      <c r="K12" t="str">
-        <f t="shared" si="2"/>
+      <c r="M12" t="str">
+        <f t="shared" si="4"/>
         <v>TR</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1115,22 +1236,30 @@
       <c r="E13">
         <v>52.3</v>
       </c>
-      <c r="G13" t="s">
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>52.3</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="2"/>
+        <v>510.97099999999995</v>
+      </c>
+      <c r="I13" t="s">
         <v>11</v>
       </c>
-      <c r="H13" t="s">
+      <c r="J13" t="s">
         <v>105</v>
       </c>
-      <c r="J13" t="str">
-        <f t="shared" si="1"/>
+      <c r="L13" t="str">
+        <f t="shared" si="3"/>
         <v>UK_LNG</v>
       </c>
-      <c r="K13" t="str">
-        <f t="shared" si="2"/>
+      <c r="M13" t="str">
+        <f t="shared" si="4"/>
         <v>UK</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>94</v>
       </c>
@@ -1141,11 +1270,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G14" t="s">
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>0.7</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="2"/>
+        <v>6.8389999999999995</v>
+      </c>
+      <c r="I14" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="D15" s="1"/>
     </row>
   </sheetData>
@@ -1155,15 +1292,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF82F4-4954-4D06-9A30-AE8575CA18DE}">
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
     <col min="2" max="2" width="12.54296875" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="3" max="4" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -1173,14 +1310,17 @@
       <c r="C1" t="s">
         <v>86</v>
       </c>
-      <c r="H1" t="s">
+      <c r="D1" t="s">
+        <v>109</v>
+      </c>
+      <c r="I1" t="s">
         <v>95</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -1188,19 +1328,23 @@
         <v>74</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="E2" t="s">
+      <c r="D2" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
         <v>106</v>
       </c>
-      <c r="H2" t="str">
-        <f>_xlfn.CONCAT(A2,$E$2)</f>
+      <c r="I2" t="str">
+        <f>_xlfn.CONCAT(A2,$F$2)</f>
         <v>AL_Prod</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>AL</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -1210,16 +1354,20 @@
       <c r="C3" s="2">
         <v>81.5</v>
       </c>
-      <c r="H3" t="str">
-        <f t="shared" ref="H3:H42" si="0">_xlfn.CONCAT(A3,$E$2)</f>
+      <c r="D3" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>796.255</v>
+      </c>
+      <c r="I3" t="str">
+        <f t="shared" ref="I3:I41" si="0">_xlfn.CONCAT(A3,$F$2)</f>
         <v>DZ_Prod</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>DZ</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -1227,16 +1375,20 @@
         <v>58</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="H4" t="str">
+      <c r="D4" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I4" t="str">
         <f t="shared" si="0"/>
         <v>AT_Prod</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>AT</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>53</v>
       </c>
@@ -1244,16 +1396,20 @@
         <v>82</v>
       </c>
       <c r="C5" s="2"/>
-      <c r="H5" t="str">
+      <c r="D5" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I5" t="str">
         <f t="shared" si="0"/>
         <v>BY_Prod</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>BY</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1261,16 +1417,20 @@
         <v>0</v>
       </c>
       <c r="C6" s="2"/>
-      <c r="H6" t="str">
+      <c r="D6" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I6" t="str">
         <f t="shared" si="0"/>
         <v>BE_Prod</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>BE</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>45</v>
       </c>
@@ -1278,16 +1438,20 @@
         <v>76</v>
       </c>
       <c r="C7" s="2"/>
-      <c r="H7" t="str">
+      <c r="D7" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I7" t="str">
         <f t="shared" si="0"/>
         <v>BA_Prod</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>BA</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1295,16 +1459,20 @@
         <v>65</v>
       </c>
       <c r="C8" s="2"/>
-      <c r="H8" t="str">
+      <c r="D8" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I8" t="str">
         <f t="shared" si="0"/>
         <v>BG_Prod</v>
       </c>
-      <c r="I8" t="str">
+      <c r="J8" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>BG</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -1312,16 +1480,20 @@
         <v>5</v>
       </c>
       <c r="C9" s="2"/>
-      <c r="H9" t="str">
+      <c r="D9" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I9" t="str">
         <f t="shared" si="0"/>
         <v>HR_Prod</v>
       </c>
-      <c r="I9" t="str">
+      <c r="J9" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>HR</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1329,16 +1501,20 @@
         <v>62</v>
       </c>
       <c r="C10" s="2"/>
-      <c r="H10" t="str">
+      <c r="D10" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I10" t="str">
         <f t="shared" si="0"/>
         <v>CZ_Prod</v>
       </c>
-      <c r="I10" t="str">
+      <c r="J10" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>CZ</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -1348,16 +1524,20 @@
       <c r="C11" s="2">
         <v>1.4</v>
       </c>
-      <c r="H11" t="str">
+      <c r="D11" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>13.677999999999999</v>
+      </c>
+      <c r="I11" t="str">
         <f t="shared" si="0"/>
         <v>DK_Prod</v>
       </c>
-      <c r="I11" t="str">
+      <c r="J11" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>DK</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>37</v>
       </c>
@@ -1365,16 +1545,20 @@
         <v>67</v>
       </c>
       <c r="C12" s="2"/>
-      <c r="H12" t="str">
+      <c r="D12" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I12" t="str">
         <f t="shared" si="0"/>
         <v>ES_Prod</v>
       </c>
-      <c r="I12" t="str">
+      <c r="J12" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>ES</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>54</v>
       </c>
@@ -1382,16 +1566,20 @@
         <v>67</v>
       </c>
       <c r="C13" s="2"/>
-      <c r="H13" t="str">
+      <c r="D13" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I13" t="str">
         <f t="shared" si="0"/>
         <v>EE_Prod</v>
       </c>
-      <c r="I13" t="str">
+      <c r="J13" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>EE</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>55</v>
       </c>
@@ -1399,16 +1587,20 @@
         <v>87</v>
       </c>
       <c r="C14" s="2"/>
-      <c r="H14" t="str">
+      <c r="D14" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I14" t="str">
         <f t="shared" si="0"/>
         <v>FI_Prod</v>
       </c>
-      <c r="I14" t="str">
+      <c r="J14" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>FI</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -1416,16 +1608,20 @@
         <v>2</v>
       </c>
       <c r="C15" s="2"/>
-      <c r="H15" t="str">
+      <c r="D15" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I15" t="str">
         <f t="shared" si="0"/>
         <v>FR_Prod</v>
       </c>
-      <c r="I15" t="str">
+      <c r="J15" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>FR</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -1435,16 +1631,20 @@
       <c r="C16" s="2">
         <v>4.5</v>
       </c>
-      <c r="H16" t="str">
+      <c r="D16" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>43.964999999999996</v>
+      </c>
+      <c r="I16" t="str">
         <f t="shared" si="0"/>
         <v>DE_Prod</v>
       </c>
-      <c r="I16" t="str">
+      <c r="J16" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>DE</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -1452,16 +1652,20 @@
         <v>3</v>
       </c>
       <c r="C17" s="2"/>
-      <c r="H17" t="str">
+      <c r="D17" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I17" t="str">
         <f t="shared" si="0"/>
         <v>GR_Prod</v>
       </c>
-      <c r="I17" t="str">
+      <c r="J17" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>GR</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1469,16 +1673,20 @@
         <v>64</v>
       </c>
       <c r="C18" s="2"/>
-      <c r="H18" t="str">
+      <c r="D18" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I18" t="str">
         <f t="shared" si="0"/>
         <v>HU_Prod</v>
       </c>
-      <c r="I18" t="str">
+      <c r="J18" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>HU</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>44</v>
       </c>
@@ -1486,16 +1694,20 @@
         <v>75</v>
       </c>
       <c r="C19" s="2"/>
-      <c r="H19" t="str">
+      <c r="D19" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I19" t="str">
         <f t="shared" si="0"/>
         <v>IE_Prod</v>
       </c>
-      <c r="I19" t="str">
+      <c r="J19" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>IE</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1505,16 +1717,20 @@
       <c r="C20" s="2">
         <v>3.9</v>
       </c>
-      <c r="H20" t="str">
+      <c r="D20" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>38.102999999999994</v>
+      </c>
+      <c r="I20" t="str">
         <f t="shared" si="0"/>
         <v>IT_Prod</v>
       </c>
-      <c r="I20" t="str">
+      <c r="J20" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>IT</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -1522,16 +1738,20 @@
         <v>66</v>
       </c>
       <c r="C21" s="2"/>
-      <c r="H21" t="str">
+      <c r="D21" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I21" t="str">
         <f t="shared" si="0"/>
         <v>LV_Prod</v>
       </c>
-      <c r="I21" t="str">
+      <c r="J21" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>LV</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>52</v>
       </c>
@@ -1541,16 +1761,20 @@
       <c r="C22" s="2">
         <v>13.3</v>
       </c>
-      <c r="H22" t="str">
+      <c r="D22" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>129.941</v>
+      </c>
+      <c r="I22" t="str">
         <f t="shared" si="0"/>
         <v>LY_Prod</v>
       </c>
-      <c r="I22" t="str">
+      <c r="J22" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>LY</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>35</v>
       </c>
@@ -1558,16 +1782,20 @@
         <v>6</v>
       </c>
       <c r="C23" s="2"/>
-      <c r="H23" t="str">
+      <c r="D23" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I23" t="str">
         <f t="shared" si="0"/>
         <v>LT_Prod</v>
       </c>
-      <c r="I23" t="str">
+      <c r="J23" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>LT</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>43</v>
       </c>
@@ -1575,16 +1803,20 @@
         <v>71</v>
       </c>
       <c r="C24" s="2"/>
-      <c r="H24" t="str">
+      <c r="D24" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I24" t="str">
         <f t="shared" si="0"/>
         <v>LU_Prod</v>
       </c>
-      <c r="I24" t="str">
+      <c r="J24" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>LU</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>40</v>
       </c>
@@ -1592,16 +1824,20 @@
         <v>69</v>
       </c>
       <c r="C25" s="2"/>
-      <c r="H25" t="str">
+      <c r="D25" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I25" t="str">
         <f t="shared" si="0"/>
         <v>MD_Prod</v>
       </c>
-      <c r="I25" t="str">
+      <c r="J25" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>MD</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -1611,16 +1847,20 @@
       <c r="C26" s="2">
         <v>20</v>
       </c>
-      <c r="H26" t="str">
+      <c r="D26" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>195.39999999999998</v>
+      </c>
+      <c r="I26" t="str">
         <f t="shared" si="0"/>
         <v>NL_Prod</v>
       </c>
-      <c r="I26" t="str">
+      <c r="J26" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>NL</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>46</v>
       </c>
@@ -1628,16 +1868,20 @@
         <v>77</v>
       </c>
       <c r="C27" s="2"/>
-      <c r="H27" t="str">
+      <c r="D27" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I27" t="str">
         <f t="shared" si="0"/>
         <v>MK_Prod</v>
       </c>
-      <c r="I27" t="str">
+      <c r="J27" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>MK</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>49</v>
       </c>
@@ -1647,16 +1891,20 @@
       <c r="C28" s="2">
         <v>111.5</v>
       </c>
-      <c r="H28" t="str">
+      <c r="D28" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>1089.355</v>
+      </c>
+      <c r="I28" t="str">
         <f t="shared" si="0"/>
         <v>NO_Prod</v>
       </c>
-      <c r="I28" t="str">
+      <c r="J28" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>NO</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1666,16 +1914,20 @@
       <c r="C29" s="2">
         <v>3.9</v>
       </c>
-      <c r="H29" t="str">
+      <c r="D29" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>38.102999999999994</v>
+      </c>
+      <c r="I29" t="str">
         <f t="shared" si="0"/>
         <v>PL_Prod</v>
       </c>
-      <c r="I29" t="str">
+      <c r="J29" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>PL</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>38</v>
       </c>
@@ -1683,16 +1935,20 @@
         <v>1</v>
       </c>
       <c r="C30" s="2"/>
-      <c r="H30" t="str">
+      <c r="D30" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I30" t="str">
         <f t="shared" si="0"/>
         <v>PT_Prod</v>
       </c>
-      <c r="I30" t="str">
+      <c r="J30" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>PT</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -1702,16 +1958,20 @@
       <c r="C31" s="2">
         <v>8.6999999999999993</v>
       </c>
-      <c r="H31" t="str">
+      <c r="D31" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>84.998999999999995</v>
+      </c>
+      <c r="I31" t="str">
         <f t="shared" si="0"/>
         <v>RO_Prod</v>
       </c>
-      <c r="I31" t="str">
+      <c r="J31" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>RO</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>41</v>
       </c>
@@ -1721,16 +1981,20 @@
       <c r="C32" s="2">
         <v>638.5</v>
       </c>
-      <c r="H32" t="str">
+      <c r="D32" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>6238.1449999999995</v>
+      </c>
+      <c r="I32" t="str">
         <f t="shared" si="0"/>
         <v>RU_Prod</v>
       </c>
-      <c r="I32" t="str">
+      <c r="J32" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>RU</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>48</v>
       </c>
@@ -1738,16 +2002,20 @@
         <v>78</v>
       </c>
       <c r="C33" s="2"/>
-      <c r="H33" t="str">
+      <c r="D33" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I33" t="str">
         <f t="shared" si="0"/>
         <v>SM_Prod</v>
       </c>
-      <c r="I33" t="str">
+      <c r="J33" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>SM</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>31</v>
       </c>
@@ -1755,16 +2023,20 @@
         <v>73</v>
       </c>
       <c r="C34" s="2"/>
-      <c r="H34" t="str">
+      <c r="D34" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I34" t="str">
         <f t="shared" si="0"/>
         <v>RS_Prod</v>
       </c>
-      <c r="I34" t="str">
+      <c r="J34" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>RS</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>29</v>
       </c>
@@ -1772,16 +2044,20 @@
         <v>63</v>
       </c>
       <c r="C35" s="2"/>
-      <c r="H35" t="str">
+      <c r="D35" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I35" t="str">
         <f t="shared" si="0"/>
         <v>SK_Prod</v>
       </c>
-      <c r="I35" t="str">
+      <c r="J35" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>SK</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>23</v>
       </c>
@@ -1789,16 +2065,20 @@
         <v>60</v>
       </c>
       <c r="C36" s="2"/>
-      <c r="H36" t="str">
+      <c r="D36" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I36" t="str">
         <f t="shared" si="0"/>
         <v>SI_Prod</v>
       </c>
-      <c r="I36" t="str">
+      <c r="J36" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>SI</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -1806,16 +2086,20 @@
         <v>59</v>
       </c>
       <c r="C37" s="2"/>
-      <c r="H37" t="str">
+      <c r="D37" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I37" t="str">
         <f t="shared" si="0"/>
         <v>CH_Prod</v>
       </c>
-      <c r="I37" t="str">
+      <c r="J37" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>CH</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>51</v>
       </c>
@@ -1825,16 +2109,20 @@
       <c r="C38" s="2">
         <v>1.9</v>
       </c>
-      <c r="H38" t="str">
+      <c r="D38" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>18.562999999999999</v>
+      </c>
+      <c r="I38" t="str">
         <f t="shared" si="0"/>
         <v>TN_Prod</v>
       </c>
-      <c r="I38" t="str">
+      <c r="J38" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>TN</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>47</v>
       </c>
@@ -1842,16 +2130,20 @@
         <v>10</v>
       </c>
       <c r="C39" s="2"/>
-      <c r="H39" t="str">
+      <c r="D39" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>0</v>
+      </c>
+      <c r="I39" t="str">
         <f t="shared" si="0"/>
         <v>TR_Prod</v>
       </c>
-      <c r="I39" t="str">
+      <c r="J39" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>TR</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>11</v>
       </c>
@@ -1861,16 +2153,20 @@
       <c r="C40" s="2">
         <v>39.5</v>
       </c>
-      <c r="H40" t="str">
+      <c r="D40" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>385.91499999999996</v>
+      </c>
+      <c r="I40" t="str">
         <f t="shared" si="0"/>
         <v>UK_Prod</v>
       </c>
-      <c r="I40" t="str">
+      <c r="J40" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>UK</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>39</v>
       </c>
@@ -1880,16 +2176,20 @@
       <c r="C41" s="2">
         <v>19</v>
       </c>
-      <c r="H41" t="str">
+      <c r="D41" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>185.63</v>
+      </c>
+      <c r="I41" t="str">
         <f t="shared" si="0"/>
         <v>UA_Prod</v>
       </c>
-      <c r="I41" t="str">
+      <c r="J41" t="str">
         <f>Table2[[#This Row],[Country]]</f>
         <v>UA</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>90</v>
       </c>
@@ -1899,8 +2199,12 @@
       <c r="C42" s="2">
         <v>6.3</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D42" s="2">
+        <f>Table2[[#This Row],[Mrd m3 '[2020']]]*9.77</f>
+        <v>61.550999999999995</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>85</v>
       </c>
@@ -1923,7 +2227,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE55996C-4401-4161-B17D-CF2A8462856A}">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:D51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -1931,7 +2235,7 @@
     <col min="3" max="3" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -1941,8 +2245,11 @@
       <c r="C1" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -1950,8 +2257,12 @@
         <v>74</v>
       </c>
       <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D2">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1961,8 +2272,12 @@
       <c r="C3" s="2">
         <v>8.5</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D3">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-83.045000000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -1972,8 +2287,12 @@
       <c r="C4" s="2">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D4">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-166.09</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>45</v>
       </c>
@@ -1981,8 +2300,12 @@
         <v>76</v>
       </c>
       <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D5">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>32</v>
       </c>
@@ -1990,8 +2313,12 @@
         <v>65</v>
       </c>
       <c r="C6" s="2"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D6">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1999,8 +2326,12 @@
         <v>5</v>
       </c>
       <c r="C7" s="2"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D7">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -2010,8 +2341,12 @@
       <c r="C8" s="2">
         <v>8.5</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D8">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-83.045000000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -2019,8 +2354,12 @@
         <v>61</v>
       </c>
       <c r="C9" s="2"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D9">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>54</v>
       </c>
@@ -2028,8 +2367,12 @@
         <v>67</v>
       </c>
       <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D10">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>37</v>
       </c>
@@ -2037,8 +2380,12 @@
         <v>67</v>
       </c>
       <c r="C11" s="2"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D11">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>55</v>
       </c>
@@ -2048,8 +2395,12 @@
       <c r="C12" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D12">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-19.54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -2059,8 +2410,12 @@
       <c r="C13" s="2">
         <v>40.700000000000003</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D13">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-397.63900000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -2070,8 +2425,12 @@
       <c r="C14" s="2">
         <v>86.5</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D14">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-845.10500000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -2081,8 +2440,12 @@
       <c r="C15" s="2">
         <v>5.7</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D15">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-55.689</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -2092,8 +2455,12 @@
       <c r="C16" s="2">
         <v>10.199999999999999</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D16">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-99.653999999999982</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>44</v>
       </c>
@@ -2101,8 +2468,12 @@
         <v>75</v>
       </c>
       <c r="C17" s="2"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D17">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -2112,8 +2483,12 @@
       <c r="C18" s="2">
         <v>67.7</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D18">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-661.42899999999997</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -2121,8 +2496,12 @@
         <v>66</v>
       </c>
       <c r="C19" s="2"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D19">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -2130,8 +2509,12 @@
         <v>6</v>
       </c>
       <c r="C20" s="2"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D20">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -2139,8 +2522,12 @@
         <v>71</v>
       </c>
       <c r="C21" s="2"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D21">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -2148,8 +2535,12 @@
         <v>69</v>
       </c>
       <c r="C22" s="2"/>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D22">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>18</v>
       </c>
@@ -2159,8 +2550,12 @@
       <c r="C23" s="2">
         <v>36.6</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D23">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-357.58199999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>46</v>
       </c>
@@ -2168,8 +2563,12 @@
         <v>77</v>
       </c>
       <c r="C24" s="2"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D24">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>49</v>
       </c>
@@ -2179,8 +2578,12 @@
       <c r="C25" s="2">
         <v>4.4000000000000004</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D25">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-42.988</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>90</v>
       </c>
@@ -2190,8 +2593,12 @@
       <c r="C26" s="2">
         <v>29.6</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D26">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-289.19200000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -2201,8 +2608,12 @@
       <c r="C27" s="2">
         <v>21.6</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D27">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-211.03200000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>38</v>
       </c>
@@ -2212,8 +2623,12 @@
       <c r="C28" s="2">
         <v>6</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D28">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-58.62</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -2223,8 +2638,12 @@
       <c r="C29" s="2">
         <v>11.3</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D29">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-110.401</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>48</v>
       </c>
@@ -2232,8 +2651,12 @@
         <v>78</v>
       </c>
       <c r="C30" s="2"/>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D30">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>31</v>
       </c>
@@ -2241,8 +2664,12 @@
         <v>73</v>
       </c>
       <c r="C31" s="2"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D31">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>29</v>
       </c>
@@ -2250,8 +2677,12 @@
         <v>63</v>
       </c>
       <c r="C32" s="2"/>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D32">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -2259,8 +2690,12 @@
         <v>60</v>
       </c>
       <c r="C33" s="2"/>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D33">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>89</v>
       </c>
@@ -2270,8 +2705,12 @@
       <c r="C34" s="2">
         <v>32.4</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D34">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-316.54799999999994</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>83</v>
       </c>
@@ -2281,8 +2720,12 @@
       <c r="C35" s="2">
         <v>1.1000000000000001</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D35">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-10.747</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>22</v>
       </c>
@@ -2292,8 +2735,12 @@
       <c r="C36" s="2">
         <v>3.2</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D36">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-31.263999999999999</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>47</v>
       </c>
@@ -2303,8 +2750,12 @@
       <c r="C37" s="2">
         <v>46.4</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D37">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-453.32799999999997</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>11</v>
       </c>
@@ -2314,8 +2765,12 @@
       <c r="C38" s="2">
         <v>72.5</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D38">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-708.32499999999993</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>39</v>
       </c>
@@ -2324,6 +2779,10 @@
       </c>
       <c r="C39" s="2">
         <v>29.3</v>
+      </c>
+      <c r="D39">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-286.26099999999997</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
@@ -2341,10 +2800,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD7211D-DC17-4DD6-B657-CA08F8FBC20F}">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>95</v>
       </c>
@@ -2354,8 +2813,14 @@
       <c r="C1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -2365,8 +2830,16 @@
       <c r="C2">
         <v>651.70000000000005</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D2">
+        <f>C2*365</f>
+        <v>237870.50000000003</v>
+      </c>
+      <c r="E2">
+        <f>D2/1000</f>
+        <v>237.87050000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -2376,8 +2849,16 @@
       <c r="C3">
         <v>386.9</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D3">
+        <f t="shared" ref="D3:D66" si="0">C3*365</f>
+        <v>141218.5</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E66" si="1">D3/1000</f>
+        <v>141.21850000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -2387,8 +2868,16 @@
       <c r="C4">
         <v>803.4</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>293241</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="1"/>
+        <v>293.24099999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -2398,8 +2887,16 @@
       <c r="C5">
         <v>331.2</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>120888</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>120.88800000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -2409,8 +2906,16 @@
       <c r="C6">
         <v>322.77</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>117811.04999999999</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="1"/>
+        <v>117.81104999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -2420,8 +2925,16 @@
       <c r="C7">
         <v>870</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>317550</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>317.55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -2431,8 +2944,16 @@
       <c r="C8">
         <v>1397.2</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>509978</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="1"/>
+        <v>509.97800000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -2442,8 +2963,16 @@
       <c r="C9">
         <v>1925.7729999999999</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>702907.14500000002</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>702.90714500000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -2453,8 +2982,16 @@
       <c r="C10">
         <v>396.15000000000003</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>144594.75</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="1"/>
+        <v>144.59475</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -2464,8 +3001,16 @@
       <c r="C11">
         <v>1628.3030000000001</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D11">
+        <f t="shared" si="0"/>
+        <v>594330.59500000009</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="1"/>
+        <v>594.33059500000013</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -2475,8 +3020,16 @@
       <c r="C12">
         <v>344.24799999999993</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D12">
+        <f t="shared" si="0"/>
+        <v>125650.51999999997</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="1"/>
+        <v>125.65051999999997</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -2486,8 +3039,16 @@
       <c r="C13">
         <v>328</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>119720</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="1"/>
+        <v>119.72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -2497,8 +3058,16 @@
       <c r="C14">
         <v>613.71600000000001</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D14">
+        <f t="shared" si="0"/>
+        <v>224006.34</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="1"/>
+        <v>224.00633999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -2508,8 +3077,16 @@
       <c r="C15">
         <v>136.11199999999999</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D15">
+        <f t="shared" si="0"/>
+        <v>49680.88</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="1"/>
+        <v>49.680879999999995</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -2519,8 +3096,16 @@
       <c r="C16">
         <v>233.5</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D16">
+        <f t="shared" si="0"/>
+        <v>85227.5</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="1"/>
+        <v>85.227500000000006</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -2530,8 +3115,16 @@
       <c r="C17">
         <v>1803.77</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D17">
+        <f t="shared" si="0"/>
+        <v>658376.05000000005</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="1"/>
+        <v>658.37605000000008</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -2541,8 +3134,16 @@
       <c r="C18">
         <v>26.71</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D18">
+        <f t="shared" si="0"/>
+        <v>9749.15</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="1"/>
+        <v>9.7491500000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -2552,8 +3153,16 @@
       <c r="C19">
         <v>339.96799999999996</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D19">
+        <f t="shared" si="0"/>
+        <v>124088.31999999999</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="1"/>
+        <v>124.08832</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -2563,8 +3172,16 @@
       <c r="C20">
         <v>1150</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D20">
+        <f t="shared" si="0"/>
+        <v>419750</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="1"/>
+        <v>419.75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2574,8 +3191,16 @@
       <c r="C21">
         <v>112.5</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D21">
+        <f t="shared" si="0"/>
+        <v>41062.5</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="1"/>
+        <v>41.0625</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -2585,8 +3210,16 @@
       <c r="C22">
         <v>246.5</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D22">
+        <f t="shared" si="0"/>
+        <v>89972.5</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="1"/>
+        <v>89.972499999999997</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -2596,8 +3229,16 @@
       <c r="C23">
         <v>153.1</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D23">
+        <f t="shared" si="0"/>
+        <v>55881.5</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="1"/>
+        <v>55.881500000000003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -2607,8 +3248,16 @@
       <c r="C24">
         <v>193.5</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D24">
+        <f t="shared" si="0"/>
+        <v>70627.5</v>
+      </c>
+      <c r="E24">
+        <f t="shared" si="1"/>
+        <v>70.627499999999998</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -2618,8 +3267,16 @@
       <c r="C25">
         <v>431.4</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D25">
+        <f t="shared" si="0"/>
+        <v>157461</v>
+      </c>
+      <c r="E25">
+        <f t="shared" si="1"/>
+        <v>157.46100000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -2629,8 +3286,16 @@
       <c r="C26">
         <v>28.5</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D26">
+        <f t="shared" si="0"/>
+        <v>10402.5</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="1"/>
+        <v>10.4025</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -2640,8 +3305,16 @@
       <c r="C27">
         <v>4.3</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D27">
+        <f t="shared" si="0"/>
+        <v>1569.5</v>
+      </c>
+      <c r="E27">
+        <f t="shared" si="1"/>
+        <v>1.5694999999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -2651,8 +3324,16 @@
       <c r="C28">
         <v>172.8</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D28">
+        <f t="shared" si="0"/>
+        <v>63072.000000000007</v>
+      </c>
+      <c r="E28">
+        <f t="shared" si="1"/>
+        <v>63.07200000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>22</v>
       </c>
@@ -2662,8 +3343,16 @@
       <c r="C29">
         <v>640.4</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D29">
+        <f t="shared" si="0"/>
+        <v>233746</v>
+      </c>
+      <c r="E29">
+        <f t="shared" si="1"/>
+        <v>233.74600000000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>22</v>
       </c>
@@ -2673,8 +3362,16 @@
       <c r="C30">
         <v>100</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D30">
+        <f t="shared" si="0"/>
+        <v>36500</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="1"/>
+        <v>36.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -2684,8 +3381,16 @@
       <c r="C31">
         <v>21.5</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D31">
+        <f t="shared" si="0"/>
+        <v>7847.5</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="1"/>
+        <v>7.8475000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -2695,8 +3400,16 @@
       <c r="C32">
         <v>53.7</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D32">
+        <f t="shared" si="0"/>
+        <v>19600.5</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="1"/>
+        <v>19.6005</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>24</v>
       </c>
@@ -2706,8 +3419,16 @@
       <c r="C33">
         <v>7.7</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D33">
+        <f t="shared" si="0"/>
+        <v>2810.5</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="1"/>
+        <v>2.8105000000000002</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>24</v>
       </c>
@@ -2717,8 +3438,16 @@
       <c r="C34">
         <v>48.57</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D34">
+        <f t="shared" si="0"/>
+        <v>17728.05</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="1"/>
+        <v>17.72805</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>25</v>
       </c>
@@ -2728,8 +3457,16 @@
       <c r="C35">
         <v>270</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D35">
+        <f t="shared" si="0"/>
+        <v>98550</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="1"/>
+        <v>98.55</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>25</v>
       </c>
@@ -2739,8 +3476,16 @@
       <c r="C36">
         <v>223</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D36">
+        <f t="shared" si="0"/>
+        <v>81395</v>
+      </c>
+      <c r="E36">
+        <f t="shared" si="1"/>
+        <v>81.394999999999996</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>25</v>
       </c>
@@ -2750,8 +3495,16 @@
       <c r="C37">
         <v>164.572</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D37">
+        <f t="shared" si="0"/>
+        <v>60068.78</v>
+      </c>
+      <c r="E37">
+        <f t="shared" si="1"/>
+        <v>60.068779999999997</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>26</v>
       </c>
@@ -2761,8 +3514,16 @@
       <c r="C38">
         <v>4.1189999999999998</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D38">
+        <f t="shared" si="0"/>
+        <v>1503.4349999999999</v>
+      </c>
+      <c r="E38">
+        <f t="shared" si="1"/>
+        <v>1.5034349999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>27</v>
       </c>
@@ -2772,8 +3533,16 @@
       <c r="C39">
         <v>931.6</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D39">
+        <f t="shared" si="0"/>
+        <v>340034</v>
+      </c>
+      <c r="E39">
+        <f t="shared" si="1"/>
+        <v>340.03399999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>28</v>
       </c>
@@ -2783,8 +3552,16 @@
       <c r="C40">
         <v>1231.759</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D40">
+        <f t="shared" si="0"/>
+        <v>449592.03500000003</v>
+      </c>
+      <c r="E40">
+        <f t="shared" si="1"/>
+        <v>449.59203500000001</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>28</v>
       </c>
@@ -2794,8 +3571,16 @@
       <c r="C41">
         <v>28</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D41">
+        <f t="shared" si="0"/>
+        <v>10220</v>
+      </c>
+      <c r="E41">
+        <f t="shared" si="1"/>
+        <v>10.220000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>28</v>
       </c>
@@ -2805,8 +3590,16 @@
       <c r="C42">
         <v>1246.4000000000001</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D42">
+        <f t="shared" si="0"/>
+        <v>454936.00000000006</v>
+      </c>
+      <c r="E42">
+        <f t="shared" si="1"/>
+        <v>454.93600000000004</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>29</v>
       </c>
@@ -2816,8 +3609,16 @@
       <c r="C43">
         <v>1570.4</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D43">
+        <f t="shared" si="0"/>
+        <v>573196</v>
+      </c>
+      <c r="E43">
+        <f t="shared" si="1"/>
+        <v>573.19600000000003</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>29</v>
       </c>
@@ -2827,8 +3628,16 @@
       <c r="C44">
         <v>457.6</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D44">
+        <f t="shared" si="0"/>
+        <v>167024</v>
+      </c>
+      <c r="E44">
+        <f t="shared" si="1"/>
+        <v>167.024</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>29</v>
       </c>
@@ -2838,8 +3647,16 @@
       <c r="C45">
         <v>128.9</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D45">
+        <f t="shared" si="0"/>
+        <v>47048.5</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="1"/>
+        <v>47.048499999999997</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>29</v>
       </c>
@@ -2849,8 +3666,16 @@
       <c r="C46">
         <v>416</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D46">
+        <f t="shared" si="0"/>
+        <v>151840</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="1"/>
+        <v>151.84</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>30</v>
       </c>
@@ -2860,8 +3685,16 @@
       <c r="C47">
         <v>77.400000000000006</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D47">
+        <f t="shared" si="0"/>
+        <v>28251.000000000004</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="1"/>
+        <v>28.251000000000005</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>30</v>
       </c>
@@ -2871,8 +3704,16 @@
       <c r="C48">
         <v>50.883000000000003</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D48">
+        <f t="shared" si="0"/>
+        <v>18572.295000000002</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="1"/>
+        <v>18.572295</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>30</v>
       </c>
@@ -2882,8 +3723,16 @@
       <c r="C49">
         <v>142</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D49">
+        <f t="shared" si="0"/>
+        <v>51830</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="1"/>
+        <v>51.83</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>30</v>
       </c>
@@ -2893,8 +3742,16 @@
       <c r="C50">
         <v>77.5</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D50">
+        <f t="shared" si="0"/>
+        <v>28287.5</v>
+      </c>
+      <c r="E50">
+        <f t="shared" si="1"/>
+        <v>28.287500000000001</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>31</v>
       </c>
@@ -2904,8 +3761,16 @@
       <c r="C51">
         <v>335.26</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D51">
+        <f t="shared" si="0"/>
+        <v>122369.9</v>
+      </c>
+      <c r="E51">
+        <f t="shared" si="1"/>
+        <v>122.3699</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>31</v>
       </c>
@@ -2915,8 +3780,16 @@
       <c r="C52">
         <v>17.98</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D52">
+        <f t="shared" si="0"/>
+        <v>6562.7</v>
+      </c>
+      <c r="E52">
+        <f t="shared" si="1"/>
+        <v>6.5626999999999995</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>32</v>
       </c>
@@ -2926,8 +3799,16 @@
       <c r="C53">
         <v>398.13</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D53">
+        <f t="shared" si="0"/>
+        <v>145317.45000000001</v>
+      </c>
+      <c r="E53">
+        <f t="shared" si="1"/>
+        <v>145.31745000000001</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>32</v>
       </c>
@@ -2937,8 +3818,16 @@
       <c r="C54">
         <v>117.8</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D54">
+        <f t="shared" si="0"/>
+        <v>42997</v>
+      </c>
+      <c r="E54">
+        <f t="shared" si="1"/>
+        <v>42.997</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>32</v>
       </c>
@@ -2948,8 +3837,16 @@
       <c r="C55">
         <v>148.15</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D55">
+        <f t="shared" si="0"/>
+        <v>54074.75</v>
+      </c>
+      <c r="E55">
+        <f t="shared" si="1"/>
+        <v>54.074750000000002</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>32</v>
       </c>
@@ -2959,8 +3856,16 @@
       <c r="C56">
         <v>27.38</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D56">
+        <f t="shared" si="0"/>
+        <v>9993.6999999999989</v>
+      </c>
+      <c r="E56">
+        <f t="shared" si="1"/>
+        <v>9.9936999999999987</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>32</v>
       </c>
@@ -2970,8 +3875,16 @@
       <c r="C57">
         <v>497.16</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D57">
+        <f t="shared" si="0"/>
+        <v>181463.40000000002</v>
+      </c>
+      <c r="E57">
+        <f t="shared" si="1"/>
+        <v>181.46340000000004</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>33</v>
       </c>
@@ -2981,8 +3894,16 @@
       <c r="C58">
         <v>64.819999999999993</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D58">
+        <f t="shared" si="0"/>
+        <v>23659.3</v>
+      </c>
+      <c r="E58">
+        <f t="shared" si="1"/>
+        <v>23.659299999999998</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>33</v>
       </c>
@@ -2992,8 +3913,16 @@
       <c r="C59">
         <v>53.4</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D59">
+        <f t="shared" si="0"/>
+        <v>19491</v>
+      </c>
+      <c r="E59">
+        <f t="shared" si="1"/>
+        <v>19.491</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>34</v>
       </c>
@@ -3003,8 +3932,16 @@
       <c r="C60">
         <v>50.3</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D60">
+        <f t="shared" si="0"/>
+        <v>18359.5</v>
+      </c>
+      <c r="E60">
+        <f t="shared" si="1"/>
+        <v>18.359500000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>34</v>
       </c>
@@ -3014,8 +3951,16 @@
       <c r="C61">
         <v>805.75000000000011</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D61">
+        <f t="shared" si="0"/>
+        <v>294098.75000000006</v>
+      </c>
+      <c r="E61">
+        <f t="shared" si="1"/>
+        <v>294.09875000000005</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>34</v>
       </c>
@@ -3025,8 +3970,16 @@
       <c r="C62">
         <v>122.2</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D62">
+        <f t="shared" si="0"/>
+        <v>44603</v>
+      </c>
+      <c r="E62">
+        <f t="shared" si="1"/>
+        <v>44.603000000000002</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>34</v>
       </c>
@@ -3036,8 +3989,16 @@
       <c r="C63">
         <v>16.100000000000001</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D63">
+        <f t="shared" si="0"/>
+        <v>5876.5000000000009</v>
+      </c>
+      <c r="E63">
+        <f t="shared" si="1"/>
+        <v>5.8765000000000009</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>35</v>
       </c>
@@ -3047,8 +4008,16 @@
       <c r="C64">
         <v>67.599999999999994</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D64">
+        <f t="shared" si="0"/>
+        <v>24673.999999999996</v>
+      </c>
+      <c r="E64">
+        <f t="shared" si="1"/>
+        <v>24.673999999999996</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>35</v>
       </c>
@@ -3058,8 +4027,16 @@
       <c r="C65">
         <v>114.2</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D65">
+        <f t="shared" si="0"/>
+        <v>41683</v>
+      </c>
+      <c r="E65">
+        <f t="shared" si="1"/>
+        <v>41.683</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>36</v>
       </c>
@@ -3069,8 +4046,16 @@
       <c r="C66">
         <v>65.099999999999994</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D66">
+        <f t="shared" si="0"/>
+        <v>23761.499999999996</v>
+      </c>
+      <c r="E66">
+        <f t="shared" si="1"/>
+        <v>23.761499999999998</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>36</v>
       </c>
@@ -3080,8 +4065,16 @@
       <c r="C67">
         <v>85</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D67">
+        <f t="shared" ref="D67:D90" si="2">C67*365</f>
+        <v>31025</v>
+      </c>
+      <c r="E67">
+        <f t="shared" ref="E67:E90" si="3">D67/1000</f>
+        <v>31.024999999999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>37</v>
       </c>
@@ -3091,8 +4084,16 @@
       <c r="C68">
         <v>224.4</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D68">
+        <f t="shared" si="2"/>
+        <v>81906</v>
+      </c>
+      <c r="E68">
+        <f t="shared" si="3"/>
+        <v>81.906000000000006</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>37</v>
       </c>
@@ -3102,8 +4103,16 @@
       <c r="C69">
         <v>144</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D69">
+        <f t="shared" si="2"/>
+        <v>52560</v>
+      </c>
+      <c r="E69">
+        <f t="shared" si="3"/>
+        <v>52.56</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>38</v>
       </c>
@@ -3113,8 +4122,16 @@
       <c r="C70">
         <v>80</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D70">
+        <f t="shared" si="2"/>
+        <v>29200</v>
+      </c>
+      <c r="E70">
+        <f t="shared" si="3"/>
+        <v>29.2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>39</v>
       </c>
@@ -3124,8 +4141,16 @@
       <c r="C71">
         <v>135.6</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D71">
+        <f t="shared" si="2"/>
+        <v>49494</v>
+      </c>
+      <c r="E71">
+        <f t="shared" si="3"/>
+        <v>49.494</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>39</v>
       </c>
@@ -3135,8 +4160,16 @@
       <c r="C72">
         <v>2277.6</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D72">
+        <f t="shared" si="2"/>
+        <v>831324</v>
+      </c>
+      <c r="E72">
+        <f t="shared" si="3"/>
+        <v>831.32399999999996</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>39</v>
       </c>
@@ -3146,8 +4179,16 @@
       <c r="C73">
         <v>515.6</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D73">
+        <f t="shared" si="2"/>
+        <v>188194</v>
+      </c>
+      <c r="E73">
+        <f t="shared" si="3"/>
+        <v>188.19399999999999</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>39</v>
       </c>
@@ -3157,8 +4198,16 @@
       <c r="C74">
         <v>1163.4000000000001</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D74">
+        <f t="shared" si="2"/>
+        <v>424641.00000000006</v>
+      </c>
+      <c r="E74">
+        <f t="shared" si="3"/>
+        <v>424.64100000000008</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>40</v>
       </c>
@@ -3168,8 +4217,16 @@
       <c r="C75">
         <v>2.2000000000000002</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D75">
+        <f t="shared" si="2"/>
+        <v>803.00000000000011</v>
+      </c>
+      <c r="E75">
+        <f t="shared" si="3"/>
+        <v>0.80300000000000016</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>41</v>
       </c>
@@ -3179,8 +4236,16 @@
       <c r="C76">
         <v>1742</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D76">
+        <f t="shared" si="2"/>
+        <v>635830</v>
+      </c>
+      <c r="E76">
+        <f t="shared" si="3"/>
+        <v>635.83000000000004</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>41</v>
       </c>
@@ -3190,8 +4255,16 @@
       <c r="C77">
         <v>168</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D77">
+        <f t="shared" si="2"/>
+        <v>61320</v>
+      </c>
+      <c r="E77">
+        <f t="shared" si="3"/>
+        <v>61.32</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>41</v>
       </c>
@@ -3201,8 +4274,16 @@
       <c r="C78">
         <v>220</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D78">
+        <f t="shared" si="2"/>
+        <v>80300</v>
+      </c>
+      <c r="E78">
+        <f t="shared" si="3"/>
+        <v>80.3</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>42</v>
       </c>
@@ -3212,8 +4293,16 @@
       <c r="C79">
         <v>487.1</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D79">
+        <f t="shared" si="2"/>
+        <v>177791.5</v>
+      </c>
+      <c r="E79">
+        <f t="shared" si="3"/>
+        <v>177.79150000000001</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>47</v>
       </c>
@@ -3223,8 +4312,16 @@
       <c r="C80">
         <v>576.03</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D80">
+        <f t="shared" si="2"/>
+        <v>210250.94999999998</v>
+      </c>
+      <c r="E80">
+        <f t="shared" si="3"/>
+        <v>210.25094999999999</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>47</v>
       </c>
@@ -3234,8 +4331,16 @@
       <c r="C81">
         <v>398.6</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D81">
+        <f t="shared" si="2"/>
+        <v>145489</v>
+      </c>
+      <c r="E81">
+        <f t="shared" si="3"/>
+        <v>145.489</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>49</v>
       </c>
@@ -3245,8 +4350,16 @@
       <c r="C82">
         <v>1499.1</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D82">
+        <f t="shared" si="2"/>
+        <v>547171.5</v>
+      </c>
+      <c r="E82">
+        <f t="shared" si="3"/>
+        <v>547.17150000000004</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>49</v>
       </c>
@@ -3256,8 +4369,16 @@
       <c r="C83">
         <v>488</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D83">
+        <f t="shared" si="2"/>
+        <v>178120</v>
+      </c>
+      <c r="E83">
+        <f t="shared" si="3"/>
+        <v>178.12</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>49</v>
       </c>
@@ -3267,8 +4388,16 @@
       <c r="C84">
         <v>2210.5639999999999</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D84">
+        <f t="shared" si="2"/>
+        <v>806855.86</v>
+      </c>
+      <c r="E84">
+        <f t="shared" si="3"/>
+        <v>806.85586000000001</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>49</v>
       </c>
@@ -3278,8 +4407,16 @@
       <c r="C85">
         <v>570</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D85">
+        <f t="shared" si="2"/>
+        <v>208050</v>
+      </c>
+      <c r="E85">
+        <f t="shared" si="3"/>
+        <v>208.05</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>50</v>
       </c>
@@ -3289,8 +4426,16 @@
       <c r="C86">
         <v>731.7</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D86">
+        <f t="shared" si="2"/>
+        <v>267070.5</v>
+      </c>
+      <c r="E86">
+        <f t="shared" si="3"/>
+        <v>267.07049999999998</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>51</v>
       </c>
@@ -3300,8 +4445,16 @@
       <c r="C87">
         <v>1138.0999999999999</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D87">
+        <f t="shared" si="2"/>
+        <v>415406.49999999994</v>
+      </c>
+      <c r="E87">
+        <f t="shared" si="3"/>
+        <v>415.40649999999994</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>52</v>
       </c>
@@ -3311,8 +4464,16 @@
       <c r="C88">
         <v>475.8</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D88">
+        <f t="shared" si="2"/>
+        <v>173667</v>
+      </c>
+      <c r="E88">
+        <f t="shared" si="3"/>
+        <v>173.667</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>53</v>
       </c>
@@ -3322,8 +4483,16 @@
       <c r="C89">
         <v>1203.4999999999998</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D89">
+        <f t="shared" si="2"/>
+        <v>439277.49999999994</v>
+      </c>
+      <c r="E89">
+        <f t="shared" si="3"/>
+        <v>439.27749999999992</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>53</v>
       </c>
@@ -3332,6 +4501,14 @@
       </c>
       <c r="C90">
         <v>325.39999999999998</v>
+      </c>
+      <c r="D90">
+        <f t="shared" si="2"/>
+        <v>118770.99999999999</v>
+      </c>
+      <c r="E90">
+        <f t="shared" si="3"/>
+        <v>118.77099999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3344,7 +4521,7 @@
   <dimension ref="A1:E30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>95</v>
       </c>
@@ -3354,8 +4531,14 @@
       <c r="C1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -3365,8 +4548,16 @@
       <c r="C2">
         <v>1334</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D2">
+        <f>C2*365</f>
+        <v>486910</v>
+      </c>
+      <c r="E2">
+        <f>D2/1000</f>
+        <v>486.91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>99</v>
       </c>
@@ -3376,8 +4567,16 @@
       <c r="C3">
         <v>395</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D3">
+        <f t="shared" ref="D3:D24" si="0">C3*365</f>
+        <v>144175</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E24" si="1">D3/1000</f>
+        <v>144.17500000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -3387,8 +4586,16 @@
       <c r="C4">
         <v>135.6</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>49494</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="1"/>
+        <v>49.494</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -3399,8 +4606,16 @@
         <f>1799+436.8</f>
         <v>2235.8000000000002</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>816067.00000000012</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>816.06700000000012</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>39</v>
       </c>
@@ -3410,8 +4625,16 @@
       <c r="C6">
         <v>517.5</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>188887.5</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="1"/>
+        <v>188.88749999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -3421,8 +4644,16 @@
       <c r="C7">
         <v>245.8</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>89717</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>89.716999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -3432,8 +4663,16 @@
       <c r="C8">
         <v>467.5</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>170637.5</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="1"/>
+        <v>170.63749999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>32</v>
       </c>
@@ -3443,8 +4682,16 @@
       <c r="C9">
         <v>33.380000000000003</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>12183.7</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>12.1837</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -3454,8 +4701,16 @@
       <c r="C10">
         <v>701.8</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>256156.99999999997</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="1"/>
+        <v>256.15699999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -3465,8 +4720,16 @@
       <c r="C11">
         <v>168</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D11">
+        <f t="shared" si="0"/>
+        <v>61320</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="1"/>
+        <v>61.32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>41</v>
       </c>
@@ -3476,8 +4739,16 @@
       <c r="C12">
         <v>220</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D12">
+        <f t="shared" si="0"/>
+        <v>80300</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="1"/>
+        <v>80.3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>52</v>
       </c>
@@ -3487,8 +4758,16 @@
       <c r="C13">
         <v>493.7</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>180200.5</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="1"/>
+        <v>180.20050000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>51</v>
       </c>
@@ -3498,8 +4777,16 @@
       <c r="C14">
         <v>1154</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D14">
+        <f t="shared" si="0"/>
+        <v>421210</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="1"/>
+        <v>421.21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>42</v>
       </c>
@@ -3509,8 +4796,16 @@
       <c r="C15">
         <v>337.1</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D15">
+        <f t="shared" si="0"/>
+        <v>123041.50000000001</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="1"/>
+        <v>123.04150000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>101</v>
       </c>
@@ -3519,6 +4814,14 @@
       </c>
       <c r="C16">
         <v>442.8</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="0"/>
+        <v>161622</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="1"/>
+        <v>161.62200000000001</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -3531,6 +4834,14 @@
       <c r="C17">
         <v>1247</v>
       </c>
+      <c r="D17">
+        <f t="shared" si="0"/>
+        <v>455155</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="1"/>
+        <v>455.15499999999997</v>
+      </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
@@ -3542,6 +4853,14 @@
       <c r="C18">
         <v>963.6</v>
       </c>
+      <c r="D18">
+        <f t="shared" si="0"/>
+        <v>351714</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="1"/>
+        <v>351.714</v>
+      </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
@@ -3553,6 +4872,14 @@
       <c r="C19">
         <v>459.6</v>
       </c>
+      <c r="D19">
+        <f t="shared" si="0"/>
+        <v>167754</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="1"/>
+        <v>167.75399999999999</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
@@ -3564,6 +4891,14 @@
       <c r="C20">
         <v>568.5</v>
       </c>
+      <c r="D20">
+        <f t="shared" si="0"/>
+        <v>207502.5</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="1"/>
+        <v>207.5025</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
@@ -3575,6 +4910,14 @@
       <c r="C21">
         <v>1406</v>
       </c>
+      <c r="D21">
+        <f t="shared" si="0"/>
+        <v>513190</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="1"/>
+        <v>513.19000000000005</v>
+      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
@@ -3586,6 +4929,14 @@
       <c r="C22">
         <v>385</v>
       </c>
+      <c r="D22">
+        <f t="shared" si="0"/>
+        <v>140525</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="1"/>
+        <v>140.52500000000001</v>
+      </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
@@ -3597,6 +4948,14 @@
       <c r="C23">
         <v>227.2</v>
       </c>
+      <c r="D23">
+        <f t="shared" si="0"/>
+        <v>82928</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="1"/>
+        <v>82.927999999999997</v>
+      </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
@@ -3607,6 +4966,14 @@
       </c>
       <c r="C24">
         <v>184.8</v>
+      </c>
+      <c r="D24">
+        <f t="shared" si="0"/>
+        <v>67452</v>
+      </c>
+      <c r="E24">
+        <f t="shared" si="1"/>
+        <v>67.451999999999998</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
start fix Estonian capacity bug
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6CD0683-BCB8-4740-AFB6-18E523E2C013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9DAFECF-8536-43C8-8E46-D869DDE91305}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="136">
   <si>
     <t>Belgium</t>
   </si>
@@ -582,14 +582,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}" name="Table3" displayName="Table3" ref="A1:E90" totalsRowShown="0">
-  <autoFilter ref="A1:E90" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="UA"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}" name="Table3" displayName="Table3" ref="A1:E92" totalsRowShown="0">
+  <autoFilter ref="A1:E92" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E90">
     <sortCondition ref="B1:B90"/>
   </sortState>
@@ -3771,7 +3765,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD7211D-DC17-4DD6-B657-CA08F8FBC20F}">
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="8.90625" customWidth="1"/>
@@ -3795,7 +3789,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -3814,7 +3808,7 @@
         <v>125.65051999999997</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -3833,7 +3827,7 @@
         <v>70.627499999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -3852,7 +3846,7 @@
         <v>573.19600000000003</v>
       </c>
     </row>
-    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -3871,7 +3865,7 @@
         <v>6.5626999999999995</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -3890,7 +3884,7 @@
         <v>237.87050000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -3909,7 +3903,7 @@
         <v>509.97800000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -3928,7 +3922,7 @@
         <v>144.59475</v>
       </c>
     </row>
-    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -3947,7 +3941,7 @@
         <v>98.55</v>
       </c>
     </row>
-    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>49</v>
       </c>
@@ -3966,7 +3960,7 @@
         <v>178.12</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>31</v>
       </c>
@@ -3985,7 +3979,7 @@
         <v>122.3699</v>
       </c>
     </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -4004,7 +3998,7 @@
         <v>23.659299999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -4023,7 +4017,7 @@
         <v>294.09875000000005</v>
       </c>
     </row>
-    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>47</v>
       </c>
@@ -4042,7 +4036,7 @@
         <v>210.25094999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -4061,7 +4055,7 @@
         <v>119.72</v>
       </c>
     </row>
-    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -4080,7 +4074,7 @@
         <v>157.46100000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -4099,7 +4093,7 @@
         <v>81.394999999999996</v>
       </c>
     </row>
-    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -4118,7 +4112,7 @@
         <v>658.37605000000008</v>
       </c>
     </row>
-    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -4137,7 +4131,7 @@
         <v>167.024</v>
       </c>
     </row>
-    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -4156,7 +4150,7 @@
         <v>117.81104999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -4175,7 +4169,7 @@
         <v>702.90714500000001</v>
       </c>
     </row>
-    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -4194,7 +4188,7 @@
         <v>124.08832</v>
       </c>
     </row>
-    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -4213,7 +4207,7 @@
         <v>63.07200000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>26</v>
       </c>
@@ -4232,7 +4226,7 @@
         <v>1.5034349999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -4251,7 +4245,7 @@
         <v>340.03399999999999</v>
       </c>
     </row>
-    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>28</v>
       </c>
@@ -4270,7 +4264,7 @@
         <v>449.59203500000001</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>41</v>
       </c>
@@ -4289,7 +4283,7 @@
         <v>635.83000000000004</v>
       </c>
     </row>
-    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>49</v>
       </c>
@@ -4308,7 +4302,7 @@
         <v>806.85586000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>19</v>
       </c>
@@ -4327,7 +4321,7 @@
         <v>49.680879999999995</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>25</v>
       </c>
@@ -4346,7 +4340,7 @@
         <v>60.068779999999997</v>
       </c>
     </row>
-    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>38</v>
       </c>
@@ -4365,7 +4359,7 @@
         <v>29.2</v>
       </c>
     </row>
-    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>50</v>
       </c>
@@ -4384,7 +4378,7 @@
         <v>267.07049999999998</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>41</v>
       </c>
@@ -4403,7 +4397,7 @@
         <v>80.3</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>17</v>
       </c>
@@ -4422,7 +4416,7 @@
         <v>317.55</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>19</v>
       </c>
@@ -4441,7 +4435,7 @@
         <v>224.00633999999999</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>22</v>
       </c>
@@ -4460,7 +4454,7 @@
         <v>36.5</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>37</v>
       </c>
@@ -4479,7 +4473,7 @@
         <v>81.906000000000006</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>49</v>
       </c>
@@ -4498,7 +4492,7 @@
         <v>208.05</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>32</v>
       </c>
@@ -4517,7 +4511,7 @@
         <v>42.997</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>33</v>
       </c>
@@ -4536,7 +4530,7 @@
         <v>19.491</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>47</v>
       </c>
@@ -4555,7 +4549,7 @@
         <v>145.489</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>23</v>
       </c>
@@ -4574,7 +4568,7 @@
         <v>19.6005</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>30</v>
       </c>
@@ -4593,7 +4587,7 @@
         <v>28.251000000000005</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>20</v>
       </c>
@@ -4612,7 +4606,7 @@
         <v>55.881500000000003</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>24</v>
       </c>
@@ -4631,7 +4625,7 @@
         <v>17.72805</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>29</v>
       </c>
@@ -4650,7 +4644,7 @@
         <v>47.048499999999997</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>34</v>
       </c>
@@ -4688,7 +4682,7 @@
         <v>188.19399999999999</v>
       </c>
     </row>
-    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>11</v>
       </c>
@@ -4707,7 +4701,7 @@
         <v>141.21850000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>20</v>
       </c>
@@ -4726,7 +4720,7 @@
         <v>419.75</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>22</v>
       </c>
@@ -4745,7 +4739,7 @@
         <v>233.74600000000001</v>
       </c>
     </row>
-    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>23</v>
       </c>
@@ -4764,7 +4758,7 @@
         <v>7.8475000000000001</v>
       </c>
     </row>
-    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>42</v>
       </c>
@@ -4783,7 +4777,7 @@
         <v>177.79150000000001</v>
       </c>
     </row>
-    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>51</v>
       </c>
@@ -4802,7 +4796,7 @@
         <v>415.40649999999994</v>
       </c>
     </row>
-    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>52</v>
       </c>
@@ -4821,7 +4815,7 @@
         <v>173.667</v>
       </c>
     </row>
-    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>36</v>
       </c>
@@ -4840,7 +4834,7 @@
         <v>23.761499999999998</v>
       </c>
     </row>
-    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>53</v>
       </c>
@@ -4859,7 +4853,7 @@
         <v>118.77099999999999</v>
       </c>
     </row>
-    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>19</v>
       </c>
@@ -4878,7 +4872,7 @@
         <v>9.7491500000000002</v>
       </c>
     </row>
-    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>35</v>
       </c>
@@ -4897,7 +4891,7 @@
         <v>24.673999999999996</v>
       </c>
     </row>
-    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>41</v>
       </c>
@@ -4916,7 +4910,7 @@
         <v>61.32</v>
       </c>
     </row>
-    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>34</v>
       </c>
@@ -4935,7 +4929,7 @@
         <v>20.330500000000001</v>
       </c>
     </row>
-    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>32</v>
       </c>
@@ -4954,7 +4948,7 @@
         <v>9.9936999999999987</v>
       </c>
     </row>
-    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>17</v>
       </c>
@@ -4973,7 +4967,7 @@
         <v>120.88800000000001</v>
       </c>
     </row>
-    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>19</v>
       </c>
@@ -4992,7 +4986,7 @@
         <v>594.33059500000013</v>
       </c>
     </row>
-    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>19</v>
       </c>
@@ -5011,7 +5005,7 @@
         <v>85.227500000000006</v>
       </c>
     </row>
-    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>28</v>
       </c>
@@ -5049,7 +5043,7 @@
         <v>49.494</v>
       </c>
     </row>
-    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>53</v>
       </c>
@@ -5068,7 +5062,7 @@
         <v>439.27749999999992</v>
       </c>
     </row>
-    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>37</v>
       </c>
@@ -5087,7 +5081,7 @@
         <v>52.56</v>
       </c>
     </row>
-    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>30</v>
       </c>
@@ -5106,7 +5100,7 @@
         <v>28.287500000000001</v>
       </c>
     </row>
-    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>32</v>
       </c>
@@ -5144,7 +5138,7 @@
         <v>424.64100000000008</v>
       </c>
     </row>
-    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>40</v>
       </c>
@@ -5163,7 +5157,7 @@
         <v>0.80300000000000016</v>
       </c>
     </row>
-    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>30</v>
       </c>
@@ -5182,7 +5176,7 @@
         <v>51.83</v>
       </c>
     </row>
-    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>32</v>
       </c>
@@ -5201,7 +5195,7 @@
         <v>145.31745000000001</v>
       </c>
     </row>
-    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>35</v>
       </c>
@@ -5220,7 +5214,7 @@
         <v>41.683</v>
       </c>
     </row>
-    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>36</v>
       </c>
@@ -5239,7 +5233,7 @@
         <v>31.024999999999999</v>
       </c>
     </row>
-    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>20</v>
       </c>
@@ -5258,7 +5252,7 @@
         <v>41.0625</v>
       </c>
     </row>
-    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>21</v>
       </c>
@@ -5277,7 +5271,7 @@
         <v>10.4025</v>
       </c>
     </row>
-    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>24</v>
       </c>
@@ -5296,7 +5290,7 @@
         <v>2.8105000000000002</v>
       </c>
     </row>
-    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>20</v>
       </c>
@@ -5315,7 +5309,7 @@
         <v>89.972499999999997</v>
       </c>
     </row>
-    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>28</v>
       </c>
@@ -5334,7 +5328,7 @@
         <v>454.93600000000004</v>
       </c>
     </row>
-    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>30</v>
       </c>
@@ -5372,7 +5366,7 @@
         <v>831.32399999999996</v>
       </c>
     </row>
-    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>21</v>
       </c>
@@ -5391,7 +5385,7 @@
         <v>1.5694999999999999</v>
       </c>
     </row>
-    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>32</v>
       </c>
@@ -5410,7 +5404,7 @@
         <v>181.46340000000004</v>
       </c>
     </row>
-    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>29</v>
       </c>
@@ -5429,7 +5423,7 @@
         <v>151.84</v>
       </c>
     </row>
-    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>34</v>
       </c>
@@ -5448,7 +5442,7 @@
         <v>44.603000000000002</v>
       </c>
     </row>
-    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>17</v>
       </c>
@@ -5467,7 +5461,7 @@
         <v>293.24099999999999</v>
       </c>
     </row>
-    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>49</v>
       </c>
@@ -5484,6 +5478,37 @@
       <c r="E90">
         <f t="shared" si="5"/>
         <v>547.17150000000004</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A91" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C91" s="4"/>
+      <c r="D91" s="4">
+        <f>C91*365</f>
+        <v>0</v>
+      </c>
+      <c r="E91" s="4">
+        <v>24.424999999999997</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>36</v>
+      </c>
+      <c r="B92" t="s">
+        <v>54</v>
+      </c>
+      <c r="D92">
+        <f>C92*365</f>
+        <v>0</v>
+      </c>
+      <c r="E92" s="4">
+        <v>24.424999999999997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bug fix in demand calculation for other Europe
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0B00252-E19F-4602-A4C1-AEEF3F20F204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{441A09C5-75FF-4221-BA74-C8AF2F57A9CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="137">
   <si>
     <t>Belgium</t>
   </si>
@@ -459,9 +459,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="173" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -599,23 +599,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -628,7 +617,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="44">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyFill="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -643,9 +632,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyFill="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyFill="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
@@ -658,7 +644,7 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="173" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0">
       <alignment horizontal="right"/>
@@ -667,7 +653,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyNumberFormat="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyNumberFormat="0" applyAlignment="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
@@ -679,13 +665,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyFill="0" applyBorder="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="173" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyFill="0" applyBorder="0"/>
-    <xf numFmtId="179" fontId="5" fillId="0" borderId="0">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="179" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -701,51 +687,50 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="44">
-    <cellStyle name="02_Rule above and below" xfId="7" xr:uid="{986163A9-ABD7-4B23-BF51-4DC5B73EBE7F}"/>
+  <cellStyles count="43">
     <cellStyle name="03_Table Notes" xfId="5" xr:uid="{957BCF11-BB00-461F-A0F4-0368139C34F0}"/>
     <cellStyle name="04_Table text" xfId="3" xr:uid="{60FAF7FD-D988-4AB0-B86F-CAD4D7C5E89B}"/>
-    <cellStyle name="C01_Main head" xfId="25" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
-    <cellStyle name="C02_Column heads" xfId="19" xr:uid="{6AA76714-52DD-4B3B-9F1F-E7ED06188786}"/>
-    <cellStyle name="C03_Sub head bold" xfId="20" xr:uid="{71BDF15F-8FAB-4B9D-BF56-0C82A383AA8E}"/>
-    <cellStyle name="C04_Total text white bold" xfId="23" xr:uid="{287E28E8-DA9A-4DA7-94AD-5AF1C537F15F}"/>
-    <cellStyle name="C04a_Total text black with rule" xfId="22" xr:uid="{16CE27B2-E630-4389-8700-BC6F07A207BB}"/>
-    <cellStyle name="C05_Main text" xfId="21" xr:uid="{19A3C003-4A4D-4B53-B889-86660BE2F4A7}"/>
-    <cellStyle name="C06_Figs" xfId="27" xr:uid="{6EF7291D-EE46-4629-B94D-1ECDF30BDA6F}"/>
-    <cellStyle name="C07_Figs 1 dec percent" xfId="35" xr:uid="{47221C8E-FC37-465A-9665-18759B74A6CE}"/>
-    <cellStyle name="C09_Notes" xfId="10" xr:uid="{9085F154-117F-416B-8D81-36A9DB81FB8C}"/>
-    <cellStyle name="Comma 2" xfId="17" xr:uid="{C220F88A-4F55-4623-B6C1-AD23C8E74659}"/>
-    <cellStyle name="Comma 5" xfId="32" xr:uid="{0067ED6D-11E5-44AC-9D53-C45880789330}"/>
+    <cellStyle name="C01_Main head" xfId="24" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
+    <cellStyle name="C02_Column heads" xfId="18" xr:uid="{6AA76714-52DD-4B3B-9F1F-E7ED06188786}"/>
+    <cellStyle name="C03_Sub head bold" xfId="19" xr:uid="{71BDF15F-8FAB-4B9D-BF56-0C82A383AA8E}"/>
+    <cellStyle name="C04_Total text white bold" xfId="22" xr:uid="{287E28E8-DA9A-4DA7-94AD-5AF1C537F15F}"/>
+    <cellStyle name="C04a_Total text black with rule" xfId="21" xr:uid="{16CE27B2-E630-4389-8700-BC6F07A207BB}"/>
+    <cellStyle name="C05_Main text" xfId="20" xr:uid="{19A3C003-4A4D-4B53-B889-86660BE2F4A7}"/>
+    <cellStyle name="C06_Figs" xfId="26" xr:uid="{6EF7291D-EE46-4629-B94D-1ECDF30BDA6F}"/>
+    <cellStyle name="C07_Figs 1 dec percent" xfId="34" xr:uid="{47221C8E-FC37-465A-9665-18759B74A6CE}"/>
+    <cellStyle name="C09_Notes" xfId="9" xr:uid="{9085F154-117F-416B-8D81-36A9DB81FB8C}"/>
+    <cellStyle name="Comma 2" xfId="16" xr:uid="{C220F88A-4F55-4623-B6C1-AD23C8E74659}"/>
+    <cellStyle name="Comma 5" xfId="31" xr:uid="{0067ED6D-11E5-44AC-9D53-C45880789330}"/>
     <cellStyle name="Hyperlink 2" xfId="2" xr:uid="{BA9329EA-B184-49A9-9DC3-748FF9EBB7D9}"/>
     <cellStyle name="Hyperlink 2 2" xfId="4" xr:uid="{F9103865-4F21-4889-8B72-20BE8654C338}"/>
-    <cellStyle name="Hyperlink 2 2 2" xfId="15" xr:uid="{5BCD4CE7-6B2C-456F-8FB9-324AD7E49CAD}"/>
-    <cellStyle name="Hyperlink 3" xfId="16" xr:uid="{94940656-2676-4A09-B05D-BC18288B254C}"/>
+    <cellStyle name="Hyperlink 2 2 2" xfId="14" xr:uid="{5BCD4CE7-6B2C-456F-8FB9-324AD7E49CAD}"/>
+    <cellStyle name="Hyperlink 3" xfId="15" xr:uid="{94940656-2676-4A09-B05D-BC18288B254C}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 18" xfId="33" xr:uid="{E7EAE102-3B70-42A2-97BE-6613C6991711}"/>
+    <cellStyle name="Normal 18" xfId="32" xr:uid="{E7EAE102-3B70-42A2-97BE-6613C6991711}"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{190F2216-BF41-4842-8670-90BCBED25C1F}"/>
-    <cellStyle name="Normal 2 2" xfId="11" xr:uid="{BBA1F6BA-F8D2-45BD-89F2-5F79E7C1C329}"/>
-    <cellStyle name="Normal 2 2 2" xfId="29" xr:uid="{AD51099B-D49D-45FE-80D3-1F4120CAB713}"/>
-    <cellStyle name="Normal 2 2 3" xfId="34" xr:uid="{685F2931-69F1-4742-862E-8D36BACD9F1A}"/>
-    <cellStyle name="Normal 2 2 9 2" xfId="40" xr:uid="{1D997E3D-2769-4905-B0EB-950CAA58DB0A}"/>
-    <cellStyle name="Normal 2 3" xfId="43" xr:uid="{1A02E014-9D0A-45BD-84AD-CEF3659D5A24}"/>
-    <cellStyle name="Normal 2 5" xfId="30" xr:uid="{BA56A082-19D7-4317-9FF5-DEC1FFBEF23C}"/>
-    <cellStyle name="Normal 2 6" xfId="12" xr:uid="{A9C605D1-161F-4025-811E-28DABC062934}"/>
-    <cellStyle name="Normal 20" xfId="24" xr:uid="{648D11FF-279B-4F0E-B09D-8C1EC6061892}"/>
-    <cellStyle name="Normal 3" xfId="13" xr:uid="{C48EB3F3-1975-4918-BAB7-BE900719A5F7}"/>
-    <cellStyle name="Normal 33" xfId="8" xr:uid="{5CD1E707-8667-45EC-ABF6-B60F6E9E59D3}"/>
-    <cellStyle name="Normal 4" xfId="42" xr:uid="{6FD259F4-48D1-4A86-985F-41950DBD9149}"/>
+    <cellStyle name="Normal 2 2" xfId="10" xr:uid="{BBA1F6BA-F8D2-45BD-89F2-5F79E7C1C329}"/>
+    <cellStyle name="Normal 2 2 2" xfId="28" xr:uid="{AD51099B-D49D-45FE-80D3-1F4120CAB713}"/>
+    <cellStyle name="Normal 2 2 3" xfId="33" xr:uid="{685F2931-69F1-4742-862E-8D36BACD9F1A}"/>
+    <cellStyle name="Normal 2 2 9 2" xfId="39" xr:uid="{1D997E3D-2769-4905-B0EB-950CAA58DB0A}"/>
+    <cellStyle name="Normal 2 3" xfId="42" xr:uid="{1A02E014-9D0A-45BD-84AD-CEF3659D5A24}"/>
+    <cellStyle name="Normal 2 5" xfId="29" xr:uid="{BA56A082-19D7-4317-9FF5-DEC1FFBEF23C}"/>
+    <cellStyle name="Normal 2 6" xfId="11" xr:uid="{A9C605D1-161F-4025-811E-28DABC062934}"/>
+    <cellStyle name="Normal 20" xfId="23" xr:uid="{648D11FF-279B-4F0E-B09D-8C1EC6061892}"/>
+    <cellStyle name="Normal 3" xfId="12" xr:uid="{C48EB3F3-1975-4918-BAB7-BE900719A5F7}"/>
+    <cellStyle name="Normal 33" xfId="7" xr:uid="{5CD1E707-8667-45EC-ABF6-B60F6E9E59D3}"/>
+    <cellStyle name="Normal 4" xfId="41" xr:uid="{6FD259F4-48D1-4A86-985F-41950DBD9149}"/>
     <cellStyle name="Normal 4 2 2" xfId="6" xr:uid="{919221B1-42A4-4700-9239-2DAFE893779F}"/>
-    <cellStyle name="Normal 5" xfId="39" xr:uid="{7566378D-1084-4857-A4BB-1DAAB3764B14}"/>
-    <cellStyle name="Normal 5 8 2" xfId="41" xr:uid="{AEB2F650-B345-44F9-857E-1FF7EFC5D55E}"/>
-    <cellStyle name="Normal 6" xfId="14" xr:uid="{D03254E9-8E42-4BF4-8A58-7DE6DA4A8303}"/>
-    <cellStyle name="Normal 8" xfId="9" xr:uid="{90F0E83A-EA1A-48E1-A5EE-D67EB082C60D}"/>
-    <cellStyle name="Normal 8 2" xfId="26" xr:uid="{A358C3D2-DBD8-459F-9B06-BAA976C32485}"/>
-    <cellStyle name="Normal 8 7" xfId="28" xr:uid="{76B13E51-C838-4F8D-AADA-E10D7E632F63}"/>
-    <cellStyle name="Percent 2" xfId="18" xr:uid="{8FA158A0-20DC-4018-9CF3-EDDF9FADF72C}"/>
-    <cellStyle name="Percent 2 2" xfId="31" xr:uid="{0AA4CE3F-8960-4102-9CAE-7448A8126969}"/>
-    <cellStyle name="Percent 3" xfId="37" xr:uid="{8AB380C1-64CC-421C-8275-BF15C8D4F870}"/>
-    <cellStyle name="Percent 4" xfId="38" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
-    <cellStyle name="Percent 8" xfId="36" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
+    <cellStyle name="Normal 5" xfId="38" xr:uid="{7566378D-1084-4857-A4BB-1DAAB3764B14}"/>
+    <cellStyle name="Normal 5 8 2" xfId="40" xr:uid="{AEB2F650-B345-44F9-857E-1FF7EFC5D55E}"/>
+    <cellStyle name="Normal 6" xfId="13" xr:uid="{D03254E9-8E42-4BF4-8A58-7DE6DA4A8303}"/>
+    <cellStyle name="Normal 8" xfId="8" xr:uid="{90F0E83A-EA1A-48E1-A5EE-D67EB082C60D}"/>
+    <cellStyle name="Normal 8 2" xfId="25" xr:uid="{A358C3D2-DBD8-459F-9B06-BAA976C32485}"/>
+    <cellStyle name="Normal 8 7" xfId="27" xr:uid="{76B13E51-C838-4F8D-AADA-E10D7E632F63}"/>
+    <cellStyle name="Percent 2" xfId="17" xr:uid="{8FA158A0-20DC-4018-9CF3-EDDF9FADF72C}"/>
+    <cellStyle name="Percent 2 2" xfId="30" xr:uid="{0AA4CE3F-8960-4102-9CAE-7448A8126969}"/>
+    <cellStyle name="Percent 3" xfId="36" xr:uid="{8AB380C1-64CC-421C-8275-BF15C8D4F870}"/>
+    <cellStyle name="Percent 4" xfId="37" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
+    <cellStyle name="Percent 8" xfId="35" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
   <dxfs count="10">
     <dxf>
@@ -828,7 +813,7 @@
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
     <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="3">
-      <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E2/$E$27,0)</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -850,7 +835,7 @@
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
     <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="0">
-      <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E2/$E$27,0)</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3168,8 +3153,8 @@
         <v>2846</v>
       </c>
       <c r="F2">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E2/$E$27,0)</f>
-        <v>-2.6268792942111183</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</f>
+        <v>-7.7179334425266708</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -3190,7 +3175,7 @@
         <v>8901.1</v>
       </c>
       <c r="F3">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E3/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E3/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3212,7 +3197,7 @@
         <v>11549.9</v>
       </c>
       <c r="F4">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E4/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E4/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3232,8 +3217,8 @@
         <v>3492</v>
       </c>
       <c r="F5">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E5/$E$27,0)</f>
-        <v>-3.2231421276827916</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E5/$E$27),0)</f>
+        <v>-9.4697904361571084</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -3254,7 +3239,7 @@
         <v>6951.5</v>
       </c>
       <c r="F6">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E6/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E6/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3276,7 +3261,7 @@
         <v>4058.2</v>
       </c>
       <c r="F7">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E7/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E7/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3298,7 +3283,7 @@
         <v>10693.9</v>
       </c>
       <c r="F8">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E8/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E8/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3320,7 +3305,7 @@
         <v>5822.8</v>
       </c>
       <c r="F9">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E9/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E9/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3342,7 +3327,7 @@
         <v>1329</v>
       </c>
       <c r="F10">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E10/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E10/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3364,7 +3349,7 @@
         <v>5525.3</v>
       </c>
       <c r="F11">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E11/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E11/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3386,7 +3371,7 @@
         <v>67098.8</v>
       </c>
       <c r="F12">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E12/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E12/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3408,7 +3393,7 @@
         <v>83166.7</v>
       </c>
       <c r="F13">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E13/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E13/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3430,7 +3415,7 @@
         <v>10709.7</v>
       </c>
       <c r="F14">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E14/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E14/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3452,7 +3437,7 @@
         <v>9769.5</v>
       </c>
       <c r="F15">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E15/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E15/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3474,7 +3459,7 @@
         <v>4963.8</v>
       </c>
       <c r="F16">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E16/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E16/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3496,7 +3481,7 @@
         <v>60244.6</v>
       </c>
       <c r="F17">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E17/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E17/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3518,7 +3503,7 @@
         <v>1907.7</v>
       </c>
       <c r="F18">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E18/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E18/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3540,7 +3525,7 @@
         <v>2794.1</v>
       </c>
       <c r="F19">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E19/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E19/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3562,7 +3547,7 @@
         <v>626.1</v>
       </c>
       <c r="F20">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E20/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E20/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3582,8 +3567,8 @@
         <v>514.6</v>
       </c>
       <c r="F21">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E21/$E$27,0)</f>
-        <v>-0.47497965031659928</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E21/$E$27),0)</f>
+        <v>-1.395519518455455</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -3602,8 +3587,8 @@
         <v>2579</v>
       </c>
       <c r="F22">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E22/$E$27,0)</f>
-        <v>-2.3804362964759216</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E22/$E$27),0)</f>
+        <v>-6.9938687098651737</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -3619,8 +3604,8 @@
         <v>621.9</v>
       </c>
       <c r="F23">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E23/$E$27,0)</f>
-        <v>-0.57401835315175476</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E23/$E$27),0)</f>
+        <v>-1.6865013379857121</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -3641,7 +3626,7 @@
         <v>17407.599999999999</v>
       </c>
       <c r="F24">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E24/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E24/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3663,7 +3648,7 @@
         <v>2076.3000000000002</v>
       </c>
       <c r="F25">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E25/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E25/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3685,7 +3670,7 @@
         <v>5367.6</v>
       </c>
       <c r="F26">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E26/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E26/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3704,11 +3689,11 @@
         <v>-53.28845247095488</v>
       </c>
       <c r="E27">
-        <f>E2+E5+E6+E7+E9+E10+E16+E18+E19+E20+E21+E22+E23+E25+E32+E33+E34+E41+E42</f>
-        <v>57733.5</v>
+        <f>SUMIF(D2:D26,"=0",E2:E26)+SUMIF(D28:D42,"=0",E28:E42)</f>
+        <v>19650.2</v>
       </c>
       <c r="F27">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E27/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E27/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3730,7 +3715,7 @@
         <v>37958.1</v>
       </c>
       <c r="F28">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E28/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E28/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3752,7 +3737,7 @@
         <v>10295.9</v>
       </c>
       <c r="F29">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E29/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E29/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3774,7 +3759,7 @@
         <v>19318</v>
       </c>
       <c r="F30">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E30/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E30/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3790,8 +3775,12 @@
         <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>0</v>
       </c>
-      <c r="E31" t="s">
-        <v>103</v>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E31/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -3810,8 +3799,8 @@
         <v>6926.7</v>
       </c>
       <c r="F32">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E32/$E$27,0)</f>
-        <v>-6.3933959266381413</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E32/$E$27),0)</f>
+        <v>-18.784191699349783</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -3832,7 +3821,7 @@
         <v>5457.9</v>
       </c>
       <c r="F33">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E33/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E33/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3854,7 +3843,7 @@
         <v>2095.9</v>
       </c>
       <c r="F34">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E34/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E34/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3876,7 +3865,7 @@
         <v>47330</v>
       </c>
       <c r="F35">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E35/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E35/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3898,7 +3887,7 @@
         <v>10327.6</v>
       </c>
       <c r="F36">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E36/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E36/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3920,7 +3909,7 @@
         <v>8606</v>
       </c>
       <c r="F37">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E37/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E37/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3942,7 +3931,7 @@
         <v>83155</v>
       </c>
       <c r="F38">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E38/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E38/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3964,7 +3953,7 @@
         <v>67025.5</v>
       </c>
       <c r="F39">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E39/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E39/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -3986,7 +3975,7 @@
         <v>41733</v>
       </c>
       <c r="F40">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E40/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E40/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4006,8 +3995,8 @@
         <v>888</v>
       </c>
       <c r="F41">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E41/$E$27,0)</f>
-        <v>-0.81963064415301234</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E41/$E$27),0)</f>
+        <v>-2.4081254030090244</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -4023,8 +4012,8 @@
         <v>1782</v>
       </c>
       <c r="F42">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*E42/$E$27,0)</f>
-        <v>-1.6447993331989503</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E42/$E$27),0)</f>
+        <v>-4.8325219236059471</v>
       </c>
     </row>
     <row r="50" spans="1:2">
@@ -4109,8 +4098,8 @@
         <v>2846</v>
       </c>
       <c r="F2">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E2/$E$27,0)</f>
-        <v>-14.255855473858333</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</f>
+        <v>-3.3547123739475664</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -4131,7 +4120,7 @@
         <v>8901.1</v>
       </c>
       <c r="F3">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E3/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E3/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4153,7 +4142,7 @@
         <v>11549.9</v>
       </c>
       <c r="F4">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E4/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E4/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4173,8 +4162,8 @@
         <v>3492</v>
       </c>
       <c r="F5">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E5/$E$27,0)</f>
-        <v>-17.491724284860609</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E5/$E$27),0)</f>
+        <v>-4.1161825754830996</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -4193,8 +4182,8 @@
         <v>6951.5</v>
       </c>
       <c r="F6">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E6/$E$27,0)</f>
-        <v>-34.820653312201756</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E6/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -4213,8 +4202,8 @@
         <v>4058.2</v>
       </c>
       <c r="F7">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E7/$E$27,0)</f>
-        <v>-20.327868125092017</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E7/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -4235,7 +4224,7 @@
         <v>10693.9</v>
       </c>
       <c r="F8">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E8/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E8/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4255,8 +4244,8 @@
         <v>5822.8</v>
       </c>
       <c r="F9">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E9/$E$27,0)</f>
-        <v>-29.166899245671924</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E9/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -4275,8 +4264,8 @@
         <v>1329</v>
       </c>
       <c r="F10">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E10/$E$27,0)</f>
-        <v>-6.6570737613344075</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E10/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -4297,7 +4286,7 @@
         <v>5525.3</v>
       </c>
       <c r="F11">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E11/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E11/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4319,7 +4308,7 @@
         <v>67098.8</v>
       </c>
       <c r="F12">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E12/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E12/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4341,7 +4330,7 @@
         <v>83166.7</v>
       </c>
       <c r="F13">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E13/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E13/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4363,7 +4352,7 @@
         <v>10709.7</v>
       </c>
       <c r="F14">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E14/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E14/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4385,7 +4374,7 @@
         <v>9769.5</v>
       </c>
       <c r="F15">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E15/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E15/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4405,8 +4394,8 @@
         <v>4963.8</v>
       </c>
       <c r="F16">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E16/$E$27,0)</f>
-        <v>-24.864095362311311</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E16/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -4427,7 +4416,7 @@
         <v>60244.6</v>
       </c>
       <c r="F17">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E17/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E17/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4447,8 +4436,8 @@
         <v>1907.7</v>
       </c>
       <c r="F18">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E18/$E$27,0)</f>
-        <v>-9.5558311621502252</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E18/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -4467,8 +4456,8 @@
         <v>2794.1</v>
       </c>
       <c r="F19">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E19/$E$27,0)</f>
-        <v>-13.995883970311864</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E19/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -4487,8 +4476,8 @@
         <v>626.1</v>
       </c>
       <c r="F20">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E20/$E$27,0)</f>
-        <v>-3.1361880225518983</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E20/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -4507,8 +4496,8 @@
         <v>514.6</v>
       </c>
       <c r="F21">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E21/$E$27,0)</f>
-        <v>-2.5776750621389666</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E21/$E$27),0)</f>
+        <v>-0.60658291905601469</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -4527,8 +4516,8 @@
         <v>2579</v>
       </c>
       <c r="F22">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E22/$E$27,0)</f>
-        <v>-12.918429819775348</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E22/$E$27),0)</f>
+        <v>-3.0399870739321062</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -4544,8 +4533,8 @@
         <v>621.9</v>
       </c>
       <c r="F23">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E23/$E$27,0)</f>
-        <v>-3.1151498661955364</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E23/$E$27),0)</f>
+        <v>-0.73306241228320157</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -4566,7 +4555,7 @@
         <v>17407.599999999999</v>
       </c>
       <c r="F24">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E24/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E24/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4586,8 +4575,8 @@
         <v>2076.3000000000002</v>
       </c>
       <c r="F25">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E25/$E$27,0)</f>
-        <v>-10.40036286731274</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E25/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -4608,7 +4597,7 @@
         <v>5367.6</v>
       </c>
       <c r="F26">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E26/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E26/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4620,18 +4609,18 @@
         <v>90</v>
       </c>
       <c r="C27" s="2">
-        <v>29.6</v>
+        <v>6.9655227952428636</v>
       </c>
       <c r="D27">
         <f>Table15[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-289.19200000000001</v>
+        <v>-68.053157709522779</v>
       </c>
       <c r="E27">
-        <f>E2+E5+E6+E7+E9+E10+E16+E18+E19+E20+E21+E22+E23+E25+E32+E33+E34+E41+E42</f>
+        <f>SUMIF(D2:D26,"=0",E2:E26)+SUMIF(D28:D42,"=0",E28:E42)</f>
         <v>57733.5</v>
       </c>
       <c r="F27">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E27/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E27/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4653,7 +4642,7 @@
         <v>37958.1</v>
       </c>
       <c r="F28">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E28/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E28/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4675,7 +4664,7 @@
         <v>10295.9</v>
       </c>
       <c r="F29">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E29/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E29/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4697,7 +4686,7 @@
         <v>19318</v>
       </c>
       <c r="F30">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E30/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E30/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4713,8 +4702,12 @@
         <f>Table15[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>0</v>
       </c>
-      <c r="E31" t="s">
-        <v>103</v>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E31/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -4733,8 +4726,8 @@
         <v>6926.7</v>
       </c>
       <c r="F32">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E32/$E$27,0)</f>
-        <v>-34.696428008002286</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E32/$E$27),0)</f>
+        <v>-8.1648229798392862</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -4753,8 +4746,8 @@
         <v>5457.9</v>
       </c>
       <c r="F33">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E33/$E$27,0)</f>
-        <v>-27.339084185091842</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E33/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -4773,8 +4766,8 @@
         <v>2095.9</v>
       </c>
       <c r="F34">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E34/$E$27,0)</f>
-        <v>-10.498540930309094</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E34/$E$27),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -4795,7 +4788,7 @@
         <v>47330</v>
       </c>
       <c r="F35">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E35/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E35/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4817,7 +4810,7 @@
         <v>10327.6</v>
       </c>
       <c r="F36">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E36/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E36/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4839,7 +4832,7 @@
         <v>8606</v>
       </c>
       <c r="F37">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E37/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E37/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4861,7 +4854,7 @@
         <v>83155</v>
       </c>
       <c r="F38">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E38/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E38/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4883,7 +4876,7 @@
         <v>67025.5</v>
       </c>
       <c r="F39">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E39/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E39/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4905,7 +4898,7 @@
         <v>41733</v>
       </c>
       <c r="F40">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E40/$E$27,0)</f>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E40/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4925,8 +4918,8 @@
         <v>888</v>
       </c>
       <c r="F41">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E41/$E$27,0)</f>
-        <v>-4.4480673439164438</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E41/$E$27),0)</f>
+        <v>-1.046726840500857</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -4942,8 +4935,8 @@
         <v>1782</v>
       </c>
       <c r="F42">
-        <f>IF(Table15[[#This Row],[TWh '[2020']]]=0,$D$27*E42/$E$27,0)</f>
-        <v>-8.9261891969134037</v>
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E42/$E$27),0)</f>
+        <v>-2.1005261596537466</v>
       </c>
     </row>
     <row r="50" spans="1:2">

</xml_diff>

<commit_message>
update production data for 2020
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A8BFAD9-B3F8-4153-8762-D9C5883BA897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A42C35-6F73-4CF3-A238-6CD046593CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
-    <sheet name="nodes_gas_prod" sheetId="2" r:id="rId2"/>
+    <sheet name="nodes_gas_prod_2020" sheetId="2" r:id="rId2"/>
     <sheet name="nodes_demand_2020" sheetId="3" r:id="rId3"/>
     <sheet name="nodes_demand_2023" sheetId="6" r:id="rId4"/>
     <sheet name="Connections" sheetId="4" r:id="rId5"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="138">
   <si>
     <t>Belgium</t>
   </si>
@@ -296,9 +296,6 @@
   </si>
   <si>
     <t>Sweden</t>
-  </si>
-  <si>
-    <t>https://www.bp.com/content/dam/bp/business-sites/en/global/corporate/pdfs/energy-economics/statistical-review/bp-stats-review-2021-full-report.pdf</t>
   </si>
   <si>
     <t>Mrd m3 [2020]</t>
@@ -623,15 +620,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyFill="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyFill="0" applyBorder="0">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -690,49 +684,48 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="42">
-    <cellStyle name="04_Table text" xfId="3" xr:uid="{60FAF7FD-D988-4AB0-B86F-CAD4D7C5E89B}"/>
-    <cellStyle name="C01_Main head" xfId="23" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
-    <cellStyle name="C02_Column heads" xfId="17" xr:uid="{6AA76714-52DD-4B3B-9F1F-E7ED06188786}"/>
-    <cellStyle name="C03_Sub head bold" xfId="18" xr:uid="{71BDF15F-8FAB-4B9D-BF56-0C82A383AA8E}"/>
-    <cellStyle name="C04_Total text white bold" xfId="21" xr:uid="{287E28E8-DA9A-4DA7-94AD-5AF1C537F15F}"/>
-    <cellStyle name="C04a_Total text black with rule" xfId="20" xr:uid="{16CE27B2-E630-4389-8700-BC6F07A207BB}"/>
-    <cellStyle name="C05_Main text" xfId="19" xr:uid="{19A3C003-4A4D-4B53-B889-86660BE2F4A7}"/>
-    <cellStyle name="C06_Figs" xfId="25" xr:uid="{6EF7291D-EE46-4629-B94D-1ECDF30BDA6F}"/>
-    <cellStyle name="C07_Figs 1 dec percent" xfId="33" xr:uid="{47221C8E-FC37-465A-9665-18759B74A6CE}"/>
-    <cellStyle name="C09_Notes" xfId="8" xr:uid="{9085F154-117F-416B-8D81-36A9DB81FB8C}"/>
-    <cellStyle name="Comma 2" xfId="15" xr:uid="{C220F88A-4F55-4623-B6C1-AD23C8E74659}"/>
-    <cellStyle name="Comma 5" xfId="30" xr:uid="{0067ED6D-11E5-44AC-9D53-C45880789330}"/>
+  <cellStyles count="41">
+    <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
+    <cellStyle name="C02_Column heads" xfId="16" xr:uid="{6AA76714-52DD-4B3B-9F1F-E7ED06188786}"/>
+    <cellStyle name="C03_Sub head bold" xfId="17" xr:uid="{71BDF15F-8FAB-4B9D-BF56-0C82A383AA8E}"/>
+    <cellStyle name="C04_Total text white bold" xfId="20" xr:uid="{287E28E8-DA9A-4DA7-94AD-5AF1C537F15F}"/>
+    <cellStyle name="C04a_Total text black with rule" xfId="19" xr:uid="{16CE27B2-E630-4389-8700-BC6F07A207BB}"/>
+    <cellStyle name="C05_Main text" xfId="18" xr:uid="{19A3C003-4A4D-4B53-B889-86660BE2F4A7}"/>
+    <cellStyle name="C06_Figs" xfId="24" xr:uid="{6EF7291D-EE46-4629-B94D-1ECDF30BDA6F}"/>
+    <cellStyle name="C07_Figs 1 dec percent" xfId="32" xr:uid="{47221C8E-FC37-465A-9665-18759B74A6CE}"/>
+    <cellStyle name="C09_Notes" xfId="7" xr:uid="{9085F154-117F-416B-8D81-36A9DB81FB8C}"/>
+    <cellStyle name="Comma 2" xfId="14" xr:uid="{C220F88A-4F55-4623-B6C1-AD23C8E74659}"/>
+    <cellStyle name="Comma 5" xfId="29" xr:uid="{0067ED6D-11E5-44AC-9D53-C45880789330}"/>
     <cellStyle name="Hyperlink 2" xfId="2" xr:uid="{BA9329EA-B184-49A9-9DC3-748FF9EBB7D9}"/>
-    <cellStyle name="Hyperlink 2 2" xfId="4" xr:uid="{F9103865-4F21-4889-8B72-20BE8654C338}"/>
-    <cellStyle name="Hyperlink 2 2 2" xfId="13" xr:uid="{5BCD4CE7-6B2C-456F-8FB9-324AD7E49CAD}"/>
-    <cellStyle name="Hyperlink 3" xfId="14" xr:uid="{94940656-2676-4A09-B05D-BC18288B254C}"/>
+    <cellStyle name="Hyperlink 2 2" xfId="3" xr:uid="{F9103865-4F21-4889-8B72-20BE8654C338}"/>
+    <cellStyle name="Hyperlink 2 2 2" xfId="12" xr:uid="{5BCD4CE7-6B2C-456F-8FB9-324AD7E49CAD}"/>
+    <cellStyle name="Hyperlink 3" xfId="13" xr:uid="{94940656-2676-4A09-B05D-BC18288B254C}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 18" xfId="31" xr:uid="{E7EAE102-3B70-42A2-97BE-6613C6991711}"/>
+    <cellStyle name="Normal 18" xfId="30" xr:uid="{E7EAE102-3B70-42A2-97BE-6613C6991711}"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{190F2216-BF41-4842-8670-90BCBED25C1F}"/>
-    <cellStyle name="Normal 2 2" xfId="9" xr:uid="{BBA1F6BA-F8D2-45BD-89F2-5F79E7C1C329}"/>
-    <cellStyle name="Normal 2 2 2" xfId="27" xr:uid="{AD51099B-D49D-45FE-80D3-1F4120CAB713}"/>
-    <cellStyle name="Normal 2 2 3" xfId="32" xr:uid="{685F2931-69F1-4742-862E-8D36BACD9F1A}"/>
-    <cellStyle name="Normal 2 2 9 2" xfId="38" xr:uid="{1D997E3D-2769-4905-B0EB-950CAA58DB0A}"/>
-    <cellStyle name="Normal 2 3" xfId="41" xr:uid="{1A02E014-9D0A-45BD-84AD-CEF3659D5A24}"/>
-    <cellStyle name="Normal 2 5" xfId="28" xr:uid="{BA56A082-19D7-4317-9FF5-DEC1FFBEF23C}"/>
-    <cellStyle name="Normal 2 6" xfId="10" xr:uid="{A9C605D1-161F-4025-811E-28DABC062934}"/>
-    <cellStyle name="Normal 20" xfId="22" xr:uid="{648D11FF-279B-4F0E-B09D-8C1EC6061892}"/>
-    <cellStyle name="Normal 3" xfId="11" xr:uid="{C48EB3F3-1975-4918-BAB7-BE900719A5F7}"/>
-    <cellStyle name="Normal 33" xfId="6" xr:uid="{5CD1E707-8667-45EC-ABF6-B60F6E9E59D3}"/>
-    <cellStyle name="Normal 4" xfId="40" xr:uid="{6FD259F4-48D1-4A86-985F-41950DBD9149}"/>
-    <cellStyle name="Normal 4 2 2" xfId="5" xr:uid="{919221B1-42A4-4700-9239-2DAFE893779F}"/>
-    <cellStyle name="Normal 5" xfId="37" xr:uid="{7566378D-1084-4857-A4BB-1DAAB3764B14}"/>
-    <cellStyle name="Normal 5 8 2" xfId="39" xr:uid="{AEB2F650-B345-44F9-857E-1FF7EFC5D55E}"/>
-    <cellStyle name="Normal 6" xfId="12" xr:uid="{D03254E9-8E42-4BF4-8A58-7DE6DA4A8303}"/>
-    <cellStyle name="Normal 8" xfId="7" xr:uid="{90F0E83A-EA1A-48E1-A5EE-D67EB082C60D}"/>
-    <cellStyle name="Normal 8 2" xfId="24" xr:uid="{A358C3D2-DBD8-459F-9B06-BAA976C32485}"/>
-    <cellStyle name="Normal 8 7" xfId="26" xr:uid="{76B13E51-C838-4F8D-AADA-E10D7E632F63}"/>
-    <cellStyle name="Percent 2" xfId="16" xr:uid="{8FA158A0-20DC-4018-9CF3-EDDF9FADF72C}"/>
-    <cellStyle name="Percent 2 2" xfId="29" xr:uid="{0AA4CE3F-8960-4102-9CAE-7448A8126969}"/>
-    <cellStyle name="Percent 3" xfId="35" xr:uid="{8AB380C1-64CC-421C-8275-BF15C8D4F870}"/>
-    <cellStyle name="Percent 4" xfId="36" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
-    <cellStyle name="Percent 8" xfId="34" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
+    <cellStyle name="Normal 2 2" xfId="8" xr:uid="{BBA1F6BA-F8D2-45BD-89F2-5F79E7C1C329}"/>
+    <cellStyle name="Normal 2 2 2" xfId="26" xr:uid="{AD51099B-D49D-45FE-80D3-1F4120CAB713}"/>
+    <cellStyle name="Normal 2 2 3" xfId="31" xr:uid="{685F2931-69F1-4742-862E-8D36BACD9F1A}"/>
+    <cellStyle name="Normal 2 2 9 2" xfId="37" xr:uid="{1D997E3D-2769-4905-B0EB-950CAA58DB0A}"/>
+    <cellStyle name="Normal 2 3" xfId="40" xr:uid="{1A02E014-9D0A-45BD-84AD-CEF3659D5A24}"/>
+    <cellStyle name="Normal 2 5" xfId="27" xr:uid="{BA56A082-19D7-4317-9FF5-DEC1FFBEF23C}"/>
+    <cellStyle name="Normal 2 6" xfId="9" xr:uid="{A9C605D1-161F-4025-811E-28DABC062934}"/>
+    <cellStyle name="Normal 20" xfId="21" xr:uid="{648D11FF-279B-4F0E-B09D-8C1EC6061892}"/>
+    <cellStyle name="Normal 3" xfId="10" xr:uid="{C48EB3F3-1975-4918-BAB7-BE900719A5F7}"/>
+    <cellStyle name="Normal 33" xfId="5" xr:uid="{5CD1E707-8667-45EC-ABF6-B60F6E9E59D3}"/>
+    <cellStyle name="Normal 4" xfId="39" xr:uid="{6FD259F4-48D1-4A86-985F-41950DBD9149}"/>
+    <cellStyle name="Normal 4 2 2" xfId="4" xr:uid="{919221B1-42A4-4700-9239-2DAFE893779F}"/>
+    <cellStyle name="Normal 5" xfId="36" xr:uid="{7566378D-1084-4857-A4BB-1DAAB3764B14}"/>
+    <cellStyle name="Normal 5 8 2" xfId="38" xr:uid="{AEB2F650-B345-44F9-857E-1FF7EFC5D55E}"/>
+    <cellStyle name="Normal 6" xfId="11" xr:uid="{D03254E9-8E42-4BF4-8A58-7DE6DA4A8303}"/>
+    <cellStyle name="Normal 8" xfId="6" xr:uid="{90F0E83A-EA1A-48E1-A5EE-D67EB082C60D}"/>
+    <cellStyle name="Normal 8 2" xfId="23" xr:uid="{A358C3D2-DBD8-459F-9B06-BAA976C32485}"/>
+    <cellStyle name="Normal 8 7" xfId="25" xr:uid="{76B13E51-C838-4F8D-AADA-E10D7E632F63}"/>
+    <cellStyle name="Percent 2" xfId="15" xr:uid="{8FA158A0-20DC-4018-9CF3-EDDF9FADF72C}"/>
+    <cellStyle name="Percent 2 2" xfId="28" xr:uid="{0AA4CE3F-8960-4102-9CAE-7448A8126969}"/>
+    <cellStyle name="Percent 3" xfId="34" xr:uid="{8AB380C1-64CC-421C-8275-BF15C8D4F870}"/>
+    <cellStyle name="Percent 4" xfId="35" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
+    <cellStyle name="Percent 8" xfId="33" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
   <dxfs count="10">
     <dxf>
@@ -1139,7 +1132,7 @@
         <v>15</v>
       </c>
       <c r="C1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D1" t="s">
         <v>13</v>
@@ -1148,16 +1141,16 @@
         <v>14</v>
       </c>
       <c r="F1" t="s">
+        <v>105</v>
+      </c>
+      <c r="G1" t="s">
         <v>106</v>
       </c>
-      <c r="G1" t="s">
-        <v>107</v>
-      </c>
       <c r="L1" t="s">
+        <v>93</v>
+      </c>
+      <c r="M1" t="s">
         <v>94</v>
-      </c>
-      <c r="M1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -1189,7 +1182,7 @@
         <v>17</v>
       </c>
       <c r="J2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L2" t="str">
         <f>_xlfn.CONCAT(I2,J2)</f>
@@ -1229,7 +1222,7 @@
         <v>25</v>
       </c>
       <c r="J3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L3" t="str">
         <f t="shared" ref="L3:L19" si="2">_xlfn.CONCAT(I3,J3)</f>
@@ -1269,7 +1262,7 @@
         <v>33</v>
       </c>
       <c r="J4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="2"/>
@@ -1309,7 +1302,7 @@
         <v>21</v>
       </c>
       <c r="J5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="2"/>
@@ -1349,7 +1342,7 @@
         <v>24</v>
       </c>
       <c r="J6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="2"/>
@@ -1389,7 +1382,7 @@
         <v>35</v>
       </c>
       <c r="J7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="2"/>
@@ -1429,7 +1422,7 @@
         <v>18</v>
       </c>
       <c r="J8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L8" t="str">
         <f t="shared" si="2"/>
@@ -1469,7 +1462,7 @@
         <v>27</v>
       </c>
       <c r="J9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L9" t="str">
         <f t="shared" si="2"/>
@@ -1509,7 +1502,7 @@
         <v>38</v>
       </c>
       <c r="J10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L10" t="str">
         <f t="shared" si="2"/>
@@ -1549,7 +1542,7 @@
         <v>37</v>
       </c>
       <c r="J11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L11" t="str">
         <f t="shared" si="2"/>
@@ -1589,7 +1582,7 @@
         <v>47</v>
       </c>
       <c r="J12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L12" t="str">
         <f t="shared" si="2"/>
@@ -1629,7 +1622,7 @@
         <v>11</v>
       </c>
       <c r="J13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L13" t="str">
         <f t="shared" si="2"/>
@@ -1642,7 +1635,7 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B14">
         <v>0.7</v>
@@ -1660,12 +1653,12 @@
         <v>6.8389999999999995</v>
       </c>
       <c r="I14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B15">
         <v>2.5</v>
@@ -1686,7 +1679,7 @@
         <v>54</v>
       </c>
       <c r="J15" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L15" t="str">
         <f t="shared" si="2"/>
@@ -1699,7 +1692,7 @@
     </row>
     <row r="16" spans="1:13">
       <c r="A16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B16">
         <v>5</v>
@@ -1720,7 +1713,7 @@
         <v>55</v>
       </c>
       <c r="J16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L16" t="str">
         <f t="shared" si="2"/>
@@ -1733,7 +1726,7 @@
     </row>
     <row r="17" spans="1:13">
       <c r="A17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B17">
         <v>31.2</v>
@@ -1754,7 +1747,7 @@
         <v>19</v>
       </c>
       <c r="J17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L17" t="str">
         <f t="shared" si="2"/>
@@ -1767,7 +1760,7 @@
     </row>
     <row r="18" spans="1:13">
       <c r="A18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B18">
         <v>2.6</v>
@@ -1788,7 +1781,7 @@
         <v>44</v>
       </c>
       <c r="J18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L18" t="str">
         <f t="shared" si="2"/>
@@ -1801,7 +1794,7 @@
     </row>
     <row r="19" spans="1:13">
       <c r="A19" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B19">
         <v>1.5</v>
@@ -1822,7 +1815,7 @@
         <v>36</v>
       </c>
       <c r="J19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L19" t="str">
         <f t="shared" si="2"/>
@@ -1856,22 +1849,22 @@
         <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L1" t="s">
+        <v>93</v>
+      </c>
+      <c r="M1" t="s">
         <v>94</v>
-      </c>
-      <c r="M1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -1895,7 +1888,7 @@
       </c>
       <c r="G2" s="2"/>
       <c r="I2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="L2" t="str">
         <f t="shared" ref="L2:L40" si="0">_xlfn.CONCAT(A2,$I$2)</f>
@@ -1914,7 +1907,7 @@
         <v>79</v>
       </c>
       <c r="C3" s="2">
-        <v>81.5</v>
+        <v>81.424612499999995</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2">
@@ -1923,7 +1916,7 @@
       </c>
       <c r="F3" s="3">
         <f>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>796.255</v>
+        <v>795.51846412499992</v>
       </c>
       <c r="G3" s="2"/>
       <c r="L3" t="str">
@@ -2142,18 +2135,18 @@
         <v>61</v>
       </c>
       <c r="C11" s="2">
-        <v>1.4</v>
+        <v>1.3796929768583337</v>
       </c>
       <c r="D11" s="2">
-        <v>1427.5409999999997</v>
+        <v>1427.5409999999999</v>
       </c>
       <c r="E11" s="2">
         <f>Table2[[#This Row],[Mil m3 EU '[2020']]]/1000</f>
-        <v>1.4275409999999997</v>
+        <v>1.4275409999999999</v>
       </c>
       <c r="F11" s="3">
         <f>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>13.947075569999997</v>
+        <v>13.947075569999999</v>
       </c>
       <c r="G11" s="2"/>
       <c r="L11" t="str">
@@ -2199,7 +2192,7 @@
         <v>55</v>
       </c>
       <c r="B13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -2258,7 +2251,7 @@
         <v>57</v>
       </c>
       <c r="C15" s="2">
-        <v>4.5</v>
+        <v>4.5324203399999998</v>
       </c>
       <c r="D15" s="2">
         <v>4874</v>
@@ -2376,7 +2369,7 @@
         <v>4</v>
       </c>
       <c r="C19" s="2">
-        <v>3.9</v>
+        <v>3.9120907084594152</v>
       </c>
       <c r="D19" s="2">
         <v>3932</v>
@@ -2434,7 +2427,7 @@
         <v>81</v>
       </c>
       <c r="C21" s="2">
-        <v>13.3</v>
+        <v>12.699712072345603</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2">
@@ -2443,7 +2436,7 @@
       </c>
       <c r="F21" s="3">
         <f>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>129.941</v>
+        <v>124.07618694681653</v>
       </c>
       <c r="G21" s="2"/>
       <c r="L21" t="str">
@@ -2544,7 +2537,7 @@
         <v>7</v>
       </c>
       <c r="C25" s="2">
-        <v>20</v>
+        <v>20.091666666666669</v>
       </c>
       <c r="D25" s="2">
         <v>23966.123</v>
@@ -2602,7 +2595,7 @@
         <v>72</v>
       </c>
       <c r="C27" s="2">
-        <v>111.5</v>
+        <v>111.71588259981999</v>
       </c>
       <c r="D27" s="2">
         <v>116206.11699999998</v>
@@ -2633,7 +2626,7 @@
         <v>8</v>
       </c>
       <c r="C28" s="2">
-        <v>3.9</v>
+        <v>3.9287777777777784</v>
       </c>
       <c r="D28" s="2">
         <v>5592.88</v>
@@ -2688,10 +2681,10 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C30" s="2">
-        <v>8.6999999999999993</v>
+        <v>8.5963213888888905</v>
       </c>
       <c r="D30" s="2">
         <v>9017</v>
@@ -2722,7 +2715,7 @@
         <v>70</v>
       </c>
       <c r="C31" s="2">
-        <v>638.5</v>
+        <v>638.44665603244835</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2">
@@ -2731,7 +2724,7 @@
       </c>
       <c r="F31" s="3">
         <f>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>6238.1449999999995</v>
+        <v>6237.6238294370205</v>
       </c>
       <c r="G31" s="2"/>
       <c r="L31" t="str">
@@ -2950,7 +2943,7 @@
         <v>11</v>
       </c>
       <c r="C39" s="2">
-        <v>39.5</v>
+        <v>39.571421400000006</v>
       </c>
       <c r="D39" s="2">
         <v>32836.551999999996</v>
@@ -2981,7 +2974,7 @@
         <v>68</v>
       </c>
       <c r="C40" s="2">
-        <v>19</v>
+        <v>19.117502458210424</v>
       </c>
       <c r="D40" s="2">
         <v>19516</v>
@@ -3006,13 +2999,13 @@
     </row>
     <row r="41" spans="1:13">
       <c r="A41" t="s">
+        <v>88</v>
+      </c>
+      <c r="B41" t="s">
         <v>89</v>
       </c>
-      <c r="B41" t="s">
-        <v>90</v>
-      </c>
       <c r="C41" s="2">
-        <v>6.3</v>
+        <v>6.2834748117948553</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2">
@@ -3021,7 +3014,7 @@
       </c>
       <c r="F41" s="3">
         <f>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>61.550999999999995</v>
+        <v>61.389548911235735</v>
       </c>
       <c r="G41" s="2"/>
       <c r="L41" t="str">
@@ -3064,11 +3057,11 @@
     <row r="44" spans="1:13">
       <c r="C44" s="2">
         <f>SUM(Table2[Mrd m3 '[2020']])</f>
-        <v>953.9</v>
+        <v>953.60023173327022</v>
       </c>
       <c r="D44" s="2">
         <f>SUM(Table2[Mil m3 EU '[2020']])/1000+C31+C37+C21+C3</f>
-        <v>959.24681999999996</v>
+        <v>958.51780060479393</v>
       </c>
       <c r="E44">
         <f>SUMIF(Table2[Mil m3 EU '[2020']],"&gt;0",Table2[Mrd m3 EU '[2020']])</f>
@@ -3080,7 +3073,7 @@
     </row>
     <row r="47" spans="1:13">
       <c r="A47" t="s">
-        <v>85</v>
+        <v>135</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -3088,15 +3081,15 @@
         <v>80</v>
       </c>
       <c r="B48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B49" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -3127,16 +3120,16 @@
         <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -3338,7 +3331,7 @@
         <v>55</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C11" s="2">
         <v>2.0718055555555557</v>
@@ -3555,10 +3548,10 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21">
@@ -3595,7 +3588,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="B23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23">
@@ -3678,10 +3671,10 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" t="s">
         <v>89</v>
-      </c>
-      <c r="B27" t="s">
-        <v>90</v>
       </c>
       <c r="C27" s="2">
         <v>5.4542940093096091</v>
@@ -3748,7 +3741,7 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C30" s="2">
         <v>11.262552972222222</v>
@@ -3983,10 +3976,10 @@
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
+        <v>111</v>
+      </c>
+      <c r="B41" t="s">
         <v>112</v>
-      </c>
-      <c r="B41" t="s">
-        <v>113</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41">
@@ -4003,7 +3996,7 @@
     </row>
     <row r="42" spans="1:6">
       <c r="B42" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42">
@@ -4020,28 +4013,28 @@
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" t="s">
+        <v>116</v>
+      </c>
+      <c r="B52" t="s">
         <v>117</v>
-      </c>
-      <c r="B52" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" t="s">
+        <v>118</v>
+      </c>
+      <c r="B53" t="s">
         <v>119</v>
-      </c>
-      <c r="B53" t="s">
-        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -4072,16 +4065,16 @@
         <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -4283,7 +4276,7 @@
         <v>55</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C11" s="2">
         <v>1.1944166666666667</v>
@@ -4500,10 +4493,10 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21">
@@ -4540,7 +4533,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="B23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23">
@@ -4623,10 +4616,10 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" t="s">
         <v>89</v>
-      </c>
-      <c r="B27" t="s">
-        <v>90</v>
       </c>
       <c r="C27" s="2">
         <v>6.9655227952428636</v>
@@ -4693,7 +4686,7 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C30" s="2">
         <v>9.0859916688941222</v>
@@ -4928,10 +4921,10 @@
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
+        <v>111</v>
+      </c>
+      <c r="B41" t="s">
         <v>112</v>
-      </c>
-      <c r="B41" t="s">
-        <v>113</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41">
@@ -4948,7 +4941,7 @@
     </row>
     <row r="42" spans="1:6">
       <c r="B42" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42">
@@ -4965,28 +4958,28 @@
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" t="s">
+        <v>116</v>
+      </c>
+      <c r="B52" t="s">
         <v>117</v>
-      </c>
-      <c r="B52" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" t="s">
+        <v>118</v>
+      </c>
+      <c r="B53" t="s">
         <v>119</v>
-      </c>
-      <c r="B53" t="s">
-        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -5008,19 +5001,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" t="s">
         <v>94</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>95</v>
       </c>
-      <c r="C1" t="s">
-        <v>96</v>
-      </c>
       <c r="D1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E1" t="s">
         <v>109</v>
-      </c>
-      <c r="E1" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -6760,19 +6753,19 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" t="s">
         <v>94</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>95</v>
       </c>
-      <c r="C1" t="s">
-        <v>96</v>
-      </c>
       <c r="D1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E1" t="s">
         <v>109</v>
-      </c>
-      <c r="E1" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -6796,10 +6789,10 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" t="s">
         <v>98</v>
-      </c>
-      <c r="B3" t="s">
-        <v>99</v>
       </c>
       <c r="C3">
         <v>395</v>
@@ -7044,7 +7037,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B16" t="s">
         <v>37</v>
@@ -7161,7 +7154,7 @@
         <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C22">
         <v>385</v>
@@ -7253,7 +7246,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B27" t="s">
         <v>33</v>
@@ -7275,7 +7268,7 @@
         <v>50</v>
       </c>
       <c r="B28" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C28">
         <f>C15</f>
@@ -7290,7 +7283,7 @@
         <v>123.04150000000001</v>
       </c>
       <c r="F28" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -7312,7 +7305,7 @@
         <v>421.21</v>
       </c>
       <c r="F29" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -7334,7 +7327,7 @@
         <v>14.965</v>
       </c>
       <c r="F30" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -7345,7 +7338,7 @@
         <v>53</v>
       </c>
       <c r="F31" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -7367,7 +7360,7 @@
         <v>117.49349999999998</v>
       </c>
       <c r="F33" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -7389,12 +7382,12 @@
         <v>117.49349999999998</v>
       </c>
       <c r="F34" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add 2025 entsog capacities
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4FA34C9-A7BB-4E36-9388-A00A8B3D0AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65FC2583-9393-4B12-92C7-C994959F149C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="nodes_gas_prod_2024" sheetId="7" r:id="rId3"/>
     <sheet name="nodes_demand_2020" sheetId="3" r:id="rId4"/>
     <sheet name="nodes_demand_2023" sheetId="6" r:id="rId5"/>
-    <sheet name="Connections" sheetId="4" r:id="rId6"/>
+    <sheet name="Connections_2020" sheetId="4" r:id="rId6"/>
     <sheet name="Import_Connections" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -739,13 +739,10 @@
   </cellStyles>
   <dxfs count="14">
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
@@ -760,10 +757,13 @@
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
@@ -824,12 +824,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="1">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="7">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="0">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="6">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -846,12 +846,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="8">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="4">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="7">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="3">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -868,12 +868,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="5">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="1">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="4">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="0">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>

</xml_diff>

<commit_message>
update capacity values from gasdashboard by entsog
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{723F7426-73C0-40B6-B690-D0B6E6F42466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{832237F2-9583-4190-A328-0990B39D810F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,8 @@
     <sheet name="nodes_demand_2020" sheetId="3" r:id="rId4"/>
     <sheet name="nodes_demand_2023" sheetId="6" r:id="rId5"/>
     <sheet name="Connections_2021" sheetId="4" r:id="rId6"/>
-    <sheet name="Import_Connections" sheetId="5" r:id="rId7"/>
+    <sheet name="Connections_2024" sheetId="8" r:id="rId7"/>
+    <sheet name="Import_Connections" sheetId="5" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="985" uniqueCount="152">
   <si>
     <t>Belgium</t>
   </si>
@@ -726,14 +727,12 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -778,7 +777,10 @@
     <cellStyle name="Percent 4" xfId="35" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
     <cellStyle name="Percent 8" xfId="33" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -846,12 +848,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D3465064-BCEE-4D04-A8E6-DEAE11BBDA92}" name="Country"/>
     <tableColumn id="2" xr3:uid="{D66D54B4-4DED-47C6-BE50-755A236428ED}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="12">
+    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="13">
       <calculatedColumnFormula>Table2[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="11">
+    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="12">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -868,12 +870,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="8">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="9">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="7">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="8">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -890,12 +892,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="5">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="6">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="4">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="5">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -912,12 +914,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="2">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="3">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="1">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="2">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -937,13 +939,37 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="0">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="1">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
       <calculatedColumnFormula>F2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{E4B126C2-804B-4928-BF8B-8FE6229310A1}" name="Comment"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FC7F2F97-F859-4A2C-9657-17C35EEFE785}" name="Table37" displayName="Table37" ref="A1:H111" totalsRowShown="0">
+  <autoFilter ref="A1:H111" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H111">
+    <sortCondition ref="B1:B111"/>
+  </sortState>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{F94559DC-2602-4FF1-9531-3B8A374512C0}" name="From"/>
+    <tableColumn id="2" xr3:uid="{C59F5B7E-5BA7-48FA-B638-C3CA1C390D23}" name="To"/>
+    <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
+    <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
+    <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="0">
+      <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
+      <calculatedColumnFormula>F2/1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{18E94D69-5388-4B9B-8C8E-7A29BC79BE42}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6353,7 +6379,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD7211D-DC17-4DD6-B657-CA08F8FBC20F}">
-  <dimension ref="A1:M111"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="20.453125" customWidth="1"/>
@@ -6363,7 +6389,7 @@
     <col min="11" max="12" width="10.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>93</v>
       </c>
@@ -6389,7 +6415,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -6399,19 +6425,19 @@
       <c r="C2">
         <v>487.1</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>177791.5</v>
       </c>
       <c r="G2">
-        <f>F2/1000</f>
+        <f t="shared" ref="G2:G33" si="0">F2/1000</f>
         <v>177.79150000000001</v>
       </c>
       <c r="H2" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -6426,11 +6452,11 @@
         <v>125650.51999999997</v>
       </c>
       <c r="G3">
-        <f>F3/1000</f>
+        <f t="shared" si="0"/>
         <v>125.65051999999997</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -6445,11 +6471,11 @@
         <v>70627.5</v>
       </c>
       <c r="G4">
-        <f>F4/1000</f>
+        <f t="shared" si="0"/>
         <v>70.627499999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -6464,11 +6490,11 @@
         <v>573196</v>
       </c>
       <c r="G5">
-        <f>F5/1000</f>
+        <f t="shared" si="0"/>
         <v>573.19600000000003</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -6483,11 +6509,11 @@
         <v>6562.7</v>
       </c>
       <c r="G6">
-        <f>F6/1000</f>
+        <f t="shared" si="0"/>
         <v>6.5626999999999995</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -6502,11 +6528,11 @@
         <v>95301.500000000015</v>
       </c>
       <c r="G7">
-        <f>F7/1000</f>
+        <f t="shared" si="0"/>
         <v>95.301500000000019</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -6521,11 +6547,11 @@
         <v>509978</v>
       </c>
       <c r="G8">
-        <f>F8/1000</f>
+        <f t="shared" si="0"/>
         <v>509.97800000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -6540,11 +6566,11 @@
         <v>144594.75</v>
       </c>
       <c r="G9">
-        <f>F9/1000</f>
+        <f t="shared" si="0"/>
         <v>144.59475</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -6559,11 +6585,11 @@
         <v>98550</v>
       </c>
       <c r="G10">
-        <f>F10/1000</f>
+        <f t="shared" si="0"/>
         <v>98.55</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>49</v>
       </c>
@@ -6581,11 +6607,11 @@
         <v>124209.5</v>
       </c>
       <c r="G11">
-        <f>F11/1000</f>
+        <f t="shared" si="0"/>
         <v>124.20950000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -6595,17 +6621,16 @@
       <c r="E12">
         <v>41.973541999999995</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>15320.342829999998</v>
       </c>
       <c r="G12">
-        <f>F12/1000</f>
+        <f t="shared" si="0"/>
         <v>15.320342829999998</v>
       </c>
-      <c r="M12" s="5"/>
-    </row>
-    <row r="13" spans="1:13">
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -6620,11 +6645,11 @@
         <v>122369.9</v>
       </c>
       <c r="G13">
-        <f>F13/1000</f>
+        <f t="shared" si="0"/>
         <v>122.3699</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:8">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -6639,11 +6664,11 @@
         <v>23659.3</v>
       </c>
       <c r="G14">
-        <f>F14/1000</f>
+        <f t="shared" si="0"/>
         <v>23.659299999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:8">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -6658,11 +6683,11 @@
         <v>294098.75000000006</v>
       </c>
       <c r="G15">
-        <f>F15/1000</f>
+        <f t="shared" si="0"/>
         <v>294.09875000000005</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:8">
       <c r="A16" t="s">
         <v>47</v>
       </c>
@@ -6677,7 +6702,7 @@
         <v>210250.94999999998</v>
       </c>
       <c r="G16">
-        <f>F16/1000</f>
+        <f t="shared" si="0"/>
         <v>210.25094999999999</v>
       </c>
     </row>
@@ -6691,12 +6716,12 @@
       <c r="C17">
         <v>1203.4999999999998</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>439277.49999999994</v>
       </c>
       <c r="G17">
-        <f>F17/1000</f>
+        <f t="shared" si="0"/>
         <v>439.27749999999992</v>
       </c>
     </row>
@@ -6715,7 +6740,7 @@
         <v>119720</v>
       </c>
       <c r="G18">
-        <f>F18/1000</f>
+        <f t="shared" si="0"/>
         <v>119.72</v>
       </c>
     </row>
@@ -6734,7 +6759,7 @@
         <v>157461</v>
       </c>
       <c r="G19">
-        <f>F19/1000</f>
+        <f t="shared" si="0"/>
         <v>157.46100000000001</v>
       </c>
     </row>
@@ -6753,7 +6778,7 @@
         <v>81395</v>
       </c>
       <c r="G20">
-        <f>F20/1000</f>
+        <f t="shared" si="0"/>
         <v>81.394999999999996</v>
       </c>
     </row>
@@ -6772,7 +6797,7 @@
         <v>658376.05000000005</v>
       </c>
       <c r="G21">
-        <f>F21/1000</f>
+        <f t="shared" si="0"/>
         <v>658.37605000000008</v>
       </c>
     </row>
@@ -6791,7 +6816,7 @@
         <v>167024</v>
       </c>
       <c r="G22">
-        <f>F22/1000</f>
+        <f t="shared" si="0"/>
         <v>167.024</v>
       </c>
     </row>
@@ -6810,7 +6835,7 @@
         <v>117811.04999999999</v>
       </c>
       <c r="G23">
-        <f>F23/1000</f>
+        <f t="shared" si="0"/>
         <v>117.81104999999999</v>
       </c>
     </row>
@@ -6829,7 +6854,7 @@
         <v>702907.14500000002</v>
       </c>
       <c r="G24">
-        <f>F24/1000</f>
+        <f t="shared" si="0"/>
         <v>702.90714500000001</v>
       </c>
     </row>
@@ -6848,7 +6873,7 @@
         <v>124088.31999999999</v>
       </c>
       <c r="G25">
-        <f>F25/1000</f>
+        <f t="shared" si="0"/>
         <v>124.08832</v>
       </c>
     </row>
@@ -6867,7 +6892,7 @@
         <v>63072.000000000007</v>
       </c>
       <c r="G26">
-        <f>F26/1000</f>
+        <f t="shared" si="0"/>
         <v>63.07200000000001</v>
       </c>
     </row>
@@ -6886,7 +6911,7 @@
         <v>1503.4349999999999</v>
       </c>
       <c r="G27">
-        <f>F27/1000</f>
+        <f t="shared" si="0"/>
         <v>1.5034349999999999</v>
       </c>
     </row>
@@ -6905,7 +6930,7 @@
         <v>340034</v>
       </c>
       <c r="G28">
-        <f>F28/1000</f>
+        <f t="shared" si="0"/>
         <v>340.03399999999999</v>
       </c>
     </row>
@@ -6924,7 +6949,7 @@
         <v>449592.03500000003</v>
       </c>
       <c r="G29">
-        <f>F29/1000</f>
+        <f t="shared" si="0"/>
         <v>449.59203500000001</v>
       </c>
     </row>
@@ -6946,7 +6971,7 @@
         <v>513190</v>
       </c>
       <c r="G30">
-        <f>F30/1000</f>
+        <f t="shared" si="0"/>
         <v>513.19000000000005</v>
       </c>
     </row>
@@ -6968,7 +6993,7 @@
         <v>440555</v>
       </c>
       <c r="G31">
-        <f>F31/1000</f>
+        <f t="shared" si="0"/>
         <v>440.55500000000001</v>
       </c>
     </row>
@@ -6987,11 +7012,11 @@
         <v>49680.88</v>
       </c>
       <c r="G32">
-        <f>F32/1000</f>
+        <f t="shared" si="0"/>
         <v>49.680879999999995</v>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:7">
       <c r="A33" t="s">
         <v>36</v>
       </c>
@@ -7006,28 +7031,27 @@
         <v>24710.5</v>
       </c>
       <c r="G33">
-        <f>F33/1000</f>
+        <f t="shared" si="0"/>
         <v>24.7105</v>
       </c>
     </row>
-    <row r="34" spans="1:13">
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
         <v>41</v>
       </c>
       <c r="B34" t="s">
         <v>54</v>
       </c>
-      <c r="F34" s="5">
+      <c r="F34">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
       <c r="G34">
-        <f>F34/1000</f>
-        <v>0</v>
-      </c>
-      <c r="M34" s="5"/>
-    </row>
-    <row r="35" spans="1:13">
+        <f t="shared" ref="G34:G65" si="1">F34/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" t="s">
         <v>55</v>
       </c>
@@ -7037,17 +7061,16 @@
       <c r="E35">
         <v>32.802250000000008</v>
       </c>
-      <c r="F35" s="5">
+      <c r="F35">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>11972.821250000003</v>
       </c>
       <c r="G35">
-        <f>F35/1000</f>
+        <f t="shared" si="1"/>
         <v>11.972821250000003</v>
       </c>
-      <c r="M35" s="5"/>
-    </row>
-    <row r="36" spans="1:13">
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
         <v>25</v>
       </c>
@@ -7062,11 +7085,11 @@
         <v>60068.78</v>
       </c>
       <c r="G36">
-        <f>F36/1000</f>
+        <f t="shared" si="1"/>
         <v>60.068779999999997</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
         <v>38</v>
       </c>
@@ -7081,11 +7104,11 @@
         <v>29200</v>
       </c>
       <c r="G37">
-        <f>F37/1000</f>
+        <f t="shared" si="1"/>
         <v>29.2</v>
       </c>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
         <v>99</v>
       </c>
@@ -7095,16 +7118,16 @@
       <c r="D38">
         <v>442.8</v>
       </c>
-      <c r="F38" s="5">
+      <c r="F38">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>161622</v>
       </c>
       <c r="G38">
-        <f>F38/1000</f>
+        <f t="shared" si="1"/>
         <v>161.62200000000001</v>
       </c>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
         <v>50</v>
       </c>
@@ -7122,11 +7145,11 @@
         <v>83329.5</v>
       </c>
       <c r="G39">
-        <f>F39/1000</f>
+        <f t="shared" si="1"/>
         <v>83.329499999999996</v>
       </c>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
         <v>41</v>
       </c>
@@ -7144,11 +7167,11 @@
         <v>80300</v>
       </c>
       <c r="G40">
-        <f>F40/1000</f>
+        <f t="shared" si="1"/>
         <v>80.3</v>
       </c>
     </row>
-    <row r="41" spans="1:13">
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
         <v>54</v>
       </c>
@@ -7158,17 +7181,16 @@
       <c r="E41">
         <v>61.341321000000001</v>
       </c>
-      <c r="F41" s="5">
+      <c r="F41">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>22389.582165</v>
       </c>
       <c r="G41">
-        <f>F41/1000</f>
+        <f t="shared" si="1"/>
         <v>22.389582165</v>
       </c>
-      <c r="M41" s="5"/>
-    </row>
-    <row r="42" spans="1:13">
+    </row>
+    <row r="42" spans="1:7">
       <c r="A42" t="s">
         <v>17</v>
       </c>
@@ -7183,11 +7205,11 @@
         <v>317550</v>
       </c>
       <c r="G42">
-        <f>F42/1000</f>
+        <f t="shared" si="1"/>
         <v>317.55</v>
       </c>
     </row>
-    <row r="43" spans="1:13">
+    <row r="43" spans="1:7">
       <c r="A43" t="s">
         <v>19</v>
       </c>
@@ -7202,11 +7224,11 @@
         <v>224006.34</v>
       </c>
       <c r="G43">
-        <f>F43/1000</f>
+        <f t="shared" si="1"/>
         <v>224.00633999999999</v>
       </c>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:7">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -7221,11 +7243,11 @@
         <v>36500</v>
       </c>
       <c r="G44">
-        <f>F44/1000</f>
+        <f t="shared" si="1"/>
         <v>36.5</v>
       </c>
     </row>
-    <row r="45" spans="1:13">
+    <row r="45" spans="1:7">
       <c r="A45" t="s">
         <v>37</v>
       </c>
@@ -7240,11 +7262,11 @@
         <v>81906</v>
       </c>
       <c r="G45">
-        <f>F45/1000</f>
+        <f t="shared" si="1"/>
         <v>81.906000000000006</v>
       </c>
     </row>
-    <row r="46" spans="1:13">
+    <row r="46" spans="1:7">
       <c r="A46" t="s">
         <v>49</v>
       </c>
@@ -7262,11 +7284,11 @@
         <v>208050</v>
       </c>
       <c r="G46">
-        <f>F46/1000</f>
+        <f t="shared" si="1"/>
         <v>208.05</v>
       </c>
     </row>
-    <row r="47" spans="1:13">
+    <row r="47" spans="1:7">
       <c r="A47" t="s">
         <v>32</v>
       </c>
@@ -7281,11 +7303,11 @@
         <v>42997</v>
       </c>
       <c r="G47">
-        <f>F47/1000</f>
+        <f t="shared" si="1"/>
         <v>42.997</v>
       </c>
     </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:7">
       <c r="A48" t="s">
         <v>47</v>
       </c>
@@ -7300,7 +7322,7 @@
         <v>145489</v>
       </c>
       <c r="G48">
-        <f>F48/1000</f>
+        <f t="shared" si="1"/>
         <v>145.489</v>
       </c>
     </row>
@@ -7319,7 +7341,7 @@
         <v>19600.5</v>
       </c>
       <c r="G49">
-        <f>F49/1000</f>
+        <f t="shared" si="1"/>
         <v>19.6005</v>
       </c>
     </row>
@@ -7338,7 +7360,7 @@
         <v>28251.000000000004</v>
       </c>
       <c r="G50">
-        <f>F50/1000</f>
+        <f t="shared" si="1"/>
         <v>28.251000000000005</v>
       </c>
     </row>
@@ -7357,7 +7379,7 @@
         <v>55881.5</v>
       </c>
       <c r="G51">
-        <f>F51/1000</f>
+        <f t="shared" si="1"/>
         <v>55.881500000000003</v>
       </c>
     </row>
@@ -7376,7 +7398,7 @@
         <v>17728.05</v>
       </c>
       <c r="G52">
-        <f>F52/1000</f>
+        <f t="shared" si="1"/>
         <v>17.72805</v>
       </c>
     </row>
@@ -7395,7 +7417,7 @@
         <v>47048.5</v>
       </c>
       <c r="G53">
-        <f>F53/1000</f>
+        <f t="shared" si="1"/>
         <v>47.048499999999997</v>
       </c>
     </row>
@@ -7414,7 +7436,7 @@
         <v>18359.5</v>
       </c>
       <c r="G54">
-        <f>F54/1000</f>
+        <f t="shared" si="1"/>
         <v>18.359500000000001</v>
       </c>
     </row>
@@ -7436,7 +7458,7 @@
         <v>188194</v>
       </c>
       <c r="G55">
-        <f>F55/1000</f>
+        <f t="shared" si="1"/>
         <v>188.19399999999999</v>
       </c>
     </row>
@@ -7450,12 +7472,12 @@
       <c r="D56">
         <v>0</v>
       </c>
-      <c r="F56" s="5">
+      <c r="F56">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
       <c r="G56">
-        <f>F56/1000</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H56" t="s">
@@ -7480,7 +7502,7 @@
         <v>140525</v>
       </c>
       <c r="G57">
-        <f>F57/1000</f>
+        <f t="shared" si="1"/>
         <v>140.52500000000001</v>
       </c>
     </row>
@@ -7499,7 +7521,7 @@
         <v>419750</v>
       </c>
       <c r="G58">
-        <f>F58/1000</f>
+        <f t="shared" si="1"/>
         <v>419.75</v>
       </c>
     </row>
@@ -7518,7 +7540,7 @@
         <v>233746</v>
       </c>
       <c r="G59">
-        <f>F59/1000</f>
+        <f t="shared" si="1"/>
         <v>233.74600000000001</v>
       </c>
     </row>
@@ -7537,7 +7559,7 @@
         <v>7847.5</v>
       </c>
       <c r="G60">
-        <f>F60/1000</f>
+        <f t="shared" si="1"/>
         <v>7.8475000000000001</v>
       </c>
     </row>
@@ -7556,7 +7578,7 @@
         <v>177791.5</v>
       </c>
       <c r="G61">
-        <f>F61/1000</f>
+        <f t="shared" si="1"/>
         <v>177.79150000000001</v>
       </c>
     </row>
@@ -7578,7 +7600,7 @@
         <v>415370</v>
       </c>
       <c r="G62">
-        <f>F62/1000</f>
+        <f t="shared" si="1"/>
         <v>415.37</v>
       </c>
     </row>
@@ -7600,7 +7622,7 @@
         <v>153409.5</v>
       </c>
       <c r="G63">
-        <f>F63/1000</f>
+        <f t="shared" si="1"/>
         <v>153.40950000000001</v>
       </c>
     </row>
@@ -7619,11 +7641,11 @@
         <v>23761.499999999996</v>
       </c>
       <c r="G64">
-        <f>F64/1000</f>
+        <f t="shared" si="1"/>
         <v>23.761499999999998</v>
       </c>
     </row>
-    <row r="65" spans="1:13">
+    <row r="65" spans="1:8">
       <c r="A65" t="s">
         <v>53</v>
       </c>
@@ -7641,11 +7663,11 @@
         <v>118770.99999999999</v>
       </c>
       <c r="G65">
-        <f>F65/1000</f>
+        <f t="shared" si="1"/>
         <v>118.77099999999999</v>
       </c>
     </row>
-    <row r="66" spans="1:13">
+    <row r="66" spans="1:8">
       <c r="A66" t="s">
         <v>19</v>
       </c>
@@ -7660,11 +7682,11 @@
         <v>9749.15</v>
       </c>
       <c r="G66">
-        <f>F66/1000</f>
+        <f t="shared" ref="G66:G97" si="2">F66/1000</f>
         <v>9.7491500000000002</v>
       </c>
     </row>
-    <row r="67" spans="1:13">
+    <row r="67" spans="1:8">
       <c r="A67" t="s">
         <v>17</v>
       </c>
@@ -7674,17 +7696,16 @@
       <c r="E67">
         <v>41.973541999999995</v>
       </c>
-      <c r="F67" s="5">
+      <c r="F67">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>15320.342829999998</v>
       </c>
       <c r="G67">
-        <f>F67/1000</f>
+        <f t="shared" si="2"/>
         <v>15.320342829999998</v>
       </c>
-      <c r="M67" s="5"/>
-    </row>
-    <row r="68" spans="1:13">
+    </row>
+    <row r="68" spans="1:8">
       <c r="A68" t="s">
         <v>35</v>
       </c>
@@ -7699,11 +7720,11 @@
         <v>24673.999999999996</v>
       </c>
       <c r="G68">
-        <f>F68/1000</f>
+        <f t="shared" si="2"/>
         <v>24.673999999999996</v>
       </c>
     </row>
-    <row r="69" spans="1:13">
+    <row r="69" spans="1:8">
       <c r="A69" t="s">
         <v>41</v>
       </c>
@@ -7721,11 +7742,11 @@
         <v>43070</v>
       </c>
       <c r="G69">
-        <f>F69/1000</f>
+        <f t="shared" si="2"/>
         <v>43.07</v>
       </c>
     </row>
-    <row r="70" spans="1:13">
+    <row r="70" spans="1:8">
       <c r="A70" t="s">
         <v>54</v>
       </c>
@@ -7740,33 +7761,33 @@
         <v>24710.5</v>
       </c>
       <c r="G70">
-        <f>F70/1000</f>
+        <f t="shared" si="2"/>
         <v>24.7105</v>
       </c>
     </row>
-    <row r="71" spans="1:13">
+    <row r="71" spans="1:8">
       <c r="A71" t="s">
         <v>50</v>
       </c>
       <c r="B71" t="s">
         <v>99</v>
       </c>
-      <c r="C71">
+      <c r="D71">
         <v>442.8</v>
       </c>
-      <c r="F71" s="5">
+      <c r="F71">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>161622</v>
       </c>
       <c r="G71">
-        <f>F71/1000</f>
+        <f t="shared" si="2"/>
         <v>161.62200000000001</v>
       </c>
       <c r="H71" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="72" spans="1:13">
+    <row r="72" spans="1:8">
       <c r="A72" t="s">
         <v>34</v>
       </c>
@@ -7784,11 +7805,11 @@
         <v>5876.5000000000009</v>
       </c>
       <c r="G72">
-        <f>F72/1000</f>
+        <f t="shared" si="2"/>
         <v>5.8765000000000009</v>
       </c>
     </row>
-    <row r="73" spans="1:13">
+    <row r="73" spans="1:8">
       <c r="A73" t="s">
         <v>39</v>
       </c>
@@ -7798,17 +7819,16 @@
       <c r="E73">
         <v>255.46047452000005</v>
       </c>
-      <c r="F73" s="5">
+      <c r="F73">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>93243.073199800012</v>
       </c>
       <c r="G73">
-        <f>F73/1000</f>
+        <f t="shared" si="2"/>
         <v>93.243073199800008</v>
       </c>
-      <c r="M73" s="5"/>
-    </row>
-    <row r="74" spans="1:13">
+    </row>
+    <row r="74" spans="1:8">
       <c r="A74" t="s">
         <v>32</v>
       </c>
@@ -7826,11 +7846,11 @@
         <v>9993.6999999999989</v>
       </c>
       <c r="G74">
-        <f>F74/1000</f>
+        <f t="shared" si="2"/>
         <v>9.9936999999999987</v>
       </c>
     </row>
-    <row r="75" spans="1:13">
+    <row r="75" spans="1:8">
       <c r="A75" t="s">
         <v>17</v>
       </c>
@@ -7845,11 +7865,11 @@
         <v>120888</v>
       </c>
       <c r="G75">
-        <f>F75/1000</f>
+        <f t="shared" si="2"/>
         <v>120.88800000000001</v>
       </c>
     </row>
-    <row r="76" spans="1:13">
+    <row r="76" spans="1:8">
       <c r="A76" t="s">
         <v>19</v>
       </c>
@@ -7864,11 +7884,11 @@
         <v>594330.59500000009</v>
       </c>
       <c r="G76">
-        <f>F76/1000</f>
+        <f t="shared" si="2"/>
         <v>594.33059500000013</v>
       </c>
     </row>
-    <row r="77" spans="1:13">
+    <row r="77" spans="1:8">
       <c r="A77" t="s">
         <v>49</v>
       </c>
@@ -7878,16 +7898,16 @@
       <c r="D77">
         <v>963.6</v>
       </c>
-      <c r="F77" s="5">
+      <c r="F77">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>351714</v>
       </c>
       <c r="G77">
-        <f>F77/1000</f>
+        <f t="shared" si="2"/>
         <v>351.714</v>
       </c>
     </row>
-    <row r="78" spans="1:13">
+    <row r="78" spans="1:8">
       <c r="A78" t="s">
         <v>11</v>
       </c>
@@ -7897,16 +7917,16 @@
       <c r="C78">
         <v>494.4</v>
       </c>
-      <c r="F78" s="5">
+      <c r="F78">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>180456</v>
       </c>
       <c r="G78">
-        <f>F78/1000</f>
+        <f t="shared" si="2"/>
         <v>180.45599999999999</v>
       </c>
     </row>
-    <row r="79" spans="1:13">
+    <row r="79" spans="1:8">
       <c r="A79" t="s">
         <v>19</v>
       </c>
@@ -7921,11 +7941,11 @@
         <v>85227.5</v>
       </c>
       <c r="G79">
-        <f>F79/1000</f>
+        <f t="shared" si="2"/>
         <v>85.227500000000006</v>
       </c>
     </row>
-    <row r="80" spans="1:13">
+    <row r="80" spans="1:8">
       <c r="A80" t="s">
         <v>28</v>
       </c>
@@ -7940,7 +7960,7 @@
         <v>10220</v>
       </c>
       <c r="G80">
-        <f>F80/1000</f>
+        <f t="shared" si="2"/>
         <v>10.220000000000001</v>
       </c>
     </row>
@@ -7954,7 +7974,7 @@
       <c r="C81">
         <v>135.6</v>
       </c>
-      <c r="D81" s="6">
+      <c r="D81">
         <v>135.6</v>
       </c>
       <c r="F81">
@@ -7962,7 +7982,7 @@
         <v>49494</v>
       </c>
       <c r="G81">
-        <f>F81/1000</f>
+        <f t="shared" si="2"/>
         <v>49.494</v>
       </c>
     </row>
@@ -7984,7 +8004,7 @@
         <v>439277.49999999994</v>
       </c>
       <c r="G82">
-        <f>F82/1000</f>
+        <f t="shared" si="2"/>
         <v>439.27749999999992</v>
       </c>
     </row>
@@ -8003,7 +8023,7 @@
         <v>52560</v>
       </c>
       <c r="G83">
-        <f>F83/1000</f>
+        <f t="shared" si="2"/>
         <v>52.56</v>
       </c>
     </row>
@@ -8022,7 +8042,7 @@
         <v>28287.5</v>
       </c>
       <c r="G84">
-        <f>F84/1000</f>
+        <f t="shared" si="2"/>
         <v>28.287500000000001</v>
       </c>
     </row>
@@ -8041,7 +8061,7 @@
         <v>54074.75</v>
       </c>
       <c r="G85">
-        <f>F85/1000</f>
+        <f t="shared" si="2"/>
         <v>54.074750000000002</v>
       </c>
     </row>
@@ -8063,7 +8083,7 @@
         <v>73584</v>
       </c>
       <c r="G86">
-        <f>F86/1000</f>
+        <f t="shared" si="2"/>
         <v>73.584000000000003</v>
       </c>
     </row>
@@ -8082,7 +8102,7 @@
         <v>803.00000000000011</v>
       </c>
       <c r="G87">
-        <f>F87/1000</f>
+        <f t="shared" si="2"/>
         <v>0.80300000000000016</v>
       </c>
     </row>
@@ -8104,7 +8124,7 @@
         <v>51830</v>
       </c>
       <c r="G88">
-        <f>F88/1000</f>
+        <f t="shared" si="2"/>
         <v>51.83</v>
       </c>
     </row>
@@ -8126,7 +8146,7 @@
         <v>63546.5</v>
       </c>
       <c r="G89">
-        <f>F89/1000</f>
+        <f t="shared" si="2"/>
         <v>63.546500000000002</v>
       </c>
     </row>
@@ -8145,7 +8165,7 @@
         <v>41683</v>
       </c>
       <c r="G90">
-        <f>F90/1000</f>
+        <f t="shared" si="2"/>
         <v>41.683</v>
       </c>
     </row>
@@ -8167,7 +8187,7 @@
         <v>31025</v>
       </c>
       <c r="G91">
-        <f>F91/1000</f>
+        <f t="shared" si="2"/>
         <v>31.024999999999999</v>
       </c>
     </row>
@@ -8181,12 +8201,12 @@
       <c r="E92">
         <v>30</v>
       </c>
-      <c r="F92" s="5">
+      <c r="F92">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>10950</v>
       </c>
       <c r="G92">
-        <f>F92/1000</f>
+        <f t="shared" si="2"/>
         <v>10.95</v>
       </c>
       <c r="H92" t="s">
@@ -8208,7 +8228,7 @@
         <v>41062.5</v>
       </c>
       <c r="G93">
-        <f>F93/1000</f>
+        <f t="shared" si="2"/>
         <v>41.0625</v>
       </c>
     </row>
@@ -8227,7 +8247,7 @@
         <v>10402.5</v>
       </c>
       <c r="G94">
-        <f>F94/1000</f>
+        <f t="shared" si="2"/>
         <v>10.4025</v>
       </c>
     </row>
@@ -8246,7 +8266,7 @@
         <v>2810.5</v>
       </c>
       <c r="G95">
-        <f>F95/1000</f>
+        <f t="shared" si="2"/>
         <v>2.8105000000000002</v>
       </c>
     </row>
@@ -8265,11 +8285,11 @@
         <v>89972.5</v>
       </c>
       <c r="G96">
-        <f>F96/1000</f>
+        <f t="shared" si="2"/>
         <v>89.972499999999997</v>
       </c>
     </row>
-    <row r="97" spans="1:13">
+    <row r="97" spans="1:8">
       <c r="A97" t="s">
         <v>28</v>
       </c>
@@ -8284,11 +8304,11 @@
         <v>454936.00000000006</v>
       </c>
       <c r="G97">
-        <f>F97/1000</f>
+        <f t="shared" si="2"/>
         <v>454.93600000000004</v>
       </c>
     </row>
-    <row r="98" spans="1:13">
+    <row r="98" spans="1:8">
       <c r="A98" t="s">
         <v>30</v>
       </c>
@@ -8303,11 +8323,11 @@
         <v>18572.295000000002</v>
       </c>
       <c r="G98">
-        <f>F98/1000</f>
+        <f t="shared" ref="G98:G129" si="3">F98/1000</f>
         <v>18.572295</v>
       </c>
     </row>
-    <row r="99" spans="1:13">
+    <row r="99" spans="1:8">
       <c r="A99" t="s">
         <v>39</v>
       </c>
@@ -8325,11 +8345,11 @@
         <v>740220</v>
       </c>
       <c r="G99">
-        <f>F99/1000</f>
+        <f t="shared" si="3"/>
         <v>740.22</v>
       </c>
     </row>
-    <row r="100" spans="1:13">
+    <row r="100" spans="1:8">
       <c r="A100" t="s">
         <v>50</v>
       </c>
@@ -8339,19 +8359,19 @@
       <c r="C100">
         <v>1138.0999999999999</v>
       </c>
-      <c r="F100" s="5">
+      <c r="F100">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>415406.49999999994</v>
       </c>
       <c r="G100">
-        <f>F100/1000</f>
+        <f t="shared" si="3"/>
         <v>415.40649999999994</v>
       </c>
       <c r="H100" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="101" spans="1:13">
+    <row r="101" spans="1:8">
       <c r="A101" t="s">
         <v>32</v>
       </c>
@@ -8369,11 +8389,11 @@
         <v>181463.40000000002</v>
       </c>
       <c r="G101">
-        <f>F101/1000</f>
+        <f t="shared" si="3"/>
         <v>181.46340000000004</v>
       </c>
     </row>
-    <row r="102" spans="1:13">
+    <row r="102" spans="1:8">
       <c r="A102" t="s">
         <v>41</v>
       </c>
@@ -8383,20 +8403,19 @@
       <c r="E102">
         <v>958.9</v>
       </c>
-      <c r="F102" s="5">
+      <c r="F102">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>349998.5</v>
       </c>
       <c r="G102">
-        <f>F102/1000</f>
+        <f t="shared" si="3"/>
         <v>349.99849999999998</v>
       </c>
       <c r="H102" t="s">
         <v>144</v>
       </c>
-      <c r="M102" s="5"/>
-    </row>
-    <row r="103" spans="1:13">
+    </row>
+    <row r="103" spans="1:8">
       <c r="A103" t="s">
         <v>97</v>
       </c>
@@ -8406,19 +8425,19 @@
       <c r="D103">
         <v>349.9</v>
       </c>
-      <c r="F103" s="5">
+      <c r="F103">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>127713.49999999999</v>
       </c>
       <c r="G103">
-        <f>F103/1000</f>
+        <f t="shared" si="3"/>
         <v>127.71349999999998</v>
       </c>
       <c r="H103" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="104" spans="1:13">
+    <row r="104" spans="1:8">
       <c r="A104" t="s">
         <v>29</v>
       </c>
@@ -8436,11 +8455,11 @@
         <v>102492</v>
       </c>
       <c r="G104">
-        <f>F104/1000</f>
+        <f t="shared" si="3"/>
         <v>102.492</v>
       </c>
     </row>
-    <row r="105" spans="1:13">
+    <row r="105" spans="1:8">
       <c r="A105" t="s">
         <v>34</v>
       </c>
@@ -8455,11 +8474,11 @@
         <v>44603</v>
       </c>
       <c r="G105">
-        <f>F105/1000</f>
+        <f t="shared" si="3"/>
         <v>44.603000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:13">
+    <row r="106" spans="1:8">
       <c r="A106" t="s">
         <v>41</v>
       </c>
@@ -8469,16 +8488,16 @@
       <c r="E106">
         <v>5459.5088498999994</v>
       </c>
-      <c r="F106" s="5">
+      <c r="F106">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>1992720.7302134999</v>
       </c>
       <c r="G106">
-        <f>F106/1000</f>
+        <f t="shared" si="3"/>
         <v>1992.7207302134998</v>
       </c>
     </row>
-    <row r="107" spans="1:13">
+    <row r="107" spans="1:8">
       <c r="A107" t="s">
         <v>40</v>
       </c>
@@ -8488,17 +8507,16 @@
       <c r="E107">
         <v>80.846503979999994</v>
       </c>
-      <c r="F107" s="5">
+      <c r="F107">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>29508.973952699998</v>
       </c>
       <c r="G107">
-        <f>F107/1000</f>
+        <f t="shared" si="3"/>
         <v>29.5089739527</v>
       </c>
-      <c r="M107" s="5"/>
-    </row>
-    <row r="108" spans="1:13">
+    </row>
+    <row r="108" spans="1:8">
       <c r="A108" t="s">
         <v>53</v>
       </c>
@@ -8508,17 +8526,16 @@
       <c r="E108">
         <v>35.53171072</v>
       </c>
-      <c r="F108" s="5">
+      <c r="F108">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>12969.074412800001</v>
       </c>
       <c r="G108">
-        <f>F108/1000</f>
+        <f t="shared" si="3"/>
         <v>12.969074412800001</v>
       </c>
-      <c r="M108" s="5"/>
-    </row>
-    <row r="109" spans="1:13">
+    </row>
+    <row r="109" spans="1:8">
       <c r="A109" t="s">
         <v>17</v>
       </c>
@@ -8536,11 +8553,11 @@
         <v>95301.500000000015</v>
       </c>
       <c r="G109">
-        <f>F109/1000</f>
+        <f t="shared" si="3"/>
         <v>95.301500000000019</v>
       </c>
     </row>
-    <row r="110" spans="1:13">
+    <row r="110" spans="1:8">
       <c r="A110" t="s">
         <v>49</v>
       </c>
@@ -8558,11 +8575,11 @@
         <v>513190</v>
       </c>
       <c r="G110">
-        <f>F110/1000</f>
+        <f t="shared" si="3"/>
         <v>513.19000000000005</v>
       </c>
     </row>
-    <row r="111" spans="1:13">
+    <row r="111" spans="1:8">
       <c r="A111" t="s">
         <v>18</v>
       </c>
@@ -8572,15 +8589,14 @@
       <c r="C111">
         <v>494.4</v>
       </c>
-      <c r="F111" s="5">
+      <c r="F111">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>180456</v>
       </c>
       <c r="G111">
-        <f>F111/1000</f>
+        <f t="shared" si="3"/>
         <v>180.45599999999999</v>
       </c>
-      <c r="M111" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
@@ -8592,6 +8608,2220 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67CAB708-6819-43AD-B444-2B653F840206}">
+  <dimension ref="A1:H111"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="3" max="3" width="20.453125" customWidth="1"/>
+    <col min="4" max="4" width="17.26953125" customWidth="1"/>
+    <col min="5" max="5" width="16.1796875" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" customWidth="1"/>
+    <col min="11" max="12" width="10.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2">
+        <v>487.1</v>
+      </c>
+      <c r="F2">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>177791.5</v>
+      </c>
+      <c r="G2">
+        <f t="shared" ref="G2:G65" si="0">F2/1000</f>
+        <v>177.79150000000001</v>
+      </c>
+      <c r="H2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <v>344.24799999999993</v>
+      </c>
+      <c r="F3">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>125650.51999999997</v>
+      </c>
+      <c r="G3">
+        <f t="shared" si="0"/>
+        <v>125.65051999999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4">
+        <v>193.5</v>
+      </c>
+      <c r="F4">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>70627.5</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="0"/>
+        <v>70.627499999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5">
+        <v>1570.4</v>
+      </c>
+      <c r="F5">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>573196</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="0"/>
+        <v>573.19600000000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6">
+        <v>17.98</v>
+      </c>
+      <c r="F6">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>6562.7</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>6.5626999999999995</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7">
+        <v>205.9</v>
+      </c>
+      <c r="F7">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>75153.5</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="0"/>
+        <v>75.153499999999994</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8">
+        <v>1397.2</v>
+      </c>
+      <c r="F8">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>509978</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="0"/>
+        <v>509.97800000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>396.15000000000003</v>
+      </c>
+      <c r="F9">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>144594.75</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="0"/>
+        <v>144.59475</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10">
+        <v>270</v>
+      </c>
+      <c r="F10">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>98550</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="0"/>
+        <v>98.55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11">
+        <v>488</v>
+      </c>
+      <c r="D11">
+        <v>453.2</v>
+      </c>
+      <c r="F11">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>165418</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="0"/>
+        <v>165.41800000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E12">
+        <v>41.973541999999995</v>
+      </c>
+      <c r="F12">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>15320.342829999998</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="0"/>
+        <v>15.320342829999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13">
+        <v>335.26</v>
+      </c>
+      <c r="F13">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>122369.9</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="0"/>
+        <v>122.3699</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14">
+        <v>64.819999999999993</v>
+      </c>
+      <c r="F14">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>23659.3</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="0"/>
+        <v>23.659299999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15">
+        <v>805.75000000000011</v>
+      </c>
+      <c r="F15">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>294098.75000000006</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="0"/>
+        <v>294.09875000000005</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16">
+        <v>576.03</v>
+      </c>
+      <c r="F16">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>210250.94999999998</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="0"/>
+        <v>210.25094999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17">
+        <v>1203.4999999999998</v>
+      </c>
+      <c r="F17">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>439277.49999999994</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="0"/>
+        <v>439.27749999999992</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18">
+        <v>328</v>
+      </c>
+      <c r="F18">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>119720</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="0"/>
+        <v>119.72</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19">
+        <v>431.4</v>
+      </c>
+      <c r="F19">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>157461</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="0"/>
+        <v>157.46100000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20">
+        <v>223</v>
+      </c>
+      <c r="F20">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>81395</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="0"/>
+        <v>81.394999999999996</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21">
+        <v>1803.77</v>
+      </c>
+      <c r="F21">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>658376.05000000005</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="0"/>
+        <v>658.37605000000008</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22">
+        <v>457.6</v>
+      </c>
+      <c r="F22">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>167024</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="0"/>
+        <v>167.024</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23">
+        <v>322.77</v>
+      </c>
+      <c r="F23">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>117811.04999999999</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="0"/>
+        <v>117.81104999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24">
+        <v>1925.7729999999999</v>
+      </c>
+      <c r="F24">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>702907.14500000002</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="0"/>
+        <v>702.90714500000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25">
+        <v>339.96799999999996</v>
+      </c>
+      <c r="F25">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>124088.31999999999</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="0"/>
+        <v>124.08832</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26">
+        <v>172.8</v>
+      </c>
+      <c r="F26">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>63072.000000000007</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="0"/>
+        <v>63.07200000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27">
+        <v>4.1189999999999998</v>
+      </c>
+      <c r="F27">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>1503.4349999999999</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="0"/>
+        <v>1.5034349999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28">
+        <v>931.6</v>
+      </c>
+      <c r="F28">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>340034</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="0"/>
+        <v>340.03399999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29">
+        <v>1231.759</v>
+      </c>
+      <c r="F29">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>449592.03500000003</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="0"/>
+        <v>449.59203500000001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30" t="s">
+        <v>19</v>
+      </c>
+      <c r="D30">
+        <v>0</v>
+      </c>
+      <c r="F30">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" t="s">
+        <v>49</v>
+      </c>
+      <c r="B31" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31">
+        <v>2210.5639999999999</v>
+      </c>
+      <c r="D31">
+        <v>1226</v>
+      </c>
+      <c r="F31">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>447490</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="0"/>
+        <v>447.49</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" t="s">
+        <v>19</v>
+      </c>
+      <c r="B32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32">
+        <v>136.11199999999999</v>
+      </c>
+      <c r="F32">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>49680.88</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="0"/>
+        <v>49.680879999999995</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" t="s">
+        <v>36</v>
+      </c>
+      <c r="B33" t="s">
+        <v>54</v>
+      </c>
+      <c r="E33">
+        <v>67.7</v>
+      </c>
+      <c r="F33">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>24710.5</v>
+      </c>
+      <c r="G33">
+        <f t="shared" si="0"/>
+        <v>24.7105</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34" t="s">
+        <v>54</v>
+      </c>
+      <c r="F34">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G34">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" t="s">
+        <v>55</v>
+      </c>
+      <c r="B35" t="s">
+        <v>54</v>
+      </c>
+      <c r="E35">
+        <v>32.802250000000008</v>
+      </c>
+      <c r="F35">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>11972.821250000003</v>
+      </c>
+      <c r="G35">
+        <f t="shared" si="0"/>
+        <v>11.972821250000003</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" t="s">
+        <v>25</v>
+      </c>
+      <c r="B36" t="s">
+        <v>37</v>
+      </c>
+      <c r="C36">
+        <v>164.572</v>
+      </c>
+      <c r="F36">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>60068.78</v>
+      </c>
+      <c r="G36">
+        <f t="shared" si="0"/>
+        <v>60.068779999999997</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" t="s">
+        <v>38</v>
+      </c>
+      <c r="B37" t="s">
+        <v>37</v>
+      </c>
+      <c r="C37">
+        <v>80</v>
+      </c>
+      <c r="F37">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>29200</v>
+      </c>
+      <c r="G37">
+        <f t="shared" si="0"/>
+        <v>29.2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" t="s">
+        <v>99</v>
+      </c>
+      <c r="B38" t="s">
+        <v>37</v>
+      </c>
+      <c r="D38">
+        <v>31.92</v>
+      </c>
+      <c r="F38">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>11650.800000000001</v>
+      </c>
+      <c r="G38">
+        <f t="shared" si="0"/>
+        <v>11.6508</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39" t="s">
+        <v>37</v>
+      </c>
+      <c r="C39">
+        <v>731.7</v>
+      </c>
+      <c r="D39">
+        <v>337.1</v>
+      </c>
+      <c r="F39">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>123041.50000000001</v>
+      </c>
+      <c r="G39">
+        <f t="shared" si="0"/>
+        <v>123.04150000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" t="s">
+        <v>41</v>
+      </c>
+      <c r="B40" t="s">
+        <v>55</v>
+      </c>
+      <c r="D40">
+        <v>0</v>
+      </c>
+      <c r="F40">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" t="s">
+        <v>55</v>
+      </c>
+      <c r="E41">
+        <v>61.341321000000001</v>
+      </c>
+      <c r="F41">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>22389.582165</v>
+      </c>
+      <c r="G41">
+        <f t="shared" si="0"/>
+        <v>22.389582165</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" t="s">
+        <v>25</v>
+      </c>
+      <c r="C42">
+        <v>870</v>
+      </c>
+      <c r="F42">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>317550</v>
+      </c>
+      <c r="G42">
+        <f t="shared" si="0"/>
+        <v>317.55</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" t="s">
+        <v>19</v>
+      </c>
+      <c r="B43" t="s">
+        <v>25</v>
+      </c>
+      <c r="C43">
+        <v>613.71600000000001</v>
+      </c>
+      <c r="F43">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>224006.34</v>
+      </c>
+      <c r="G43">
+        <f t="shared" si="0"/>
+        <v>224.00633999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" t="s">
+        <v>22</v>
+      </c>
+      <c r="B44" t="s">
+        <v>25</v>
+      </c>
+      <c r="C44">
+        <v>100</v>
+      </c>
+      <c r="F44">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>36500</v>
+      </c>
+      <c r="G44">
+        <f t="shared" si="0"/>
+        <v>36.5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" t="s">
+        <v>37</v>
+      </c>
+      <c r="B45" t="s">
+        <v>25</v>
+      </c>
+      <c r="C45">
+        <v>224.4</v>
+      </c>
+      <c r="F45">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>81906</v>
+      </c>
+      <c r="G45">
+        <f t="shared" si="0"/>
+        <v>81.906000000000006</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46" t="s">
+        <v>49</v>
+      </c>
+      <c r="B46" t="s">
+        <v>25</v>
+      </c>
+      <c r="C46">
+        <v>570</v>
+      </c>
+      <c r="D46">
+        <v>568.5</v>
+      </c>
+      <c r="F46">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>207502.5</v>
+      </c>
+      <c r="G46">
+        <f t="shared" si="0"/>
+        <v>207.5025</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
+      <c r="A47" t="s">
+        <v>32</v>
+      </c>
+      <c r="B47" t="s">
+        <v>33</v>
+      </c>
+      <c r="C47">
+        <v>117.8</v>
+      </c>
+      <c r="F47">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>42997</v>
+      </c>
+      <c r="G47">
+        <f t="shared" si="0"/>
+        <v>42.997</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" t="s">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>33</v>
+      </c>
+      <c r="C48">
+        <v>398.6</v>
+      </c>
+      <c r="F48">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>145489</v>
+      </c>
+      <c r="G48">
+        <f t="shared" si="0"/>
+        <v>145.489</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" t="s">
+        <v>23</v>
+      </c>
+      <c r="B49" t="s">
+        <v>24</v>
+      </c>
+      <c r="C49">
+        <v>53.7</v>
+      </c>
+      <c r="F49">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>19600.5</v>
+      </c>
+      <c r="G49">
+        <f t="shared" si="0"/>
+        <v>19.6005</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50" t="s">
+        <v>30</v>
+      </c>
+      <c r="B50" t="s">
+        <v>24</v>
+      </c>
+      <c r="C50">
+        <v>77.400000000000006</v>
+      </c>
+      <c r="F50">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>28251.000000000004</v>
+      </c>
+      <c r="G50">
+        <f t="shared" si="0"/>
+        <v>28.251000000000005</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
+      <c r="A51" t="s">
+        <v>20</v>
+      </c>
+      <c r="B51" t="s">
+        <v>30</v>
+      </c>
+      <c r="C51">
+        <v>153.1</v>
+      </c>
+      <c r="F51">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>55881.5</v>
+      </c>
+      <c r="G51">
+        <f t="shared" si="0"/>
+        <v>55.881500000000003</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
+      <c r="A52" t="s">
+        <v>24</v>
+      </c>
+      <c r="B52" t="s">
+        <v>30</v>
+      </c>
+      <c r="C52">
+        <v>48.57</v>
+      </c>
+      <c r="F52">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>17728.05</v>
+      </c>
+      <c r="G52">
+        <f t="shared" si="0"/>
+        <v>17.72805</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
+      <c r="A53" t="s">
+        <v>29</v>
+      </c>
+      <c r="B53" t="s">
+        <v>30</v>
+      </c>
+      <c r="C53">
+        <v>128.9</v>
+      </c>
+      <c r="F53">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>47048.5</v>
+      </c>
+      <c r="G53">
+        <f t="shared" si="0"/>
+        <v>47.048499999999997</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54" t="s">
+        <v>34</v>
+      </c>
+      <c r="B54" t="s">
+        <v>30</v>
+      </c>
+      <c r="C54">
+        <v>50.3</v>
+      </c>
+      <c r="F54">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>18359.5</v>
+      </c>
+      <c r="G54">
+        <f t="shared" si="0"/>
+        <v>18.359500000000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
+      <c r="A55" t="s">
+        <v>39</v>
+      </c>
+      <c r="B55" t="s">
+        <v>30</v>
+      </c>
+      <c r="C55">
+        <v>515.6</v>
+      </c>
+      <c r="D55">
+        <v>84.77</v>
+      </c>
+      <c r="F55">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>30941.05</v>
+      </c>
+      <c r="G55">
+        <f t="shared" si="0"/>
+        <v>30.941050000000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
+      <c r="A56" t="s">
+        <v>31</v>
+      </c>
+      <c r="B56" t="s">
+        <v>30</v>
+      </c>
+      <c r="D56">
+        <v>245.8</v>
+      </c>
+      <c r="F56">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>89717</v>
+      </c>
+      <c r="G56">
+        <f t="shared" si="0"/>
+        <v>89.716999999999999</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
+      <c r="A57" t="s">
+        <v>11</v>
+      </c>
+      <c r="B57" t="s">
+        <v>44</v>
+      </c>
+      <c r="C57">
+        <v>386.9</v>
+      </c>
+      <c r="D57">
+        <v>385</v>
+      </c>
+      <c r="F57">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>140525</v>
+      </c>
+      <c r="G57">
+        <f t="shared" si="0"/>
+        <v>140.52500000000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
+      <c r="A58" t="s">
+        <v>20</v>
+      </c>
+      <c r="B58" t="s">
+        <v>21</v>
+      </c>
+      <c r="C58">
+        <v>1150</v>
+      </c>
+      <c r="F58">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>419750</v>
+      </c>
+      <c r="G58">
+        <f t="shared" si="0"/>
+        <v>419.75</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
+      <c r="A59" t="s">
+        <v>22</v>
+      </c>
+      <c r="B59" t="s">
+        <v>21</v>
+      </c>
+      <c r="C59">
+        <v>640.4</v>
+      </c>
+      <c r="F59">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>233746</v>
+      </c>
+      <c r="G59">
+        <f t="shared" si="0"/>
+        <v>233.74600000000001</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
+      <c r="A60" t="s">
+        <v>23</v>
+      </c>
+      <c r="B60" t="s">
+        <v>21</v>
+      </c>
+      <c r="C60">
+        <v>21.5</v>
+      </c>
+      <c r="F60">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>7847.5</v>
+      </c>
+      <c r="G60">
+        <f t="shared" si="0"/>
+        <v>7.8475000000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
+      <c r="A61" t="s">
+        <v>42</v>
+      </c>
+      <c r="B61" t="s">
+        <v>21</v>
+      </c>
+      <c r="C61">
+        <v>487.1</v>
+      </c>
+      <c r="F61">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>177791.5</v>
+      </c>
+      <c r="G61">
+        <f t="shared" si="0"/>
+        <v>177.79150000000001</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
+      <c r="A62" t="s">
+        <v>51</v>
+      </c>
+      <c r="B62" t="s">
+        <v>21</v>
+      </c>
+      <c r="C62">
+        <v>1138.0999999999999</v>
+      </c>
+      <c r="D62">
+        <v>1154</v>
+      </c>
+      <c r="F62">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>415406.49999999994</v>
+      </c>
+      <c r="G62">
+        <f t="shared" si="0"/>
+        <v>415.40649999999994</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
+      <c r="A63" t="s">
+        <v>52</v>
+      </c>
+      <c r="B63" t="s">
+        <v>21</v>
+      </c>
+      <c r="C63">
+        <v>475.8</v>
+      </c>
+      <c r="D63">
+        <v>493.7</v>
+      </c>
+      <c r="F63">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>173667</v>
+      </c>
+      <c r="G63">
+        <f t="shared" si="0"/>
+        <v>173.667</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
+      <c r="A64" t="s">
+        <v>36</v>
+      </c>
+      <c r="B64" t="s">
+        <v>35</v>
+      </c>
+      <c r="C64">
+        <v>65.099999999999994</v>
+      </c>
+      <c r="F64">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>23761.499999999996</v>
+      </c>
+      <c r="G64">
+        <f t="shared" si="0"/>
+        <v>23.761499999999998</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" t="s">
+        <v>53</v>
+      </c>
+      <c r="B65" t="s">
+        <v>35</v>
+      </c>
+      <c r="C65">
+        <v>325.39999999999998</v>
+      </c>
+      <c r="D65">
+        <v>325.39999999999998</v>
+      </c>
+      <c r="F65">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>118770.99999999999</v>
+      </c>
+      <c r="G65">
+        <f t="shared" si="0"/>
+        <v>118.77099999999999</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" t="s">
+        <v>19</v>
+      </c>
+      <c r="B66" t="s">
+        <v>43</v>
+      </c>
+      <c r="C66">
+        <v>26.71</v>
+      </c>
+      <c r="F66">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>9749.15</v>
+      </c>
+      <c r="G66">
+        <f t="shared" ref="G66:G111" si="1">F66/1000</f>
+        <v>9.7491500000000002</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
+      <c r="A67" t="s">
+        <v>17</v>
+      </c>
+      <c r="B67" t="s">
+        <v>43</v>
+      </c>
+      <c r="E67">
+        <v>41.973541999999995</v>
+      </c>
+      <c r="F67">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>15320.342829999998</v>
+      </c>
+      <c r="G67">
+        <f t="shared" si="1"/>
+        <v>15.320342829999998</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68" t="s">
+        <v>35</v>
+      </c>
+      <c r="B68" t="s">
+        <v>36</v>
+      </c>
+      <c r="C68">
+        <v>67.599999999999994</v>
+      </c>
+      <c r="F68">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>24673.999999999996</v>
+      </c>
+      <c r="G68">
+        <f t="shared" si="1"/>
+        <v>24.673999999999996</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69" t="s">
+        <v>41</v>
+      </c>
+      <c r="B69" t="s">
+        <v>36</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G69">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70" t="s">
+        <v>54</v>
+      </c>
+      <c r="B70" t="s">
+        <v>36</v>
+      </c>
+      <c r="E70">
+        <v>67.7</v>
+      </c>
+      <c r="F70">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>24710.5</v>
+      </c>
+      <c r="G70">
+        <f t="shared" si="1"/>
+        <v>24.7105</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71" t="s">
+        <v>50</v>
+      </c>
+      <c r="B71" t="s">
+        <v>99</v>
+      </c>
+      <c r="D71">
+        <v>31.92</v>
+      </c>
+      <c r="F71">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>11650.800000000001</v>
+      </c>
+      <c r="G71">
+        <f t="shared" si="1"/>
+        <v>11.6508</v>
+      </c>
+      <c r="H71" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72" t="s">
+        <v>34</v>
+      </c>
+      <c r="B72" t="s">
+        <v>40</v>
+      </c>
+      <c r="C72">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="E72">
+        <v>55.7</v>
+      </c>
+      <c r="F72">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>5876.5000000000009</v>
+      </c>
+      <c r="G72">
+        <f t="shared" si="1"/>
+        <v>5.8765000000000009</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73" t="s">
+        <v>39</v>
+      </c>
+      <c r="B73" t="s">
+        <v>40</v>
+      </c>
+      <c r="E73">
+        <v>255.46047452000005</v>
+      </c>
+      <c r="F73">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>93243.073199800012</v>
+      </c>
+      <c r="G73">
+        <f t="shared" si="1"/>
+        <v>93.243073199800008</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8">
+      <c r="A74" t="s">
+        <v>32</v>
+      </c>
+      <c r="B74" t="s">
+        <v>46</v>
+      </c>
+      <c r="C74">
+        <v>27.38</v>
+      </c>
+      <c r="D74">
+        <v>33.28</v>
+      </c>
+      <c r="F74">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>9993.6999999999989</v>
+      </c>
+      <c r="G74">
+        <f t="shared" si="1"/>
+        <v>9.9936999999999987</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75" t="s">
+        <v>17</v>
+      </c>
+      <c r="B75" t="s">
+        <v>18</v>
+      </c>
+      <c r="C75">
+        <v>331.2</v>
+      </c>
+      <c r="F75">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>120888</v>
+      </c>
+      <c r="G75">
+        <f t="shared" si="1"/>
+        <v>120.88800000000001</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
+      <c r="A76" t="s">
+        <v>19</v>
+      </c>
+      <c r="B76" t="s">
+        <v>18</v>
+      </c>
+      <c r="C76">
+        <v>1628.3030000000001</v>
+      </c>
+      <c r="F76">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>594330.59500000009</v>
+      </c>
+      <c r="G76">
+        <f t="shared" si="1"/>
+        <v>594.33059500000013</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
+      <c r="A77" t="s">
+        <v>49</v>
+      </c>
+      <c r="B77" t="s">
+        <v>18</v>
+      </c>
+      <c r="D77">
+        <v>963.6</v>
+      </c>
+      <c r="F77">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>351714</v>
+      </c>
+      <c r="G77">
+        <f t="shared" si="1"/>
+        <v>351.714</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
+      <c r="A78" t="s">
+        <v>11</v>
+      </c>
+      <c r="B78" t="s">
+        <v>18</v>
+      </c>
+      <c r="C78">
+        <v>494.4</v>
+      </c>
+      <c r="F78">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>180456</v>
+      </c>
+      <c r="G78">
+        <f t="shared" si="1"/>
+        <v>180.45599999999999</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8">
+      <c r="A79" t="s">
+        <v>19</v>
+      </c>
+      <c r="B79" t="s">
+        <v>27</v>
+      </c>
+      <c r="C79">
+        <v>233.5</v>
+      </c>
+      <c r="F79">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>85227.5</v>
+      </c>
+      <c r="G79">
+        <f t="shared" si="1"/>
+        <v>85.227500000000006</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8">
+      <c r="A80" t="s">
+        <v>28</v>
+      </c>
+      <c r="B80" t="s">
+        <v>27</v>
+      </c>
+      <c r="C80">
+        <v>28</v>
+      </c>
+      <c r="F80">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>10220</v>
+      </c>
+      <c r="G80">
+        <f t="shared" si="1"/>
+        <v>10.220000000000001</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8">
+      <c r="A81" t="s">
+        <v>39</v>
+      </c>
+      <c r="B81" t="s">
+        <v>27</v>
+      </c>
+      <c r="C81">
+        <v>135.6</v>
+      </c>
+      <c r="D81">
+        <v>135.6</v>
+      </c>
+      <c r="F81">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>49494</v>
+      </c>
+      <c r="G81">
+        <f t="shared" si="1"/>
+        <v>49.494</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8">
+      <c r="A82" t="s">
+        <v>53</v>
+      </c>
+      <c r="B82" t="s">
+        <v>27</v>
+      </c>
+      <c r="C82">
+        <v>1203.4999999999998</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+      <c r="F82">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G82">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8">
+      <c r="A83" t="s">
+        <v>37</v>
+      </c>
+      <c r="B83" t="s">
+        <v>38</v>
+      </c>
+      <c r="C83">
+        <v>144</v>
+      </c>
+      <c r="F83">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>52560</v>
+      </c>
+      <c r="G83">
+        <f t="shared" si="1"/>
+        <v>52.56</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8">
+      <c r="A84" t="s">
+        <v>30</v>
+      </c>
+      <c r="B84" t="s">
+        <v>34</v>
+      </c>
+      <c r="C84">
+        <v>77.5</v>
+      </c>
+      <c r="F84">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>28287.5</v>
+      </c>
+      <c r="G84">
+        <f t="shared" si="1"/>
+        <v>28.287500000000001</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8">
+      <c r="A85" t="s">
+        <v>32</v>
+      </c>
+      <c r="B85" t="s">
+        <v>34</v>
+      </c>
+      <c r="C85">
+        <v>148.15</v>
+      </c>
+      <c r="F85">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>54074.75</v>
+      </c>
+      <c r="G85">
+        <f t="shared" si="1"/>
+        <v>54.074750000000002</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8">
+      <c r="A86" t="s">
+        <v>39</v>
+      </c>
+      <c r="B86" t="s">
+        <v>34</v>
+      </c>
+      <c r="C86">
+        <v>1163.4000000000001</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="F86">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G86">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8">
+      <c r="A87" t="s">
+        <v>40</v>
+      </c>
+      <c r="B87" t="s">
+        <v>34</v>
+      </c>
+      <c r="C87">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="F87">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>803.00000000000011</v>
+      </c>
+      <c r="G87">
+        <f t="shared" si="1"/>
+        <v>0.80300000000000016</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8">
+      <c r="A88" t="s">
+        <v>30</v>
+      </c>
+      <c r="B88" t="s">
+        <v>31</v>
+      </c>
+      <c r="C88">
+        <v>142</v>
+      </c>
+      <c r="D88">
+        <v>245.8</v>
+      </c>
+      <c r="F88">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>51830</v>
+      </c>
+      <c r="G88">
+        <f t="shared" si="1"/>
+        <v>51.83</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8">
+      <c r="A89" t="s">
+        <v>32</v>
+      </c>
+      <c r="B89" t="s">
+        <v>31</v>
+      </c>
+      <c r="C89">
+        <v>398.13</v>
+      </c>
+      <c r="D89">
+        <v>467.5</v>
+      </c>
+      <c r="F89">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>145317.45000000001</v>
+      </c>
+      <c r="G89">
+        <f t="shared" si="1"/>
+        <v>145.31745000000001</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8">
+      <c r="A90" t="s">
+        <v>35</v>
+      </c>
+      <c r="B90" t="s">
+        <v>41</v>
+      </c>
+      <c r="C90">
+        <v>114.2</v>
+      </c>
+      <c r="F90">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>41683</v>
+      </c>
+      <c r="G90">
+        <f t="shared" si="1"/>
+        <v>41.683</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8">
+      <c r="A91" t="s">
+        <v>36</v>
+      </c>
+      <c r="B91" t="s">
+        <v>41</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="F91">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G91">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8">
+      <c r="A92" t="s">
+        <v>26</v>
+      </c>
+      <c r="B92" t="s">
+        <v>83</v>
+      </c>
+      <c r="E92">
+        <v>30</v>
+      </c>
+      <c r="F92">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>10950</v>
+      </c>
+      <c r="G92">
+        <f t="shared" si="1"/>
+        <v>10.95</v>
+      </c>
+      <c r="H92" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8">
+      <c r="A93" t="s">
+        <v>20</v>
+      </c>
+      <c r="B93" t="s">
+        <v>23</v>
+      </c>
+      <c r="C93">
+        <v>112.5</v>
+      </c>
+      <c r="F93">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>41062.5</v>
+      </c>
+      <c r="G93">
+        <f t="shared" si="1"/>
+        <v>41.0625</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8">
+      <c r="A94" t="s">
+        <v>21</v>
+      </c>
+      <c r="B94" t="s">
+        <v>23</v>
+      </c>
+      <c r="C94">
+        <v>28.5</v>
+      </c>
+      <c r="F94">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>10402.5</v>
+      </c>
+      <c r="G94">
+        <f t="shared" si="1"/>
+        <v>10.4025</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8">
+      <c r="A95" t="s">
+        <v>24</v>
+      </c>
+      <c r="B95" t="s">
+        <v>23</v>
+      </c>
+      <c r="C95">
+        <v>7.7</v>
+      </c>
+      <c r="F95">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>2810.5</v>
+      </c>
+      <c r="G95">
+        <f t="shared" si="1"/>
+        <v>2.8105000000000002</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8">
+      <c r="A96" t="s">
+        <v>20</v>
+      </c>
+      <c r="B96" t="s">
+        <v>29</v>
+      </c>
+      <c r="C96">
+        <v>246.5</v>
+      </c>
+      <c r="F96">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>89972.5</v>
+      </c>
+      <c r="G96">
+        <f t="shared" si="1"/>
+        <v>89.972499999999997</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8">
+      <c r="A97" t="s">
+        <v>28</v>
+      </c>
+      <c r="B97" t="s">
+        <v>29</v>
+      </c>
+      <c r="C97">
+        <v>1246.4000000000001</v>
+      </c>
+      <c r="F97">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>454936.00000000006</v>
+      </c>
+      <c r="G97">
+        <f t="shared" si="1"/>
+        <v>454.93600000000004</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8">
+      <c r="A98" t="s">
+        <v>30</v>
+      </c>
+      <c r="B98" t="s">
+        <v>29</v>
+      </c>
+      <c r="C98">
+        <v>50.883000000000003</v>
+      </c>
+      <c r="F98">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>18572.295000000002</v>
+      </c>
+      <c r="G98">
+        <f t="shared" si="1"/>
+        <v>18.572295</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8">
+      <c r="A99" t="s">
+        <v>39</v>
+      </c>
+      <c r="B99" t="s">
+        <v>29</v>
+      </c>
+      <c r="C99">
+        <v>2277.6</v>
+      </c>
+      <c r="D99">
+        <v>1799</v>
+      </c>
+      <c r="F99">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>656635</v>
+      </c>
+      <c r="G99">
+        <f t="shared" si="1"/>
+        <v>656.63499999999999</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8">
+      <c r="A100" t="s">
+        <v>50</v>
+      </c>
+      <c r="B100" t="s">
+        <v>51</v>
+      </c>
+      <c r="C100">
+        <v>1138.0999999999999</v>
+      </c>
+      <c r="F100">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>415406.49999999994</v>
+      </c>
+      <c r="G100">
+        <f t="shared" si="1"/>
+        <v>415.40649999999994</v>
+      </c>
+      <c r="H100" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8">
+      <c r="A101" t="s">
+        <v>32</v>
+      </c>
+      <c r="B101" t="s">
+        <v>47</v>
+      </c>
+      <c r="C101">
+        <v>497.16</v>
+      </c>
+      <c r="D101">
+        <v>701.8</v>
+      </c>
+      <c r="F101">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>181463.40000000002</v>
+      </c>
+      <c r="G101">
+        <f t="shared" si="1"/>
+        <v>181.46340000000004</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8">
+      <c r="A102" t="s">
+        <v>41</v>
+      </c>
+      <c r="B102" t="s">
+        <v>47</v>
+      </c>
+      <c r="E102">
+        <v>958.9</v>
+      </c>
+      <c r="F102">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>349998.5</v>
+      </c>
+      <c r="G102">
+        <f t="shared" si="1"/>
+        <v>349.99849999999998</v>
+      </c>
+      <c r="H102" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8">
+      <c r="A103" t="s">
+        <v>97</v>
+      </c>
+      <c r="B103" t="s">
+        <v>47</v>
+      </c>
+      <c r="D103">
+        <v>375</v>
+      </c>
+      <c r="F103">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>136875</v>
+      </c>
+      <c r="G103">
+        <f t="shared" si="1"/>
+        <v>136.875</v>
+      </c>
+      <c r="H103" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8">
+      <c r="A104" t="s">
+        <v>29</v>
+      </c>
+      <c r="B104" t="s">
+        <v>39</v>
+      </c>
+      <c r="C104">
+        <v>416</v>
+      </c>
+      <c r="D104">
+        <v>280.8</v>
+      </c>
+      <c r="F104">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>102492</v>
+      </c>
+      <c r="G104">
+        <f t="shared" si="1"/>
+        <v>102.492</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8">
+      <c r="A105" t="s">
+        <v>34</v>
+      </c>
+      <c r="B105" t="s">
+        <v>39</v>
+      </c>
+      <c r="C105">
+        <v>122.2</v>
+      </c>
+      <c r="F105">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>44603</v>
+      </c>
+      <c r="G105">
+        <f t="shared" si="1"/>
+        <v>44.603000000000002</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8">
+      <c r="A106" t="s">
+        <v>41</v>
+      </c>
+      <c r="B106" t="s">
+        <v>39</v>
+      </c>
+      <c r="E106">
+        <v>5459.5088498999994</v>
+      </c>
+      <c r="F106">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>1992720.7302134999</v>
+      </c>
+      <c r="G106">
+        <f t="shared" si="1"/>
+        <v>1992.7207302134998</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8">
+      <c r="A107" t="s">
+        <v>40</v>
+      </c>
+      <c r="B107" t="s">
+        <v>39</v>
+      </c>
+      <c r="E107">
+        <v>80.846503979999994</v>
+      </c>
+      <c r="F107">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>29508.973952699998</v>
+      </c>
+      <c r="G107">
+        <f t="shared" si="1"/>
+        <v>29.5089739527</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8">
+      <c r="A108" t="s">
+        <v>53</v>
+      </c>
+      <c r="B108" t="s">
+        <v>39</v>
+      </c>
+      <c r="E108">
+        <v>35.53171072</v>
+      </c>
+      <c r="F108">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>12969.074412800001</v>
+      </c>
+      <c r="G108">
+        <f t="shared" si="1"/>
+        <v>12.969074412800001</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8">
+      <c r="A109" t="s">
+        <v>17</v>
+      </c>
+      <c r="B109" t="s">
+        <v>11</v>
+      </c>
+      <c r="C109">
+        <v>803.4</v>
+      </c>
+      <c r="D109">
+        <v>205.9</v>
+      </c>
+      <c r="F109">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>75153.5</v>
+      </c>
+      <c r="G109">
+        <f t="shared" si="1"/>
+        <v>75.153499999999994</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8">
+      <c r="A110" t="s">
+        <v>49</v>
+      </c>
+      <c r="B110" t="s">
+        <v>11</v>
+      </c>
+      <c r="C110">
+        <v>1499.1</v>
+      </c>
+      <c r="D110">
+        <v>1406</v>
+      </c>
+      <c r="F110">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>513190</v>
+      </c>
+      <c r="G110">
+        <f t="shared" si="1"/>
+        <v>513.19000000000005</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8">
+      <c r="A111" t="s">
+        <v>18</v>
+      </c>
+      <c r="B111" t="s">
+        <v>11</v>
+      </c>
+      <c r="C111">
+        <v>494.4</v>
+      </c>
+      <c r="F111">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>180456</v>
+      </c>
+      <c r="G111">
+        <f t="shared" si="1"/>
+        <v>180.45599999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58F6DC53-AE01-4DBE-BF9B-43427CD51EF0}">
   <dimension ref="A1:F37"/>
   <sheetFormatPr defaultRowHeight="14.5"/>

</xml_diff>

<commit_message>
update capacity values from capacity map by entsog
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{832237F2-9583-4190-A328-0990B39D810F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF85F68E-ECFD-472C-BDEE-E1260FD9D93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="985" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="154">
   <si>
     <t>Belgium</t>
   </si>
@@ -499,6 +499,12 @@
   </si>
   <si>
     <t>Assumption, same as MA to ES</t>
+  </si>
+  <si>
+    <t>in entsog capacity as DZ to italy</t>
+  </si>
+  <si>
+    <t>not in entsog capacity anymore</t>
   </si>
 </sst>
 </file>
@@ -510,7 +516,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -637,6 +643,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -727,12 +738,14 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -952,10 +965,10 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FC7F2F97-F859-4A2C-9657-17C35EEFE785}" name="Table37" displayName="Table37" ref="A1:H111" totalsRowShown="0">
-  <autoFilter ref="A1:H111" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H111">
-    <sortCondition ref="B1:B111"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FC7F2F97-F859-4A2C-9657-17C35EEFE785}" name="Table37" displayName="Table37" ref="A1:H117" totalsRowShown="0">
+  <autoFilter ref="A1:H117" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H117">
+    <sortCondition ref="B1:B117"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{F94559DC-2602-4FF1-9531-3B8A374512C0}" name="From"/>
@@ -8323,7 +8336,7 @@
         <v>18572.295000000002</v>
       </c>
       <c r="G98">
-        <f t="shared" ref="G98:G129" si="3">F98/1000</f>
+        <f t="shared" ref="G98:G111" si="3">F98/1000</f>
         <v>18.572295</v>
       </c>
     </row>
@@ -8609,7 +8622,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67CAB708-6819-43AD-B444-2B653F840206}">
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H117"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="20.453125" customWidth="1"/>
@@ -8660,7 +8673,7 @@
         <v>177791.5</v>
       </c>
       <c r="G2">
-        <f t="shared" ref="G2:G65" si="0">F2/1000</f>
+        <f t="shared" ref="G2:G67" si="0">F2/1000</f>
         <v>177.79150000000001</v>
       </c>
       <c r="H2" t="s">
@@ -8675,15 +8688,15 @@
         <v>20</v>
       </c>
       <c r="C3">
-        <v>344.24799999999993</v>
+        <v>710.94036800000003</v>
       </c>
       <c r="F3">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>125650.51999999997</v>
+        <v>259493.23432000002</v>
       </c>
       <c r="G3">
         <f t="shared" si="0"/>
-        <v>125.65051999999997</v>
+        <v>259.49323432</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -8694,15 +8707,15 @@
         <v>20</v>
       </c>
       <c r="C4">
-        <v>193.5</v>
+        <v>194.05</v>
       </c>
       <c r="F4">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>70627.5</v>
+        <v>70828.25</v>
       </c>
       <c r="G4">
         <f t="shared" si="0"/>
-        <v>70.627499999999998</v>
+        <v>70.828249999999997</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -8713,15 +8726,15 @@
         <v>20</v>
       </c>
       <c r="C5">
-        <v>1570.4</v>
+        <v>1708.7</v>
       </c>
       <c r="F5">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>573196</v>
+        <v>623675.5</v>
       </c>
       <c r="G5">
         <f t="shared" si="0"/>
-        <v>573.19600000000003</v>
+        <v>623.67550000000006</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -8732,15 +8745,15 @@
         <v>45</v>
       </c>
       <c r="C6">
-        <v>17.98</v>
+        <v>14</v>
       </c>
       <c r="F6">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>6562.7</v>
+        <v>5110</v>
       </c>
       <c r="G6">
         <f t="shared" si="0"/>
-        <v>6.5626999999999995</v>
+        <v>5.1100000000000003</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -8750,6 +8763,9 @@
       <c r="B7" t="s">
         <v>17</v>
       </c>
+      <c r="C7">
+        <v>651.70000000000005</v>
+      </c>
       <c r="D7">
         <v>205.9</v>
       </c>
@@ -8770,15 +8786,15 @@
         <v>17</v>
       </c>
       <c r="C8">
-        <v>1397.2</v>
+        <v>1387.5634559999999</v>
       </c>
       <c r="F8">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>509978</v>
+        <v>506460.66143999994</v>
       </c>
       <c r="G8">
         <f t="shared" si="0"/>
-        <v>509.97800000000001</v>
+        <v>506.46066143999991</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -8789,15 +8805,15 @@
         <v>17</v>
       </c>
       <c r="C9">
-        <v>396.15000000000003</v>
+        <v>356</v>
       </c>
       <c r="F9">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>144594.75</v>
+        <v>129940</v>
       </c>
       <c r="G9">
         <f t="shared" si="0"/>
-        <v>144.59475</v>
+        <v>129.94</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -8827,7 +8843,7 @@
         <v>17</v>
       </c>
       <c r="C11">
-        <v>488</v>
+        <v>488.4</v>
       </c>
       <c r="D11">
         <v>453.2</v>
@@ -8868,15 +8884,15 @@
         <v>32</v>
       </c>
       <c r="C13">
-        <v>335.26</v>
+        <v>350.11200000000002</v>
       </c>
       <c r="F13">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>122369.9</v>
+        <v>127790.88</v>
       </c>
       <c r="G13">
         <f t="shared" si="0"/>
-        <v>122.3699</v>
+        <v>127.79088</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -8887,15 +8903,15 @@
         <v>32</v>
       </c>
       <c r="C14">
-        <v>64.819999999999993</v>
+        <v>172.57</v>
       </c>
       <c r="F14">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>23659.3</v>
+        <v>62988.049999999996</v>
       </c>
       <c r="G14">
         <f t="shared" si="0"/>
-        <v>23.659299999999998</v>
+        <v>62.988049999999994</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -8906,15 +8922,15 @@
         <v>32</v>
       </c>
       <c r="C15">
-        <v>805.75000000000011</v>
+        <v>231.417</v>
       </c>
       <c r="F15">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>294098.75000000006</v>
+        <v>84467.205000000002</v>
       </c>
       <c r="G15">
         <f t="shared" si="0"/>
-        <v>294.09875000000005</v>
+        <v>84.467205000000007</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -8963,15 +8979,15 @@
         <v>22</v>
       </c>
       <c r="C18">
-        <v>328</v>
+        <v>353.83</v>
       </c>
       <c r="F18">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>119720</v>
+        <v>129147.95</v>
       </c>
       <c r="G18">
         <f t="shared" si="0"/>
-        <v>119.72</v>
+        <v>129.14795000000001</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -8982,15 +8998,15 @@
         <v>22</v>
       </c>
       <c r="C19">
-        <v>431.4</v>
+        <v>387.85</v>
       </c>
       <c r="F19">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>157461</v>
+        <v>141565.25</v>
       </c>
       <c r="G19">
         <f t="shared" si="0"/>
-        <v>157.46100000000001</v>
+        <v>141.56524999999999</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -9001,15 +9017,15 @@
         <v>22</v>
       </c>
       <c r="C20">
-        <v>223</v>
+        <v>259.02</v>
       </c>
       <c r="F20">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>81395</v>
+        <v>94542.299999999988</v>
       </c>
       <c r="G20">
         <f t="shared" si="0"/>
-        <v>81.394999999999996</v>
+        <v>94.542299999999983</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -9020,15 +9036,15 @@
         <v>28</v>
       </c>
       <c r="C21">
-        <v>1803.77</v>
+        <v>1628</v>
       </c>
       <c r="F21">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>658376.05000000005</v>
+        <v>594220</v>
       </c>
       <c r="G21">
         <f t="shared" si="0"/>
-        <v>658.37605000000008</v>
+        <v>594.22</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -9039,15 +9055,15 @@
         <v>28</v>
       </c>
       <c r="C22">
-        <v>457.6</v>
+        <v>395.2</v>
       </c>
       <c r="F22">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>167024</v>
+        <v>144248</v>
       </c>
       <c r="G22">
         <f t="shared" si="0"/>
-        <v>167.024</v>
+        <v>144.24799999999999</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -9058,15 +9074,15 @@
         <v>19</v>
       </c>
       <c r="C23">
-        <v>322.77</v>
+        <v>542</v>
       </c>
       <c r="F23">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>117811.04999999999</v>
+        <v>197830</v>
       </c>
       <c r="G23">
         <f t="shared" si="0"/>
-        <v>117.81104999999999</v>
+        <v>197.83</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -9077,15 +9093,15 @@
         <v>19</v>
       </c>
       <c r="C24">
-        <v>1925.7729999999999</v>
+        <v>1849.1500000000003</v>
       </c>
       <c r="F24">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>702907.14500000002</v>
+        <v>674939.75000000012</v>
       </c>
       <c r="G24">
         <f t="shared" si="0"/>
-        <v>702.90714500000001</v>
+        <v>674.93975000000012</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -9096,15 +9112,15 @@
         <v>19</v>
       </c>
       <c r="C25">
-        <v>339.96799999999996</v>
+        <v>797.93600000000004</v>
       </c>
       <c r="F25">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>124088.31999999999</v>
+        <v>291246.64</v>
       </c>
       <c r="G25">
         <f t="shared" si="0"/>
-        <v>124.08832</v>
+        <v>291.24664000000001</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -9115,1172 +9131,1172 @@
         <v>19</v>
       </c>
       <c r="C26">
-        <v>172.8</v>
+        <v>240</v>
       </c>
       <c r="F26">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>63072.000000000007</v>
+        <v>87600</v>
       </c>
       <c r="G26">
         <f t="shared" si="0"/>
-        <v>63.07200000000001</v>
+        <v>87.6</v>
       </c>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s">
         <v>19</v>
       </c>
       <c r="C27">
-        <v>4.1189999999999998</v>
-      </c>
-      <c r="F27">
+        <v>100</v>
+      </c>
+      <c r="F27" s="5">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>1503.4349999999999</v>
+        <v>36500</v>
       </c>
       <c r="G27">
-        <f t="shared" si="0"/>
-        <v>1.5034349999999999</v>
+        <f>F27/1000</f>
+        <v>36.5</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" t="s">
         <v>19</v>
       </c>
       <c r="C28">
-        <v>931.6</v>
+        <v>15.7</v>
       </c>
       <c r="F28">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>340034</v>
+        <v>5730.5</v>
       </c>
       <c r="G28">
         <f t="shared" si="0"/>
-        <v>340.03399999999999</v>
+        <v>5.7305000000000001</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" t="s">
         <v>19</v>
       </c>
       <c r="C29">
-        <v>1231.759</v>
+        <v>0.09</v>
       </c>
       <c r="F29">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>449592.03500000003</v>
+        <v>32.85</v>
       </c>
       <c r="G29">
         <f t="shared" si="0"/>
-        <v>449.59203500000001</v>
+        <v>3.2850000000000004E-2</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="B30" t="s">
         <v>19</v>
       </c>
-      <c r="D30">
-        <v>0</v>
+      <c r="C30">
+        <v>960.97</v>
       </c>
       <c r="F30">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
+        <v>350754.05</v>
       </c>
       <c r="G30">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>350.75405000000001</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B31" t="s">
         <v>19</v>
       </c>
-      <c r="C31">
-        <v>2210.5639999999999</v>
-      </c>
       <c r="D31">
-        <v>1226</v>
+        <v>0</v>
       </c>
       <c r="F31">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>447490</v>
+        <v>0</v>
       </c>
       <c r="G31">
         <f t="shared" si="0"/>
-        <v>447.49</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" t="s">
+        <v>49</v>
+      </c>
+      <c r="B32" t="s">
         <v>19</v>
       </c>
-      <c r="B32" t="s">
-        <v>26</v>
-      </c>
       <c r="C32">
-        <v>136.11199999999999</v>
+        <v>2195.9271199999998</v>
+      </c>
+      <c r="D32">
+        <v>1226</v>
       </c>
       <c r="F32">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>49680.88</v>
+        <v>447490</v>
       </c>
       <c r="G32">
         <f t="shared" si="0"/>
-        <v>49.680879999999995</v>
+        <v>447.49</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="B33" t="s">
-        <v>54</v>
-      </c>
-      <c r="E33">
-        <v>67.7</v>
+        <v>26</v>
+      </c>
+      <c r="C33">
+        <v>123.627</v>
       </c>
       <c r="F33">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>24710.5</v>
+        <v>45123.854999999996</v>
       </c>
       <c r="G33">
         <f t="shared" si="0"/>
-        <v>24.7105</v>
+        <v>45.123854999999999</v>
       </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="B34" t="s">
-        <v>54</v>
-      </c>
-      <c r="F34">
+        <v>26</v>
+      </c>
+      <c r="C34">
+        <v>91.2</v>
+      </c>
+      <c r="F34" s="5">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
+        <v>33288</v>
       </c>
       <c r="G34">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f>F34/1000</f>
+        <v>33.287999999999997</v>
       </c>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="B35" t="s">
         <v>54</v>
       </c>
       <c r="E35">
-        <v>32.802250000000008</v>
+        <v>67.7</v>
       </c>
       <c r="F35">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>11972.821250000003</v>
+        <v>24710.5</v>
       </c>
       <c r="G35">
         <f t="shared" si="0"/>
-        <v>11.972821250000003</v>
+        <v>24.7105</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
-      </c>
-      <c r="C36">
-        <v>164.572</v>
+        <v>54</v>
       </c>
       <c r="F36">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>60068.78</v>
+        <v>0</v>
       </c>
       <c r="G36">
         <f t="shared" si="0"/>
-        <v>60.068779999999997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="B37" t="s">
-        <v>37</v>
-      </c>
-      <c r="C37">
-        <v>80</v>
+        <v>54</v>
+      </c>
+      <c r="C37" s="6">
+        <v>78</v>
+      </c>
+      <c r="E37">
+        <v>32.802250000000008</v>
       </c>
       <c r="F37">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>29200</v>
+        <v>11972.821250000003</v>
       </c>
       <c r="G37">
         <f t="shared" si="0"/>
-        <v>29.2</v>
+        <v>11.972821250000003</v>
       </c>
     </row>
     <row r="38" spans="1:7">
       <c r="A38" t="s">
-        <v>99</v>
+        <v>25</v>
       </c>
       <c r="B38" t="s">
         <v>37</v>
       </c>
-      <c r="D38">
-        <v>31.92</v>
+      <c r="C38">
+        <v>164.57</v>
       </c>
       <c r="F38">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>11650.800000000001</v>
+        <v>60068.049999999996</v>
       </c>
       <c r="G38">
         <f t="shared" si="0"/>
-        <v>11.6508</v>
+        <v>60.068049999999992</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="B39" t="s">
         <v>37</v>
       </c>
       <c r="C39">
-        <v>731.7</v>
-      </c>
-      <c r="D39">
-        <v>337.1</v>
+        <v>80</v>
       </c>
       <c r="F39">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>123041.50000000001</v>
+        <v>29200</v>
       </c>
       <c r="G39">
         <f t="shared" si="0"/>
-        <v>123.04150000000001</v>
+        <v>29.2</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>41</v>
+        <v>99</v>
       </c>
       <c r="B40" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="D40">
-        <v>0</v>
+        <v>31.92</v>
       </c>
       <c r="F40">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
+        <v>11650.800000000001</v>
       </c>
       <c r="G40">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>11.6508</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B41" t="s">
-        <v>55</v>
-      </c>
-      <c r="E41">
-        <v>61.341321000000001</v>
+        <v>37</v>
+      </c>
+      <c r="C41">
+        <v>337.12</v>
+      </c>
+      <c r="D41">
+        <v>337.1</v>
       </c>
       <c r="F41">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>22389.582165</v>
+        <v>123041.50000000001</v>
       </c>
       <c r="G41">
         <f t="shared" si="0"/>
-        <v>22.389582165</v>
+        <v>123.04150000000001</v>
       </c>
     </row>
     <row r="42" spans="1:7">
       <c r="A42" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>25</v>
-      </c>
-      <c r="C42">
-        <v>870</v>
+        <v>55</v>
+      </c>
+      <c r="D42">
+        <v>0</v>
       </c>
       <c r="F42">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>317550</v>
+        <v>0</v>
       </c>
       <c r="G42">
         <f t="shared" si="0"/>
-        <v>317.55</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:7">
       <c r="A43" t="s">
-        <v>19</v>
+        <v>54</v>
       </c>
       <c r="B43" t="s">
-        <v>25</v>
-      </c>
-      <c r="C43">
-        <v>613.71600000000001</v>
+        <v>55</v>
+      </c>
+      <c r="E43">
+        <v>61.341321000000001</v>
       </c>
       <c r="F43">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>224006.34</v>
+        <v>22389.582165</v>
       </c>
       <c r="G43">
         <f t="shared" si="0"/>
-        <v>224.00633999999999</v>
+        <v>22.389582165</v>
       </c>
     </row>
     <row r="44" spans="1:7">
       <c r="A44" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B44" t="s">
         <v>25</v>
       </c>
       <c r="C44">
-        <v>100</v>
+        <v>530</v>
       </c>
       <c r="F44">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>36500</v>
+        <v>193450</v>
       </c>
       <c r="G44">
         <f t="shared" si="0"/>
-        <v>36.5</v>
+        <v>193.45</v>
       </c>
     </row>
     <row r="45" spans="1:7">
       <c r="A45" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="B45" t="s">
         <v>25</v>
       </c>
       <c r="C45">
-        <v>224.4</v>
+        <v>613.74174400000004</v>
       </c>
       <c r="F45">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>81906</v>
+        <v>224015.73656000002</v>
       </c>
       <c r="G45">
         <f t="shared" si="0"/>
-        <v>81.906000000000006</v>
+        <v>224.01573656000002</v>
       </c>
     </row>
     <row r="46" spans="1:7">
       <c r="A46" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="B46" t="s">
         <v>25</v>
       </c>
       <c r="C46">
-        <v>570</v>
-      </c>
-      <c r="D46">
-        <v>568.5</v>
+        <v>100</v>
       </c>
       <c r="F46">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>207502.5</v>
+        <v>36500</v>
       </c>
       <c r="G46">
         <f t="shared" si="0"/>
-        <v>207.5025</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B47" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C47">
-        <v>117.8</v>
+        <v>224.4</v>
       </c>
       <c r="F47">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>42997</v>
+        <v>81906</v>
       </c>
       <c r="G47">
         <f t="shared" si="0"/>
-        <v>42.997</v>
+        <v>81.906000000000006</v>
       </c>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B48" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C48">
-        <v>398.6</v>
+        <v>575</v>
+      </c>
+      <c r="D48">
+        <v>568.5</v>
       </c>
       <c r="F48">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>145489</v>
+        <v>207502.5</v>
       </c>
       <c r="G48">
         <f t="shared" si="0"/>
-        <v>145.489</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7">
+        <v>207.5025</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="B49" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C49">
-        <v>53.7</v>
+        <v>120.36</v>
       </c>
       <c r="F49">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>19600.5</v>
+        <v>43931.4</v>
       </c>
       <c r="G49">
         <f t="shared" si="0"/>
-        <v>19.6005</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7">
+        <v>43.931400000000004</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="B50" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="C50">
-        <v>77.400000000000006</v>
+        <v>398.6</v>
       </c>
       <c r="F50">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>28251.000000000004</v>
+        <v>145489</v>
       </c>
       <c r="G50">
         <f t="shared" si="0"/>
-        <v>28.251000000000005</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7">
+        <v>145.489</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B51" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C51">
-        <v>153.1</v>
+        <v>53.7</v>
       </c>
       <c r="F51">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>55881.5</v>
+        <v>19600.5</v>
       </c>
       <c r="G51">
         <f t="shared" si="0"/>
-        <v>55.881500000000003</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7">
+        <v>19.6005</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52" t="s">
+        <v>30</v>
+      </c>
+      <c r="B52" t="s">
         <v>24</v>
       </c>
-      <c r="B52" t="s">
-        <v>30</v>
-      </c>
       <c r="C52">
-        <v>48.57</v>
+        <v>77.2</v>
       </c>
       <c r="F52">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>17728.05</v>
+        <v>28178</v>
       </c>
       <c r="G52">
         <f t="shared" si="0"/>
-        <v>17.72805</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7">
+        <v>28.178000000000001</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
       <c r="A53" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B53" t="s">
         <v>30</v>
       </c>
       <c r="C53">
-        <v>128.9</v>
+        <v>153.08000000000001</v>
       </c>
       <c r="F53">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>47048.5</v>
+        <v>55874.200000000004</v>
       </c>
       <c r="G53">
         <f t="shared" si="0"/>
-        <v>47.048499999999997</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7">
+        <v>55.874200000000002</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
       <c r="A54" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="B54" t="s">
         <v>30</v>
       </c>
       <c r="C54">
-        <v>50.3</v>
+        <v>50.9</v>
       </c>
       <c r="F54">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>18359.5</v>
+        <v>18578.5</v>
       </c>
       <c r="G54">
         <f t="shared" si="0"/>
-        <v>18.359500000000001</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7">
+        <v>18.578499999999998</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
       <c r="A55" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="B55" t="s">
         <v>30</v>
       </c>
       <c r="C55">
-        <v>515.6</v>
-      </c>
-      <c r="D55">
-        <v>84.77</v>
+        <v>128.97</v>
       </c>
       <c r="F55">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>30941.05</v>
+        <v>47074.05</v>
       </c>
       <c r="G55">
         <f t="shared" si="0"/>
-        <v>30.941050000000001</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7">
+        <v>47.07405</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
       <c r="A56" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B56" t="s">
         <v>30</v>
       </c>
-      <c r="D56">
-        <v>245.8</v>
+      <c r="C56">
+        <v>73.37</v>
       </c>
       <c r="F56">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>89717</v>
+        <v>26780.050000000003</v>
       </c>
       <c r="G56">
         <f t="shared" si="0"/>
-        <v>89.716999999999999</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7">
+        <v>26.780050000000003</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
       <c r="A57" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="B57" t="s">
-        <v>44</v>
-      </c>
-      <c r="C57">
-        <v>386.9</v>
+        <v>30</v>
       </c>
       <c r="D57">
-        <v>385</v>
+        <v>84.77</v>
       </c>
       <c r="F57">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>140525</v>
+        <v>30941.05</v>
       </c>
       <c r="G57">
         <f t="shared" si="0"/>
-        <v>140.52500000000001</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7">
+        <v>30.941050000000001</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
       <c r="A58" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="B58" t="s">
-        <v>21</v>
-      </c>
-      <c r="C58">
-        <v>1150</v>
+        <v>30</v>
+      </c>
+      <c r="D58">
+        <v>245.8</v>
       </c>
       <c r="F58">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>419750</v>
+        <v>89717</v>
       </c>
       <c r="G58">
         <f t="shared" si="0"/>
-        <v>419.75</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7">
+        <v>89.716999999999999</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
       <c r="A59" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B59" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="C59">
-        <v>640.4</v>
+        <v>386.58</v>
+      </c>
+      <c r="D59">
+        <v>385</v>
       </c>
       <c r="F59">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>233746</v>
+        <v>140525</v>
       </c>
       <c r="G59">
         <f t="shared" si="0"/>
-        <v>233.74600000000001</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7">
+        <v>140.52500000000001</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
       <c r="A60" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B60" t="s">
         <v>21</v>
       </c>
       <c r="C60">
-        <v>21.5</v>
+        <v>1176.1099999999999</v>
       </c>
       <c r="F60">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>7847.5</v>
+        <v>429280.14999999997</v>
       </c>
       <c r="G60">
         <f t="shared" si="0"/>
-        <v>7.8475000000000001</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7">
+        <v>429.28014999999999</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
       <c r="A61" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="B61" t="s">
         <v>21</v>
       </c>
       <c r="C61">
-        <v>487.1</v>
+        <v>640.48</v>
       </c>
       <c r="F61">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>177791.5</v>
+        <v>233775.2</v>
       </c>
       <c r="G61">
         <f t="shared" si="0"/>
-        <v>177.79150000000001</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7">
+        <v>233.77520000000001</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
       <c r="A62" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="B62" t="s">
         <v>21</v>
       </c>
       <c r="C62">
-        <v>1138.0999999999999</v>
-      </c>
-      <c r="D62">
-        <v>1154</v>
+        <v>25.77</v>
       </c>
       <c r="F62">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>415406.49999999994</v>
+        <v>9406.0499999999993</v>
       </c>
       <c r="G62">
         <f t="shared" si="0"/>
-        <v>415.40649999999994</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7">
+        <v>9.4060499999999987</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
       <c r="A63" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B63" t="s">
         <v>21</v>
       </c>
       <c r="C63">
-        <v>475.8</v>
-      </c>
-      <c r="D63">
-        <v>493.7</v>
+        <v>494.33</v>
       </c>
       <c r="F63">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>173667</v>
+        <v>180430.44999999998</v>
       </c>
       <c r="G63">
         <f t="shared" si="0"/>
-        <v>173.667</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7">
+        <v>180.43044999999998</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
       <c r="A64" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="B64" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="C64">
-        <v>65.099999999999994</v>
+        <v>1154.47</v>
+      </c>
+      <c r="D64">
+        <v>1154</v>
       </c>
       <c r="F64">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>23761.499999999996</v>
+        <v>421210</v>
       </c>
       <c r="G64">
         <f t="shared" si="0"/>
-        <v>23.761499999999998</v>
+        <v>421.21</v>
+      </c>
+      <c r="H64" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="65" spans="1:8">
       <c r="A65" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B65" t="s">
-        <v>35</v>
-      </c>
-      <c r="C65">
-        <v>325.39999999999998</v>
+        <v>21</v>
       </c>
       <c r="D65">
-        <v>325.39999999999998</v>
+        <v>493.7</v>
       </c>
       <c r="F65">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>118770.99999999999</v>
+        <v>180200.5</v>
       </c>
       <c r="G65">
         <f t="shared" si="0"/>
-        <v>118.77099999999999</v>
+        <v>180.20050000000001</v>
+      </c>
+      <c r="H65" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="66" spans="1:8">
       <c r="A66" t="s">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="B66" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C66">
-        <v>26.71</v>
+        <v>82</v>
       </c>
       <c r="F66">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>9749.15</v>
+        <v>29930</v>
       </c>
       <c r="G66">
-        <f t="shared" ref="G66:G111" si="1">F66/1000</f>
-        <v>9.7491500000000002</v>
+        <f t="shared" si="0"/>
+        <v>29.93</v>
       </c>
     </row>
     <row r="67" spans="1:8">
       <c r="A67" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="B67" t="s">
-        <v>43</v>
-      </c>
-      <c r="E67">
-        <v>41.973541999999995</v>
+        <v>35</v>
+      </c>
+      <c r="D67">
+        <v>325.39999999999998</v>
       </c>
       <c r="F67">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>15320.342829999998</v>
+        <v>118770.99999999999</v>
       </c>
       <c r="G67">
-        <f t="shared" si="1"/>
-        <v>15.320342829999998</v>
+        <f t="shared" si="0"/>
+        <v>118.77099999999999</v>
+      </c>
+      <c r="H67" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="68" spans="1:8">
       <c r="A68" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B68" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="C68">
-        <v>67.599999999999994</v>
+        <v>24</v>
       </c>
       <c r="F68">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>24673.999999999996</v>
+        <v>8760</v>
       </c>
       <c r="G68">
-        <f t="shared" si="1"/>
-        <v>24.673999999999996</v>
+        <f t="shared" ref="G68:G117" si="1">F68/1000</f>
+        <v>8.76</v>
       </c>
     </row>
     <row r="69" spans="1:8">
       <c r="A69" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="B69" t="s">
-        <v>36</v>
-      </c>
-      <c r="D69">
-        <v>0</v>
+        <v>43</v>
+      </c>
+      <c r="C69">
+        <v>48.8</v>
+      </c>
+      <c r="E69">
+        <v>41.973541999999995</v>
       </c>
       <c r="F69">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
+        <v>15320.342829999998</v>
       </c>
       <c r="G69">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>15.320342829999998</v>
       </c>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="B70" t="s">
         <v>36</v>
       </c>
-      <c r="E70">
-        <v>67.7</v>
+      <c r="C70">
+        <v>90</v>
       </c>
       <c r="F70">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>24710.5</v>
+        <v>32850</v>
       </c>
       <c r="G70">
         <f t="shared" si="1"/>
-        <v>24.7105</v>
+        <v>32.85</v>
       </c>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="B71" t="s">
-        <v>99</v>
+        <v>36</v>
       </c>
       <c r="D71">
-        <v>31.92</v>
+        <v>0</v>
       </c>
       <c r="F71">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>11650.800000000001</v>
+        <v>0</v>
       </c>
       <c r="G71">
         <f t="shared" si="1"/>
-        <v>11.6508</v>
-      </c>
-      <c r="H71" t="s">
-        <v>151</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:8">
       <c r="A72" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="B72" t="s">
-        <v>40</v>
-      </c>
-      <c r="C72">
-        <v>16.100000000000001</v>
+        <v>36</v>
       </c>
       <c r="E72">
-        <v>55.7</v>
+        <v>67.7</v>
       </c>
       <c r="F72">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>5876.5000000000009</v>
+        <v>24710.5</v>
       </c>
       <c r="G72">
         <f t="shared" si="1"/>
-        <v>5.8765000000000009</v>
+        <v>24.7105</v>
       </c>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="B73" t="s">
-        <v>40</v>
-      </c>
-      <c r="E73">
-        <v>255.46047452000005</v>
+        <v>99</v>
+      </c>
+      <c r="D73">
+        <v>31.92</v>
       </c>
       <c r="F73">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>93243.073199800012</v>
+        <v>11650.800000000001</v>
       </c>
       <c r="G73">
         <f t="shared" si="1"/>
-        <v>93.243073199800008</v>
+        <v>11.6508</v>
+      </c>
+      <c r="H73" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="74" spans="1:8">
       <c r="A74" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B74" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C74">
-        <v>27.38</v>
-      </c>
-      <c r="D74">
-        <v>33.28</v>
+        <v>55.7</v>
+      </c>
+      <c r="E74">
+        <v>55.7</v>
       </c>
       <c r="F74">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>9993.6999999999989</v>
+        <v>20330.5</v>
       </c>
       <c r="G74">
         <f t="shared" si="1"/>
-        <v>9.9936999999999987</v>
+        <v>20.330500000000001</v>
       </c>
     </row>
     <row r="75" spans="1:8">
       <c r="A75" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="B75" t="s">
-        <v>18</v>
-      </c>
-      <c r="C75">
-        <v>331.2</v>
+        <v>40</v>
+      </c>
+      <c r="E75">
+        <v>255.46047452000005</v>
       </c>
       <c r="F75">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>120888</v>
+        <v>93243.073199800012</v>
       </c>
       <c r="G75">
         <f t="shared" si="1"/>
-        <v>120.88800000000001</v>
+        <v>93.243073199800008</v>
       </c>
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="B76" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="C76">
-        <v>1628.3030000000001</v>
+        <v>33.28</v>
+      </c>
+      <c r="D76">
+        <v>33.28</v>
       </c>
       <c r="F76">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>594330.59500000009</v>
+        <v>12147.2</v>
       </c>
       <c r="G76">
         <f t="shared" si="1"/>
-        <v>594.33059500000013</v>
+        <v>12.147200000000002</v>
       </c>
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="B77" t="s">
         <v>18</v>
       </c>
-      <c r="D77">
-        <v>963.6</v>
+      <c r="C77">
+        <v>428</v>
       </c>
       <c r="F77">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>351714</v>
+        <v>156220</v>
       </c>
       <c r="G77">
         <f t="shared" si="1"/>
-        <v>351.714</v>
+        <v>156.22</v>
       </c>
     </row>
     <row r="78" spans="1:8">
       <c r="A78" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B78" t="s">
         <v>18</v>
       </c>
       <c r="C78">
-        <v>494.4</v>
+        <v>1513.9</v>
       </c>
       <c r="F78">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>180456</v>
+        <v>552573.5</v>
       </c>
       <c r="G78">
         <f t="shared" si="1"/>
-        <v>180.45599999999999</v>
+        <v>552.57349999999997</v>
       </c>
     </row>
     <row r="79" spans="1:8">
       <c r="A79" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="B79" t="s">
-        <v>27</v>
-      </c>
-      <c r="C79">
-        <v>233.5</v>
+        <v>18</v>
+      </c>
+      <c r="D79">
+        <v>963.6</v>
       </c>
       <c r="F79">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>85227.5</v>
+        <v>351714</v>
       </c>
       <c r="G79">
         <f t="shared" si="1"/>
-        <v>85.227500000000006</v>
+        <v>351.714</v>
       </c>
     </row>
     <row r="80" spans="1:8">
       <c r="A80" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="C80">
-        <v>28</v>
+        <v>168</v>
       </c>
       <c r="F80">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>10220</v>
+        <v>61320</v>
       </c>
       <c r="G80">
         <f t="shared" si="1"/>
-        <v>10.220000000000001</v>
+        <v>61.32</v>
       </c>
     </row>
     <row r="81" spans="1:8">
       <c r="A81" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="B81" t="s">
         <v>27</v>
       </c>
       <c r="C81">
-        <v>135.6</v>
-      </c>
-      <c r="D81">
-        <v>135.6</v>
+        <v>326.27999999999997</v>
       </c>
       <c r="F81">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>49494</v>
+        <v>119092.2</v>
       </c>
       <c r="G81">
         <f t="shared" si="1"/>
-        <v>49.494</v>
+        <v>119.09219999999999</v>
       </c>
     </row>
     <row r="82" spans="1:8">
       <c r="A82" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="B82" t="s">
         <v>27</v>
       </c>
       <c r="C82">
-        <v>1203.4999999999998</v>
-      </c>
-      <c r="D82">
-        <v>0</v>
-      </c>
-      <c r="F82">
+        <v>321.60000000000002</v>
+      </c>
+      <c r="F82" s="5">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
+        <v>117384.00000000001</v>
       </c>
       <c r="G82">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f>F82/1000</f>
+        <v>117.38400000000001</v>
       </c>
     </row>
     <row r="83" spans="1:8">
       <c r="A83" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B83" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C83">
-        <v>144</v>
+        <v>28.03</v>
       </c>
       <c r="F83">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>52560</v>
+        <v>10230.950000000001</v>
       </c>
       <c r="G83">
         <f t="shared" si="1"/>
-        <v>52.56</v>
+        <v>10.23095</v>
       </c>
     </row>
     <row r="84" spans="1:8">
       <c r="A84" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B84" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C84">
-        <v>77.5</v>
-      </c>
-      <c r="F84">
+        <v>58.069200000000002</v>
+      </c>
+      <c r="F84" s="5">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>28287.5</v>
+        <v>21195.258000000002</v>
       </c>
       <c r="G84">
-        <f t="shared" si="1"/>
-        <v>28.287500000000001</v>
+        <f>F84/1000</f>
+        <v>21.195258000000003</v>
       </c>
     </row>
     <row r="85" spans="1:8">
       <c r="A85" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B85" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C85">
-        <v>148.15</v>
-      </c>
-      <c r="F85">
+        <v>144.50399999999999</v>
+      </c>
+      <c r="F85" s="5">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>54074.75</v>
+        <v>52743.96</v>
       </c>
       <c r="G85">
-        <f t="shared" si="1"/>
-        <v>54.074750000000002</v>
+        <f>F85/1000</f>
+        <v>52.743960000000001</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -10288,111 +10304,111 @@
         <v>39</v>
       </c>
       <c r="B86" t="s">
-        <v>34</v>
-      </c>
-      <c r="C86">
-        <v>1163.4000000000001</v>
+        <v>27</v>
       </c>
       <c r="D86">
-        <v>0</v>
+        <v>135.6</v>
       </c>
       <c r="F86">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
+        <v>49494</v>
       </c>
       <c r="G86">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>49.494</v>
+      </c>
+      <c r="H86" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="87" spans="1:8">
       <c r="A87" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="B87" t="s">
-        <v>34</v>
-      </c>
-      <c r="C87">
-        <v>2.2000000000000002</v>
+        <v>27</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
       </c>
       <c r="F87">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>803.00000000000011</v>
+        <v>0</v>
       </c>
       <c r="G87">
         <f t="shared" si="1"/>
-        <v>0.80300000000000016</v>
+        <v>0</v>
+      </c>
+      <c r="H87" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="88" spans="1:8">
       <c r="A88" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="B88" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C88">
-        <v>142</v>
-      </c>
-      <c r="D88">
-        <v>245.8</v>
+        <v>144</v>
       </c>
       <c r="F88">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>51830</v>
+        <v>52560</v>
       </c>
       <c r="G88">
         <f t="shared" si="1"/>
-        <v>51.83</v>
+        <v>52.56</v>
       </c>
     </row>
     <row r="89" spans="1:8">
       <c r="A89" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B89" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C89">
-        <v>398.13</v>
-      </c>
-      <c r="D89">
-        <v>467.5</v>
+        <v>77.459999999999994</v>
       </c>
       <c r="F89">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>145317.45000000001</v>
+        <v>28272.899999999998</v>
       </c>
       <c r="G89">
         <f t="shared" si="1"/>
-        <v>145.31745000000001</v>
+        <v>28.272899999999996</v>
       </c>
     </row>
     <row r="90" spans="1:8">
       <c r="A90" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B90" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="C90">
-        <v>114.2</v>
+        <v>211.73400000000001</v>
       </c>
       <c r="F90">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>41683</v>
+        <v>77282.91</v>
       </c>
       <c r="G90">
         <f t="shared" si="1"/>
-        <v>41.683</v>
+        <v>77.282910000000001</v>
       </c>
     </row>
     <row r="91" spans="1:8">
       <c r="A91" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B91" t="s">
-        <v>41</v>
+        <v>34</v>
+      </c>
+      <c r="C91">
+        <v>0</v>
       </c>
       <c r="D91">
         <v>0</v>
@@ -10405,410 +10421,536 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="H91" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="92" spans="1:8">
       <c r="A92" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="B92" t="s">
-        <v>83</v>
-      </c>
-      <c r="E92">
-        <v>30</v>
+        <v>34</v>
+      </c>
+      <c r="C92">
+        <v>2.2000000000000002</v>
       </c>
       <c r="F92">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>10950</v>
+        <v>803.00000000000011</v>
       </c>
       <c r="G92">
         <f t="shared" si="1"/>
-        <v>10.95</v>
-      </c>
-      <c r="H92" t="s">
-        <v>150</v>
+        <v>0.80300000000000016</v>
       </c>
     </row>
     <row r="93" spans="1:8">
       <c r="A93" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B93" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C93">
-        <v>112.5</v>
+        <v>141.97999999999999</v>
+      </c>
+      <c r="D93">
+        <v>245.8</v>
       </c>
       <c r="F93">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>41062.5</v>
+        <v>51822.7</v>
       </c>
       <c r="G93">
         <f t="shared" si="1"/>
-        <v>41.0625</v>
+        <v>51.822699999999998</v>
       </c>
     </row>
     <row r="94" spans="1:8">
       <c r="A94" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B94" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C94">
-        <v>28.5</v>
+        <v>459.76800000000003</v>
+      </c>
+      <c r="D94">
+        <v>467.5</v>
       </c>
       <c r="F94">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>10402.5</v>
+        <v>167815.32</v>
       </c>
       <c r="G94">
         <f t="shared" si="1"/>
-        <v>10.4025</v>
+        <v>167.81532000000001</v>
       </c>
     </row>
     <row r="95" spans="1:8">
       <c r="A95" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="B95" t="s">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="C95">
-        <v>7.7</v>
+        <v>0</v>
       </c>
       <c r="F95">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>2810.5</v>
+        <v>0</v>
       </c>
       <c r="G95">
         <f t="shared" si="1"/>
-        <v>2.8105000000000002</v>
+        <v>0</v>
+      </c>
+      <c r="H95" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="96" spans="1:8">
       <c r="A96" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="B96" t="s">
-        <v>29</v>
-      </c>
-      <c r="C96">
-        <v>246.5</v>
+        <v>41</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
       </c>
       <c r="F96">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>89972.5</v>
+        <v>0</v>
       </c>
       <c r="G96">
         <f t="shared" si="1"/>
-        <v>89.972499999999997</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97" spans="1:8">
       <c r="A97" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B97" t="s">
-        <v>29</v>
-      </c>
-      <c r="C97">
-        <v>1246.4000000000001</v>
+        <v>83</v>
+      </c>
+      <c r="E97">
+        <v>30</v>
       </c>
       <c r="F97">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>454936.00000000006</v>
+        <v>10950</v>
       </c>
       <c r="G97">
         <f t="shared" si="1"/>
-        <v>454.93600000000004</v>
+        <v>10.95</v>
+      </c>
+      <c r="H97" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="98" spans="1:8">
       <c r="A98" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B98" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C98">
-        <v>50.883000000000003</v>
+        <v>112.5</v>
       </c>
       <c r="F98">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>18572.295000000002</v>
+        <v>41062.5</v>
       </c>
       <c r="G98">
         <f t="shared" si="1"/>
-        <v>18.572295</v>
+        <v>41.0625</v>
       </c>
     </row>
     <row r="99" spans="1:8">
       <c r="A99" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="B99" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C99">
-        <v>2277.6</v>
-      </c>
-      <c r="D99">
-        <v>1799</v>
+        <v>38.99</v>
       </c>
       <c r="F99">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>656635</v>
+        <v>14231.35</v>
       </c>
       <c r="G99">
         <f t="shared" si="1"/>
-        <v>656.63499999999999</v>
+        <v>14.231350000000001</v>
       </c>
     </row>
     <row r="100" spans="1:8">
       <c r="A100" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="B100" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="C100">
-        <v>1138.0999999999999</v>
+        <v>7.7</v>
       </c>
       <c r="F100">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>415406.49999999994</v>
+        <v>2810.5</v>
       </c>
       <c r="G100">
         <f t="shared" si="1"/>
-        <v>415.40649999999994</v>
-      </c>
-      <c r="H100" t="s">
-        <v>149</v>
+        <v>2.8105000000000002</v>
       </c>
     </row>
     <row r="101" spans="1:8">
       <c r="A101" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B101" t="s">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="C101">
-        <v>497.16</v>
-      </c>
-      <c r="D101">
-        <v>701.8</v>
+        <v>384.8</v>
       </c>
       <c r="F101">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>181463.40000000002</v>
+        <v>140452</v>
       </c>
       <c r="G101">
         <f t="shared" si="1"/>
-        <v>181.46340000000004</v>
+        <v>140.452</v>
       </c>
     </row>
     <row r="102" spans="1:8">
       <c r="A102" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="B102" t="s">
-        <v>47</v>
-      </c>
-      <c r="E102">
-        <v>958.9</v>
+        <v>29</v>
+      </c>
+      <c r="C102">
+        <v>1399</v>
       </c>
       <c r="F102">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>349998.5</v>
+        <v>510635</v>
       </c>
       <c r="G102">
         <f t="shared" si="1"/>
-        <v>349.99849999999998</v>
-      </c>
-      <c r="H102" t="s">
-        <v>144</v>
+        <v>510.63499999999999</v>
       </c>
     </row>
     <row r="103" spans="1:8">
       <c r="A103" t="s">
-        <v>97</v>
+        <v>30</v>
       </c>
       <c r="B103" t="s">
-        <v>47</v>
-      </c>
-      <c r="D103">
-        <v>375</v>
+        <v>29</v>
+      </c>
+      <c r="C103">
+        <v>50.88</v>
       </c>
       <c r="F103">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>136875</v>
+        <v>18571.2</v>
       </c>
       <c r="G103">
         <f t="shared" si="1"/>
-        <v>136.875</v>
-      </c>
-      <c r="H103" t="s">
-        <v>148</v>
+        <v>18.571200000000001</v>
       </c>
     </row>
     <row r="104" spans="1:8">
       <c r="A104" t="s">
+        <v>27</v>
+      </c>
+      <c r="B104" t="s">
         <v>29</v>
       </c>
-      <c r="B104" t="s">
+      <c r="C104">
+        <v>173.94</v>
+      </c>
+      <c r="F104" s="5">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>63488.1</v>
+      </c>
+      <c r="G104">
+        <f>F104/1000</f>
+        <v>63.488099999999996</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8">
+      <c r="A105" t="s">
         <v>39</v>
       </c>
-      <c r="C104">
-        <v>416</v>
-      </c>
-      <c r="D104">
+      <c r="B105" t="s">
+        <v>29</v>
+      </c>
+      <c r="C105">
+        <v>249.6</v>
+      </c>
+      <c r="D105">
+        <v>1799</v>
+      </c>
+      <c r="F105">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>91104</v>
+      </c>
+      <c r="G105">
+        <f t="shared" si="1"/>
+        <v>91.103999999999999</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8">
+      <c r="A106" t="s">
+        <v>50</v>
+      </c>
+      <c r="B106" t="s">
+        <v>51</v>
+      </c>
+      <c r="C106">
+        <v>1154.47</v>
+      </c>
+      <c r="F106">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>421381.55</v>
+      </c>
+      <c r="G106">
+        <f t="shared" si="1"/>
+        <v>421.38155</v>
+      </c>
+      <c r="H106" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8">
+      <c r="A107" t="s">
+        <v>32</v>
+      </c>
+      <c r="B107" t="s">
+        <v>47</v>
+      </c>
+      <c r="D107">
+        <v>701.8</v>
+      </c>
+      <c r="F107">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>256156.99999999997</v>
+      </c>
+      <c r="G107">
+        <f t="shared" si="1"/>
+        <v>256.15699999999998</v>
+      </c>
+      <c r="H107" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8">
+      <c r="A108" t="s">
+        <v>41</v>
+      </c>
+      <c r="B108" t="s">
+        <v>47</v>
+      </c>
+      <c r="E108">
+        <v>958.9</v>
+      </c>
+      <c r="F108">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>349998.5</v>
+      </c>
+      <c r="G108">
+        <f t="shared" si="1"/>
+        <v>349.99849999999998</v>
+      </c>
+      <c r="H108" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8">
+      <c r="A109" t="s">
+        <v>97</v>
+      </c>
+      <c r="B109" t="s">
+        <v>47</v>
+      </c>
+      <c r="D109">
+        <v>375</v>
+      </c>
+      <c r="F109">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>136875</v>
+      </c>
+      <c r="G109">
+        <f t="shared" si="1"/>
+        <v>136.875</v>
+      </c>
+      <c r="H109" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8">
+      <c r="A110" t="s">
+        <v>29</v>
+      </c>
+      <c r="B110" t="s">
+        <v>39</v>
+      </c>
+      <c r="C110">
+        <v>436.8</v>
+      </c>
+      <c r="D110">
         <v>280.8</v>
       </c>
-      <c r="F104">
+      <c r="F110">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>102492</v>
       </c>
-      <c r="G104">
+      <c r="G110">
         <f t="shared" si="1"/>
         <v>102.492</v>
       </c>
     </row>
-    <row r="105" spans="1:8">
-      <c r="A105" t="s">
+    <row r="111" spans="1:8">
+      <c r="A111" t="s">
         <v>34</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B111" t="s">
         <v>39</v>
       </c>
-      <c r="C105">
+      <c r="C111">
         <v>122.2</v>
       </c>
-      <c r="F105">
+      <c r="F111">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>44603</v>
       </c>
-      <c r="G105">
+      <c r="G111">
         <f t="shared" si="1"/>
         <v>44.603000000000002</v>
       </c>
     </row>
-    <row r="106" spans="1:8">
-      <c r="A106" t="s">
+    <row r="112" spans="1:8">
+      <c r="A112" t="s">
         <v>41</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B112" t="s">
         <v>39</v>
       </c>
-      <c r="E106">
+      <c r="E112">
         <v>5459.5088498999994</v>
       </c>
-      <c r="F106">
+      <c r="F112">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>1992720.7302134999</v>
       </c>
-      <c r="G106">
+      <c r="G112">
         <f t="shared" si="1"/>
         <v>1992.7207302134998</v>
       </c>
     </row>
-    <row r="107" spans="1:8">
-      <c r="A107" t="s">
+    <row r="113" spans="1:7">
+      <c r="A113" t="s">
         <v>40</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B113" t="s">
         <v>39</v>
       </c>
-      <c r="E107">
+      <c r="E113">
         <v>80.846503979999994</v>
       </c>
-      <c r="F107">
+      <c r="F113">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>29508.973952699998</v>
       </c>
-      <c r="G107">
+      <c r="G113">
         <f t="shared" si="1"/>
         <v>29.5089739527</v>
       </c>
     </row>
-    <row r="108" spans="1:8">
-      <c r="A108" t="s">
+    <row r="114" spans="1:7">
+      <c r="A114" t="s">
         <v>53</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B114" t="s">
         <v>39</v>
       </c>
-      <c r="E108">
+      <c r="E114">
         <v>35.53171072</v>
       </c>
-      <c r="F108">
+      <c r="F114">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>12969.074412800001</v>
       </c>
-      <c r="G108">
+      <c r="G114">
         <f t="shared" si="1"/>
         <v>12.969074412800001</v>
       </c>
     </row>
-    <row r="109" spans="1:8">
-      <c r="A109" t="s">
+    <row r="115" spans="1:7">
+      <c r="A115" t="s">
         <v>17</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B115" t="s">
         <v>11</v>
       </c>
-      <c r="C109">
+      <c r="C115">
         <v>803.4</v>
       </c>
-      <c r="D109">
+      <c r="D115">
         <v>205.9</v>
       </c>
-      <c r="F109">
+      <c r="F115">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>75153.5</v>
       </c>
-      <c r="G109">
+      <c r="G115">
         <f t="shared" si="1"/>
         <v>75.153499999999994</v>
       </c>
     </row>
-    <row r="110" spans="1:8">
-      <c r="A110" t="s">
+    <row r="116" spans="1:7">
+      <c r="A116" t="s">
         <v>49</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B116" t="s">
         <v>11</v>
       </c>
-      <c r="C110">
+      <c r="C116">
         <v>1499.1</v>
       </c>
-      <c r="D110">
+      <c r="D116">
         <v>1406</v>
       </c>
-      <c r="F110">
+      <c r="F116">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>513190</v>
       </c>
-      <c r="G110">
+      <c r="G116">
         <f t="shared" si="1"/>
         <v>513.19000000000005</v>
       </c>
     </row>
-    <row r="111" spans="1:8">
-      <c r="A111" t="s">
+    <row r="117" spans="1:7">
+      <c r="A117" t="s">
         <v>18</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B117" t="s">
         <v>11</v>
       </c>
-      <c r="C111">
+      <c r="C117">
         <v>494.4</v>
       </c>
-      <c r="F111">
+      <c r="F117">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>180456</v>
       </c>
-      <c r="G111">
+      <c r="G117">
         <f t="shared" si="1"/>
         <v>180.45599999999999</v>
       </c>

</xml_diff>

<commit_message>
add demand for further world regions
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF85F68E-ECFD-472C-BDEE-E1260FD9D93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F1019F-A729-43DD-88B4-109E6B40F1C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="181">
   <si>
     <t>Belgium</t>
   </si>
@@ -336,9 +336,6 @@
     <t>https://gasdashboard.entsog.eu/</t>
   </si>
   <si>
-    <t>AZ</t>
-  </si>
-  <si>
     <t>TK</t>
   </si>
   <si>
@@ -505,6 +502,90 @@
   </si>
   <si>
     <t>not in entsog capacity anymore</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>SA</t>
+  </si>
+  <si>
+    <t>TT</t>
+  </si>
+  <si>
+    <t>ME</t>
+  </si>
+  <si>
+    <t>QA</t>
+  </si>
+  <si>
+    <t>AF</t>
+  </si>
+  <si>
+    <t>AU</t>
+  </si>
+  <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>JS</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>AS</t>
+  </si>
+  <si>
+    <t>North America</t>
+  </si>
+  <si>
+    <t>South America</t>
+  </si>
+  <si>
+    <t>Trinidad &amp; Tobago</t>
+  </si>
+  <si>
+    <t>Middle East</t>
+  </si>
+  <si>
+    <t>Quatar</t>
+  </si>
+  <si>
+    <t>Africa</t>
+  </si>
+  <si>
+    <t>Australia</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>Japan &amp; South Korea</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Asia</t>
+  </si>
+  <si>
+    <t>Mil m3 [2020]</t>
+  </si>
+  <si>
+    <t>Mrd m3 [2020]2</t>
+  </si>
+  <si>
+    <t>CR</t>
+  </si>
+  <si>
+    <t>Caspian Region</t>
+  </si>
+  <si>
+    <t>TAP from TR to GR</t>
   </si>
 </sst>
 </file>
@@ -516,7 +597,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -648,8 +729,16 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -662,8 +751,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -677,6 +778,48 @@
       <top/>
       <bottom style="thin">
         <color indexed="50"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
       </bottom>
       <diagonal/>
     </border>
@@ -738,14 +881,18 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -790,7 +937,95 @@
     <cellStyle name="Percent 4" xfId="35" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
     <cellStyle name="Percent 8" xfId="33" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="26">
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -861,12 +1096,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D3465064-BCEE-4D04-A8E6-DEAE11BBDA92}" name="Country"/>
     <tableColumn id="2" xr3:uid="{D66D54B4-4DED-47C6-BE50-755A236428ED}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="13">
+    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="23">
       <calculatedColumnFormula>Table2[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="12">
+    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="22">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -875,6 +1110,25 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F67" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="8" tableBorderDxfId="9">
+  <autoFilter ref="A53:F67" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{3F684FB4-9656-4C92-BAF4-456019B2B924}" name="Country"/>
+    <tableColumn id="2" xr3:uid="{082B059D-405D-407D-8F97-297DCD23D3B2}" name="Long_name"/>
+    <tableColumn id="3" xr3:uid="{388F462C-127F-4CB7-B46A-1DD19D06D0E8}" name="Mrd m3 [2020]"/>
+    <tableColumn id="4" xr3:uid="{ACDF4345-6201-4524-A8D7-A0CE31D137A6}" name="Mil m3 [2020]"/>
+    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="5">
+      <calculatedColumnFormula>Table7[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="6">
+      <calculatedColumnFormula>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{7149C479-1393-40B9-97BF-B292D48CAD19}" name="Table26" displayName="Table26" ref="A1:F42" totalsRowShown="0">
   <autoFilter ref="A1:F42" xr:uid="{D12A1D17-871E-4E66-A144-F2ADD46C5E00}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C40">
@@ -883,12 +1137,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="9">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="19">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="8">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="18">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -896,7 +1150,26 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F66" totalsRowShown="0" headerRowDxfId="4" headerRowBorderDxfId="2" tableBorderDxfId="3">
+  <autoFilter ref="A52:F66" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
+    <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
+    <tableColumn id="3" xr3:uid="{02819FD0-F6B6-484E-B4DA-8262AECE7052}" name="Mrd m3 [2020]"/>
+    <tableColumn id="4" xr3:uid="{A15C284E-E91C-44C6-B3BB-CC2DD205DA84}" name="Mil m3 [2020]"/>
+    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="1">
+      <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="0">
+      <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}" name="Table1" displayName="Table1" ref="A1:F42" totalsRowShown="0">
   <autoFilter ref="A1:F42" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E41">
@@ -905,12 +1178,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="6">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="16">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="5">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="15">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -918,7 +1191,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9FAAA988-46A0-43D3-858D-474206C07928}" name="Table15" displayName="Table15" ref="A1:F42" totalsRowShown="0">
   <autoFilter ref="A1:F42" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E41">
@@ -927,12 +1200,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="3">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="13">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="2">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="12">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -940,7 +1213,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}" name="Table3" displayName="Table3" ref="A1:H111" totalsRowShown="0">
   <autoFilter ref="A1:H111" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H111">
@@ -952,7 +1225,7 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="1">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="11">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
@@ -964,7 +1237,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FC7F2F97-F859-4A2C-9657-17C35EEFE785}" name="Table37" displayName="Table37" ref="A1:H117" totalsRowShown="0">
   <autoFilter ref="A1:H117" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H117">
@@ -976,7 +1249,7 @@
     <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="0">
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="10">
       <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
@@ -1271,10 +1544,10 @@
         <v>14</v>
       </c>
       <c r="F1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G1" t="s">
         <v>105</v>
-      </c>
-      <c r="G1" t="s">
-        <v>106</v>
       </c>
       <c r="L1" t="s">
         <v>93</v>
@@ -1312,7 +1585,7 @@
         <v>17</v>
       </c>
       <c r="J2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L2" t="str">
         <f>_xlfn.CONCAT(I2,J2)</f>
@@ -1352,7 +1625,7 @@
         <v>25</v>
       </c>
       <c r="J3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L3" t="str">
         <f t="shared" ref="L3:L19" si="2">_xlfn.CONCAT(I3,J3)</f>
@@ -1392,7 +1665,7 @@
         <v>33</v>
       </c>
       <c r="J4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L4" t="str">
         <f t="shared" si="2"/>
@@ -1432,7 +1705,7 @@
         <v>21</v>
       </c>
       <c r="J5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L5" t="str">
         <f t="shared" si="2"/>
@@ -1472,7 +1745,7 @@
         <v>24</v>
       </c>
       <c r="J6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L6" t="str">
         <f t="shared" si="2"/>
@@ -1512,7 +1785,7 @@
         <v>35</v>
       </c>
       <c r="J7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L7" t="str">
         <f t="shared" si="2"/>
@@ -1552,7 +1825,7 @@
         <v>18</v>
       </c>
       <c r="J8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L8" t="str">
         <f t="shared" si="2"/>
@@ -1592,7 +1865,7 @@
         <v>27</v>
       </c>
       <c r="J9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L9" t="str">
         <f t="shared" si="2"/>
@@ -1632,7 +1905,7 @@
         <v>38</v>
       </c>
       <c r="J10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L10" t="str">
         <f t="shared" si="2"/>
@@ -1672,7 +1945,7 @@
         <v>37</v>
       </c>
       <c r="J11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L11" t="str">
         <f t="shared" si="2"/>
@@ -1712,7 +1985,7 @@
         <v>47</v>
       </c>
       <c r="J12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L12" t="str">
         <f t="shared" si="2"/>
@@ -1752,7 +2025,7 @@
         <v>11</v>
       </c>
       <c r="J13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L13" t="str">
         <f t="shared" si="2"/>
@@ -1783,12 +2056,12 @@
         <v>6.8389999999999995</v>
       </c>
       <c r="I14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B15">
         <v>2.5</v>
@@ -1809,7 +2082,7 @@
         <v>54</v>
       </c>
       <c r="J15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L15" t="str">
         <f t="shared" si="2"/>
@@ -1822,7 +2095,7 @@
     </row>
     <row r="16" spans="1:13">
       <c r="A16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B16">
         <v>5</v>
@@ -1843,7 +2116,7 @@
         <v>55</v>
       </c>
       <c r="J16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L16" t="str">
         <f t="shared" si="2"/>
@@ -1856,7 +2129,7 @@
     </row>
     <row r="17" spans="1:13">
       <c r="A17" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B17">
         <v>31.2</v>
@@ -1877,7 +2150,7 @@
         <v>19</v>
       </c>
       <c r="J17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L17" t="str">
         <f t="shared" si="2"/>
@@ -1890,7 +2163,7 @@
     </row>
     <row r="18" spans="1:13">
       <c r="A18" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B18">
         <v>2.6</v>
@@ -1911,7 +2184,7 @@
         <v>44</v>
       </c>
       <c r="J18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L18" t="str">
         <f t="shared" si="2"/>
@@ -1924,7 +2197,7 @@
     </row>
     <row r="19" spans="1:13">
       <c r="A19" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B19">
         <v>1.5</v>
@@ -1945,7 +2218,7 @@
         <v>36</v>
       </c>
       <c r="J19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L19" t="str">
         <f t="shared" si="2"/>
@@ -1963,12 +2236,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF82F4-4954-4D06-9A30-AE8575CA18DE}">
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M67"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" customWidth="1"/>
-    <col min="3" max="7" width="15" customWidth="1"/>
+    <col min="2" max="2" width="19.26953125" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="17.08984375" customWidth="1"/>
+    <col min="5" max="5" width="17.7265625" customWidth="1"/>
+    <col min="6" max="7" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -1982,13 +2258,13 @@
         <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L1" t="s">
         <v>93</v>
@@ -2018,7 +2294,7 @@
       </c>
       <c r="G2" s="2"/>
       <c r="I2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L2" t="str">
         <f t="shared" ref="L2:L40" si="0">_xlfn.CONCAT(A2,$I$2)</f>
@@ -2467,7 +2743,7 @@
         <v>44</v>
       </c>
       <c r="B18" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2">
@@ -3203,7 +3479,7 @@
     </row>
     <row r="47" spans="1:13">
       <c r="A47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -3214,28 +3490,322 @@
         <v>90</v>
       </c>
       <c r="H48" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
       <c r="A49" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B49" t="s">
-        <v>123</v>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="F53" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" t="s">
+        <v>153</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C54" s="7">
+        <v>924.81292668594142</v>
+      </c>
+      <c r="D54" s="7"/>
+      <c r="E54" s="7">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F54" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>9035.4222937216473</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" t="s">
+        <v>154</v>
+      </c>
+      <c r="B55" t="s">
+        <v>165</v>
+      </c>
+      <c r="C55">
+        <f>165.613+35.5252809102083</f>
+        <v>201.13828091020829</v>
+      </c>
+      <c r="E55" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F55" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1965.121004492735</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" t="s">
+        <v>155</v>
+      </c>
+      <c r="B56" t="s">
+        <v>166</v>
+      </c>
+      <c r="C56">
+        <f>156.619145389645-29.4652641615749</f>
+        <v>127.15388122807011</v>
+      </c>
+      <c r="E56" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F56" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1242.2934195982448</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" t="s">
+        <v>156</v>
+      </c>
+      <c r="B57" t="s">
+        <v>167</v>
+      </c>
+      <c r="C57">
+        <v>29.4652641615749</v>
+      </c>
+      <c r="E57" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F57" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>287.87563085858676</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" t="s">
+        <v>157</v>
+      </c>
+      <c r="B58" t="s">
+        <v>168</v>
+      </c>
+      <c r="C58">
+        <f>667.939379731508-174.9348378172</f>
+        <v>493.00454191430799</v>
+      </c>
+      <c r="E58" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>4816.6543745027893</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" t="s">
+        <v>158</v>
+      </c>
+      <c r="B59" t="s">
+        <v>169</v>
+      </c>
+      <c r="C59">
+        <v>174.93483781719999</v>
+      </c>
+      <c r="E59" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1709.1133654740438</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" t="s">
+        <v>159</v>
+      </c>
+      <c r="B60" t="s">
+        <v>170</v>
+      </c>
+      <c r="C60" s="2">
+        <f>231.909048813308-C21-C3-C37</f>
+        <v>135.88472424096241</v>
+      </c>
+      <c r="E60" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F60" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1327.5937558342027</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" t="s">
+        <v>160</v>
+      </c>
+      <c r="B61" t="s">
+        <v>171</v>
+      </c>
+      <c r="C61">
+        <v>145.71638020075315</v>
+      </c>
+      <c r="E61" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F61" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1423.6490345613581</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" t="s">
+        <v>161</v>
+      </c>
+      <c r="B62" t="s">
+        <v>172</v>
+      </c>
+      <c r="C62">
+        <v>194.00921828908548</v>
+      </c>
+      <c r="E62" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F62" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1895.4700626843651</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" t="s">
+        <v>162</v>
+      </c>
+      <c r="B63" t="s">
+        <v>173</v>
+      </c>
+      <c r="C63">
+        <v>0</v>
+      </c>
+      <c r="E63" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F63" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" t="s">
+        <v>163</v>
+      </c>
+      <c r="B64" t="s">
+        <v>174</v>
+      </c>
+      <c r="C64">
+        <v>23.760626555099513</v>
+      </c>
+      <c r="E64" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F64" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>232.14132144332223</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" t="s">
+        <v>164</v>
+      </c>
+      <c r="B65" t="s">
+        <v>175</v>
+      </c>
+      <c r="C65">
+        <f>656.2735508682-C64-C62-C61-C63</f>
+        <v>292.78732582326188</v>
+      </c>
+      <c r="E65" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F65" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2860.5321732932684</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
+      <c r="A66" t="s">
+        <v>178</v>
+      </c>
+      <c r="B66" t="s">
+        <v>179</v>
+      </c>
+      <c r="C66">
+        <f>808.357450256401-638.446656032448</f>
+        <v>169.91079422395296</v>
+      </c>
+      <c r="E66" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F66" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1660.0284595680205</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" t="s">
+        <v>41</v>
+      </c>
+      <c r="B67" t="s">
+        <v>70</v>
+      </c>
+      <c r="C67">
+        <v>638.446656032448</v>
+      </c>
+      <c r="E67" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F67" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>6237.6238294370169</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{036BBBE1-80BC-4BBB-9141-C576056723F9}">
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -3255,13 +3825,13 @@
         <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L1" t="s">
         <v>93</v>
@@ -3291,7 +3861,7 @@
       </c>
       <c r="G2" s="2"/>
       <c r="I2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L2" t="str">
         <f t="shared" ref="L2:L42" si="0">_xlfn.CONCAT(A2,$I$2)</f>
@@ -3740,7 +4310,7 @@
         <v>44</v>
       </c>
       <c r="B18" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2">
@@ -4470,7 +5040,7 @@
     </row>
     <row r="47" spans="1:13">
       <c r="A47" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -4478,24 +5048,318 @@
         <v>80</v>
       </c>
       <c r="B48" t="s">
+        <v>138</v>
+      </c>
+      <c r="H48" t="s">
         <v>139</v>
       </c>
-      <c r="H48" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2">
+    </row>
+    <row r="49" spans="1:6">
       <c r="A49" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B49" t="s">
-        <v>123</v>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="F52" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" t="s">
+        <v>153</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C53" s="7">
+        <v>1035.2966874829399</v>
+      </c>
+      <c r="D53" s="7"/>
+      <c r="E53" s="7">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F53" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>10114.848636708322</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" t="s">
+        <v>154</v>
+      </c>
+      <c r="B54" t="s">
+        <v>165</v>
+      </c>
+      <c r="C54">
+        <f>1261.13549926252-1035.29668748294</f>
+        <v>225.83881177958006</v>
+      </c>
+      <c r="E54" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F54" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2206.4451910864968</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" t="s">
+        <v>155</v>
+      </c>
+      <c r="B55" t="s">
+        <v>166</v>
+      </c>
+      <c r="C55">
+        <f>162.021478179314-24.9936060429938</f>
+        <v>137.02787213632018</v>
+      </c>
+      <c r="E55" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F55" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1338.7623107718482</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" t="s">
+        <v>156</v>
+      </c>
+      <c r="B56" t="s">
+        <v>167</v>
+      </c>
+      <c r="C56">
+        <v>24.9936060429938</v>
+      </c>
+      <c r="E56" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F56" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>244.18753104004941</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" t="s">
+        <v>157</v>
+      </c>
+      <c r="B57" t="s">
+        <v>168</v>
+      </c>
+      <c r="C57">
+        <f>712.704008488226-180.976586566424</f>
+        <v>531.72742192180203</v>
+      </c>
+      <c r="E57" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F57" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>5194.9769121760055</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" t="s">
+        <v>158</v>
+      </c>
+      <c r="B58" t="s">
+        <v>169</v>
+      </c>
+      <c r="C58">
+        <v>180.976586566424</v>
+      </c>
+      <c r="E58" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1768.1412507539624</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" t="s">
+        <v>159</v>
+      </c>
+      <c r="B59" t="s">
+        <v>170</v>
+      </c>
+      <c r="C59" s="2">
+        <f>253.649617284986-C21-C3-C37</f>
+        <v>133.95499124326935</v>
+      </c>
+      <c r="E59" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1308.7402644467415</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" t="s">
+        <v>160</v>
+      </c>
+      <c r="B60" t="s">
+        <v>171</v>
+      </c>
+      <c r="C60">
+        <v>151.74021373996112</v>
+      </c>
+      <c r="E60" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F60" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1482.5018882394202</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" t="s">
+        <v>161</v>
+      </c>
+      <c r="B61" t="s">
+        <v>172</v>
+      </c>
+      <c r="C61">
+        <v>234.25835791543756</v>
+      </c>
+      <c r="E61" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F61" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2288.704156833825</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" t="s">
+        <v>162</v>
+      </c>
+      <c r="B62" t="s">
+        <v>173</v>
+      </c>
+      <c r="C62">
+        <v>0</v>
+      </c>
+      <c r="E62" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F62" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" t="s">
+        <v>163</v>
+      </c>
+      <c r="B63" t="s">
+        <v>174</v>
+      </c>
+      <c r="C63">
+        <v>31.585488535476742</v>
+      </c>
+      <c r="E63" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F63" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>308.59022299160773</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" t="s">
+        <v>164</v>
+      </c>
+      <c r="B64" t="s">
+        <v>175</v>
+      </c>
+      <c r="C64">
+        <f>691.83903700697-C63-C61-C60-C62</f>
+        <v>274.25497681609454</v>
+      </c>
+      <c r="E64" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F64" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2679.4711234932433</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" t="s">
+        <v>178</v>
+      </c>
+      <c r="B65" t="s">
+        <v>179</v>
+      </c>
+      <c r="C65">
+        <f>773.5530598751-586.382199872419</f>
+        <v>187.17086000268091</v>
+      </c>
+      <c r="E65" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F65" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1828.6593022261925</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
+      <c r="A66" t="s">
+        <v>41</v>
+      </c>
+      <c r="B66" t="s">
+        <v>70</v>
+      </c>
+      <c r="C66">
+        <v>586.38219987241905</v>
+      </c>
+      <c r="E66" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F66" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>5728.9540927535336</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4523,13 +5387,13 @@
         <v>85</v>
       </c>
       <c r="D1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -4948,7 +5812,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B21" t="s">
         <v>92</v>
@@ -4988,7 +5852,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="B23" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23">
@@ -5376,10 +6240,10 @@
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
+        <v>110</v>
+      </c>
+      <c r="B41" t="s">
         <v>111</v>
-      </c>
-      <c r="B41" t="s">
-        <v>112</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41">
@@ -5396,7 +6260,7 @@
     </row>
     <row r="42" spans="1:6">
       <c r="B42" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42">
@@ -5413,28 +6277,28 @@
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" t="s">
+        <v>115</v>
+      </c>
+      <c r="B52" t="s">
         <v>116</v>
-      </c>
-      <c r="B52" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" t="s">
+        <v>117</v>
+      </c>
+      <c r="B53" t="s">
         <v>118</v>
-      </c>
-      <c r="B53" t="s">
-        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -5465,16 +6329,16 @@
         <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -5893,7 +6757,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B21" t="s">
         <v>92</v>
@@ -5933,7 +6797,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="B23" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23">
@@ -6321,10 +7185,10 @@
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
+        <v>110</v>
+      </c>
+      <c r="B41" t="s">
         <v>111</v>
-      </c>
-      <c r="B41" t="s">
-        <v>112</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41">
@@ -6341,7 +7205,7 @@
     </row>
     <row r="42" spans="1:6">
       <c r="B42" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42">
@@ -6358,28 +7222,28 @@
     </row>
     <row r="50" spans="1:2">
       <c r="A50" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52" t="s">
+        <v>115</v>
+      </c>
+      <c r="B52" t="s">
         <v>116</v>
-      </c>
-      <c r="B52" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53" t="s">
+        <v>117</v>
+      </c>
+      <c r="B53" t="s">
         <v>118</v>
-      </c>
-      <c r="B53" t="s">
-        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -6410,22 +7274,22 @@
         <v>94</v>
       </c>
       <c r="C1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" t="s">
         <v>141</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>142</v>
       </c>
-      <c r="E1" t="s">
-        <v>143</v>
-      </c>
       <c r="F1" t="s">
+        <v>107</v>
+      </c>
+      <c r="G1" t="s">
         <v>108</v>
       </c>
-      <c r="G1" t="s">
-        <v>109</v>
-      </c>
       <c r="H1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -6447,7 +7311,7 @@
         <v>177.79150000000001</v>
       </c>
       <c r="H2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -7123,7 +7987,7 @@
     </row>
     <row r="38" spans="1:7">
       <c r="A38" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B38" t="s">
         <v>37</v>
@@ -7494,7 +8358,7 @@
         <v>0</v>
       </c>
       <c r="H56" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -7783,7 +8647,7 @@
         <v>50</v>
       </c>
       <c r="B71" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D71">
         <v>442.8</v>
@@ -7797,7 +8661,7 @@
         <v>161.62200000000001</v>
       </c>
       <c r="H71" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -8223,7 +9087,7 @@
         <v>10.95</v>
       </c>
       <c r="H92" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -8381,7 +9245,7 @@
         <v>415.40649999999994</v>
       </c>
       <c r="H100" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="101" spans="1:8">
@@ -8425,12 +9289,12 @@
         <v>349.99849999999998</v>
       </c>
       <c r="H102" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="103" spans="1:8">
       <c r="A103" t="s">
-        <v>97</v>
+        <v>178</v>
       </c>
       <c r="B103" t="s">
         <v>47</v>
@@ -8447,7 +9311,7 @@
         <v>127.71349999999998</v>
       </c>
       <c r="H103" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="104" spans="1:8">
@@ -8640,22 +9504,22 @@
         <v>94</v>
       </c>
       <c r="C1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D1" t="s">
         <v>141</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>142</v>
       </c>
-      <c r="E1" t="s">
-        <v>143</v>
-      </c>
       <c r="F1" t="s">
+        <v>107</v>
+      </c>
+      <c r="G1" t="s">
         <v>108</v>
       </c>
-      <c r="G1" t="s">
-        <v>109</v>
-      </c>
       <c r="H1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -8677,7 +9541,7 @@
         <v>177.79150000000001</v>
       </c>
       <c r="H2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -9152,7 +10016,7 @@
       <c r="C27">
         <v>100</v>
       </c>
-      <c r="F27" s="5">
+      <c r="F27">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>36500</v>
       </c>
@@ -9288,7 +10152,7 @@
       <c r="C34">
         <v>91.2</v>
       </c>
-      <c r="F34" s="5">
+      <c r="F34">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>33288</v>
       </c>
@@ -9339,7 +10203,7 @@
       <c r="B37" t="s">
         <v>54</v>
       </c>
-      <c r="C37" s="6">
+      <c r="C37" s="5">
         <v>78</v>
       </c>
       <c r="E37">
@@ -9394,7 +10258,7 @@
     </row>
     <row r="40" spans="1:7">
       <c r="A40" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B40" t="s">
         <v>37</v>
@@ -9879,7 +10743,7 @@
         <v>421.21</v>
       </c>
       <c r="H64" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -9901,7 +10765,7 @@
         <v>180.20050000000001</v>
       </c>
       <c r="H65" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -9942,7 +10806,7 @@
         <v>118.77099999999999</v>
       </c>
       <c r="H67" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -10048,7 +10912,7 @@
         <v>50</v>
       </c>
       <c r="B73" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D73">
         <v>31.92</v>
@@ -10062,7 +10926,7 @@
         <v>11.6508</v>
       </c>
       <c r="H73" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -10233,7 +11097,7 @@
       <c r="C82">
         <v>321.60000000000002</v>
       </c>
-      <c r="F82" s="5">
+      <c r="F82">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>117384.00000000001</v>
       </c>
@@ -10271,7 +11135,7 @@
       <c r="C84">
         <v>58.069200000000002</v>
       </c>
-      <c r="F84" s="5">
+      <c r="F84">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>21195.258000000002</v>
       </c>
@@ -10290,7 +11154,7 @@
       <c r="C85">
         <v>144.50399999999999</v>
       </c>
-      <c r="F85" s="5">
+      <c r="F85">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>52743.96</v>
       </c>
@@ -10318,7 +11182,7 @@
         <v>49.494</v>
       </c>
       <c r="H86" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="87" spans="1:8">
@@ -10340,7 +11204,7 @@
         <v>0</v>
       </c>
       <c r="H87" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -10422,7 +11286,7 @@
         <v>0</v>
       </c>
       <c r="H91" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -10507,7 +11371,7 @@
         <v>0</v>
       </c>
       <c r="H95" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="96" spans="1:8">
@@ -10548,7 +11412,7 @@
         <v>10.95</v>
       </c>
       <c r="H97" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -10675,7 +11539,7 @@
       <c r="C104">
         <v>173.94</v>
       </c>
-      <c r="F104" s="5">
+      <c r="F104">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>63488.1</v>
       </c>
@@ -10725,7 +11589,7 @@
         <v>421.38155</v>
       </c>
       <c r="H106" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="107" spans="1:8">
@@ -10747,7 +11611,7 @@
         <v>256.15699999999998</v>
       </c>
       <c r="H107" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="108" spans="1:8">
@@ -10769,12 +11633,12 @@
         <v>349.99849999999998</v>
       </c>
       <c r="H108" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="109" spans="1:8">
       <c r="A109" t="s">
-        <v>97</v>
+        <v>178</v>
       </c>
       <c r="B109" t="s">
         <v>47</v>
@@ -10791,7 +11655,7 @@
         <v>136.875</v>
       </c>
       <c r="H109" t="s">
-        <v>148</v>
+        <v>180</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -10979,10 +11843,10 @@
         <v>95</v>
       </c>
       <c r="D1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" t="s">
         <v>108</v>
-      </c>
-      <c r="E1" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -11006,10 +11870,10 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
+        <v>178</v>
+      </c>
+      <c r="B3" t="s">
         <v>97</v>
-      </c>
-      <c r="B3" t="s">
-        <v>98</v>
       </c>
       <c r="C3">
         <v>395</v>
@@ -11254,7 +12118,7 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B16" t="s">
         <v>37</v>
@@ -11371,7 +12235,7 @@
         <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C22">
         <v>385</v>
@@ -11463,7 +12327,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B27" t="s">
         <v>33</v>
@@ -11485,7 +12349,7 @@
         <v>50</v>
       </c>
       <c r="B28" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C28">
         <f>C15</f>
@@ -11500,7 +12364,7 @@
         <v>123.04150000000001</v>
       </c>
       <c r="F28" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -11522,7 +12386,7 @@
         <v>421.21</v>
       </c>
       <c r="F29" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -11544,7 +12408,7 @@
         <v>14.965</v>
       </c>
       <c r="F30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -11555,7 +12419,7 @@
         <v>53</v>
       </c>
       <c r="F31" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -11577,7 +12441,7 @@
         <v>117.49349999999998</v>
       </c>
       <c r="F33" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -11599,7 +12463,7 @@
         <v>117.49349999999998</v>
       </c>
       <c r="F34" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37" spans="1:6">

</xml_diff>

<commit_message>
add production for further world regions
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F1019F-A729-43DD-88B4-109E6B40F1C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6817EC08-3183-4381-9A7B-AF9246AFDA86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,8 @@
     <sheet name="nodes_demand_2023" sheetId="6" r:id="rId5"/>
     <sheet name="Connections_2021" sheetId="4" r:id="rId6"/>
     <sheet name="Connections_2024" sheetId="8" r:id="rId7"/>
-    <sheet name="Import_Connections" sheetId="5" r:id="rId8"/>
+    <sheet name="Import_Connections_EU" sheetId="5" r:id="rId8"/>
+    <sheet name="Sheet1" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="186">
   <si>
     <t>Belgium</t>
   </si>
@@ -586,6 +587,21 @@
   </si>
   <si>
     <t>TAP from TR to GR</t>
+  </si>
+  <si>
+    <t>Qatar</t>
+  </si>
+  <si>
+    <t>Morroco</t>
+  </si>
+  <si>
+    <t>https://www.gecf.org/_resources/files/events/release-of-the-gecf-annual-statistical-bulletin-2023/gecf-asb-2023.pdf</t>
+  </si>
+  <si>
+    <t>EG</t>
+  </si>
+  <si>
+    <t>Egypt</t>
   </si>
 </sst>
 </file>
@@ -881,18 +897,19 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -937,7 +954,19 @@
     <cellStyle name="Percent 4" xfId="35" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
     <cellStyle name="Percent 8" xfId="33" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="36">
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -983,10 +1012,24 @@
       </fill>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1027,6 +1070,30 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -1063,6 +1130,44 @@
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
@@ -1096,12 +1201,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D3465064-BCEE-4D04-A8E6-DEAE11BBDA92}" name="Country"/>
     <tableColumn id="2" xr3:uid="{D66D54B4-4DED-47C6-BE50-755A236428ED}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="25"/>
-    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="23">
+    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="35"/>
+    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="34"/>
+    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="33">
       <calculatedColumnFormula>Table2[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="22">
+    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="32">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1109,19 +1214,43 @@
 </table>
 </file>
 
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FC7F2F97-F859-4A2C-9657-17C35EEFE785}" name="Table37" displayName="Table37" ref="A1:H126" totalsRowShown="0">
+  <autoFilter ref="A1:H126" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H117">
+    <sortCondition ref="B1:B117"/>
+  </sortState>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{F94559DC-2602-4FF1-9531-3B8A374512C0}" name="From"/>
+    <tableColumn id="2" xr3:uid="{C59F5B7E-5BA7-48FA-B638-C3CA1C390D23}" name="To"/>
+    <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
+    <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
+    <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="17">
+      <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
+      <calculatedColumnFormula>F2/1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{18E94D69-5388-4B9B-8C8E-7A29BC79BE42}" name="Comment"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F67" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="8" tableBorderDxfId="9">
-  <autoFilter ref="A53:F67" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F68" totalsRowShown="0" headerRowDxfId="31" headerRowBorderDxfId="30" tableBorderDxfId="29">
+  <autoFilter ref="A53:F68" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3F684FB4-9656-4C92-BAF4-456019B2B924}" name="Country"/>
     <tableColumn id="2" xr3:uid="{082B059D-405D-407D-8F97-297DCD23D3B2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{388F462C-127F-4CB7-B46A-1DD19D06D0E8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{ACDF4345-6201-4524-A8D7-A0CE31D137A6}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="5">
-      <calculatedColumnFormula>Table7[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
+    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="1">
+      <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="6">
-      <calculatedColumnFormula>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="0">
+      <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1137,12 +1266,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="19">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="26">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="18">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="25">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1151,17 +1280,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F66" totalsRowShown="0" headerRowDxfId="4" headerRowBorderDxfId="2" tableBorderDxfId="3">
-  <autoFilter ref="A52:F66" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F67" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="11" tableBorderDxfId="12">
+  <autoFilter ref="A52:F67" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{02819FD0-F6B6-484E-B4DA-8262AECE7052}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{A15C284E-E91C-44C6-B3BB-CC2DD205DA84}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="1">
+    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="10">
       <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="9">
       <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1178,12 +1307,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="16">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="23">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="15">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="22">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1192,6 +1321,25 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F76" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="14" tableBorderDxfId="15">
+  <autoFilter ref="A57:F76" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{555371BF-8030-4257-9852-212E94829B9B}" name="Country"/>
+    <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
+    <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2020]"/>
+    <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2020]"/>
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="3">
+      <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="2">
+      <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{9FAAA988-46A0-43D3-858D-474206C07928}" name="Table15" displayName="Table15" ref="A1:F42" totalsRowShown="0">
   <autoFilter ref="A1:F42" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E41">
@@ -1200,12 +1348,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="13">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="20">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="12">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="19">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1213,9 +1361,28 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}" name="Table3" displayName="Table3" ref="A1:H111" totalsRowShown="0">
-  <autoFilter ref="A1:H111" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F76" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7">
+  <autoFilter ref="A57:F76" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
+    <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
+    <tableColumn id="3" xr3:uid="{779C3748-4ECD-495F-809A-B5DD28F5EC2F}" name="Mrd m3 [2020]"/>
+    <tableColumn id="4" xr3:uid="{94BC7314-C5A0-4AAD-895B-84E7A94D7CF7}" name="Mil m3 [2020]"/>
+    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="5">
+      <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="4">
+      <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}" name="Table3" displayName="Table3" ref="A1:H120" totalsRowShown="0">
+  <autoFilter ref="A1:H120" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H111">
     <sortCondition ref="B1:B111"/>
   </sortState>
@@ -1225,37 +1392,13 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="11">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="18">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
       <calculatedColumnFormula>F2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{E4B126C2-804B-4928-BF8B-8FE6229310A1}" name="Comment"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FC7F2F97-F859-4A2C-9657-17C35EEFE785}" name="Table37" displayName="Table37" ref="A1:H117" totalsRowShown="0">
-  <autoFilter ref="A1:H117" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H117">
-    <sortCondition ref="B1:B117"/>
-  </sortState>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{F94559DC-2602-4FF1-9531-3B8A374512C0}" name="From"/>
-    <tableColumn id="2" xr3:uid="{C59F5B7E-5BA7-48FA-B638-C3CA1C390D23}" name="To"/>
-    <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
-    <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
-    <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="10">
-      <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
-      <calculatedColumnFormula>F2/1000</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="8" xr3:uid="{18E94D69-5388-4B9B-8C8E-7A29BC79BE42}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2236,7 +2379,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF82F4-4954-4D06-9A30-AE8575CA18DE}">
-  <dimension ref="A1:M67"/>
+  <dimension ref="A1:M68"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -3533,12 +3676,12 @@
       </c>
       <c r="D54" s="7"/>
       <c r="E54" s="7">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>9035.4222937216473</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2206.4451910864968</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -3553,12 +3696,12 @@
         <v>201.13828091020829</v>
       </c>
       <c r="E55" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F55" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1965.121004492735</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1338.7623107718482</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -3573,12 +3716,12 @@
         <v>127.15388122807011</v>
       </c>
       <c r="E56" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F56" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1242.2934195982448</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>244.18753104004941</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -3592,12 +3735,12 @@
         <v>29.4652641615749</v>
       </c>
       <c r="E57" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F57" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>287.87563085858676</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>5194.9769121760055</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -3612,12 +3755,12 @@
         <v>493.00454191430799</v>
       </c>
       <c r="E58" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F58" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>4816.6543745027893</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1768.1412507539624</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -3631,12 +3774,12 @@
         <v>174.93483781719999</v>
       </c>
       <c r="E59" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F59" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1709.1133654740438</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>750.8692287163949</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -3647,16 +3790,16 @@
         <v>170</v>
       </c>
       <c r="C60" s="2">
-        <f>231.909048813308-C21-C3-C37</f>
-        <v>135.88472424096241</v>
+        <f>231.909048813308-C21-C3-C37-C68</f>
+        <v>77.419550083247572</v>
       </c>
       <c r="E60" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F60" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1327.5937558342027</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1482.5018882394202</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -3670,12 +3813,12 @@
         <v>145.71638020075315</v>
       </c>
       <c r="E61" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F61" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1423.6490345613581</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2288.704156833825</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -3689,12 +3832,12 @@
         <v>194.00921828908548</v>
       </c>
       <c r="E62" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F62" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1895.4700626843651</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -3708,12 +3851,12 @@
         <v>0</v>
       </c>
       <c r="E63" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F63" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>0</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>308.59022299160773</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -3727,12 +3870,12 @@
         <v>23.760626555099513</v>
       </c>
       <c r="E64" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F64" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>232.14132144332223</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2679.4711234932433</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -3747,12 +3890,12 @@
         <v>292.78732582326188</v>
       </c>
       <c r="E65" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F65" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2860.5321732932684</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1828.6593022261925</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -3767,12 +3910,12 @@
         <v>169.91079422395296</v>
       </c>
       <c r="E66" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F66" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1660.0284595680205</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>5728.9540927535336</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -3786,12 +3929,31 @@
         <v>638.446656032448</v>
       </c>
       <c r="E67" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F67" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>6237.6238294370169</v>
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>557.87103573034665</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" t="s">
+        <v>184</v>
+      </c>
+      <c r="B68" t="s">
+        <v>185</v>
+      </c>
+      <c r="C68">
+        <v>58.465174157714841</v>
+      </c>
+      <c r="E68" s="2" t="e">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F68" s="3" t="e">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>#VALUE!</v>
       </c>
     </row>
   </sheetData>
@@ -3805,13 +3967,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{036BBBE1-80BC-4BBB-9141-C576056723F9}">
-  <dimension ref="A1:M66"/>
+  <dimension ref="A1:M67"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
     <col min="2" max="2" width="12.54296875" customWidth="1"/>
     <col min="3" max="7" width="15" customWidth="1"/>
     <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="15.453125" customWidth="1"/>
+    <col min="16" max="16" width="18.1796875" customWidth="1"/>
+    <col min="17" max="17" width="14.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -5208,8 +5373,8 @@
         <v>170</v>
       </c>
       <c r="C59" s="2">
-        <f>253.649617284986-C21-C3-C37</f>
-        <v>133.95499124326935</v>
+        <f>253.649617284986-C21-C3-C37-C67</f>
+        <v>76.854578169538883</v>
       </c>
       <c r="E59" s="2">
         <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
@@ -5217,7 +5382,7 @@
       </c>
       <c r="F59" s="3">
         <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1308.7402644467415</v>
+        <v>750.8692287163949</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -5353,6 +5518,25 @@
       <c r="F66" s="3">
         <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
         <v>5728.9540927535336</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" t="s">
+        <v>184</v>
+      </c>
+      <c r="B67" t="s">
+        <v>185</v>
+      </c>
+      <c r="C67">
+        <v>57.100413073730465</v>
+      </c>
+      <c r="E67" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F67" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>557.87103573034665</v>
       </c>
     </row>
   </sheetData>
@@ -5366,7 +5550,1363 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE55996C-4401-4161-B17D-CF2A8462856A}">
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:H80"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="9.54296875" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="22.26953125" customWidth="1"/>
+    <col min="14" max="14" width="11.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>2846</v>
+      </c>
+      <c r="F2">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</f>
+        <v>-7.7179334425266708</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C3" s="2">
+        <v>8.5272482121300026</v>
+      </c>
+      <c r="D3">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-83.31121503251012</v>
+      </c>
+      <c r="E3">
+        <v>8901.1</v>
+      </c>
+      <c r="F3">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E3/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2">
+        <v>16.998179999999998</v>
+      </c>
+      <c r="D4">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-166.07221859999999</v>
+      </c>
+      <c r="E4">
+        <v>11549.9</v>
+      </c>
+      <c r="F4">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E4/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>3492</v>
+      </c>
+      <c r="F5">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E5/$E$27),0)</f>
+        <v>-9.4697904361571084</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C6" s="2">
+        <v>2.9206500000000002</v>
+      </c>
+      <c r="D6">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-28.534750500000001</v>
+      </c>
+      <c r="E6">
+        <v>6951.5</v>
+      </c>
+      <c r="F6">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E6/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2.9368094170890702</v>
+      </c>
+      <c r="D7">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-28.692628004960213</v>
+      </c>
+      <c r="E7">
+        <v>4058.2</v>
+      </c>
+      <c r="F7">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E7/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="2">
+        <v>8.4623749999999998</v>
+      </c>
+      <c r="D8">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-82.677403749999996</v>
+      </c>
+      <c r="E8">
+        <v>10693.9</v>
+      </c>
+      <c r="F8">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E8/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2.3225881808696536</v>
+      </c>
+      <c r="D9">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-22.691686527096515</v>
+      </c>
+      <c r="E9">
+        <v>5822.8</v>
+      </c>
+      <c r="F9">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E9/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.43005000000000004</v>
+      </c>
+      <c r="D10">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-4.2015885000000006</v>
+      </c>
+      <c r="E10">
+        <v>1329</v>
+      </c>
+      <c r="F10">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E10/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2.0718055555555557</v>
+      </c>
+      <c r="D11">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-20.241540277777776</v>
+      </c>
+      <c r="E11">
+        <v>5525.3</v>
+      </c>
+      <c r="F11">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E11/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" s="2">
+        <v>40.582840274999995</v>
+      </c>
+      <c r="D12">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-396.49434948674991</v>
+      </c>
+      <c r="E12">
+        <v>67098.8</v>
+      </c>
+      <c r="F12">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E12/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" s="2">
+        <v>87.107500000000002</v>
+      </c>
+      <c r="D13">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-851.04027499999995</v>
+      </c>
+      <c r="E13">
+        <v>83166.7</v>
+      </c>
+      <c r="F13">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E13/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="2">
+        <v>6.3426600000000004</v>
+      </c>
+      <c r="D14">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-61.967788200000001</v>
+      </c>
+      <c r="E14">
+        <v>10709.7</v>
+      </c>
+      <c r="F14">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E14/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="2">
+        <v>10.192972222222224</v>
+      </c>
+      <c r="D15">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-99.585338611111126</v>
+      </c>
+      <c r="E15">
+        <v>9769.5</v>
+      </c>
+      <c r="F15">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E15/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" t="s">
+        <v>75</v>
+      </c>
+      <c r="C16" s="2">
+        <v>5.3080830939788495</v>
+      </c>
+      <c r="D16">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-51.859971828173357</v>
+      </c>
+      <c r="E16">
+        <v>4963.8</v>
+      </c>
+      <c r="F16">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E16/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="2">
+        <v>67.625157295559788</v>
+      </c>
+      <c r="D17">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-660.69778677761906</v>
+      </c>
+      <c r="E17">
+        <v>60244.6</v>
+      </c>
+      <c r="F17">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E17/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" s="2">
+        <v>1.0731875</v>
+      </c>
+      <c r="D18">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-10.485041874999999</v>
+      </c>
+      <c r="E18">
+        <v>1907.7</v>
+      </c>
+      <c r="F18">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E18/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="2">
+        <v>2.3604840000000005</v>
+      </c>
+      <c r="D19">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-23.061928680000005</v>
+      </c>
+      <c r="E19">
+        <v>2794.1</v>
+      </c>
+      <c r="F19">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E19/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" s="2">
+        <v>0.722536175</v>
+      </c>
+      <c r="D20">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-7.0591784297499993</v>
+      </c>
+      <c r="E20">
+        <v>626.1</v>
+      </c>
+      <c r="F20">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E20/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" t="s">
+        <v>92</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>514.6</v>
+      </c>
+      <c r="F21">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E21/$E$27),0)</f>
+        <v>-1.395519518455455</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>2579</v>
+      </c>
+      <c r="F22">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E22/$E$27),0)</f>
+        <v>-6.9938687098651737</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="B23" t="s">
+        <v>113</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>621.9</v>
+      </c>
+      <c r="F23">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E23/$E$27),0)</f>
+        <v>-1.6865013379857121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="2">
+        <v>36.094444444444456</v>
+      </c>
+      <c r="D24">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-352.64272222222229</v>
+      </c>
+      <c r="E24">
+        <v>17407.599999999999</v>
+      </c>
+      <c r="F24">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E24/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>46</v>
+      </c>
+      <c r="B25" t="s">
+        <v>77</v>
+      </c>
+      <c r="C25" s="2">
+        <v>0.324946535664</v>
+      </c>
+      <c r="D25">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-3.1747276534372797</v>
+      </c>
+      <c r="E25">
+        <v>2076.3000000000002</v>
+      </c>
+      <c r="F25">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E25/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" t="s">
+        <v>72</v>
+      </c>
+      <c r="C26" s="2">
+        <v>4.4535245861624997</v>
+      </c>
+      <c r="D26">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-43.510935206807623</v>
+      </c>
+      <c r="E26">
+        <v>5367.6</v>
+      </c>
+      <c r="F26">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E26/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" s="2">
+        <v>5.4542940093096091</v>
+      </c>
+      <c r="D27">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-53.28845247095488</v>
+      </c>
+      <c r="E27">
+        <f>SUMIF(D2:D26,"=0",E2:E26)+SUMIF(D28:D42,"=0",E28:E42)</f>
+        <v>19650.2</v>
+      </c>
+      <c r="F27">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E27/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" s="2">
+        <v>21.064583333333339</v>
+      </c>
+      <c r="D28">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-205.80097916666671</v>
+      </c>
+      <c r="E28">
+        <v>37958.1</v>
+      </c>
+      <c r="F28">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E28/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>38</v>
+      </c>
+      <c r="B29" t="s">
+        <v>1</v>
+      </c>
+      <c r="C29" s="2">
+        <v>6.0366596174639984</v>
+      </c>
+      <c r="D29">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-58.978164462623262</v>
+      </c>
+      <c r="E29">
+        <v>10295.9</v>
+      </c>
+      <c r="F29">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E29/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" s="2">
+        <v>11.262552972222222</v>
+      </c>
+      <c r="D30">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-110.03514253861111</v>
+      </c>
+      <c r="E30">
+        <v>19318</v>
+      </c>
+      <c r="F30">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E30/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" t="s">
+        <v>78</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+      <c r="F31">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E31/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" s="2"/>
+      <c r="D32">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+      <c r="E32">
+        <v>6926.7</v>
+      </c>
+      <c r="F32">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E32/$E$27),0)</f>
+        <v>-18.784191699349783</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" s="2">
+        <v>4.754638388888889</v>
+      </c>
+      <c r="D33">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-46.452817059444442</v>
+      </c>
+      <c r="E33">
+        <v>5457.9</v>
+      </c>
+      <c r="F33">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E33/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B34" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" s="2">
+        <v>0.85516059371380015</v>
+      </c>
+      <c r="D34">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-8.354919000583827</v>
+      </c>
+      <c r="E34">
+        <v>2095.9</v>
+      </c>
+      <c r="F34">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E34/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="2">
+        <v>32.490230910000008</v>
+      </c>
+      <c r="D35">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-317.42955599070007</v>
+      </c>
+      <c r="E35">
+        <v>47330</v>
+      </c>
+      <c r="F35">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E35/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" t="s">
+        <v>83</v>
+      </c>
+      <c r="B36" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" s="2">
+        <v>0.99092500000000006</v>
+      </c>
+      <c r="D36">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-9.6813372500000003</v>
+      </c>
+      <c r="E36">
+        <v>10327.6</v>
+      </c>
+      <c r="F36">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E36/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" t="s">
+        <v>22</v>
+      </c>
+      <c r="B37" t="s">
+        <v>59</v>
+      </c>
+      <c r="C37" s="2">
+        <v>3.3147222222222226</v>
+      </c>
+      <c r="D37">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-32.384836111111113</v>
+      </c>
+      <c r="E37">
+        <v>8606</v>
+      </c>
+      <c r="F37">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E37/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" t="s">
+        <v>47</v>
+      </c>
+      <c r="B38" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="2">
+        <v>46.209907500000007</v>
+      </c>
+      <c r="D38">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-451.47079627500005</v>
+      </c>
+      <c r="E38">
+        <v>83155</v>
+      </c>
+      <c r="F38">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E38/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" t="s">
+        <v>11</v>
+      </c>
+      <c r="B39" t="s">
+        <v>11</v>
+      </c>
+      <c r="C39" s="2">
+        <v>73.145389499999993</v>
+      </c>
+      <c r="D39">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-714.63045541499991</v>
+      </c>
+      <c r="E39">
+        <v>67025.5</v>
+      </c>
+      <c r="F39">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E39/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>68</v>
+      </c>
+      <c r="C40" s="2">
+        <v>29.338741396263522</v>
+      </c>
+      <c r="D40">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>-286.63950344149458</v>
+      </c>
+      <c r="E40">
+        <v>41733</v>
+      </c>
+      <c r="F40">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E40/$E$27),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" t="s">
+        <v>110</v>
+      </c>
+      <c r="B41" t="s">
+        <v>111</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>888</v>
+      </c>
+      <c r="F41">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E41/$E$27),0)</f>
+        <v>-2.4081254030090244</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="B42" t="s">
+        <v>119</v>
+      </c>
+      <c r="C42" s="2"/>
+      <c r="D42">
+        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <v>0</v>
+      </c>
+      <c r="E42">
+        <v>1782</v>
+      </c>
+      <c r="F42">
+        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E42/$E$27),0)</f>
+        <v>-4.8325219236059471</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" t="s">
+        <v>115</v>
+      </c>
+      <c r="B52" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" t="s">
+        <v>117</v>
+      </c>
+      <c r="B53" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="F57" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" t="s">
+        <v>153</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C58" s="7">
+        <v>834.54962782115695</v>
+      </c>
+      <c r="D58" s="7"/>
+      <c r="E58" s="7">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>8660.7846598998185</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" t="s">
+        <v>154</v>
+      </c>
+      <c r="B59" t="s">
+        <v>165</v>
+      </c>
+      <c r="C59">
+        <f>1042.08498320178-834.549627821157</f>
+        <v>207.53535538062306</v>
+      </c>
+      <c r="E59" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2132.7907642308792</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" t="s">
+        <v>155</v>
+      </c>
+      <c r="B60" t="s">
+        <v>166</v>
+      </c>
+      <c r="C60">
+        <f>148.570059919613-15.1856471767803</f>
+        <v>133.38441274283269</v>
+      </c>
+      <c r="E60" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F60" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1438.139604719081</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" t="s">
+        <v>156</v>
+      </c>
+      <c r="B61" t="s">
+        <v>167</v>
+      </c>
+      <c r="C61">
+        <f>15.1856471767803</f>
+        <v>15.1856471767803</v>
+      </c>
+      <c r="E61" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F61" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>141.70363816030851</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" t="s">
+        <v>157</v>
+      </c>
+      <c r="B62" t="s">
+        <v>168</v>
+      </c>
+      <c r="C62" s="2">
+        <f>552.897499957585-38.4132347090566</f>
+        <v>514.48426524852835</v>
+      </c>
+      <c r="E62" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F62" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>5212.4455255534276</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" t="s">
+        <v>158</v>
+      </c>
+      <c r="B63" t="s">
+        <v>181</v>
+      </c>
+      <c r="C63">
+        <v>38.413234709056603</v>
+      </c>
+      <c r="E63" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F63" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>431.84687643593901</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" t="s">
+        <v>159</v>
+      </c>
+      <c r="B64" t="s">
+        <v>170</v>
+      </c>
+      <c r="C64" s="2">
+        <f>154.184349315883-C72-C73-C74-C75-C76</f>
+        <v>40.449273476568081</v>
+      </c>
+      <c r="E64" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F64" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>458.53340662554189</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" t="s">
+        <v>160</v>
+      </c>
+      <c r="B65" t="s">
+        <v>171</v>
+      </c>
+      <c r="C65">
+        <v>42.317339828787539</v>
+      </c>
+      <c r="E65" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F65" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>391.98708472127618</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" t="s">
+        <v>161</v>
+      </c>
+      <c r="B66" t="s">
+        <v>172</v>
+      </c>
+      <c r="C66">
+        <v>336.61725663716805</v>
+      </c>
+      <c r="E66" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F66" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>4002.6213997252307</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
+      <c r="A67" t="s">
+        <v>162</v>
+      </c>
+      <c r="B67" t="s">
+        <v>173</v>
+      </c>
+      <c r="C67">
+        <f>104.1275049683+57.53730834</f>
+        <v>161.66481330830001</v>
+      </c>
+      <c r="E67" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F67" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1489.8809967005398</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68" t="s">
+        <v>163</v>
+      </c>
+      <c r="B68" t="s">
+        <v>174</v>
+      </c>
+      <c r="C68">
+        <v>60.360121323378813</v>
+      </c>
+      <c r="E68" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F68" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>611.70270126686103</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69" t="s">
+        <v>164</v>
+      </c>
+      <c r="B69" t="s">
+        <v>175</v>
+      </c>
+      <c r="C69">
+        <f>876.9412368709-C68-C66-C65-C67</f>
+        <v>275.9817057732655</v>
+      </c>
+      <c r="E69" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F69" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2642.5076198591928</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70" t="s">
+        <v>178</v>
+      </c>
+      <c r="B70" t="s">
+        <v>179</v>
+      </c>
+      <c r="C70">
+        <f>554.955290969357-423.483407079646</f>
+        <v>131.47188388971097</v>
+      </c>
+      <c r="E70" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F70" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1393.657265723991</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71" t="s">
+        <v>41</v>
+      </c>
+      <c r="B71" t="s">
+        <v>70</v>
+      </c>
+      <c r="C71">
+        <v>423.48340707964599</v>
+      </c>
+      <c r="E71" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F71" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>4429.4341224188756</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72" t="s">
+        <v>50</v>
+      </c>
+      <c r="B72" t="s">
+        <v>79</v>
+      </c>
+      <c r="C72">
+        <v>43.350037499999999</v>
+      </c>
+      <c r="E72" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F72" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>491.80958750000002</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73" t="s">
+        <v>52</v>
+      </c>
+      <c r="B73" t="s">
+        <v>81</v>
+      </c>
+      <c r="C73">
+        <v>7.7</v>
+      </c>
+      <c r="E73" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F73" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>98.676999999999992</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8">
+      <c r="A74" t="s">
+        <v>51</v>
+      </c>
+      <c r="B74" t="s">
+        <v>80</v>
+      </c>
+      <c r="C74">
+        <v>3.5904531497162</v>
+      </c>
+      <c r="E74" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F74" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>35.078727272727271</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75" t="s">
+        <v>98</v>
+      </c>
+      <c r="B75" t="s">
+        <v>182</v>
+      </c>
+      <c r="C75">
+        <v>0.78666131450805166</v>
+      </c>
+      <c r="E75" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F75" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2.1757375189927228</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
+      <c r="A76" t="s">
+        <v>184</v>
+      </c>
+      <c r="B76" t="s">
+        <v>185</v>
+      </c>
+      <c r="C76">
+        <v>58.307923875090665</v>
+      </c>
+      <c r="E76" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F76" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>586.63367669240563</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8">
+      <c r="A79" t="s">
+        <v>80</v>
+      </c>
+      <c r="B79" t="s">
+        <v>138</v>
+      </c>
+      <c r="H79" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8">
+      <c r="A80" t="s">
+        <v>81</v>
+      </c>
+      <c r="B80" t="s">
+        <v>183</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06AEBB83-8C6D-4234-B52F-BC23EBBF1927}">
+  <dimension ref="A1:F80"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -5384,10 +6924,10 @@
         <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>85</v>
+        <v>136</v>
       </c>
       <c r="D1" t="s">
-        <v>106</v>
+        <v>135</v>
       </c>
       <c r="E1" t="s">
         <v>109</v>
@@ -5405,15 +6945,15 @@
       </c>
       <c r="C2" s="2"/>
       <c r="D2">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
         <v>0</v>
       </c>
       <c r="E2">
         <v>2846</v>
       </c>
       <c r="F2">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</f>
-        <v>-7.7179334425266708</v>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</f>
+        <v>-9.8563519374511106</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -5424,17 +6964,17 @@
         <v>58</v>
       </c>
       <c r="C3" s="2">
-        <v>8.5272482121300026</v>
+        <v>6.881278581090001</v>
       </c>
       <c r="D3">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-83.31121503251012</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-67.23009173724931</v>
       </c>
       <c r="E3">
         <v>8901.1</v>
       </c>
       <c r="F3">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E3/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E3/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5446,17 +6986,17 @@
         <v>0</v>
       </c>
       <c r="C4" s="2">
-        <v>16.998179999999998</v>
+        <v>13.70613731198001</v>
       </c>
       <c r="D4">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-166.07221859999999</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-133.90896153804468</v>
       </c>
       <c r="E4">
         <v>11549.9</v>
       </c>
       <c r="F4">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E4/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E4/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5469,15 +7009,15 @@
       </c>
       <c r="C5" s="2"/>
       <c r="D5">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
         <v>0</v>
       </c>
       <c r="E5">
         <v>3492</v>
       </c>
       <c r="F5">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E5/$E$27),0)</f>
-        <v>-9.4697904361571084</v>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E5/$E$27),0)</f>
+        <v>-12.093598371601995</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -5488,17 +7028,17 @@
         <v>65</v>
       </c>
       <c r="C6" s="2">
-        <v>2.9206500000000002</v>
+        <v>2.5260000000000002</v>
       </c>
       <c r="D6">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-28.534750500000001</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-24.679020000000001</v>
       </c>
       <c r="E6">
         <v>6951.5</v>
       </c>
       <c r="F6">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E6/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E6/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5510,17 +7050,17 @@
         <v>5</v>
       </c>
       <c r="C7" s="2">
-        <v>2.9368094170890702</v>
+        <v>2.500143698008789</v>
       </c>
       <c r="D7">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-28.692628004960213</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-24.426403929545867</v>
       </c>
       <c r="E7">
         <v>4058.2</v>
       </c>
       <c r="F7">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E7/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E7/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5532,17 +7072,17 @@
         <v>62</v>
       </c>
       <c r="C8" s="2">
-        <v>8.4623749999999998</v>
+        <v>6.6974999999999998</v>
       </c>
       <c r="D8">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-82.677403749999996</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-65.434574999999995</v>
       </c>
       <c r="E8">
         <v>10693.9</v>
       </c>
       <c r="F8">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E8/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E8/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5554,17 +7094,17 @@
         <v>61</v>
       </c>
       <c r="C9" s="2">
-        <v>2.3225881808696536</v>
+        <v>1.6302510017201839</v>
       </c>
       <c r="D9">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-22.691686527096515</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-15.927552286806195</v>
       </c>
       <c r="E9">
         <v>5822.8</v>
       </c>
       <c r="F9">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E9/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E9/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5576,17 +7116,17 @@
         <v>67</v>
       </c>
       <c r="C10" s="2">
-        <v>0.43005000000000004</v>
+        <v>0.36988437623824216</v>
       </c>
       <c r="D10">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-4.2015885000000006</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-3.6137703558476257</v>
       </c>
       <c r="E10">
         <v>1329</v>
       </c>
       <c r="F10">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E10/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E10/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5598,17 +7138,17 @@
         <v>86</v>
       </c>
       <c r="C11" s="2">
-        <v>2.0718055555555557</v>
+        <v>1.1944166666666667</v>
       </c>
       <c r="D11">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-20.241540277777776</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-11.669450833333332</v>
       </c>
       <c r="E11">
         <v>5525.3</v>
       </c>
       <c r="F11">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E11/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E11/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5620,17 +7160,17 @@
         <v>2</v>
       </c>
       <c r="C12" s="2">
-        <v>40.582840274999995</v>
+        <v>33.864162380796365</v>
       </c>
       <c r="D12">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-396.49434948674991</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-330.85286646038048</v>
       </c>
       <c r="E12">
         <v>67098.8</v>
       </c>
       <c r="F12">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E12/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E12/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5642,17 +7182,17 @@
         <v>57</v>
       </c>
       <c r="C13" s="2">
-        <v>87.107500000000002</v>
+        <v>75.663813855200303</v>
       </c>
       <c r="D13">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-851.04027499999995</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-739.23546136530695</v>
       </c>
       <c r="E13">
         <v>83166.7</v>
       </c>
       <c r="F13">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E13/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E13/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5664,17 +7204,17 @@
         <v>3</v>
       </c>
       <c r="C14" s="2">
-        <v>6.3426600000000004</v>
+        <v>5.3821999999999992</v>
       </c>
       <c r="D14">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-61.967788200000001</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-52.584093999999993</v>
       </c>
       <c r="E14">
         <v>10709.7</v>
       </c>
       <c r="F14">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E14/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E14/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5686,17 +7226,17 @@
         <v>64</v>
       </c>
       <c r="C15" s="2">
-        <v>10.192972222222224</v>
+        <v>8.1848333333333336</v>
       </c>
       <c r="D15">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-99.585338611111126</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-79.96582166666667</v>
       </c>
       <c r="E15">
         <v>9769.5</v>
       </c>
       <c r="F15">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E15/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E15/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5708,17 +7248,17 @@
         <v>75</v>
       </c>
       <c r="C16" s="2">
-        <v>5.3080830939788495</v>
+        <v>4.8234356462169234</v>
       </c>
       <c r="D16">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-51.859971828173357</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-47.124966263539342</v>
       </c>
       <c r="E16">
         <v>4963.8</v>
       </c>
       <c r="F16">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E16/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E16/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5730,17 +7270,17 @@
         <v>4</v>
       </c>
       <c r="C17" s="2">
-        <v>67.625157295559788</v>
+        <v>58.597640207836605</v>
       </c>
       <c r="D17">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-660.69778677761906</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-572.49894483056357</v>
       </c>
       <c r="E17">
         <v>60244.6</v>
       </c>
       <c r="F17">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E17/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E17/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5752,17 +7292,17 @@
         <v>66</v>
       </c>
       <c r="C18" s="2">
-        <v>1.0731875</v>
+        <v>0.76711249999999997</v>
       </c>
       <c r="D18">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-10.485041874999999</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-7.4946891249999998</v>
       </c>
       <c r="E18">
         <v>1907.7</v>
       </c>
       <c r="F18">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E18/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E18/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5774,17 +7314,17 @@
         <v>6</v>
       </c>
       <c r="C19" s="2">
-        <v>2.3604840000000005</v>
+        <v>1.5655230000000002</v>
       </c>
       <c r="D19">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-23.061928680000005</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-15.295159710000002</v>
       </c>
       <c r="E19">
         <v>2794.1</v>
       </c>
       <c r="F19">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E19/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E19/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5796,17 +7336,17 @@
         <v>71</v>
       </c>
       <c r="C20" s="2">
-        <v>0.722536175</v>
+        <v>0.57345708050874755</v>
       </c>
       <c r="D20">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-7.0591784297499993</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-5.6026756765704633</v>
       </c>
       <c r="E20">
         <v>626.1</v>
       </c>
       <c r="F20">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E20/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E20/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5819,15 +7359,15 @@
       </c>
       <c r="C21" s="2"/>
       <c r="D21">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
         <v>0</v>
       </c>
       <c r="E21">
         <v>514.6</v>
       </c>
       <c r="F21">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E21/$E$27),0)</f>
-        <v>-1.395519518455455</v>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E21/$E$27),0)</f>
+        <v>-1.7821780418174076</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -5839,15 +7379,15 @@
       </c>
       <c r="C22" s="2"/>
       <c r="D22">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
         <v>0</v>
       </c>
       <c r="E22">
         <v>2579</v>
       </c>
       <c r="F22">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E22/$E$27),0)</f>
-        <v>-6.9938687098651737</v>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E22/$E$27),0)</f>
+        <v>-8.9316695877324026</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -5856,15 +7396,15 @@
       </c>
       <c r="C23" s="2"/>
       <c r="D23">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
         <v>0</v>
       </c>
       <c r="E23">
         <v>621.9</v>
       </c>
       <c r="F23">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E23/$E$27),0)</f>
-        <v>-1.6865013379857121</v>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E23/$E$27),0)</f>
+        <v>-2.1537825965920052</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -5875,17 +7415,17 @@
         <v>7</v>
       </c>
       <c r="C24" s="2">
-        <v>36.094444444444456</v>
+        <v>25.772222222222222</v>
       </c>
       <c r="D24">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-352.64272222222229</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-251.7946111111111</v>
       </c>
       <c r="E24">
         <v>17407.599999999999</v>
       </c>
       <c r="F24">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E24/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E24/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5897,17 +7437,17 @@
         <v>77</v>
       </c>
       <c r="C25" s="2">
-        <v>0.324946535664</v>
+        <v>0.35287261590049462</v>
       </c>
       <c r="D25">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-3.1747276534372797</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-3.4475654573478325</v>
       </c>
       <c r="E25">
         <v>2076.3000000000002</v>
       </c>
       <c r="F25">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E25/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E25/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5919,17 +7459,17 @@
         <v>72</v>
       </c>
       <c r="C26" s="2">
-        <v>4.4535245861624997</v>
+        <v>3.7932103112550002</v>
       </c>
       <c r="D26">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-43.510935206807623</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-37.059664740961352</v>
       </c>
       <c r="E26">
         <v>5367.6</v>
       </c>
       <c r="F26">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E26/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E26/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5941,18 +7481,18 @@
         <v>89</v>
       </c>
       <c r="C27" s="2">
-        <v>5.4542940093096091</v>
+        <v>6.9655227952428636</v>
       </c>
       <c r="D27">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-53.28845247095488</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-68.053157709522779</v>
       </c>
       <c r="E27">
         <f>SUMIF(D2:D26,"=0",E2:E26)+SUMIF(D28:D42,"=0",E28:E42)</f>
         <v>19650.2</v>
       </c>
       <c r="F27">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E27/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E27/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5964,17 +7504,17 @@
         <v>8</v>
       </c>
       <c r="C28" s="2">
-        <v>21.064583333333339</v>
+        <v>19.582712959636471</v>
       </c>
       <c r="D28">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-205.80097916666671</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-191.3231056156483</v>
       </c>
       <c r="E28">
         <v>37958.1</v>
       </c>
       <c r="F28">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E28/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E28/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5986,17 +7526,17 @@
         <v>1</v>
       </c>
       <c r="C29" s="2">
-        <v>6.0366596174639984</v>
+        <v>4.4804912631795961</v>
       </c>
       <c r="D29">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-58.978164462623262</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-43.774399641264651</v>
       </c>
       <c r="E29">
         <v>10295.9</v>
       </c>
       <c r="F29">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E29/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E29/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6008,17 +7548,17 @@
         <v>87</v>
       </c>
       <c r="C30" s="2">
-        <v>11.262552972222222</v>
+        <v>9.0859916688941222</v>
       </c>
       <c r="D30">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-110.03514253861111</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-88.770138605095568</v>
       </c>
       <c r="E30">
         <v>19318</v>
       </c>
       <c r="F30">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E30/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E30/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6031,14 +7571,14 @@
       </c>
       <c r="C31" s="2"/>
       <c r="D31">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
         <v>0</v>
       </c>
       <c r="E31">
         <v>0</v>
       </c>
       <c r="F31">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E31/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E31/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6051,15 +7591,15 @@
       </c>
       <c r="C32" s="2"/>
       <c r="D32">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
         <v>0</v>
       </c>
       <c r="E32">
         <v>6926.7</v>
       </c>
       <c r="F32">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E32/$E$27),0)</f>
-        <v>-18.784191699349783</v>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E32/$E$27),0)</f>
+        <v>-23.98875367714076</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -6070,17 +7610,17 @@
         <v>63</v>
       </c>
       <c r="C33" s="2">
-        <v>4.754638388888889</v>
+        <v>4.1980544937588302</v>
       </c>
       <c r="D33">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-46.452817059444442</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-41.014992404023772</v>
       </c>
       <c r="E33">
         <v>5457.9</v>
       </c>
       <c r="F33">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E33/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E33/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6092,17 +7632,17 @@
         <v>60</v>
       </c>
       <c r="C34" s="2">
-        <v>0.85516059371380015</v>
+        <v>0.76667289608525002</v>
       </c>
       <c r="D34">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-8.354919000583827</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-7.4903941947528923</v>
       </c>
       <c r="E34">
         <v>2095.9</v>
       </c>
       <c r="F34">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E34/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E34/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6114,17 +7654,17 @@
         <v>9</v>
       </c>
       <c r="C35" s="2">
-        <v>32.490230910000008</v>
+        <v>29.298304475852706</v>
       </c>
       <c r="D35">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-317.42955599070007</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-286.24443472908092</v>
       </c>
       <c r="E35">
         <v>47330</v>
       </c>
       <c r="F35">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E35/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E35/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6136,17 +7676,17 @@
         <v>84</v>
       </c>
       <c r="C36" s="2">
-        <v>0.99092500000000006</v>
+        <v>0.71619917569573466</v>
       </c>
       <c r="D36">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-9.6813372500000003</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-6.9972659465473273</v>
       </c>
       <c r="E36">
         <v>10327.6</v>
       </c>
       <c r="F36">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E36/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E36/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6158,17 +7698,17 @@
         <v>59</v>
       </c>
       <c r="C37" s="2">
-        <v>3.3147222222222226</v>
+        <v>2.7441227961633525</v>
       </c>
       <c r="D37">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-32.384836111111113</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-26.810079718515954</v>
       </c>
       <c r="E37">
         <v>8606</v>
       </c>
       <c r="F37">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E37/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E37/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6180,17 +7720,17 @@
         <v>10</v>
       </c>
       <c r="C38" s="2">
-        <v>46.209907500000007</v>
+        <v>48.429348579939109</v>
       </c>
       <c r="D38">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-451.47079627500005</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-473.15473562600505</v>
       </c>
       <c r="E38">
         <v>83155</v>
       </c>
       <c r="F38">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E38/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E38/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6202,17 +7742,17 @@
         <v>11</v>
       </c>
       <c r="C39" s="2">
-        <v>73.145389499999993</v>
+        <v>63.503524799999994</v>
       </c>
       <c r="D39">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-714.63045541499991</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-620.42943729599995</v>
       </c>
       <c r="E39">
         <v>67025.5</v>
       </c>
       <c r="F39">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E39/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E39/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6224,17 +7764,17 @@
         <v>68</v>
       </c>
       <c r="C40" s="2">
-        <v>29.338741396263522</v>
+        <v>18.73893805309735</v>
       </c>
       <c r="D40">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>-286.63950344149458</v>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
+        <v>-183.07942477876111</v>
       </c>
       <c r="E40">
         <v>41733</v>
       </c>
       <c r="F40">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E40/$E$27),0)</f>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E40/$E$27),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6247,15 +7787,15 @@
       </c>
       <c r="C41" s="2"/>
       <c r="D41">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
+        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
         <v>0</v>
       </c>
       <c r="E41">
         <v>888</v>
       </c>
       <c r="F41">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E41/$E$27),0)</f>
-        <v>-2.4081254030090244</v>
+        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E41/$E$27),0)</f>
+        <v>-3.0753480395139094</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -6264,951 +7804,6 @@
       </c>
       <c r="C42" s="2"/>
       <c r="D42">
-        <f>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
-        <v>0</v>
-      </c>
-      <c r="E42">
-        <v>1782</v>
-      </c>
-      <c r="F42">
-        <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E42/$E$27),0)</f>
-        <v>-4.8325219236059471</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2">
-      <c r="A50" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2">
-      <c r="A51" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2">
-      <c r="A52" t="s">
-        <v>115</v>
-      </c>
-      <c r="B52" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2">
-      <c r="A53" t="s">
-        <v>117</v>
-      </c>
-      <c r="B53" t="s">
-        <v>118</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06AEBB83-8C6D-4234-B52F-BC23EBBF1927}">
-  <dimension ref="A1:F53"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="1" max="1" width="9.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" t="s">
-        <v>136</v>
-      </c>
-      <c r="D1" t="s">
-        <v>135</v>
-      </c>
-      <c r="E1" t="s">
-        <v>109</v>
-      </c>
-      <c r="F1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C2" s="2"/>
-      <c r="D2">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>2846</v>
-      </c>
-      <c r="F2">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</f>
-        <v>-9.8563519374511106</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C3" s="2">
-        <v>6.881278581090001</v>
-      </c>
-      <c r="D3">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-67.23009173724931</v>
-      </c>
-      <c r="E3">
-        <v>8901.1</v>
-      </c>
-      <c r="F3">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E3/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="2">
-        <v>13.70613731198001</v>
-      </c>
-      <c r="D4">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-133.90896153804468</v>
-      </c>
-      <c r="E4">
-        <v>11549.9</v>
-      </c>
-      <c r="F4">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E4/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C5" s="2"/>
-      <c r="D5">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>3492</v>
-      </c>
-      <c r="F5">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E5/$E$27),0)</f>
-        <v>-12.093598371601995</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="2">
-        <v>2.5260000000000002</v>
-      </c>
-      <c r="D6">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-24.679020000000001</v>
-      </c>
-      <c r="E6">
-        <v>6951.5</v>
-      </c>
-      <c r="F6">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E6/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="2">
-        <v>2.500143698008789</v>
-      </c>
-      <c r="D7">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-24.426403929545867</v>
-      </c>
-      <c r="E7">
-        <v>4058.2</v>
-      </c>
-      <c r="F7">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E7/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="2">
-        <v>6.6974999999999998</v>
-      </c>
-      <c r="D8">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-65.434574999999995</v>
-      </c>
-      <c r="E8">
-        <v>10693.9</v>
-      </c>
-      <c r="F8">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E8/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="2">
-        <v>1.6302510017201839</v>
-      </c>
-      <c r="D9">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-15.927552286806195</v>
-      </c>
-      <c r="E9">
-        <v>5822.8</v>
-      </c>
-      <c r="F9">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E9/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>54</v>
-      </c>
-      <c r="B10" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="2">
-        <v>0.36988437623824216</v>
-      </c>
-      <c r="D10">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-3.6137703558476257</v>
-      </c>
-      <c r="E10">
-        <v>1329</v>
-      </c>
-      <c r="F10">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E10/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" t="s">
-        <v>86</v>
-      </c>
-      <c r="C11" s="2">
-        <v>1.1944166666666667</v>
-      </c>
-      <c r="D11">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-11.669450833333332</v>
-      </c>
-      <c r="E11">
-        <v>5525.3</v>
-      </c>
-      <c r="F11">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E11/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" t="s">
-        <v>2</v>
-      </c>
-      <c r="C12" s="2">
-        <v>33.864162380796365</v>
-      </c>
-      <c r="D12">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-330.85286646038048</v>
-      </c>
-      <c r="E12">
-        <v>67098.8</v>
-      </c>
-      <c r="F12">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E12/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B13" t="s">
-        <v>57</v>
-      </c>
-      <c r="C13" s="2">
-        <v>75.663813855200303</v>
-      </c>
-      <c r="D13">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-739.23546136530695</v>
-      </c>
-      <c r="E13">
-        <v>83166.7</v>
-      </c>
-      <c r="F13">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E13/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" t="s">
-        <v>33</v>
-      </c>
-      <c r="B14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C14" s="2">
-        <v>5.3821999999999992</v>
-      </c>
-      <c r="D14">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-52.584093999999993</v>
-      </c>
-      <c r="E14">
-        <v>10709.7</v>
-      </c>
-      <c r="F14">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E14/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" t="s">
-        <v>64</v>
-      </c>
-      <c r="C15" s="2">
-        <v>8.1848333333333336</v>
-      </c>
-      <c r="D15">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-79.96582166666667</v>
-      </c>
-      <c r="E15">
-        <v>9769.5</v>
-      </c>
-      <c r="F15">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E15/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" t="s">
-        <v>75</v>
-      </c>
-      <c r="C16" s="2">
-        <v>4.8234356462169234</v>
-      </c>
-      <c r="D16">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-47.124966263539342</v>
-      </c>
-      <c r="E16">
-        <v>4963.8</v>
-      </c>
-      <c r="F16">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E16/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" t="s">
-        <v>4</v>
-      </c>
-      <c r="C17" s="2">
-        <v>58.597640207836605</v>
-      </c>
-      <c r="D17">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-572.49894483056357</v>
-      </c>
-      <c r="E17">
-        <v>60244.6</v>
-      </c>
-      <c r="F17">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E17/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" t="s">
-        <v>36</v>
-      </c>
-      <c r="B18" t="s">
-        <v>66</v>
-      </c>
-      <c r="C18" s="2">
-        <v>0.76711249999999997</v>
-      </c>
-      <c r="D18">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-7.4946891249999998</v>
-      </c>
-      <c r="E18">
-        <v>1907.7</v>
-      </c>
-      <c r="F18">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E18/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" t="s">
-        <v>35</v>
-      </c>
-      <c r="B19" t="s">
-        <v>6</v>
-      </c>
-      <c r="C19" s="2">
-        <v>1.5655230000000002</v>
-      </c>
-      <c r="D19">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-15.295159710000002</v>
-      </c>
-      <c r="E19">
-        <v>2794.1</v>
-      </c>
-      <c r="F19">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E19/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" t="s">
-        <v>71</v>
-      </c>
-      <c r="C20" s="2">
-        <v>0.57345708050874755</v>
-      </c>
-      <c r="D20">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-5.6026756765704633</v>
-      </c>
-      <c r="E20">
-        <v>626.1</v>
-      </c>
-      <c r="F20">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E20/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" t="s">
-        <v>112</v>
-      </c>
-      <c r="B21" t="s">
-        <v>92</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>0</v>
-      </c>
-      <c r="E21">
-        <v>514.6</v>
-      </c>
-      <c r="F21">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E21/$E$27),0)</f>
-        <v>-1.7821780418174076</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" t="s">
-        <v>69</v>
-      </c>
-      <c r="C22" s="2"/>
-      <c r="D22">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>0</v>
-      </c>
-      <c r="E22">
-        <v>2579</v>
-      </c>
-      <c r="F22">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E22/$E$27),0)</f>
-        <v>-8.9316695877324026</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="B23" t="s">
-        <v>113</v>
-      </c>
-      <c r="C23" s="2"/>
-      <c r="D23">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>0</v>
-      </c>
-      <c r="E23">
-        <v>621.9</v>
-      </c>
-      <c r="F23">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E23/$E$27),0)</f>
-        <v>-2.1537825965920052</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" t="s">
-        <v>18</v>
-      </c>
-      <c r="B24" t="s">
-        <v>7</v>
-      </c>
-      <c r="C24" s="2">
-        <v>25.772222222222222</v>
-      </c>
-      <c r="D24">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-251.7946111111111</v>
-      </c>
-      <c r="E24">
-        <v>17407.599999999999</v>
-      </c>
-      <c r="F24">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E24/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" t="s">
-        <v>46</v>
-      </c>
-      <c r="B25" t="s">
-        <v>77</v>
-      </c>
-      <c r="C25" s="2">
-        <v>0.35287261590049462</v>
-      </c>
-      <c r="D25">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-3.4475654573478325</v>
-      </c>
-      <c r="E25">
-        <v>2076.3000000000002</v>
-      </c>
-      <c r="F25">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E25/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" t="s">
-        <v>49</v>
-      </c>
-      <c r="B26" t="s">
-        <v>72</v>
-      </c>
-      <c r="C26" s="2">
-        <v>3.7932103112550002</v>
-      </c>
-      <c r="D26">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-37.059664740961352</v>
-      </c>
-      <c r="E26">
-        <v>5367.6</v>
-      </c>
-      <c r="F26">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E26/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" t="s">
-        <v>88</v>
-      </c>
-      <c r="B27" t="s">
-        <v>89</v>
-      </c>
-      <c r="C27" s="2">
-        <v>6.9655227952428636</v>
-      </c>
-      <c r="D27">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-68.053157709522779</v>
-      </c>
-      <c r="E27">
-        <f>SUMIF(D2:D26,"=0",E2:E26)+SUMIF(D28:D42,"=0",E28:E42)</f>
-        <v>19650.2</v>
-      </c>
-      <c r="F27">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E27/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" t="s">
-        <v>8</v>
-      </c>
-      <c r="C28" s="2">
-        <v>19.582712959636471</v>
-      </c>
-      <c r="D28">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-191.3231056156483</v>
-      </c>
-      <c r="E28">
-        <v>37958.1</v>
-      </c>
-      <c r="F28">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E28/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" t="s">
-        <v>38</v>
-      </c>
-      <c r="B29" t="s">
-        <v>1</v>
-      </c>
-      <c r="C29" s="2">
-        <v>4.4804912631795961</v>
-      </c>
-      <c r="D29">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-43.774399641264651</v>
-      </c>
-      <c r="E29">
-        <v>10295.9</v>
-      </c>
-      <c r="F29">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E29/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="A30" t="s">
-        <v>34</v>
-      </c>
-      <c r="B30" t="s">
-        <v>87</v>
-      </c>
-      <c r="C30" s="2">
-        <v>9.0859916688941222</v>
-      </c>
-      <c r="D30">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-88.770138605095568</v>
-      </c>
-      <c r="E30">
-        <v>19318</v>
-      </c>
-      <c r="F30">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E30/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" t="s">
-        <v>48</v>
-      </c>
-      <c r="B31" t="s">
-        <v>78</v>
-      </c>
-      <c r="C31" s="2"/>
-      <c r="D31">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>0</v>
-      </c>
-      <c r="E31">
-        <v>0</v>
-      </c>
-      <c r="F31">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E31/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" t="s">
-        <v>31</v>
-      </c>
-      <c r="B32" t="s">
-        <v>73</v>
-      </c>
-      <c r="C32" s="2"/>
-      <c r="D32">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>0</v>
-      </c>
-      <c r="E32">
-        <v>6926.7</v>
-      </c>
-      <c r="F32">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E32/$E$27),0)</f>
-        <v>-23.98875367714076</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" t="s">
-        <v>29</v>
-      </c>
-      <c r="B33" t="s">
-        <v>63</v>
-      </c>
-      <c r="C33" s="2">
-        <v>4.1980544937588302</v>
-      </c>
-      <c r="D33">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-41.014992404023772</v>
-      </c>
-      <c r="E33">
-        <v>5457.9</v>
-      </c>
-      <c r="F33">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E33/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6">
-      <c r="A34" t="s">
-        <v>23</v>
-      </c>
-      <c r="B34" t="s">
-        <v>60</v>
-      </c>
-      <c r="C34" s="2">
-        <v>0.76667289608525002</v>
-      </c>
-      <c r="D34">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-7.4903941947528923</v>
-      </c>
-      <c r="E34">
-        <v>2095.9</v>
-      </c>
-      <c r="F34">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E34/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" t="s">
-        <v>37</v>
-      </c>
-      <c r="B35" t="s">
-        <v>9</v>
-      </c>
-      <c r="C35" s="2">
-        <v>29.298304475852706</v>
-      </c>
-      <c r="D35">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-286.24443472908092</v>
-      </c>
-      <c r="E35">
-        <v>47330</v>
-      </c>
-      <c r="F35">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E35/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36" t="s">
-        <v>83</v>
-      </c>
-      <c r="B36" t="s">
-        <v>84</v>
-      </c>
-      <c r="C36" s="2">
-        <v>0.71619917569573466</v>
-      </c>
-      <c r="D36">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-6.9972659465473273</v>
-      </c>
-      <c r="E36">
-        <v>10327.6</v>
-      </c>
-      <c r="F36">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E36/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37" t="s">
-        <v>22</v>
-      </c>
-      <c r="B37" t="s">
-        <v>59</v>
-      </c>
-      <c r="C37" s="2">
-        <v>2.7441227961633525</v>
-      </c>
-      <c r="D37">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-26.810079718515954</v>
-      </c>
-      <c r="E37">
-        <v>8606</v>
-      </c>
-      <c r="F37">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E37/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38" t="s">
-        <v>47</v>
-      </c>
-      <c r="B38" t="s">
-        <v>10</v>
-      </c>
-      <c r="C38" s="2">
-        <v>48.429348579939109</v>
-      </c>
-      <c r="D38">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-473.15473562600505</v>
-      </c>
-      <c r="E38">
-        <v>83155</v>
-      </c>
-      <c r="F38">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E38/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" t="s">
-        <v>11</v>
-      </c>
-      <c r="B39" t="s">
-        <v>11</v>
-      </c>
-      <c r="C39" s="2">
-        <v>63.503524799999994</v>
-      </c>
-      <c r="D39">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-620.42943729599995</v>
-      </c>
-      <c r="E39">
-        <v>67025.5</v>
-      </c>
-      <c r="F39">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E39/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40" t="s">
-        <v>39</v>
-      </c>
-      <c r="B40" t="s">
-        <v>68</v>
-      </c>
-      <c r="C40" s="2">
-        <v>18.73893805309735</v>
-      </c>
-      <c r="D40">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>-183.07942477876111</v>
-      </c>
-      <c r="E40">
-        <v>41733</v>
-      </c>
-      <c r="F40">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E40/$E$27),0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" t="s">
-        <v>110</v>
-      </c>
-      <c r="B41" t="s">
-        <v>111</v>
-      </c>
-      <c r="C41" s="2"/>
-      <c r="D41">
-        <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
-        <v>0</v>
-      </c>
-      <c r="E41">
-        <v>888</v>
-      </c>
-      <c r="F41">
-        <f>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E41/$E$27),0)</f>
-        <v>-3.0753480395139094</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="B42" t="s">
-        <v>119</v>
-      </c>
-      <c r="C42" s="2"/>
-      <c r="D42">
         <f>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</f>
         <v>0</v>
       </c>
@@ -7220,17 +7815,17 @@
         <v>-6.171475457673183</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
+    <row r="50" spans="1:6">
       <c r="A50" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
+    <row r="51" spans="1:6">
       <c r="A51" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:6">
       <c r="A52" t="s">
         <v>115</v>
       </c>
@@ -7238,7 +7833,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="1:2">
+    <row r="53" spans="1:6">
       <c r="A53" t="s">
         <v>117</v>
       </c>
@@ -7246,17 +7841,424 @@
         <v>118</v>
       </c>
     </row>
+    <row r="57" spans="1:6">
+      <c r="A57" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="F57" s="10" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" t="s">
+        <v>153</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="C58" s="7">
+        <v>886.46721186282696</v>
+      </c>
+      <c r="D58" s="7"/>
+      <c r="E58" s="7">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>8660.7846598998185</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" t="s">
+        <v>154</v>
+      </c>
+      <c r="B59" t="s">
+        <v>165</v>
+      </c>
+      <c r="C59">
+        <f>1104.76718773088-886.467211862827</f>
+        <v>218.29997586805314</v>
+      </c>
+      <c r="E59" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2132.7907642308792</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6">
+      <c r="A60" t="s">
+        <v>155</v>
+      </c>
+      <c r="B60" t="s">
+        <v>166</v>
+      </c>
+      <c r="C60">
+        <f>161.703504900654-14.503954775876</f>
+        <v>147.199550124778</v>
+      </c>
+      <c r="E60" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F60" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1438.139604719081</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6">
+      <c r="A61" t="s">
+        <v>156</v>
+      </c>
+      <c r="B61" t="s">
+        <v>167</v>
+      </c>
+      <c r="C61">
+        <v>14.503954775876</v>
+      </c>
+      <c r="E61" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F61" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>141.70363816030851</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" t="s">
+        <v>157</v>
+      </c>
+      <c r="B62" t="s">
+        <v>168</v>
+      </c>
+      <c r="C62" s="2">
+        <f>577.716724870969-44.2013179565956</f>
+        <v>533.51540691437333</v>
+      </c>
+      <c r="E62" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F62" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>5212.4455255534276</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" t="s">
+        <v>158</v>
+      </c>
+      <c r="B63" t="s">
+        <v>181</v>
+      </c>
+      <c r="C63">
+        <v>44.201317956595602</v>
+      </c>
+      <c r="E63" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F63" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>431.84687643593901</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" t="s">
+        <v>159</v>
+      </c>
+      <c r="B64" t="s">
+        <v>170</v>
+      </c>
+      <c r="C64" s="2">
+        <f>171.229082457489-C72-C73-C74-C75-C76</f>
+        <v>46.93279494631954</v>
+      </c>
+      <c r="E64" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F64" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>458.53340662554189</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6">
+      <c r="A65" t="s">
+        <v>160</v>
+      </c>
+      <c r="B65" t="s">
+        <v>171</v>
+      </c>
+      <c r="C65">
+        <v>40.121503042095824</v>
+      </c>
+      <c r="E65" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F65" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>391.98708472127618</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6">
+      <c r="A66" t="s">
+        <v>161</v>
+      </c>
+      <c r="B66" t="s">
+        <v>172</v>
+      </c>
+      <c r="C66">
+        <f>404.838112094395+4.84678040562862</f>
+        <v>409.68489250002364</v>
+      </c>
+      <c r="E66" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F66" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>4002.6213997252307</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6">
+      <c r="A67" t="s">
+        <v>162</v>
+      </c>
+      <c r="B67" t="s">
+        <v>173</v>
+      </c>
+      <c r="C67">
+        <f>92.4207922536915+60.0747038262</f>
+        <v>152.4954960798915</v>
+      </c>
+      <c r="E67" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F67" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1489.8809967005398</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" t="s">
+        <v>163</v>
+      </c>
+      <c r="B68" t="s">
+        <v>174</v>
+      </c>
+      <c r="C68">
+        <v>62.610307192104507</v>
+      </c>
+      <c r="E68" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F68" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>611.70270126686103</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="A69" t="s">
+        <v>164</v>
+      </c>
+      <c r="B69" t="s">
+        <v>175</v>
+      </c>
+      <c r="C69">
+        <f>935.383807806868-C68-C66-C65-C67</f>
+        <v>270.47160899275258</v>
+      </c>
+      <c r="E69" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F69" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2642.5076198591928</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="A70" t="s">
+        <v>178</v>
+      </c>
+      <c r="B70" t="s">
+        <v>179</v>
+      </c>
+      <c r="C70">
+        <f>596.017542286885-453.370943952802</f>
+        <v>142.64659833408302</v>
+      </c>
+      <c r="E70" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F70" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1393.657265723991</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
+      <c r="A71" t="s">
+        <v>41</v>
+      </c>
+      <c r="B71" t="s">
+        <v>70</v>
+      </c>
+      <c r="C71">
+        <v>453.37094395280201</v>
+      </c>
+      <c r="E71" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F71" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>4429.4341224188756</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="A72" t="s">
+        <v>50</v>
+      </c>
+      <c r="B72" t="s">
+        <v>79</v>
+      </c>
+      <c r="C72">
+        <v>50.338750000000005</v>
+      </c>
+      <c r="E72" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F72" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>491.80958750000002</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
+      <c r="A73" t="s">
+        <v>52</v>
+      </c>
+      <c r="B73" t="s">
+        <v>81</v>
+      </c>
+      <c r="C73">
+        <v>10.1</v>
+      </c>
+      <c r="E73" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F73" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>98.676999999999992</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
+      <c r="A74" t="s">
+        <v>51</v>
+      </c>
+      <c r="B74" t="s">
+        <v>80</v>
+      </c>
+      <c r="C74">
+        <v>3.5904531497162</v>
+      </c>
+      <c r="E74" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F74" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>35.078727272727271</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
+      <c r="A75" t="s">
+        <v>98</v>
+      </c>
+      <c r="B75" t="s">
+        <v>182</v>
+      </c>
+      <c r="C75">
+        <v>0.22269575424695218</v>
+      </c>
+      <c r="E75" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F75" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2.1757375189927228</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="A76" t="s">
+        <v>184</v>
+      </c>
+      <c r="B76" t="s">
+        <v>185</v>
+      </c>
+      <c r="C76">
+        <v>60.044388607206308</v>
+      </c>
+      <c r="E76" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F76" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>586.63367669240563</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
+      <c r="A79" t="s">
+        <v>80</v>
+      </c>
+      <c r="B79" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6">
+      <c r="A80" t="s">
+        <v>81</v>
+      </c>
+      <c r="B80" t="s">
+        <v>183</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD7211D-DC17-4DD6-B657-CA08F8FBC20F}">
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H128"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="20.453125" customWidth="1"/>
@@ -9475,6 +10477,174 @@
         <v>180.45599999999999</v>
       </c>
     </row>
+    <row r="112" spans="1:8">
+      <c r="A112" t="s">
+        <v>153</v>
+      </c>
+      <c r="B112" t="s">
+        <v>154</v>
+      </c>
+      <c r="F112" s="11">
+        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G112">
+        <f t="shared" ref="G112:G120" si="4">F112/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7">
+      <c r="A113" t="s">
+        <v>154</v>
+      </c>
+      <c r="B113" t="s">
+        <v>153</v>
+      </c>
+      <c r="F113" s="11">
+        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G113">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7">
+      <c r="A114" t="s">
+        <v>157</v>
+      </c>
+      <c r="B114" t="s">
+        <v>158</v>
+      </c>
+      <c r="F114" s="11">
+        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G114">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7">
+      <c r="A115" t="s">
+        <v>158</v>
+      </c>
+      <c r="B115" t="s">
+        <v>157</v>
+      </c>
+      <c r="F115" s="11">
+        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G115">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7">
+      <c r="A116" t="s">
+        <v>41</v>
+      </c>
+      <c r="B116" t="s">
+        <v>161</v>
+      </c>
+      <c r="F116" s="11">
+        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G116">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7">
+      <c r="A117" t="s">
+        <v>178</v>
+      </c>
+      <c r="B117" t="s">
+        <v>161</v>
+      </c>
+      <c r="F117" s="11">
+        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G117">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7">
+      <c r="A118" t="s">
+        <v>164</v>
+      </c>
+      <c r="B118" t="s">
+        <v>161</v>
+      </c>
+      <c r="F118" s="11">
+        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G118">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7">
+      <c r="A119" t="s">
+        <v>41</v>
+      </c>
+      <c r="B119" t="s">
+        <v>178</v>
+      </c>
+      <c r="F119" s="11">
+        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G119">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7">
+      <c r="A120" t="s">
+        <v>184</v>
+      </c>
+      <c r="B120" t="s">
+        <v>157</v>
+      </c>
+      <c r="F120" s="11">
+        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G120">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7">
+      <c r="F121" s="11"/>
+    </row>
+    <row r="122" spans="1:7">
+      <c r="F122" s="11"/>
+    </row>
+    <row r="123" spans="1:7">
+      <c r="F123" s="11"/>
+    </row>
+    <row r="124" spans="1:7">
+      <c r="F124" s="11"/>
+    </row>
+    <row r="125" spans="1:7">
+      <c r="F125" s="11"/>
+    </row>
+    <row r="126" spans="1:7">
+      <c r="F126" s="11"/>
+    </row>
+    <row r="127" spans="1:7">
+      <c r="F127" s="11"/>
+    </row>
+    <row r="128" spans="1:7">
+      <c r="F128" s="11"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9486,7 +10656,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67CAB708-6819-43AD-B444-2B653F840206}">
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:H126"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="20.453125" customWidth="1"/>
@@ -11817,6 +12987,150 @@
       <c r="G117">
         <f t="shared" si="1"/>
         <v>180.45599999999999</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7">
+      <c r="A118" t="s">
+        <v>153</v>
+      </c>
+      <c r="B118" t="s">
+        <v>154</v>
+      </c>
+      <c r="F118" s="11">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G118">
+        <f t="shared" ref="G118:G126" si="2">F118/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7">
+      <c r="A119" t="s">
+        <v>154</v>
+      </c>
+      <c r="B119" t="s">
+        <v>153</v>
+      </c>
+      <c r="F119" s="11">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G119">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7">
+      <c r="A120" t="s">
+        <v>157</v>
+      </c>
+      <c r="B120" t="s">
+        <v>158</v>
+      </c>
+      <c r="F120" s="11">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G120">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7">
+      <c r="A121" t="s">
+        <v>158</v>
+      </c>
+      <c r="B121" t="s">
+        <v>157</v>
+      </c>
+      <c r="F121" s="11">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G121">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7">
+      <c r="A122" t="s">
+        <v>41</v>
+      </c>
+      <c r="B122" t="s">
+        <v>161</v>
+      </c>
+      <c r="F122" s="11">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G122">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7">
+      <c r="A123" t="s">
+        <v>178</v>
+      </c>
+      <c r="B123" t="s">
+        <v>161</v>
+      </c>
+      <c r="F123" s="11">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G123">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7">
+      <c r="A124" t="s">
+        <v>164</v>
+      </c>
+      <c r="B124" t="s">
+        <v>161</v>
+      </c>
+      <c r="F124" s="11">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G124">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7">
+      <c r="A125" t="s">
+        <v>41</v>
+      </c>
+      <c r="B125" t="s">
+        <v>178</v>
+      </c>
+      <c r="F125" s="11">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G125">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7">
+      <c r="A126" t="s">
+        <v>184</v>
+      </c>
+      <c r="B126" t="s">
+        <v>157</v>
+      </c>
+      <c r="F126" s="11">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>0</v>
+      </c>
+      <c r="G126">
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -12474,4 +13788,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
adding non-European LNG connections
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6817EC08-3183-4381-9A7B-AF9246AFDA86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F073AE-A613-4179-B460-114D223FC2E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="Connections_2021" sheetId="4" r:id="rId6"/>
     <sheet name="Connections_2024" sheetId="8" r:id="rId7"/>
     <sheet name="Import_Connections_EU" sheetId="5" r:id="rId8"/>
-    <sheet name="Sheet1" sheetId="9" r:id="rId9"/>
+    <sheet name="global_LNG_connections" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1370" uniqueCount="204">
   <si>
     <t>Belgium</t>
   </si>
@@ -602,6 +602,60 @@
   </si>
   <si>
     <t>Egypt</t>
+  </si>
+  <si>
+    <t>USA_LNG</t>
+  </si>
+  <si>
+    <t>EU</t>
+  </si>
+  <si>
+    <t>GWh/d [capacity]</t>
+  </si>
+  <si>
+    <t>TT_LNG</t>
+  </si>
+  <si>
+    <t>ME_LNG</t>
+  </si>
+  <si>
+    <t>QA_LNG</t>
+  </si>
+  <si>
+    <t>AF_LNG</t>
+  </si>
+  <si>
+    <t>AU_LNG</t>
+  </si>
+  <si>
+    <t>SA_LNG</t>
+  </si>
+  <si>
+    <t>CN_LNG</t>
+  </si>
+  <si>
+    <t>JS_LNG</t>
+  </si>
+  <si>
+    <t>IN_LNG</t>
+  </si>
+  <si>
+    <t>AS_LNG</t>
+  </si>
+  <si>
+    <t>EG_LNG</t>
+  </si>
+  <si>
+    <t>IM</t>
+  </si>
+  <si>
+    <t>RU_LNG</t>
+  </si>
+  <si>
+    <t>IM_LNG</t>
+  </si>
+  <si>
+    <t>Indonesia &amp; Malaysia</t>
   </si>
 </sst>
 </file>
@@ -780,7 +834,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -837,6 +891,15 @@
       <bottom style="thin">
         <color theme="4" tint="0.39997558519241921"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -897,7 +960,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -909,7 +972,9 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -954,7 +1019,67 @@
     <cellStyle name="Percent 4" xfId="35" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
     <cellStyle name="Percent 8" xfId="33" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
-  <dxfs count="36">
+  <dxfs count="40">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <right style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -962,7 +1087,48 @@
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
@@ -975,16 +1141,69 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <bottom style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </bottom>
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1018,113 +1237,13 @@
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
@@ -1201,12 +1320,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D3465064-BCEE-4D04-A8E6-DEAE11BBDA92}" name="Country"/>
     <tableColumn id="2" xr3:uid="{D66D54B4-4DED-47C6-BE50-755A236428ED}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="33">
+    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="38"/>
+    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="37">
       <calculatedColumnFormula>Table2[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="32">
+    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="36">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1226,7 +1345,7 @@
     <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="17">
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="4">
       <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
@@ -1238,18 +1357,37 @@
 </table>
 </file>
 
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:F69" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="2" tableBorderDxfId="3" totalsRowBorderDxfId="1">
+  <autoFilter ref="A1:F69" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
+    <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
+    <tableColumn id="3" xr3:uid="{426DF8FF-B8EF-4473-B5C0-4A6D2531E9C8}" name="GWh/d [capacity]"/>
+    <tableColumn id="6" xr3:uid="{FE296762-E7A2-4F83-8B38-CCAC423CA9A3}" name="GWh/a">
+      <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{15452FB1-E8BF-413E-AF8B-8B2631F8DB73}" name="TWh/a">
+      <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{ECBB25E4-2145-4120-8981-E6E8E1591E5B}" name="Comment"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F68" totalsRowShown="0" headerRowDxfId="31" headerRowBorderDxfId="30" tableBorderDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F68" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33">
   <autoFilter ref="A53:F68" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3F684FB4-9656-4C92-BAF4-456019B2B924}" name="Country"/>
     <tableColumn id="2" xr3:uid="{082B059D-405D-407D-8F97-297DCD23D3B2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{388F462C-127F-4CB7-B46A-1DD19D06D0E8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{ACDF4345-6201-4524-A8D7-A0CE31D137A6}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="1">
+    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="32">
       <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="31">
       <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1266,12 +1404,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="26">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="28">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="25">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="27">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1280,17 +1418,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F67" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="11" tableBorderDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F67" totalsRowShown="0" headerRowDxfId="26" headerRowBorderDxfId="25" tableBorderDxfId="24">
   <autoFilter ref="A52:F67" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{02819FD0-F6B6-484E-B4DA-8262AECE7052}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{A15C284E-E91C-44C6-B3BB-CC2DD205DA84}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="10">
+    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="23">
       <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="9">
+    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="22">
       <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1307,12 +1445,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="23">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="20">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="22">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="19">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1321,17 +1459,17 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F76" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="14" tableBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F76" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16">
   <autoFilter ref="A57:F76" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{555371BF-8030-4257-9852-212E94829B9B}" name="Country"/>
     <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="3">
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="15">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="2">
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="14">
       <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1348,12 +1486,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="20">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="12">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="19">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="11">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1362,17 +1500,17 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F76" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="6" tableBorderDxfId="7">
-  <autoFilter ref="A57:F76" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F77" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="9" tableBorderDxfId="8">
+  <autoFilter ref="A57:F77" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{779C3748-4ECD-495F-809A-B5DD28F5EC2F}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{94BC7314-C5A0-4AAD-895B-84E7A94D7CF7}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="5">
+    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="7">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="4">
+    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="6">
       <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1392,7 +1530,7 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="18">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="5">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
@@ -6910,7 +7048,7 @@
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" customWidth="1"/>
+    <col min="2" max="2" width="20.36328125" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="22.26953125" customWidth="1"/>
@@ -8229,6 +8367,22 @@
       <c r="F76" s="3">
         <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
         <v>586.63367669240563</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="A77" t="s">
+        <v>200</v>
+      </c>
+      <c r="B77" t="s">
+        <v>203</v>
+      </c>
+      <c r="E77" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F77" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -8258,7 +8412,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD7211D-DC17-4DD6-B657-CA08F8FBC20F}">
-  <dimension ref="A1:H128"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="20.453125" customWidth="1"/>
@@ -10484,7 +10638,7 @@
       <c r="B112" t="s">
         <v>154</v>
       </c>
-      <c r="F112" s="11">
+      <c r="F112">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -10500,7 +10654,7 @@
       <c r="B113" t="s">
         <v>153</v>
       </c>
-      <c r="F113" s="11">
+      <c r="F113">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -10516,7 +10670,7 @@
       <c r="B114" t="s">
         <v>158</v>
       </c>
-      <c r="F114" s="11">
+      <c r="F114">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -10532,7 +10686,7 @@
       <c r="B115" t="s">
         <v>157</v>
       </c>
-      <c r="F115" s="11">
+      <c r="F115">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -10548,7 +10702,7 @@
       <c r="B116" t="s">
         <v>161</v>
       </c>
-      <c r="F116" s="11">
+      <c r="F116">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -10564,7 +10718,7 @@
       <c r="B117" t="s">
         <v>161</v>
       </c>
-      <c r="F117" s="11">
+      <c r="F117">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -10580,7 +10734,7 @@
       <c r="B118" t="s">
         <v>161</v>
       </c>
-      <c r="F118" s="11">
+      <c r="F118">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -10596,7 +10750,7 @@
       <c r="B119" t="s">
         <v>178</v>
       </c>
-      <c r="F119" s="11">
+      <c r="F119">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -10612,7 +10766,7 @@
       <c r="B120" t="s">
         <v>157</v>
       </c>
-      <c r="F120" s="11">
+      <c r="F120">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -10620,30 +10774,6 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="121" spans="1:7">
-      <c r="F121" s="11"/>
-    </row>
-    <row r="122" spans="1:7">
-      <c r="F122" s="11"/>
-    </row>
-    <row r="123" spans="1:7">
-      <c r="F123" s="11"/>
-    </row>
-    <row r="124" spans="1:7">
-      <c r="F124" s="11"/>
-    </row>
-    <row r="125" spans="1:7">
-      <c r="F125" s="11"/>
-    </row>
-    <row r="126" spans="1:7">
-      <c r="F126" s="11"/>
-    </row>
-    <row r="127" spans="1:7">
-      <c r="F127" s="11"/>
-    </row>
-    <row r="128" spans="1:7">
-      <c r="F128" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="20" type="noConversion"/>
@@ -12996,7 +13126,7 @@
       <c r="B118" t="s">
         <v>154</v>
       </c>
-      <c r="F118" s="11">
+      <c r="F118">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -13012,7 +13142,7 @@
       <c r="B119" t="s">
         <v>153</v>
       </c>
-      <c r="F119" s="11">
+      <c r="F119">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -13028,7 +13158,7 @@
       <c r="B120" t="s">
         <v>158</v>
       </c>
-      <c r="F120" s="11">
+      <c r="F120">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -13044,7 +13174,7 @@
       <c r="B121" t="s">
         <v>157</v>
       </c>
-      <c r="F121" s="11">
+      <c r="F121">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -13060,7 +13190,7 @@
       <c r="B122" t="s">
         <v>161</v>
       </c>
-      <c r="F122" s="11">
+      <c r="F122">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -13076,7 +13206,7 @@
       <c r="B123" t="s">
         <v>161</v>
       </c>
-      <c r="F123" s="11">
+      <c r="F123">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -13092,7 +13222,7 @@
       <c r="B124" t="s">
         <v>161</v>
       </c>
-      <c r="F124" s="11">
+      <c r="F124">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -13108,7 +13238,7 @@
       <c r="B125" t="s">
         <v>178</v>
       </c>
-      <c r="F125" s="11">
+      <c r="F125">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -13124,7 +13254,7 @@
       <c r="B126" t="s">
         <v>157</v>
       </c>
-      <c r="F126" s="11">
+      <c r="F126">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>0</v>
       </c>
@@ -13792,9 +13922,911 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="21.81640625" customWidth="1"/>
+    <col min="4" max="4" width="9" customWidth="1"/>
+    <col min="6" max="6" width="11.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>187</v>
+      </c>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11">
+        <f t="shared" ref="E2:E5" si="0">D2/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F2" s="11"/>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F3" s="12"/>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F4" s="13"/>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>191</v>
+      </c>
+      <c r="B5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E5" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>192</v>
+      </c>
+      <c r="B6" t="s">
+        <v>187</v>
+      </c>
+      <c r="E6">
+        <f>D6/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>193</v>
+      </c>
+      <c r="B7" t="s">
+        <v>187</v>
+      </c>
+      <c r="E7">
+        <f>D7/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L7" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>186</v>
+      </c>
+      <c r="B8" t="s">
+        <v>194</v>
+      </c>
+      <c r="E8">
+        <f>D8/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L8" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>186</v>
+      </c>
+      <c r="B9" t="s">
+        <v>192</v>
+      </c>
+      <c r="E9">
+        <f>D9/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L9" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" t="s">
+        <v>195</v>
+      </c>
+      <c r="E10">
+        <f>D10/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L10" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>186</v>
+      </c>
+      <c r="B11" t="s">
+        <v>196</v>
+      </c>
+      <c r="E11">
+        <f>D11/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L11" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>186</v>
+      </c>
+      <c r="B12" t="s">
+        <v>197</v>
+      </c>
+      <c r="E12">
+        <f>D12/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L12" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>186</v>
+      </c>
+      <c r="B13" t="s">
+        <v>198</v>
+      </c>
+      <c r="E13">
+        <f>D13/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L13" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>186</v>
+      </c>
+      <c r="B14" t="s">
+        <v>199</v>
+      </c>
+      <c r="E14">
+        <f>D14/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L14" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B15" t="s">
+        <v>194</v>
+      </c>
+      <c r="E15">
+        <f>D15/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L15" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" t="s">
+        <v>189</v>
+      </c>
+      <c r="B16" t="s">
+        <v>192</v>
+      </c>
+      <c r="E16">
+        <f>D16/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L16" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" t="s">
+        <v>189</v>
+      </c>
+      <c r="B17" t="s">
+        <v>195</v>
+      </c>
+      <c r="E17">
+        <f>D17/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L17" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" t="s">
+        <v>189</v>
+      </c>
+      <c r="B18" t="s">
+        <v>196</v>
+      </c>
+      <c r="E18">
+        <f>D18/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L18" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" t="s">
+        <v>189</v>
+      </c>
+      <c r="B19" t="s">
+        <v>197</v>
+      </c>
+      <c r="E19">
+        <f>D19/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L19" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" t="s">
+        <v>189</v>
+      </c>
+      <c r="B20" t="s">
+        <v>198</v>
+      </c>
+      <c r="E20">
+        <f>D20/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" t="s">
+        <v>189</v>
+      </c>
+      <c r="B21" t="s">
+        <v>199</v>
+      </c>
+      <c r="E21">
+        <f>D21/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L21" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" t="s">
+        <v>190</v>
+      </c>
+      <c r="B22" t="s">
+        <v>194</v>
+      </c>
+      <c r="E22">
+        <f>D22/1000</f>
+        <v>0</v>
+      </c>
+      <c r="L22" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" t="s">
+        <v>190</v>
+      </c>
+      <c r="B23" t="s">
+        <v>192</v>
+      </c>
+      <c r="E23">
+        <f>D23/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" t="s">
+        <v>190</v>
+      </c>
+      <c r="B24" t="s">
+        <v>195</v>
+      </c>
+      <c r="E24">
+        <f>D24/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" t="s">
+        <v>190</v>
+      </c>
+      <c r="B25" t="s">
+        <v>196</v>
+      </c>
+      <c r="E25">
+        <f>D25/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" t="s">
+        <v>190</v>
+      </c>
+      <c r="B26" t="s">
+        <v>197</v>
+      </c>
+      <c r="E26">
+        <f>D26/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" t="s">
+        <v>190</v>
+      </c>
+      <c r="B27" t="s">
+        <v>198</v>
+      </c>
+      <c r="E27">
+        <f>D27/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" t="s">
+        <v>190</v>
+      </c>
+      <c r="B28" t="s">
+        <v>199</v>
+      </c>
+      <c r="E28">
+        <f>D28/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" t="s">
+        <v>191</v>
+      </c>
+      <c r="B29" t="s">
+        <v>194</v>
+      </c>
+      <c r="E29">
+        <f>D29/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" t="s">
+        <v>191</v>
+      </c>
+      <c r="B30" t="s">
+        <v>192</v>
+      </c>
+      <c r="E30">
+        <f t="shared" ref="E30:E35" si="1">D30/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" t="s">
+        <v>191</v>
+      </c>
+      <c r="B31" t="s">
+        <v>195</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" t="s">
+        <v>191</v>
+      </c>
+      <c r="B32" t="s">
+        <v>196</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" t="s">
+        <v>191</v>
+      </c>
+      <c r="B33" t="s">
+        <v>197</v>
+      </c>
+      <c r="E33">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" t="s">
+        <v>191</v>
+      </c>
+      <c r="B34" t="s">
+        <v>198</v>
+      </c>
+      <c r="E34">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" t="s">
+        <v>191</v>
+      </c>
+      <c r="B35" t="s">
+        <v>199</v>
+      </c>
+      <c r="E35">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" t="s">
+        <v>192</v>
+      </c>
+      <c r="B36" t="s">
+        <v>194</v>
+      </c>
+      <c r="E36">
+        <f>D36/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" t="s">
+        <v>192</v>
+      </c>
+      <c r="B37" t="s">
+        <v>192</v>
+      </c>
+      <c r="E37">
+        <f t="shared" ref="E37:E42" si="2">D37/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" t="s">
+        <v>192</v>
+      </c>
+      <c r="B38" t="s">
+        <v>195</v>
+      </c>
+      <c r="E38">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" t="s">
+        <v>192</v>
+      </c>
+      <c r="B39" t="s">
+        <v>196</v>
+      </c>
+      <c r="E39">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" t="s">
+        <v>192</v>
+      </c>
+      <c r="B40" t="s">
+        <v>197</v>
+      </c>
+      <c r="E40">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" t="s">
+        <v>192</v>
+      </c>
+      <c r="B41" t="s">
+        <v>198</v>
+      </c>
+      <c r="E41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" t="s">
+        <v>192</v>
+      </c>
+      <c r="B42" t="s">
+        <v>199</v>
+      </c>
+      <c r="E42">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" t="s">
+        <v>193</v>
+      </c>
+      <c r="B43" t="s">
+        <v>194</v>
+      </c>
+      <c r="E43">
+        <f>D43/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" t="s">
+        <v>193</v>
+      </c>
+      <c r="B44" t="s">
+        <v>192</v>
+      </c>
+      <c r="E44">
+        <f t="shared" ref="E44:E49" si="3">D44/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" t="s">
+        <v>193</v>
+      </c>
+      <c r="B45" t="s">
+        <v>195</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" t="s">
+        <v>193</v>
+      </c>
+      <c r="B46" t="s">
+        <v>196</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" t="s">
+        <v>193</v>
+      </c>
+      <c r="B47" t="s">
+        <v>197</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" t="s">
+        <v>193</v>
+      </c>
+      <c r="B48" t="s">
+        <v>198</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49" t="s">
+        <v>193</v>
+      </c>
+      <c r="B49" t="s">
+        <v>199</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" t="s">
+        <v>201</v>
+      </c>
+      <c r="B50" t="s">
+        <v>194</v>
+      </c>
+      <c r="E50">
+        <f>D50/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51" t="s">
+        <v>201</v>
+      </c>
+      <c r="B51" t="s">
+        <v>192</v>
+      </c>
+      <c r="E51">
+        <f t="shared" ref="E51:E56" si="4">D51/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52" t="s">
+        <v>201</v>
+      </c>
+      <c r="B52" t="s">
+        <v>195</v>
+      </c>
+      <c r="E52">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53" t="s">
+        <v>201</v>
+      </c>
+      <c r="B53" t="s">
+        <v>196</v>
+      </c>
+      <c r="E53">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54" t="s">
+        <v>201</v>
+      </c>
+      <c r="B54" t="s">
+        <v>197</v>
+      </c>
+      <c r="E54">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55" t="s">
+        <v>201</v>
+      </c>
+      <c r="B55" t="s">
+        <v>198</v>
+      </c>
+      <c r="E55">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" t="s">
+        <v>201</v>
+      </c>
+      <c r="B56" t="s">
+        <v>199</v>
+      </c>
+      <c r="E56">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" t="s">
+        <v>199</v>
+      </c>
+      <c r="B57" t="s">
+        <v>194</v>
+      </c>
+      <c r="E57">
+        <f>D57/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" t="s">
+        <v>199</v>
+      </c>
+      <c r="B58" t="s">
+        <v>192</v>
+      </c>
+      <c r="E58">
+        <f t="shared" ref="E58:E63" si="5">D58/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" t="s">
+        <v>199</v>
+      </c>
+      <c r="B59" t="s">
+        <v>195</v>
+      </c>
+      <c r="E59">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" t="s">
+        <v>199</v>
+      </c>
+      <c r="B60" t="s">
+        <v>196</v>
+      </c>
+      <c r="E60">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" t="s">
+        <v>199</v>
+      </c>
+      <c r="B61" t="s">
+        <v>197</v>
+      </c>
+      <c r="E61">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" t="s">
+        <v>199</v>
+      </c>
+      <c r="B62" t="s">
+        <v>198</v>
+      </c>
+      <c r="E62">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63" t="s">
+        <v>202</v>
+      </c>
+      <c r="B63" t="s">
+        <v>194</v>
+      </c>
+      <c r="E63">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" t="s">
+        <v>202</v>
+      </c>
+      <c r="B64" t="s">
+        <v>192</v>
+      </c>
+      <c r="E64">
+        <f t="shared" ref="E64:E69" si="6">D64/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65" t="s">
+        <v>202</v>
+      </c>
+      <c r="B65" t="s">
+        <v>195</v>
+      </c>
+      <c r="E65">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" t="s">
+        <v>202</v>
+      </c>
+      <c r="B66" t="s">
+        <v>196</v>
+      </c>
+      <c r="E66">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" t="s">
+        <v>202</v>
+      </c>
+      <c r="B67" t="s">
+        <v>197</v>
+      </c>
+      <c r="E67">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" t="s">
+        <v>202</v>
+      </c>
+      <c r="B68" t="s">
+        <v>198</v>
+      </c>
+      <c r="E68">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" t="s">
+        <v>202</v>
+      </c>
+      <c r="B69" t="s">
+        <v>199</v>
+      </c>
+      <c r="E69">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add Indonesia+Malaysia as new region in Asia
relevant to depict LNG-Imports and Exports in the region.
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F073AE-A613-4179-B460-114D223FC2E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60F18701-D4B7-4083-9494-0B080BCDF8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1370" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1360" uniqueCount="204">
   <si>
     <t>Belgium</t>
   </si>
@@ -960,7 +960,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -972,9 +972,8 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -1021,6 +1020,42 @@
   </cellStyles>
   <dxfs count="40">
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <right style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -1043,36 +1078,6 @@
           <bgColor theme="4"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </left>
-        <right style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </right>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1243,12 +1248,6 @@
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -1345,7 +1344,7 @@
     <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="4">
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="6">
       <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
@@ -1358,7 +1357,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:F69" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="2" tableBorderDxfId="3" totalsRowBorderDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:F69" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
   <autoFilter ref="A1:F69" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
@@ -1377,18 +1376,18 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F68" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33">
-  <autoFilter ref="A53:F68" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F69" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33">
+  <autoFilter ref="A53:F69" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3F684FB4-9656-4C92-BAF4-456019B2B924}" name="Country"/>
     <tableColumn id="2" xr3:uid="{082B059D-405D-407D-8F97-297DCD23D3B2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{388F462C-127F-4CB7-B46A-1DD19D06D0E8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{ACDF4345-6201-4524-A8D7-A0CE31D137A6}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="32">
-      <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
+    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="1">
+      <calculatedColumnFormula>Table7[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="31">
-      <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="0">
+      <calculatedColumnFormula>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1404,12 +1403,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="28">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="30">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="27">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="29">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1418,17 +1417,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F67" totalsRowShown="0" headerRowDxfId="26" headerRowBorderDxfId="25" tableBorderDxfId="24">
-  <autoFilter ref="A52:F67" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F68" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="27" tableBorderDxfId="26">
+  <autoFilter ref="A52:F68" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{02819FD0-F6B6-484E-B4DA-8262AECE7052}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{A15C284E-E91C-44C6-B3BB-CC2DD205DA84}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="23">
+    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="25">
       <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="22">
+    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="24">
       <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1445,12 +1444,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="20">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="22">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="19">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="21">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1459,17 +1458,17 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F76" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16">
-  <autoFilter ref="A57:F76" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F77" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18">
+  <autoFilter ref="A57:F77" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{555371BF-8030-4257-9852-212E94829B9B}" name="Country"/>
     <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="15">
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="17">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="14">
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="16">
       <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1486,12 +1485,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="12">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="14">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="11">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="13">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1500,17 +1499,17 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F77" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="9" tableBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F77" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10">
   <autoFilter ref="A57:F77" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{779C3748-4ECD-495F-809A-B5DD28F5EC2F}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{94BC7314-C5A0-4AAD-895B-84E7A94D7CF7}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="7">
+    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="9">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="6">
+    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="8">
       <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1530,7 +1529,7 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="5">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="7">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
@@ -2517,7 +2516,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF82F4-4954-4D06-9A30-AE8575CA18DE}">
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -3814,12 +3813,12 @@
       </c>
       <c r="D54" s="7"/>
       <c r="E54" s="7">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F54" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2206.4451910864968</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>9035.4222937216473</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -3834,12 +3833,12 @@
         <v>201.13828091020829</v>
       </c>
       <c r="E55" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F55" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1338.7623107718482</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1965.121004492735</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -3854,12 +3853,12 @@
         <v>127.15388122807011</v>
       </c>
       <c r="E56" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F56" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>244.18753104004941</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1242.2934195982448</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -3873,12 +3872,12 @@
         <v>29.4652641615749</v>
       </c>
       <c r="E57" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F57" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>5194.9769121760055</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>287.87563085858676</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -3893,12 +3892,12 @@
         <v>493.00454191430799</v>
       </c>
       <c r="E58" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F58" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1768.1412507539624</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>4816.6543745027893</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -3912,12 +3911,12 @@
         <v>174.93483781719999</v>
       </c>
       <c r="E59" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F59" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>750.8692287163949</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1709.1133654740438</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -3932,12 +3931,12 @@
         <v>77.419550083247572</v>
       </c>
       <c r="E60" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F60" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1482.5018882394202</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>756.38900431332877</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -3951,12 +3950,12 @@
         <v>145.71638020075315</v>
       </c>
       <c r="E61" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F61" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2288.704156833825</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1423.6490345613581</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -3970,12 +3969,12 @@
         <v>194.00921828908548</v>
       </c>
       <c r="E62" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F62" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>0</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1895.4700626843651</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -3989,12 +3988,12 @@
         <v>0</v>
       </c>
       <c r="E63" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F63" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>308.59022299160773</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -4008,12 +4007,12 @@
         <v>23.760626555099513</v>
       </c>
       <c r="E64" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F64" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2679.4711234932433</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>232.14132144332223</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -4024,16 +4023,16 @@
         <v>175</v>
       </c>
       <c r="C65">
-        <f>656.2735508682-C64-C62-C61-C63</f>
-        <v>292.78732582326188</v>
+        <f>656.2735508682-C64-C62-C61-C63-C69</f>
+        <v>154.99710695848057</v>
       </c>
       <c r="E65" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F65" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1828.6593022261925</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1514.3217349843551</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -4048,12 +4047,12 @@
         <v>169.91079422395296</v>
       </c>
       <c r="E66" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F66" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>5728.9540927535336</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1660.0284595680205</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -4067,12 +4066,12 @@
         <v>638.446656032448</v>
       </c>
       <c r="E67" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F67" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>557.87103573034665</v>
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>6237.6238294370169</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -4085,13 +4084,33 @@
       <c r="C68">
         <v>58.465174157714841</v>
       </c>
-      <c r="E68" s="2" t="e">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F68" s="3" t="e">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>#VALUE!</v>
+      <c r="E68" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F68" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>571.20475152087397</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="A69" t="s">
+        <v>200</v>
+      </c>
+      <c r="B69" t="s">
+        <v>203</v>
+      </c>
+      <c r="C69">
+        <f>64.6974253845862+73.0927934801951</f>
+        <v>137.79021886478131</v>
+      </c>
+      <c r="E69" s="2">
+        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F69" s="3">
+        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1346.2104383089134</v>
       </c>
     </row>
   </sheetData>
@@ -4105,7 +4124,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{036BBBE1-80BC-4BBB-9141-C576056723F9}">
-  <dimension ref="A1:M67"/>
+  <dimension ref="A1:M68"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -5607,8 +5626,8 @@
         <v>175</v>
       </c>
       <c r="C64">
-        <f>691.83903700697-C63-C61-C60-C62</f>
-        <v>274.25497681609454</v>
+        <f>691.83903700697-C63-C61-C60-C62-C68</f>
+        <v>128.91680453343903</v>
       </c>
       <c r="E64" s="2">
         <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
@@ -5616,7 +5635,7 @@
       </c>
       <c r="F64" s="3">
         <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2679.4711234932433</v>
+        <v>1259.5171802916993</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -5675,6 +5694,26 @@
       <c r="F67" s="3">
         <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
         <v>557.87103573034665</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" t="s">
+        <v>200</v>
+      </c>
+      <c r="B68" t="s">
+        <v>203</v>
+      </c>
+      <c r="C68">
+        <f>64.2640381356325+81.074134147023</f>
+        <v>145.33817228265551</v>
+      </c>
+      <c r="E68" s="2">
+        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F68" s="3">
+        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1419.9539432015442</v>
       </c>
     </row>
   </sheetData>
@@ -6868,8 +6907,8 @@
         <v>175</v>
       </c>
       <c r="C69">
-        <f>876.9412368709-C68-C66-C65-C67</f>
-        <v>275.9817057732655</v>
+        <f>876.9412368709-C68-C66-C65-C67-C77</f>
+        <v>189.7875106376263</v>
       </c>
       <c r="E69" s="2">
         <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
@@ -6877,7 +6916,7 @@
       </c>
       <c r="F69" s="3">
         <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2642.5076198591928</v>
+        <v>1748.3915086808172</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -7012,6 +7051,26 @@
       <c r="F76" s="3">
         <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
         <v>586.63367669240563</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
+      <c r="A77" t="s">
+        <v>200</v>
+      </c>
+      <c r="B77" t="s">
+        <v>203</v>
+      </c>
+      <c r="C77">
+        <f>42.5805321356392+43.613663</f>
+        <v>86.194195135639205</v>
+      </c>
+      <c r="E77" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F77" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>894.11611117837549</v>
       </c>
     </row>
     <row r="79" spans="1:8">
@@ -8223,8 +8282,8 @@
         <v>175</v>
       </c>
       <c r="C69">
-        <f>935.383807806868-C68-C66-C65-C67</f>
-        <v>270.47160899275258</v>
+        <f>935.383807806868-C68-C66-C65-C67-C77</f>
+        <v>178.95511859578477</v>
       </c>
       <c r="E69" s="2">
         <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
@@ -8232,7 +8291,7 @@
       </c>
       <c r="F69" s="3">
         <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2642.5076198591928</v>
+        <v>1748.3915086808172</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -8376,13 +8435,17 @@
       <c r="B77" t="s">
         <v>203</v>
       </c>
+      <c r="C77">
+        <f>45.4449851278232+46.0715052691446</f>
+        <v>91.516490396967811</v>
+      </c>
       <c r="E77" s="2">
         <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F77" s="3">
         <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>0</v>
+        <v>894.11611117837549</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -13922,7 +13985,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="21.81640625" customWidth="1"/>
@@ -13930,7 +13993,7 @@
     <col min="6" max="6" width="11.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:6">
       <c r="A1" s="9" t="s">
         <v>93</v>
       </c>
@@ -13950,64 +14013,64 @@
         <v>144</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:6">
+      <c r="A2" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11">
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6">
         <f t="shared" ref="E2:E5" si="0">D2/1000</f>
         <v>0</v>
       </c>
-      <c r="F2" s="11"/>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="A3" s="12" t="s">
+      <c r="F2" s="6"/>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="11" t="s">
         <v>189</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>187</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F3" s="12"/>
-    </row>
-    <row r="4" spans="1:12">
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F3" s="11"/>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>190</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="F4" s="13"/>
-    </row>
-    <row r="5" spans="1:12">
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F4" s="12"/>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>191</v>
       </c>
       <c r="B5" t="s">
         <v>187</v>
       </c>
-      <c r="E5" s="12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
+      <c r="E5" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>192</v>
       </c>
@@ -14015,11 +14078,11 @@
         <v>187</v>
       </c>
       <c r="E6">
-        <f>D6/1000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
+        <f t="shared" ref="E6:E29" si="1">D6/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>193</v>
       </c>
@@ -14027,14 +14090,11 @@
         <v>187</v>
       </c>
       <c r="E7">
-        <f>D7/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L7" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>186</v>
       </c>
@@ -14042,14 +14102,11 @@
         <v>194</v>
       </c>
       <c r="E8">
-        <f>D8/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L8" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>186</v>
       </c>
@@ -14057,14 +14114,11 @@
         <v>192</v>
       </c>
       <c r="E9">
-        <f>D9/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L9" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>186</v>
       </c>
@@ -14072,14 +14126,11 @@
         <v>195</v>
       </c>
       <c r="E10">
-        <f>D10/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L10" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>186</v>
       </c>
@@ -14087,14 +14138,11 @@
         <v>196</v>
       </c>
       <c r="E11">
-        <f>D11/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L11" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>186</v>
       </c>
@@ -14102,14 +14150,11 @@
         <v>197</v>
       </c>
       <c r="E12">
-        <f>D12/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L12" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>186</v>
       </c>
@@ -14117,14 +14162,11 @@
         <v>198</v>
       </c>
       <c r="E13">
-        <f>D13/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L13" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>186</v>
       </c>
@@ -14132,14 +14174,11 @@
         <v>199</v>
       </c>
       <c r="E14">
-        <f>D14/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L14" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>189</v>
       </c>
@@ -14147,14 +14186,11 @@
         <v>194</v>
       </c>
       <c r="E15">
-        <f>D15/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L15" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>189</v>
       </c>
@@ -14162,14 +14198,11 @@
         <v>192</v>
       </c>
       <c r="E16">
-        <f>D16/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L16" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17" t="s">
         <v>189</v>
       </c>
@@ -14177,14 +14210,11 @@
         <v>195</v>
       </c>
       <c r="E17">
-        <f>D17/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L17" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
       <c r="A18" t="s">
         <v>189</v>
       </c>
@@ -14192,14 +14222,11 @@
         <v>196</v>
       </c>
       <c r="E18">
-        <f>D18/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L18" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
       <c r="A19" t="s">
         <v>189</v>
       </c>
@@ -14207,14 +14234,11 @@
         <v>197</v>
       </c>
       <c r="E19">
-        <f>D19/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L19" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
         <v>189</v>
       </c>
@@ -14222,14 +14246,11 @@
         <v>198</v>
       </c>
       <c r="E20">
-        <f>D20/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L20" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
       <c r="A21" t="s">
         <v>189</v>
       </c>
@@ -14237,14 +14258,11 @@
         <v>199</v>
       </c>
       <c r="E21">
-        <f>D21/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L21" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
       <c r="A22" t="s">
         <v>190</v>
       </c>
@@ -14252,14 +14270,11 @@
         <v>194</v>
       </c>
       <c r="E22">
-        <f>D22/1000</f>
-        <v>0</v>
-      </c>
-      <c r="L22" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
       <c r="A23" t="s">
         <v>190</v>
       </c>
@@ -14267,11 +14282,11 @@
         <v>192</v>
       </c>
       <c r="E23">
-        <f>D23/1000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
       <c r="A24" t="s">
         <v>190</v>
       </c>
@@ -14279,11 +14294,11 @@
         <v>195</v>
       </c>
       <c r="E24">
-        <f>D24/1000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
       <c r="A25" t="s">
         <v>190</v>
       </c>
@@ -14291,11 +14306,11 @@
         <v>196</v>
       </c>
       <c r="E25">
-        <f>D25/1000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
       <c r="A26" t="s">
         <v>190</v>
       </c>
@@ -14303,11 +14318,11 @@
         <v>197</v>
       </c>
       <c r="E26">
-        <f>D26/1000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
       <c r="A27" t="s">
         <v>190</v>
       </c>
@@ -14315,11 +14330,11 @@
         <v>198</v>
       </c>
       <c r="E27">
-        <f>D27/1000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
       <c r="A28" t="s">
         <v>190</v>
       </c>
@@ -14327,11 +14342,11 @@
         <v>199</v>
       </c>
       <c r="E28">
-        <f>D28/1000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
       <c r="A29" t="s">
         <v>191</v>
       </c>
@@ -14339,11 +14354,11 @@
         <v>194</v>
       </c>
       <c r="E29">
-        <f>D29/1000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
       <c r="A30" t="s">
         <v>191</v>
       </c>
@@ -14351,11 +14366,11 @@
         <v>192</v>
       </c>
       <c r="E30">
-        <f t="shared" ref="E30:E35" si="1">D30/1000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12">
+        <f t="shared" ref="E30:E35" si="2">D30/1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
       <c r="A31" t="s">
         <v>191</v>
       </c>
@@ -14363,11 +14378,11 @@
         <v>195</v>
       </c>
       <c r="E31">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
       <c r="A32" t="s">
         <v>191</v>
       </c>
@@ -14375,7 +14390,7 @@
         <v>196</v>
       </c>
       <c r="E32">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -14387,7 +14402,7 @@
         <v>197</v>
       </c>
       <c r="E33">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -14399,7 +14414,7 @@
         <v>198</v>
       </c>
       <c r="E34">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -14411,7 +14426,7 @@
         <v>199</v>
       </c>
       <c r="E35">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -14435,7 +14450,7 @@
         <v>192</v>
       </c>
       <c r="E37">
-        <f t="shared" ref="E37:E42" si="2">D37/1000</f>
+        <f t="shared" ref="E37:E42" si="3">D37/1000</f>
         <v>0</v>
       </c>
     </row>
@@ -14447,7 +14462,7 @@
         <v>195</v>
       </c>
       <c r="E38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -14459,7 +14474,7 @@
         <v>196</v>
       </c>
       <c r="E39">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -14471,7 +14486,7 @@
         <v>197</v>
       </c>
       <c r="E40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -14483,7 +14498,7 @@
         <v>198</v>
       </c>
       <c r="E41">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -14495,7 +14510,7 @@
         <v>199</v>
       </c>
       <c r="E42">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
@@ -14519,7 +14534,7 @@
         <v>192</v>
       </c>
       <c r="E44">
-        <f t="shared" ref="E44:E49" si="3">D44/1000</f>
+        <f t="shared" ref="E44:E49" si="4">D44/1000</f>
         <v>0</v>
       </c>
     </row>
@@ -14531,7 +14546,7 @@
         <v>195</v>
       </c>
       <c r="E45">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -14543,7 +14558,7 @@
         <v>196</v>
       </c>
       <c r="E46">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -14555,7 +14570,7 @@
         <v>197</v>
       </c>
       <c r="E47">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -14567,7 +14582,7 @@
         <v>198</v>
       </c>
       <c r="E48">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -14579,7 +14594,7 @@
         <v>199</v>
       </c>
       <c r="E49">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -14603,7 +14618,7 @@
         <v>192</v>
       </c>
       <c r="E51">
-        <f t="shared" ref="E51:E56" si="4">D51/1000</f>
+        <f t="shared" ref="E51:E56" si="5">D51/1000</f>
         <v>0</v>
       </c>
     </row>
@@ -14615,7 +14630,7 @@
         <v>195</v>
       </c>
       <c r="E52">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -14627,7 +14642,7 @@
         <v>196</v>
       </c>
       <c r="E53">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -14639,7 +14654,7 @@
         <v>197</v>
       </c>
       <c r="E54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -14651,7 +14666,7 @@
         <v>198</v>
       </c>
       <c r="E55">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -14663,7 +14678,7 @@
         <v>199</v>
       </c>
       <c r="E56">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
@@ -14687,7 +14702,7 @@
         <v>192</v>
       </c>
       <c r="E58">
-        <f t="shared" ref="E58:E63" si="5">D58/1000</f>
+        <f t="shared" ref="E58:E63" si="6">D58/1000</f>
         <v>0</v>
       </c>
     </row>
@@ -14699,7 +14714,7 @@
         <v>195</v>
       </c>
       <c r="E59">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -14711,7 +14726,7 @@
         <v>196</v>
       </c>
       <c r="E60">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -14723,7 +14738,7 @@
         <v>197</v>
       </c>
       <c r="E61">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -14735,7 +14750,7 @@
         <v>198</v>
       </c>
       <c r="E62">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -14747,7 +14762,7 @@
         <v>194</v>
       </c>
       <c r="E63">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -14759,7 +14774,7 @@
         <v>192</v>
       </c>
       <c r="E64">
-        <f t="shared" ref="E64:E69" si="6">D64/1000</f>
+        <f t="shared" ref="E64:E69" si="7">D64/1000</f>
         <v>0</v>
       </c>
     </row>
@@ -14771,7 +14786,7 @@
         <v>195</v>
       </c>
       <c r="E65">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -14783,7 +14798,7 @@
         <v>196</v>
       </c>
       <c r="E66">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -14795,7 +14810,7 @@
         <v>197</v>
       </c>
       <c r="E67">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -14807,7 +14822,7 @@
         <v>198</v>
       </c>
       <c r="E68">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -14819,7 +14834,7 @@
         <v>199</v>
       </c>
       <c r="E69">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add data to input sheet for the model
for testing
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60F18701-D4B7-4083-9494-0B080BCDF8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63999AC2-7D26-46E1-A4D0-CBA0ECD083B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1360" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1364" uniqueCount="203">
   <si>
     <t>Belgium</t>
   </si>
@@ -551,9 +551,6 @@
   </si>
   <si>
     <t>Middle East</t>
-  </si>
-  <si>
-    <t>Quatar</t>
   </si>
   <si>
     <t>Africa</t>
@@ -1139,12 +1136,6 @@
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -1243,6 +1234,12 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
@@ -1383,10 +1380,10 @@
     <tableColumn id="2" xr3:uid="{082B059D-405D-407D-8F97-297DCD23D3B2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{388F462C-127F-4CB7-B46A-1DD19D06D0E8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{ACDF4345-6201-4524-A8D7-A0CE31D137A6}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="1">
+    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="32">
       <calculatedColumnFormula>Table7[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="31">
       <calculatedColumnFormula>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1403,12 +1400,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="30">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="28">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="29">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="27">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1417,17 +1414,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F68" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="27" tableBorderDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F68" totalsRowShown="0" headerRowDxfId="26" headerRowBorderDxfId="25" tableBorderDxfId="24">
   <autoFilter ref="A52:F68" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{02819FD0-F6B6-484E-B4DA-8262AECE7052}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{A15C284E-E91C-44C6-B3BB-CC2DD205DA84}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="25">
+    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="23">
       <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="24">
+    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="22">
       <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1444,12 +1441,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="22">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="20">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="21">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="19">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1458,18 +1455,18 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F77" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18">
-  <autoFilter ref="A57:F77" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F78" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16">
+  <autoFilter ref="A57:F78" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{555371BF-8030-4257-9852-212E94829B9B}" name="Country"/>
     <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="17">
-      <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="1">
+      <calculatedColumnFormula>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="16">
-      <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="0">
+      <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1499,8 +1496,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F77" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10">
-  <autoFilter ref="A57:F77" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F78" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10">
+  <autoFilter ref="A57:F78" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
@@ -3792,10 +3789,10 @@
         <v>85</v>
       </c>
       <c r="D53" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="E53" s="9" t="s">
         <v>176</v>
-      </c>
-      <c r="E53" s="9" t="s">
-        <v>177</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>106</v>
@@ -3905,7 +3902,7 @@
         <v>158</v>
       </c>
       <c r="B59" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="C59">
         <v>174.93483781719999</v>
@@ -3924,7 +3921,7 @@
         <v>159</v>
       </c>
       <c r="B60" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C60" s="2">
         <f>231.909048813308-C21-C3-C37-C68</f>
@@ -3944,7 +3941,7 @@
         <v>160</v>
       </c>
       <c r="B61" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C61">
         <v>145.71638020075315</v>
@@ -3963,7 +3960,7 @@
         <v>161</v>
       </c>
       <c r="B62" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C62">
         <v>194.00921828908548</v>
@@ -3982,7 +3979,7 @@
         <v>162</v>
       </c>
       <c r="B63" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -4001,7 +3998,7 @@
         <v>163</v>
       </c>
       <c r="B64" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C64">
         <v>23.760626555099513</v>
@@ -4020,7 +4017,7 @@
         <v>164</v>
       </c>
       <c r="B65" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C65">
         <f>656.2735508682-C64-C62-C61-C63-C69</f>
@@ -4037,10 +4034,10 @@
     </row>
     <row r="66" spans="1:6">
       <c r="A66" t="s">
+        <v>177</v>
+      </c>
+      <c r="B66" t="s">
         <v>178</v>
-      </c>
-      <c r="B66" t="s">
-        <v>179</v>
       </c>
       <c r="C66">
         <f>808.357450256401-638.446656032448</f>
@@ -4076,10 +4073,10 @@
     </row>
     <row r="68" spans="1:6">
       <c r="A68" t="s">
+        <v>183</v>
+      </c>
+      <c r="B68" t="s">
         <v>184</v>
-      </c>
-      <c r="B68" t="s">
-        <v>185</v>
       </c>
       <c r="C68">
         <v>58.465174157714841</v>
@@ -4095,10 +4092,10 @@
     </row>
     <row r="69" spans="1:6">
       <c r="A69" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B69" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C69">
         <f>64.6974253845862+73.0927934801951</f>
@@ -5395,10 +5392,10 @@
         <v>85</v>
       </c>
       <c r="D52" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="E52" s="9" t="s">
         <v>176</v>
-      </c>
-      <c r="E52" s="9" t="s">
-        <v>177</v>
       </c>
       <c r="F52" s="10" t="s">
         <v>106</v>
@@ -5508,7 +5505,7 @@
         <v>158</v>
       </c>
       <c r="B58" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="C58">
         <v>180.976586566424</v>
@@ -5527,7 +5524,7 @@
         <v>159</v>
       </c>
       <c r="B59" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C59" s="2">
         <f>253.649617284986-C21-C3-C37-C67</f>
@@ -5547,7 +5544,7 @@
         <v>160</v>
       </c>
       <c r="B60" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C60">
         <v>151.74021373996112</v>
@@ -5566,7 +5563,7 @@
         <v>161</v>
       </c>
       <c r="B61" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C61">
         <v>234.25835791543756</v>
@@ -5585,7 +5582,7 @@
         <v>162</v>
       </c>
       <c r="B62" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -5604,7 +5601,7 @@
         <v>163</v>
       </c>
       <c r="B63" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C63">
         <v>31.585488535476742</v>
@@ -5623,7 +5620,7 @@
         <v>164</v>
       </c>
       <c r="B64" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C64">
         <f>691.83903700697-C63-C61-C60-C62-C68</f>
@@ -5640,10 +5637,10 @@
     </row>
     <row r="65" spans="1:6">
       <c r="A65" t="s">
+        <v>177</v>
+      </c>
+      <c r="B65" t="s">
         <v>178</v>
-      </c>
-      <c r="B65" t="s">
-        <v>179</v>
       </c>
       <c r="C65">
         <f>773.5530598751-586.382199872419</f>
@@ -5679,10 +5676,10 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" t="s">
+        <v>183</v>
+      </c>
+      <c r="B67" t="s">
         <v>184</v>
-      </c>
-      <c r="B67" t="s">
-        <v>185</v>
       </c>
       <c r="C67">
         <v>57.100413073730465</v>
@@ -5698,10 +5695,10 @@
     </row>
     <row r="68" spans="1:6">
       <c r="A68" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B68" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C68">
         <f>64.2640381356325+81.074134147023</f>
@@ -5727,7 +5724,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE55996C-4401-4161-B17D-CF2A8462856A}">
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -6674,10 +6671,10 @@
         <v>85</v>
       </c>
       <c r="D57" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="E57" s="9" t="s">
         <v>176</v>
-      </c>
-      <c r="E57" s="9" t="s">
-        <v>177</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>106</v>
@@ -6695,12 +6692,12 @@
       </c>
       <c r="D58" s="7"/>
       <c r="E58" s="7">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F58" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>8660.7846598998185</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>8153.5498638127028</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -6715,12 +6712,12 @@
         <v>207.53535538062306</v>
       </c>
       <c r="E59" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F59" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2132.7907642308792</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>2027.6204220686873</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -6735,12 +6732,12 @@
         <v>133.38441274283269</v>
       </c>
       <c r="E60" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F60" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1438.139604719081</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1303.1657124974754</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -6755,12 +6752,12 @@
         <v>15.1856471767803</v>
       </c>
       <c r="E61" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F61" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>141.70363816030851</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>148.36377291714354</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -6775,12 +6772,12 @@
         <v>514.48426524852835</v>
       </c>
       <c r="E62" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F62" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>5212.4455255534276</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>5026.5112714781217</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -6788,18 +6785,18 @@
         <v>158</v>
       </c>
       <c r="B63" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C63">
         <v>38.413234709056603</v>
       </c>
       <c r="E63" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F63" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>431.84687643593901</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>375.297303107483</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -6807,19 +6804,19 @@
         <v>159</v>
       </c>
       <c r="B64" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C64" s="2">
         <f>154.184349315883-C72-C73-C74-C75-C76</f>
         <v>40.449273476568081</v>
       </c>
       <c r="E64" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F64" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>458.53340662554189</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>395.18940186607011</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -6827,18 +6824,18 @@
         <v>160</v>
       </c>
       <c r="B65" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C65">
         <v>42.317339828787539</v>
       </c>
       <c r="E65" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F65" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>391.98708472127618</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>413.44041012725421</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -6846,18 +6843,18 @@
         <v>161</v>
       </c>
       <c r="B66" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C66">
         <v>336.61725663716805</v>
       </c>
       <c r="E66" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F66" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>4002.6213997252307</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>3288.7505973451316</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -6865,19 +6862,19 @@
         <v>162</v>
       </c>
       <c r="B67" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C67">
         <f>104.1275049683+57.53730834</f>
         <v>161.66481330830001</v>
       </c>
       <c r="E67" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F67" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1489.8809967005398</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1579.465226022091</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -6885,18 +6882,18 @@
         <v>163</v>
       </c>
       <c r="B68" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C68">
         <v>60.360121323378813</v>
       </c>
       <c r="E68" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F68" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>611.70270126686103</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>589.71838532941092</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -6904,39 +6901,39 @@
         <v>164</v>
       </c>
       <c r="B69" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C69">
         <f>876.9412368709-C68-C66-C65-C67-C77</f>
         <v>189.7875106376263</v>
       </c>
       <c r="E69" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F69" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1748.3915086808172</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1854.2239789296088</v>
       </c>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
+        <v>177</v>
+      </c>
+      <c r="B70" t="s">
         <v>178</v>
-      </c>
-      <c r="B70" t="s">
-        <v>179</v>
       </c>
       <c r="C70">
         <f>554.955290969357-423.483407079646</f>
         <v>131.47188388971097</v>
       </c>
       <c r="E70" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F70" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1393.657265723991</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>1284.4803056024762</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -6950,12 +6947,12 @@
         <v>423.48340707964599</v>
       </c>
       <c r="E71" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F71" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>4429.4341224188756</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>4137.432887168141</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -6969,12 +6966,12 @@
         <v>43.350037499999999</v>
       </c>
       <c r="E72" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F72" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>491.80958750000002</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>423.52986637499998</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -6988,12 +6985,12 @@
         <v>7.7</v>
       </c>
       <c r="E73" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F73" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>98.676999999999992</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>75.228999999999999</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -7007,11 +7004,11 @@
         <v>3.5904531497162</v>
       </c>
       <c r="E74" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F74" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
         <v>35.078727272727271</v>
       </c>
     </row>
@@ -7020,76 +7017,95 @@
         <v>98</v>
       </c>
       <c r="B75" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C75">
         <v>0.78666131450805166</v>
       </c>
       <c r="E75" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F75" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2.1757375189927228</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>7.6856810427436644</v>
       </c>
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
+        <v>183</v>
+      </c>
+      <c r="B76" t="s">
         <v>184</v>
-      </c>
-      <c r="B76" t="s">
-        <v>185</v>
       </c>
       <c r="C76">
         <v>58.307923875090665</v>
       </c>
       <c r="E76" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F76" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>586.63367669240563</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>569.66841625963582</v>
       </c>
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B77" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C77">
         <f>42.5805321356392+43.613663</f>
         <v>86.194195135639205</v>
       </c>
       <c r="E77" s="2">
-        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F77" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>894.11611117837549</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8">
-      <c r="A79" t="s">
-        <v>80</v>
-      </c>
-      <c r="B79" t="s">
-        <v>138</v>
-      </c>
-      <c r="H79" t="s">
-        <v>139</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>842.11728647519499</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
+      <c r="A78" t="s">
+        <v>53</v>
+      </c>
+      <c r="B78" t="s">
+        <v>82</v>
+      </c>
+      <c r="C78">
+        <v>17.751008849557518</v>
+      </c>
+      <c r="E78" s="2">
+        <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="3">
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>173.42735646017695</v>
       </c>
     </row>
     <row r="80" spans="1:8">
       <c r="A80" t="s">
+        <v>80</v>
+      </c>
+      <c r="B80" t="s">
+        <v>138</v>
+      </c>
+      <c r="H80" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
         <v>81</v>
       </c>
-      <c r="B80" t="s">
-        <v>183</v>
+      <c r="B81" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -7103,7 +7119,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06AEBB83-8C6D-4234-B52F-BC23EBBF1927}">
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -8049,10 +8065,10 @@
         <v>85</v>
       </c>
       <c r="D57" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="E57" s="9" t="s">
         <v>176</v>
-      </c>
-      <c r="E57" s="9" t="s">
-        <v>177</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>106</v>
@@ -8162,7 +8178,7 @@
         <v>158</v>
       </c>
       <c r="B63" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C63">
         <v>44.201317956595602</v>
@@ -8181,7 +8197,7 @@
         <v>159</v>
       </c>
       <c r="B64" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C64" s="2">
         <f>171.229082457489-C72-C73-C74-C75-C76</f>
@@ -8201,7 +8217,7 @@
         <v>160</v>
       </c>
       <c r="B65" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C65">
         <v>40.121503042095824</v>
@@ -8220,7 +8236,7 @@
         <v>161</v>
       </c>
       <c r="B66" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C66">
         <f>404.838112094395+4.84678040562862</f>
@@ -8240,7 +8256,7 @@
         <v>162</v>
       </c>
       <c r="B67" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C67">
         <f>92.4207922536915+60.0747038262</f>
@@ -8260,7 +8276,7 @@
         <v>163</v>
       </c>
       <c r="B68" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C68">
         <v>62.610307192104507</v>
@@ -8279,7 +8295,7 @@
         <v>164</v>
       </c>
       <c r="B69" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C69">
         <f>935.383807806868-C68-C66-C65-C67-C77</f>
@@ -8296,10 +8312,10 @@
     </row>
     <row r="70" spans="1:6">
       <c r="A70" t="s">
+        <v>177</v>
+      </c>
+      <c r="B70" t="s">
         <v>178</v>
-      </c>
-      <c r="B70" t="s">
-        <v>179</v>
       </c>
       <c r="C70">
         <f>596.017542286885-453.370943952802</f>
@@ -8395,7 +8411,7 @@
         <v>98</v>
       </c>
       <c r="B75" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C75">
         <v>0.22269575424695218</v>
@@ -8411,10 +8427,10 @@
     </row>
     <row r="76" spans="1:6">
       <c r="A76" t="s">
+        <v>183</v>
+      </c>
+      <c r="B76" t="s">
         <v>184</v>
-      </c>
-      <c r="B76" t="s">
-        <v>185</v>
       </c>
       <c r="C76">
         <v>60.044388607206308</v>
@@ -8430,10 +8446,10 @@
     </row>
     <row r="77" spans="1:6">
       <c r="A77" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B77" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C77">
         <f>45.4449851278232+46.0715052691446</f>
@@ -8448,20 +8464,39 @@
         <v>894.11611117837549</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
-      <c r="A79" t="s">
-        <v>80</v>
-      </c>
-      <c r="B79" t="s">
-        <v>138</v>
+    <row r="78" spans="1:6">
+      <c r="A78" t="s">
+        <v>53</v>
+      </c>
+      <c r="B78" t="s">
+        <v>82</v>
+      </c>
+      <c r="C78">
+        <v>16.784035990584055</v>
+      </c>
+      <c r="E78" s="2">
+        <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="3">
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
+        <v>163.9800316280062</v>
       </c>
     </row>
     <row r="80" spans="1:6">
       <c r="A80" t="s">
+        <v>80</v>
+      </c>
+      <c r="B80" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
         <v>81</v>
       </c>
-      <c r="B80" t="s">
-        <v>183</v>
+      <c r="B81" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -10513,7 +10548,7 @@
     </row>
     <row r="103" spans="1:8">
       <c r="A103" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B103" t="s">
         <v>47</v>
@@ -10776,7 +10811,7 @@
     </row>
     <row r="117" spans="1:7">
       <c r="A117" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B117" t="s">
         <v>161</v>
@@ -10811,7 +10846,7 @@
         <v>41</v>
       </c>
       <c r="B119" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F119">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -10824,7 +10859,7 @@
     </row>
     <row r="120" spans="1:7">
       <c r="A120" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B120" t="s">
         <v>157</v>
@@ -13001,7 +13036,7 @@
     </row>
     <row r="109" spans="1:8">
       <c r="A109" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B109" t="s">
         <v>47</v>
@@ -13018,7 +13053,7 @@
         <v>136.875</v>
       </c>
       <c r="H109" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -13264,7 +13299,7 @@
     </row>
     <row r="123" spans="1:7">
       <c r="A123" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B123" t="s">
         <v>161</v>
@@ -13299,7 +13334,7 @@
         <v>41</v>
       </c>
       <c r="B125" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F125">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -13312,7 +13347,7 @@
     </row>
     <row r="126" spans="1:7">
       <c r="A126" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B126" t="s">
         <v>157</v>
@@ -13377,7 +13412,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B3" t="s">
         <v>97</v>
@@ -14001,7 +14036,7 @@
         <v>94</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>107</v>
@@ -14015,10 +14050,10 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -14030,10 +14065,10 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="11" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
@@ -14045,10 +14080,10 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="12"/>
@@ -14060,10 +14095,10 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E5" s="11">
         <f t="shared" si="0"/>
@@ -14072,10 +14107,10 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E6">
         <f t="shared" ref="E6:E29" si="1">D6/1000</f>
@@ -14084,10 +14119,10 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E7">
         <f t="shared" si="1"/>
@@ -14096,10 +14131,10 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E8">
         <f t="shared" si="1"/>
@@ -14108,10 +14143,10 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E9">
         <f t="shared" si="1"/>
@@ -14120,10 +14155,10 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B10" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E10">
         <f t="shared" si="1"/>
@@ -14132,10 +14167,10 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E11">
         <f t="shared" si="1"/>
@@ -14144,10 +14179,10 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E12">
         <f t="shared" si="1"/>
@@ -14156,10 +14191,10 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E13">
         <f t="shared" si="1"/>
@@ -14168,10 +14203,10 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B14" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E14">
         <f t="shared" si="1"/>
@@ -14180,10 +14215,10 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B15" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E15">
         <f t="shared" si="1"/>
@@ -14192,10 +14227,10 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B16" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E16">
         <f t="shared" si="1"/>
@@ -14204,10 +14239,10 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B17" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E17">
         <f t="shared" si="1"/>
@@ -14216,10 +14251,10 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B18" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E18">
         <f t="shared" si="1"/>
@@ -14228,10 +14263,10 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B19" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E19">
         <f t="shared" si="1"/>
@@ -14240,10 +14275,10 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B20" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E20">
         <f t="shared" si="1"/>
@@ -14252,10 +14287,10 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B21" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E21">
         <f t="shared" si="1"/>
@@ -14264,10 +14299,10 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B22" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E22">
         <f t="shared" si="1"/>
@@ -14276,10 +14311,10 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B23" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E23">
         <f t="shared" si="1"/>
@@ -14288,10 +14323,10 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B24" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E24">
         <f t="shared" si="1"/>
@@ -14300,10 +14335,10 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B25" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E25">
         <f t="shared" si="1"/>
@@ -14312,10 +14347,10 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B26" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E26">
         <f t="shared" si="1"/>
@@ -14324,10 +14359,10 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B27" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E27">
         <f t="shared" si="1"/>
@@ -14336,10 +14371,10 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B28" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E28">
         <f t="shared" si="1"/>
@@ -14348,10 +14383,10 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B29" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E29">
         <f t="shared" si="1"/>
@@ -14360,10 +14395,10 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
+        <v>190</v>
+      </c>
+      <c r="B30" t="s">
         <v>191</v>
-      </c>
-      <c r="B30" t="s">
-        <v>192</v>
       </c>
       <c r="E30">
         <f t="shared" ref="E30:E35" si="2">D30/1000</f>
@@ -14372,10 +14407,10 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B31" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E31">
         <f t="shared" si="2"/>
@@ -14384,10 +14419,10 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B32" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E32">
         <f t="shared" si="2"/>
@@ -14396,10 +14431,10 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B33" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E33">
         <f t="shared" si="2"/>
@@ -14408,10 +14443,10 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B34" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E34">
         <f t="shared" si="2"/>
@@ -14420,10 +14455,10 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B35" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E35">
         <f t="shared" si="2"/>
@@ -14432,10 +14467,10 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B36" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E36">
         <f>D36/1000</f>
@@ -14444,10 +14479,10 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B37" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E37">
         <f t="shared" ref="E37:E42" si="3">D37/1000</f>
@@ -14456,10 +14491,10 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B38" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E38">
         <f t="shared" si="3"/>
@@ -14468,10 +14503,10 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B39" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E39">
         <f t="shared" si="3"/>
@@ -14480,10 +14515,10 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B40" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E40">
         <f t="shared" si="3"/>
@@ -14492,10 +14527,10 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B41" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E41">
         <f t="shared" si="3"/>
@@ -14504,10 +14539,10 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B42" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E42">
         <f t="shared" si="3"/>
@@ -14516,10 +14551,10 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
+        <v>192</v>
+      </c>
+      <c r="B43" t="s">
         <v>193</v>
-      </c>
-      <c r="B43" t="s">
-        <v>194</v>
       </c>
       <c r="E43">
         <f>D43/1000</f>
@@ -14528,10 +14563,10 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B44" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E44">
         <f t="shared" ref="E44:E49" si="4">D44/1000</f>
@@ -14540,10 +14575,10 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B45" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E45">
         <f t="shared" si="4"/>
@@ -14552,10 +14587,10 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B46" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E46">
         <f t="shared" si="4"/>
@@ -14564,10 +14599,10 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B47" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E47">
         <f t="shared" si="4"/>
@@ -14576,10 +14611,10 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B48" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E48">
         <f t="shared" si="4"/>
@@ -14588,10 +14623,10 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B49" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E49">
         <f t="shared" si="4"/>
@@ -14600,10 +14635,10 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B50" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E50">
         <f>D50/1000</f>
@@ -14612,10 +14647,10 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B51" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E51">
         <f t="shared" ref="E51:E56" si="5">D51/1000</f>
@@ -14624,10 +14659,10 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B52" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E52">
         <f t="shared" si="5"/>
@@ -14636,10 +14671,10 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B53" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E53">
         <f t="shared" si="5"/>
@@ -14648,10 +14683,10 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B54" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E54">
         <f t="shared" si="5"/>
@@ -14660,10 +14695,10 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B55" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E55">
         <f t="shared" si="5"/>
@@ -14672,10 +14707,10 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B56" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E56">
         <f t="shared" si="5"/>
@@ -14684,10 +14719,10 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B57" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E57">
         <f>D57/1000</f>
@@ -14696,10 +14731,10 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B58" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E58">
         <f t="shared" ref="E58:E63" si="6">D58/1000</f>
@@ -14708,10 +14743,10 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B59" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E59">
         <f t="shared" si="6"/>
@@ -14720,10 +14755,10 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B60" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E60">
         <f t="shared" si="6"/>
@@ -14732,10 +14767,10 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B61" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E61">
         <f t="shared" si="6"/>
@@ -14744,10 +14779,10 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B62" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E62">
         <f t="shared" si="6"/>
@@ -14756,10 +14791,10 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B63" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E63">
         <f t="shared" si="6"/>
@@ -14768,10 +14803,10 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B64" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E64">
         <f t="shared" ref="E64:E69" si="7">D64/1000</f>
@@ -14780,10 +14815,10 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B65" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E65">
         <f t="shared" si="7"/>
@@ -14792,10 +14827,10 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B66" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E66">
         <f t="shared" si="7"/>
@@ -14804,10 +14839,10 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B67" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E67">
         <f t="shared" si="7"/>
@@ -14816,10 +14851,10 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B68" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E68">
         <f t="shared" si="7"/>
@@ -14828,10 +14863,10 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B69" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E69">
         <f t="shared" si="7"/>

</xml_diff>

<commit_message>
bug fixing and testing
global LNG implemented and working with dummy data
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63999AC2-7D26-46E1-A4D0-CBA0ECD083B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0812907-7258-43E0-9AE0-161193AE3962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -508,9 +508,6 @@
     <t>USA</t>
   </si>
   <si>
-    <t>NA</t>
-  </si>
-  <si>
     <t>SA</t>
   </si>
   <si>
@@ -653,6 +650,9 @@
   </si>
   <si>
     <t>Indonesia &amp; Malaysia</t>
+  </si>
+  <si>
+    <t>CM</t>
   </si>
 </sst>
 </file>
@@ -1017,12 +1017,6 @@
   </cellStyles>
   <dxfs count="40">
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -1131,6 +1125,12 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
@@ -1341,7 +1341,7 @@
     <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="6">
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="4">
       <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
@@ -1354,7 +1354,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:F69" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:F69" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2" tableBorderDxfId="1" totalsRowBorderDxfId="0">
   <autoFilter ref="A1:F69" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
@@ -1462,10 +1462,10 @@
     <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="1">
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="15">
       <calculatedColumnFormula>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="14">
       <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1482,12 +1482,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="14">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="12">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="13">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="11">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1496,17 +1496,17 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F78" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F78" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="9" tableBorderDxfId="8">
   <autoFilter ref="A57:F78" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{779C3748-4ECD-495F-809A-B5DD28F5EC2F}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{94BC7314-C5A0-4AAD-895B-84E7A94D7CF7}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="9">
+    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="7">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="8">
+    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="6">
       <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1526,7 +1526,7 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="7">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="5">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
@@ -3789,10 +3789,10 @@
         <v>85</v>
       </c>
       <c r="D53" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="E53" s="9" t="s">
         <v>175</v>
-      </c>
-      <c r="E53" s="9" t="s">
-        <v>176</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>106</v>
@@ -3820,10 +3820,10 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="B55" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C55">
         <f>165.613+35.5252809102083</f>
@@ -3840,10 +3840,10 @@
     </row>
     <row r="56" spans="1:6">
       <c r="A56" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B56" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C56">
         <f>156.619145389645-29.4652641615749</f>
@@ -3860,10 +3860,10 @@
     </row>
     <row r="57" spans="1:6">
       <c r="A57" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B57" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C57">
         <v>29.4652641615749</v>
@@ -3879,10 +3879,10 @@
     </row>
     <row r="58" spans="1:6">
       <c r="A58" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B58" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C58">
         <f>667.939379731508-174.9348378172</f>
@@ -3899,10 +3899,10 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B59" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C59">
         <v>174.93483781719999</v>
@@ -3918,10 +3918,10 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B60" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C60" s="2">
         <f>231.909048813308-C21-C3-C37-C68</f>
@@ -3938,10 +3938,10 @@
     </row>
     <row r="61" spans="1:6">
       <c r="A61" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B61" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C61">
         <v>145.71638020075315</v>
@@ -3957,10 +3957,10 @@
     </row>
     <row r="62" spans="1:6">
       <c r="A62" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B62" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C62">
         <v>194.00921828908548</v>
@@ -3976,10 +3976,10 @@
     </row>
     <row r="63" spans="1:6">
       <c r="A63" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B63" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -3995,10 +3995,10 @@
     </row>
     <row r="64" spans="1:6">
       <c r="A64" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B64" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C64">
         <v>23.760626555099513</v>
@@ -4014,10 +4014,10 @@
     </row>
     <row r="65" spans="1:6">
       <c r="A65" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B65" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C65">
         <f>656.2735508682-C64-C62-C61-C63-C69</f>
@@ -4034,10 +4034,10 @@
     </row>
     <row r="66" spans="1:6">
       <c r="A66" t="s">
+        <v>176</v>
+      </c>
+      <c r="B66" t="s">
         <v>177</v>
-      </c>
-      <c r="B66" t="s">
-        <v>178</v>
       </c>
       <c r="C66">
         <f>808.357450256401-638.446656032448</f>
@@ -4073,10 +4073,10 @@
     </row>
     <row r="68" spans="1:6">
       <c r="A68" t="s">
+        <v>182</v>
+      </c>
+      <c r="B68" t="s">
         <v>183</v>
-      </c>
-      <c r="B68" t="s">
-        <v>184</v>
       </c>
       <c r="C68">
         <v>58.465174157714841</v>
@@ -4092,10 +4092,10 @@
     </row>
     <row r="69" spans="1:6">
       <c r="A69" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B69" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C69">
         <f>64.6974253845862+73.0927934801951</f>
@@ -5392,10 +5392,10 @@
         <v>85</v>
       </c>
       <c r="D52" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="E52" s="9" t="s">
         <v>175</v>
-      </c>
-      <c r="E52" s="9" t="s">
-        <v>176</v>
       </c>
       <c r="F52" s="10" t="s">
         <v>106</v>
@@ -5423,10 +5423,10 @@
     </row>
     <row r="54" spans="1:6">
       <c r="A54" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="B54" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C54">
         <f>1261.13549926252-1035.29668748294</f>
@@ -5443,10 +5443,10 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B55" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C55">
         <f>162.021478179314-24.9936060429938</f>
@@ -5463,10 +5463,10 @@
     </row>
     <row r="56" spans="1:6">
       <c r="A56" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B56" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C56">
         <v>24.9936060429938</v>
@@ -5482,10 +5482,10 @@
     </row>
     <row r="57" spans="1:6">
       <c r="A57" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C57">
         <f>712.704008488226-180.976586566424</f>
@@ -5502,10 +5502,10 @@
     </row>
     <row r="58" spans="1:6">
       <c r="A58" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B58" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C58">
         <v>180.976586566424</v>
@@ -5521,10 +5521,10 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B59" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C59" s="2">
         <f>253.649617284986-C21-C3-C37-C67</f>
@@ -5541,10 +5541,10 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B60" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C60">
         <v>151.74021373996112</v>
@@ -5560,10 +5560,10 @@
     </row>
     <row r="61" spans="1:6">
       <c r="A61" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B61" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C61">
         <v>234.25835791543756</v>
@@ -5579,10 +5579,10 @@
     </row>
     <row r="62" spans="1:6">
       <c r="A62" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B62" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -5598,10 +5598,10 @@
     </row>
     <row r="63" spans="1:6">
       <c r="A63" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B63" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C63">
         <v>31.585488535476742</v>
@@ -5617,10 +5617,10 @@
     </row>
     <row r="64" spans="1:6">
       <c r="A64" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B64" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C64">
         <f>691.83903700697-C63-C61-C60-C62-C68</f>
@@ -5637,10 +5637,10 @@
     </row>
     <row r="65" spans="1:6">
       <c r="A65" t="s">
+        <v>176</v>
+      </c>
+      <c r="B65" t="s">
         <v>177</v>
-      </c>
-      <c r="B65" t="s">
-        <v>178</v>
       </c>
       <c r="C65">
         <f>773.5530598751-586.382199872419</f>
@@ -5676,10 +5676,10 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" t="s">
+        <v>182</v>
+      </c>
+      <c r="B67" t="s">
         <v>183</v>
-      </c>
-      <c r="B67" t="s">
-        <v>184</v>
       </c>
       <c r="C67">
         <v>57.100413073730465</v>
@@ -5695,10 +5695,10 @@
     </row>
     <row r="68" spans="1:6">
       <c r="A68" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B68" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C68">
         <f>64.2640381356325+81.074134147023</f>
@@ -6671,10 +6671,10 @@
         <v>85</v>
       </c>
       <c r="D57" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="E57" s="9" t="s">
         <v>175</v>
-      </c>
-      <c r="E57" s="9" t="s">
-        <v>176</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>106</v>
@@ -6702,10 +6702,10 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="B59" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C59">
         <f>1042.08498320178-834.549627821157</f>
@@ -6722,10 +6722,10 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B60" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C60">
         <f>148.570059919613-15.1856471767803</f>
@@ -6742,10 +6742,10 @@
     </row>
     <row r="61" spans="1:6">
       <c r="A61" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B61" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C61">
         <f>15.1856471767803</f>
@@ -6762,10 +6762,10 @@
     </row>
     <row r="62" spans="1:6">
       <c r="A62" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B62" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C62" s="2">
         <f>552.897499957585-38.4132347090566</f>
@@ -6782,10 +6782,10 @@
     </row>
     <row r="63" spans="1:6">
       <c r="A63" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B63" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C63">
         <v>38.413234709056603</v>
@@ -6801,10 +6801,10 @@
     </row>
     <row r="64" spans="1:6">
       <c r="A64" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B64" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C64" s="2">
         <f>154.184349315883-C72-C73-C74-C75-C76</f>
@@ -6821,10 +6821,10 @@
     </row>
     <row r="65" spans="1:8">
       <c r="A65" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B65" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C65">
         <v>42.317339828787539</v>
@@ -6840,10 +6840,10 @@
     </row>
     <row r="66" spans="1:8">
       <c r="A66" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B66" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C66">
         <v>336.61725663716805</v>
@@ -6859,10 +6859,10 @@
     </row>
     <row r="67" spans="1:8">
       <c r="A67" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B67" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C67">
         <f>104.1275049683+57.53730834</f>
@@ -6879,10 +6879,10 @@
     </row>
     <row r="68" spans="1:8">
       <c r="A68" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B68" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C68">
         <v>60.360121323378813</v>
@@ -6898,10 +6898,10 @@
     </row>
     <row r="69" spans="1:8">
       <c r="A69" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B69" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C69">
         <f>876.9412368709-C68-C66-C65-C67-C77</f>
@@ -6918,10 +6918,10 @@
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
+        <v>176</v>
+      </c>
+      <c r="B70" t="s">
         <v>177</v>
-      </c>
-      <c r="B70" t="s">
-        <v>178</v>
       </c>
       <c r="C70">
         <f>554.955290969357-423.483407079646</f>
@@ -7017,7 +7017,7 @@
         <v>98</v>
       </c>
       <c r="B75" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C75">
         <v>0.78666131450805166</v>
@@ -7033,10 +7033,10 @@
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
+        <v>182</v>
+      </c>
+      <c r="B76" t="s">
         <v>183</v>
-      </c>
-      <c r="B76" t="s">
-        <v>184</v>
       </c>
       <c r="C76">
         <v>58.307923875090665</v>
@@ -7052,10 +7052,10 @@
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B77" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C77">
         <f>42.5805321356392+43.613663</f>
@@ -7105,7 +7105,7 @@
         <v>81</v>
       </c>
       <c r="B81" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -8065,10 +8065,10 @@
         <v>85</v>
       </c>
       <c r="D57" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="E57" s="9" t="s">
         <v>175</v>
-      </c>
-      <c r="E57" s="9" t="s">
-        <v>176</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>106</v>
@@ -8096,10 +8096,10 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="B59" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C59">
         <f>1104.76718773088-886.467211862827</f>
@@ -8116,10 +8116,10 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B60" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C60">
         <f>161.703504900654-14.503954775876</f>
@@ -8136,10 +8136,10 @@
     </row>
     <row r="61" spans="1:6">
       <c r="A61" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B61" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C61">
         <v>14.503954775876</v>
@@ -8155,10 +8155,10 @@
     </row>
     <row r="62" spans="1:6">
       <c r="A62" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B62" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C62" s="2">
         <f>577.716724870969-44.2013179565956</f>
@@ -8175,10 +8175,10 @@
     </row>
     <row r="63" spans="1:6">
       <c r="A63" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B63" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C63">
         <v>44.201317956595602</v>
@@ -8194,10 +8194,10 @@
     </row>
     <row r="64" spans="1:6">
       <c r="A64" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B64" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C64" s="2">
         <f>171.229082457489-C72-C73-C74-C75-C76</f>
@@ -8214,10 +8214,10 @@
     </row>
     <row r="65" spans="1:6">
       <c r="A65" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B65" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C65">
         <v>40.121503042095824</v>
@@ -8233,10 +8233,10 @@
     </row>
     <row r="66" spans="1:6">
       <c r="A66" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B66" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C66">
         <f>404.838112094395+4.84678040562862</f>
@@ -8253,10 +8253,10 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B67" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C67">
         <f>92.4207922536915+60.0747038262</f>
@@ -8273,10 +8273,10 @@
     </row>
     <row r="68" spans="1:6">
       <c r="A68" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B68" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C68">
         <v>62.610307192104507</v>
@@ -8292,10 +8292,10 @@
     </row>
     <row r="69" spans="1:6">
       <c r="A69" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B69" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C69">
         <f>935.383807806868-C68-C66-C65-C67-C77</f>
@@ -8312,10 +8312,10 @@
     </row>
     <row r="70" spans="1:6">
       <c r="A70" t="s">
+        <v>176</v>
+      </c>
+      <c r="B70" t="s">
         <v>177</v>
-      </c>
-      <c r="B70" t="s">
-        <v>178</v>
       </c>
       <c r="C70">
         <f>596.017542286885-453.370943952802</f>
@@ -8411,7 +8411,7 @@
         <v>98</v>
       </c>
       <c r="B75" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C75">
         <v>0.22269575424695218</v>
@@ -8427,10 +8427,10 @@
     </row>
     <row r="76" spans="1:6">
       <c r="A76" t="s">
+        <v>182</v>
+      </c>
+      <c r="B76" t="s">
         <v>183</v>
-      </c>
-      <c r="B76" t="s">
-        <v>184</v>
       </c>
       <c r="C76">
         <v>60.044388607206308</v>
@@ -8446,10 +8446,10 @@
     </row>
     <row r="77" spans="1:6">
       <c r="A77" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B77" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C77">
         <f>45.4449851278232+46.0715052691446</f>
@@ -8496,7 +8496,7 @@
         <v>81</v>
       </c>
       <c r="B81" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -10548,7 +10548,7 @@
     </row>
     <row r="103" spans="1:8">
       <c r="A103" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B103" t="s">
         <v>47</v>
@@ -10734,7 +10734,7 @@
         <v>153</v>
       </c>
       <c r="B112" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="F112">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -10747,7 +10747,7 @@
     </row>
     <row r="113" spans="1:7">
       <c r="A113" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="B113" t="s">
         <v>153</v>
@@ -10763,10 +10763,10 @@
     </row>
     <row r="114" spans="1:7">
       <c r="A114" t="s">
+        <v>156</v>
+      </c>
+      <c r="B114" t="s">
         <v>157</v>
-      </c>
-      <c r="B114" t="s">
-        <v>158</v>
       </c>
       <c r="F114">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -10779,10 +10779,10 @@
     </row>
     <row r="115" spans="1:7">
       <c r="A115" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B115" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F115">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -10798,7 +10798,7 @@
         <v>41</v>
       </c>
       <c r="B116" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F116">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -10811,10 +10811,10 @@
     </row>
     <row r="117" spans="1:7">
       <c r="A117" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B117" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F117">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -10827,10 +10827,10 @@
     </row>
     <row r="118" spans="1:7">
       <c r="A118" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B118" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F118">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -10846,7 +10846,7 @@
         <v>41</v>
       </c>
       <c r="B119" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F119">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -10859,10 +10859,10 @@
     </row>
     <row r="120" spans="1:7">
       <c r="A120" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B120" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F120">
         <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -13036,7 +13036,7 @@
     </row>
     <row r="109" spans="1:8">
       <c r="A109" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B109" t="s">
         <v>47</v>
@@ -13053,7 +13053,7 @@
         <v>136.875</v>
       </c>
       <c r="H109" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -13222,7 +13222,7 @@
         <v>153</v>
       </c>
       <c r="B118" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="F118">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -13235,7 +13235,7 @@
     </row>
     <row r="119" spans="1:7">
       <c r="A119" t="s">
-        <v>154</v>
+        <v>202</v>
       </c>
       <c r="B119" t="s">
         <v>153</v>
@@ -13251,10 +13251,10 @@
     </row>
     <row r="120" spans="1:7">
       <c r="A120" t="s">
+        <v>156</v>
+      </c>
+      <c r="B120" t="s">
         <v>157</v>
-      </c>
-      <c r="B120" t="s">
-        <v>158</v>
       </c>
       <c r="F120">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -13267,10 +13267,10 @@
     </row>
     <row r="121" spans="1:7">
       <c r="A121" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B121" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F121">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -13286,7 +13286,7 @@
         <v>41</v>
       </c>
       <c r="B122" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F122">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -13299,10 +13299,10 @@
     </row>
     <row r="123" spans="1:7">
       <c r="A123" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B123" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F123">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -13315,10 +13315,10 @@
     </row>
     <row r="124" spans="1:7">
       <c r="A124" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B124" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F124">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -13334,7 +13334,7 @@
         <v>41</v>
       </c>
       <c r="B125" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F125">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -13347,10 +13347,10 @@
     </row>
     <row r="126" spans="1:7">
       <c r="A126" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B126" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F126">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
@@ -13412,7 +13412,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B3" t="s">
         <v>97</v>
@@ -14036,7 +14036,7 @@
         <v>94</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>107</v>
@@ -14050,10 +14050,10 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>185</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>186</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -14065,10 +14065,10 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
@@ -14080,10 +14080,10 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="12"/>
@@ -14095,10 +14095,10 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E5" s="11">
         <f t="shared" si="0"/>
@@ -14107,10 +14107,10 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E6">
         <f t="shared" ref="E6:E29" si="1">D6/1000</f>
@@ -14119,10 +14119,10 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E7">
         <f t="shared" si="1"/>
@@ -14131,10 +14131,10 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E8">
         <f t="shared" si="1"/>
@@ -14143,10 +14143,10 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E9">
         <f t="shared" si="1"/>
@@ -14155,10 +14155,10 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E10">
         <f t="shared" si="1"/>
@@ -14167,10 +14167,10 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E11">
         <f t="shared" si="1"/>
@@ -14179,10 +14179,10 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E12">
         <f t="shared" si="1"/>
@@ -14191,10 +14191,10 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E13">
         <f t="shared" si="1"/>
@@ -14203,10 +14203,10 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B14" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E14">
         <f t="shared" si="1"/>
@@ -14215,10 +14215,10 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E15">
         <f t="shared" si="1"/>
@@ -14227,10 +14227,10 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B16" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E16">
         <f t="shared" si="1"/>
@@ -14239,10 +14239,10 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E17">
         <f t="shared" si="1"/>
@@ -14251,10 +14251,10 @@
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B18" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E18">
         <f t="shared" si="1"/>
@@ -14263,10 +14263,10 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B19" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E19">
         <f t="shared" si="1"/>
@@ -14275,10 +14275,10 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B20" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E20">
         <f t="shared" si="1"/>
@@ -14287,10 +14287,10 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B21" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E21">
         <f t="shared" si="1"/>
@@ -14299,10 +14299,10 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B22" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E22">
         <f t="shared" si="1"/>
@@ -14311,10 +14311,10 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B23" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E23">
         <f t="shared" si="1"/>
@@ -14323,10 +14323,10 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B24" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E24">
         <f t="shared" si="1"/>
@@ -14335,10 +14335,10 @@
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B25" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E25">
         <f t="shared" si="1"/>
@@ -14347,10 +14347,10 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B26" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E26">
         <f t="shared" si="1"/>
@@ -14359,10 +14359,10 @@
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B27" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E27">
         <f t="shared" si="1"/>
@@ -14371,10 +14371,10 @@
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B28" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E28">
         <f t="shared" si="1"/>
@@ -14383,10 +14383,10 @@
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B29" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E29">
         <f t="shared" si="1"/>
@@ -14395,10 +14395,10 @@
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
+        <v>189</v>
+      </c>
+      <c r="B30" t="s">
         <v>190</v>
-      </c>
-      <c r="B30" t="s">
-        <v>191</v>
       </c>
       <c r="E30">
         <f t="shared" ref="E30:E35" si="2">D30/1000</f>
@@ -14407,10 +14407,10 @@
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B31" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E31">
         <f t="shared" si="2"/>
@@ -14419,10 +14419,10 @@
     </row>
     <row r="32" spans="1:5">
       <c r="A32" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B32" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E32">
         <f t="shared" si="2"/>
@@ -14431,10 +14431,10 @@
     </row>
     <row r="33" spans="1:5">
       <c r="A33" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B33" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E33">
         <f t="shared" si="2"/>
@@ -14443,10 +14443,10 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B34" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E34">
         <f t="shared" si="2"/>
@@ -14455,10 +14455,10 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B35" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E35">
         <f t="shared" si="2"/>
@@ -14467,10 +14467,10 @@
     </row>
     <row r="36" spans="1:5">
       <c r="A36" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E36">
         <f>D36/1000</f>
@@ -14479,10 +14479,10 @@
     </row>
     <row r="37" spans="1:5">
       <c r="A37" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B37" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E37">
         <f t="shared" ref="E37:E42" si="3">D37/1000</f>
@@ -14491,10 +14491,10 @@
     </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B38" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E38">
         <f t="shared" si="3"/>
@@ -14503,10 +14503,10 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B39" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E39">
         <f t="shared" si="3"/>
@@ -14515,10 +14515,10 @@
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B40" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E40">
         <f t="shared" si="3"/>
@@ -14527,10 +14527,10 @@
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B41" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E41">
         <f t="shared" si="3"/>
@@ -14539,10 +14539,10 @@
     </row>
     <row r="42" spans="1:5">
       <c r="A42" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B42" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E42">
         <f t="shared" si="3"/>
@@ -14551,10 +14551,10 @@
     </row>
     <row r="43" spans="1:5">
       <c r="A43" t="s">
+        <v>191</v>
+      </c>
+      <c r="B43" t="s">
         <v>192</v>
-      </c>
-      <c r="B43" t="s">
-        <v>193</v>
       </c>
       <c r="E43">
         <f>D43/1000</f>
@@ -14563,10 +14563,10 @@
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B44" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E44">
         <f t="shared" ref="E44:E49" si="4">D44/1000</f>
@@ -14575,10 +14575,10 @@
     </row>
     <row r="45" spans="1:5">
       <c r="A45" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B45" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E45">
         <f t="shared" si="4"/>
@@ -14587,10 +14587,10 @@
     </row>
     <row r="46" spans="1:5">
       <c r="A46" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B46" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E46">
         <f t="shared" si="4"/>
@@ -14599,10 +14599,10 @@
     </row>
     <row r="47" spans="1:5">
       <c r="A47" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B47" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E47">
         <f t="shared" si="4"/>
@@ -14611,10 +14611,10 @@
     </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B48" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E48">
         <f t="shared" si="4"/>
@@ -14623,10 +14623,10 @@
     </row>
     <row r="49" spans="1:5">
       <c r="A49" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B49" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E49">
         <f t="shared" si="4"/>
@@ -14635,10 +14635,10 @@
     </row>
     <row r="50" spans="1:5">
       <c r="A50" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B50" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E50">
         <f>D50/1000</f>
@@ -14647,10 +14647,10 @@
     </row>
     <row r="51" spans="1:5">
       <c r="A51" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E51">
         <f t="shared" ref="E51:E56" si="5">D51/1000</f>
@@ -14659,10 +14659,10 @@
     </row>
     <row r="52" spans="1:5">
       <c r="A52" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B52" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E52">
         <f t="shared" si="5"/>
@@ -14671,10 +14671,10 @@
     </row>
     <row r="53" spans="1:5">
       <c r="A53" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B53" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E53">
         <f t="shared" si="5"/>
@@ -14683,10 +14683,10 @@
     </row>
     <row r="54" spans="1:5">
       <c r="A54" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B54" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E54">
         <f t="shared" si="5"/>
@@ -14695,10 +14695,10 @@
     </row>
     <row r="55" spans="1:5">
       <c r="A55" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B55" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E55">
         <f t="shared" si="5"/>
@@ -14707,10 +14707,10 @@
     </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B56" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E56">
         <f t="shared" si="5"/>
@@ -14719,10 +14719,10 @@
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B57" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E57">
         <f>D57/1000</f>
@@ -14731,10 +14731,10 @@
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B58" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E58">
         <f t="shared" ref="E58:E63" si="6">D58/1000</f>
@@ -14743,10 +14743,10 @@
     </row>
     <row r="59" spans="1:5">
       <c r="A59" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B59" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E59">
         <f t="shared" si="6"/>
@@ -14755,10 +14755,10 @@
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B60" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E60">
         <f t="shared" si="6"/>
@@ -14767,10 +14767,10 @@
     </row>
     <row r="61" spans="1:5">
       <c r="A61" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B61" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E61">
         <f t="shared" si="6"/>
@@ -14779,10 +14779,10 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B62" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E62">
         <f t="shared" si="6"/>
@@ -14791,10 +14791,10 @@
     </row>
     <row r="63" spans="1:5">
       <c r="A63" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B63" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E63">
         <f t="shared" si="6"/>
@@ -14803,10 +14803,10 @@
     </row>
     <row r="64" spans="1:5">
       <c r="A64" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B64" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E64">
         <f t="shared" ref="E64:E69" si="7">D64/1000</f>
@@ -14815,10 +14815,10 @@
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B65" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E65">
         <f t="shared" si="7"/>
@@ -14827,10 +14827,10 @@
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B66" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E66">
         <f t="shared" si="7"/>
@@ -14839,10 +14839,10 @@
     </row>
     <row r="67" spans="1:5">
       <c r="A67" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B67" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E67">
         <f t="shared" si="7"/>
@@ -14851,10 +14851,10 @@
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B68" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E68">
         <f t="shared" si="7"/>
@@ -14863,10 +14863,10 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B69" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E69">
         <f t="shared" si="7"/>

</xml_diff>

<commit_message>
bug fixing by checking input values
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0812907-7258-43E0-9AE0-161193AE3962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A989FBAA-632B-406A-AC79-4F814B2DEBD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1364" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1360" uniqueCount="203">
   <si>
     <t>Belgium</t>
   </si>
@@ -1017,6 +1017,12 @@
   </cellStyles>
   <dxfs count="40">
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -1077,9 +1083,6 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
@@ -1128,9 +1131,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
@@ -1341,7 +1341,7 @@
     <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="4">
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="6">
       <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
@@ -1354,7 +1354,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:F69" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2" tableBorderDxfId="1" totalsRowBorderDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:F69" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
   <autoFilter ref="A1:F69" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
@@ -1373,8 +1373,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F69" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33">
-  <autoFilter ref="A53:F69" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F68" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33">
+  <autoFilter ref="A53:F68" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3F684FB4-9656-4C92-BAF4-456019B2B924}" name="Country"/>
     <tableColumn id="2" xr3:uid="{082B059D-405D-407D-8F97-297DCD23D3B2}" name="Long_name"/>
@@ -1414,8 +1414,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F68" totalsRowShown="0" headerRowDxfId="26" headerRowBorderDxfId="25" tableBorderDxfId="24">
-  <autoFilter ref="A52:F68" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F67" totalsRowShown="0" headerRowDxfId="26" headerRowBorderDxfId="25" tableBorderDxfId="24">
+  <autoFilter ref="A52:F67" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
@@ -1465,8 +1465,8 @@
     <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="15">
       <calculatedColumnFormula>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="14">
-      <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="1">
+      <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1482,12 +1482,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="12">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="13">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="11">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="12">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1496,18 +1496,18 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F78" totalsRowShown="0" headerRowDxfId="10" headerRowBorderDxfId="9" tableBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F78" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9">
   <autoFilter ref="A57:F78" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{779C3748-4ECD-495F-809A-B5DD28F5EC2F}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{94BC7314-C5A0-4AAD-895B-84E7A94D7CF7}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="7">
+    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="8">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="6">
-      <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="0">
+      <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1526,7 +1526,7 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="5">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="7">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
@@ -2513,7 +2513,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF82F4-4954-4D06-9A30-AE8575CA18DE}">
-  <dimension ref="A1:M69"/>
+  <dimension ref="A1:M68"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -3924,7 +3924,7 @@
         <v>168</v>
       </c>
       <c r="C60" s="2">
-        <f>231.909048813308-C21-C3-C37-C68</f>
+        <f>231.909048813308-C21-C3-C37-C67</f>
         <v>77.419550083247572</v>
       </c>
       <c r="E60" s="2">
@@ -4020,7 +4020,7 @@
         <v>173</v>
       </c>
       <c r="C65">
-        <f>656.2735508682-C64-C62-C61-C63-C69</f>
+        <f>656.2735508682-C64-C62-C61-C63-C68</f>
         <v>154.99710695848057</v>
       </c>
       <c r="E65" s="2">
@@ -4054,13 +4054,13 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" t="s">
-        <v>41</v>
+        <v>182</v>
       </c>
       <c r="B67" t="s">
-        <v>70</v>
+        <v>183</v>
       </c>
       <c r="C67">
-        <v>638.446656032448</v>
+        <v>58.465174157714841</v>
       </c>
       <c r="E67" s="2">
         <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
@@ -4068,44 +4068,25 @@
       </c>
       <c r="F67" s="3">
         <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>6237.6238294370169</v>
+        <v>571.20475152087397</v>
       </c>
     </row>
     <row r="68" spans="1:6">
       <c r="A68" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="B68" t="s">
-        <v>183</v>
+        <v>201</v>
       </c>
       <c r="C68">
-        <v>58.465174157714841</v>
+        <f>64.6974253845862+73.0927934801951</f>
+        <v>137.79021886478131</v>
       </c>
       <c r="E68" s="2">
         <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F68" s="3">
-        <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>571.20475152087397</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6">
-      <c r="A69" t="s">
-        <v>198</v>
-      </c>
-      <c r="B69" t="s">
-        <v>201</v>
-      </c>
-      <c r="C69">
-        <f>64.6974253845862+73.0927934801951</f>
-        <v>137.79021886478131</v>
-      </c>
-      <c r="E69" s="2">
-        <f>Table7[[#This Row],[Mil m3 '[2020']]]/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F69" s="3">
         <f>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
         <v>1346.2104383089134</v>
       </c>
@@ -4121,7 +4102,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{036BBBE1-80BC-4BBB-9141-C576056723F9}">
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:M67"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -5527,7 +5508,7 @@
         <v>168</v>
       </c>
       <c r="C59" s="2">
-        <f>253.649617284986-C21-C3-C37-C67</f>
+        <f>253.649617284986-C21-C3-C37-C66</f>
         <v>76.854578169538883</v>
       </c>
       <c r="E59" s="2">
@@ -5623,7 +5604,7 @@
         <v>173</v>
       </c>
       <c r="C64">
-        <f>691.83903700697-C63-C61-C60-C62-C68</f>
+        <f>691.83903700697-C63-C61-C60-C62-C67</f>
         <v>128.91680453343903</v>
       </c>
       <c r="E64" s="2">
@@ -5657,13 +5638,13 @@
     </row>
     <row r="66" spans="1:6">
       <c r="A66" t="s">
-        <v>41</v>
+        <v>182</v>
       </c>
       <c r="B66" t="s">
-        <v>70</v>
+        <v>183</v>
       </c>
       <c r="C66">
-        <v>586.38219987241905</v>
+        <v>57.100413073730465</v>
       </c>
       <c r="E66" s="2">
         <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
@@ -5671,44 +5652,25 @@
       </c>
       <c r="F66" s="3">
         <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>5728.9540927535336</v>
+        <v>557.87103573034665</v>
       </c>
     </row>
     <row r="67" spans="1:6">
       <c r="A67" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="B67" t="s">
-        <v>183</v>
+        <v>201</v>
       </c>
       <c r="C67">
-        <v>57.100413073730465</v>
+        <f>64.2640381356325+81.074134147023</f>
+        <v>145.33817228265551</v>
       </c>
       <c r="E67" s="2">
         <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F67" s="3">
-        <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>557.87103573034665</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6">
-      <c r="A68" t="s">
-        <v>198</v>
-      </c>
-      <c r="B68" t="s">
-        <v>201</v>
-      </c>
-      <c r="C68">
-        <f>64.2640381356325+81.074134147023</f>
-        <v>145.33817228265551</v>
-      </c>
-      <c r="E68" s="2">
-        <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F68" s="3">
         <f>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
         <v>1419.9539432015442</v>
       </c>
@@ -6634,6 +6596,12 @@
         <v>-4.8325219236059471</v>
       </c>
     </row>
+    <row r="44" spans="1:6">
+      <c r="C44" s="2">
+        <f>SUM(Table1[Mrd m3 '[2020']])</f>
+        <v>541.77584793709366</v>
+      </c>
+    </row>
     <row r="50" spans="1:6">
       <c r="A50" t="s">
         <v>134</v>
@@ -6696,8 +6664,8 @@
         <v>0</v>
       </c>
       <c r="F58" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>8153.5498638127028</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-8153.5498638127028</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -6716,8 +6684,8 @@
         <v>0</v>
       </c>
       <c r="F59" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2027.6204220686873</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-2027.6204220686873</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -6736,8 +6704,8 @@
         <v>0</v>
       </c>
       <c r="F60" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1303.1657124974754</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-1303.1657124974754</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -6756,8 +6724,8 @@
         <v>0</v>
       </c>
       <c r="F61" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>148.36377291714354</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-148.36377291714354</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -6776,8 +6744,8 @@
         <v>0</v>
       </c>
       <c r="F62" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>5026.5112714781217</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-5026.5112714781217</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -6795,8 +6763,8 @@
         <v>0</v>
       </c>
       <c r="F63" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>375.297303107483</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-375.297303107483</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -6815,8 +6783,8 @@
         <v>0</v>
       </c>
       <c r="F64" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>395.18940186607011</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-395.18940186607011</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -6834,8 +6802,8 @@
         <v>0</v>
       </c>
       <c r="F65" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>413.44041012725421</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-413.44041012725421</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -6853,8 +6821,8 @@
         <v>0</v>
       </c>
       <c r="F66" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>3288.7505973451316</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-3288.7505973451316</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -6873,8 +6841,8 @@
         <v>0</v>
       </c>
       <c r="F67" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1579.465226022091</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-1579.465226022091</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -6892,8 +6860,8 @@
         <v>0</v>
       </c>
       <c r="F68" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>589.71838532941092</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-589.71838532941092</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -6912,8 +6880,8 @@
         <v>0</v>
       </c>
       <c r="F69" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1854.2239789296088</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-1854.2239789296088</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -6924,16 +6892,16 @@
         <v>177</v>
       </c>
       <c r="C70">
-        <f>554.955290969357-423.483407079646</f>
-        <v>131.47188388971097</v>
+        <f>554.955290969357-423.483407079646-17.7510088495575</f>
+        <v>113.72087504015346</v>
       </c>
       <c r="E70" s="2">
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F70" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1284.4803056024762</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-1111.0529491422992</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -6951,8 +6919,8 @@
         <v>0</v>
       </c>
       <c r="F71" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>4137.432887168141</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-4137.432887168141</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -6970,8 +6938,8 @@
         <v>0</v>
       </c>
       <c r="F72" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>423.52986637499998</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-423.52986637499998</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -6989,8 +6957,8 @@
         <v>0</v>
       </c>
       <c r="F73" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>75.228999999999999</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-75.228999999999999</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -7008,8 +6976,8 @@
         <v>0</v>
       </c>
       <c r="F74" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>35.078727272727271</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-35.078727272727271</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -7027,8 +6995,8 @@
         <v>0</v>
       </c>
       <c r="F75" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>7.6856810427436644</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-7.6856810427436644</v>
       </c>
     </row>
     <row r="76" spans="1:8">
@@ -7046,8 +7014,8 @@
         <v>0</v>
       </c>
       <c r="F76" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>569.66841625963582</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-569.66841625963582</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -7066,8 +7034,8 @@
         <v>0</v>
       </c>
       <c r="F77" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>842.11728647519499</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-842.11728647519499</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -7078,15 +7046,15 @@
         <v>82</v>
       </c>
       <c r="C78">
-        <v>17.751008849557518</v>
+        <v>17.7510088495575</v>
       </c>
       <c r="E78" s="2">
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F78" s="3">
-        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>173.42735646017695</v>
+        <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-173.42735646017678</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -8090,8 +8058,8 @@
         <v>0</v>
       </c>
       <c r="F58" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>8660.7846598998185</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-8660.7846598998185</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -8110,8 +8078,8 @@
         <v>0</v>
       </c>
       <c r="F59" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2132.7907642308792</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-2132.7907642308792</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -8130,8 +8098,8 @@
         <v>0</v>
       </c>
       <c r="F60" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1438.139604719081</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-1438.139604719081</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -8149,8 +8117,8 @@
         <v>0</v>
       </c>
       <c r="F61" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>141.70363816030851</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-141.70363816030851</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -8169,8 +8137,8 @@
         <v>0</v>
       </c>
       <c r="F62" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>5212.4455255534276</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-5212.4455255534276</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -8188,8 +8156,8 @@
         <v>0</v>
       </c>
       <c r="F63" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>431.84687643593901</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-431.84687643593901</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -8208,8 +8176,8 @@
         <v>0</v>
       </c>
       <c r="F64" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>458.53340662554189</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-458.53340662554189</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -8227,8 +8195,8 @@
         <v>0</v>
       </c>
       <c r="F65" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>391.98708472127618</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-391.98708472127618</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -8247,8 +8215,8 @@
         <v>0</v>
       </c>
       <c r="F66" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>4002.6213997252307</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-4002.6213997252307</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -8267,8 +8235,8 @@
         <v>0</v>
       </c>
       <c r="F67" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1489.8809967005398</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-1489.8809967005398</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -8286,8 +8254,8 @@
         <v>0</v>
       </c>
       <c r="F68" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>611.70270126686103</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-611.70270126686103</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -8306,8 +8274,8 @@
         <v>0</v>
       </c>
       <c r="F69" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1748.3915086808172</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-1748.3915086808172</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -8318,16 +8286,16 @@
         <v>177</v>
       </c>
       <c r="C70">
-        <f>596.017542286885-453.370943952802</f>
-        <v>142.64659833408302</v>
+        <f>596.017542286885-453.370943952802-16.7840359905841</f>
+        <v>125.86256234349892</v>
       </c>
       <c r="E70" s="2">
         <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F70" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>1393.657265723991</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-1229.6772340959844</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -8345,8 +8313,8 @@
         <v>0</v>
       </c>
       <c r="F71" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>4429.4341224188756</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-4429.4341224188756</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -8364,8 +8332,8 @@
         <v>0</v>
       </c>
       <c r="F72" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>491.80958750000002</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-491.80958750000002</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -8383,8 +8351,8 @@
         <v>0</v>
       </c>
       <c r="F73" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>98.676999999999992</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-98.676999999999992</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -8402,8 +8370,8 @@
         <v>0</v>
       </c>
       <c r="F74" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>35.078727272727271</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-35.078727272727271</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -8421,8 +8389,8 @@
         <v>0</v>
       </c>
       <c r="F75" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>2.1757375189927228</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-2.1757375189927228</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -8440,8 +8408,8 @@
         <v>0</v>
       </c>
       <c r="F76" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>586.63367669240563</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-586.63367669240563</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -8460,8 +8428,8 @@
         <v>0</v>
       </c>
       <c r="F77" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>894.11611117837549</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-894.11611117837549</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -8472,15 +8440,15 @@
         <v>82</v>
       </c>
       <c r="C78">
-        <v>16.784035990584055</v>
+        <v>16.784035990584101</v>
       </c>
       <c r="E78" s="2">
         <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
       <c r="F78" s="3">
-        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77</f>
-        <v>163.9800316280062</v>
+        <f>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
+        <v>-163.98003162800666</v>
       </c>
     </row>
     <row r="80" spans="1:6">

</xml_diff>

<commit_message>
add LNG transport distances from Qatar
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A989FBAA-632B-406A-AC79-4F814B2DEBD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8EC2038-C6D4-4C86-BAE9-F1B63CC72F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1360" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1439" uniqueCount="249">
   <si>
     <t>Belgium</t>
   </si>
@@ -653,6 +653,144 @@
   </si>
   <si>
     <t>CM</t>
+  </si>
+  <si>
+    <t>Distance [km]</t>
+  </si>
+  <si>
+    <t>Distance [miles]</t>
+  </si>
+  <si>
+    <t>distance from https://sea-distances.org/advanced</t>
+  </si>
+  <si>
+    <t>to Tokyo</t>
+  </si>
+  <si>
+    <t>to Mumbai</t>
+  </si>
+  <si>
+    <t>to Dalian</t>
+  </si>
+  <si>
+    <t>to Suez</t>
+  </si>
+  <si>
+    <t>to Port Harcourt</t>
+  </si>
+  <si>
+    <t>to Rio</t>
+  </si>
+  <si>
+    <t>to Bangkok</t>
+  </si>
+  <si>
+    <t>BE_LNG</t>
+  </si>
+  <si>
+    <t>FR_LNG</t>
+  </si>
+  <si>
+    <t>GR_LNG</t>
+  </si>
+  <si>
+    <t>IT_LNG</t>
+  </si>
+  <si>
+    <t>HR_LNG</t>
+  </si>
+  <si>
+    <t>LT_LNG</t>
+  </si>
+  <si>
+    <t>NL_LNG</t>
+  </si>
+  <si>
+    <t>PL_LNG</t>
+  </si>
+  <si>
+    <t>PT_LNG</t>
+  </si>
+  <si>
+    <t>ES_LNG</t>
+  </si>
+  <si>
+    <t>TR_LNG</t>
+  </si>
+  <si>
+    <t>UK_LNG</t>
+  </si>
+  <si>
+    <t>to Zeebrugge</t>
+  </si>
+  <si>
+    <t>Suez or Panama</t>
+  </si>
+  <si>
+    <t>Suez</t>
+  </si>
+  <si>
+    <t>Fos</t>
+  </si>
+  <si>
+    <t>Megara</t>
+  </si>
+  <si>
+    <t>La Spezia</t>
+  </si>
+  <si>
+    <t>Omisalj</t>
+  </si>
+  <si>
+    <t>Klaipeda</t>
+  </si>
+  <si>
+    <t>Rotterdam</t>
+  </si>
+  <si>
+    <t>Swinoujscie</t>
+  </si>
+  <si>
+    <t>Setubal</t>
+  </si>
+  <si>
+    <t>Barcelona</t>
+  </si>
+  <si>
+    <t>Izmir</t>
+  </si>
+  <si>
+    <t>Pembroke</t>
+  </si>
+  <si>
+    <t>EE_LNG</t>
+  </si>
+  <si>
+    <t>FI_LNG</t>
+  </si>
+  <si>
+    <t>DE_LNG</t>
+  </si>
+  <si>
+    <t>IE_LNG</t>
+  </si>
+  <si>
+    <t>LV_LNG</t>
+  </si>
+  <si>
+    <t>Talinn</t>
+  </si>
+  <si>
+    <t>Inkoo</t>
+  </si>
+  <si>
+    <t>Wilhelmshaven</t>
+  </si>
+  <si>
+    <t>Cork</t>
+  </si>
+  <si>
+    <t>Riga</t>
   </si>
 </sst>
 </file>
@@ -957,7 +1095,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -971,6 +1109,8 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -1015,12 +1155,12 @@
     <cellStyle name="Percent 4" xfId="35" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
     <cellStyle name="Percent 8" xfId="33" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
-  <dxfs count="40">
+  <dxfs count="42">
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1083,6 +1223,9 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
@@ -1131,6 +1274,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
@@ -1316,12 +1462,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D3465064-BCEE-4D04-A8E6-DEAE11BBDA92}" name="Country"/>
     <tableColumn id="2" xr3:uid="{D66D54B4-4DED-47C6-BE50-755A236428ED}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="39"/>
-    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="38"/>
-    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="37">
+    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="41"/>
+    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="40"/>
+    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="39">
       <calculatedColumnFormula>Table2[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="36">
+    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="38">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1354,9 +1500,9 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:F69" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
-  <autoFilter ref="A1:F69" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:I86" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+  <autoFilter ref="A1:I86" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
+  <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
     <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
     <tableColumn id="3" xr3:uid="{426DF8FF-B8EF-4473-B5C0-4A6D2531E9C8}" name="GWh/d [capacity]"/>
@@ -1366,6 +1512,11 @@
     <tableColumn id="7" xr3:uid="{15452FB1-E8BF-413E-AF8B-8B2631F8DB73}" name="TWh/a">
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
+    <tableColumn id="5" xr3:uid="{7E7B8CB5-D54F-4427-813D-93B66C13FCBB}" name="Distance [miles]"/>
+    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="1">
+      <calculatedColumnFormula>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="0"/>
     <tableColumn id="8" xr3:uid="{ECBB25E4-2145-4120-8981-E6E8E1591E5B}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1373,17 +1524,17 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F68" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F68" totalsRowShown="0" headerRowDxfId="37" headerRowBorderDxfId="36" tableBorderDxfId="35">
   <autoFilter ref="A53:F68" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3F684FB4-9656-4C92-BAF4-456019B2B924}" name="Country"/>
     <tableColumn id="2" xr3:uid="{082B059D-405D-407D-8F97-297DCD23D3B2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{388F462C-127F-4CB7-B46A-1DD19D06D0E8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{ACDF4345-6201-4524-A8D7-A0CE31D137A6}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="32">
+    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="34">
       <calculatedColumnFormula>Table7[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="31">
+    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="33">
       <calculatedColumnFormula>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1400,12 +1551,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="28">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="30">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="27">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="29">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1414,17 +1565,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F67" totalsRowShown="0" headerRowDxfId="26" headerRowBorderDxfId="25" tableBorderDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F67" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="27" tableBorderDxfId="26">
   <autoFilter ref="A52:F67" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{02819FD0-F6B6-484E-B4DA-8262AECE7052}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{A15C284E-E91C-44C6-B3BB-CC2DD205DA84}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="23">
+    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="25">
       <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="22">
+    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="24">
       <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1441,12 +1592,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="20">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="22">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="19">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="21">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1455,17 +1606,17 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F78" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F78" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18">
   <autoFilter ref="A57:F78" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{555371BF-8030-4257-9852-212E94829B9B}" name="Country"/>
     <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="15">
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="17">
       <calculatedColumnFormula>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="1">
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="16">
       <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1482,12 +1633,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="13">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="14">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="12">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="13">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1496,17 +1647,17 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F78" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F78" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10">
   <autoFilter ref="A57:F78" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{779C3748-4ECD-495F-809A-B5DD28F5EC2F}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{94BC7314-C5A0-4AAD-895B-84E7A94D7CF7}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="8">
+    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="9">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="8">
       <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -13988,15 +14139,17 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
-  <dimension ref="A1:F69"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:M86"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="21.81640625" customWidth="1"/>
     <col min="4" max="4" width="9" customWidth="1"/>
-    <col min="6" max="6" width="11.1796875" customWidth="1"/>
+    <col min="6" max="6" width="16.453125" customWidth="1"/>
+    <col min="7" max="7" width="15.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:13">
       <c r="A1" s="9" t="s">
         <v>93</v>
       </c>
@@ -14013,10 +14166,22 @@
         <v>108</v>
       </c>
       <c r="F1" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="I1" s="9" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="M1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="6" t="s">
         <v>184</v>
       </c>
@@ -14030,8 +14195,14 @@
         <v>0</v>
       </c>
       <c r="F2" s="6"/>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2" s="6">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="11" t="s">
         <v>187</v>
       </c>
@@ -14045,8 +14216,14 @@
         <v>0</v>
       </c>
       <c r="F3" s="11"/>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="G3" s="11">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" t="s">
         <v>188</v>
       </c>
@@ -14060,8 +14237,14 @@
         <v>0</v>
       </c>
       <c r="F4" s="12"/>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4" s="12">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
         <v>189</v>
       </c>
@@ -14072,8 +14255,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="F5" s="13"/>
+      <c r="G5" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="13"/>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" t="s">
         <v>190</v>
       </c>
@@ -14084,8 +14273,12 @@
         <f t="shared" ref="E6:E29" si="1">D6/1000</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" t="s">
         <v>191</v>
       </c>
@@ -14096,8 +14289,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G7">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" t="s">
         <v>184</v>
       </c>
@@ -14108,8 +14305,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="G8">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" t="s">
         <v>184</v>
       </c>
@@ -14120,8 +14321,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="G9">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" t="s">
         <v>184</v>
       </c>
@@ -14132,8 +14337,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
+      <c r="G10">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" t="s">
         <v>184</v>
       </c>
@@ -14144,8 +14353,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
+      <c r="G11">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12" t="s">
         <v>184</v>
       </c>
@@ -14156,8 +14369,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:6">
+      <c r="G12">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
       <c r="A13" t="s">
         <v>184</v>
       </c>
@@ -14168,8 +14385,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:6">
+      <c r="G13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
       <c r="A14" t="s">
         <v>184</v>
       </c>
@@ -14180,8 +14401,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
+      <c r="G14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
       <c r="A15" t="s">
         <v>187</v>
       </c>
@@ -14192,8 +14417,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
+      <c r="G15">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
       <c r="A16" t="s">
         <v>187</v>
       </c>
@@ -14204,8 +14433,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="G16">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>187</v>
       </c>
@@ -14216,8 +14449,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="G17">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>187</v>
       </c>
@@ -14228,8 +14465,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="G18">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>187</v>
       </c>
@@ -14240,8 +14481,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="G19">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>187</v>
       </c>
@@ -14252,8 +14497,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:5">
+      <c r="G20">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>187</v>
       </c>
@@ -14264,8 +14513,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:5">
+      <c r="G21">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
         <v>188</v>
       </c>
@@ -14276,8 +14529,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:5">
+      <c r="G22">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
       <c r="A23" t="s">
         <v>188</v>
       </c>
@@ -14288,8 +14545,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:5">
+      <c r="G23">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
         <v>188</v>
       </c>
@@ -14300,8 +14561,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:5">
+      <c r="G24">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
       <c r="A25" t="s">
         <v>188</v>
       </c>
@@ -14312,8 +14577,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:5">
+      <c r="G25">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
         <v>188</v>
       </c>
@@ -14324,8 +14593,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:5">
+      <c r="G26">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
         <v>188</v>
       </c>
@@ -14336,8 +14609,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:5">
+      <c r="G27">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
         <v>188</v>
       </c>
@@ -14348,8 +14625,12 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:5">
+      <c r="G28">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
       <c r="A29" t="s">
         <v>189</v>
       </c>
@@ -14360,8 +14641,18 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:5">
+      <c r="F29">
+        <v>8158</v>
+      </c>
+      <c r="G29">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>13129.032413807505</v>
+      </c>
+      <c r="I29" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
         <v>189</v>
       </c>
@@ -14372,8 +14663,18 @@
         <f t="shared" ref="E30:E35" si="2">D30/1000</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:5">
+      <c r="F30">
+        <v>7349</v>
+      </c>
+      <c r="G30">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11827.072715012424</v>
+      </c>
+      <c r="I30" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
         <v>189</v>
       </c>
@@ -14384,8 +14685,18 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:5">
+      <c r="F31">
+        <v>6227</v>
+      </c>
+      <c r="G31">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>10021.38818837697</v>
+      </c>
+      <c r="I31" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
       <c r="A32" t="s">
         <v>189</v>
       </c>
@@ -14396,8 +14707,18 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="F32">
+        <v>6512</v>
+      </c>
+      <c r="G32">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>10480.051370276351</v>
+      </c>
+      <c r="I32" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
       <c r="A33" t="s">
         <v>189</v>
       </c>
@@ -14408,8 +14729,18 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="F33">
+        <v>1300</v>
+      </c>
+      <c r="G33">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>2092.147847260328</v>
+      </c>
+      <c r="I33" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
       <c r="A34" t="s">
         <v>189</v>
       </c>
@@ -14420,8 +14751,18 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:5">
+      <c r="F34">
+        <v>4439</v>
+      </c>
+      <c r="G34">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7143.8802261450737</v>
+      </c>
+      <c r="I34" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
       <c r="A35" t="s">
         <v>189</v>
       </c>
@@ -14432,8 +14773,18 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:5">
+      <c r="F35">
+        <v>2982</v>
+      </c>
+      <c r="G35">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4799.0652927156134</v>
+      </c>
+      <c r="I35" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
       <c r="A36" t="s">
         <v>190</v>
       </c>
@@ -14444,8 +14795,12 @@
         <f>D36/1000</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:5">
+      <c r="G36">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
       <c r="A37" t="s">
         <v>190</v>
       </c>
@@ -14456,8 +14811,12 @@
         <f t="shared" ref="E37:E42" si="3">D37/1000</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:5">
+      <c r="G37">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
       <c r="A38" t="s">
         <v>190</v>
       </c>
@@ -14468,8 +14827,12 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:5">
+      <c r="G38">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
       <c r="A39" t="s">
         <v>190</v>
       </c>
@@ -14480,8 +14843,12 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:5">
+      <c r="G39">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
       <c r="A40" t="s">
         <v>190</v>
       </c>
@@ -14492,8 +14859,12 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:5">
+      <c r="G40">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
       <c r="A41" t="s">
         <v>190</v>
       </c>
@@ -14504,8 +14875,12 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:5">
+      <c r="G41">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
       <c r="A42" t="s">
         <v>190</v>
       </c>
@@ -14516,8 +14891,12 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:5">
+      <c r="G42">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
       <c r="A43" t="s">
         <v>191</v>
       </c>
@@ -14528,8 +14907,12 @@
         <f>D43/1000</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:5">
+      <c r="G43">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
       <c r="A44" t="s">
         <v>191</v>
       </c>
@@ -14540,8 +14923,12 @@
         <f t="shared" ref="E44:E49" si="4">D44/1000</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:5">
+      <c r="G44">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
       <c r="A45" t="s">
         <v>191</v>
       </c>
@@ -14552,8 +14939,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:5">
+      <c r="G45">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
       <c r="A46" t="s">
         <v>191</v>
       </c>
@@ -14564,8 +14955,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:5">
+      <c r="G46">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
       <c r="A47" t="s">
         <v>191</v>
       </c>
@@ -14576,8 +14971,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:5">
+      <c r="G47">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
       <c r="A48" t="s">
         <v>191</v>
       </c>
@@ -14588,8 +14987,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:5">
+      <c r="G48">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
       <c r="A49" t="s">
         <v>191</v>
       </c>
@@ -14600,8 +15003,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:5">
+      <c r="G49">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
       <c r="A50" t="s">
         <v>199</v>
       </c>
@@ -14612,8 +15019,12 @@
         <f>D50/1000</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:5">
+      <c r="G50">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
       <c r="A51" t="s">
         <v>199</v>
       </c>
@@ -14624,8 +15035,12 @@
         <f t="shared" ref="E51:E56" si="5">D51/1000</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:5">
+      <c r="G51">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
       <c r="A52" t="s">
         <v>199</v>
       </c>
@@ -14636,8 +15051,12 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:5">
+      <c r="G52">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
       <c r="A53" t="s">
         <v>199</v>
       </c>
@@ -14648,8 +15067,12 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:5">
+      <c r="G53">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
       <c r="A54" t="s">
         <v>199</v>
       </c>
@@ -14660,8 +15083,12 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:5">
+      <c r="G54">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
       <c r="A55" t="s">
         <v>199</v>
       </c>
@@ -14672,8 +15099,12 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:5">
+      <c r="G55">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
       <c r="A56" t="s">
         <v>199</v>
       </c>
@@ -14684,8 +15115,12 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:5">
+      <c r="G56">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
       <c r="A57" t="s">
         <v>197</v>
       </c>
@@ -14696,8 +15131,12 @@
         <f>D57/1000</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="58" spans="1:5">
+      <c r="G57">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
       <c r="A58" t="s">
         <v>197</v>
       </c>
@@ -14708,8 +15147,12 @@
         <f t="shared" ref="E58:E63" si="6">D58/1000</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:5">
+      <c r="G58">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
       <c r="A59" t="s">
         <v>197</v>
       </c>
@@ -14720,8 +15163,12 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:5">
+      <c r="G59">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
       <c r="A60" t="s">
         <v>197</v>
       </c>
@@ -14732,8 +15179,12 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:5">
+      <c r="G60">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
       <c r="A61" t="s">
         <v>197</v>
       </c>
@@ -14744,8 +15195,12 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:5">
+      <c r="G61">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
       <c r="A62" t="s">
         <v>197</v>
       </c>
@@ -14756,8 +15211,12 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:5">
+      <c r="G62">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
       <c r="A63" t="s">
         <v>200</v>
       </c>
@@ -14768,8 +15227,12 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:5">
+      <c r="G63">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
       <c r="A64" t="s">
         <v>200</v>
       </c>
@@ -14780,8 +15243,12 @@
         <f t="shared" ref="E64:E69" si="7">D64/1000</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:5">
+      <c r="G64">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9">
       <c r="A65" t="s">
         <v>200</v>
       </c>
@@ -14792,8 +15259,12 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="66" spans="1:5">
+      <c r="G65">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9">
       <c r="A66" t="s">
         <v>200</v>
       </c>
@@ -14804,8 +15275,12 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:5">
+      <c r="G66">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9">
       <c r="A67" t="s">
         <v>200</v>
       </c>
@@ -14816,8 +15291,12 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:5">
+      <c r="G67">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9">
       <c r="A68" t="s">
         <v>200</v>
       </c>
@@ -14828,8 +15307,12 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:5">
+      <c r="G68">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9">
       <c r="A69" t="s">
         <v>200</v>
       </c>
@@ -14839,6 +15322,435 @@
       <c r="E69">
         <f t="shared" si="7"/>
         <v>0</v>
+      </c>
+      <c r="G69">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9">
+      <c r="A70" t="s">
+        <v>189</v>
+      </c>
+      <c r="B70" t="s">
+        <v>213</v>
+      </c>
+      <c r="E70">
+        <f>D70/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F70">
+        <v>6277</v>
+      </c>
+      <c r="G70" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>10101.855413271598</v>
+      </c>
+      <c r="H70" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I70" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9">
+      <c r="A71" t="s">
+        <v>189</v>
+      </c>
+      <c r="B71" t="s">
+        <v>214</v>
+      </c>
+      <c r="E71">
+        <f t="shared" ref="E71:E81" si="8">D71/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F71">
+        <v>4581</v>
+      </c>
+      <c r="G71" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7372.4071448458171</v>
+      </c>
+      <c r="H71" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I71" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9">
+      <c r="A72" t="s">
+        <v>189</v>
+      </c>
+      <c r="B72" t="s">
+        <v>215</v>
+      </c>
+      <c r="E72">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F72">
+        <v>3668</v>
+      </c>
+      <c r="G72" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5903.0756182699097</v>
+      </c>
+      <c r="H72" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I72" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9">
+      <c r="A73" t="s">
+        <v>189</v>
+      </c>
+      <c r="B73" t="s">
+        <v>216</v>
+      </c>
+      <c r="E73">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F73">
+        <v>4452</v>
+      </c>
+      <c r="G73" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7164.8017046176765</v>
+      </c>
+      <c r="H73" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I73" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9">
+      <c r="A74" t="s">
+        <v>189</v>
+      </c>
+      <c r="B74" t="s">
+        <v>217</v>
+      </c>
+      <c r="E74">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F74">
+        <v>4327</v>
+      </c>
+      <c r="G74" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6963.6336423811072</v>
+      </c>
+      <c r="H74" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I74" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9">
+      <c r="A75" t="s">
+        <v>189</v>
+      </c>
+      <c r="B75" t="s">
+        <v>218</v>
+      </c>
+      <c r="E75">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F75">
+        <v>7211</v>
+      </c>
+      <c r="G75" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11604.98317430325</v>
+      </c>
+      <c r="H75" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I75" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9">
+      <c r="A76" t="s">
+        <v>189</v>
+      </c>
+      <c r="B76" t="s">
+        <v>219</v>
+      </c>
+      <c r="E76">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F76">
+        <v>6346</v>
+      </c>
+      <c r="G76" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>10212.900183626185</v>
+      </c>
+      <c r="H76" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I76" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9">
+      <c r="A77" t="s">
+        <v>189</v>
+      </c>
+      <c r="B77" t="s">
+        <v>220</v>
+      </c>
+      <c r="E77">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F77">
+        <v>7020</v>
+      </c>
+      <c r="G77" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11297.598375205771</v>
+      </c>
+      <c r="H77" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I77" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9">
+      <c r="A78" t="s">
+        <v>189</v>
+      </c>
+      <c r="B78" t="s">
+        <v>221</v>
+      </c>
+      <c r="E78">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F78">
+        <v>5266</v>
+      </c>
+      <c r="G78" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8474.8081259022201</v>
+      </c>
+      <c r="H78" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I78" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9">
+      <c r="A79" t="s">
+        <v>189</v>
+      </c>
+      <c r="B79" t="s">
+        <v>222</v>
+      </c>
+      <c r="E79">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F79">
+        <v>4657</v>
+      </c>
+      <c r="G79" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7494.7173266856516</v>
+      </c>
+      <c r="H79" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I79" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9">
+      <c r="A80" t="s">
+        <v>189</v>
+      </c>
+      <c r="B80" t="s">
+        <v>223</v>
+      </c>
+      <c r="E80">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F80">
+        <v>3667</v>
+      </c>
+      <c r="G80" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5901.4662737720173</v>
+      </c>
+      <c r="H80" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I80" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9">
+      <c r="A81" t="s">
+        <v>189</v>
+      </c>
+      <c r="B81" t="s">
+        <v>224</v>
+      </c>
+      <c r="E81">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F81">
+        <v>6094</v>
+      </c>
+      <c r="G81" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>9807.3453701572598</v>
+      </c>
+      <c r="H81" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I81" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9">
+      <c r="A82" t="s">
+        <v>189</v>
+      </c>
+      <c r="B82" t="s">
+        <v>239</v>
+      </c>
+      <c r="E82">
+        <f t="shared" ref="E82:E86" si="9">D82/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F82">
+        <v>7423</v>
+      </c>
+      <c r="G82" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11946.164207856473</v>
+      </c>
+      <c r="H82" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I82" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9">
+      <c r="A83" t="s">
+        <v>189</v>
+      </c>
+      <c r="B83" t="s">
+        <v>240</v>
+      </c>
+      <c r="E83">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>7423</v>
+      </c>
+      <c r="G83" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11946.164207856473</v>
+      </c>
+      <c r="H83" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I83" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9">
+      <c r="A84" t="s">
+        <v>189</v>
+      </c>
+      <c r="B84" t="s">
+        <v>241</v>
+      </c>
+      <c r="E84">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F84">
+        <v>6540</v>
+      </c>
+      <c r="G84" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>10525.113016217341</v>
+      </c>
+      <c r="H84" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I84" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9">
+      <c r="A85" t="s">
+        <v>189</v>
+      </c>
+      <c r="B85" t="s">
+        <v>242</v>
+      </c>
+      <c r="E85">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F85">
+        <v>6078</v>
+      </c>
+      <c r="G85" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>9781.5958581909799</v>
+      </c>
+      <c r="H85" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I85" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9">
+      <c r="A86" t="s">
+        <v>189</v>
+      </c>
+      <c r="B86" t="s">
+        <v>243</v>
+      </c>
+      <c r="E86">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F86">
+        <v>7363</v>
+      </c>
+      <c r="G86" s="14">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11849.603537982919</v>
+      </c>
+      <c r="H86" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I86" t="s">
+        <v>248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add LNG transport distances from Trinidad
from Point Fortin to the different regions
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D437736-9726-409F-94A3-BB11E9CBA2EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB956D2-320F-4869-BA15-A23B770D3500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1503" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="254">
   <si>
     <t>Belgium</t>
   </si>
@@ -796,9 +796,6 @@
     <t>Tokyo</t>
   </si>
   <si>
-    <t>Mumbai</t>
-  </si>
-  <si>
     <t>Okha</t>
   </si>
   <si>
@@ -806,6 +803,9 @@
   </si>
   <si>
     <t>Port Said</t>
+  </si>
+  <si>
+    <t>Trinidad from Point Fortin</t>
   </si>
 </sst>
 </file>
@@ -1514,8 +1514,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:I103" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
-  <autoFilter ref="A1:I103" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:I120" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+  <autoFilter ref="A1:I120" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
     <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
@@ -14154,7 +14154,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M103"/>
+  <dimension ref="A1:M120"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="21.81640625" customWidth="1"/>
@@ -14263,6 +14263,9 @@
       </c>
       <c r="H4" s="12"/>
       <c r="I4" s="12"/>
+      <c r="M4" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
@@ -14418,11 +14421,11 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <v>9727</v>
+        <v>9568</v>
       </c>
       <c r="G12">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>15654.093931000931</v>
+        <v>15398.208155836013</v>
       </c>
       <c r="H12" t="s">
         <v>219</v>
@@ -14453,7 +14456,7 @@
         <v>247</v>
       </c>
       <c r="I13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -14475,7 +14478,7 @@
         <v>10752.030590420192</v>
       </c>
       <c r="I14" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -14489,9 +14492,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F15">
+        <v>3136</v>
+      </c>
       <c r="G15">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>5046.9043453910681</v>
+      </c>
+      <c r="I15" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -14505,9 +14514,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F16">
+        <v>4174</v>
+      </c>
       <c r="G16">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>6717.4039342035448</v>
+      </c>
+      <c r="I16" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -14521,9 +14536,18 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F17">
+        <v>9806</v>
+      </c>
       <c r="G17">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>15781.232146334443</v>
+      </c>
+      <c r="H17" t="s">
+        <v>247</v>
+      </c>
+      <c r="I17" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -14537,9 +14561,18 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F18">
+        <v>8878</v>
+      </c>
       <c r="G18">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>14287.760452290147</v>
+      </c>
+      <c r="H18" t="s">
+        <v>247</v>
+      </c>
+      <c r="I18" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -14553,9 +14586,18 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F19">
+        <v>8211</v>
+      </c>
       <c r="G19">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>13214.32767219581</v>
+      </c>
+      <c r="H19" t="s">
+        <v>219</v>
+      </c>
+      <c r="I19" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -14569,9 +14611,18 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F20">
+        <v>11169</v>
+      </c>
       <c r="G20">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>17974.768696962001</v>
+      </c>
+      <c r="H20" t="s">
+        <v>219</v>
+      </c>
+      <c r="I20" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -14585,9 +14636,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F21">
+        <v>5324</v>
+      </c>
       <c r="G21">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>8568.1501067799891</v>
+      </c>
+      <c r="I21" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -14809,7 +14866,7 @@
         <v>1638.312698854626</v>
       </c>
       <c r="I33" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -14831,7 +14888,7 @@
         <v>7143.8802261450737</v>
       </c>
       <c r="I34" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -15839,11 +15896,10 @@
       <c r="F87">
         <v>4986</v>
       </c>
-      <c r="G87" s="13">
+      <c r="G87">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8024.1916664923037</v>
       </c>
-      <c r="H87" s="13"/>
       <c r="I87" t="s">
         <v>240</v>
       </c>
@@ -15862,11 +15918,10 @@
       <c r="F88">
         <v>4815</v>
       </c>
-      <c r="G88" s="13">
+      <c r="G88">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7748.9937573526759</v>
       </c>
-      <c r="H88" s="13"/>
       <c r="I88" t="s">
         <v>220</v>
       </c>
@@ -15885,11 +15940,10 @@
       <c r="F89">
         <v>6255</v>
       </c>
-      <c r="G89" s="13">
+      <c r="G89">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10066.449834317962</v>
       </c>
-      <c r="H89" s="13"/>
       <c r="I89" t="s">
         <v>221</v>
       </c>
@@ -15908,11 +15962,10 @@
       <c r="F90">
         <v>5637</v>
       </c>
-      <c r="G90" s="13">
+      <c r="G90">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9071.8749346203604</v>
       </c>
-      <c r="H90" s="13"/>
       <c r="I90" t="s">
         <v>222</v>
       </c>
@@ -15931,11 +15984,10 @@
       <c r="F91">
         <v>6380</v>
       </c>
-      <c r="G91" s="13">
+      <c r="G91">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10267.617896554533</v>
       </c>
-      <c r="H91" s="13"/>
       <c r="I91" t="s">
         <v>223</v>
       </c>
@@ -15954,11 +16006,10 @@
       <c r="F92">
         <v>5634</v>
       </c>
-      <c r="G92" s="13">
+      <c r="G92">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9067.0469011266832</v>
       </c>
-      <c r="H92" s="13"/>
       <c r="I92" t="s">
         <v>224</v>
       </c>
@@ -15977,11 +16028,10 @@
       <c r="F93">
         <v>5052</v>
       </c>
-      <c r="G93" s="13">
+      <c r="G93">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8130.4084033532126</v>
       </c>
-      <c r="H93" s="13"/>
       <c r="I93" t="s">
         <v>225</v>
       </c>
@@ -16000,11 +16050,10 @@
       <c r="F94">
         <v>5443</v>
       </c>
-      <c r="G94" s="13">
+      <c r="G94">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8759.6621020292041</v>
       </c>
-      <c r="H94" s="13"/>
       <c r="I94" t="s">
         <v>226</v>
       </c>
@@ -16023,11 +16072,10 @@
       <c r="F95">
         <v>4565</v>
       </c>
-      <c r="G95" s="13">
+      <c r="G95">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7346.6576328795363</v>
       </c>
-      <c r="H95" s="13"/>
       <c r="I95" t="s">
         <v>227</v>
       </c>
@@ -16046,11 +16094,10 @@
       <c r="F96">
         <v>4786</v>
       </c>
-      <c r="G96" s="13">
+      <c r="G96">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7702.3227669137923</v>
       </c>
-      <c r="H96" s="13"/>
       <c r="I96" t="s">
         <v>243</v>
       </c>
@@ -16069,11 +16116,10 @@
       <c r="F97">
         <v>6409</v>
       </c>
-      <c r="G97" s="13">
+      <c r="G97">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10314.288886993416</v>
       </c>
-      <c r="H97" s="13"/>
       <c r="I97" t="s">
         <v>229</v>
       </c>
@@ -16092,11 +16138,10 @@
       <c r="F98">
         <v>4666</v>
       </c>
-      <c r="G98" s="13">
+      <c r="G98">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7509.2014271666849</v>
       </c>
-      <c r="H98" s="13"/>
       <c r="I98" t="s">
         <v>244</v>
       </c>
@@ -16115,11 +16160,10 @@
       <c r="F99">
         <v>5846</v>
       </c>
-      <c r="G99" s="13">
+      <c r="G99">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9408.227934679906</v>
       </c>
-      <c r="H99" s="13"/>
       <c r="I99" t="s">
         <v>235</v>
       </c>
@@ -16138,11 +16182,10 @@
       <c r="F100">
         <v>5846</v>
       </c>
-      <c r="G100" s="13">
+      <c r="G100">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9408.227934679906</v>
       </c>
-      <c r="H100" s="13"/>
       <c r="I100" t="s">
         <v>236</v>
       </c>
@@ -16161,11 +16204,10 @@
       <c r="F101">
         <v>5215</v>
       </c>
-      <c r="G101" s="13">
+      <c r="G101">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8392.7315565096997</v>
       </c>
-      <c r="H101" s="13"/>
       <c r="I101" t="s">
         <v>237</v>
       </c>
@@ -16184,11 +16226,10 @@
       <c r="F102">
         <v>4564</v>
       </c>
-      <c r="G102" s="13">
+      <c r="G102">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7345.0482883816439</v>
       </c>
-      <c r="H102" s="13"/>
       <c r="I102" t="s">
         <v>238</v>
       </c>
@@ -16207,12 +16248,402 @@
       <c r="F103">
         <v>5786</v>
       </c>
-      <c r="G103" s="13">
+      <c r="G103">
         <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9311.6672648063523</v>
       </c>
-      <c r="H103" s="13"/>
       <c r="I103" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9">
+      <c r="A104" t="s">
+        <v>187</v>
+      </c>
+      <c r="B104" t="s">
+        <v>206</v>
+      </c>
+      <c r="E104">
+        <f>D104/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F104">
+        <v>3985</v>
+      </c>
+      <c r="G104" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6413.2378241018514</v>
+      </c>
+      <c r="H104" s="13"/>
+      <c r="I104" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9">
+      <c r="A105" t="s">
+        <v>187</v>
+      </c>
+      <c r="B105" t="s">
+        <v>207</v>
+      </c>
+      <c r="E105">
+        <f t="shared" ref="E105:E120" si="11">D105/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F105">
+        <v>4101</v>
+      </c>
+      <c r="G105" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6599.9217858573884</v>
+      </c>
+      <c r="H105" s="13"/>
+      <c r="I105" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9">
+      <c r="A106" t="s">
+        <v>187</v>
+      </c>
+      <c r="B106" t="s">
+        <v>208</v>
+      </c>
+      <c r="E106">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F106">
+        <v>4898</v>
+      </c>
+      <c r="G106" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7882.5693506777588</v>
+      </c>
+      <c r="H106" s="13"/>
+      <c r="I106" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9">
+      <c r="A107" t="s">
+        <v>187</v>
+      </c>
+      <c r="B107" t="s">
+        <v>209</v>
+      </c>
+      <c r="E107">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F107">
+        <v>4280</v>
+      </c>
+      <c r="G107" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6887.9944509801562</v>
+      </c>
+      <c r="H107" s="13"/>
+      <c r="I107" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9">
+      <c r="A108" t="s">
+        <v>187</v>
+      </c>
+      <c r="B108" t="s">
+        <v>210</v>
+      </c>
+      <c r="E108">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F108">
+        <v>5023</v>
+      </c>
+      <c r="G108" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8083.7374129143291</v>
+      </c>
+      <c r="H108" s="13"/>
+      <c r="I108" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9">
+      <c r="A109" t="s">
+        <v>187</v>
+      </c>
+      <c r="B109" t="s">
+        <v>211</v>
+      </c>
+      <c r="E109">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F109">
+        <v>4823</v>
+      </c>
+      <c r="G109" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7761.8685133358167</v>
+      </c>
+      <c r="H109" s="13"/>
+      <c r="I109" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9">
+      <c r="A110" t="s">
+        <v>187</v>
+      </c>
+      <c r="B110" t="s">
+        <v>212</v>
+      </c>
+      <c r="E110">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F110">
+        <v>4051</v>
+      </c>
+      <c r="G110" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6519.4545609627603</v>
+      </c>
+      <c r="H110" s="13"/>
+      <c r="I110" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9">
+      <c r="A111" t="s">
+        <v>187</v>
+      </c>
+      <c r="B111" t="s">
+        <v>213</v>
+      </c>
+      <c r="E111">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F111">
+        <v>4632</v>
+      </c>
+      <c r="G111" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7454.4837142383376</v>
+      </c>
+      <c r="H111" s="13"/>
+      <c r="I111" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9">
+      <c r="A112" t="s">
+        <v>187</v>
+      </c>
+      <c r="B112" t="s">
+        <v>214</v>
+      </c>
+      <c r="E112">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F112">
+        <v>3299</v>
+      </c>
+      <c r="G112" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5309.2274985475551</v>
+      </c>
+      <c r="H112" s="13"/>
+      <c r="I112" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9">
+      <c r="A113" t="s">
+        <v>187</v>
+      </c>
+      <c r="B113" t="s">
+        <v>215</v>
+      </c>
+      <c r="E113">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F113">
+        <v>3645</v>
+      </c>
+      <c r="G113" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5866.0606948183813</v>
+      </c>
+      <c r="H113" s="13"/>
+      <c r="I113" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9">
+      <c r="A114" t="s">
+        <v>187</v>
+      </c>
+      <c r="B114" t="s">
+        <v>216</v>
+      </c>
+      <c r="E114">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F114">
+        <v>5052</v>
+      </c>
+      <c r="G114" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8130.4084033532126</v>
+      </c>
+      <c r="H114" s="13"/>
+      <c r="I114" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9">
+      <c r="A115" t="s">
+        <v>187</v>
+      </c>
+      <c r="B115" t="s">
+        <v>217</v>
+      </c>
+      <c r="E115">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F115">
+        <v>3733</v>
+      </c>
+      <c r="G115" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6007.6830106329262</v>
+      </c>
+      <c r="H115" s="13"/>
+      <c r="I115" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9">
+      <c r="A116" t="s">
+        <v>187</v>
+      </c>
+      <c r="B116" t="s">
+        <v>230</v>
+      </c>
+      <c r="E116">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F116">
+        <v>5035</v>
+      </c>
+      <c r="G116" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8103.0495468890394</v>
+      </c>
+      <c r="H116" s="13"/>
+      <c r="I116" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9">
+      <c r="A117" t="s">
+        <v>187</v>
+      </c>
+      <c r="B117" t="s">
+        <v>231</v>
+      </c>
+      <c r="E117">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F117">
+        <v>5035</v>
+      </c>
+      <c r="G117" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8103.0495468890394</v>
+      </c>
+      <c r="H117" s="13"/>
+      <c r="I117" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9">
+      <c r="A118" t="s">
+        <v>187</v>
+      </c>
+      <c r="B118" t="s">
+        <v>232</v>
+      </c>
+      <c r="E118">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F118">
+        <v>4248</v>
+      </c>
+      <c r="G118" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6836.4954270475946</v>
+      </c>
+      <c r="H118" s="13"/>
+      <c r="I118" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9">
+      <c r="A119" t="s">
+        <v>187</v>
+      </c>
+      <c r="B119" t="s">
+        <v>233</v>
+      </c>
+      <c r="E119">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F119">
+        <v>3599</v>
+      </c>
+      <c r="G119" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5792.0308479153236</v>
+      </c>
+      <c r="H119" s="13"/>
+      <c r="I119" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9">
+      <c r="A120" t="s">
+        <v>187</v>
+      </c>
+      <c r="B120" t="s">
+        <v>234</v>
+      </c>
+      <c r="E120">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="F120">
+        <v>4975</v>
+      </c>
+      <c r="G120" s="13">
+        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8006.4888770154857</v>
+      </c>
+      <c r="H120" s="13"/>
+      <c r="I120" t="s">
         <v>239</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add LNG transport distances from ME
from Das Island (UAE) to the different regions
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DB956D2-320F-4869-BA15-A23B770D3500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7555382-E962-4D0A-9BCF-DC91D0C33829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1642" uniqueCount="255">
   <si>
     <t>Belgium</t>
   </si>
@@ -806,6 +806,9 @@
   </si>
   <si>
     <t>Trinidad from Point Fortin</t>
+  </si>
+  <si>
+    <t>ME from Das Island (UAE)</t>
   </si>
 </sst>
 </file>
@@ -1514,8 +1517,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="Table11" displayName="Table11" ref="A1:I120" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
-  <autoFilter ref="A1:I120" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I137" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+  <autoFilter ref="A1:I137" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
     <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
@@ -1528,7 +1531,7 @@
     </tableColumn>
     <tableColumn id="5" xr3:uid="{7E7B8CB5-D54F-4427-813D-93B66C13FCBB}" name="Distance [miles]"/>
     <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="1">
-      <calculatedColumnFormula>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
+      <calculatedColumnFormula>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="0"/>
     <tableColumn id="8" xr3:uid="{ECBB25E4-2145-4120-8981-E6E8E1591E5B}" name="Comment"/>
@@ -14154,7 +14157,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M120"/>
+  <dimension ref="A1:M137"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="21.81640625" customWidth="1"/>
@@ -14210,7 +14213,7 @@
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="6">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
       <c r="H2" s="6"/>
@@ -14234,7 +14237,7 @@
       </c>
       <c r="F3" s="11"/>
       <c r="G3" s="11">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
       <c r="H3" s="11"/>
@@ -14258,7 +14261,7 @@
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
       <c r="H4" s="12"/>
@@ -14279,8 +14282,11 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="M5" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -14295,7 +14301,7 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -14311,7 +14317,7 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -14330,7 +14336,7 @@
         <v>5323</v>
       </c>
       <c r="G8">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8566.5407622820967</v>
       </c>
       <c r="I8" t="s">
@@ -14352,7 +14358,7 @@
         <v>6194</v>
       </c>
       <c r="G9">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9968.279819946516</v>
       </c>
       <c r="I9" t="s">
@@ -14374,7 +14380,7 @@
         <v>10194</v>
       </c>
       <c r="G10">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>16405.657811516758</v>
       </c>
       <c r="H10" t="s">
@@ -14399,7 +14405,7 @@
         <v>9266</v>
       </c>
       <c r="G11">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>14912.18611747246</v>
       </c>
       <c r="H11" t="s">
@@ -14424,7 +14430,7 @@
         <v>9568</v>
       </c>
       <c r="G12">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>15398.208155836013</v>
       </c>
       <c r="H12" t="s">
@@ -14449,7 +14455,7 @@
         <v>12151</v>
       </c>
       <c r="G13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>19555.144993892496</v>
       </c>
       <c r="H13" t="s">
@@ -14474,7 +14480,7 @@
         <v>6681</v>
       </c>
       <c r="G14">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10752.030590420192</v>
       </c>
       <c r="I14" t="s">
@@ -14496,7 +14502,7 @@
         <v>3136</v>
       </c>
       <c r="G15">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5046.9043453910681</v>
       </c>
       <c r="I15" t="s">
@@ -14518,7 +14524,7 @@
         <v>4174</v>
       </c>
       <c r="G16">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6717.4039342035448</v>
       </c>
       <c r="I16" t="s">
@@ -14540,7 +14546,7 @@
         <v>9806</v>
       </c>
       <c r="G17">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>15781.232146334443</v>
       </c>
       <c r="H17" t="s">
@@ -14565,7 +14571,7 @@
         <v>8878</v>
       </c>
       <c r="G18">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>14287.760452290147</v>
       </c>
       <c r="H18" t="s">
@@ -14590,7 +14596,7 @@
         <v>8211</v>
       </c>
       <c r="G19">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>13214.32767219581</v>
       </c>
       <c r="H19" t="s">
@@ -14615,7 +14621,7 @@
         <v>11169</v>
       </c>
       <c r="G20">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>17974.768696962001</v>
       </c>
       <c r="H20" t="s">
@@ -14640,7 +14646,7 @@
         <v>5324</v>
       </c>
       <c r="G21">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8568.1501067799891</v>
       </c>
       <c r="I21" t="s">
@@ -14658,9 +14664,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F22">
+        <v>8091</v>
+      </c>
       <c r="G22">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>13021.206332448703</v>
+      </c>
+      <c r="I22" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -14674,9 +14686,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F23">
+        <v>7282</v>
+      </c>
       <c r="G23">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11719.246633653622</v>
+      </c>
+      <c r="I23" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -14690,9 +14708,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F24">
+        <v>6160</v>
+      </c>
       <c r="G24">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>9913.5621070181696</v>
+      </c>
+      <c r="I24" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -14706,9 +14730,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F25">
+        <v>6445</v>
+      </c>
       <c r="G25">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>10372.225288917549</v>
+      </c>
+      <c r="I25" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -14722,9 +14752,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F26">
+        <v>951</v>
+      </c>
       <c r="G26">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>1530.4866174958245</v>
+      </c>
+      <c r="I26" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -14738,9 +14774,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F27">
+        <v>4372</v>
+      </c>
       <c r="G27">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7036.0541447862724</v>
+      </c>
+      <c r="I27" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -14754,9 +14796,15 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="F28">
+        <v>2915</v>
+      </c>
       <c r="G28">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4691.2392113568121</v>
+      </c>
+      <c r="I28" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -14774,7 +14822,7 @@
         <v>8158</v>
       </c>
       <c r="G29">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>13129.032413807505</v>
       </c>
       <c r="I29" t="s">
@@ -14796,7 +14844,7 @@
         <v>7349</v>
       </c>
       <c r="G30">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>11827.072715012424</v>
       </c>
       <c r="I30" t="s">
@@ -14818,7 +14866,7 @@
         <v>6227</v>
       </c>
       <c r="G31">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10021.38818837697</v>
       </c>
       <c r="I31" t="s">
@@ -14840,7 +14888,7 @@
         <v>6512</v>
       </c>
       <c r="G32">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10480.051370276351</v>
       </c>
       <c r="I32" t="s">
@@ -14862,7 +14910,7 @@
         <v>1018</v>
       </c>
       <c r="G33">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>1638.312698854626</v>
       </c>
       <c r="I33" t="s">
@@ -14884,7 +14932,7 @@
         <v>4439</v>
       </c>
       <c r="G34">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7143.8802261450737</v>
       </c>
       <c r="I34" t="s">
@@ -14906,7 +14954,7 @@
         <v>2982</v>
       </c>
       <c r="G35">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>4799.0652927156134</v>
       </c>
       <c r="I35" t="s">
@@ -14925,7 +14973,7 @@
         <v>0</v>
       </c>
       <c r="G36">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -14941,7 +14989,7 @@
         <v>0</v>
       </c>
       <c r="G37">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -14957,7 +15005,7 @@
         <v>0</v>
       </c>
       <c r="G38">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -14973,7 +15021,7 @@
         <v>0</v>
       </c>
       <c r="G39">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -14989,7 +15037,7 @@
         <v>0</v>
       </c>
       <c r="G40">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15005,7 +15053,7 @@
         <v>0</v>
       </c>
       <c r="G41">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15021,7 +15069,7 @@
         <v>0</v>
       </c>
       <c r="G42">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15037,7 +15085,7 @@
         <v>0</v>
       </c>
       <c r="G43">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15053,7 +15101,7 @@
         <v>0</v>
       </c>
       <c r="G44">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15069,7 +15117,7 @@
         <v>0</v>
       </c>
       <c r="G45">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15085,7 +15133,7 @@
         <v>0</v>
       </c>
       <c r="G46">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15101,7 +15149,7 @@
         <v>0</v>
       </c>
       <c r="G47">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15117,7 +15165,7 @@
         <v>0</v>
       </c>
       <c r="G48">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15133,7 +15181,7 @@
         <v>0</v>
       </c>
       <c r="G49">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15149,7 +15197,7 @@
         <v>0</v>
       </c>
       <c r="G50">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15165,7 +15213,7 @@
         <v>0</v>
       </c>
       <c r="G51">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15181,7 +15229,7 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15197,7 +15245,7 @@
         <v>0</v>
       </c>
       <c r="G53">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15213,7 +15261,7 @@
         <v>0</v>
       </c>
       <c r="G54">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15229,7 +15277,7 @@
         <v>0</v>
       </c>
       <c r="G55">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15245,7 +15293,7 @@
         <v>0</v>
       </c>
       <c r="G56">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15261,7 +15309,7 @@
         <v>0</v>
       </c>
       <c r="G57">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15277,7 +15325,7 @@
         <v>0</v>
       </c>
       <c r="G58">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15293,7 +15341,7 @@
         <v>0</v>
       </c>
       <c r="G59">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15309,7 +15357,7 @@
         <v>0</v>
       </c>
       <c r="G60">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15325,7 +15373,7 @@
         <v>0</v>
       </c>
       <c r="G61">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15341,7 +15389,7 @@
         <v>0</v>
       </c>
       <c r="G62">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15357,7 +15405,7 @@
         <v>0</v>
       </c>
       <c r="G63">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15373,7 +15421,7 @@
         <v>0</v>
       </c>
       <c r="G64">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15389,7 +15437,7 @@
         <v>0</v>
       </c>
       <c r="G65">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15405,7 +15453,7 @@
         <v>0</v>
       </c>
       <c r="G66">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15421,7 +15469,7 @@
         <v>0</v>
       </c>
       <c r="G67">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15437,7 +15485,7 @@
         <v>0</v>
       </c>
       <c r="G68">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15453,7 +15501,7 @@
         <v>0</v>
       </c>
       <c r="G69">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
     </row>
@@ -15472,7 +15520,7 @@
         <v>6277</v>
       </c>
       <c r="G70">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10101.855413271598</v>
       </c>
       <c r="H70" t="s">
@@ -15497,7 +15545,7 @@
         <v>4581</v>
       </c>
       <c r="G71">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7372.4071448458171</v>
       </c>
       <c r="H71" t="s">
@@ -15522,7 +15570,7 @@
         <v>3668</v>
       </c>
       <c r="G72">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5903.0756182699097</v>
       </c>
       <c r="H72" t="s">
@@ -15547,7 +15595,7 @@
         <v>4452</v>
       </c>
       <c r="G73">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7164.8017046176765</v>
       </c>
       <c r="H73" t="s">
@@ -15572,7 +15620,7 @@
         <v>4327</v>
       </c>
       <c r="G74">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6963.6336423811072</v>
       </c>
       <c r="H74" t="s">
@@ -15597,7 +15645,7 @@
         <v>7211</v>
       </c>
       <c r="G75">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>11604.98317430325</v>
       </c>
       <c r="H75" t="s">
@@ -15622,7 +15670,7 @@
         <v>6346</v>
       </c>
       <c r="G76">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10212.900183626185</v>
       </c>
       <c r="H76" t="s">
@@ -15647,7 +15695,7 @@
         <v>7020</v>
       </c>
       <c r="G77">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>11297.598375205771</v>
       </c>
       <c r="H77" t="s">
@@ -15672,7 +15720,7 @@
         <v>5266</v>
       </c>
       <c r="G78">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8474.8081259022201</v>
       </c>
       <c r="H78" t="s">
@@ -15697,7 +15745,7 @@
         <v>4657</v>
       </c>
       <c r="G79">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7494.7173266856516</v>
       </c>
       <c r="H79" t="s">
@@ -15722,7 +15770,7 @@
         <v>3667</v>
       </c>
       <c r="G80">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5901.4662737720173</v>
       </c>
       <c r="H80" t="s">
@@ -15747,7 +15795,7 @@
         <v>6091</v>
       </c>
       <c r="G81">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9802.5173366635827</v>
       </c>
       <c r="H81" t="s">
@@ -15772,7 +15820,7 @@
         <v>7423</v>
       </c>
       <c r="G82">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>11946.164207856473</v>
       </c>
       <c r="H82" t="s">
@@ -15797,7 +15845,7 @@
         <v>7423</v>
       </c>
       <c r="G83">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>11946.164207856473</v>
       </c>
       <c r="H83" t="s">
@@ -15822,7 +15870,7 @@
         <v>6540</v>
       </c>
       <c r="G84">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10525.113016217341</v>
       </c>
       <c r="H84" t="s">
@@ -15847,7 +15895,7 @@
         <v>6078</v>
       </c>
       <c r="G85">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9781.5958581909799</v>
       </c>
       <c r="H85" t="s">
@@ -15872,7 +15920,7 @@
         <v>7363</v>
       </c>
       <c r="G86">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>11849.603537982919</v>
       </c>
       <c r="H86" t="s">
@@ -15897,7 +15945,7 @@
         <v>4986</v>
       </c>
       <c r="G87">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8024.1916664923037</v>
       </c>
       <c r="I87" t="s">
@@ -15919,7 +15967,7 @@
         <v>4815</v>
       </c>
       <c r="G88">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7748.9937573526759</v>
       </c>
       <c r="I88" t="s">
@@ -15941,7 +15989,7 @@
         <v>6255</v>
       </c>
       <c r="G89">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10066.449834317962</v>
       </c>
       <c r="I89" t="s">
@@ -15963,7 +16011,7 @@
         <v>5637</v>
       </c>
       <c r="G90">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9071.8749346203604</v>
       </c>
       <c r="I90" t="s">
@@ -15985,7 +16033,7 @@
         <v>6380</v>
       </c>
       <c r="G91">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10267.617896554533</v>
       </c>
       <c r="I91" t="s">
@@ -16007,7 +16055,7 @@
         <v>5634</v>
       </c>
       <c r="G92">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9067.0469011266832</v>
       </c>
       <c r="I92" t="s">
@@ -16029,7 +16077,7 @@
         <v>5052</v>
       </c>
       <c r="G93">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8130.4084033532126</v>
       </c>
       <c r="I93" t="s">
@@ -16051,7 +16099,7 @@
         <v>5443</v>
       </c>
       <c r="G94">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8759.6621020292041</v>
       </c>
       <c r="I94" t="s">
@@ -16073,7 +16121,7 @@
         <v>4565</v>
       </c>
       <c r="G95">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7346.6576328795363</v>
       </c>
       <c r="I95" t="s">
@@ -16095,7 +16143,7 @@
         <v>4786</v>
       </c>
       <c r="G96">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7702.3227669137923</v>
       </c>
       <c r="I96" t="s">
@@ -16117,7 +16165,7 @@
         <v>6409</v>
       </c>
       <c r="G97">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10314.288886993416</v>
       </c>
       <c r="I97" t="s">
@@ -16139,7 +16187,7 @@
         <v>4666</v>
       </c>
       <c r="G98">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7509.2014271666849</v>
       </c>
       <c r="I98" t="s">
@@ -16161,7 +16209,7 @@
         <v>5846</v>
       </c>
       <c r="G99">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9408.227934679906</v>
       </c>
       <c r="I99" t="s">
@@ -16183,7 +16231,7 @@
         <v>5846</v>
       </c>
       <c r="G100">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9408.227934679906</v>
       </c>
       <c r="I100" t="s">
@@ -16205,7 +16253,7 @@
         <v>5215</v>
       </c>
       <c r="G101">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8392.7315565096997</v>
       </c>
       <c r="I101" t="s">
@@ -16227,7 +16275,7 @@
         <v>4564</v>
       </c>
       <c r="G102">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7345.0482883816439</v>
       </c>
       <c r="I102" t="s">
@@ -16249,7 +16297,7 @@
         <v>5786</v>
       </c>
       <c r="G103">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9311.6672648063523</v>
       </c>
       <c r="I103" t="s">
@@ -16270,11 +16318,10 @@
       <c r="F104">
         <v>3985</v>
       </c>
-      <c r="G104" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G104">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6413.2378241018514</v>
       </c>
-      <c r="H104" s="13"/>
       <c r="I104" t="s">
         <v>240</v>
       </c>
@@ -16293,11 +16340,10 @@
       <c r="F105">
         <v>4101</v>
       </c>
-      <c r="G105" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G105">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6599.9217858573884</v>
       </c>
-      <c r="H105" s="13"/>
       <c r="I105" t="s">
         <v>220</v>
       </c>
@@ -16316,11 +16362,10 @@
       <c r="F106">
         <v>4898</v>
       </c>
-      <c r="G106" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G106">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7882.5693506777588</v>
       </c>
-      <c r="H106" s="13"/>
       <c r="I106" t="s">
         <v>221</v>
       </c>
@@ -16339,11 +16384,10 @@
       <c r="F107">
         <v>4280</v>
       </c>
-      <c r="G107" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G107">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6887.9944509801562</v>
       </c>
-      <c r="H107" s="13"/>
       <c r="I107" t="s">
         <v>222</v>
       </c>
@@ -16362,11 +16406,10 @@
       <c r="F108">
         <v>5023</v>
       </c>
-      <c r="G108" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G108">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8083.7374129143291</v>
       </c>
-      <c r="H108" s="13"/>
       <c r="I108" t="s">
         <v>223</v>
       </c>
@@ -16385,11 +16428,10 @@
       <c r="F109">
         <v>4823</v>
       </c>
-      <c r="G109" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G109">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7761.8685133358167</v>
       </c>
-      <c r="H109" s="13"/>
       <c r="I109" t="s">
         <v>224</v>
       </c>
@@ -16408,11 +16450,10 @@
       <c r="F110">
         <v>4051</v>
       </c>
-      <c r="G110" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G110">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6519.4545609627603</v>
       </c>
-      <c r="H110" s="13"/>
       <c r="I110" t="s">
         <v>225</v>
       </c>
@@ -16431,11 +16472,10 @@
       <c r="F111">
         <v>4632</v>
       </c>
-      <c r="G111" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G111">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7454.4837142383376</v>
       </c>
-      <c r="H111" s="13"/>
       <c r="I111" t="s">
         <v>226</v>
       </c>
@@ -16454,11 +16494,10 @@
       <c r="F112">
         <v>3299</v>
       </c>
-      <c r="G112" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G112">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5309.2274985475551</v>
       </c>
-      <c r="H112" s="13"/>
       <c r="I112" t="s">
         <v>227</v>
       </c>
@@ -16477,11 +16516,10 @@
       <c r="F113">
         <v>3645</v>
       </c>
-      <c r="G113" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G113">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5866.0606948183813</v>
       </c>
-      <c r="H113" s="13"/>
       <c r="I113" t="s">
         <v>243</v>
       </c>
@@ -16500,11 +16538,10 @@
       <c r="F114">
         <v>5052</v>
       </c>
-      <c r="G114" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G114">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8130.4084033532126</v>
       </c>
-      <c r="H114" s="13"/>
       <c r="I114" t="s">
         <v>229</v>
       </c>
@@ -16523,11 +16560,10 @@
       <c r="F115">
         <v>3733</v>
       </c>
-      <c r="G115" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G115">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6007.6830106329262</v>
       </c>
-      <c r="H115" s="13"/>
       <c r="I115" t="s">
         <v>244</v>
       </c>
@@ -16546,11 +16582,10 @@
       <c r="F116">
         <v>5035</v>
       </c>
-      <c r="G116" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G116">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8103.0495468890394</v>
       </c>
-      <c r="H116" s="13"/>
       <c r="I116" t="s">
         <v>235</v>
       </c>
@@ -16569,11 +16604,10 @@
       <c r="F117">
         <v>5035</v>
       </c>
-      <c r="G117" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G117">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8103.0495468890394</v>
       </c>
-      <c r="H117" s="13"/>
       <c r="I117" t="s">
         <v>236</v>
       </c>
@@ -16592,11 +16626,10 @@
       <c r="F118">
         <v>4248</v>
       </c>
-      <c r="G118" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G118">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6836.4954270475946</v>
       </c>
-      <c r="H118" s="13"/>
       <c r="I118" t="s">
         <v>237</v>
       </c>
@@ -16615,11 +16648,10 @@
       <c r="F119">
         <v>3599</v>
       </c>
-      <c r="G119" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G119">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5792.0308479153236</v>
       </c>
-      <c r="H119" s="13"/>
       <c r="I119" t="s">
         <v>238</v>
       </c>
@@ -16638,12 +16670,436 @@
       <c r="F120">
         <v>4975</v>
       </c>
-      <c r="G120" s="13">
-        <f>Table11[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+      <c r="G120">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8006.4888770154857</v>
       </c>
-      <c r="H120" s="13"/>
       <c r="I120" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9">
+      <c r="A121" t="s">
+        <v>188</v>
+      </c>
+      <c r="B121" t="s">
+        <v>206</v>
+      </c>
+      <c r="E121">
+        <f>D121/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F121">
+        <v>6210</v>
+      </c>
+      <c r="G121" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>9994.0293319127977</v>
+      </c>
+      <c r="H121" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I121" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9">
+      <c r="A122" t="s">
+        <v>188</v>
+      </c>
+      <c r="B122" t="s">
+        <v>207</v>
+      </c>
+      <c r="E122">
+        <f t="shared" ref="E122:E137" si="12">D122/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F122">
+        <v>4514</v>
+      </c>
+      <c r="G122" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7264.5810634870159</v>
+      </c>
+      <c r="H122" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I122" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9">
+      <c r="A123" t="s">
+        <v>188</v>
+      </c>
+      <c r="B123" t="s">
+        <v>208</v>
+      </c>
+      <c r="E123">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F123">
+        <v>3601</v>
+      </c>
+      <c r="G123" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5795.2495369111084</v>
+      </c>
+      <c r="H123" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I123" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9">
+      <c r="A124" t="s">
+        <v>188</v>
+      </c>
+      <c r="B124" t="s">
+        <v>209</v>
+      </c>
+      <c r="E124">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F124">
+        <v>4385</v>
+      </c>
+      <c r="G124" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7056.9756232588752</v>
+      </c>
+      <c r="H124" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I124" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9">
+      <c r="A125" t="s">
+        <v>188</v>
+      </c>
+      <c r="B125" t="s">
+        <v>210</v>
+      </c>
+      <c r="E125">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F125">
+        <v>4260</v>
+      </c>
+      <c r="G125" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6855.807561022305</v>
+      </c>
+      <c r="H125" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I125" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9">
+      <c r="A126" t="s">
+        <v>188</v>
+      </c>
+      <c r="B126" t="s">
+        <v>211</v>
+      </c>
+      <c r="E126">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F126">
+        <v>7144</v>
+      </c>
+      <c r="G126" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11497.157092944448</v>
+      </c>
+      <c r="H126" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I126" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9">
+      <c r="A127" t="s">
+        <v>188</v>
+      </c>
+      <c r="B127" t="s">
+        <v>212</v>
+      </c>
+      <c r="E127">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F127">
+        <v>6276</v>
+      </c>
+      <c r="G127" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>10100.246068773706</v>
+      </c>
+      <c r="H127" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I127" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9">
+      <c r="A128" t="s">
+        <v>188</v>
+      </c>
+      <c r="B128" t="s">
+        <v>213</v>
+      </c>
+      <c r="E128">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F128">
+        <v>6953</v>
+      </c>
+      <c r="G128" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11189.772293846969</v>
+      </c>
+      <c r="H128" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I128" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9">
+      <c r="A129" t="s">
+        <v>188</v>
+      </c>
+      <c r="B129" t="s">
+        <v>214</v>
+      </c>
+      <c r="E129">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F129">
+        <v>5199</v>
+      </c>
+      <c r="G129" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8366.9820445434198</v>
+      </c>
+      <c r="H129" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I129" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9">
+      <c r="A130" t="s">
+        <v>188</v>
+      </c>
+      <c r="B130" t="s">
+        <v>215</v>
+      </c>
+      <c r="E130">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F130">
+        <v>4590</v>
+      </c>
+      <c r="G130" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7386.8912453268504</v>
+      </c>
+      <c r="H130" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I130" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9">
+      <c r="A131" t="s">
+        <v>188</v>
+      </c>
+      <c r="B131" t="s">
+        <v>216</v>
+      </c>
+      <c r="E131">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F131">
+        <v>3600</v>
+      </c>
+      <c r="G131" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5793.640192413216</v>
+      </c>
+      <c r="H131" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I131" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9">
+      <c r="A132" t="s">
+        <v>188</v>
+      </c>
+      <c r="B132" t="s">
+        <v>217</v>
+      </c>
+      <c r="E132">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F132">
+        <v>6024</v>
+      </c>
+      <c r="G132" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>9694.6912553047805</v>
+      </c>
+      <c r="H132" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I132" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9">
+      <c r="A133" t="s">
+        <v>188</v>
+      </c>
+      <c r="B133" t="s">
+        <v>230</v>
+      </c>
+      <c r="E133">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F133">
+        <v>7356</v>
+      </c>
+      <c r="G133" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11838.338126497671</v>
+      </c>
+      <c r="H133" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I133" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9">
+      <c r="A134" t="s">
+        <v>188</v>
+      </c>
+      <c r="B134" t="s">
+        <v>231</v>
+      </c>
+      <c r="E134">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F134">
+        <v>7356</v>
+      </c>
+      <c r="G134" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11838.338126497671</v>
+      </c>
+      <c r="H134" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I134" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9">
+      <c r="A135" t="s">
+        <v>188</v>
+      </c>
+      <c r="B135" t="s">
+        <v>232</v>
+      </c>
+      <c r="E135">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F135">
+        <v>6473</v>
+      </c>
+      <c r="G135" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>10417.286934858541</v>
+      </c>
+      <c r="H135" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I135" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9">
+      <c r="A136" t="s">
+        <v>188</v>
+      </c>
+      <c r="B136" t="s">
+        <v>233</v>
+      </c>
+      <c r="E136">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F136">
+        <v>6011</v>
+      </c>
+      <c r="G136" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>9673.7697768321777</v>
+      </c>
+      <c r="H136" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I136" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9">
+      <c r="A137" t="s">
+        <v>188</v>
+      </c>
+      <c r="B137" t="s">
+        <v>234</v>
+      </c>
+      <c r="E137">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F137">
+        <v>7296</v>
+      </c>
+      <c r="G137" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11741.777456624117</v>
+      </c>
+      <c r="H137" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I137" t="s">
         <v>239</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add LNG transport distances from AF
from Port Harcourt (Nigeria) to the different regions
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7555382-E962-4D0A-9BCF-DC91D0C33829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F07001EF-28A2-421E-9DE8-4EC031747CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1642" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1698" uniqueCount="258">
   <si>
     <t>Belgium</t>
   </si>
@@ -809,6 +809,15 @@
   </si>
   <si>
     <t>ME from Das Island (UAE)</t>
+  </si>
+  <si>
+    <t>AF from Port Harcourt (Nigeria)</t>
+  </si>
+  <si>
+    <t>Huelva</t>
+  </si>
+  <si>
+    <t>Mumbai</t>
   </si>
 </sst>
 </file>
@@ -1517,8 +1526,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I137" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
-  <autoFilter ref="A1:I137" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I153" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+  <autoFilter ref="A1:I153" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
     <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
@@ -14157,7 +14166,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M137"/>
+  <dimension ref="A1:M153"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="21.81640625" customWidth="1"/>
@@ -14304,6 +14313,9 @@
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
+      <c r="M6" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
@@ -14972,9 +14984,15 @@
         <f>D36/1000</f>
         <v>0</v>
       </c>
+      <c r="F36">
+        <v>3420</v>
+      </c>
       <c r="G36">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>5503.9581827925549</v>
+      </c>
+      <c r="I36" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -14982,15 +15000,21 @@
         <v>190</v>
       </c>
       <c r="B37" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E37">
-        <f t="shared" ref="E37:E42" si="3">D37/1000</f>
-        <v>0</v>
+        <f t="shared" ref="E37:E41" si="3">D37/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>10496</v>
       </c>
       <c r="G37">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>16891.679849880311</v>
+      </c>
+      <c r="I37" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -14998,15 +15022,21 @@
         <v>190</v>
       </c>
       <c r="B38" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E38">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
+      <c r="F38">
+        <v>10780</v>
+      </c>
       <c r="G38">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>17348.733687281798</v>
+      </c>
+      <c r="I38" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -15014,15 +15044,21 @@
         <v>190</v>
       </c>
       <c r="B39" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E39">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
+      <c r="F39">
+        <v>7016</v>
+      </c>
       <c r="G39">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>11291.160997214201</v>
+      </c>
+      <c r="I39" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -15030,15 +15066,21 @@
         <v>190</v>
       </c>
       <c r="B40" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E40">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
+      <c r="F40">
+        <v>8836</v>
+      </c>
       <c r="G40">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>14220.16798337866</v>
+      </c>
+      <c r="I40" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -15046,26 +15088,32 @@
         <v>190</v>
       </c>
       <c r="B41" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E41">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
+      <c r="F41">
+        <v>5250</v>
+      </c>
       <c r="G41">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>8449.0586139359402</v>
+      </c>
+      <c r="I41" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="42" spans="1:9">
       <c r="A42" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B42" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E42">
-        <f t="shared" si="3"/>
+        <f>D42/1000</f>
         <v>0</v>
       </c>
       <c r="G42">
@@ -15078,10 +15126,10 @@
         <v>191</v>
       </c>
       <c r="B43" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E43">
-        <f>D43/1000</f>
+        <f t="shared" ref="E43:E48" si="4">D43/1000</f>
         <v>0</v>
       </c>
       <c r="G43">
@@ -15094,10 +15142,10 @@
         <v>191</v>
       </c>
       <c r="B44" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E44">
-        <f t="shared" ref="E44:E49" si="4">D44/1000</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="G44">
@@ -15110,7 +15158,7 @@
         <v>191</v>
       </c>
       <c r="B45" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E45">
         <f t="shared" si="4"/>
@@ -15126,7 +15174,7 @@
         <v>191</v>
       </c>
       <c r="B46" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E46">
         <f t="shared" si="4"/>
@@ -15142,7 +15190,7 @@
         <v>191</v>
       </c>
       <c r="B47" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E47">
         <f t="shared" si="4"/>
@@ -15158,7 +15206,7 @@
         <v>191</v>
       </c>
       <c r="B48" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E48">
         <f t="shared" si="4"/>
@@ -15171,13 +15219,13 @@
     </row>
     <row r="49" spans="1:7">
       <c r="A49" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="B49" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E49">
-        <f t="shared" si="4"/>
+        <f>D49/1000</f>
         <v>0</v>
       </c>
       <c r="G49">
@@ -15190,10 +15238,10 @@
         <v>199</v>
       </c>
       <c r="B50" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E50">
-        <f>D50/1000</f>
+        <f t="shared" ref="E50:E55" si="5">D50/1000</f>
         <v>0</v>
       </c>
       <c r="G50">
@@ -15206,10 +15254,10 @@
         <v>199</v>
       </c>
       <c r="B51" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E51">
-        <f t="shared" ref="E51:E56" si="5">D51/1000</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="G51">
@@ -15222,7 +15270,7 @@
         <v>199</v>
       </c>
       <c r="B52" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E52">
         <f t="shared" si="5"/>
@@ -15238,7 +15286,7 @@
         <v>199</v>
       </c>
       <c r="B53" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E53">
         <f t="shared" si="5"/>
@@ -15254,7 +15302,7 @@
         <v>199</v>
       </c>
       <c r="B54" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E54">
         <f t="shared" si="5"/>
@@ -15270,7 +15318,7 @@
         <v>199</v>
       </c>
       <c r="B55" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E55">
         <f t="shared" si="5"/>
@@ -15283,13 +15331,13 @@
     </row>
     <row r="56" spans="1:7">
       <c r="A56" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B56" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="E56">
-        <f t="shared" si="5"/>
+        <f>D56/1000</f>
         <v>0</v>
       </c>
       <c r="G56">
@@ -15302,10 +15350,10 @@
         <v>197</v>
       </c>
       <c r="B57" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E57">
-        <f>D57/1000</f>
+        <f t="shared" ref="E57:E62" si="6">D57/1000</f>
         <v>0</v>
       </c>
       <c r="G57">
@@ -15318,10 +15366,10 @@
         <v>197</v>
       </c>
       <c r="B58" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E58">
-        <f t="shared" ref="E58:E63" si="6">D58/1000</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="G58">
@@ -15334,7 +15382,7 @@
         <v>197</v>
       </c>
       <c r="B59" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E59">
         <f t="shared" si="6"/>
@@ -15350,7 +15398,7 @@
         <v>197</v>
       </c>
       <c r="B60" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E60">
         <f t="shared" si="6"/>
@@ -15366,7 +15414,7 @@
         <v>197</v>
       </c>
       <c r="B61" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E61">
         <f t="shared" si="6"/>
@@ -15379,10 +15427,10 @@
     </row>
     <row r="62" spans="1:7">
       <c r="A62" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B62" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="E62">
         <f t="shared" si="6"/>
@@ -15398,10 +15446,10 @@
         <v>200</v>
       </c>
       <c r="B63" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E63">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="E63:E68" si="7">D63/1000</f>
         <v>0</v>
       </c>
       <c r="G63">
@@ -15414,10 +15462,10 @@
         <v>200</v>
       </c>
       <c r="B64" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E64">
-        <f t="shared" ref="E64:E69" si="7">D64/1000</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G64">
@@ -15430,7 +15478,7 @@
         <v>200</v>
       </c>
       <c r="B65" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E65">
         <f t="shared" si="7"/>
@@ -15446,7 +15494,7 @@
         <v>200</v>
       </c>
       <c r="B66" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E66">
         <f t="shared" si="7"/>
@@ -15462,7 +15510,7 @@
         <v>200</v>
       </c>
       <c r="B67" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="E67">
         <f t="shared" si="7"/>
@@ -15478,7 +15526,7 @@
         <v>200</v>
       </c>
       <c r="B68" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="E68">
         <f t="shared" si="7"/>
@@ -15491,18 +15539,27 @@
     </row>
     <row r="69" spans="1:9">
       <c r="A69" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="B69" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="E69">
-        <f t="shared" si="7"/>
-        <v>0</v>
+        <f>D69/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F69">
+        <v>6277</v>
       </c>
       <c r="G69">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>10101.855413271598</v>
+      </c>
+      <c r="H69" t="s">
+        <v>219</v>
+      </c>
+      <c r="I69" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -15510,24 +15567,24 @@
         <v>189</v>
       </c>
       <c r="B70" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E70">
-        <f>D70/1000</f>
+        <f t="shared" ref="E70:E80" si="8">D70/1000</f>
         <v>0</v>
       </c>
       <c r="F70">
-        <v>6277</v>
+        <v>4581</v>
       </c>
       <c r="G70">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10101.855413271598</v>
+        <v>7372.4071448458171</v>
       </c>
       <c r="H70" t="s">
         <v>219</v>
       </c>
       <c r="I70" t="s">
-        <v>240</v>
+        <v>220</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -15535,24 +15592,24 @@
         <v>189</v>
       </c>
       <c r="B71" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E71">
-        <f t="shared" ref="E71:E81" si="8">D71/1000</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F71">
-        <v>4581</v>
+        <v>3668</v>
       </c>
       <c r="G71">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7372.4071448458171</v>
+        <v>5903.0756182699097</v>
       </c>
       <c r="H71" t="s">
         <v>219</v>
       </c>
       <c r="I71" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -15560,24 +15617,24 @@
         <v>189</v>
       </c>
       <c r="B72" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E72">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F72">
-        <v>3668</v>
+        <v>4452</v>
       </c>
       <c r="G72">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5903.0756182699097</v>
+        <v>7164.8017046176765</v>
       </c>
       <c r="H72" t="s">
         <v>219</v>
       </c>
       <c r="I72" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -15585,24 +15642,24 @@
         <v>189</v>
       </c>
       <c r="B73" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E73">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F73">
-        <v>4452</v>
+        <v>4327</v>
       </c>
       <c r="G73">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7164.8017046176765</v>
+        <v>6963.6336423811072</v>
       </c>
       <c r="H73" t="s">
         <v>219</v>
       </c>
       <c r="I73" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -15610,24 +15667,24 @@
         <v>189</v>
       </c>
       <c r="B74" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E74">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F74">
-        <v>4327</v>
+        <v>7211</v>
       </c>
       <c r="G74">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6963.6336423811072</v>
+        <v>11604.98317430325</v>
       </c>
       <c r="H74" t="s">
         <v>219</v>
       </c>
       <c r="I74" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -15635,24 +15692,24 @@
         <v>189</v>
       </c>
       <c r="B75" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E75">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F75">
-        <v>7211</v>
+        <v>6346</v>
       </c>
       <c r="G75">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11604.98317430325</v>
+        <v>10212.900183626185</v>
       </c>
       <c r="H75" t="s">
         <v>219</v>
       </c>
       <c r="I75" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -15660,24 +15717,24 @@
         <v>189</v>
       </c>
       <c r="B76" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E76">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F76">
-        <v>6346</v>
+        <v>7020</v>
       </c>
       <c r="G76">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10212.900183626185</v>
+        <v>11297.598375205771</v>
       </c>
       <c r="H76" t="s">
         <v>219</v>
       </c>
       <c r="I76" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -15685,24 +15742,24 @@
         <v>189</v>
       </c>
       <c r="B77" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E77">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F77">
-        <v>7020</v>
+        <v>5266</v>
       </c>
       <c r="G77">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11297.598375205771</v>
+        <v>8474.8081259022201</v>
       </c>
       <c r="H77" t="s">
         <v>219</v>
       </c>
       <c r="I77" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -15710,24 +15767,24 @@
         <v>189</v>
       </c>
       <c r="B78" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E78">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F78">
-        <v>5266</v>
+        <v>4657</v>
       </c>
       <c r="G78">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8474.8081259022201</v>
+        <v>7494.7173266856516</v>
       </c>
       <c r="H78" t="s">
         <v>219</v>
       </c>
       <c r="I78" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -15735,24 +15792,24 @@
         <v>189</v>
       </c>
       <c r="B79" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E79">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F79">
-        <v>4657</v>
+        <v>3667</v>
       </c>
       <c r="G79">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7494.7173266856516</v>
+        <v>5901.4662737720173</v>
       </c>
       <c r="H79" t="s">
         <v>219</v>
       </c>
       <c r="I79" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -15760,24 +15817,24 @@
         <v>189</v>
       </c>
       <c r="B80" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E80">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F80">
-        <v>3667</v>
+        <v>6091</v>
       </c>
       <c r="G80">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5901.4662737720173</v>
+        <v>9802.5173366635827</v>
       </c>
       <c r="H80" t="s">
         <v>219</v>
       </c>
       <c r="I80" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -15785,24 +15842,24 @@
         <v>189</v>
       </c>
       <c r="B81" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="E81">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="E81:E85" si="9">D81/1000</f>
         <v>0</v>
       </c>
       <c r="F81">
-        <v>6091</v>
+        <v>7423</v>
       </c>
       <c r="G81">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9802.5173366635827</v>
+        <v>11946.164207856473</v>
       </c>
       <c r="H81" t="s">
         <v>219</v>
       </c>
       <c r="I81" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -15810,10 +15867,10 @@
         <v>189</v>
       </c>
       <c r="B82" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E82">
-        <f t="shared" ref="E82:E86" si="9">D82/1000</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F82">
@@ -15827,7 +15884,7 @@
         <v>219</v>
       </c>
       <c r="I82" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -15835,24 +15892,24 @@
         <v>189</v>
       </c>
       <c r="B83" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E83">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F83">
-        <v>7423</v>
+        <v>6540</v>
       </c>
       <c r="G83">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11946.164207856473</v>
+        <v>10525.113016217341</v>
       </c>
       <c r="H83" t="s">
         <v>219</v>
       </c>
       <c r="I83" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -15860,24 +15917,24 @@
         <v>189</v>
       </c>
       <c r="B84" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E84">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F84">
-        <v>6540</v>
+        <v>6078</v>
       </c>
       <c r="G84">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10525.113016217341</v>
+        <v>9781.5958581909799</v>
       </c>
       <c r="H84" t="s">
         <v>219</v>
       </c>
       <c r="I84" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="85" spans="1:9">
@@ -15885,49 +15942,46 @@
         <v>189</v>
       </c>
       <c r="B85" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E85">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F85">
-        <v>6078</v>
+        <v>7363</v>
       </c>
       <c r="G85">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9781.5958581909799</v>
+        <v>11849.603537982919</v>
       </c>
       <c r="H85" t="s">
         <v>219</v>
       </c>
       <c r="I85" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="86" spans="1:9">
       <c r="A86" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B86" t="s">
-        <v>234</v>
+        <v>206</v>
       </c>
       <c r="E86">
-        <f t="shared" si="9"/>
+        <f>D86/1000</f>
         <v>0</v>
       </c>
       <c r="F86">
-        <v>7363</v>
+        <v>4986</v>
       </c>
       <c r="G86">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11849.603537982919</v>
-      </c>
-      <c r="H86" t="s">
-        <v>219</v>
+        <v>8024.1916664923037</v>
       </c>
       <c r="I86" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="87" spans="1:9">
@@ -15935,21 +15989,21 @@
         <v>184</v>
       </c>
       <c r="B87" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E87">
-        <f>D87/1000</f>
+        <f t="shared" ref="E87:E102" si="10">D87/1000</f>
         <v>0</v>
       </c>
       <c r="F87">
-        <v>4986</v>
+        <v>4815</v>
       </c>
       <c r="G87">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8024.1916664923037</v>
+        <v>7748.9937573526759</v>
       </c>
       <c r="I87" t="s">
-        <v>240</v>
+        <v>220</v>
       </c>
     </row>
     <row r="88" spans="1:9">
@@ -15957,21 +16011,21 @@
         <v>184</v>
       </c>
       <c r="B88" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E88">
-        <f t="shared" ref="E88:E103" si="10">D88/1000</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F88">
-        <v>4815</v>
+        <v>6255</v>
       </c>
       <c r="G88">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7748.9937573526759</v>
+        <v>10066.449834317962</v>
       </c>
       <c r="I88" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="89" spans="1:9">
@@ -15979,21 +16033,21 @@
         <v>184</v>
       </c>
       <c r="B89" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E89">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F89">
-        <v>6255</v>
+        <v>5637</v>
       </c>
       <c r="G89">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10066.449834317962</v>
+        <v>9071.8749346203604</v>
       </c>
       <c r="I89" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -16001,21 +16055,21 @@
         <v>184</v>
       </c>
       <c r="B90" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E90">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F90">
-        <v>5637</v>
+        <v>6380</v>
       </c>
       <c r="G90">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9071.8749346203604</v>
+        <v>10267.617896554533</v>
       </c>
       <c r="I90" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="91" spans="1:9">
@@ -16023,21 +16077,21 @@
         <v>184</v>
       </c>
       <c r="B91" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E91">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F91">
-        <v>6380</v>
+        <v>5634</v>
       </c>
       <c r="G91">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10267.617896554533</v>
+        <v>9067.0469011266832</v>
       </c>
       <c r="I91" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="92" spans="1:9">
@@ -16045,21 +16099,21 @@
         <v>184</v>
       </c>
       <c r="B92" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E92">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F92">
-        <v>5634</v>
+        <v>5052</v>
       </c>
       <c r="G92">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9067.0469011266832</v>
+        <v>8130.4084033532126</v>
       </c>
       <c r="I92" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="93" spans="1:9">
@@ -16067,21 +16121,21 @@
         <v>184</v>
       </c>
       <c r="B93" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E93">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F93">
-        <v>5052</v>
+        <v>5443</v>
       </c>
       <c r="G93">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8130.4084033532126</v>
+        <v>8759.6621020292041</v>
       </c>
       <c r="I93" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="94" spans="1:9">
@@ -16089,21 +16143,21 @@
         <v>184</v>
       </c>
       <c r="B94" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E94">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F94">
-        <v>5443</v>
+        <v>4565</v>
       </c>
       <c r="G94">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8759.6621020292041</v>
+        <v>7346.6576328795363</v>
       </c>
       <c r="I94" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="95" spans="1:9">
@@ -16111,21 +16165,21 @@
         <v>184</v>
       </c>
       <c r="B95" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E95">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F95">
-        <v>4565</v>
+        <v>4786</v>
       </c>
       <c r="G95">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7346.6576328795363</v>
+        <v>7702.3227669137923</v>
       </c>
       <c r="I95" t="s">
-        <v>227</v>
+        <v>243</v>
       </c>
     </row>
     <row r="96" spans="1:9">
@@ -16133,21 +16187,21 @@
         <v>184</v>
       </c>
       <c r="B96" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E96">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F96">
-        <v>4786</v>
+        <v>6409</v>
       </c>
       <c r="G96">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7702.3227669137923</v>
+        <v>10314.288886993416</v>
       </c>
       <c r="I96" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="97" spans="1:9">
@@ -16155,21 +16209,21 @@
         <v>184</v>
       </c>
       <c r="B97" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E97">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F97">
-        <v>6409</v>
+        <v>4666</v>
       </c>
       <c r="G97">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10314.288886993416</v>
+        <v>7509.2014271666849</v>
       </c>
       <c r="I97" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
     </row>
     <row r="98" spans="1:9">
@@ -16177,21 +16231,21 @@
         <v>184</v>
       </c>
       <c r="B98" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="E98">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F98">
-        <v>4666</v>
+        <v>5846</v>
       </c>
       <c r="G98">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7509.2014271666849</v>
+        <v>9408.227934679906</v>
       </c>
       <c r="I98" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
     </row>
     <row r="99" spans="1:9">
@@ -16199,7 +16253,7 @@
         <v>184</v>
       </c>
       <c r="B99" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E99">
         <f t="shared" si="10"/>
@@ -16213,7 +16267,7 @@
         <v>9408.227934679906</v>
       </c>
       <c r="I99" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="100" spans="1:9">
@@ -16221,21 +16275,21 @@
         <v>184</v>
       </c>
       <c r="B100" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E100">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F100">
-        <v>5846</v>
+        <v>5215</v>
       </c>
       <c r="G100">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9408.227934679906</v>
+        <v>8392.7315565096997</v>
       </c>
       <c r="I100" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="101" spans="1:9">
@@ -16243,21 +16297,21 @@
         <v>184</v>
       </c>
       <c r="B101" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E101">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F101">
-        <v>5215</v>
+        <v>4564</v>
       </c>
       <c r="G101">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8392.7315565096997</v>
+        <v>7345.0482883816439</v>
       </c>
       <c r="I101" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="102" spans="1:9">
@@ -16265,43 +16319,43 @@
         <v>184</v>
       </c>
       <c r="B102" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E102">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F102">
-        <v>4564</v>
+        <v>5786</v>
       </c>
       <c r="G102">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7345.0482883816439</v>
+        <v>9311.6672648063523</v>
       </c>
       <c r="I102" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="103" spans="1:9">
       <c r="A103" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B103" t="s">
-        <v>234</v>
+        <v>206</v>
       </c>
       <c r="E103">
-        <f t="shared" si="10"/>
+        <f>D103/1000</f>
         <v>0</v>
       </c>
       <c r="F103">
-        <v>5786</v>
+        <v>3985</v>
       </c>
       <c r="G103">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9311.6672648063523</v>
+        <v>6413.2378241018514</v>
       </c>
       <c r="I103" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="104" spans="1:9">
@@ -16309,21 +16363,21 @@
         <v>187</v>
       </c>
       <c r="B104" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E104">
-        <f>D104/1000</f>
+        <f t="shared" ref="E104:E119" si="11">D104/1000</f>
         <v>0</v>
       </c>
       <c r="F104">
-        <v>3985</v>
+        <v>4101</v>
       </c>
       <c r="G104">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6413.2378241018514</v>
+        <v>6599.9217858573884</v>
       </c>
       <c r="I104" t="s">
-        <v>240</v>
+        <v>220</v>
       </c>
     </row>
     <row r="105" spans="1:9">
@@ -16331,21 +16385,21 @@
         <v>187</v>
       </c>
       <c r="B105" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E105">
-        <f t="shared" ref="E105:E120" si="11">D105/1000</f>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F105">
-        <v>4101</v>
+        <v>4898</v>
       </c>
       <c r="G105">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6599.9217858573884</v>
+        <v>7882.5693506777588</v>
       </c>
       <c r="I105" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="106" spans="1:9">
@@ -16353,21 +16407,21 @@
         <v>187</v>
       </c>
       <c r="B106" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E106">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F106">
-        <v>4898</v>
+        <v>4280</v>
       </c>
       <c r="G106">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7882.5693506777588</v>
+        <v>6887.9944509801562</v>
       </c>
       <c r="I106" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="107" spans="1:9">
@@ -16375,21 +16429,21 @@
         <v>187</v>
       </c>
       <c r="B107" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E107">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F107">
-        <v>4280</v>
+        <v>5023</v>
       </c>
       <c r="G107">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6887.9944509801562</v>
+        <v>8083.7374129143291</v>
       </c>
       <c r="I107" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="108" spans="1:9">
@@ -16397,21 +16451,21 @@
         <v>187</v>
       </c>
       <c r="B108" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E108">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F108">
-        <v>5023</v>
+        <v>4823</v>
       </c>
       <c r="G108">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8083.7374129143291</v>
+        <v>7761.8685133358167</v>
       </c>
       <c r="I108" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="109" spans="1:9">
@@ -16419,21 +16473,21 @@
         <v>187</v>
       </c>
       <c r="B109" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E109">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F109">
-        <v>4823</v>
+        <v>4051</v>
       </c>
       <c r="G109">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7761.8685133358167</v>
+        <v>6519.4545609627603</v>
       </c>
       <c r="I109" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="110" spans="1:9">
@@ -16441,21 +16495,21 @@
         <v>187</v>
       </c>
       <c r="B110" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E110">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F110">
-        <v>4051</v>
+        <v>4632</v>
       </c>
       <c r="G110">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6519.4545609627603</v>
+        <v>7454.4837142383376</v>
       </c>
       <c r="I110" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="111" spans="1:9">
@@ -16463,21 +16517,21 @@
         <v>187</v>
       </c>
       <c r="B111" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E111">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F111">
-        <v>4632</v>
+        <v>3299</v>
       </c>
       <c r="G111">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7454.4837142383376</v>
+        <v>5309.2274985475551</v>
       </c>
       <c r="I111" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="112" spans="1:9">
@@ -16485,21 +16539,21 @@
         <v>187</v>
       </c>
       <c r="B112" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E112">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F112">
-        <v>3299</v>
+        <v>3366</v>
       </c>
       <c r="G112">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5309.2274985475551</v>
+        <v>5417.0535799063564</v>
       </c>
       <c r="I112" t="s">
-        <v>227</v>
+        <v>256</v>
       </c>
     </row>
     <row r="113" spans="1:9">
@@ -16507,21 +16561,21 @@
         <v>187</v>
       </c>
       <c r="B113" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E113">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F113">
-        <v>3645</v>
+        <v>5052</v>
       </c>
       <c r="G113">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5866.0606948183813</v>
+        <v>8130.4084033532126</v>
       </c>
       <c r="I113" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
     </row>
     <row r="114" spans="1:9">
@@ -16529,21 +16583,21 @@
         <v>187</v>
       </c>
       <c r="B114" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E114">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F114">
-        <v>5052</v>
+        <v>3733</v>
       </c>
       <c r="G114">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8130.4084033532126</v>
+        <v>6007.6830106329262</v>
       </c>
       <c r="I114" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
     </row>
     <row r="115" spans="1:9">
@@ -16551,21 +16605,21 @@
         <v>187</v>
       </c>
       <c r="B115" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="E115">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F115">
-        <v>3733</v>
+        <v>5035</v>
       </c>
       <c r="G115">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6007.6830106329262</v>
+        <v>8103.0495468890394</v>
       </c>
       <c r="I115" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
     </row>
     <row r="116" spans="1:9">
@@ -16573,7 +16627,7 @@
         <v>187</v>
       </c>
       <c r="B116" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E116">
         <f t="shared" si="11"/>
@@ -16587,7 +16641,7 @@
         <v>8103.0495468890394</v>
       </c>
       <c r="I116" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="117" spans="1:9">
@@ -16595,21 +16649,21 @@
         <v>187</v>
       </c>
       <c r="B117" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E117">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F117">
-        <v>5035</v>
+        <v>4248</v>
       </c>
       <c r="G117">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8103.0495468890394</v>
+        <v>6836.4954270475946</v>
       </c>
       <c r="I117" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="118" spans="1:9">
@@ -16617,21 +16671,21 @@
         <v>187</v>
       </c>
       <c r="B118" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E118">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F118">
-        <v>4248</v>
+        <v>3599</v>
       </c>
       <c r="G118">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6836.4954270475946</v>
+        <v>5792.0308479153236</v>
       </c>
       <c r="I118" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="119" spans="1:9">
@@ -16639,43 +16693,46 @@
         <v>187</v>
       </c>
       <c r="B119" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E119">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F119">
-        <v>3599</v>
+        <v>4975</v>
       </c>
       <c r="G119">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5792.0308479153236</v>
+        <v>8006.4888770154857</v>
       </c>
       <c r="I119" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="120" spans="1:9">
       <c r="A120" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B120" t="s">
-        <v>234</v>
+        <v>206</v>
       </c>
       <c r="E120">
-        <f t="shared" si="11"/>
+        <f>D120/1000</f>
         <v>0</v>
       </c>
       <c r="F120">
-        <v>4975</v>
+        <v>6210</v>
       </c>
       <c r="G120">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8006.4888770154857</v>
+        <v>9994.0293319127977</v>
+      </c>
+      <c r="H120" t="s">
+        <v>219</v>
       </c>
       <c r="I120" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="121" spans="1:9">
@@ -16683,24 +16740,24 @@
         <v>188</v>
       </c>
       <c r="B121" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E121">
-        <f>D121/1000</f>
+        <f t="shared" ref="E121:E136" si="12">D121/1000</f>
         <v>0</v>
       </c>
       <c r="F121">
-        <v>6210</v>
-      </c>
-      <c r="G121" s="13">
+        <v>4514</v>
+      </c>
+      <c r="G121">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9994.0293319127977</v>
-      </c>
-      <c r="H121" s="13" t="s">
+        <v>7264.5810634870159</v>
+      </c>
+      <c r="H121" t="s">
         <v>219</v>
       </c>
       <c r="I121" t="s">
-        <v>240</v>
+        <v>220</v>
       </c>
     </row>
     <row r="122" spans="1:9">
@@ -16708,24 +16765,24 @@
         <v>188</v>
       </c>
       <c r="B122" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E122">
-        <f t="shared" ref="E122:E137" si="12">D122/1000</f>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F122">
-        <v>4514</v>
-      </c>
-      <c r="G122" s="13">
+        <v>3601</v>
+      </c>
+      <c r="G122">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7264.5810634870159</v>
-      </c>
-      <c r="H122" s="13" t="s">
+        <v>5795.2495369111084</v>
+      </c>
+      <c r="H122" t="s">
         <v>219</v>
       </c>
       <c r="I122" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="123" spans="1:9">
@@ -16733,24 +16790,24 @@
         <v>188</v>
       </c>
       <c r="B123" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E123">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F123">
-        <v>3601</v>
-      </c>
-      <c r="G123" s="13">
+        <v>4385</v>
+      </c>
+      <c r="G123">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5795.2495369111084</v>
-      </c>
-      <c r="H123" s="13" t="s">
+        <v>7056.9756232588752</v>
+      </c>
+      <c r="H123" t="s">
         <v>219</v>
       </c>
       <c r="I123" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="124" spans="1:9">
@@ -16758,24 +16815,24 @@
         <v>188</v>
       </c>
       <c r="B124" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E124">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F124">
-        <v>4385</v>
-      </c>
-      <c r="G124" s="13">
+        <v>4260</v>
+      </c>
+      <c r="G124">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7056.9756232588752</v>
-      </c>
-      <c r="H124" s="13" t="s">
+        <v>6855.807561022305</v>
+      </c>
+      <c r="H124" t="s">
         <v>219</v>
       </c>
       <c r="I124" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="125" spans="1:9">
@@ -16783,24 +16840,24 @@
         <v>188</v>
       </c>
       <c r="B125" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E125">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F125">
-        <v>4260</v>
-      </c>
-      <c r="G125" s="13">
+        <v>7144</v>
+      </c>
+      <c r="G125">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6855.807561022305</v>
-      </c>
-      <c r="H125" s="13" t="s">
+        <v>11497.157092944448</v>
+      </c>
+      <c r="H125" t="s">
         <v>219</v>
       </c>
       <c r="I125" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="126" spans="1:9">
@@ -16808,24 +16865,24 @@
         <v>188</v>
       </c>
       <c r="B126" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E126">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F126">
-        <v>7144</v>
-      </c>
-      <c r="G126" s="13">
+        <v>6276</v>
+      </c>
+      <c r="G126">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11497.157092944448</v>
-      </c>
-      <c r="H126" s="13" t="s">
+        <v>10100.246068773706</v>
+      </c>
+      <c r="H126" t="s">
         <v>219</v>
       </c>
       <c r="I126" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="127" spans="1:9">
@@ -16833,24 +16890,24 @@
         <v>188</v>
       </c>
       <c r="B127" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E127">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F127">
-        <v>6276</v>
-      </c>
-      <c r="G127" s="13">
+        <v>6953</v>
+      </c>
+      <c r="G127">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10100.246068773706</v>
-      </c>
-      <c r="H127" s="13" t="s">
+        <v>11189.772293846969</v>
+      </c>
+      <c r="H127" t="s">
         <v>219</v>
       </c>
       <c r="I127" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="128" spans="1:9">
@@ -16858,24 +16915,24 @@
         <v>188</v>
       </c>
       <c r="B128" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E128">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F128">
-        <v>6953</v>
-      </c>
-      <c r="G128" s="13">
+        <v>5199</v>
+      </c>
+      <c r="G128">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11189.772293846969</v>
-      </c>
-      <c r="H128" s="13" t="s">
+        <v>8366.9820445434198</v>
+      </c>
+      <c r="H128" t="s">
         <v>219</v>
       </c>
       <c r="I128" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="129" spans="1:9">
@@ -16883,24 +16940,24 @@
         <v>188</v>
       </c>
       <c r="B129" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E129">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F129">
-        <v>5199</v>
-      </c>
-      <c r="G129" s="13">
+        <v>4590</v>
+      </c>
+      <c r="G129">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8366.9820445434198</v>
-      </c>
-      <c r="H129" s="13" t="s">
+        <v>7386.8912453268504</v>
+      </c>
+      <c r="H129" t="s">
         <v>219</v>
       </c>
       <c r="I129" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="130" spans="1:9">
@@ -16908,24 +16965,24 @@
         <v>188</v>
       </c>
       <c r="B130" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E130">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F130">
-        <v>4590</v>
-      </c>
-      <c r="G130" s="13">
+        <v>3600</v>
+      </c>
+      <c r="G130">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7386.8912453268504</v>
-      </c>
-      <c r="H130" s="13" t="s">
+        <v>5793.640192413216</v>
+      </c>
+      <c r="H130" t="s">
         <v>219</v>
       </c>
       <c r="I130" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="131" spans="1:9">
@@ -16933,24 +16990,24 @@
         <v>188</v>
       </c>
       <c r="B131" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E131">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F131">
-        <v>3600</v>
-      </c>
-      <c r="G131" s="13">
+        <v>6024</v>
+      </c>
+      <c r="G131">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5793.640192413216</v>
-      </c>
-      <c r="H131" s="13" t="s">
+        <v>9694.6912553047805</v>
+      </c>
+      <c r="H131" t="s">
         <v>219</v>
       </c>
       <c r="I131" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
     </row>
     <row r="132" spans="1:9">
@@ -16958,24 +17015,24 @@
         <v>188</v>
       </c>
       <c r="B132" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="E132">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F132">
-        <v>6024</v>
-      </c>
-      <c r="G132" s="13">
+        <v>7356</v>
+      </c>
+      <c r="G132">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9694.6912553047805</v>
-      </c>
-      <c r="H132" s="13" t="s">
+        <v>11838.338126497671</v>
+      </c>
+      <c r="H132" t="s">
         <v>219</v>
       </c>
       <c r="I132" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
     </row>
     <row r="133" spans="1:9">
@@ -16983,7 +17040,7 @@
         <v>188</v>
       </c>
       <c r="B133" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E133">
         <f t="shared" si="12"/>
@@ -16992,15 +17049,15 @@
       <c r="F133">
         <v>7356</v>
       </c>
-      <c r="G133" s="13">
+      <c r="G133">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>11838.338126497671</v>
       </c>
-      <c r="H133" s="13" t="s">
+      <c r="H133" t="s">
         <v>219</v>
       </c>
       <c r="I133" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="134" spans="1:9">
@@ -17008,24 +17065,24 @@
         <v>188</v>
       </c>
       <c r="B134" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E134">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F134">
-        <v>7356</v>
-      </c>
-      <c r="G134" s="13">
+        <v>6473</v>
+      </c>
+      <c r="G134">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11838.338126497671</v>
-      </c>
-      <c r="H134" s="13" t="s">
+        <v>10417.286934858541</v>
+      </c>
+      <c r="H134" t="s">
         <v>219</v>
       </c>
       <c r="I134" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="135" spans="1:9">
@@ -17033,24 +17090,24 @@
         <v>188</v>
       </c>
       <c r="B135" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E135">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F135">
-        <v>6473</v>
-      </c>
-      <c r="G135" s="13">
+        <v>6011</v>
+      </c>
+      <c r="G135">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10417.286934858541</v>
-      </c>
-      <c r="H135" s="13" t="s">
+        <v>9673.7697768321777</v>
+      </c>
+      <c r="H135" t="s">
         <v>219</v>
       </c>
       <c r="I135" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="136" spans="1:9">
@@ -17058,48 +17115,414 @@
         <v>188</v>
       </c>
       <c r="B136" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="E136">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F136">
-        <v>6011</v>
-      </c>
-      <c r="G136" s="13">
+        <v>7296</v>
+      </c>
+      <c r="G136">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9673.7697768321777</v>
-      </c>
-      <c r="H136" s="13" t="s">
+        <v>11741.777456624117</v>
+      </c>
+      <c r="H136" t="s">
         <v>219</v>
       </c>
       <c r="I136" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="137" spans="1:9">
       <c r="A137" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B137" t="s">
-        <v>234</v>
+        <v>206</v>
       </c>
       <c r="E137">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="E137:E153" si="13">D137/1000</f>
         <v>0</v>
       </c>
       <c r="F137">
-        <v>7296</v>
+        <v>4348</v>
       </c>
       <c r="G137" s="13">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11741.777456624117</v>
-      </c>
-      <c r="H137" s="13" t="s">
-        <v>219</v>
-      </c>
+        <v>6997.4298768368508</v>
+      </c>
+      <c r="H137" s="13"/>
       <c r="I137" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9">
+      <c r="A138" t="s">
+        <v>190</v>
+      </c>
+      <c r="B138" t="s">
+        <v>207</v>
+      </c>
+      <c r="E138">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F138">
+        <v>4027</v>
+      </c>
+      <c r="G138" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6480.8302930133386</v>
+      </c>
+      <c r="H138" s="13"/>
+      <c r="I138" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9">
+      <c r="A139" t="s">
+        <v>190</v>
+      </c>
+      <c r="B139" t="s">
+        <v>208</v>
+      </c>
+      <c r="E139">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F139">
+        <v>4824</v>
+      </c>
+      <c r="G139" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7763.4778578337091</v>
+      </c>
+      <c r="H139" s="13"/>
+      <c r="I139" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9">
+      <c r="A140" t="s">
+        <v>190</v>
+      </c>
+      <c r="B140" t="s">
+        <v>209</v>
+      </c>
+      <c r="E140">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F140">
+        <v>4206</v>
+      </c>
+      <c r="G140" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6768.9029581361074</v>
+      </c>
+      <c r="H140" s="13"/>
+      <c r="I140" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9">
+      <c r="A141" t="s">
+        <v>190</v>
+      </c>
+      <c r="B141" t="s">
+        <v>210</v>
+      </c>
+      <c r="E141">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F141">
+        <v>4949</v>
+      </c>
+      <c r="G141" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7964.6459200702793</v>
+      </c>
+      <c r="H141" s="13"/>
+      <c r="I141" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9">
+      <c r="A142" t="s">
+        <v>190</v>
+      </c>
+      <c r="B142" t="s">
+        <v>211</v>
+      </c>
+      <c r="E142">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F142">
+        <v>5282</v>
+      </c>
+      <c r="G142" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8500.5576378685018</v>
+      </c>
+      <c r="H142" s="13"/>
+      <c r="I142" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9">
+      <c r="A143" t="s">
+        <v>190</v>
+      </c>
+      <c r="B143" t="s">
+        <v>212</v>
+      </c>
+      <c r="E143">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F143">
+        <v>4414</v>
+      </c>
+      <c r="G143" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7103.6466136977597</v>
+      </c>
+      <c r="H143" s="13"/>
+      <c r="I143" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9">
+      <c r="A144" t="s">
+        <v>190</v>
+      </c>
+      <c r="B144" t="s">
+        <v>213</v>
+      </c>
+      <c r="E144">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F144">
+        <v>5091</v>
+      </c>
+      <c r="G144" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8193.1728387710227</v>
+      </c>
+      <c r="H144" s="13"/>
+      <c r="I144" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9">
+      <c r="A145" t="s">
+        <v>190</v>
+      </c>
+      <c r="B145" t="s">
+        <v>214</v>
+      </c>
+      <c r="E145">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F145">
+        <v>3389</v>
+      </c>
+      <c r="G145" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5454.0685033578857</v>
+      </c>
+      <c r="H145" s="13"/>
+      <c r="I145" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9">
+      <c r="A146" t="s">
+        <v>190</v>
+      </c>
+      <c r="B146" t="s">
+        <v>215</v>
+      </c>
+      <c r="E146">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F146">
+        <v>3359</v>
+      </c>
+      <c r="G146" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5405.7881684211088</v>
+      </c>
+      <c r="H146" s="13"/>
+      <c r="I146" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9">
+      <c r="A147" t="s">
+        <v>190</v>
+      </c>
+      <c r="B147" t="s">
+        <v>216</v>
+      </c>
+      <c r="E147">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F147">
+        <v>4978</v>
+      </c>
+      <c r="G147" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8011.3169105091638</v>
+      </c>
+      <c r="H147" s="13"/>
+      <c r="I147" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9">
+      <c r="A148" t="s">
+        <v>190</v>
+      </c>
+      <c r="B148" t="s">
+        <v>217</v>
+      </c>
+      <c r="E148">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F148">
+        <v>4162</v>
+      </c>
+      <c r="G148" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6698.0918002288345</v>
+      </c>
+      <c r="H148" s="13"/>
+      <c r="I148" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9">
+      <c r="A149" t="s">
+        <v>190</v>
+      </c>
+      <c r="B149" t="s">
+        <v>230</v>
+      </c>
+      <c r="E149">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F149">
+        <v>5494</v>
+      </c>
+      <c r="G149" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8841.7386714217246</v>
+      </c>
+      <c r="H149" s="13"/>
+      <c r="I149" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9">
+      <c r="A150" t="s">
+        <v>190</v>
+      </c>
+      <c r="B150" t="s">
+        <v>231</v>
+      </c>
+      <c r="E150">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F150">
+        <v>5494</v>
+      </c>
+      <c r="G150" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8841.7386714217246</v>
+      </c>
+      <c r="H150" s="13"/>
+      <c r="I150" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9">
+      <c r="A151" t="s">
+        <v>190</v>
+      </c>
+      <c r="B151" t="s">
+        <v>232</v>
+      </c>
+      <c r="E151">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F151">
+        <v>4611</v>
+      </c>
+      <c r="G151" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7420.687479782594</v>
+      </c>
+      <c r="H151" s="13"/>
+      <c r="I151" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9">
+      <c r="A152" t="s">
+        <v>190</v>
+      </c>
+      <c r="B152" t="s">
+        <v>233</v>
+      </c>
+      <c r="E152">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F152">
+        <v>4149</v>
+      </c>
+      <c r="G152" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6677.1703217562308</v>
+      </c>
+      <c r="H152" s="13"/>
+      <c r="I152" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9">
+      <c r="A153" t="s">
+        <v>190</v>
+      </c>
+      <c r="B153" t="s">
+        <v>234</v>
+      </c>
+      <c r="E153">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+      <c r="F153">
+        <v>5434</v>
+      </c>
+      <c r="G153" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8745.1780015481709</v>
+      </c>
+      <c r="H153" s="13"/>
+      <c r="I153" t="s">
         <v>239</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add LNG transport distances from AU
from Darwin to the different regions
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F07001EF-28A2-421E-9DE8-4EC031747CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A646E4F-5121-428B-8DAB-A36538638524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1698" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1774" uniqueCount="260">
   <si>
     <t>Belgium</t>
   </si>
@@ -818,6 +818,12 @@
   </si>
   <si>
     <t>Mumbai</t>
+  </si>
+  <si>
+    <t>AU from Darwin</t>
+  </si>
+  <si>
+    <t>Quintero (Chile)</t>
   </si>
 </sst>
 </file>
@@ -1526,8 +1532,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I153" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
-  <autoFilter ref="A1:I153" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I170" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+  <autoFilter ref="A1:I170" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
     <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
@@ -14166,7 +14172,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M153"/>
+  <dimension ref="A1:M170"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="21.81640625" customWidth="1"/>
@@ -14332,6 +14338,9 @@
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
+      <c r="M7" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
@@ -15116,9 +15125,15 @@
         <f>D42/1000</f>
         <v>0</v>
       </c>
+      <c r="F42">
+        <v>8575</v>
+      </c>
       <c r="G42">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>13800.129069428702</v>
+      </c>
+      <c r="I42" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -15132,9 +15147,15 @@
         <f t="shared" ref="E43:E48" si="4">D43/1000</f>
         <v>0</v>
       </c>
+      <c r="F43">
+        <v>8554</v>
+      </c>
       <c r="G43">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>13766.332834972958</v>
+      </c>
+      <c r="I43" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -15148,9 +15169,15 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="F44">
+        <v>3175</v>
+      </c>
       <c r="G44">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>5109.6687808088782</v>
+      </c>
+      <c r="I44" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -15164,9 +15191,15 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="F45">
+        <v>3033</v>
+      </c>
       <c r="G45">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>4881.1418621081348</v>
+      </c>
+      <c r="I45" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -15180,9 +15213,15 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="F46">
+        <v>4180</v>
+      </c>
       <c r="G46">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>6727.0600011909009</v>
+      </c>
+      <c r="I46" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -15196,9 +15235,15 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="F47">
+        <v>2612</v>
+      </c>
       <c r="G47">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>4203.6078284953664</v>
+      </c>
+      <c r="I47" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -15212,9 +15257,15 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="F48">
+        <v>6655</v>
+      </c>
       <c r="G48">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>10710.187633474987</v>
+      </c>
+      <c r="I48" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -17149,11 +17200,10 @@
       <c r="F137">
         <v>4348</v>
       </c>
-      <c r="G137" s="13">
+      <c r="G137">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6997.4298768368508</v>
       </c>
-      <c r="H137" s="13"/>
       <c r="I137" t="s">
         <v>240</v>
       </c>
@@ -17172,11 +17222,10 @@
       <c r="F138">
         <v>4027</v>
       </c>
-      <c r="G138" s="13">
+      <c r="G138">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6480.8302930133386</v>
       </c>
-      <c r="H138" s="13"/>
       <c r="I138" t="s">
         <v>220</v>
       </c>
@@ -17195,11 +17244,10 @@
       <c r="F139">
         <v>4824</v>
       </c>
-      <c r="G139" s="13">
+      <c r="G139">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7763.4778578337091</v>
       </c>
-      <c r="H139" s="13"/>
       <c r="I139" t="s">
         <v>221</v>
       </c>
@@ -17218,11 +17266,10 @@
       <c r="F140">
         <v>4206</v>
       </c>
-      <c r="G140" s="13">
+      <c r="G140">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6768.9029581361074</v>
       </c>
-      <c r="H140" s="13"/>
       <c r="I140" t="s">
         <v>222</v>
       </c>
@@ -17241,11 +17288,10 @@
       <c r="F141">
         <v>4949</v>
       </c>
-      <c r="G141" s="13">
+      <c r="G141">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7964.6459200702793</v>
       </c>
-      <c r="H141" s="13"/>
       <c r="I141" t="s">
         <v>223</v>
       </c>
@@ -17264,11 +17310,10 @@
       <c r="F142">
         <v>5282</v>
       </c>
-      <c r="G142" s="13">
+      <c r="G142">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8500.5576378685018</v>
       </c>
-      <c r="H142" s="13"/>
       <c r="I142" t="s">
         <v>224</v>
       </c>
@@ -17287,11 +17332,10 @@
       <c r="F143">
         <v>4414</v>
       </c>
-      <c r="G143" s="13">
+      <c r="G143">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7103.6466136977597</v>
       </c>
-      <c r="H143" s="13"/>
       <c r="I143" t="s">
         <v>225</v>
       </c>
@@ -17310,11 +17354,10 @@
       <c r="F144">
         <v>5091</v>
       </c>
-      <c r="G144" s="13">
+      <c r="G144">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8193.1728387710227</v>
       </c>
-      <c r="H144" s="13"/>
       <c r="I144" t="s">
         <v>226</v>
       </c>
@@ -17333,11 +17376,10 @@
       <c r="F145">
         <v>3389</v>
       </c>
-      <c r="G145" s="13">
+      <c r="G145">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5454.0685033578857</v>
       </c>
-      <c r="H145" s="13"/>
       <c r="I145" t="s">
         <v>227</v>
       </c>
@@ -17356,11 +17398,10 @@
       <c r="F146">
         <v>3359</v>
       </c>
-      <c r="G146" s="13">
+      <c r="G146">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5405.7881684211088</v>
       </c>
-      <c r="H146" s="13"/>
       <c r="I146" t="s">
         <v>256</v>
       </c>
@@ -17379,11 +17420,10 @@
       <c r="F147">
         <v>4978</v>
       </c>
-      <c r="G147" s="13">
+      <c r="G147">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8011.3169105091638</v>
       </c>
-      <c r="H147" s="13"/>
       <c r="I147" t="s">
         <v>229</v>
       </c>
@@ -17402,11 +17442,10 @@
       <c r="F148">
         <v>4162</v>
       </c>
-      <c r="G148" s="13">
+      <c r="G148">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6698.0918002288345</v>
       </c>
-      <c r="H148" s="13"/>
       <c r="I148" t="s">
         <v>244</v>
       </c>
@@ -17425,11 +17464,10 @@
       <c r="F149">
         <v>5494</v>
       </c>
-      <c r="G149" s="13">
+      <c r="G149">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8841.7386714217246</v>
       </c>
-      <c r="H149" s="13"/>
       <c r="I149" t="s">
         <v>235</v>
       </c>
@@ -17448,11 +17486,10 @@
       <c r="F150">
         <v>5494</v>
       </c>
-      <c r="G150" s="13">
+      <c r="G150">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8841.7386714217246</v>
       </c>
-      <c r="H150" s="13"/>
       <c r="I150" t="s">
         <v>236</v>
       </c>
@@ -17471,11 +17508,10 @@
       <c r="F151">
         <v>4611</v>
       </c>
-      <c r="G151" s="13">
+      <c r="G151">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7420.687479782594</v>
       </c>
-      <c r="H151" s="13"/>
       <c r="I151" t="s">
         <v>237</v>
       </c>
@@ -17494,11 +17530,10 @@
       <c r="F152">
         <v>4149</v>
       </c>
-      <c r="G152" s="13">
+      <c r="G152">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6677.1703217562308</v>
       </c>
-      <c r="H152" s="13"/>
       <c r="I152" t="s">
         <v>238</v>
       </c>
@@ -17517,12 +17552,436 @@
       <c r="F153">
         <v>5434</v>
       </c>
-      <c r="G153" s="13">
+      <c r="G153">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8745.1780015481709</v>
       </c>
-      <c r="H153" s="13"/>
       <c r="I153" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9">
+      <c r="A154" t="s">
+        <v>191</v>
+      </c>
+      <c r="B154" t="s">
+        <v>206</v>
+      </c>
+      <c r="E154">
+        <f>D154/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F154">
+        <v>9950</v>
+      </c>
+      <c r="G154" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>16012.977754030971</v>
+      </c>
+      <c r="H154" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I154" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9">
+      <c r="A155" t="s">
+        <v>191</v>
+      </c>
+      <c r="B155" t="s">
+        <v>207</v>
+      </c>
+      <c r="E155">
+        <f t="shared" ref="E155:E170" si="14">D155/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F155">
+        <v>8254</v>
+      </c>
+      <c r="G155" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>13283.52948560519</v>
+      </c>
+      <c r="H155" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I155" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9">
+      <c r="A156" t="s">
+        <v>191</v>
+      </c>
+      <c r="B156" t="s">
+        <v>208</v>
+      </c>
+      <c r="E156">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F156">
+        <v>7341</v>
+      </c>
+      <c r="G156" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11814.197959029283</v>
+      </c>
+      <c r="H156" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I156" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9">
+      <c r="A157" t="s">
+        <v>191</v>
+      </c>
+      <c r="B157" t="s">
+        <v>209</v>
+      </c>
+      <c r="E157">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F157">
+        <v>8125</v>
+      </c>
+      <c r="G157" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>13075.924045377049</v>
+      </c>
+      <c r="H157" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I157" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="158" spans="1:9">
+      <c r="A158" t="s">
+        <v>191</v>
+      </c>
+      <c r="B158" t="s">
+        <v>210</v>
+      </c>
+      <c r="E158">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F158">
+        <v>8000</v>
+      </c>
+      <c r="G158" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>12874.75598314048</v>
+      </c>
+      <c r="H158" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I158" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="159" spans="1:9">
+      <c r="A159" t="s">
+        <v>191</v>
+      </c>
+      <c r="B159" t="s">
+        <v>211</v>
+      </c>
+      <c r="E159">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F159">
+        <v>10884</v>
+      </c>
+      <c r="G159" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>17516.105515062623</v>
+      </c>
+      <c r="H159" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I159" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="160" spans="1:9">
+      <c r="A160" t="s">
+        <v>191</v>
+      </c>
+      <c r="B160" t="s">
+        <v>212</v>
+      </c>
+      <c r="E160">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F160">
+        <v>10016</v>
+      </c>
+      <c r="G160" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>16119.194490891881</v>
+      </c>
+      <c r="H160" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I160" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="161" spans="1:9">
+      <c r="A161" t="s">
+        <v>191</v>
+      </c>
+      <c r="B161" t="s">
+        <v>213</v>
+      </c>
+      <c r="E161">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F161">
+        <v>10693</v>
+      </c>
+      <c r="G161" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>17208.720715965144</v>
+      </c>
+      <c r="H161" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I161" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="162" spans="1:9">
+      <c r="A162" t="s">
+        <v>191</v>
+      </c>
+      <c r="B162" t="s">
+        <v>214</v>
+      </c>
+      <c r="E162">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F162">
+        <v>8939</v>
+      </c>
+      <c r="G162" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>14385.930466661594</v>
+      </c>
+      <c r="H162" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I162" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9">
+      <c r="A163" t="s">
+        <v>191</v>
+      </c>
+      <c r="B163" t="s">
+        <v>215</v>
+      </c>
+      <c r="E163">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F163">
+        <v>8330</v>
+      </c>
+      <c r="G163" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>13405.839667445025</v>
+      </c>
+      <c r="H163" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I163" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="164" spans="1:9">
+      <c r="A164" t="s">
+        <v>191</v>
+      </c>
+      <c r="B164" t="s">
+        <v>216</v>
+      </c>
+      <c r="E164">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F164">
+        <v>7340</v>
+      </c>
+      <c r="G164" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11812.588614531391</v>
+      </c>
+      <c r="H164" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I164" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9">
+      <c r="A165" t="s">
+        <v>191</v>
+      </c>
+      <c r="B165" t="s">
+        <v>217</v>
+      </c>
+      <c r="E165">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F165">
+        <v>9764</v>
+      </c>
+      <c r="G165" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>15713.639677422956</v>
+      </c>
+      <c r="H165" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I165" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9">
+      <c r="A166" t="s">
+        <v>191</v>
+      </c>
+      <c r="B166" t="s">
+        <v>230</v>
+      </c>
+      <c r="E166">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F166">
+        <v>11096</v>
+      </c>
+      <c r="G166" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>17857.286548615844</v>
+      </c>
+      <c r="H166" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I166" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9">
+      <c r="A167" t="s">
+        <v>191</v>
+      </c>
+      <c r="B167" t="s">
+        <v>231</v>
+      </c>
+      <c r="E167">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F167">
+        <v>11096</v>
+      </c>
+      <c r="G167" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>17857.286548615844</v>
+      </c>
+      <c r="H167" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I167" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9">
+      <c r="A168" t="s">
+        <v>191</v>
+      </c>
+      <c r="B168" t="s">
+        <v>232</v>
+      </c>
+      <c r="E168">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F168">
+        <v>10213</v>
+      </c>
+      <c r="G168" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>16436.235356976715</v>
+      </c>
+      <c r="H168" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I168" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9">
+      <c r="A169" t="s">
+        <v>191</v>
+      </c>
+      <c r="B169" t="s">
+        <v>233</v>
+      </c>
+      <c r="E169">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F169">
+        <v>9751</v>
+      </c>
+      <c r="G169" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>15692.718198950352</v>
+      </c>
+      <c r="H169" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I169" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9">
+      <c r="A170" t="s">
+        <v>191</v>
+      </c>
+      <c r="B170" t="s">
+        <v>234</v>
+      </c>
+      <c r="E170">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="F170">
+        <v>11036</v>
+      </c>
+      <c r="G170" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>17760.725878742291</v>
+      </c>
+      <c r="H170" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I170" t="s">
         <v>239</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add LNG transport distances from EG
from Port Said to Europe, AF, SA and from Suez to Asian Regions
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A646E4F-5121-428B-8DAB-A36538638524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380CEC8A-544C-4AF6-8966-243C38A929FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1774" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1832" uniqueCount="261">
   <si>
     <t>Belgium</t>
   </si>
@@ -824,6 +824,9 @@
   </si>
   <si>
     <t>Quintero (Chile)</t>
+  </si>
+  <si>
+    <t>EG from Port Said to Europe, AF and from Suez to Asian Regions</t>
   </si>
 </sst>
 </file>
@@ -1128,7 +1131,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1142,7 +1145,6 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -1532,8 +1534,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I170" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
-  <autoFilter ref="A1:I170" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I187" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+  <autoFilter ref="A1:I187" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
     <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
@@ -14172,7 +14174,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M170"/>
+  <dimension ref="A1:M187"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="21.81640625" customWidth="1"/>
@@ -14363,6 +14365,9 @@
       <c r="I8" t="s">
         <v>245</v>
       </c>
+      <c r="M8" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" t="s">
@@ -15268,7 +15273,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="49" spans="1:7">
+    <row r="49" spans="1:9">
       <c r="A49" t="s">
         <v>199</v>
       </c>
@@ -15284,7 +15289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7">
+    <row r="50" spans="1:9">
       <c r="A50" t="s">
         <v>199</v>
       </c>
@@ -15300,7 +15305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7">
+    <row r="51" spans="1:9">
       <c r="A51" t="s">
         <v>199</v>
       </c>
@@ -15316,7 +15321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:9">
       <c r="A52" t="s">
         <v>199</v>
       </c>
@@ -15332,7 +15337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:7">
+    <row r="53" spans="1:9">
       <c r="A53" t="s">
         <v>199</v>
       </c>
@@ -15348,7 +15353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:9">
       <c r="A54" t="s">
         <v>199</v>
       </c>
@@ -15364,7 +15369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:9">
       <c r="A55" t="s">
         <v>199</v>
       </c>
@@ -15380,7 +15385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7">
+    <row r="56" spans="1:9">
       <c r="A56" t="s">
         <v>197</v>
       </c>
@@ -15391,12 +15396,18 @@
         <f>D56/1000</f>
         <v>0</v>
       </c>
+      <c r="F56">
+        <v>6103</v>
+      </c>
       <c r="G56">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7">
+        <v>9821.8294706382931</v>
+      </c>
+      <c r="I56" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9">
       <c r="A57" t="s">
         <v>197</v>
       </c>
@@ -15407,12 +15418,18 @@
         <f t="shared" ref="E57:E62" si="6">D57/1000</f>
         <v>0</v>
       </c>
+      <c r="F57">
+        <v>5250</v>
+      </c>
       <c r="G57">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7">
+        <v>8449.0586139359402</v>
+      </c>
+      <c r="I57" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9">
       <c r="A58" t="s">
         <v>197</v>
       </c>
@@ -15423,12 +15440,18 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
+      <c r="F58">
+        <v>7546</v>
+      </c>
       <c r="G58">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7">
+        <v>12144.113581097257</v>
+      </c>
+      <c r="I58" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9">
       <c r="A59" t="s">
         <v>197</v>
       </c>
@@ -15439,12 +15462,18 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
+      <c r="F59">
+        <v>7831</v>
+      </c>
       <c r="G59">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7">
+        <v>12602.776762996637</v>
+      </c>
+      <c r="I59" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9">
       <c r="A60" t="s">
         <v>197</v>
       </c>
@@ -15455,12 +15484,18 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
+      <c r="F60">
+        <v>2800</v>
+      </c>
       <c r="G60">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7">
+        <v>4506.1645940991675</v>
+      </c>
+      <c r="I60" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9">
       <c r="A61" t="s">
         <v>197</v>
       </c>
@@ -15471,12 +15506,18 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
+      <c r="F61">
+        <v>5758</v>
+      </c>
       <c r="G61">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7">
+        <v>9266.6056188653602</v>
+      </c>
+      <c r="I61" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9">
       <c r="A62" t="s">
         <v>200</v>
       </c>
@@ -15492,7 +15533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:9">
       <c r="A63" t="s">
         <v>200</v>
       </c>
@@ -15508,7 +15549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:7">
+    <row r="64" spans="1:9">
       <c r="A64" t="s">
         <v>200</v>
       </c>
@@ -17574,11 +17615,11 @@
       <c r="F154">
         <v>9950</v>
       </c>
-      <c r="G154" s="13">
+      <c r="G154">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>16012.977754030971</v>
       </c>
-      <c r="H154" s="13" t="s">
+      <c r="H154" t="s">
         <v>219</v>
       </c>
       <c r="I154" t="s">
@@ -17599,11 +17640,11 @@
       <c r="F155">
         <v>8254</v>
       </c>
-      <c r="G155" s="13">
+      <c r="G155">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>13283.52948560519</v>
       </c>
-      <c r="H155" s="13" t="s">
+      <c r="H155" t="s">
         <v>219</v>
       </c>
       <c r="I155" t="s">
@@ -17624,11 +17665,11 @@
       <c r="F156">
         <v>7341</v>
       </c>
-      <c r="G156" s="13">
+      <c r="G156">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>11814.197959029283</v>
       </c>
-      <c r="H156" s="13" t="s">
+      <c r="H156" t="s">
         <v>219</v>
       </c>
       <c r="I156" t="s">
@@ -17649,11 +17690,11 @@
       <c r="F157">
         <v>8125</v>
       </c>
-      <c r="G157" s="13">
+      <c r="G157">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>13075.924045377049</v>
       </c>
-      <c r="H157" s="13" t="s">
+      <c r="H157" t="s">
         <v>219</v>
       </c>
       <c r="I157" t="s">
@@ -17674,11 +17715,11 @@
       <c r="F158">
         <v>8000</v>
       </c>
-      <c r="G158" s="13">
+      <c r="G158">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>12874.75598314048</v>
       </c>
-      <c r="H158" s="13" t="s">
+      <c r="H158" t="s">
         <v>219</v>
       </c>
       <c r="I158" t="s">
@@ -17699,11 +17740,11 @@
       <c r="F159">
         <v>10884</v>
       </c>
-      <c r="G159" s="13">
+      <c r="G159">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>17516.105515062623</v>
       </c>
-      <c r="H159" s="13" t="s">
+      <c r="H159" t="s">
         <v>219</v>
       </c>
       <c r="I159" t="s">
@@ -17724,11 +17765,11 @@
       <c r="F160">
         <v>10016</v>
       </c>
-      <c r="G160" s="13">
+      <c r="G160">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>16119.194490891881</v>
       </c>
-      <c r="H160" s="13" t="s">
+      <c r="H160" t="s">
         <v>219</v>
       </c>
       <c r="I160" t="s">
@@ -17749,11 +17790,11 @@
       <c r="F161">
         <v>10693</v>
       </c>
-      <c r="G161" s="13">
+      <c r="G161">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>17208.720715965144</v>
       </c>
-      <c r="H161" s="13" t="s">
+      <c r="H161" t="s">
         <v>219</v>
       </c>
       <c r="I161" t="s">
@@ -17774,11 +17815,11 @@
       <c r="F162">
         <v>8939</v>
       </c>
-      <c r="G162" s="13">
+      <c r="G162">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>14385.930466661594</v>
       </c>
-      <c r="H162" s="13" t="s">
+      <c r="H162" t="s">
         <v>219</v>
       </c>
       <c r="I162" t="s">
@@ -17799,11 +17840,11 @@
       <c r="F163">
         <v>8330</v>
       </c>
-      <c r="G163" s="13">
+      <c r="G163">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>13405.839667445025</v>
       </c>
-      <c r="H163" s="13" t="s">
+      <c r="H163" t="s">
         <v>219</v>
       </c>
       <c r="I163" t="s">
@@ -17824,11 +17865,11 @@
       <c r="F164">
         <v>7340</v>
       </c>
-      <c r="G164" s="13">
+      <c r="G164">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>11812.588614531391</v>
       </c>
-      <c r="H164" s="13" t="s">
+      <c r="H164" t="s">
         <v>219</v>
       </c>
       <c r="I164" t="s">
@@ -17849,11 +17890,11 @@
       <c r="F165">
         <v>9764</v>
       </c>
-      <c r="G165" s="13">
+      <c r="G165">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>15713.639677422956</v>
       </c>
-      <c r="H165" s="13" t="s">
+      <c r="H165" t="s">
         <v>219</v>
       </c>
       <c r="I165" t="s">
@@ -17874,11 +17915,11 @@
       <c r="F166">
         <v>11096</v>
       </c>
-      <c r="G166" s="13">
+      <c r="G166">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>17857.286548615844</v>
       </c>
-      <c r="H166" s="13" t="s">
+      <c r="H166" t="s">
         <v>219</v>
       </c>
       <c r="I166" t="s">
@@ -17899,11 +17940,11 @@
       <c r="F167">
         <v>11096</v>
       </c>
-      <c r="G167" s="13">
+      <c r="G167">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>17857.286548615844</v>
       </c>
-      <c r="H167" s="13" t="s">
+      <c r="H167" t="s">
         <v>219</v>
       </c>
       <c r="I167" t="s">
@@ -17924,11 +17965,11 @@
       <c r="F168">
         <v>10213</v>
       </c>
-      <c r="G168" s="13">
+      <c r="G168">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>16436.235356976715</v>
       </c>
-      <c r="H168" s="13" t="s">
+      <c r="H168" t="s">
         <v>219</v>
       </c>
       <c r="I168" t="s">
@@ -17949,11 +17990,11 @@
       <c r="F169">
         <v>9751</v>
       </c>
-      <c r="G169" s="13">
+      <c r="G169">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>15692.718198950352</v>
       </c>
-      <c r="H169" s="13" t="s">
+      <c r="H169" t="s">
         <v>219</v>
       </c>
       <c r="I169" t="s">
@@ -17974,14 +18015,388 @@
       <c r="F170">
         <v>11036</v>
       </c>
-      <c r="G170" s="13">
+      <c r="G170">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>17760.725878742291</v>
       </c>
-      <c r="H170" s="13" t="s">
+      <c r="H170" t="s">
         <v>219</v>
       </c>
       <c r="I170" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9">
+      <c r="A171" t="s">
+        <v>197</v>
+      </c>
+      <c r="B171" t="s">
+        <v>206</v>
+      </c>
+      <c r="E171">
+        <f>D171/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F171">
+        <v>3208</v>
+      </c>
+      <c r="G171">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5162.7771492393322</v>
+      </c>
+      <c r="I171" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9">
+      <c r="A172" t="s">
+        <v>197</v>
+      </c>
+      <c r="B172" t="s">
+        <v>207</v>
+      </c>
+      <c r="E172">
+        <f t="shared" ref="E172:E187" si="15">D172/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F172">
+        <v>1512</v>
+      </c>
+      <c r="G172">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>2433.3288808135508</v>
+      </c>
+      <c r="I172" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9">
+      <c r="A173" t="s">
+        <v>197</v>
+      </c>
+      <c r="B173" t="s">
+        <v>208</v>
+      </c>
+      <c r="E173">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F173">
+        <v>599</v>
+      </c>
+      <c r="G173">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>963.99735423764344</v>
+      </c>
+      <c r="I173" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9">
+      <c r="A174" t="s">
+        <v>197</v>
+      </c>
+      <c r="B174" t="s">
+        <v>209</v>
+      </c>
+      <c r="E174">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F174">
+        <v>1383</v>
+      </c>
+      <c r="G174">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>2225.7234405854106</v>
+      </c>
+      <c r="I174" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="175" spans="1:9">
+      <c r="A175" t="s">
+        <v>197</v>
+      </c>
+      <c r="B175" t="s">
+        <v>210</v>
+      </c>
+      <c r="E175">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F175">
+        <v>1258</v>
+      </c>
+      <c r="G175">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>2024.5553783488403</v>
+      </c>
+      <c r="I175" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="176" spans="1:9">
+      <c r="A176" t="s">
+        <v>197</v>
+      </c>
+      <c r="B176" t="s">
+        <v>211</v>
+      </c>
+      <c r="E176">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F176">
+        <v>4142</v>
+      </c>
+      <c r="G176">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6665.9049102709832</v>
+      </c>
+      <c r="I176" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="177" spans="1:9">
+      <c r="A177" t="s">
+        <v>197</v>
+      </c>
+      <c r="B177" t="s">
+        <v>212</v>
+      </c>
+      <c r="E177">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F177">
+        <v>3274</v>
+      </c>
+      <c r="G177">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5268.9938861002411</v>
+      </c>
+      <c r="I177" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="178" spans="1:9">
+      <c r="A178" t="s">
+        <v>197</v>
+      </c>
+      <c r="B178" t="s">
+        <v>213</v>
+      </c>
+      <c r="E178">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F178">
+        <v>3951</v>
+      </c>
+      <c r="G178">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6358.5201111735041</v>
+      </c>
+      <c r="I178" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="179" spans="1:9">
+      <c r="A179" t="s">
+        <v>197</v>
+      </c>
+      <c r="B179" t="s">
+        <v>214</v>
+      </c>
+      <c r="E179">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F179">
+        <v>2197</v>
+      </c>
+      <c r="G179">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>3535.7298618699542</v>
+      </c>
+      <c r="I179" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="180" spans="1:9">
+      <c r="A180" t="s">
+        <v>197</v>
+      </c>
+      <c r="B180" t="s">
+        <v>215</v>
+      </c>
+      <c r="E180">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F180">
+        <v>1588</v>
+      </c>
+      <c r="G180">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>2555.6390626533853</v>
+      </c>
+      <c r="I180" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="181" spans="1:9">
+      <c r="A181" t="s">
+        <v>197</v>
+      </c>
+      <c r="B181" t="s">
+        <v>216</v>
+      </c>
+      <c r="E181">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F181">
+        <v>598</v>
+      </c>
+      <c r="G181">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>962.38800973975083</v>
+      </c>
+      <c r="I181" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="182" spans="1:9">
+      <c r="A182" t="s">
+        <v>197</v>
+      </c>
+      <c r="B182" t="s">
+        <v>217</v>
+      </c>
+      <c r="E182">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F182">
+        <v>3022</v>
+      </c>
+      <c r="G182">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4863.4390726313159</v>
+      </c>
+      <c r="I182" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="183" spans="1:9">
+      <c r="A183" t="s">
+        <v>197</v>
+      </c>
+      <c r="B183" t="s">
+        <v>230</v>
+      </c>
+      <c r="E183">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F183">
+        <v>4354</v>
+      </c>
+      <c r="G183">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7007.085943824206</v>
+      </c>
+      <c r="I183" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="184" spans="1:9">
+      <c r="A184" t="s">
+        <v>197</v>
+      </c>
+      <c r="B184" t="s">
+        <v>231</v>
+      </c>
+      <c r="E184">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F184">
+        <v>4354</v>
+      </c>
+      <c r="G184">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7007.085943824206</v>
+      </c>
+      <c r="I184" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="185" spans="1:9">
+      <c r="A185" t="s">
+        <v>197</v>
+      </c>
+      <c r="B185" t="s">
+        <v>232</v>
+      </c>
+      <c r="E185">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F185">
+        <v>3471</v>
+      </c>
+      <c r="G185">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5586.0347521850754</v>
+      </c>
+      <c r="I185" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="186" spans="1:9">
+      <c r="A186" t="s">
+        <v>197</v>
+      </c>
+      <c r="B186" t="s">
+        <v>233</v>
+      </c>
+      <c r="E186">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F186">
+        <v>3009</v>
+      </c>
+      <c r="G186">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4842.5175941587131</v>
+      </c>
+      <c r="I186" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="187" spans="1:9">
+      <c r="A187" t="s">
+        <v>197</v>
+      </c>
+      <c r="B187" t="s">
+        <v>234</v>
+      </c>
+      <c r="E187">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
+      <c r="F187">
+        <v>4294</v>
+      </c>
+      <c r="G187">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6910.5252739506523</v>
+      </c>
+      <c r="I187" t="s">
         <v>239</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add LNG transport distances from IM
from Balikpapan (best guess  in the middle) to the different regions
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380CEC8A-544C-4AF6-8966-243C38A929FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B548B0-C9A1-42F6-BEFD-CB062C92EDAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1832" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1908" uniqueCount="262">
   <si>
     <t>Belgium</t>
   </si>
@@ -827,6 +827,9 @@
   </si>
   <si>
     <t>EG from Port Said to Europe, AF and from Suez to Asian Regions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IM from Balikpapan (bestguess  in the middle) </t>
   </si>
 </sst>
 </file>
@@ -1131,7 +1134,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1145,6 +1148,7 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -1534,8 +1538,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I187" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
-  <autoFilter ref="A1:I187" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I204" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+  <autoFilter ref="A1:I204" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
     <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
@@ -14174,7 +14178,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M187"/>
+  <dimension ref="A1:M204"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="21.81640625" customWidth="1"/>
@@ -14390,6 +14394,9 @@
       <c r="I9" t="s">
         <v>246</v>
       </c>
+      <c r="M9" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" t="s">
@@ -15288,6 +15295,7 @@
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
+      <c r="H49" s="13"/>
     </row>
     <row r="50" spans="1:9">
       <c r="A50" t="s">
@@ -15304,6 +15312,7 @@
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
+      <c r="H50" s="13"/>
     </row>
     <row r="51" spans="1:9">
       <c r="A51" t="s">
@@ -15320,6 +15329,7 @@
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
+      <c r="H51" s="13"/>
     </row>
     <row r="52" spans="1:9">
       <c r="A52" t="s">
@@ -15336,6 +15346,7 @@
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>0</v>
       </c>
+      <c r="H52" s="13"/>
     </row>
     <row r="53" spans="1:9">
       <c r="A53" t="s">
@@ -15528,9 +15539,15 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
+      <c r="F62">
+        <v>9163</v>
+      </c>
       <c r="G62">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>14746.423634189527</v>
+      </c>
+      <c r="I62" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -15544,9 +15561,15 @@
         <f t="shared" ref="E63:E68" si="7">D63/1000</f>
         <v>0</v>
       </c>
+      <c r="F63">
+        <v>8354</v>
+      </c>
       <c r="G63">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>13444.463935394446</v>
+      </c>
+      <c r="I63" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -15560,9 +15583,15 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
+      <c r="F64">
+        <v>2583</v>
+      </c>
       <c r="G64">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>4156.936838056482</v>
+      </c>
+      <c r="I64" t="s">
+        <v>248</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -15576,9 +15605,15 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
+      <c r="F65">
+        <v>2657</v>
+      </c>
       <c r="G65">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>4276.0283309005317</v>
+      </c>
+      <c r="I65" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -15592,9 +15627,15 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
+      <c r="F66">
+        <v>3463</v>
+      </c>
       <c r="G66">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>5573.1599962019354</v>
+      </c>
+      <c r="I66" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -15608,9 +15649,15 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
+      <c r="F67">
+        <v>1775</v>
+      </c>
       <c r="G67">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>2856.586483759294</v>
+      </c>
+      <c r="I67" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -15624,9 +15671,15 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
+      <c r="F68">
+        <v>5942</v>
+      </c>
       <c r="G68">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>9562.7250064775908</v>
+      </c>
+      <c r="I68" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -18397,6 +18450,431 @@
         <v>6910.5252739506523</v>
       </c>
       <c r="I187" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="188" spans="1:9">
+      <c r="A188" t="s">
+        <v>200</v>
+      </c>
+      <c r="B188" t="s">
+        <v>206</v>
+      </c>
+      <c r="E188">
+        <f>D188/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F188">
+        <v>9237</v>
+      </c>
+      <c r="G188" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>14865.515127033575</v>
+      </c>
+      <c r="H188" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I188" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="189" spans="1:9">
+      <c r="A189" t="s">
+        <v>200</v>
+      </c>
+      <c r="B189" t="s">
+        <v>207</v>
+      </c>
+      <c r="E189">
+        <f t="shared" ref="E189:E204" si="16">D189/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F189">
+        <v>7541</v>
+      </c>
+      <c r="G189" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>12136.066858607795</v>
+      </c>
+      <c r="H189" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I189" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="190" spans="1:9">
+      <c r="A190" t="s">
+        <v>200</v>
+      </c>
+      <c r="B190" t="s">
+        <v>208</v>
+      </c>
+      <c r="E190">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F190">
+        <v>6628</v>
+      </c>
+      <c r="G190" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>10666.735332031887</v>
+      </c>
+      <c r="H190" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I190" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="191" spans="1:9">
+      <c r="A191" t="s">
+        <v>200</v>
+      </c>
+      <c r="B191" t="s">
+        <v>209</v>
+      </c>
+      <c r="E191">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F191">
+        <v>7412</v>
+      </c>
+      <c r="G191" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11928.461418379655</v>
+      </c>
+      <c r="H191" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I191" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="192" spans="1:9">
+      <c r="A192" t="s">
+        <v>200</v>
+      </c>
+      <c r="B192" t="s">
+        <v>210</v>
+      </c>
+      <c r="E192">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F192">
+        <v>7287</v>
+      </c>
+      <c r="G192" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>11727.293356143084</v>
+      </c>
+      <c r="H192" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I192" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="193" spans="1:9">
+      <c r="A193" t="s">
+        <v>200</v>
+      </c>
+      <c r="B193" t="s">
+        <v>211</v>
+      </c>
+      <c r="E193">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F193">
+        <v>10171</v>
+      </c>
+      <c r="G193" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>16368.642888065227</v>
+      </c>
+      <c r="H193" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I193" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="194" spans="1:9">
+      <c r="A194" t="s">
+        <v>200</v>
+      </c>
+      <c r="B194" t="s">
+        <v>212</v>
+      </c>
+      <c r="E194">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F194">
+        <v>9303</v>
+      </c>
+      <c r="G194" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>14971.731863894485</v>
+      </c>
+      <c r="H194" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I194" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="195" spans="1:9">
+      <c r="A195" t="s">
+        <v>200</v>
+      </c>
+      <c r="B195" t="s">
+        <v>213</v>
+      </c>
+      <c r="E195">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F195">
+        <v>9980</v>
+      </c>
+      <c r="G195" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>16061.258088967748</v>
+      </c>
+      <c r="H195" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I195" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9">
+      <c r="A196" t="s">
+        <v>200</v>
+      </c>
+      <c r="B196" t="s">
+        <v>214</v>
+      </c>
+      <c r="E196">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F196">
+        <v>8226</v>
+      </c>
+      <c r="G196" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>13238.467839664198</v>
+      </c>
+      <c r="H196" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I196" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="197" spans="1:9">
+      <c r="A197" t="s">
+        <v>200</v>
+      </c>
+      <c r="B197" t="s">
+        <v>215</v>
+      </c>
+      <c r="E197">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F197">
+        <v>7617</v>
+      </c>
+      <c r="G197" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>12258.377040447629</v>
+      </c>
+      <c r="H197" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I197" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="198" spans="1:9">
+      <c r="A198" t="s">
+        <v>200</v>
+      </c>
+      <c r="B198" t="s">
+        <v>216</v>
+      </c>
+      <c r="E198">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F198">
+        <v>6627</v>
+      </c>
+      <c r="G198" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>10665.125987533995</v>
+      </c>
+      <c r="H198" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I198" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="199" spans="1:9">
+      <c r="A199" t="s">
+        <v>200</v>
+      </c>
+      <c r="B199" t="s">
+        <v>217</v>
+      </c>
+      <c r="E199">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F199">
+        <v>9051</v>
+      </c>
+      <c r="G199" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>14566.17705042556</v>
+      </c>
+      <c r="H199" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I199" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="200" spans="1:9">
+      <c r="A200" t="s">
+        <v>200</v>
+      </c>
+      <c r="B200" t="s">
+        <v>230</v>
+      </c>
+      <c r="E200">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F200">
+        <v>10383</v>
+      </c>
+      <c r="G200" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>16709.823921618448</v>
+      </c>
+      <c r="H200" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I200" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9">
+      <c r="A201" t="s">
+        <v>200</v>
+      </c>
+      <c r="B201" t="s">
+        <v>231</v>
+      </c>
+      <c r="E201">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F201">
+        <v>10383</v>
+      </c>
+      <c r="G201" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>16709.823921618448</v>
+      </c>
+      <c r="H201" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I201" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9">
+      <c r="A202" t="s">
+        <v>200</v>
+      </c>
+      <c r="B202" t="s">
+        <v>232</v>
+      </c>
+      <c r="E202">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F202">
+        <v>9500</v>
+      </c>
+      <c r="G202" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>15288.772729979319</v>
+      </c>
+      <c r="H202" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I202" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9">
+      <c r="A203" t="s">
+        <v>200</v>
+      </c>
+      <c r="B203" t="s">
+        <v>233</v>
+      </c>
+      <c r="E203">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F203">
+        <v>9038</v>
+      </c>
+      <c r="G203" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>14545.255571952957</v>
+      </c>
+      <c r="H203" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I203" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="204" spans="1:9">
+      <c r="A204" t="s">
+        <v>200</v>
+      </c>
+      <c r="B204" t="s">
+        <v>234</v>
+      </c>
+      <c r="E204">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F204">
+        <v>10323</v>
+      </c>
+      <c r="G204" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>16613.263251744895</v>
+      </c>
+      <c r="H204" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="I204" t="s">
         <v>239</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add LNG transport distances from RU
from Sabetta (plus 1200 mi to the west as Murmansk is the closest port) except for JS, there it comes from Vladivostok
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7B548B0-C9A1-42F6-BEFD-CB062C92EDAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973892C0-654D-443E-8E9E-C458535F6BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1908" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1970" uniqueCount="265">
   <si>
     <t>Belgium</t>
   </si>
@@ -830,6 +830,15 @@
   </si>
   <si>
     <t xml:space="preserve">IM from Balikpapan (bestguess  in the middle) </t>
+  </si>
+  <si>
+    <t>Isle of Grain</t>
+  </si>
+  <si>
+    <t>Dunkirk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RU from Sabetta (plus 1200 mi to west, minus 1200 mi to east as Murmansk is the closest port) except for JS, there it's from Vladivostok </t>
   </si>
 </sst>
 </file>
@@ -1538,8 +1547,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I204" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
-  <autoFilter ref="A1:I204" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I221" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+  <autoFilter ref="A1:I221" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
     <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
@@ -14178,7 +14187,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M204"/>
+  <dimension ref="A1:M221"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="21.81640625" customWidth="1"/>
@@ -14422,6 +14431,9 @@
       <c r="I10" t="s">
         <v>248</v>
       </c>
+      <c r="M10" t="s">
+        <v>264</v>
+      </c>
     </row>
     <row r="11" spans="1:13">
       <c r="A11" t="s">
@@ -15291,11 +15303,16 @@
         <f>D49/1000</f>
         <v>0</v>
       </c>
+      <c r="F49">
+        <v>7893</v>
+      </c>
       <c r="G49">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H49" s="13"/>
+        <v>12702.556121865975</v>
+      </c>
+      <c r="I49" t="s">
+        <v>245</v>
+      </c>
     </row>
     <row r="50" spans="1:9">
       <c r="A50" t="s">
@@ -15308,11 +15325,16 @@
         <f t="shared" ref="E50:E55" si="5">D50/1000</f>
         <v>0</v>
       </c>
+      <c r="F50">
+        <v>7122</v>
+      </c>
       <c r="G50">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H50" s="13"/>
+        <v>11461.751513990812</v>
+      </c>
+      <c r="I50" t="s">
+        <v>246</v>
+      </c>
     </row>
     <row r="51" spans="1:9">
       <c r="A51" t="s">
@@ -15325,11 +15347,19 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
+      <c r="F51">
+        <v>13641</v>
+      </c>
       <c r="G51">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H51" s="13"/>
+        <v>21953.068295752411</v>
+      </c>
+      <c r="H51" t="s">
+        <v>219</v>
+      </c>
+      <c r="I51" t="s">
+        <v>248</v>
+      </c>
     </row>
     <row r="52" spans="1:9">
       <c r="A52" t="s">
@@ -15342,11 +15372,16 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
+      <c r="F52">
+        <v>949</v>
+      </c>
       <c r="G52">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H52" s="13"/>
+        <v>1527.2679285000395</v>
+      </c>
+      <c r="I52" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="53" spans="1:9">
       <c r="A53" t="s">
@@ -15359,9 +15394,18 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
+      <c r="F53">
+        <v>8895</v>
+      </c>
       <c r="G53">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>14315.119308754322</v>
+      </c>
+      <c r="H53" t="s">
+        <v>219</v>
+      </c>
+      <c r="I53" t="s">
+        <v>250</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -15375,9 +15419,18 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
+      <c r="F54">
+        <v>11853</v>
+      </c>
       <c r="G54">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>19075.560333520512</v>
+      </c>
+      <c r="H54" t="s">
+        <v>219</v>
+      </c>
+      <c r="I54" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -15391,9 +15444,15 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
+      <c r="F55">
+        <v>6008</v>
+      </c>
       <c r="G55">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>0</v>
+        <v>9668.9417433385006</v>
+      </c>
+      <c r="I55" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -18467,11 +18526,11 @@
       <c r="F188">
         <v>9237</v>
       </c>
-      <c r="G188" s="13">
+      <c r="G188">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>14865.515127033575</v>
       </c>
-      <c r="H188" s="13" t="s">
+      <c r="H188" t="s">
         <v>219</v>
       </c>
       <c r="I188" t="s">
@@ -18492,11 +18551,11 @@
       <c r="F189">
         <v>7541</v>
       </c>
-      <c r="G189" s="13">
+      <c r="G189">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>12136.066858607795</v>
       </c>
-      <c r="H189" s="13" t="s">
+      <c r="H189" t="s">
         <v>219</v>
       </c>
       <c r="I189" t="s">
@@ -18517,11 +18576,11 @@
       <c r="F190">
         <v>6628</v>
       </c>
-      <c r="G190" s="13">
+      <c r="G190">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10666.735332031887</v>
       </c>
-      <c r="H190" s="13" t="s">
+      <c r="H190" t="s">
         <v>219</v>
       </c>
       <c r="I190" t="s">
@@ -18542,11 +18601,11 @@
       <c r="F191">
         <v>7412</v>
       </c>
-      <c r="G191" s="13">
+      <c r="G191">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>11928.461418379655</v>
       </c>
-      <c r="H191" s="13" t="s">
+      <c r="H191" t="s">
         <v>219</v>
       </c>
       <c r="I191" t="s">
@@ -18567,11 +18626,11 @@
       <c r="F192">
         <v>7287</v>
       </c>
-      <c r="G192" s="13">
+      <c r="G192">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>11727.293356143084</v>
       </c>
-      <c r="H192" s="13" t="s">
+      <c r="H192" t="s">
         <v>219</v>
       </c>
       <c r="I192" t="s">
@@ -18592,11 +18651,11 @@
       <c r="F193">
         <v>10171</v>
       </c>
-      <c r="G193" s="13">
+      <c r="G193">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>16368.642888065227</v>
       </c>
-      <c r="H193" s="13" t="s">
+      <c r="H193" t="s">
         <v>219</v>
       </c>
       <c r="I193" t="s">
@@ -18617,11 +18676,11 @@
       <c r="F194">
         <v>9303</v>
       </c>
-      <c r="G194" s="13">
+      <c r="G194">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>14971.731863894485</v>
       </c>
-      <c r="H194" s="13" t="s">
+      <c r="H194" t="s">
         <v>219</v>
       </c>
       <c r="I194" t="s">
@@ -18642,11 +18701,11 @@
       <c r="F195">
         <v>9980</v>
       </c>
-      <c r="G195" s="13">
+      <c r="G195">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>16061.258088967748</v>
       </c>
-      <c r="H195" s="13" t="s">
+      <c r="H195" t="s">
         <v>219</v>
       </c>
       <c r="I195" t="s">
@@ -18667,11 +18726,11 @@
       <c r="F196">
         <v>8226</v>
       </c>
-      <c r="G196" s="13">
+      <c r="G196">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>13238.467839664198</v>
       </c>
-      <c r="H196" s="13" t="s">
+      <c r="H196" t="s">
         <v>219</v>
       </c>
       <c r="I196" t="s">
@@ -18692,11 +18751,11 @@
       <c r="F197">
         <v>7617</v>
       </c>
-      <c r="G197" s="13">
+      <c r="G197">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>12258.377040447629</v>
       </c>
-      <c r="H197" s="13" t="s">
+      <c r="H197" t="s">
         <v>219</v>
       </c>
       <c r="I197" t="s">
@@ -18717,11 +18776,11 @@
       <c r="F198">
         <v>6627</v>
       </c>
-      <c r="G198" s="13">
+      <c r="G198">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>10665.125987533995</v>
       </c>
-      <c r="H198" s="13" t="s">
+      <c r="H198" t="s">
         <v>219</v>
       </c>
       <c r="I198" t="s">
@@ -18742,11 +18801,11 @@
       <c r="F199">
         <v>9051</v>
       </c>
-      <c r="G199" s="13">
+      <c r="G199">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>14566.17705042556</v>
       </c>
-      <c r="H199" s="13" t="s">
+      <c r="H199" t="s">
         <v>219</v>
       </c>
       <c r="I199" t="s">
@@ -18767,11 +18826,11 @@
       <c r="F200">
         <v>10383</v>
       </c>
-      <c r="G200" s="13">
+      <c r="G200">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>16709.823921618448</v>
       </c>
-      <c r="H200" s="13" t="s">
+      <c r="H200" t="s">
         <v>219</v>
       </c>
       <c r="I200" t="s">
@@ -18792,11 +18851,11 @@
       <c r="F201">
         <v>10383</v>
       </c>
-      <c r="G201" s="13">
+      <c r="G201">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>16709.823921618448</v>
       </c>
-      <c r="H201" s="13" t="s">
+      <c r="H201" t="s">
         <v>219</v>
       </c>
       <c r="I201" t="s">
@@ -18817,11 +18876,11 @@
       <c r="F202">
         <v>9500</v>
       </c>
-      <c r="G202" s="13">
+      <c r="G202">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>15288.772729979319</v>
       </c>
-      <c r="H202" s="13" t="s">
+      <c r="H202" t="s">
         <v>219</v>
       </c>
       <c r="I202" t="s">
@@ -18842,11 +18901,11 @@
       <c r="F203">
         <v>9038</v>
       </c>
-      <c r="G203" s="13">
+      <c r="G203">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>14545.255571952957</v>
       </c>
-      <c r="H203" s="13" t="s">
+      <c r="H203" t="s">
         <v>219</v>
       </c>
       <c r="I203" t="s">
@@ -18867,14 +18926,405 @@
       <c r="F204">
         <v>10323</v>
       </c>
-      <c r="G204" s="13">
+      <c r="G204">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>16613.263251744895</v>
       </c>
-      <c r="H204" s="13" t="s">
+      <c r="H204" t="s">
         <v>219</v>
       </c>
       <c r="I204" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="205" spans="1:9">
+      <c r="A205" t="s">
+        <v>199</v>
+      </c>
+      <c r="B205" t="s">
+        <v>206</v>
+      </c>
+      <c r="E205">
+        <f>D205/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F205">
+        <v>2843</v>
+      </c>
+      <c r="G205" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4575.366407508548</v>
+      </c>
+      <c r="H205" s="13"/>
+      <c r="I205" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="206" spans="1:9">
+      <c r="A206" t="s">
+        <v>199</v>
+      </c>
+      <c r="B206" t="s">
+        <v>207</v>
+      </c>
+      <c r="E206">
+        <f t="shared" ref="E206:E221" si="17">D206/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F206">
+        <v>2873</v>
+      </c>
+      <c r="G206" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4623.6467424453249</v>
+      </c>
+      <c r="H206" s="13"/>
+      <c r="I206" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9">
+      <c r="A207" t="s">
+        <v>199</v>
+      </c>
+      <c r="B207" t="s">
+        <v>208</v>
+      </c>
+      <c r="E207">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F207">
+        <v>5582</v>
+      </c>
+      <c r="G207" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>8983.3609872362704</v>
+      </c>
+      <c r="H207" s="13"/>
+      <c r="I207" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9">
+      <c r="A208" t="s">
+        <v>199</v>
+      </c>
+      <c r="B208" t="s">
+        <v>209</v>
+      </c>
+      <c r="E208">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F208">
+        <v>4964</v>
+      </c>
+      <c r="G208" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>7988.7860875386677</v>
+      </c>
+      <c r="H208" s="13"/>
+      <c r="I208" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="209" spans="1:9">
+      <c r="A209" t="s">
+        <v>199</v>
+      </c>
+      <c r="B209" t="s">
+        <v>210</v>
+      </c>
+      <c r="E209">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F209">
+        <v>5707</v>
+      </c>
+      <c r="G209" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>9184.5290494728397</v>
+      </c>
+      <c r="H209" s="13"/>
+      <c r="I209" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="210" spans="1:9">
+      <c r="A210" t="s">
+        <v>199</v>
+      </c>
+      <c r="B210" t="s">
+        <v>211</v>
+      </c>
+      <c r="E210">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F210">
+        <v>3047</v>
+      </c>
+      <c r="G210" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4903.6726850786299</v>
+      </c>
+      <c r="H210" s="13"/>
+      <c r="I210" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="211" spans="1:9">
+      <c r="A211" t="s">
+        <v>199</v>
+      </c>
+      <c r="B211" t="s">
+        <v>212</v>
+      </c>
+      <c r="E211">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F211">
+        <v>2827</v>
+      </c>
+      <c r="G211" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4549.6168955422672</v>
+      </c>
+      <c r="H211" s="13"/>
+      <c r="I211" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="212" spans="1:9">
+      <c r="A212" t="s">
+        <v>199</v>
+      </c>
+      <c r="B212" t="s">
+        <v>213</v>
+      </c>
+      <c r="E212">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F212">
+        <v>2856</v>
+      </c>
+      <c r="G212" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4596.2878859811508</v>
+      </c>
+      <c r="H212" s="13"/>
+      <c r="I212" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="213" spans="1:9">
+      <c r="A213" t="s">
+        <v>199</v>
+      </c>
+      <c r="B213" t="s">
+        <v>214</v>
+      </c>
+      <c r="E213">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F213">
+        <v>3840</v>
+      </c>
+      <c r="G213" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>6179.8828719074299</v>
+      </c>
+      <c r="H213" s="13"/>
+      <c r="I213" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="214" spans="1:9">
+      <c r="A214" t="s">
+        <v>199</v>
+      </c>
+      <c r="B214" t="s">
+        <v>215</v>
+      </c>
+      <c r="E214">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F214">
+        <v>3499</v>
+      </c>
+      <c r="G214" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5631.0963981260675</v>
+      </c>
+      <c r="H214" s="13"/>
+      <c r="I214" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="215" spans="1:9">
+      <c r="A215" t="s">
+        <v>199</v>
+      </c>
+      <c r="B215" t="s">
+        <v>216</v>
+      </c>
+      <c r="E215">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F215">
+        <v>5736</v>
+      </c>
+      <c r="G215" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>9231.2000399117242</v>
+      </c>
+      <c r="H215" s="13"/>
+      <c r="I215" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="216" spans="1:9">
+      <c r="A216" t="s">
+        <v>199</v>
+      </c>
+      <c r="B216" t="s">
+        <v>217</v>
+      </c>
+      <c r="E216">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F216">
+        <v>2866</v>
+      </c>
+      <c r="G216" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4612.3813309600764</v>
+      </c>
+      <c r="H216" s="13"/>
+      <c r="I216" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="217" spans="1:9">
+      <c r="A217" t="s">
+        <v>199</v>
+      </c>
+      <c r="B217" t="s">
+        <v>230</v>
+      </c>
+      <c r="E217">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F217">
+        <v>3259</v>
+      </c>
+      <c r="G217" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5244.8537186318526</v>
+      </c>
+      <c r="H217" s="13"/>
+      <c r="I217" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="218" spans="1:9">
+      <c r="A218" t="s">
+        <v>199</v>
+      </c>
+      <c r="B218" t="s">
+        <v>231</v>
+      </c>
+      <c r="E218">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F218">
+        <v>3259</v>
+      </c>
+      <c r="G218" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5244.8537186318526</v>
+      </c>
+      <c r="H218" s="13"/>
+      <c r="I218" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="219" spans="1:9">
+      <c r="A219" t="s">
+        <v>199</v>
+      </c>
+      <c r="B219" t="s">
+        <v>232</v>
+      </c>
+      <c r="E219">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F219">
+        <v>2730</v>
+      </c>
+      <c r="G219" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4393.5104792466891</v>
+      </c>
+      <c r="H219" s="13"/>
+      <c r="I219" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="220" spans="1:9">
+      <c r="A220" t="s">
+        <v>199</v>
+      </c>
+      <c r="B220" t="s">
+        <v>233</v>
+      </c>
+      <c r="E220">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F220">
+        <v>3077</v>
+      </c>
+      <c r="G220" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>4951.9530200154068</v>
+      </c>
+      <c r="H220" s="13"/>
+      <c r="I220" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="221" spans="1:9">
+      <c r="A221" t="s">
+        <v>199</v>
+      </c>
+      <c r="B221" t="s">
+        <v>234</v>
+      </c>
+      <c r="E221">
+        <f t="shared" si="17"/>
+        <v>0</v>
+      </c>
+      <c r="F221">
+        <v>3199</v>
+      </c>
+      <c r="G221" s="13">
+        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
+        <v>5148.2930487582989</v>
+      </c>
+      <c r="H221" s="13"/>
+      <c r="I221" t="s">
         <v>239</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add pipeline connections other than in Europe
so far just the links not the capacity and distance
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973892C0-654D-443E-8E9E-C458535F6BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5181B180-8DAA-41E0-AE08-BEE2B0DBE783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="Connections_2024" sheetId="8" r:id="rId7"/>
     <sheet name="Import_Connections_EU" sheetId="5" r:id="rId8"/>
     <sheet name="global_LNG_connections" sheetId="9" r:id="rId9"/>
+    <sheet name="Global_Connections" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1970" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2003" uniqueCount="268">
   <si>
     <t>Belgium</t>
   </si>
@@ -839,6 +840,15 @@
   </si>
   <si>
     <t xml:space="preserve">RU from Sabetta (plus 1200 mi to west, minus 1200 mi to east as Murmansk is the closest port) except for JS, there it's from Vladivostok </t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>AZ data?</t>
   </si>
 </sst>
 </file>
@@ -1143,7 +1153,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1157,7 +1167,9 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -1202,7 +1214,43 @@
     <cellStyle name="Percent 4" xfId="35" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
     <cellStyle name="Percent 8" xfId="33" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
-  <dxfs count="42">
+  <dxfs count="43">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1509,12 +1557,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D3465064-BCEE-4D04-A8E6-DEAE11BBDA92}" name="Country"/>
     <tableColumn id="2" xr3:uid="{D66D54B4-4DED-47C6-BE50-755A236428ED}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="41"/>
-    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="40"/>
-    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="39">
+    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="42"/>
+    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="41"/>
+    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="40">
       <calculatedColumnFormula>Table2[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="38">
+    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="39">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1534,7 +1582,7 @@
     <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="6">
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="7">
       <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
@@ -1547,7 +1595,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I221" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I221" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4" totalsRowBorderDxfId="3">
   <autoFilter ref="A1:I221" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
@@ -1560,28 +1608,49 @@
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{7E7B8CB5-D54F-4427-813D-93B66C13FCBB}" name="Distance [miles]"/>
-    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="1">
+    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="2">
       <calculatedColumnFormula>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="1"/>
     <tableColumn id="8" xr3:uid="{ECBB25E4-2145-4120-8981-E6E8E1591E5B}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{8104487F-10A3-408B-96B9-D54FDBF0F8A7}" name="Table12" displayName="Table12" ref="A1:H13" totalsRowShown="0">
+  <autoFilter ref="A1:H13" xr:uid="{8104487F-10A3-408B-96B9-D54FDBF0F8A7}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{8DC4F854-8C96-4C42-AF47-2C64D82D363F}" name="From"/>
+    <tableColumn id="2" xr3:uid="{9178F7D7-E3CA-468B-8BE5-E203B9CC620E}" name="To"/>
+    <tableColumn id="3" xr3:uid="{9BB01476-57DE-4D59-8170-98FAC18CF80C}" name="GWh/d [capacity]"/>
+    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a"/>
+    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="0">
+      <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{19F26947-5FDD-4F06-A68D-DB6766B439A7}" name="Distance [miles]"/>
+    <tableColumn id="7" xr3:uid="{2F09491D-CBE5-4483-9E89-48B7C57273C2}" name="Distance [km]">
+      <calculatedColumnFormula>F2*1.60934449789256</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{684836E2-9F64-48D9-962B-C15DC90900B8}" name="comment"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F68" totalsRowShown="0" headerRowDxfId="37" headerRowBorderDxfId="36" tableBorderDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F68" totalsRowShown="0" headerRowDxfId="38" headerRowBorderDxfId="37" tableBorderDxfId="36">
   <autoFilter ref="A53:F68" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3F684FB4-9656-4C92-BAF4-456019B2B924}" name="Country"/>
     <tableColumn id="2" xr3:uid="{082B059D-405D-407D-8F97-297DCD23D3B2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{388F462C-127F-4CB7-B46A-1DD19D06D0E8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{ACDF4345-6201-4524-A8D7-A0CE31D137A6}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="34">
+    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="35">
       <calculatedColumnFormula>Table7[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="33">
+    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="34">
       <calculatedColumnFormula>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1598,12 +1667,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="30">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="31">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="29">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="30">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1612,17 +1681,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F67" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="27" tableBorderDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F67" totalsRowShown="0" headerRowDxfId="29" headerRowBorderDxfId="28" tableBorderDxfId="27">
   <autoFilter ref="A52:F67" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{02819FD0-F6B6-484E-B4DA-8262AECE7052}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{A15C284E-E91C-44C6-B3BB-CC2DD205DA84}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="25">
+    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="26">
       <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="24">
+    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="25">
       <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1639,12 +1708,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="22">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="23">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="21">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="22">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1653,17 +1722,17 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F78" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F78" totalsRowShown="0" headerRowDxfId="21" headerRowBorderDxfId="20" tableBorderDxfId="19">
   <autoFilter ref="A57:F78" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{555371BF-8030-4257-9852-212E94829B9B}" name="Country"/>
     <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="17">
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="18">
       <calculatedColumnFormula>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="16">
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="17">
       <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1680,12 +1749,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="14">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="15">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="13">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="14">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1694,17 +1763,17 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F78" totalsRowShown="0" headerRowDxfId="12" headerRowBorderDxfId="11" tableBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F78" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11">
   <autoFilter ref="A57:F78" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{779C3748-4ECD-495F-809A-B5DD28F5EC2F}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{94BC7314-C5A0-4AAD-895B-84E7A94D7CF7}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="9">
+    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="10">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="8">
+    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="9">
       <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1724,7 +1793,7 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="7">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="8">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
@@ -2709,6 +2778,288 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B77213A-E4EC-469C-967C-1084709D3A56}">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="8.81640625" customWidth="1"/>
+    <col min="6" max="6" width="16.08984375" customWidth="1"/>
+    <col min="7" max="7" width="14.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" t="s">
+        <v>186</v>
+      </c>
+      <c r="D1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" t="s">
+        <v>204</v>
+      </c>
+      <c r="G1" t="s">
+        <v>203</v>
+      </c>
+      <c r="H1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E2" s="13">
+        <f>D2/1000</f>
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <f>F2*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14">
+        <f>D3/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14">
+        <f>F3*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="15">
+        <f>D4/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14">
+        <f>F4*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="14"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14">
+        <f>D5/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14">
+        <f>F5*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="14"/>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="15">
+        <f>D6/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14">
+        <f>F6*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14">
+        <f>D7/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14">
+        <f>F7*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="13">
+        <f>D8/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14">
+        <f>F8*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="14" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14">
+        <f>D9/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14">
+        <f>F9*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14">
+        <f>D10/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14">
+        <f>F10*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14">
+        <f>D11/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14">
+        <f>F11*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="14"/>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14">
+        <f>D12/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14">
+        <f>F12*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H12" s="14"/>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14">
+        <f>D13/1000</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14">
+        <f>F13*1.60934449789256</f>
+        <v>0</v>
+      </c>
+      <c r="H13" s="14"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF82F4-4954-4D06-9A30-AE8575CA18DE}">
   <dimension ref="A1:M68"/>
@@ -18951,11 +19302,10 @@
       <c r="F205">
         <v>2843</v>
       </c>
-      <c r="G205" s="13">
+      <c r="G205">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>4575.366407508548</v>
       </c>
-      <c r="H205" s="13"/>
       <c r="I205" t="s">
         <v>240</v>
       </c>
@@ -18974,11 +19324,10 @@
       <c r="F206">
         <v>2873</v>
       </c>
-      <c r="G206" s="13">
+      <c r="G206">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>4623.6467424453249</v>
       </c>
-      <c r="H206" s="13"/>
       <c r="I206" t="s">
         <v>263</v>
       </c>
@@ -18997,11 +19346,10 @@
       <c r="F207">
         <v>5582</v>
       </c>
-      <c r="G207" s="13">
+      <c r="G207">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>8983.3609872362704</v>
       </c>
-      <c r="H207" s="13"/>
       <c r="I207" t="s">
         <v>221</v>
       </c>
@@ -19020,11 +19368,10 @@
       <c r="F208">
         <v>4964</v>
       </c>
-      <c r="G208" s="13">
+      <c r="G208">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>7988.7860875386677</v>
       </c>
-      <c r="H208" s="13"/>
       <c r="I208" t="s">
         <v>222</v>
       </c>
@@ -19043,11 +19390,10 @@
       <c r="F209">
         <v>5707</v>
       </c>
-      <c r="G209" s="13">
+      <c r="G209">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9184.5290494728397</v>
       </c>
-      <c r="H209" s="13"/>
       <c r="I209" t="s">
         <v>223</v>
       </c>
@@ -19066,11 +19412,10 @@
       <c r="F210">
         <v>3047</v>
       </c>
-      <c r="G210" s="13">
+      <c r="G210">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>4903.6726850786299</v>
       </c>
-      <c r="H210" s="13"/>
       <c r="I210" t="s">
         <v>224</v>
       </c>
@@ -19089,11 +19434,10 @@
       <c r="F211">
         <v>2827</v>
       </c>
-      <c r="G211" s="13">
+      <c r="G211">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>4549.6168955422672</v>
       </c>
-      <c r="H211" s="13"/>
       <c r="I211" t="s">
         <v>225</v>
       </c>
@@ -19112,11 +19456,10 @@
       <c r="F212">
         <v>2856</v>
       </c>
-      <c r="G212" s="13">
+      <c r="G212">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>4596.2878859811508</v>
       </c>
-      <c r="H212" s="13"/>
       <c r="I212" t="s">
         <v>226</v>
       </c>
@@ -19135,11 +19478,10 @@
       <c r="F213">
         <v>3840</v>
       </c>
-      <c r="G213" s="13">
+      <c r="G213">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>6179.8828719074299</v>
       </c>
-      <c r="H213" s="13"/>
       <c r="I213" t="s">
         <v>227</v>
       </c>
@@ -19158,11 +19500,10 @@
       <c r="F214">
         <v>3499</v>
       </c>
-      <c r="G214" s="13">
+      <c r="G214">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5631.0963981260675</v>
       </c>
-      <c r="H214" s="13"/>
       <c r="I214" t="s">
         <v>243</v>
       </c>
@@ -19181,11 +19522,10 @@
       <c r="F215">
         <v>5736</v>
       </c>
-      <c r="G215" s="13">
+      <c r="G215">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>9231.2000399117242</v>
       </c>
-      <c r="H215" s="13"/>
       <c r="I215" t="s">
         <v>229</v>
       </c>
@@ -19204,11 +19544,10 @@
       <c r="F216">
         <v>2866</v>
       </c>
-      <c r="G216" s="13">
+      <c r="G216">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>4612.3813309600764</v>
       </c>
-      <c r="H216" s="13"/>
       <c r="I216" t="s">
         <v>262</v>
       </c>
@@ -19227,11 +19566,10 @@
       <c r="F217">
         <v>3259</v>
       </c>
-      <c r="G217" s="13">
+      <c r="G217">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5244.8537186318526</v>
       </c>
-      <c r="H217" s="13"/>
       <c r="I217" t="s">
         <v>235</v>
       </c>
@@ -19250,11 +19588,10 @@
       <c r="F218">
         <v>3259</v>
       </c>
-      <c r="G218" s="13">
+      <c r="G218">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5244.8537186318526</v>
       </c>
-      <c r="H218" s="13"/>
       <c r="I218" t="s">
         <v>236</v>
       </c>
@@ -19273,11 +19610,10 @@
       <c r="F219">
         <v>2730</v>
       </c>
-      <c r="G219" s="13">
+      <c r="G219">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>4393.5104792466891</v>
       </c>
-      <c r="H219" s="13"/>
       <c r="I219" t="s">
         <v>237</v>
       </c>
@@ -19296,11 +19632,10 @@
       <c r="F220">
         <v>3077</v>
       </c>
-      <c r="G220" s="13">
+      <c r="G220">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>4951.9530200154068</v>
       </c>
-      <c r="H220" s="13"/>
       <c r="I220" t="s">
         <v>238</v>
       </c>
@@ -19319,11 +19654,10 @@
       <c r="F221">
         <v>3199</v>
       </c>
-      <c r="G221" s="13">
+      <c r="G221">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
         <v>5148.2930487582989</v>
       </c>
-      <c r="H221" s="13"/>
       <c r="I221" t="s">
         <v>239</v>
       </c>

</xml_diff>

<commit_message>
add pipeline connections other than in Europe data
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5181B180-8DAA-41E0-AE08-BEE2B0DBE783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77B37497-DFF3-45AC-96AC-229DFC9A7EF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2003" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2015" uniqueCount="279">
   <si>
     <t>Belgium</t>
   </si>
@@ -849,6 +849,39 @@
   </si>
   <si>
     <t>AZ data?</t>
+  </si>
+  <si>
+    <t>bcm/a  [capacity]</t>
+  </si>
+  <si>
+    <t>Data from: https://globalenergymonitor.org/projects/global-gas-infrastructure-tracker/tracker/</t>
+  </si>
+  <si>
+    <t>https://www.gem.wiki/Sino-Myanmar_Gas_Pipeline</t>
+  </si>
+  <si>
+    <t>additional source</t>
+  </si>
+  <si>
+    <t>https://www.gem.wiki/Dolphin_Qatar%E2%80%93UAE_Natural_Gas_Pipeline</t>
+  </si>
+  <si>
+    <t>https://www.gem.wiki/Arab_Gas_Pipeline</t>
+  </si>
+  <si>
+    <t>https://www.gem.wiki/West-East_Gas_Pipeline_3</t>
+  </si>
+  <si>
+    <t>https://www.gem.wiki/Central_Asia%E2%80%93Center_Gas_Pipeline, https://www.gem.wiki/Bukhara-Ural_Gas_Pipeline</t>
+  </si>
+  <si>
+    <t>assumption of both to be on the safe side</t>
+  </si>
+  <si>
+    <t>https://www.reuters.com/business/energy/china-completes-full-pipeline-power-of-siberia-gas-2024-12-02/</t>
+  </si>
+  <si>
+    <t>https://www.gem.wiki/Korpeje-Kordkuy_Gas_Pipeline</t>
   </si>
 </sst>
 </file>
@@ -1153,7 +1186,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1167,9 +1200,6 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -1214,7 +1244,10 @@
     <cellStyle name="Percent 4" xfId="35" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
     <cellStyle name="Percent 8" xfId="33" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
-  <dxfs count="43">
+  <dxfs count="44">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1557,12 +1590,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D3465064-BCEE-4D04-A8E6-DEAE11BBDA92}" name="Country"/>
     <tableColumn id="2" xr3:uid="{D66D54B4-4DED-47C6-BE50-755A236428ED}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="40">
+    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="43"/>
+    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="41">
       <calculatedColumnFormula>Table2[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="39">
+    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]" dataDxfId="40">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1582,7 +1615,7 @@
     <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="7">
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="8">
       <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
@@ -1595,7 +1628,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I221" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="5" tableBorderDxfId="4" totalsRowBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I221" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5" totalsRowBorderDxfId="4">
   <autoFilter ref="A1:I221" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
@@ -1608,10 +1641,10 @@
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{7E7B8CB5-D54F-4427-813D-93B66C13FCBB}" name="Distance [miles]"/>
-    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="2">
+    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="3">
       <calculatedColumnFormula>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="2"/>
     <tableColumn id="8" xr3:uid="{ECBB25E4-2145-4120-8981-E6E8E1591E5B}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1619,14 +1652,16 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{8104487F-10A3-408B-96B9-D54FDBF0F8A7}" name="Table12" displayName="Table12" ref="A1:H13" totalsRowShown="0">
-  <autoFilter ref="A1:H13" xr:uid="{8104487F-10A3-408B-96B9-D54FDBF0F8A7}"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{8104487F-10A3-408B-96B9-D54FDBF0F8A7}" name="Table12" displayName="Table12" ref="A1:I13" totalsRowShown="0">
+  <autoFilter ref="A1:I13" xr:uid="{8104487F-10A3-408B-96B9-D54FDBF0F8A7}"/>
+  <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{8DC4F854-8C96-4C42-AF47-2C64D82D363F}" name="From"/>
     <tableColumn id="2" xr3:uid="{9178F7D7-E3CA-468B-8BE5-E203B9CC620E}" name="To"/>
-    <tableColumn id="3" xr3:uid="{9BB01476-57DE-4D59-8170-98FAC18CF80C}" name="GWh/d [capacity]"/>
-    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a"/>
-    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="0">
+    <tableColumn id="3" xr3:uid="{9BB01476-57DE-4D59-8170-98FAC18CF80C}" name="bcm/a  [capacity]"/>
+    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a" dataDxfId="0">
+      <calculatedColumnFormula>C2*9.77*1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="1">
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{19F26947-5FDD-4F06-A68D-DB6766B439A7}" name="Distance [miles]"/>
@@ -1634,23 +1669,24 @@
       <calculatedColumnFormula>F2*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{684836E2-9F64-48D9-962B-C15DC90900B8}" name="comment"/>
+    <tableColumn id="9" xr3:uid="{A609EF7B-5D9A-46E3-BA4B-384CB20A964B}" name="additional source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F68" totalsRowShown="0" headerRowDxfId="38" headerRowBorderDxfId="37" tableBorderDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A53:F68" totalsRowShown="0" headerRowDxfId="39" headerRowBorderDxfId="38" tableBorderDxfId="37">
   <autoFilter ref="A53:F68" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3F684FB4-9656-4C92-BAF4-456019B2B924}" name="Country"/>
     <tableColumn id="2" xr3:uid="{082B059D-405D-407D-8F97-297DCD23D3B2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{388F462C-127F-4CB7-B46A-1DD19D06D0E8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{ACDF4345-6201-4524-A8D7-A0CE31D137A6}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="35">
+    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="36">
       <calculatedColumnFormula>Table7[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="34">
+    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]" dataDxfId="35">
       <calculatedColumnFormula>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1667,12 +1703,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="33"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="31">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="32">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="30">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="31">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1681,17 +1717,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F67" totalsRowShown="0" headerRowDxfId="29" headerRowBorderDxfId="28" tableBorderDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A52:F67" totalsRowShown="0" headerRowDxfId="30" headerRowBorderDxfId="29" tableBorderDxfId="28">
   <autoFilter ref="A52:F67" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{02819FD0-F6B6-484E-B4DA-8262AECE7052}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{A15C284E-E91C-44C6-B3BB-CC2DD205DA84}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="26">
+    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="27">
       <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="25">
+    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="26">
       <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1708,12 +1744,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="23">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="24">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="22">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="23">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1722,17 +1758,17 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F78" totalsRowShown="0" headerRowDxfId="21" headerRowBorderDxfId="20" tableBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A57:F78" totalsRowShown="0" headerRowDxfId="22" headerRowBorderDxfId="21" tableBorderDxfId="20">
   <autoFilter ref="A57:F78" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{555371BF-8030-4257-9852-212E94829B9B}" name="Country"/>
     <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="18">
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="19">
       <calculatedColumnFormula>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="17">
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="18">
       <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1749,12 +1785,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="15">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="16">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="14">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="15">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1763,17 +1799,17 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F78" totalsRowShown="0" headerRowDxfId="13" headerRowBorderDxfId="12" tableBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A57:F78" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="13" tableBorderDxfId="12">
   <autoFilter ref="A57:F78" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{779C3748-4ECD-495F-809A-B5DD28F5EC2F}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{94BC7314-C5A0-4AAD-895B-84E7A94D7CF7}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="10">
+    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="11">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="9">
+    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="10">
       <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1793,7 +1829,7 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="8">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="9">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
@@ -2780,7 +2816,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B77213A-E4EC-469C-967C-1084709D3A56}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="17.453125" customWidth="1"/>
@@ -2789,7 +2825,7 @@
     <col min="7" max="7" width="14.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>93</v>
       </c>
@@ -2797,7 +2833,7 @@
         <v>94</v>
       </c>
       <c r="C1" t="s">
-        <v>186</v>
+        <v>268</v>
       </c>
       <c r="D1" t="s">
         <v>107</v>
@@ -2814,243 +2850,328 @@
       <c r="H1" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" t="s">
+        <v>271</v>
+      </c>
+      <c r="L1" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
         <v>41</v>
       </c>
       <c r="B2" t="s">
         <v>160</v>
       </c>
-      <c r="E2" s="13">
-        <f>D2/1000</f>
-        <v>0</v>
+      <c r="C2">
+        <v>38</v>
+      </c>
+      <c r="D2">
+        <f t="shared" ref="D2:D13" si="0">C2*9.77*1000</f>
+        <v>371260</v>
+      </c>
+      <c r="E2" s="6">
+        <f t="shared" ref="E2:E13" si="1">D2/1000</f>
+        <v>371.26</v>
       </c>
       <c r="G2">
-        <f>F2*1.60934449789256</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="14" t="s">
+        <v>5000</v>
+      </c>
+      <c r="I2" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" t="s">
         <v>53</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14">
-        <f>D3/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14">
-        <f>F3*1.60934449789256</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="14" t="s">
+      <c r="C3">
+        <f>40+22</f>
+        <v>62</v>
+      </c>
+      <c r="D3">
+        <f t="shared" si="0"/>
+        <v>605740</v>
+      </c>
+      <c r="E3">
+        <f t="shared" si="1"/>
+        <v>605.74</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G2:G13" si="2">F3*1.60934449789256</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
         <v>41</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" t="s">
         <v>176</v>
       </c>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="15">
-        <f>D4/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14">
-        <f>F4*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H4" s="14"/>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="14" t="s">
+      <c r="C4">
+        <f>60.2+21</f>
+        <v>81.2</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>793324</v>
+      </c>
+      <c r="E4" s="12">
+        <f t="shared" si="1"/>
+        <v>793.32399999999996</v>
+      </c>
+      <c r="G4">
+        <v>2400</v>
+      </c>
+      <c r="I4" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
         <v>153</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" t="s">
         <v>266</v>
       </c>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14">
-        <f>D5/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14">
-        <f>F5*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H5" s="14"/>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="14" t="s">
+      <c r="C5">
+        <v>500</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>4885000</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>4885</v>
+      </c>
+      <c r="F5">
+        <v>3000</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="2"/>
+        <v>4828.0334936776799</v>
+      </c>
+      <c r="I5" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
         <v>266</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" t="s">
         <v>153</v>
       </c>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="15">
-        <f>D6/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14">
-        <f>F6*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H6" s="14"/>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="14" t="s">
+      <c r="C6">
+        <v>500</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>4885000</v>
+      </c>
+      <c r="E6" s="12">
+        <f t="shared" si="1"/>
+        <v>4885</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
         <v>176</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" t="s">
         <v>160</v>
       </c>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14">
-        <f>D7/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14">
-        <f>F7*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H7" s="14"/>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="14" t="s">
+      <c r="C7">
+        <v>36</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>351719.99999999994</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>351.71999999999991</v>
+      </c>
+      <c r="G7">
+        <v>7378</v>
+      </c>
+      <c r="I7" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
         <v>176</v>
       </c>
-      <c r="B8" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="13">
-        <f>D8/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14">
-        <f>F8*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H8" s="14" t="s">
+      <c r="B8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8">
+        <f>16+14</f>
+        <v>30</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>293099.99999999994</v>
+      </c>
+      <c r="E8" s="6">
+        <f t="shared" si="1"/>
+        <v>293.09999999999997</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="14" t="s">
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
         <v>156</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" t="s">
         <v>158</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14">
-        <f>D9/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14">
-        <f>F9*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="14"/>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="14" t="s">
+      <c r="C9">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>97699.999999999985</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>97.699999999999989</v>
+      </c>
+      <c r="G9">
+        <v>1200</v>
+      </c>
+      <c r="I9" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
         <v>156</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" t="s">
         <v>176</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14">
-        <f>D10/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14">
-        <f>F10*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="14"/>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="14" t="s">
+      <c r="C10">
+        <f>8</f>
+        <v>8</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>78160</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="1"/>
+        <v>78.16</v>
+      </c>
+      <c r="G10">
+        <v>200</v>
+      </c>
+      <c r="I10" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
         <v>157</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" t="s">
         <v>156</v>
       </c>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14">
-        <f>D11/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14">
-        <f>F11*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H11" s="14"/>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="14" t="s">
+      <c r="C11">
+        <v>33.1</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="0"/>
+        <v>323387</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="1"/>
+        <v>323.387</v>
+      </c>
+      <c r="F11">
+        <v>230</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="2"/>
+        <v>370.14923451528881</v>
+      </c>
+      <c r="I11" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
         <v>156</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" t="s">
         <v>157</v>
       </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14">
-        <f>D12/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14">
-        <f>F12*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="14"/>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="14" t="s">
+      <c r="C12">
+        <v>33.1</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="0"/>
+        <v>323387</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="1"/>
+        <v>323.387</v>
+      </c>
+      <c r="F12">
+        <v>230</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="2"/>
+        <v>370.14923451528881</v>
+      </c>
+      <c r="I12" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
         <v>163</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="B13" t="s">
         <v>160</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14">
-        <f>D13/1000</f>
-        <v>0</v>
-      </c>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14">
-        <f>F13*1.60934449789256</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="14"/>
+      <c r="C13">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>127009.99999999999</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="1"/>
+        <v>127.00999999999999</v>
+      </c>
+      <c r="G13">
+        <v>2520</v>
+      </c>
+      <c r="I13" t="s">
+        <v>270</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
adjust function to create input structure for supply and demand
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BC5C993-06C4-45F9-B65F-0E00B046BADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FA69DBD-B29E-4B43-9881-D1C99B79FA3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5070" yWindow="-21720" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-5070" yWindow="-21720" windowWidth="38640" windowHeight="21120" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2008" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2009" uniqueCount="281">
   <si>
     <t>Belgium</t>
   </si>
@@ -1216,7 +1216,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1232,6 +1232,7 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -1276,138 +1277,12 @@
     <cellStyle name="Percent 4" xfId="35" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
     <cellStyle name="Percent 8" xfId="33" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
-  <dxfs count="46">
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
+  <dxfs count="48">
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <font>
@@ -1515,6 +1390,50 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -1524,6 +1443,50 @@
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -1531,6 +1494,50 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1628,15 +1635,15 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{D3465064-BCEE-4D04-A8E6-DEAE11BBDA92}" name="Country"/>
     <tableColumn id="2" xr3:uid="{D66D54B4-4DED-47C6-BE50-755A236428ED}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="44"/>
-    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="43">
+    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="46"/>
+    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="45">
       <calculatedColumnFormula>Table2[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{337F5DC2-FD6B-445B-A2F7-5464B34B589E}" name="GWh [2020]" dataDxfId="42">
+    <tableColumn id="7" xr3:uid="{337F5DC2-FD6B-445B-A2F7-5464B34B589E}" name="GWh [2020]" dataDxfId="44">
       <calculatedColumnFormula>Table2[[#This Row],[TWh '[2020']2]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]2" dataDxfId="41">
+    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]2" dataDxfId="43">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1656,7 +1663,7 @@
     <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="23">
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="10">
       <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
@@ -1669,7 +1676,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I215" totalsRowShown="0" headerRowDxfId="22" headerRowBorderDxfId="21" tableBorderDxfId="20" totalsRowBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I215" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7" totalsRowBorderDxfId="6">
   <autoFilter ref="A1:I215" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
@@ -1682,10 +1689,10 @@
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{7E7B8CB5-D54F-4427-813D-93B66C13FCBB}" name="Distance [miles]"/>
-    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="18">
+    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="5">
       <calculatedColumnFormula>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="17"/>
+    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="4"/>
     <tableColumn id="8" xr3:uid="{ECBB25E4-2145-4120-8981-E6E8E1591E5B}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1699,10 +1706,10 @@
     <tableColumn id="1" xr3:uid="{8DC4F854-8C96-4C42-AF47-2C64D82D363F}" name="From"/>
     <tableColumn id="2" xr3:uid="{9178F7D7-E3CA-468B-8BE5-E203B9CC620E}" name="To"/>
     <tableColumn id="3" xr3:uid="{9BB01476-57DE-4D59-8170-98FAC18CF80C}" name="bcm/a  [capacity]"/>
-    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a" dataDxfId="16">
+    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a" dataDxfId="3">
       <calculatedColumnFormula>C2*9.77*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="15">
+    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="2">
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{19F26947-5FDD-4F06-A68D-DB6766B439A7}" name="Distance [miles]"/>
@@ -1717,20 +1724,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A1:G16" totalsRowShown="0" headerRowDxfId="40" headerRowBorderDxfId="39" tableBorderDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A1:G16" totalsRowShown="0" headerRowDxfId="42" headerRowBorderDxfId="41" tableBorderDxfId="40">
   <autoFilter ref="A1:G16" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{3F684FB4-9656-4C92-BAF4-456019B2B924}" name="Country"/>
     <tableColumn id="2" xr3:uid="{082B059D-405D-407D-8F97-297DCD23D3B2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{388F462C-127F-4CB7-B46A-1DD19D06D0E8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{ACDF4345-6201-4524-A8D7-A0CE31D137A6}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="37">
+    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="39">
       <calculatedColumnFormula>Table7[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{4A1E0E2A-2ECC-45EB-9D63-EC01B197BAA8}" name="GWh [2020]" dataDxfId="36">
+    <tableColumn id="7" xr3:uid="{4A1E0E2A-2ECC-45EB-9D63-EC01B197BAA8}" name="GWh [2020]" dataDxfId="38">
       <calculatedColumnFormula>Table7[[#This Row],[TWh '[2020']2]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]2" dataDxfId="35">
+    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]2" dataDxfId="37">
       <calculatedColumnFormula>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1747,12 +1754,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="34"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="33"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="32">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="34">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="31">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="33">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1761,17 +1768,17 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A1:F16" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="12" tableBorderDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A1:F16" totalsRowShown="0" headerRowDxfId="32" headerRowBorderDxfId="31" tableBorderDxfId="30">
   <autoFilter ref="A1:F16" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{02819FD0-F6B6-484E-B4DA-8262AECE7052}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{A15C284E-E91C-44C6-B3BB-CC2DD205DA84}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="11">
+    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="29">
       <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="10">
+    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="28">
       <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1780,21 +1787,24 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}" name="Table1" displayName="Table1" ref="A1:F42" totalsRowShown="0">
-  <autoFilter ref="A1:F42" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}" name="Table1" displayName="Table1" ref="A1:G42" totalsRowShown="0">
+  <autoFilter ref="A1:G42" xr:uid="{B73A1919-17A7-42D3-8518-97DC2C923D0A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E41">
     <sortCondition ref="B1:B41"/>
   </sortState>
-  <tableColumns count="6">
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="29">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="27"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="26">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="28">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="25">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{53C148C2-CAF7-47BC-9950-964805B82325}" name="GWh [2020]" dataDxfId="1">
+      <calculatedColumnFormula>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1802,17 +1812,20 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A1:F22" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="7" tableBorderDxfId="8">
-  <autoFilter ref="A1:F22" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A1:G22" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22">
+  <autoFilter ref="A1:G22" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{555371BF-8030-4257-9852-212E94829B9B}" name="Country"/>
     <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="6">
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="21">
       <calculatedColumnFormula>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="5">
+    <tableColumn id="7" xr3:uid="{95C698CF-3EBE-40E8-840D-A6C3E41CFB2C}" name="GWh [2020]" dataDxfId="0">
+      <calculatedColumnFormula>Table7910[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="20">
       <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1829,12 +1842,12 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="26">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="18">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="25">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="17">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1843,17 +1856,17 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A1:F22" totalsRowShown="0" headerRowDxfId="4" headerRowBorderDxfId="2" tableBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A1:F22" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14">
   <autoFilter ref="A1:F22" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{779C3748-4ECD-495F-809A-B5DD28F5EC2F}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{94BC7314-C5A0-4AAD-895B-84E7A94D7CF7}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="1">
+    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="13">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="12">
       <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1873,7 +1886,7 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="24">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="11">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
@@ -17217,7 +17230,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE55996C-4401-4161-B17D-CF2A8462856A}">
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
@@ -17228,7 +17241,7 @@
     <col min="14" max="14" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -17247,8 +17260,11 @@
       <c r="F1" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -17267,8 +17283,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</f>
         <v>-7.7179334425266708</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-7717.9334425266707</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -17289,8 +17309,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E3/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="G3">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-83311.215032510125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -17311,8 +17335,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E4/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-166072.21859999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>45</v>
       </c>
@@ -17331,8 +17359,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E5/$E$27),0)</f>
         <v>-9.4697904361571084</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="G5">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-9469.7904361571091</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>32</v>
       </c>
@@ -17353,8 +17385,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E6/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-28534.750500000002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -17375,8 +17411,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E7/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G7">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-28692.628004960214</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -17397,8 +17437,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E8/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="G8">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-82677.403749999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -17419,8 +17463,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E9/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="G9">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-22691.686527096514</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
         <v>54</v>
       </c>
@@ -17441,8 +17489,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E10/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
+      <c r="G10">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-4201.5885000000007</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>55</v>
       </c>
@@ -17463,8 +17515,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E11/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:6">
+      <c r="G11">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-20241.540277777778</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -17485,8 +17541,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E12/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:6">
+      <c r="G12">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-396494.34948674991</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -17507,8 +17567,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E13/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:6">
+      <c r="G13">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-851040.27499999991</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -17529,8 +17593,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E14/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
+      <c r="G14">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-61967.788200000003</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -17551,8 +17619,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E15/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
+      <c r="G15">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-99585.338611111132</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>44</v>
       </c>
@@ -17573,8 +17645,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E16/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:6">
+      <c r="G16">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-51859.971828173359</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -17595,8 +17671,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E17/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:6">
+      <c r="G17">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-660697.78677761904</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -17617,8 +17697,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E18/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:6">
+      <c r="G18">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-10485.041874999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -17639,8 +17723,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E19/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:6">
+      <c r="G19">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-23061.928680000005</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -17661,8 +17749,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E20/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:6">
+      <c r="G20">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-7059.1784297499989</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21" t="s">
         <v>112</v>
       </c>
@@ -17681,8 +17773,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E21/$E$27),0)</f>
         <v>-1.395519518455455</v>
       </c>
-    </row>
-    <row r="22" spans="1:6">
+      <c r="G21">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-1395.519518455455</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -17701,8 +17797,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E22/$E$27),0)</f>
         <v>-6.9938687098651737</v>
       </c>
-    </row>
-    <row r="23" spans="1:6">
+      <c r="G22">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-6993.8687098651735</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
       <c r="B23" t="s">
         <v>113</v>
       </c>
@@ -17718,8 +17818,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E23/$E$27),0)</f>
         <v>-1.6865013379857121</v>
       </c>
-    </row>
-    <row r="24" spans="1:6">
+      <c r="G23">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-1686.5013379857121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
         <v>18</v>
       </c>
@@ -17740,8 +17844,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E24/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:6">
+      <c r="G24">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-352642.72222222231</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" t="s">
         <v>46</v>
       </c>
@@ -17762,8 +17870,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E25/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:6">
+      <c r="G25">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-3174.7276534372795</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" t="s">
         <v>49</v>
       </c>
@@ -17784,8 +17896,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E26/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
+      <c r="G26">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-43510.935206807626</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
       <c r="A27" t="s">
         <v>88</v>
       </c>
@@ -17807,8 +17923,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E27/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:6">
+      <c r="G27">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-53288.452470954879</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -17829,8 +17949,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E28/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:6">
+      <c r="G28">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-205800.97916666672</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
       <c r="A29" t="s">
         <v>38</v>
       </c>
@@ -17851,8 +17975,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E29/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:6">
+      <c r="G29">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-58978.164462623259</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -17873,8 +18001,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E30/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="31" spans="1:6">
+      <c r="G30">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-110035.14253861111</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
       <c r="A31" t="s">
         <v>48</v>
       </c>
@@ -17893,8 +18025,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E31/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:6">
+      <c r="G31">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -17913,8 +18049,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E32/$E$27),0)</f>
         <v>-18.784191699349783</v>
       </c>
-    </row>
-    <row r="33" spans="1:6">
+      <c r="G32">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-18784.191699349783</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" t="s">
         <v>29</v>
       </c>
@@ -17935,8 +18075,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E33/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:6">
+      <c r="G33">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-46452.817059444438</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -17957,8 +18101,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E34/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:6">
+      <c r="G34">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-8354.9190005838263</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" t="s">
         <v>37</v>
       </c>
@@ -17979,8 +18127,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E35/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:6">
+      <c r="G35">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-317429.55599070009</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
         <v>83</v>
       </c>
@@ -18001,8 +18153,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E36/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:6">
+      <c r="G36">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-9681.3372500000005</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -18023,8 +18179,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E37/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:6">
+      <c r="G37">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-32384.836111111112</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
         <v>47</v>
       </c>
@@ -18045,8 +18205,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E38/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:6">
+      <c r="G38">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-451470.79627500003</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
         <v>11</v>
       </c>
@@ -18067,8 +18231,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E39/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:6">
+      <c r="G39">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-714630.45541499986</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -18089,8 +18257,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E40/$E$27),0)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:6">
+      <c r="G40">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-286639.5034414946</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
         <v>110</v>
       </c>
@@ -18109,8 +18281,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E41/$E$27),0)</f>
         <v>-2.4081254030090244</v>
       </c>
-    </row>
-    <row r="42" spans="1:6">
+      <c r="G41">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-2408.1254030090245</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
       <c r="B42" t="s">
         <v>119</v>
       </c>
@@ -18126,8 +18302,12 @@
         <f>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E42/$E$27),0)</f>
         <v>-4.8325219236059471</v>
       </c>
-    </row>
-    <row r="44" spans="1:6">
+      <c r="G42">
+        <f>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</f>
+        <v>-4832.5219236059474</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="C44" s="2">
         <f>SUM(Table1[Mrd m3 '[2020']])</f>
         <v>541.77584793709366</v>
@@ -18157,11 +18337,6 @@
       </c>
       <c r="B53" t="s">
         <v>118</v>
-      </c>
-    </row>
-    <row r="80" spans="8:8">
-      <c r="H80" t="s">
-        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -18174,18 +18349,18 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FF12057-E499-4FE6-95AB-7A9B585F85EC}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="9.54296875" customWidth="1"/>
     <col min="2" max="2" width="12.54296875" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" customWidth="1"/>
-    <col min="14" max="14" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="22.26953125" customWidth="1"/>
+    <col min="15" max="15" width="11.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" s="8" t="s">
         <v>16</v>
       </c>
@@ -18201,11 +18376,14 @@
       <c r="E1" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="G1" s="10" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>153</v>
       </c>
@@ -18220,12 +18398,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="15">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-8153549.8638127027</v>
+      </c>
+      <c r="G2" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-8153.5498638127028</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>201</v>
       </c>
@@ -18240,12 +18422,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-2027620.4220686874</v>
+      </c>
+      <c r="G3" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-2027.6204220686873</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>154</v>
       </c>
@@ -18260,12 +18446,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-1303165.7124974753</v>
+      </c>
+      <c r="G4" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-1303.1657124974754</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>155</v>
       </c>
@@ -18280,12 +18470,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-148363.77291714353</v>
+      </c>
+      <c r="G5" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-148.36377291714354</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>156</v>
       </c>
@@ -18300,12 +18494,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-5026511.2714781221</v>
+      </c>
+      <c r="G6" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-5026.5112714781217</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>157</v>
       </c>
@@ -18319,12 +18517,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-375297.30310748302</v>
+      </c>
+      <c r="G7" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-375.297303107483</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>158</v>
       </c>
@@ -18339,12 +18541,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-395189.40186607011</v>
+      </c>
+      <c r="G8" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-395.18940186607011</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>159</v>
       </c>
@@ -18358,12 +18564,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-413440.4101272542</v>
+      </c>
+      <c r="G9" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-413.44041012725421</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
         <v>160</v>
       </c>
@@ -18377,12 +18587,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-3288750.5973451314</v>
+      </c>
+      <c r="G10" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-3288.7505973451316</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>161</v>
       </c>
@@ -18397,12 +18611,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-1579465.226022091</v>
+      </c>
+      <c r="G11" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-1579.465226022091</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>162</v>
       </c>
@@ -18416,12 +18634,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F12" s="3">
+      <c r="F12" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-589718.3853294109</v>
+      </c>
+      <c r="G12" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-589.71838532941092</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>163</v>
       </c>
@@ -18436,12 +18658,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F13" s="3">
+      <c r="F13" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-1854223.9789296088</v>
+      </c>
+      <c r="G13" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-1854.2239789296088</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>176</v>
       </c>
@@ -18456,12 +18682,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F14" s="3">
+      <c r="F14" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-1111052.9491422991</v>
+      </c>
+      <c r="G14" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-1111.0529491422992</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>41</v>
       </c>
@@ -18475,12 +18705,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-4137432.8871681411</v>
+      </c>
+      <c r="G15" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-4137.432887168141</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>50</v>
       </c>
@@ -18494,12 +18728,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F16" s="3">
+      <c r="F16" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-423529.86637499998</v>
+      </c>
+      <c r="G16" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-423.52986637499998</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>52</v>
       </c>
@@ -18513,12 +18751,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F17" s="3">
+      <c r="F17" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-75229</v>
+      </c>
+      <c r="G17" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-75.228999999999999</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>51</v>
       </c>
@@ -18532,12 +18774,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F18" s="3">
+      <c r="F18" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-35078.727272727272</v>
+      </c>
+      <c r="G18" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-35.078727272727271</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>98</v>
       </c>
@@ -18551,12 +18797,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-7685.681042743664</v>
+      </c>
+      <c r="G19" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-7.6856810427436644</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>182</v>
       </c>
@@ -18570,12 +18820,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F20" s="3">
+      <c r="F20" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-569668.41625963582</v>
+      </c>
+      <c r="G20" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-569.66841625963582</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>197</v>
       </c>
@@ -18590,12 +18844,16 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-842117.28647519497</v>
+      </c>
+      <c r="G21" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-842.11728647519499</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -18609,23 +18867,27 @@
         <f>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F22" s="3">
+      <c r="F22" s="2">
+        <f>Table7910[[#This Row],[TWh '[2020']]]*1000</f>
+        <v>-173427.35646017679</v>
+      </c>
+      <c r="G22" s="3">
         <f>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</f>
         <v>-173.42735646017678</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
         <v>80</v>
       </c>
       <c r="B24" t="s">
         <v>138</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:9">
       <c r="A25" t="s">
         <v>81</v>
       </c>
@@ -18634,6 +18896,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
integrate pipelines into edges parameters sheet
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00637CD8-A532-4FC2-9824-C8E70CD437B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0314ECA2-2793-4816-A4B9-C13942589E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5070" yWindow="-21720" windowWidth="38640" windowHeight="21120" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng" sheetId="1" r:id="rId1"/>
@@ -25,8 +25,8 @@
     <sheet name="Connections_2021" sheetId="4" r:id="rId10"/>
     <sheet name="Connections_2024" sheetId="8" r:id="rId11"/>
     <sheet name="Import_Connections_EU" sheetId="5" r:id="rId12"/>
-    <sheet name="global_LNG_connections" sheetId="9" r:id="rId13"/>
-    <sheet name="Global_Connections" sheetId="10" r:id="rId14"/>
+    <sheet name="Global_Connections" sheetId="10" r:id="rId13"/>
+    <sheet name="global_LNG_connections" sheetId="9" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2009" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1992" uniqueCount="284">
   <si>
     <t>Belgium</t>
   </si>
@@ -837,9 +837,6 @@
     <t>NA</t>
   </si>
   <si>
-    <t>AZ data?</t>
-  </si>
-  <si>
     <t>bcm/a  [capacity]</t>
   </si>
   <si>
@@ -892,6 +889,18 @@
   </si>
   <si>
     <t>Isle of ELain</t>
+  </si>
+  <si>
+    <t>assumption for distance</t>
+  </si>
+  <si>
+    <t>https://www.gem.wiki/Torzhok-Minsk-Ivatsevichy_Gas_Pipeline</t>
+  </si>
+  <si>
+    <t>distance [km]</t>
+  </si>
+  <si>
+    <t>distance [miles]</t>
   </si>
 </sst>
 </file>
@@ -1675,6 +1684,30 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{8104487F-10A3-408B-96B9-D54FDBF0F8A7}" name="Table12" displayName="Table12" ref="A1:I13" totalsRowShown="0">
+  <autoFilter ref="A1:I13" xr:uid="{8104487F-10A3-408B-96B9-D54FDBF0F8A7}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{8DC4F854-8C96-4C42-AF47-2C64D82D363F}" name="From"/>
+    <tableColumn id="2" xr3:uid="{9178F7D7-E3CA-468B-8BE5-E203B9CC620E}" name="To"/>
+    <tableColumn id="3" xr3:uid="{9BB01476-57DE-4D59-8170-98FAC18CF80C}" name="bcm/a  [capacity]"/>
+    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a" dataDxfId="1">
+      <calculatedColumnFormula>C2*9.77*1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="0">
+      <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="6" xr3:uid="{19F26947-5FDD-4F06-A68D-DB6766B439A7}" name="distance [miles]"/>
+    <tableColumn id="7" xr3:uid="{2F09491D-CBE5-4483-9E89-48B7C57273C2}" name="distance [km]">
+      <calculatedColumnFormula>F2*1.60934449789256</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{684836E2-9F64-48D9-962B-C15DC90900B8}" name="comment"/>
+    <tableColumn id="9" xr3:uid="{A609EF7B-5D9A-46E3-BA4B-384CB20A964B}" name="additional source"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I215" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5" totalsRowBorderDxfId="4">
   <autoFilter ref="A1:I215" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
@@ -1693,30 +1726,6 @@
     </tableColumn>
     <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="2"/>
     <tableColumn id="8" xr3:uid="{ECBB25E4-2145-4120-8981-E6E8E1591E5B}" name="Comment"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{8104487F-10A3-408B-96B9-D54FDBF0F8A7}" name="Table12" displayName="Table12" ref="A1:I13" totalsRowShown="0">
-  <autoFilter ref="A1:I13" xr:uid="{8104487F-10A3-408B-96B9-D54FDBF0F8A7}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{8DC4F854-8C96-4C42-AF47-2C64D82D363F}" name="From"/>
-    <tableColumn id="2" xr3:uid="{9178F7D7-E3CA-468B-8BE5-E203B9CC620E}" name="To"/>
-    <tableColumn id="3" xr3:uid="{9BB01476-57DE-4D59-8170-98FAC18CF80C}" name="bcm/a  [capacity]"/>
-    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a" dataDxfId="1">
-      <calculatedColumnFormula>C2*9.77*1000</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="0">
-      <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="6" xr3:uid="{19F26947-5FDD-4F06-A68D-DB6766B439A7}" name="Distance [miles]"/>
-    <tableColumn id="7" xr3:uid="{2F09491D-CBE5-4483-9E89-48B7C57273C2}" name="Distance [km]">
-      <calculatedColumnFormula>F2*1.60934449789256</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="8" xr3:uid="{684836E2-9F64-48D9-962B-C15DC90900B8}" name="comment"/>
-    <tableColumn id="9" xr3:uid="{A609EF7B-5D9A-46E3-BA4B-384CB20A964B}" name="additional source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1874,8 +1883,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}" name="Table3" displayName="Table3" ref="A1:H120" totalsRowShown="0">
-  <autoFilter ref="A1:H120" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}" name="Table3" displayName="Table3" ref="A1:H111" totalsRowShown="0">
+  <autoFilter ref="A1:H111" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H111">
     <sortCondition ref="B1:B111"/>
   </sortState>
@@ -2298,7 +2307,7 @@
         <v>73.274999999999991</v>
       </c>
       <c r="I4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J4" t="s">
         <v>102</v>
@@ -2872,7 +2881,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD7211D-DC17-4DD6-B657-CA08F8FBC20F}">
-  <dimension ref="A1:H120"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="20.453125" customWidth="1"/>
@@ -2910,7 +2919,7 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B2" t="s">
         <v>42</v>
@@ -3144,7 +3153,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
@@ -3786,7 +3795,7 @@
         <v>32</v>
       </c>
       <c r="B47" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C47">
         <v>117.8</v>
@@ -3805,7 +3814,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C48">
         <v>398.6</v>
@@ -4927,7 +4936,7 @@
         <v>127.71349999999998</v>
       </c>
       <c r="H103" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="104" spans="1:8">
@@ -5089,150 +5098,6 @@
       <c r="G111">
         <f t="shared" si="3"/>
         <v>180.45599999999999</v>
-      </c>
-    </row>
-    <row r="112" spans="1:8">
-      <c r="A112" t="s">
-        <v>152</v>
-      </c>
-      <c r="B112" t="s">
-        <v>199</v>
-      </c>
-      <c r="F112">
-        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
-      </c>
-      <c r="G112">
-        <f t="shared" ref="G112:G120" si="4">F112/1000</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7">
-      <c r="A113" t="s">
-        <v>199</v>
-      </c>
-      <c r="B113" t="s">
-        <v>152</v>
-      </c>
-      <c r="F113">
-        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
-      </c>
-      <c r="G113">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="114" spans="1:7">
-      <c r="A114" t="s">
-        <v>155</v>
-      </c>
-      <c r="B114" t="s">
-        <v>156</v>
-      </c>
-      <c r="F114">
-        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
-      </c>
-      <c r="G114">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7">
-      <c r="A115" t="s">
-        <v>156</v>
-      </c>
-      <c r="B115" t="s">
-        <v>155</v>
-      </c>
-      <c r="F115">
-        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
-      </c>
-      <c r="G115">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7">
-      <c r="A116" t="s">
-        <v>41</v>
-      </c>
-      <c r="B116" t="s">
-        <v>159</v>
-      </c>
-      <c r="F116">
-        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
-      </c>
-      <c r="G116">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7">
-      <c r="A117" t="s">
-        <v>175</v>
-      </c>
-      <c r="B117" t="s">
-        <v>159</v>
-      </c>
-      <c r="F117">
-        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
-      </c>
-      <c r="G117">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="118" spans="1:7">
-      <c r="A118" t="s">
-        <v>162</v>
-      </c>
-      <c r="B118" t="s">
-        <v>159</v>
-      </c>
-      <c r="F118">
-        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
-      </c>
-      <c r="G118">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="119" spans="1:7">
-      <c r="A119" t="s">
-        <v>41</v>
-      </c>
-      <c r="B119" t="s">
-        <v>175</v>
-      </c>
-      <c r="F119">
-        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
-      </c>
-      <c r="G119">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="120" spans="1:7">
-      <c r="A120" t="s">
-        <v>180</v>
-      </c>
-      <c r="B120" t="s">
-        <v>155</v>
-      </c>
-      <c r="F120">
-        <f>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
-      </c>
-      <c r="G120">
-        <f t="shared" si="4"/>
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5284,7 +5149,7 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B2" t="s">
         <v>42</v>
@@ -5521,7 +5386,7 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B14" t="s">
         <v>32</v>
@@ -6198,7 +6063,7 @@
         <v>32</v>
       </c>
       <c r="B49" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C49">
         <v>120.36</v>
@@ -6217,7 +6082,7 @@
         <v>47</v>
       </c>
       <c r="B50" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C50">
         <v>398.6</v>
@@ -7415,7 +7280,7 @@
         <v>136.875</v>
       </c>
       <c r="H109" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -8212,7 +8077,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B26" t="s">
         <v>42</v>
@@ -8234,7 +8099,7 @@
         <v>97</v>
       </c>
       <c r="B27" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C27">
         <v>395</v>
@@ -8381,6 +8246,377 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B77213A-E4EC-469C-967C-1084709D3A56}">
+  <dimension ref="A1:L13"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="8.81640625" customWidth="1"/>
+    <col min="6" max="6" width="16.08984375" customWidth="1"/>
+    <col min="7" max="7" width="14.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" t="s">
+        <v>262</v>
+      </c>
+      <c r="D1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" t="s">
+        <v>283</v>
+      </c>
+      <c r="G1" t="s">
+        <v>282</v>
+      </c>
+      <c r="H1" t="s">
+        <v>260</v>
+      </c>
+      <c r="I1" t="s">
+        <v>265</v>
+      </c>
+      <c r="L1" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C2">
+        <v>38</v>
+      </c>
+      <c r="D2">
+        <f t="shared" ref="D2:D13" si="0">C2*9.77*1000</f>
+        <v>371260</v>
+      </c>
+      <c r="E2" s="6">
+        <f t="shared" ref="E2:E13" si="1">D2/1000</f>
+        <v>371.26</v>
+      </c>
+      <c r="G2">
+        <v>5000</v>
+      </c>
+      <c r="I2" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3">
+        <f>40+22</f>
+        <v>62</v>
+      </c>
+      <c r="D3">
+        <f t="shared" si="0"/>
+        <v>605740</v>
+      </c>
+      <c r="E3">
+        <f t="shared" si="1"/>
+        <v>605.74</v>
+      </c>
+      <c r="G3">
+        <v>850</v>
+      </c>
+      <c r="I3" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" t="s">
+        <v>175</v>
+      </c>
+      <c r="C4">
+        <f>60.2+21</f>
+        <v>81.2</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>793324</v>
+      </c>
+      <c r="E4" s="11">
+        <f t="shared" si="1"/>
+        <v>793.32399999999996</v>
+      </c>
+      <c r="G4">
+        <v>2400</v>
+      </c>
+      <c r="I4" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
+      <c r="A5" t="s">
+        <v>152</v>
+      </c>
+      <c r="B5" t="s">
+        <v>261</v>
+      </c>
+      <c r="C5">
+        <v>500</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>4885000</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>4885</v>
+      </c>
+      <c r="F5">
+        <v>3000</v>
+      </c>
+      <c r="G5">
+        <f t="shared" ref="G3:G12" si="2">F5*1.60934449789256</f>
+        <v>4828.0334936776799</v>
+      </c>
+      <c r="I5" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>261</v>
+      </c>
+      <c r="B6" t="s">
+        <v>152</v>
+      </c>
+      <c r="C6">
+        <v>500</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>4885000</v>
+      </c>
+      <c r="E6" s="11">
+        <f t="shared" si="1"/>
+        <v>4885</v>
+      </c>
+      <c r="F6">
+        <v>3000</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="2"/>
+        <v>4828.0334936776799</v>
+      </c>
+      <c r="I6" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B7" t="s">
+        <v>159</v>
+      </c>
+      <c r="C7">
+        <v>36</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>351719.99999999994</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>351.71999999999991</v>
+      </c>
+      <c r="G7">
+        <v>7378</v>
+      </c>
+      <c r="I7" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>175</v>
+      </c>
+      <c r="B8" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8">
+        <f>16+14</f>
+        <v>30</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>293099.99999999994</v>
+      </c>
+      <c r="E8" s="6">
+        <f t="shared" si="1"/>
+        <v>293.09999999999997</v>
+      </c>
+      <c r="G8">
+        <v>1000</v>
+      </c>
+      <c r="I8" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" t="s">
+        <v>157</v>
+      </c>
+      <c r="C9">
+        <v>10</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>97699.999999999985</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>97.699999999999989</v>
+      </c>
+      <c r="G9">
+        <v>1200</v>
+      </c>
+      <c r="I9" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B10" t="s">
+        <v>175</v>
+      </c>
+      <c r="C10">
+        <f>8</f>
+        <v>8</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>78160</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="1"/>
+        <v>78.16</v>
+      </c>
+      <c r="G10">
+        <v>200</v>
+      </c>
+      <c r="I10" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>156</v>
+      </c>
+      <c r="B11" t="s">
+        <v>155</v>
+      </c>
+      <c r="C11">
+        <v>33.1</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="0"/>
+        <v>323387</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="1"/>
+        <v>323.387</v>
+      </c>
+      <c r="F11">
+        <v>230</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="2"/>
+        <v>370.14923451528881</v>
+      </c>
+      <c r="I11" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>155</v>
+      </c>
+      <c r="B12" t="s">
+        <v>156</v>
+      </c>
+      <c r="C12">
+        <v>33.1</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="0"/>
+        <v>323387</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="1"/>
+        <v>323.387</v>
+      </c>
+      <c r="F12">
+        <v>230</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="2"/>
+        <v>370.14923451528881</v>
+      </c>
+      <c r="I12" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>162</v>
+      </c>
+      <c r="B13" t="s">
+        <v>159</v>
+      </c>
+      <c r="C13">
+        <v>13</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>127009.99999999999</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="1"/>
+        <v>127.00999999999999</v>
+      </c>
+      <c r="G13">
+        <v>2520</v>
+      </c>
+      <c r="I13" t="s">
+        <v>264</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:M215"/>
@@ -9881,7 +10117,7 @@
         <v>186</v>
       </c>
       <c r="B65" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E65">
         <f t="shared" si="7"/>
@@ -10300,7 +10536,7 @@
         <v>182</v>
       </c>
       <c r="B82" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E82">
         <f t="shared" si="9"/>
@@ -10674,7 +10910,7 @@
         <v>184</v>
       </c>
       <c r="B99" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E99">
         <f t="shared" si="10"/>
@@ -11054,7 +11290,7 @@
         <v>185</v>
       </c>
       <c r="B116" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E116">
         <f t="shared" si="11"/>
@@ -11473,7 +11709,7 @@
         <v>187</v>
       </c>
       <c r="B133" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E133">
         <f t="shared" si="12"/>
@@ -11853,7 +12089,7 @@
         <v>188</v>
       </c>
       <c r="B150" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E150">
         <f t="shared" si="13"/>
@@ -12272,7 +12508,7 @@
         <v>194</v>
       </c>
       <c r="B167" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E167">
         <f t="shared" si="14"/>
@@ -12652,7 +12888,7 @@
         <v>197</v>
       </c>
       <c r="B184" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E184">
         <f t="shared" si="15"/>
@@ -13071,7 +13307,7 @@
         <v>196</v>
       </c>
       <c r="B201" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E201">
         <f t="shared" si="16"/>
@@ -13283,7 +13519,7 @@
         <v>4612.3813309600764</v>
       </c>
       <c r="I210" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="211" spans="1:9">
@@ -13394,373 +13630,6 @@
       </c>
       <c r="I215" t="s">
         <v>235</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B77213A-E4EC-469C-967C-1084709D3A56}">
-  <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
-  <cols>
-    <col min="3" max="3" width="17.453125" customWidth="1"/>
-    <col min="4" max="4" width="8.81640625" customWidth="1"/>
-    <col min="6" max="6" width="16.08984375" customWidth="1"/>
-    <col min="7" max="7" width="14.36328125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12">
-      <c r="A1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C1" t="s">
-        <v>263</v>
-      </c>
-      <c r="D1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E1" t="s">
-        <v>108</v>
-      </c>
-      <c r="F1" t="s">
-        <v>201</v>
-      </c>
-      <c r="G1" t="s">
-        <v>200</v>
-      </c>
-      <c r="H1" t="s">
-        <v>260</v>
-      </c>
-      <c r="I1" t="s">
-        <v>266</v>
-      </c>
-      <c r="L1" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12">
-      <c r="A2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B2" t="s">
-        <v>159</v>
-      </c>
-      <c r="C2">
-        <v>38</v>
-      </c>
-      <c r="D2">
-        <f t="shared" ref="D2:D13" si="0">C2*9.77*1000</f>
-        <v>371260</v>
-      </c>
-      <c r="E2" s="6">
-        <f t="shared" ref="E2:E13" si="1">D2/1000</f>
-        <v>371.26</v>
-      </c>
-      <c r="G2">
-        <v>5000</v>
-      </c>
-      <c r="I2" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="A3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C3">
-        <f>40+22</f>
-        <v>62</v>
-      </c>
-      <c r="D3">
-        <f t="shared" si="0"/>
-        <v>605740</v>
-      </c>
-      <c r="E3">
-        <f t="shared" si="1"/>
-        <v>605.74</v>
-      </c>
-      <c r="G3">
-        <f t="shared" ref="G3:G12" si="2">F3*1.60934449789256</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12">
-      <c r="A4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B4" t="s">
-        <v>175</v>
-      </c>
-      <c r="C4">
-        <f>60.2+21</f>
-        <v>81.2</v>
-      </c>
-      <c r="D4">
-        <f t="shared" si="0"/>
-        <v>793324</v>
-      </c>
-      <c r="E4" s="11">
-        <f t="shared" si="1"/>
-        <v>793.32399999999996</v>
-      </c>
-      <c r="G4">
-        <v>2400</v>
-      </c>
-      <c r="I4" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" t="s">
-        <v>152</v>
-      </c>
-      <c r="B5" t="s">
-        <v>261</v>
-      </c>
-      <c r="C5">
-        <v>500</v>
-      </c>
-      <c r="D5">
-        <f t="shared" si="0"/>
-        <v>4885000</v>
-      </c>
-      <c r="E5">
-        <f t="shared" si="1"/>
-        <v>4885</v>
-      </c>
-      <c r="F5">
-        <v>3000</v>
-      </c>
-      <c r="G5">
-        <f t="shared" si="2"/>
-        <v>4828.0334936776799</v>
-      </c>
-      <c r="I5" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" t="s">
-        <v>261</v>
-      </c>
-      <c r="B6" t="s">
-        <v>152</v>
-      </c>
-      <c r="C6">
-        <v>500</v>
-      </c>
-      <c r="D6">
-        <f t="shared" si="0"/>
-        <v>4885000</v>
-      </c>
-      <c r="E6" s="11">
-        <f t="shared" si="1"/>
-        <v>4885</v>
-      </c>
-      <c r="G6">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I6" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" t="s">
-        <v>175</v>
-      </c>
-      <c r="B7" t="s">
-        <v>159</v>
-      </c>
-      <c r="C7">
-        <v>36</v>
-      </c>
-      <c r="D7">
-        <f t="shared" si="0"/>
-        <v>351719.99999999994</v>
-      </c>
-      <c r="E7">
-        <f t="shared" si="1"/>
-        <v>351.71999999999991</v>
-      </c>
-      <c r="G7">
-        <v>7378</v>
-      </c>
-      <c r="I7" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" t="s">
-        <v>175</v>
-      </c>
-      <c r="B8" t="s">
-        <v>97</v>
-      </c>
-      <c r="C8">
-        <f>16+14</f>
-        <v>30</v>
-      </c>
-      <c r="D8">
-        <f t="shared" si="0"/>
-        <v>293099.99999999994</v>
-      </c>
-      <c r="E8" s="6">
-        <f t="shared" si="1"/>
-        <v>293.09999999999997</v>
-      </c>
-      <c r="G8">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H8" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" t="s">
-        <v>155</v>
-      </c>
-      <c r="B9" t="s">
-        <v>157</v>
-      </c>
-      <c r="C9">
-        <v>10</v>
-      </c>
-      <c r="D9">
-        <f t="shared" si="0"/>
-        <v>97699.999999999985</v>
-      </c>
-      <c r="E9">
-        <f t="shared" si="1"/>
-        <v>97.699999999999989</v>
-      </c>
-      <c r="G9">
-        <v>1200</v>
-      </c>
-      <c r="I9" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="A10" t="s">
-        <v>155</v>
-      </c>
-      <c r="B10" t="s">
-        <v>175</v>
-      </c>
-      <c r="C10">
-        <f>8</f>
-        <v>8</v>
-      </c>
-      <c r="D10">
-        <f t="shared" si="0"/>
-        <v>78160</v>
-      </c>
-      <c r="E10">
-        <f t="shared" si="1"/>
-        <v>78.16</v>
-      </c>
-      <c r="G10">
-        <v>200</v>
-      </c>
-      <c r="I10" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12">
-      <c r="A11" t="s">
-        <v>156</v>
-      </c>
-      <c r="B11" t="s">
-        <v>155</v>
-      </c>
-      <c r="C11">
-        <v>33.1</v>
-      </c>
-      <c r="D11">
-        <f t="shared" si="0"/>
-        <v>323387</v>
-      </c>
-      <c r="E11">
-        <f t="shared" si="1"/>
-        <v>323.387</v>
-      </c>
-      <c r="F11">
-        <v>230</v>
-      </c>
-      <c r="G11">
-        <f t="shared" si="2"/>
-        <v>370.14923451528881</v>
-      </c>
-      <c r="I11" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="A12" t="s">
-        <v>155</v>
-      </c>
-      <c r="B12" t="s">
-        <v>156</v>
-      </c>
-      <c r="C12">
-        <v>33.1</v>
-      </c>
-      <c r="D12">
-        <f t="shared" si="0"/>
-        <v>323387</v>
-      </c>
-      <c r="E12">
-        <f t="shared" si="1"/>
-        <v>323.387</v>
-      </c>
-      <c r="F12">
-        <v>230</v>
-      </c>
-      <c r="G12">
-        <f t="shared" si="2"/>
-        <v>370.14923451528881</v>
-      </c>
-      <c r="I12" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="A13" t="s">
-        <v>162</v>
-      </c>
-      <c r="B13" t="s">
-        <v>159</v>
-      </c>
-      <c r="C13">
-        <v>13</v>
-      </c>
-      <c r="D13">
-        <f t="shared" si="0"/>
-        <v>127009.99999999999</v>
-      </c>
-      <c r="E13">
-        <f t="shared" si="1"/>
-        <v>127.00999999999999</v>
-      </c>
-      <c r="G13">
-        <v>2520</v>
-      </c>
-      <c r="I13" t="s">
-        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -13801,10 +13670,10 @@
         <v>123</v>
       </c>
       <c r="F1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="M1" t="s">
         <v>93</v>
@@ -14278,7 +14147,7 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B16" t="s">
         <v>3</v>
@@ -15244,10 +15113,10 @@
         <v>174</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -17260,7 +17129,7 @@
         <v>120</v>
       </c>
       <c r="G1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -17573,7 +17442,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B14" t="s">
         <v>3</v>
@@ -18376,7 +18245,7 @@
         <v>174</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>106</v>
@@ -19197,7 +19066,7 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B14" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
bug fix part 1
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16C72ABE-F2A6-4CDF-A7C1-037725C31093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66ED207B-A354-4CD7-BA43-5202FFB0D9F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-5070" yWindow="-21720" windowWidth="38640" windowHeight="21120" firstSheet="8" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng_europe_2020" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2054" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2054" uniqueCount="282">
   <si>
     <t>Belgium</t>
   </si>
@@ -830,9 +830,6 @@
   </si>
   <si>
     <t>comment</t>
-  </si>
-  <si>
-    <t>NA</t>
   </si>
   <si>
     <t>bcm/a  [capacity]</t>
@@ -2234,7 +2231,7 @@
         <v>111378</v>
       </c>
       <c r="I2">
-        <f>G2*9.77</f>
+        <f t="shared" ref="I2:I14" si="0">G2*9.77</f>
         <v>111.378</v>
       </c>
       <c r="K2" t="s">
@@ -2266,7 +2263,7 @@
         <v>19.600000000000001</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" ref="E3:E14" si="0">D3/C3</f>
+        <f t="shared" ref="E3:E14" si="1">D3/C3</f>
         <v>0.59393939393939399</v>
       </c>
       <c r="F3">
@@ -2277,11 +2274,11 @@
         <v>33</v>
       </c>
       <c r="H3">
-        <f t="shared" ref="H3:H14" si="1">I3*1000</f>
+        <f t="shared" ref="H3:H14" si="2">I3*1000</f>
         <v>322409.99999999994</v>
       </c>
       <c r="I3">
-        <f>G3*9.77</f>
+        <f t="shared" si="0"/>
         <v>322.40999999999997</v>
       </c>
       <c r="K3" t="s">
@@ -2291,11 +2288,11 @@
         <v>102</v>
       </c>
       <c r="N3" t="str">
-        <f t="shared" ref="N3:N13" si="2">_xlfn.CONCAT(K3,L3)</f>
+        <f t="shared" ref="N3:N13" si="3">_xlfn.CONCAT(K3,L3)</f>
         <v>FR_LNG</v>
       </c>
       <c r="O3" t="str">
-        <f t="shared" ref="O3:O13" si="3">K3</f>
+        <f t="shared" ref="O3:O13" si="4">K3</f>
         <v>FR</v>
       </c>
     </row>
@@ -2304,7 +2301,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C4">
         <v>7</v>
@@ -2313,7 +2310,7 @@
         <v>2.5</v>
       </c>
       <c r="E4" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.35714285714285715</v>
       </c>
       <c r="F4">
@@ -2324,25 +2321,25 @@
         <v>7.5</v>
       </c>
       <c r="H4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>73274.999999999985</v>
       </c>
       <c r="I4">
-        <f>G4*9.77</f>
+        <f t="shared" si="0"/>
         <v>73.274999999999991</v>
       </c>
       <c r="K4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="L4" t="s">
         <v>102</v>
       </c>
       <c r="N4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>EL_LNG</v>
       </c>
       <c r="O4" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>EL</v>
       </c>
     </row>
@@ -2360,7 +2357,7 @@
         <v>12.1</v>
       </c>
       <c r="E5" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.75862068965517238</v>
       </c>
       <c r="F5">
@@ -2371,11 +2368,11 @@
         <v>15.95</v>
       </c>
       <c r="H5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>155831.49999999997</v>
       </c>
       <c r="I5">
-        <f>G5*9.77</f>
+        <f t="shared" si="0"/>
         <v>155.83149999999998</v>
       </c>
       <c r="K5" t="s">
@@ -2385,11 +2382,11 @@
         <v>102</v>
       </c>
       <c r="N5" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>IT_LNG</v>
       </c>
       <c r="O5" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>IT</v>
       </c>
     </row>
@@ -2407,22 +2404,22 @@
         <v>0.4</v>
       </c>
       <c r="E6" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.15384615384615385</v>
       </c>
       <c r="F6">
         <v>2.6</v>
       </c>
       <c r="G6">
-        <f t="shared" ref="G6:G14" si="4">IF(C6&gt;F6,C6,F6)</f>
+        <f t="shared" ref="G6:G14" si="5">IF(C6&gt;F6,C6,F6)</f>
         <v>2.6</v>
       </c>
       <c r="H6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>25402</v>
       </c>
       <c r="I6">
-        <f>G6*9.77</f>
+        <f t="shared" si="0"/>
         <v>25.402000000000001</v>
       </c>
       <c r="K6" t="s">
@@ -2432,11 +2429,11 @@
         <v>102</v>
       </c>
       <c r="N6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>HR_LNG</v>
       </c>
       <c r="O6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>HR</v>
       </c>
     </row>
@@ -2454,22 +2451,22 @@
         <v>1.6</v>
       </c>
       <c r="E7" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.4</v>
       </c>
       <c r="F7">
         <v>4</v>
       </c>
       <c r="G7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>4</v>
       </c>
       <c r="H7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>39080</v>
       </c>
       <c r="I7">
-        <f>G7*9.77</f>
+        <f t="shared" si="0"/>
         <v>39.08</v>
       </c>
       <c r="K7" t="s">
@@ -2479,11 +2476,11 @@
         <v>102</v>
       </c>
       <c r="N7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>LT_LNG</v>
       </c>
       <c r="O7" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>LT</v>
       </c>
     </row>
@@ -2501,22 +2498,22 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="E8" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.68333333333333324</v>
       </c>
       <c r="F8">
         <v>12.5</v>
       </c>
       <c r="G8">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>12.5</v>
       </c>
       <c r="H8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>122125</v>
       </c>
       <c r="I8">
-        <f>G8*9.77</f>
+        <f t="shared" si="0"/>
         <v>122.125</v>
       </c>
       <c r="K8" t="s">
@@ -2526,11 +2523,11 @@
         <v>102</v>
       </c>
       <c r="N8" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>NL_LNG</v>
       </c>
       <c r="O8" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>NL</v>
       </c>
     </row>
@@ -2548,22 +2545,22 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="E9" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.66129032258064513</v>
       </c>
       <c r="F9">
         <v>5.8</v>
       </c>
       <c r="G9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>6.2</v>
       </c>
       <c r="H9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>60574</v>
       </c>
       <c r="I9">
-        <f>G9*9.77</f>
+        <f t="shared" si="0"/>
         <v>60.573999999999998</v>
       </c>
       <c r="K9" t="s">
@@ -2573,11 +2570,11 @@
         <v>102</v>
       </c>
       <c r="N9" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>PL_LNG</v>
       </c>
       <c r="O9" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>PL</v>
       </c>
     </row>
@@ -2595,22 +2592,22 @@
         <v>6.1</v>
       </c>
       <c r="E10" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.80263157894736836</v>
       </c>
       <c r="F10">
         <v>7.3</v>
       </c>
       <c r="G10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>7.6</v>
       </c>
       <c r="H10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>74252</v>
       </c>
       <c r="I10">
-        <f>G10*9.77</f>
+        <f t="shared" si="0"/>
         <v>74.251999999999995</v>
       </c>
       <c r="K10" t="s">
@@ -2620,11 +2617,11 @@
         <v>102</v>
       </c>
       <c r="N10" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>PT_LNG</v>
       </c>
       <c r="O10" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>PT</v>
       </c>
     </row>
@@ -2642,22 +2639,22 @@
         <v>20.9</v>
       </c>
       <c r="E11" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.3477537437603993</v>
       </c>
       <c r="F11">
         <v>67.099999999999994</v>
       </c>
       <c r="G11">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>67.099999999999994</v>
       </c>
       <c r="H11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>655566.99999999988</v>
       </c>
       <c r="I11">
-        <f>G11*9.77</f>
+        <f t="shared" si="0"/>
         <v>655.56699999999989</v>
       </c>
       <c r="K11" t="s">
@@ -2667,11 +2664,11 @@
         <v>102</v>
       </c>
       <c r="N11" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>ES_LNG</v>
       </c>
       <c r="O11" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>ES</v>
       </c>
     </row>
@@ -2689,22 +2686,22 @@
         <v>14.8</v>
       </c>
       <c r="E12" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.33944954128440369</v>
       </c>
       <c r="F12">
         <v>14.8</v>
       </c>
       <c r="G12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>43.6</v>
       </c>
       <c r="H12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>425972</v>
       </c>
       <c r="I12">
-        <f>G12*9.77</f>
+        <f t="shared" si="0"/>
         <v>425.97199999999998</v>
       </c>
       <c r="K12" t="s">
@@ -2714,11 +2711,11 @@
         <v>102</v>
       </c>
       <c r="N12" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>TR_LNG</v>
       </c>
       <c r="O12" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>TR</v>
       </c>
     </row>
@@ -2736,22 +2733,22 @@
         <v>18.600000000000001</v>
       </c>
       <c r="E13" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.38669438669438672</v>
       </c>
       <c r="F13">
         <v>52.3</v>
       </c>
       <c r="G13">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>52.3</v>
       </c>
       <c r="H13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>510970.99999999994</v>
       </c>
       <c r="I13">
-        <f>G13*9.77</f>
+        <f t="shared" si="0"/>
         <v>510.97099999999995</v>
       </c>
       <c r="K13" t="s">
@@ -2761,11 +2758,11 @@
         <v>102</v>
       </c>
       <c r="N13" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>UK_LNG</v>
       </c>
       <c r="O13" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>UK</v>
       </c>
     </row>
@@ -2780,19 +2777,19 @@
         <v>0.7</v>
       </c>
       <c r="E14" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.7</v>
       </c>
       <c r="H14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6838.9999999999991</v>
       </c>
       <c r="I14">
-        <f>G14*9.77</f>
+        <f t="shared" si="0"/>
         <v>6.8389999999999995</v>
       </c>
       <c r="K14" t="s">
@@ -3325,7 +3322,7 @@
         <v>177791.5</v>
       </c>
       <c r="G2">
-        <f>F2/1000</f>
+        <f t="shared" ref="G2:G33" si="0">F2/1000</f>
         <v>177.79150000000001</v>
       </c>
     </row>
@@ -3344,7 +3341,7 @@
         <v>124088.31999999999</v>
       </c>
       <c r="G3">
-        <f>F3/1000</f>
+        <f t="shared" si="0"/>
         <v>124.08832</v>
       </c>
     </row>
@@ -3363,7 +3360,7 @@
         <v>55881.5</v>
       </c>
       <c r="G4">
-        <f>F4/1000</f>
+        <f t="shared" si="0"/>
         <v>55.881500000000003</v>
       </c>
     </row>
@@ -3382,7 +3379,7 @@
         <v>419750</v>
       </c>
       <c r="G5">
-        <f>F5/1000</f>
+        <f t="shared" si="0"/>
         <v>419.75</v>
       </c>
     </row>
@@ -3401,7 +3398,7 @@
         <v>41062.5</v>
       </c>
       <c r="G6">
-        <f>F6/1000</f>
+        <f t="shared" si="0"/>
         <v>41.0625</v>
       </c>
     </row>
@@ -3420,7 +3417,7 @@
         <v>89972.5</v>
       </c>
       <c r="G7">
-        <f>F7/1000</f>
+        <f t="shared" si="0"/>
         <v>89.972499999999997</v>
       </c>
     </row>
@@ -3439,7 +3436,7 @@
         <v>117811.04999999999</v>
       </c>
       <c r="G8">
-        <f>F8/1000</f>
+        <f t="shared" si="0"/>
         <v>117.81104999999999</v>
       </c>
     </row>
@@ -3458,7 +3455,7 @@
         <v>317550</v>
       </c>
       <c r="G9">
-        <f>F9/1000</f>
+        <f t="shared" si="0"/>
         <v>317.55</v>
       </c>
     </row>
@@ -3477,7 +3474,7 @@
         <v>15320.342829999998</v>
       </c>
       <c r="G10">
-        <f>F10/1000</f>
+        <f t="shared" si="0"/>
         <v>15.320342829999998</v>
       </c>
     </row>
@@ -3496,7 +3493,7 @@
         <v>120888</v>
       </c>
       <c r="G11">
-        <f>F11/1000</f>
+        <f t="shared" si="0"/>
         <v>120.88800000000001</v>
       </c>
     </row>
@@ -3518,7 +3515,7 @@
         <v>95301.500000000015</v>
       </c>
       <c r="G12">
-        <f>F12/1000</f>
+        <f t="shared" si="0"/>
         <v>95.301500000000019</v>
       </c>
     </row>
@@ -3527,7 +3524,7 @@
         <v>32</v>
       </c>
       <c r="B13" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C13">
         <v>117.8</v>
@@ -3537,7 +3534,7 @@
         <v>42997</v>
       </c>
       <c r="G13">
-        <f>F13/1000</f>
+        <f t="shared" si="0"/>
         <v>42.997</v>
       </c>
     </row>
@@ -3559,7 +3556,7 @@
         <v>9993.6999999999989</v>
       </c>
       <c r="G14">
-        <f>F14/1000</f>
+        <f t="shared" si="0"/>
         <v>9.9936999999999987</v>
       </c>
     </row>
@@ -3578,7 +3575,7 @@
         <v>54074.75</v>
       </c>
       <c r="G15">
-        <f>F15/1000</f>
+        <f t="shared" si="0"/>
         <v>54.074750000000002</v>
       </c>
     </row>
@@ -3600,7 +3597,7 @@
         <v>145317.45000000001</v>
       </c>
       <c r="G16">
-        <f>F16/1000</f>
+        <f t="shared" si="0"/>
         <v>145.31745000000001</v>
       </c>
     </row>
@@ -3622,7 +3619,7 @@
         <v>181463.40000000002</v>
       </c>
       <c r="G17">
-        <f>F17/1000</f>
+        <f t="shared" si="0"/>
         <v>181.46340000000004</v>
       </c>
     </row>
@@ -3644,7 +3641,7 @@
         <v>118770.99999999999</v>
       </c>
       <c r="G18">
-        <f>F18/1000</f>
+        <f t="shared" si="0"/>
         <v>118.77099999999999</v>
       </c>
     </row>
@@ -3666,7 +3663,7 @@
         <v>439277.49999999994</v>
       </c>
       <c r="G19">
-        <f>F19/1000</f>
+        <f t="shared" si="0"/>
         <v>439.27749999999992</v>
       </c>
     </row>
@@ -3685,7 +3682,7 @@
         <v>12969.074412800001</v>
       </c>
       <c r="G20">
-        <f>F20/1000</f>
+        <f t="shared" si="0"/>
         <v>12.969074412800001</v>
       </c>
     </row>
@@ -3704,7 +3701,7 @@
         <v>63072.000000000007</v>
       </c>
       <c r="G21">
-        <f>F21/1000</f>
+        <f t="shared" si="0"/>
         <v>63.07200000000001</v>
       </c>
     </row>
@@ -3723,7 +3720,7 @@
         <v>36500</v>
       </c>
       <c r="G22">
-        <f>F22/1000</f>
+        <f t="shared" si="0"/>
         <v>36.5</v>
       </c>
     </row>
@@ -3742,7 +3739,7 @@
         <v>233746</v>
       </c>
       <c r="G23">
-        <f>F23/1000</f>
+        <f t="shared" si="0"/>
         <v>233.74600000000001</v>
       </c>
     </row>
@@ -3761,11 +3758,11 @@
         <v>144175</v>
       </c>
       <c r="G24">
-        <f>F24/1000</f>
+        <f t="shared" si="0"/>
         <v>144.17500000000001</v>
       </c>
       <c r="H24" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -3783,7 +3780,7 @@
         <v>449592.03500000003</v>
       </c>
       <c r="G25">
-        <f>F25/1000</f>
+        <f t="shared" si="0"/>
         <v>449.59203500000001</v>
       </c>
     </row>
@@ -3802,7 +3799,7 @@
         <v>10220</v>
       </c>
       <c r="G26">
-        <f>F26/1000</f>
+        <f t="shared" si="0"/>
         <v>10.220000000000001</v>
       </c>
     </row>
@@ -3821,7 +3818,7 @@
         <v>454936.00000000006</v>
       </c>
       <c r="G27">
-        <f>F27/1000</f>
+        <f t="shared" si="0"/>
         <v>454.93600000000004</v>
       </c>
     </row>
@@ -3840,7 +3837,7 @@
         <v>125650.51999999997</v>
       </c>
       <c r="G28">
-        <f>F28/1000</f>
+        <f t="shared" si="0"/>
         <v>125.65051999999997</v>
       </c>
     </row>
@@ -3859,7 +3856,7 @@
         <v>144594.75</v>
       </c>
       <c r="G29">
-        <f>F29/1000</f>
+        <f t="shared" si="0"/>
         <v>144.59475</v>
       </c>
     </row>
@@ -3878,7 +3875,7 @@
         <v>119720</v>
       </c>
       <c r="G30">
-        <f>F30/1000</f>
+        <f t="shared" si="0"/>
         <v>119.72</v>
       </c>
     </row>
@@ -3897,7 +3894,7 @@
         <v>658376.05000000005</v>
       </c>
       <c r="G31">
-        <f>F31/1000</f>
+        <f t="shared" si="0"/>
         <v>658.37605000000008</v>
       </c>
     </row>
@@ -3916,7 +3913,7 @@
         <v>49680.88</v>
       </c>
       <c r="G32">
-        <f>F32/1000</f>
+        <f t="shared" si="0"/>
         <v>49.680879999999995</v>
       </c>
     </row>
@@ -3935,7 +3932,7 @@
         <v>224006.34</v>
       </c>
       <c r="G33">
-        <f>F33/1000</f>
+        <f t="shared" si="0"/>
         <v>224.00633999999999</v>
       </c>
     </row>
@@ -3954,7 +3951,7 @@
         <v>9749.15</v>
       </c>
       <c r="G34">
-        <f>F34/1000</f>
+        <f t="shared" ref="G34:G65" si="1">F34/1000</f>
         <v>9.7491500000000002</v>
       </c>
     </row>
@@ -3973,7 +3970,7 @@
         <v>594330.59500000009</v>
       </c>
       <c r="G35">
-        <f>F35/1000</f>
+        <f t="shared" si="1"/>
         <v>594.33059500000013</v>
       </c>
     </row>
@@ -3992,7 +3989,7 @@
         <v>85227.5</v>
       </c>
       <c r="G36">
-        <f>F36/1000</f>
+        <f t="shared" si="1"/>
         <v>85.227500000000006</v>
       </c>
     </row>
@@ -4011,7 +4008,7 @@
         <v>1503.4349999999999</v>
       </c>
       <c r="G37">
-        <f>F37/1000</f>
+        <f t="shared" si="1"/>
         <v>1.5034349999999999</v>
       </c>
     </row>
@@ -4030,7 +4027,7 @@
         <v>14965</v>
       </c>
       <c r="G38">
-        <f>F38/1000</f>
+        <f t="shared" si="1"/>
         <v>14.965</v>
       </c>
       <c r="H38" t="s">
@@ -4055,7 +4052,7 @@
         <v>123041.50000000001</v>
       </c>
       <c r="G39">
-        <f>F39/1000</f>
+        <f t="shared" si="1"/>
         <v>123.04150000000001</v>
       </c>
     </row>
@@ -4074,7 +4071,7 @@
         <v>123041.50000000001</v>
       </c>
       <c r="G40">
-        <f>F40/1000</f>
+        <f t="shared" si="1"/>
         <v>123.04150000000001</v>
       </c>
       <c r="H40" t="s">
@@ -4099,7 +4096,7 @@
         <v>415406.49999999994</v>
       </c>
       <c r="G41">
-        <f>F41/1000</f>
+        <f t="shared" si="1"/>
         <v>415.40649999999994</v>
       </c>
       <c r="H41" t="s">
@@ -4121,7 +4118,7 @@
         <v>22389.582165</v>
       </c>
       <c r="G42">
-        <f>F42/1000</f>
+        <f t="shared" si="1"/>
         <v>22.389582165</v>
       </c>
     </row>
@@ -4140,13 +4137,13 @@
         <v>24710.5</v>
       </c>
       <c r="G43">
-        <f>F43/1000</f>
+        <f t="shared" si="1"/>
         <v>24.7105</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B44" t="s">
         <v>42</v>
@@ -4162,7 +4159,7 @@
         <v>177791.5</v>
       </c>
       <c r="G44">
-        <f>F44/1000</f>
+        <f t="shared" si="1"/>
         <v>177.79150000000001</v>
       </c>
       <c r="H44" t="s">
@@ -4171,7 +4168,7 @@
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B45" t="s">
         <v>32</v>
@@ -4184,7 +4181,7 @@
         <v>23659.3</v>
       </c>
       <c r="G45">
-        <f>F45/1000</f>
+        <f t="shared" si="1"/>
         <v>23.659299999999998</v>
       </c>
     </row>
@@ -4203,7 +4200,7 @@
         <v>81906</v>
       </c>
       <c r="G46">
-        <f>F46/1000</f>
+        <f t="shared" si="1"/>
         <v>81.906000000000006</v>
       </c>
     </row>
@@ -4222,7 +4219,7 @@
         <v>52560</v>
       </c>
       <c r="G47">
-        <f>F47/1000</f>
+        <f t="shared" si="1"/>
         <v>52.56</v>
       </c>
     </row>
@@ -4241,7 +4238,7 @@
         <v>11972.821250000003</v>
       </c>
       <c r="G48">
-        <f>F48/1000</f>
+        <f t="shared" si="1"/>
         <v>11.972821250000003</v>
       </c>
     </row>
@@ -4260,7 +4257,7 @@
         <v>98550</v>
       </c>
       <c r="G49">
-        <f>F49/1000</f>
+        <f t="shared" si="1"/>
         <v>98.55</v>
       </c>
     </row>
@@ -4279,7 +4276,7 @@
         <v>81395</v>
       </c>
       <c r="G50">
-        <f>F50/1000</f>
+        <f t="shared" si="1"/>
         <v>81.394999999999996</v>
       </c>
     </row>
@@ -4298,7 +4295,7 @@
         <v>60068.78</v>
       </c>
       <c r="G51">
-        <f>F51/1000</f>
+        <f t="shared" si="1"/>
         <v>60.068779999999997</v>
       </c>
     </row>
@@ -4317,7 +4314,7 @@
         <v>17728.05</v>
       </c>
       <c r="G52">
-        <f>F52/1000</f>
+        <f t="shared" si="1"/>
         <v>17.72805</v>
       </c>
     </row>
@@ -4336,7 +4333,7 @@
         <v>2810.5</v>
       </c>
       <c r="G53">
-        <f>F53/1000</f>
+        <f t="shared" si="1"/>
         <v>2.8105000000000002</v>
       </c>
     </row>
@@ -4355,7 +4352,7 @@
         <v>28251.000000000004</v>
       </c>
       <c r="G54">
-        <f>F54/1000</f>
+        <f t="shared" si="1"/>
         <v>28.251000000000005</v>
       </c>
     </row>
@@ -4374,7 +4371,7 @@
         <v>28287.5</v>
       </c>
       <c r="G55">
-        <f>F55/1000</f>
+        <f t="shared" si="1"/>
         <v>28.287500000000001</v>
       </c>
     </row>
@@ -4396,7 +4393,7 @@
         <v>51830</v>
       </c>
       <c r="G56">
-        <f>F56/1000</f>
+        <f t="shared" si="1"/>
         <v>51.83</v>
       </c>
     </row>
@@ -4415,7 +4412,7 @@
         <v>18572.295000000002</v>
       </c>
       <c r="G57">
-        <f>F57/1000</f>
+        <f t="shared" si="1"/>
         <v>18.572295</v>
       </c>
     </row>
@@ -4434,7 +4431,7 @@
         <v>70627.5</v>
       </c>
       <c r="G58">
-        <f>F58/1000</f>
+        <f t="shared" si="1"/>
         <v>70.627499999999998</v>
       </c>
     </row>
@@ -4453,7 +4450,7 @@
         <v>157461</v>
       </c>
       <c r="G59">
-        <f>F59/1000</f>
+        <f t="shared" si="1"/>
         <v>157.46100000000001</v>
       </c>
     </row>
@@ -4472,7 +4469,7 @@
         <v>10402.5</v>
       </c>
       <c r="G60">
-        <f>F60/1000</f>
+        <f t="shared" si="1"/>
         <v>10.4025</v>
       </c>
     </row>
@@ -4491,7 +4488,7 @@
         <v>24673.999999999996</v>
       </c>
       <c r="G61">
-        <f>F61/1000</f>
+        <f t="shared" si="1"/>
         <v>24.673999999999996</v>
       </c>
     </row>
@@ -4510,7 +4507,7 @@
         <v>41683</v>
       </c>
       <c r="G62">
-        <f>F62/1000</f>
+        <f t="shared" si="1"/>
         <v>41.683</v>
       </c>
     </row>
@@ -4529,7 +4526,7 @@
         <v>15320.342829999998</v>
       </c>
       <c r="G63">
-        <f>F63/1000</f>
+        <f t="shared" si="1"/>
         <v>15.320342829999998</v>
       </c>
     </row>
@@ -4548,7 +4545,7 @@
         <v>24710.5</v>
       </c>
       <c r="G64">
-        <f>F64/1000</f>
+        <f t="shared" si="1"/>
         <v>24.7105</v>
       </c>
     </row>
@@ -4567,7 +4564,7 @@
         <v>23761.499999999996</v>
       </c>
       <c r="G65">
-        <f>F65/1000</f>
+        <f t="shared" si="1"/>
         <v>23.761499999999998</v>
       </c>
     </row>
@@ -4589,7 +4586,7 @@
         <v>31025</v>
       </c>
       <c r="G66">
-        <f>F66/1000</f>
+        <f t="shared" ref="G66:G97" si="2">F66/1000</f>
         <v>31.024999999999999</v>
       </c>
     </row>
@@ -4611,7 +4608,7 @@
         <v>173667</v>
       </c>
       <c r="G67">
-        <f>F67/1000</f>
+        <f t="shared" si="2"/>
         <v>173.667</v>
       </c>
     </row>
@@ -4630,7 +4627,7 @@
         <v>161622</v>
       </c>
       <c r="G68">
-        <f>F68/1000</f>
+        <f t="shared" si="2"/>
         <v>161.62200000000001</v>
       </c>
     </row>
@@ -4649,7 +4646,7 @@
         <v>803.00000000000011</v>
       </c>
       <c r="G69">
-        <f>F69/1000</f>
+        <f t="shared" si="2"/>
         <v>0.80300000000000016</v>
       </c>
     </row>
@@ -4668,7 +4665,7 @@
         <v>29508.973952699998</v>
       </c>
       <c r="G70">
-        <f>F70/1000</f>
+        <f t="shared" si="2"/>
         <v>29.5089739527</v>
       </c>
     </row>
@@ -4687,7 +4684,7 @@
         <v>509978</v>
       </c>
       <c r="G71">
-        <f>F71/1000</f>
+        <f t="shared" si="2"/>
         <v>509.97800000000001</v>
       </c>
     </row>
@@ -4706,7 +4703,7 @@
         <v>702907.14500000002</v>
       </c>
       <c r="G72">
-        <f>F72/1000</f>
+        <f t="shared" si="2"/>
         <v>702.90714500000001</v>
       </c>
     </row>
@@ -4725,7 +4722,7 @@
         <v>180456</v>
       </c>
       <c r="G73">
-        <f>F73/1000</f>
+        <f t="shared" si="2"/>
         <v>180.45599999999999</v>
       </c>
     </row>
@@ -4747,7 +4744,7 @@
         <v>167754</v>
       </c>
       <c r="G74">
-        <f>F74/1000</f>
+        <f t="shared" si="2"/>
         <v>167.75399999999999</v>
       </c>
     </row>
@@ -4769,7 +4766,7 @@
         <v>455155</v>
       </c>
       <c r="G75">
-        <f>F75/1000</f>
+        <f t="shared" si="2"/>
         <v>455.15499999999997</v>
       </c>
     </row>
@@ -4791,7 +4788,7 @@
         <v>207502.5</v>
       </c>
       <c r="G76">
-        <f>F76/1000</f>
+        <f t="shared" si="2"/>
         <v>207.5025</v>
       </c>
     </row>
@@ -4810,7 +4807,7 @@
         <v>351714</v>
       </c>
       <c r="G77">
-        <f>F77/1000</f>
+        <f t="shared" si="2"/>
         <v>351.714</v>
       </c>
     </row>
@@ -4832,7 +4829,7 @@
         <v>513190</v>
       </c>
       <c r="G78">
-        <f>F78/1000</f>
+        <f t="shared" si="2"/>
         <v>513.19000000000005</v>
       </c>
     </row>
@@ -4851,7 +4848,7 @@
         <v>340034</v>
       </c>
       <c r="G79">
-        <f>F79/1000</f>
+        <f t="shared" si="2"/>
         <v>340.03399999999999</v>
       </c>
     </row>
@@ -4870,7 +4867,7 @@
         <v>29200</v>
       </c>
       <c r="G80">
-        <f>F80/1000</f>
+        <f t="shared" si="2"/>
         <v>29.2</v>
       </c>
     </row>
@@ -4889,7 +4886,7 @@
         <v>294098.75000000006</v>
       </c>
       <c r="G81">
-        <f>F81/1000</f>
+        <f t="shared" si="2"/>
         <v>294.09875000000005</v>
       </c>
     </row>
@@ -4908,7 +4905,7 @@
         <v>18359.5</v>
       </c>
       <c r="G82">
-        <f>F82/1000</f>
+        <f t="shared" si="2"/>
         <v>18.359500000000001</v>
       </c>
     </row>
@@ -4930,7 +4927,7 @@
         <v>5876.5000000000009</v>
       </c>
       <c r="G83">
-        <f>F83/1000</f>
+        <f t="shared" si="2"/>
         <v>5.8765000000000009</v>
       </c>
     </row>
@@ -4949,7 +4946,7 @@
         <v>44603</v>
       </c>
       <c r="G84">
-        <f>F84/1000</f>
+        <f t="shared" si="2"/>
         <v>44.603000000000002</v>
       </c>
     </row>
@@ -4968,7 +4965,7 @@
         <v>6562.7</v>
       </c>
       <c r="G85">
-        <f>F85/1000</f>
+        <f t="shared" si="2"/>
         <v>6.5626999999999995</v>
       </c>
     </row>
@@ -4987,7 +4984,7 @@
         <v>122369.9</v>
       </c>
       <c r="G86">
-        <f>F86/1000</f>
+        <f t="shared" si="2"/>
         <v>122.3699</v>
       </c>
     </row>
@@ -5006,7 +5003,7 @@
         <v>89717</v>
       </c>
       <c r="G87">
-        <f>F87/1000</f>
+        <f t="shared" si="2"/>
         <v>89.716999999999999</v>
       </c>
     </row>
@@ -5025,7 +5022,7 @@
         <v>439277.49999999994</v>
       </c>
       <c r="G88">
-        <f>F88/1000</f>
+        <f t="shared" si="2"/>
         <v>439.27749999999992</v>
       </c>
     </row>
@@ -5047,7 +5044,7 @@
         <v>513190</v>
       </c>
       <c r="G89">
-        <f>F89/1000</f>
+        <f t="shared" si="2"/>
         <v>513.19000000000005</v>
       </c>
     </row>
@@ -5063,7 +5060,7 @@
         <v>0</v>
       </c>
       <c r="G90">
-        <f>F90/1000</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -5085,7 +5082,7 @@
         <v>80300</v>
       </c>
       <c r="G91">
-        <f>F91/1000</f>
+        <f t="shared" si="2"/>
         <v>80.3</v>
       </c>
     </row>
@@ -5107,7 +5104,7 @@
         <v>61320</v>
       </c>
       <c r="G92">
-        <f>F92/1000</f>
+        <f t="shared" si="2"/>
         <v>61.32</v>
       </c>
     </row>
@@ -5126,7 +5123,7 @@
         <v>349998.5</v>
       </c>
       <c r="G93">
-        <f>F93/1000</f>
+        <f t="shared" si="2"/>
         <v>349.99849999999998</v>
       </c>
       <c r="H93" t="s">
@@ -5151,7 +5148,7 @@
         <v>486910</v>
       </c>
       <c r="G94">
-        <f>F94/1000</f>
+        <f t="shared" si="2"/>
         <v>486.91</v>
       </c>
     </row>
@@ -5170,7 +5167,7 @@
         <v>19600.5</v>
       </c>
       <c r="G95">
-        <f>F95/1000</f>
+        <f t="shared" si="2"/>
         <v>19.6005</v>
       </c>
     </row>
@@ -5189,7 +5186,7 @@
         <v>7847.5</v>
       </c>
       <c r="G96">
-        <f>F96/1000</f>
+        <f t="shared" si="2"/>
         <v>7.8475000000000001</v>
       </c>
     </row>
@@ -5208,7 +5205,7 @@
         <v>573196</v>
       </c>
       <c r="G97">
-        <f>F97/1000</f>
+        <f t="shared" si="2"/>
         <v>573.19600000000003</v>
       </c>
     </row>
@@ -5227,7 +5224,7 @@
         <v>167024</v>
       </c>
       <c r="G98">
-        <f>F98/1000</f>
+        <f t="shared" ref="G98:G129" si="3">F98/1000</f>
         <v>167.024</v>
       </c>
     </row>
@@ -5246,7 +5243,7 @@
         <v>47048.5</v>
       </c>
       <c r="G99">
-        <f>F99/1000</f>
+        <f t="shared" si="3"/>
         <v>47.048499999999997</v>
       </c>
     </row>
@@ -5268,7 +5265,7 @@
         <v>102492</v>
       </c>
       <c r="G100">
-        <f>F100/1000</f>
+        <f t="shared" si="3"/>
         <v>102.492</v>
       </c>
     </row>
@@ -5290,7 +5287,7 @@
         <v>415406.49999999994</v>
       </c>
       <c r="G101">
-        <f>F101/1000</f>
+        <f t="shared" si="3"/>
         <v>415.40649999999994</v>
       </c>
     </row>
@@ -5312,7 +5309,7 @@
         <v>210250.94999999998</v>
       </c>
       <c r="G102">
-        <f>F102/1000</f>
+        <f t="shared" si="3"/>
         <v>210.25094999999999</v>
       </c>
     </row>
@@ -5321,7 +5318,7 @@
         <v>47</v>
       </c>
       <c r="B103" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C103">
         <v>398.6</v>
@@ -5334,7 +5331,7 @@
         <v>144175</v>
       </c>
       <c r="G103">
-        <f>F103/1000</f>
+        <f t="shared" si="3"/>
         <v>144.17500000000001</v>
       </c>
     </row>
@@ -5356,7 +5353,7 @@
         <v>188194</v>
       </c>
       <c r="G104">
-        <f>F104/1000</f>
+        <f t="shared" si="3"/>
         <v>188.19399999999999</v>
       </c>
     </row>
@@ -5375,7 +5372,7 @@
         <v>93243.073199800012</v>
       </c>
       <c r="G105">
-        <f>F105/1000</f>
+        <f t="shared" si="3"/>
         <v>93.243073199800008</v>
       </c>
     </row>
@@ -5397,7 +5394,7 @@
         <v>49494</v>
       </c>
       <c r="G106">
-        <f>F106/1000</f>
+        <f t="shared" si="3"/>
         <v>49.494</v>
       </c>
     </row>
@@ -5419,7 +5416,7 @@
         <v>73584</v>
       </c>
       <c r="G107">
-        <f>F107/1000</f>
+        <f t="shared" si="3"/>
         <v>73.584000000000003</v>
       </c>
     </row>
@@ -5442,7 +5439,7 @@
         <v>816067.00000000012</v>
       </c>
       <c r="G108">
-        <f>F108/1000</f>
+        <f t="shared" si="3"/>
         <v>816.06700000000012</v>
       </c>
     </row>
@@ -5461,7 +5458,7 @@
         <v>82928</v>
       </c>
       <c r="G109">
-        <f>F109/1000</f>
+        <f t="shared" si="3"/>
         <v>82.927999999999997</v>
       </c>
     </row>
@@ -5483,7 +5480,7 @@
         <v>140525</v>
       </c>
       <c r="G110">
-        <f>F110/1000</f>
+        <f t="shared" si="3"/>
         <v>140.52500000000001</v>
       </c>
     </row>
@@ -5505,7 +5502,7 @@
         <v>67452</v>
       </c>
       <c r="G111">
-        <f>F111/1000</f>
+        <f t="shared" si="3"/>
         <v>67.451999999999998</v>
       </c>
     </row>
@@ -5999,7 +5996,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B26" t="s">
         <v>42</v>
@@ -6021,7 +6018,7 @@
         <v>97</v>
       </c>
       <c r="B27" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C27">
         <v>395</v>
@@ -6220,7 +6217,7 @@
         <v>180430.44999999998</v>
       </c>
       <c r="G2">
-        <f>F2/1000</f>
+        <f t="shared" ref="G2:G33" si="0">F2/1000</f>
         <v>180.43044999999998</v>
       </c>
     </row>
@@ -6239,7 +6236,7 @@
         <v>291246.64</v>
       </c>
       <c r="G3">
-        <f>F3/1000</f>
+        <f t="shared" si="0"/>
         <v>291.24664000000001</v>
       </c>
     </row>
@@ -6258,7 +6255,7 @@
         <v>55874.200000000004</v>
       </c>
       <c r="G4">
-        <f>F4/1000</f>
+        <f t="shared" si="0"/>
         <v>55.874200000000002</v>
       </c>
     </row>
@@ -6277,7 +6274,7 @@
         <v>429280.14999999997</v>
       </c>
       <c r="G5">
-        <f>F5/1000</f>
+        <f t="shared" si="0"/>
         <v>429.28014999999999</v>
       </c>
     </row>
@@ -6296,7 +6293,7 @@
         <v>41062.5</v>
       </c>
       <c r="G6">
-        <f>F6/1000</f>
+        <f t="shared" si="0"/>
         <v>41.0625</v>
       </c>
     </row>
@@ -6315,7 +6312,7 @@
         <v>140452</v>
       </c>
       <c r="G7">
-        <f>F7/1000</f>
+        <f t="shared" si="0"/>
         <v>140.452</v>
       </c>
     </row>
@@ -6334,7 +6331,7 @@
         <v>197830</v>
       </c>
       <c r="G8">
-        <f>F8/1000</f>
+        <f t="shared" si="0"/>
         <v>197.83</v>
       </c>
     </row>
@@ -6353,7 +6350,7 @@
         <v>193450</v>
       </c>
       <c r="G9">
-        <f>F9/1000</f>
+        <f t="shared" si="0"/>
         <v>193.45</v>
       </c>
     </row>
@@ -6375,7 +6372,7 @@
         <v>15320.342829999998</v>
       </c>
       <c r="G10">
-        <f>F10/1000</f>
+        <f t="shared" si="0"/>
         <v>15.320342829999998</v>
       </c>
     </row>
@@ -6394,7 +6391,7 @@
         <v>156220</v>
       </c>
       <c r="G11">
-        <f>F11/1000</f>
+        <f t="shared" si="0"/>
         <v>156.22</v>
       </c>
     </row>
@@ -6416,7 +6413,7 @@
         <v>75153.5</v>
       </c>
       <c r="G12">
-        <f>F12/1000</f>
+        <f t="shared" si="0"/>
         <v>75.153499999999994</v>
       </c>
     </row>
@@ -6425,7 +6422,7 @@
         <v>32</v>
       </c>
       <c r="B13" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C13">
         <v>120.36</v>
@@ -6435,7 +6432,7 @@
         <v>43931.4</v>
       </c>
       <c r="G13">
-        <f>F13/1000</f>
+        <f t="shared" si="0"/>
         <v>43.931400000000004</v>
       </c>
     </row>
@@ -6457,7 +6454,7 @@
         <v>12147.2</v>
       </c>
       <c r="G14">
-        <f>F14/1000</f>
+        <f t="shared" si="0"/>
         <v>12.147200000000002</v>
       </c>
     </row>
@@ -6476,7 +6473,7 @@
         <v>77282.91</v>
       </c>
       <c r="G15">
-        <f>F15/1000</f>
+        <f t="shared" si="0"/>
         <v>77.282910000000001</v>
       </c>
     </row>
@@ -6498,7 +6495,7 @@
         <v>167815.32</v>
       </c>
       <c r="G16">
-        <f>F16/1000</f>
+        <f t="shared" si="0"/>
         <v>167.81532000000001</v>
       </c>
     </row>
@@ -6517,7 +6514,7 @@
         <v>256156.99999999997</v>
       </c>
       <c r="G17">
-        <f>F17/1000</f>
+        <f t="shared" si="0"/>
         <v>256.15699999999998</v>
       </c>
       <c r="H17" t="s">
@@ -6539,7 +6536,7 @@
         <v>118770.99999999999</v>
       </c>
       <c r="G18">
-        <f>F18/1000</f>
+        <f t="shared" si="0"/>
         <v>118.77099999999999</v>
       </c>
       <c r="H18" t="s">
@@ -6561,7 +6558,7 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <f>F19/1000</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H19" t="s">
@@ -6583,7 +6580,7 @@
         <v>12969.074412800001</v>
       </c>
       <c r="G20">
-        <f>F20/1000</f>
+        <f t="shared" si="0"/>
         <v>12.969074412800001</v>
       </c>
     </row>
@@ -6602,7 +6599,7 @@
         <v>87600</v>
       </c>
       <c r="G21">
-        <f>F21/1000</f>
+        <f t="shared" si="0"/>
         <v>87.6</v>
       </c>
     </row>
@@ -6621,7 +6618,7 @@
         <v>36500</v>
       </c>
       <c r="G22">
-        <f>F22/1000</f>
+        <f t="shared" si="0"/>
         <v>36.5</v>
       </c>
     </row>
@@ -6640,7 +6637,7 @@
         <v>233775.2</v>
       </c>
       <c r="G23">
-        <f>F23/1000</f>
+        <f t="shared" si="0"/>
         <v>233.77520000000001</v>
       </c>
     </row>
@@ -6659,11 +6656,11 @@
         <v>136875</v>
       </c>
       <c r="G24">
-        <f>F24/1000</f>
+        <f t="shared" si="0"/>
         <v>136.875</v>
       </c>
       <c r="H24" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -6681,7 +6678,7 @@
         <v>350754.05</v>
       </c>
       <c r="G25">
-        <f>F25/1000</f>
+        <f t="shared" si="0"/>
         <v>350.75405000000001</v>
       </c>
     </row>
@@ -6700,7 +6697,7 @@
         <v>10230.950000000001</v>
       </c>
       <c r="G26">
-        <f>F26/1000</f>
+        <f t="shared" si="0"/>
         <v>10.23095</v>
       </c>
     </row>
@@ -6719,7 +6716,7 @@
         <v>510635</v>
       </c>
       <c r="G27">
-        <f>F27/1000</f>
+        <f t="shared" si="0"/>
         <v>510.63499999999999</v>
       </c>
     </row>
@@ -6738,7 +6735,7 @@
         <v>259493.23432000002</v>
       </c>
       <c r="G28">
-        <f>F28/1000</f>
+        <f t="shared" si="0"/>
         <v>259.49323432</v>
       </c>
     </row>
@@ -6757,7 +6754,7 @@
         <v>129940</v>
       </c>
       <c r="G29">
-        <f>F29/1000</f>
+        <f t="shared" si="0"/>
         <v>129.94</v>
       </c>
     </row>
@@ -6776,7 +6773,7 @@
         <v>129147.95</v>
       </c>
       <c r="G30">
-        <f>F30/1000</f>
+        <f t="shared" si="0"/>
         <v>129.14795000000001</v>
       </c>
     </row>
@@ -6795,7 +6792,7 @@
         <v>594220</v>
       </c>
       <c r="G31">
-        <f>F31/1000</f>
+        <f t="shared" si="0"/>
         <v>594.22</v>
       </c>
     </row>
@@ -6814,7 +6811,7 @@
         <v>45123.854999999996</v>
       </c>
       <c r="G32">
-        <f>F32/1000</f>
+        <f t="shared" si="0"/>
         <v>45.123854999999999</v>
       </c>
     </row>
@@ -6833,7 +6830,7 @@
         <v>224015.73656000002</v>
       </c>
       <c r="G33">
-        <f>F33/1000</f>
+        <f t="shared" si="0"/>
         <v>224.01573656000002</v>
       </c>
     </row>
@@ -6852,7 +6849,7 @@
         <v>8760</v>
       </c>
       <c r="G34">
-        <f>F34/1000</f>
+        <f t="shared" ref="G34:G65" si="1">F34/1000</f>
         <v>8.76</v>
       </c>
     </row>
@@ -6871,7 +6868,7 @@
         <v>552573.5</v>
       </c>
       <c r="G35">
-        <f>F35/1000</f>
+        <f t="shared" si="1"/>
         <v>552.57349999999997</v>
       </c>
     </row>
@@ -6890,7 +6887,7 @@
         <v>119092.2</v>
       </c>
       <c r="G36">
-        <f>F36/1000</f>
+        <f t="shared" si="1"/>
         <v>119.09219999999999</v>
       </c>
     </row>
@@ -6909,7 +6906,7 @@
         <v>5730.5</v>
       </c>
       <c r="G37">
-        <f>F37/1000</f>
+        <f t="shared" si="1"/>
         <v>5.7305000000000001</v>
       </c>
     </row>
@@ -6928,7 +6925,7 @@
         <v>117384.00000000001</v>
       </c>
       <c r="G38">
-        <f>F38/1000</f>
+        <f t="shared" si="1"/>
         <v>117.38400000000001</v>
       </c>
     </row>
@@ -6947,7 +6944,7 @@
         <v>10950</v>
       </c>
       <c r="G39">
-        <f>F39/1000</f>
+        <f t="shared" si="1"/>
         <v>10.95</v>
       </c>
       <c r="H39" t="s">
@@ -6972,7 +6969,7 @@
         <v>123041.50000000001</v>
       </c>
       <c r="G40">
-        <f>F40/1000</f>
+        <f t="shared" si="1"/>
         <v>123.04150000000001</v>
       </c>
     </row>
@@ -6991,7 +6988,7 @@
         <v>11650.800000000001</v>
       </c>
       <c r="G41">
-        <f>F41/1000</f>
+        <f t="shared" si="1"/>
         <v>11.6508</v>
       </c>
       <c r="H41" t="s">
@@ -7013,7 +7010,7 @@
         <v>421381.55</v>
       </c>
       <c r="G42">
-        <f>F42/1000</f>
+        <f t="shared" si="1"/>
         <v>421.38155</v>
       </c>
       <c r="H42" t="s">
@@ -7035,7 +7032,7 @@
         <v>22389.582165</v>
       </c>
       <c r="G43">
-        <f>F43/1000</f>
+        <f t="shared" si="1"/>
         <v>22.389582165</v>
       </c>
     </row>
@@ -7054,13 +7051,13 @@
         <v>24710.5</v>
       </c>
       <c r="G44">
-        <f>F44/1000</f>
+        <f t="shared" si="1"/>
         <v>24.7105</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B45" t="s">
         <v>42</v>
@@ -7073,7 +7070,7 @@
         <v>177791.5</v>
       </c>
       <c r="G45">
-        <f>F45/1000</f>
+        <f t="shared" si="1"/>
         <v>177.79150000000001</v>
       </c>
       <c r="H45" t="s">
@@ -7082,7 +7079,7 @@
     </row>
     <row r="46" spans="1:8">
       <c r="A46" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B46" t="s">
         <v>32</v>
@@ -7095,7 +7092,7 @@
         <v>62988.049999999996</v>
       </c>
       <c r="G46">
-        <f>F46/1000</f>
+        <f t="shared" si="1"/>
         <v>62.988049999999994</v>
       </c>
     </row>
@@ -7114,7 +7111,7 @@
         <v>81906</v>
       </c>
       <c r="G47">
-        <f>F47/1000</f>
+        <f t="shared" si="1"/>
         <v>81.906000000000006</v>
       </c>
     </row>
@@ -7133,7 +7130,7 @@
         <v>52560</v>
       </c>
       <c r="G48">
-        <f>F48/1000</f>
+        <f t="shared" si="1"/>
         <v>52.56</v>
       </c>
     </row>
@@ -7155,7 +7152,7 @@
         <v>11972.821250000003</v>
       </c>
       <c r="G49">
-        <f>F49/1000</f>
+        <f t="shared" si="1"/>
         <v>11.972821250000003</v>
       </c>
     </row>
@@ -7174,7 +7171,7 @@
         <v>98550</v>
       </c>
       <c r="G50">
-        <f>F50/1000</f>
+        <f t="shared" si="1"/>
         <v>98.55</v>
       </c>
     </row>
@@ -7193,7 +7190,7 @@
         <v>94542.299999999988</v>
       </c>
       <c r="G51">
-        <f>F51/1000</f>
+        <f t="shared" si="1"/>
         <v>94.542299999999983</v>
       </c>
     </row>
@@ -7212,7 +7209,7 @@
         <v>36500</v>
       </c>
       <c r="G52">
-        <f>F52/1000</f>
+        <f t="shared" si="1"/>
         <v>36.5</v>
       </c>
     </row>
@@ -7231,7 +7228,7 @@
         <v>60068.049999999996</v>
       </c>
       <c r="G53">
-        <f>F53/1000</f>
+        <f t="shared" si="1"/>
         <v>60.068049999999992</v>
       </c>
     </row>
@@ -7250,7 +7247,7 @@
         <v>18578.5</v>
       </c>
       <c r="G54">
-        <f>F54/1000</f>
+        <f t="shared" si="1"/>
         <v>18.578499999999998</v>
       </c>
     </row>
@@ -7269,7 +7266,7 @@
         <v>2810.5</v>
       </c>
       <c r="G55">
-        <f>F55/1000</f>
+        <f t="shared" si="1"/>
         <v>2.8105000000000002</v>
       </c>
     </row>
@@ -7288,7 +7285,7 @@
         <v>28178</v>
       </c>
       <c r="G56">
-        <f>F56/1000</f>
+        <f t="shared" si="1"/>
         <v>28.178000000000001</v>
       </c>
     </row>
@@ -7307,7 +7304,7 @@
         <v>28272.899999999998</v>
       </c>
       <c r="G57">
-        <f>F57/1000</f>
+        <f t="shared" si="1"/>
         <v>28.272899999999996</v>
       </c>
     </row>
@@ -7329,7 +7326,7 @@
         <v>51822.7</v>
       </c>
       <c r="G58">
-        <f>F58/1000</f>
+        <f t="shared" si="1"/>
         <v>51.822699999999998</v>
       </c>
     </row>
@@ -7348,7 +7345,7 @@
         <v>18571.2</v>
       </c>
       <c r="G59">
-        <f>F59/1000</f>
+        <f t="shared" si="1"/>
         <v>18.571200000000001</v>
       </c>
     </row>
@@ -7367,7 +7364,7 @@
         <v>70828.25</v>
       </c>
       <c r="G60">
-        <f>F60/1000</f>
+        <f t="shared" si="1"/>
         <v>70.828249999999997</v>
       </c>
     </row>
@@ -7386,7 +7383,7 @@
         <v>141565.25</v>
       </c>
       <c r="G61">
-        <f>F61/1000</f>
+        <f t="shared" si="1"/>
         <v>141.56524999999999</v>
       </c>
     </row>
@@ -7405,7 +7402,7 @@
         <v>14231.35</v>
       </c>
       <c r="G62">
-        <f>F62/1000</f>
+        <f t="shared" si="1"/>
         <v>14.231350000000001</v>
       </c>
     </row>
@@ -7424,7 +7421,7 @@
         <v>32850</v>
       </c>
       <c r="G63">
-        <f>F63/1000</f>
+        <f t="shared" si="1"/>
         <v>32.85</v>
       </c>
     </row>
@@ -7443,7 +7440,7 @@
         <v>21195.258000000002</v>
       </c>
       <c r="G64">
-        <f>F64/1000</f>
+        <f t="shared" si="1"/>
         <v>21.195258000000003</v>
       </c>
     </row>
@@ -7462,7 +7459,7 @@
         <v>0</v>
       </c>
       <c r="G65">
-        <f>F65/1000</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="H65" t="s">
@@ -7484,7 +7481,7 @@
         <v>15320.342829999998</v>
       </c>
       <c r="G66">
-        <f>F66/1000</f>
+        <f t="shared" ref="G66:G97" si="2">F66/1000</f>
         <v>15.320342829999998</v>
       </c>
     </row>
@@ -7503,7 +7500,7 @@
         <v>24710.5</v>
       </c>
       <c r="G67">
-        <f>F67/1000</f>
+        <f t="shared" si="2"/>
         <v>24.7105</v>
       </c>
     </row>
@@ -7522,7 +7519,7 @@
         <v>29930</v>
       </c>
       <c r="G68">
-        <f>F68/1000</f>
+        <f t="shared" si="2"/>
         <v>29.93</v>
       </c>
     </row>
@@ -7541,7 +7538,7 @@
         <v>0</v>
       </c>
       <c r="G69">
-        <f>F69/1000</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -7560,7 +7557,7 @@
         <v>180200.5</v>
       </c>
       <c r="G70">
-        <f>F70/1000</f>
+        <f t="shared" si="2"/>
         <v>180.20050000000001</v>
       </c>
       <c r="H70" t="s">
@@ -7582,7 +7579,7 @@
         <v>11650.800000000001</v>
       </c>
       <c r="G71">
-        <f>F71/1000</f>
+        <f t="shared" si="2"/>
         <v>11.6508</v>
       </c>
     </row>
@@ -7601,7 +7598,7 @@
         <v>803.00000000000011</v>
       </c>
       <c r="G72">
-        <f>F72/1000</f>
+        <f t="shared" si="2"/>
         <v>0.80300000000000016</v>
       </c>
     </row>
@@ -7620,7 +7617,7 @@
         <v>29508.973952699998</v>
       </c>
       <c r="G73">
-        <f>F73/1000</f>
+        <f t="shared" si="2"/>
         <v>29.5089739527</v>
       </c>
     </row>
@@ -7639,7 +7636,7 @@
         <v>506460.66143999994</v>
       </c>
       <c r="G74">
-        <f>F74/1000</f>
+        <f t="shared" si="2"/>
         <v>506.46066143999991</v>
       </c>
     </row>
@@ -7658,7 +7655,7 @@
         <v>674939.75000000012</v>
       </c>
       <c r="G75">
-        <f>F75/1000</f>
+        <f t="shared" si="2"/>
         <v>674.93975000000012</v>
       </c>
     </row>
@@ -7677,7 +7674,7 @@
         <v>180456</v>
       </c>
       <c r="G76">
-        <f>F76/1000</f>
+        <f t="shared" si="2"/>
         <v>180.45599999999999</v>
       </c>
     </row>
@@ -7699,7 +7696,7 @@
         <v>165418</v>
       </c>
       <c r="G77">
-        <f>F77/1000</f>
+        <f t="shared" si="2"/>
         <v>165.41800000000001</v>
       </c>
     </row>
@@ -7721,7 +7718,7 @@
         <v>447490</v>
       </c>
       <c r="G78">
-        <f>F78/1000</f>
+        <f t="shared" si="2"/>
         <v>447.49</v>
       </c>
     </row>
@@ -7743,7 +7740,7 @@
         <v>207502.5</v>
       </c>
       <c r="G79">
-        <f>F79/1000</f>
+        <f t="shared" si="2"/>
         <v>207.5025</v>
       </c>
     </row>
@@ -7762,7 +7759,7 @@
         <v>351714</v>
       </c>
       <c r="G80">
-        <f>F80/1000</f>
+        <f t="shared" si="2"/>
         <v>351.714</v>
       </c>
     </row>
@@ -7784,7 +7781,7 @@
         <v>513190</v>
       </c>
       <c r="G81">
-        <f>F81/1000</f>
+        <f t="shared" si="2"/>
         <v>513.19000000000005</v>
       </c>
     </row>
@@ -7803,7 +7800,7 @@
         <v>32.85</v>
       </c>
       <c r="G82">
-        <f>F82/1000</f>
+        <f t="shared" si="2"/>
         <v>3.2850000000000004E-2</v>
       </c>
     </row>
@@ -7822,7 +7819,7 @@
         <v>33288</v>
       </c>
       <c r="G83">
-        <f>F83/1000</f>
+        <f t="shared" si="2"/>
         <v>33.287999999999997</v>
       </c>
     </row>
@@ -7841,7 +7838,7 @@
         <v>63488.1</v>
       </c>
       <c r="G84">
-        <f>F84/1000</f>
+        <f t="shared" si="2"/>
         <v>63.488099999999996</v>
       </c>
     </row>
@@ -7860,7 +7857,7 @@
         <v>29200</v>
       </c>
       <c r="G85">
-        <f>F85/1000</f>
+        <f t="shared" si="2"/>
         <v>29.2</v>
       </c>
     </row>
@@ -7879,7 +7876,7 @@
         <v>84467.205000000002</v>
       </c>
       <c r="G86">
-        <f>F86/1000</f>
+        <f t="shared" si="2"/>
         <v>84.467205000000007</v>
       </c>
     </row>
@@ -7898,7 +7895,7 @@
         <v>26780.050000000003</v>
       </c>
       <c r="G87">
-        <f>F87/1000</f>
+        <f t="shared" si="2"/>
         <v>26.780050000000003</v>
       </c>
     </row>
@@ -7920,7 +7917,7 @@
         <v>20330.5</v>
       </c>
       <c r="G88">
-        <f>F88/1000</f>
+        <f t="shared" si="2"/>
         <v>20.330500000000001</v>
       </c>
     </row>
@@ -7939,7 +7936,7 @@
         <v>44603</v>
       </c>
       <c r="G89">
-        <f>F89/1000</f>
+        <f t="shared" si="2"/>
         <v>44.603000000000002</v>
       </c>
     </row>
@@ -7958,7 +7955,7 @@
         <v>5110</v>
       </c>
       <c r="G90">
-        <f>F90/1000</f>
+        <f t="shared" si="2"/>
         <v>5.1100000000000003</v>
       </c>
     </row>
@@ -7977,7 +7974,7 @@
         <v>127790.88</v>
       </c>
       <c r="G91">
-        <f>F91/1000</f>
+        <f t="shared" si="2"/>
         <v>127.79088</v>
       </c>
     </row>
@@ -7996,7 +7993,7 @@
         <v>89717</v>
       </c>
       <c r="G92">
-        <f>F92/1000</f>
+        <f t="shared" si="2"/>
         <v>89.716999999999999</v>
       </c>
     </row>
@@ -8015,7 +8012,7 @@
         <v>439277.49999999994</v>
       </c>
       <c r="G93">
-        <f>F93/1000</f>
+        <f t="shared" si="2"/>
         <v>439.27749999999992</v>
       </c>
     </row>
@@ -8034,7 +8031,7 @@
         <v>0</v>
       </c>
       <c r="G94">
-        <f>F94/1000</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8050,7 +8047,7 @@
         <v>0</v>
       </c>
       <c r="G95">
-        <f>F95/1000</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8069,7 +8066,7 @@
         <v>0</v>
       </c>
       <c r="G96">
-        <f>F96/1000</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8088,7 +8085,7 @@
         <v>0</v>
       </c>
       <c r="G97">
-        <f>F97/1000</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -8107,7 +8104,7 @@
         <v>349998.5</v>
       </c>
       <c r="G98">
-        <f>F98/1000</f>
+        <f t="shared" ref="G98:G129" si="3">F98/1000</f>
         <v>349.99849999999998</v>
       </c>
       <c r="H98" t="s">
@@ -8129,7 +8126,7 @@
         <v>1992720.7302134999</v>
       </c>
       <c r="G99">
-        <f>F99/1000</f>
+        <f t="shared" si="3"/>
         <v>1992.7207302134998</v>
       </c>
     </row>
@@ -8148,7 +8145,7 @@
         <v>19600.5</v>
       </c>
       <c r="G100">
-        <f>F100/1000</f>
+        <f t="shared" si="3"/>
         <v>19.6005</v>
       </c>
     </row>
@@ -8167,7 +8164,7 @@
         <v>9406.0499999999993</v>
       </c>
       <c r="G101">
-        <f>F101/1000</f>
+        <f t="shared" si="3"/>
         <v>9.4060499999999987</v>
       </c>
     </row>
@@ -8186,7 +8183,7 @@
         <v>623675.5</v>
       </c>
       <c r="G102">
-        <f>F102/1000</f>
+        <f t="shared" si="3"/>
         <v>623.67550000000006</v>
       </c>
     </row>
@@ -8205,7 +8202,7 @@
         <v>144248</v>
       </c>
       <c r="G103">
-        <f>F103/1000</f>
+        <f t="shared" si="3"/>
         <v>144.24799999999999</v>
       </c>
     </row>
@@ -8224,7 +8221,7 @@
         <v>47074.05</v>
       </c>
       <c r="G104">
-        <f>F104/1000</f>
+        <f t="shared" si="3"/>
         <v>47.07405</v>
       </c>
     </row>
@@ -8243,7 +8240,7 @@
         <v>52743.96</v>
       </c>
       <c r="G105">
-        <f>F105/1000</f>
+        <f t="shared" si="3"/>
         <v>52.743960000000001</v>
       </c>
     </row>
@@ -8265,7 +8262,7 @@
         <v>102492</v>
       </c>
       <c r="G106">
-        <f>F106/1000</f>
+        <f t="shared" si="3"/>
         <v>102.492</v>
       </c>
     </row>
@@ -8287,7 +8284,7 @@
         <v>421210</v>
       </c>
       <c r="G107">
-        <f>F107/1000</f>
+        <f t="shared" si="3"/>
         <v>421.21</v>
       </c>
       <c r="H107" t="s">
@@ -8309,7 +8306,7 @@
         <v>210250.94999999998</v>
       </c>
       <c r="G108">
-        <f>F108/1000</f>
+        <f t="shared" si="3"/>
         <v>210.25094999999999</v>
       </c>
     </row>
@@ -8318,7 +8315,7 @@
         <v>47</v>
       </c>
       <c r="B109" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C109">
         <v>398.6</v>
@@ -8328,7 +8325,7 @@
         <v>145489</v>
       </c>
       <c r="G109">
-        <f>F109/1000</f>
+        <f t="shared" si="3"/>
         <v>145.489</v>
       </c>
     </row>
@@ -8347,7 +8344,7 @@
         <v>30941.05</v>
       </c>
       <c r="G110">
-        <f>F110/1000</f>
+        <f t="shared" si="3"/>
         <v>30.941050000000001</v>
       </c>
     </row>
@@ -8366,7 +8363,7 @@
         <v>93243.073199800012</v>
       </c>
       <c r="G111">
-        <f>F111/1000</f>
+        <f t="shared" si="3"/>
         <v>93.243073199800008</v>
       </c>
     </row>
@@ -8385,7 +8382,7 @@
         <v>49494</v>
       </c>
       <c r="G112">
-        <f>F112/1000</f>
+        <f t="shared" si="3"/>
         <v>49.494</v>
       </c>
       <c r="H112" t="s">
@@ -8410,7 +8407,7 @@
         <v>0</v>
       </c>
       <c r="G113">
-        <f>F113/1000</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="H113" t="s">
@@ -8435,7 +8432,7 @@
         <v>91104</v>
       </c>
       <c r="G114">
-        <f>F114/1000</f>
+        <f t="shared" si="3"/>
         <v>91.103999999999999</v>
       </c>
     </row>
@@ -8457,7 +8454,7 @@
         <v>75153.5</v>
       </c>
       <c r="G115">
-        <f>F115/1000</f>
+        <f t="shared" si="3"/>
         <v>75.153499999999994</v>
       </c>
     </row>
@@ -8479,7 +8476,7 @@
         <v>140525</v>
       </c>
       <c r="G116">
-        <f>F116/1000</f>
+        <f t="shared" si="3"/>
         <v>140.52500000000001</v>
       </c>
     </row>
@@ -8498,7 +8495,7 @@
         <v>61320</v>
       </c>
       <c r="G117">
-        <f>F117/1000</f>
+        <f t="shared" si="3"/>
         <v>61.32</v>
       </c>
     </row>
@@ -8529,7 +8526,7 @@
         <v>94</v>
       </c>
       <c r="C1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D1" t="s">
         <v>107</v>
@@ -8538,19 +8535,19 @@
         <v>108</v>
       </c>
       <c r="F1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H1" t="s">
         <v>259</v>
       </c>
       <c r="I1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="L1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -8575,7 +8572,7 @@
         <v>5000</v>
       </c>
       <c r="I2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -8601,7 +8598,7 @@
         <v>850</v>
       </c>
       <c r="I3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -8627,7 +8624,7 @@
         <v>2400</v>
       </c>
       <c r="I4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -8635,7 +8632,7 @@
         <v>151</v>
       </c>
       <c r="B5" t="s">
-        <v>260</v>
+        <v>198</v>
       </c>
       <c r="C5">
         <v>500</v>
@@ -8656,12 +8653,12 @@
         <v>4828.0334936776799</v>
       </c>
       <c r="I5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>260</v>
+        <v>198</v>
       </c>
       <c r="B6" t="s">
         <v>151</v>
@@ -8685,7 +8682,7 @@
         <v>4828.0334936776799</v>
       </c>
       <c r="I6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -8710,7 +8707,7 @@
         <v>7378</v>
       </c>
       <c r="I7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -8736,7 +8733,7 @@
         <v>1000</v>
       </c>
       <c r="I8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -8761,7 +8758,7 @@
         <v>1200</v>
       </c>
       <c r="I9" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -8787,7 +8784,7 @@
         <v>200</v>
       </c>
       <c r="I10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -8816,7 +8813,7 @@
         <v>370.14923451528881</v>
       </c>
       <c r="I11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -8845,7 +8842,7 @@
         <v>370.14923451528881</v>
       </c>
       <c r="I12" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -8870,7 +8867,7 @@
         <v>2520</v>
       </c>
       <c r="I13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -10382,7 +10379,7 @@
         <v>185</v>
       </c>
       <c r="B65" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E65">
         <f t="shared" si="7"/>
@@ -10801,7 +10798,7 @@
         <v>181</v>
       </c>
       <c r="B82" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E82">
         <f t="shared" si="9"/>
@@ -11175,7 +11172,7 @@
         <v>183</v>
       </c>
       <c r="B99" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E99">
         <f t="shared" si="10"/>
@@ -11555,7 +11552,7 @@
         <v>184</v>
       </c>
       <c r="B116" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E116">
         <f t="shared" si="11"/>
@@ -11974,7 +11971,7 @@
         <v>186</v>
       </c>
       <c r="B133" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E133">
         <f t="shared" si="12"/>
@@ -12354,7 +12351,7 @@
         <v>187</v>
       </c>
       <c r="B150" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E150">
         <f t="shared" si="13"/>
@@ -12773,7 +12770,7 @@
         <v>193</v>
       </c>
       <c r="B167" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E167">
         <f t="shared" si="14"/>
@@ -13153,7 +13150,7 @@
         <v>196</v>
       </c>
       <c r="B184" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E184">
         <f t="shared" si="15"/>
@@ -13572,7 +13569,7 @@
         <v>195</v>
       </c>
       <c r="B201" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E201">
         <f t="shared" si="16"/>
@@ -13784,7 +13781,7 @@
         <v>4612.3813309600764</v>
       </c>
       <c r="I210" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="211" spans="1:9">
@@ -14033,7 +14030,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C4">
         <v>7</v>
@@ -14057,7 +14054,7 @@
         <v>73.274999999999991</v>
       </c>
       <c r="J4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="K4" t="s">
         <v>102</v>
@@ -14704,10 +14701,10 @@
         <v>123</v>
       </c>
       <c r="F1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="G1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="M1" t="s">
         <v>93</v>
@@ -15181,7 +15178,7 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B16" t="s">
         <v>3</v>
@@ -16147,10 +16144,10 @@
         <v>173</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -18163,7 +18160,7 @@
         <v>120</v>
       </c>
       <c r="G1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -18476,7 +18473,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B14" t="s">
         <v>3</v>
@@ -19279,7 +19276,7 @@
         <v>173</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>106</v>
@@ -20100,7 +20097,7 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B14" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
update global LNG connections 2020
update the port to port information
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B42ED01F-8A1D-48E4-BB38-7E3D3D4DC2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C918F4-F712-4020-8DA5-1C33F77A146A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="10" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng_europe_2020" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2644" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2652" uniqueCount="295">
   <si>
     <t>Belgium</t>
   </si>
@@ -894,6 +894,48 @@
   </si>
   <si>
     <t>for Morroco</t>
+  </si>
+  <si>
+    <t>Tianjin</t>
+  </si>
+  <si>
+    <t>Livorno</t>
+  </si>
+  <si>
+    <t>Hong Kong</t>
+  </si>
+  <si>
+    <t>Wadi Feiran</t>
+  </si>
+  <si>
+    <t>Montoir</t>
+  </si>
+  <si>
+    <t>Istanbul</t>
+  </si>
+  <si>
+    <t>Isle of Grain</t>
+  </si>
+  <si>
+    <t>AF from Bonny Inshore Terminal (Nigeria)</t>
+  </si>
+  <si>
+    <t>Cartagena</t>
+  </si>
+  <si>
+    <t>EG from Port Said and Alexandria</t>
+  </si>
+  <si>
+    <t>Shanghai</t>
+  </si>
+  <si>
+    <t>Kavala</t>
+  </si>
+  <si>
+    <t>Venice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RU from Sabetta (Murmansk plus 1200 mi to west, minus 1200 mi to east as Murmansk is the closest port) except for JS, there it's from Vladivostok </t>
   </si>
 </sst>
 </file>
@@ -1762,7 +1804,13 @@
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I172" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
-  <autoFilter ref="A1:I172" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
+  <autoFilter ref="A1:I172" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="Wadi Feiran"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
     <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
@@ -8928,7 +8976,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" hidden="1">
       <c r="A2" t="s">
         <v>180</v>
       </c>
@@ -8953,7 +9001,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" hidden="1">
       <c r="A3" t="s">
         <v>180</v>
       </c>
@@ -8978,7 +9026,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" hidden="1">
       <c r="A4" t="s">
         <v>180</v>
       </c>
@@ -8990,23 +9038,23 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>10194</v>
+        <v>10339</v>
       </c>
       <c r="G4">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>16405.657811516758</v>
+        <v>16639.012763711176</v>
       </c>
       <c r="H4" t="s">
         <v>241</v>
       </c>
       <c r="I4" t="s">
-        <v>242</v>
+        <v>281</v>
       </c>
       <c r="M4" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" hidden="1">
       <c r="A5" t="s">
         <v>180</v>
       </c>
@@ -9034,7 +9082,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" hidden="1">
       <c r="A6" t="s">
         <v>180</v>
       </c>
@@ -9059,10 +9107,10 @@
         <v>244</v>
       </c>
       <c r="M6" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" hidden="1">
       <c r="A7" t="s">
         <v>180</v>
       </c>
@@ -9102,20 +9150,23 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>6681</v>
+        <v>6850</v>
       </c>
       <c r="G8">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10752.030590420192</v>
+        <v>11024.009810564035</v>
+      </c>
+      <c r="H8" t="s">
+        <v>213</v>
       </c>
       <c r="I8" t="s">
-        <v>246</v>
+        <v>284</v>
       </c>
       <c r="M8" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" hidden="1">
       <c r="A9" t="s">
         <v>182</v>
       </c>
@@ -9140,7 +9191,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" hidden="1">
       <c r="A10" t="s">
         <v>182</v>
       </c>
@@ -9162,10 +9213,10 @@
         <v>240</v>
       </c>
       <c r="M10" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" hidden="1">
       <c r="A11" t="s">
         <v>182</v>
       </c>
@@ -9177,20 +9228,20 @@
         <v>0</v>
       </c>
       <c r="F11">
-        <v>9806</v>
+        <v>9750</v>
       </c>
       <c r="G11">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>15781.232146334443</v>
+        <v>15691.108854452459</v>
       </c>
       <c r="H11" t="s">
         <v>241</v>
       </c>
       <c r="I11" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" hidden="1">
       <c r="A12" t="s">
         <v>182</v>
       </c>
@@ -9215,7 +9266,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" hidden="1">
       <c r="A13" t="s">
         <v>182</v>
       </c>
@@ -9240,7 +9291,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:13" hidden="1">
       <c r="A14" t="s">
         <v>182</v>
       </c>
@@ -9277,17 +9328,20 @@
         <v>0</v>
       </c>
       <c r="F15">
-        <v>5324</v>
+        <v>5493</v>
       </c>
       <c r="G15">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8568.1501067799891</v>
+        <v>8840.1293269238322</v>
+      </c>
+      <c r="H15" t="s">
+        <v>213</v>
       </c>
       <c r="I15" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" hidden="1">
       <c r="A16" t="s">
         <v>183</v>
       </c>
@@ -9309,7 +9363,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" hidden="1">
       <c r="A17" t="s">
         <v>183</v>
       </c>
@@ -9331,7 +9385,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" hidden="1">
       <c r="A18" t="s">
         <v>183</v>
       </c>
@@ -9343,17 +9397,17 @@
         <v>0</v>
       </c>
       <c r="F18">
-        <v>6160</v>
+        <v>5001</v>
       </c>
       <c r="G18">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9913.5621070181696</v>
+        <v>8048.3318339606922</v>
       </c>
       <c r="I18" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" hidden="1">
       <c r="A19" t="s">
         <v>183</v>
       </c>
@@ -9375,7 +9429,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" hidden="1">
       <c r="A20" t="s">
         <v>183</v>
       </c>
@@ -9397,7 +9451,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" hidden="1">
       <c r="A21" t="s">
         <v>183</v>
       </c>
@@ -9419,7 +9473,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" hidden="1">
       <c r="A22" t="s">
         <v>183</v>
       </c>
@@ -9441,7 +9495,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" hidden="1">
       <c r="A23" t="s">
         <v>184</v>
       </c>
@@ -9463,7 +9517,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" hidden="1">
       <c r="A24" t="s">
         <v>184</v>
       </c>
@@ -9485,7 +9539,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" hidden="1">
       <c r="A25" t="s">
         <v>184</v>
       </c>
@@ -9497,17 +9551,17 @@
         <v>0</v>
       </c>
       <c r="F25">
-        <v>6227</v>
+        <v>5845</v>
       </c>
       <c r="G25">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10021.38818837697</v>
+        <v>9406.6185901820136</v>
       </c>
       <c r="I25" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" hidden="1">
       <c r="A26" t="s">
         <v>184</v>
       </c>
@@ -9529,7 +9583,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" hidden="1">
       <c r="A27" t="s">
         <v>184</v>
       </c>
@@ -9551,7 +9605,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" hidden="1">
       <c r="A28" t="s">
         <v>184</v>
       </c>
@@ -9585,17 +9639,17 @@
         <v>0</v>
       </c>
       <c r="F29">
-        <v>2982</v>
+        <v>2906</v>
       </c>
       <c r="G29">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4799.0652927156134</v>
+        <v>4676.7551108757789</v>
       </c>
       <c r="I29" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" hidden="1">
       <c r="A30" t="s">
         <v>185</v>
       </c>
@@ -9607,17 +9661,17 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>3420</v>
+        <v>3392</v>
       </c>
       <c r="G30">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5503.9581827925549</v>
+        <v>5458.8965368515637</v>
       </c>
       <c r="I30" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" hidden="1">
       <c r="A31" t="s">
         <v>185</v>
       </c>
@@ -9629,17 +9683,17 @@
         <v>0</v>
       </c>
       <c r="F31">
-        <v>10496</v>
+        <v>9306</v>
       </c>
       <c r="G31">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>16891.679849880311</v>
+        <v>14976.559897388162</v>
       </c>
       <c r="I31" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" hidden="1">
       <c r="A32" t="s">
         <v>185</v>
       </c>
@@ -9651,17 +9705,17 @@
         <v>0</v>
       </c>
       <c r="F32">
-        <v>10780</v>
+        <v>10752</v>
       </c>
       <c r="G32">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>17348.733687281798</v>
+        <v>17303.672041340804</v>
       </c>
       <c r="I32" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:9" hidden="1">
       <c r="A33" t="s">
         <v>185</v>
       </c>
@@ -9673,17 +9727,17 @@
         <v>0</v>
       </c>
       <c r="F33">
-        <v>7016</v>
+        <v>7030</v>
       </c>
       <c r="G33">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11291.160997214201</v>
+        <v>11313.691820184697</v>
       </c>
       <c r="I33" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" hidden="1">
       <c r="A34" t="s">
         <v>185</v>
       </c>
@@ -9695,11 +9749,11 @@
         <v>0</v>
       </c>
       <c r="F34">
-        <v>8836</v>
+        <v>8808</v>
       </c>
       <c r="G34">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>14220.16798337866</v>
+        <v>14175.106337437668</v>
       </c>
       <c r="I34" t="s">
         <v>245</v>
@@ -9717,17 +9771,20 @@
         <v>0</v>
       </c>
       <c r="F35">
-        <v>5250</v>
+        <v>5391</v>
       </c>
       <c r="G35">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8449.0586139359402</v>
+        <v>8675.9761881387913</v>
+      </c>
+      <c r="H35" t="s">
+        <v>213</v>
       </c>
       <c r="I35" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" hidden="1">
       <c r="A36" t="s">
         <v>186</v>
       </c>
@@ -9749,7 +9806,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" hidden="1">
       <c r="A37" t="s">
         <v>186</v>
       </c>
@@ -9771,7 +9828,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" hidden="1">
       <c r="A38" t="s">
         <v>186</v>
       </c>
@@ -9783,17 +9840,17 @@
         <v>0</v>
       </c>
       <c r="F38">
-        <v>3175</v>
+        <v>2353</v>
       </c>
       <c r="G38">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5109.6687808088782</v>
+        <v>3786.7876035411937</v>
       </c>
       <c r="I38" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" hidden="1">
       <c r="A39" t="s">
         <v>186</v>
       </c>
@@ -9815,7 +9872,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" hidden="1">
       <c r="A40" t="s">
         <v>186</v>
       </c>
@@ -9827,17 +9884,17 @@
         <v>0</v>
       </c>
       <c r="F40">
-        <v>4180</v>
+        <v>4477</v>
       </c>
       <c r="G40">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6727.0600011909009</v>
+        <v>7205.0353170649905</v>
       </c>
       <c r="I40" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" hidden="1">
       <c r="A41" t="s">
         <v>186</v>
       </c>
@@ -9871,17 +9928,17 @@
         <v>0</v>
       </c>
       <c r="F42">
-        <v>6655</v>
+        <v>6579</v>
       </c>
       <c r="G42">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10710.187633474987</v>
+        <v>10587.877451635151</v>
       </c>
       <c r="I42" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" hidden="1">
       <c r="A43" t="s">
         <v>194</v>
       </c>
@@ -9903,7 +9960,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="44" spans="1:9">
+    <row r="44" spans="1:9" hidden="1">
       <c r="A44" t="s">
         <v>194</v>
       </c>
@@ -9925,7 +9982,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:9" hidden="1">
       <c r="A45" t="s">
         <v>194</v>
       </c>
@@ -9937,20 +9994,20 @@
         <v>0</v>
       </c>
       <c r="F45">
-        <v>13641</v>
+        <v>13259</v>
       </c>
       <c r="G45">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>21953.068295752411</v>
+        <v>21338.298697557453</v>
       </c>
       <c r="H45" t="s">
         <v>213</v>
       </c>
       <c r="I45" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" hidden="1">
       <c r="A46" t="s">
         <v>194</v>
       </c>
@@ -9972,7 +10029,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="47" spans="1:9">
+    <row r="47" spans="1:9" hidden="1">
       <c r="A47" t="s">
         <v>194</v>
       </c>
@@ -9997,7 +10054,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" hidden="1">
       <c r="A48" t="s">
         <v>194</v>
       </c>
@@ -10034,17 +10091,20 @@
         <v>0</v>
       </c>
       <c r="F49">
-        <v>6008</v>
+        <v>6177</v>
       </c>
       <c r="G49">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9668.9417433385006</v>
+        <v>9940.9209634823437</v>
+      </c>
+      <c r="H49" t="s">
+        <v>213</v>
       </c>
       <c r="I49" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" hidden="1">
       <c r="A50" t="s">
         <v>192</v>
       </c>
@@ -10056,17 +10116,17 @@
         <v>0</v>
       </c>
       <c r="F50">
-        <v>6103</v>
+        <v>5988</v>
       </c>
       <c r="G50">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9821.8294706382931</v>
+        <v>9636.7548533806494</v>
       </c>
       <c r="I50" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="51" spans="1:9">
+    <row r="51" spans="1:9" hidden="1">
       <c r="A51" t="s">
         <v>192</v>
       </c>
@@ -10078,17 +10138,17 @@
         <v>0</v>
       </c>
       <c r="F51">
-        <v>5250</v>
+        <v>5135</v>
       </c>
       <c r="G51">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8449.0586139359402</v>
+        <v>8263.9839966782947</v>
       </c>
       <c r="I51" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="52" spans="1:9">
+    <row r="52" spans="1:9" hidden="1">
       <c r="A52" t="s">
         <v>192</v>
       </c>
@@ -10100,17 +10160,20 @@
         <v>0</v>
       </c>
       <c r="F52">
-        <v>7546</v>
+        <v>7934</v>
       </c>
       <c r="G52">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>12144.113581097257</v>
+        <v>12768.53924627957</v>
+      </c>
+      <c r="H52" t="s">
+        <v>213</v>
       </c>
       <c r="I52" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" hidden="1">
       <c r="A53" t="s">
         <v>192</v>
       </c>
@@ -10122,17 +10185,20 @@
         <v>0</v>
       </c>
       <c r="F53">
-        <v>7831</v>
+        <v>8074</v>
       </c>
       <c r="G53">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>12602.776762996637</v>
+        <v>12993.847475984529</v>
+      </c>
+      <c r="H53" t="s">
+        <v>213</v>
       </c>
       <c r="I53" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="54" spans="1:9">
+    <row r="54" spans="1:9" hidden="1">
       <c r="A54" t="s">
         <v>192</v>
       </c>
@@ -10144,17 +10210,20 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>2800</v>
+        <v>3043</v>
       </c>
       <c r="G54">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4506.1645940991675</v>
+        <v>4897.2353070870604</v>
+      </c>
+      <c r="H54" t="s">
+        <v>213</v>
       </c>
       <c r="I54" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="55" spans="1:9">
+    <row r="55" spans="1:9" hidden="1">
       <c r="A55" t="s">
         <v>192</v>
       </c>
@@ -10166,17 +10235,20 @@
         <v>0</v>
       </c>
       <c r="F55">
-        <v>5758</v>
+        <v>6001</v>
       </c>
       <c r="G55">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9266.6056188653602</v>
+        <v>9657.6763318532521</v>
+      </c>
+      <c r="H55" t="s">
+        <v>213</v>
       </c>
       <c r="I55" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="56" spans="1:9">
+    <row r="56" spans="1:9" hidden="1">
       <c r="A56" t="s">
         <v>195</v>
       </c>
@@ -10198,7 +10270,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="57" spans="1:9">
+    <row r="57" spans="1:9" hidden="1">
       <c r="A57" t="s">
         <v>195</v>
       </c>
@@ -10220,7 +10292,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="58" spans="1:9">
+    <row r="58" spans="1:9" hidden="1">
       <c r="A58" t="s">
         <v>195</v>
       </c>
@@ -10232,17 +10304,17 @@
         <v>0</v>
       </c>
       <c r="F58">
-        <v>2583</v>
+        <v>2186</v>
       </c>
       <c r="G58">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4156.936838056482</v>
+        <v>3518.0270723931362</v>
       </c>
       <c r="I58" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" hidden="1">
       <c r="A59" t="s">
         <v>195</v>
       </c>
@@ -10264,7 +10336,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="60" spans="1:9">
+    <row r="60" spans="1:9" hidden="1">
       <c r="A60" t="s">
         <v>195</v>
       </c>
@@ -10276,17 +10348,17 @@
         <v>0</v>
       </c>
       <c r="F60">
-        <v>3463</v>
+        <v>3760</v>
       </c>
       <c r="G60">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5573.1599962019354</v>
+        <v>6051.135312076025</v>
       </c>
       <c r="I60" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" hidden="1">
       <c r="A61" t="s">
         <v>195</v>
       </c>
@@ -10320,17 +10392,17 @@
         <v>0</v>
       </c>
       <c r="F62">
-        <v>5942</v>
+        <v>5866</v>
       </c>
       <c r="G62">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9562.7250064775908</v>
+        <v>9440.4148246377572</v>
       </c>
       <c r="I62" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" hidden="1">
       <c r="A63" t="s">
         <v>184</v>
       </c>
@@ -10355,7 +10427,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="64" spans="1:9">
+    <row r="64" spans="1:9" hidden="1">
       <c r="A64" t="s">
         <v>184</v>
       </c>
@@ -10380,7 +10452,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="65" spans="1:9">
+    <row r="65" spans="1:9" hidden="1">
       <c r="A65" t="s">
         <v>184</v>
       </c>
@@ -10405,7 +10477,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="66" spans="1:9">
+    <row r="66" spans="1:9" hidden="1">
       <c r="A66" t="s">
         <v>184</v>
       </c>
@@ -10417,20 +10489,20 @@
         <v>0</v>
       </c>
       <c r="F66">
-        <v>4452</v>
+        <v>4380</v>
       </c>
       <c r="G66">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7164.8017046176765</v>
+        <v>7048.9289007694124</v>
       </c>
       <c r="H66" t="s">
         <v>213</v>
       </c>
       <c r="I66" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" hidden="1">
       <c r="A67" t="s">
         <v>184</v>
       </c>
@@ -10455,7 +10527,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="68" spans="1:9">
+    <row r="68" spans="1:9" hidden="1">
       <c r="A68" t="s">
         <v>184</v>
       </c>
@@ -10480,7 +10552,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="69" spans="1:9">
+    <row r="69" spans="1:9" hidden="1">
       <c r="A69" t="s">
         <v>184</v>
       </c>
@@ -10505,7 +10577,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="70" spans="1:9">
+    <row r="70" spans="1:9" hidden="1">
       <c r="A70" t="s">
         <v>184</v>
       </c>
@@ -10530,7 +10602,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="71" spans="1:9">
+    <row r="71" spans="1:9" hidden="1">
       <c r="A71" t="s">
         <v>184</v>
       </c>
@@ -10555,7 +10627,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="72" spans="1:9">
+    <row r="72" spans="1:9" hidden="1">
       <c r="A72" t="s">
         <v>184</v>
       </c>
@@ -10580,7 +10652,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="73" spans="1:9">
+    <row r="73" spans="1:9" hidden="1">
       <c r="A73" t="s">
         <v>184</v>
       </c>
@@ -10605,7 +10677,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="74" spans="1:9">
+    <row r="74" spans="1:9" hidden="1">
       <c r="A74" t="s">
         <v>184</v>
       </c>
@@ -10630,7 +10702,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="75" spans="1:9">
+    <row r="75" spans="1:9" hidden="1">
       <c r="A75" t="s">
         <v>184</v>
       </c>
@@ -10655,7 +10727,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="76" spans="1:9">
+    <row r="76" spans="1:9" hidden="1">
       <c r="A76" t="s">
         <v>180</v>
       </c>
@@ -10677,7 +10749,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="77" spans="1:9">
+    <row r="77" spans="1:9" hidden="1">
       <c r="A77" t="s">
         <v>180</v>
       </c>
@@ -10689,17 +10761,17 @@
         <v>0</v>
       </c>
       <c r="F77">
-        <v>4815</v>
+        <v>4958</v>
       </c>
       <c r="G77">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7748.9937573526759</v>
+        <v>7979.1300205513126</v>
       </c>
       <c r="I77" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" hidden="1">
       <c r="A78" t="s">
         <v>180</v>
       </c>
@@ -10721,7 +10793,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="79" spans="1:9">
+    <row r="79" spans="1:9" hidden="1">
       <c r="A79" t="s">
         <v>180</v>
       </c>
@@ -10733,17 +10805,17 @@
         <v>0</v>
       </c>
       <c r="F79">
-        <v>5637</v>
+        <v>5631</v>
       </c>
       <c r="G79">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9071.8749346203604</v>
+        <v>9062.2188676330043</v>
       </c>
       <c r="I79" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" hidden="1">
       <c r="A80" t="s">
         <v>180</v>
       </c>
@@ -10765,7 +10837,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="81" spans="1:9">
+    <row r="81" spans="1:9" hidden="1">
       <c r="A81" t="s">
         <v>180</v>
       </c>
@@ -10787,7 +10859,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="82" spans="1:9">
+    <row r="82" spans="1:9" hidden="1">
       <c r="A82" t="s">
         <v>180</v>
       </c>
@@ -10809,7 +10881,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="83" spans="1:9">
+    <row r="83" spans="1:9" hidden="1">
       <c r="A83" t="s">
         <v>180</v>
       </c>
@@ -10831,7 +10903,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="84" spans="1:9">
+    <row r="84" spans="1:9" hidden="1">
       <c r="A84" t="s">
         <v>180</v>
       </c>
@@ -10853,7 +10925,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="85" spans="1:9">
+    <row r="85" spans="1:9" hidden="1">
       <c r="A85" t="s">
         <v>180</v>
       </c>
@@ -10865,17 +10937,17 @@
         <v>0</v>
       </c>
       <c r="F85">
-        <v>4786</v>
+        <v>4697</v>
       </c>
       <c r="G85">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7702.3227669137923</v>
+        <v>7559.0911066013541</v>
       </c>
       <c r="I85" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" hidden="1">
       <c r="A86" t="s">
         <v>180</v>
       </c>
@@ -10897,7 +10969,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="87" spans="1:9">
+    <row r="87" spans="1:9" hidden="1">
       <c r="A87" t="s">
         <v>180</v>
       </c>
@@ -10919,7 +10991,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="88" spans="1:9">
+    <row r="88" spans="1:9" hidden="1">
       <c r="A88" t="s">
         <v>180</v>
       </c>
@@ -10941,7 +11013,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="89" spans="1:9">
+    <row r="89" spans="1:9" hidden="1">
       <c r="A89" t="s">
         <v>182</v>
       </c>
@@ -10963,7 +11035,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="90" spans="1:9">
+    <row r="90" spans="1:9" hidden="1">
       <c r="A90" t="s">
         <v>182</v>
       </c>
@@ -10975,17 +11047,17 @@
         <v>0</v>
       </c>
       <c r="F90">
-        <v>4101</v>
+        <v>3952</v>
       </c>
       <c r="G90">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6599.9217858573884</v>
+        <v>6360.1294556713965</v>
       </c>
       <c r="I90" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" hidden="1">
       <c r="A91" t="s">
         <v>182</v>
       </c>
@@ -11007,7 +11079,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="92" spans="1:9">
+    <row r="92" spans="1:9" hidden="1">
       <c r="A92" t="s">
         <v>182</v>
       </c>
@@ -11019,17 +11091,17 @@
         <v>0</v>
       </c>
       <c r="F92">
-        <v>4280</v>
+        <v>5075</v>
       </c>
       <c r="G92">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6887.9944509801562</v>
+        <v>8167.4233268047419</v>
       </c>
       <c r="I92" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="93" spans="1:9">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" hidden="1">
       <c r="A93" t="s">
         <v>182</v>
       </c>
@@ -11051,7 +11123,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="94" spans="1:9">
+    <row r="94" spans="1:9" hidden="1">
       <c r="A94" t="s">
         <v>182</v>
       </c>
@@ -11073,7 +11145,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="95" spans="1:9">
+    <row r="95" spans="1:9" hidden="1">
       <c r="A95" t="s">
         <v>182</v>
       </c>
@@ -11095,7 +11167,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="96" spans="1:9">
+    <row r="96" spans="1:9" hidden="1">
       <c r="A96" t="s">
         <v>182</v>
       </c>
@@ -11117,7 +11189,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="97" spans="1:9">
+    <row r="97" spans="1:9" hidden="1">
       <c r="A97" t="s">
         <v>182</v>
       </c>
@@ -11139,7 +11211,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="98" spans="1:9">
+    <row r="98" spans="1:9" hidden="1">
       <c r="A98" t="s">
         <v>182</v>
       </c>
@@ -11151,17 +11223,17 @@
         <v>0</v>
       </c>
       <c r="F98">
-        <v>3366</v>
+        <v>3645</v>
       </c>
       <c r="G98">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5417.0535799063564</v>
+        <v>5866.0606948183813</v>
       </c>
       <c r="I98" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" hidden="1">
       <c r="A99" t="s">
         <v>182</v>
       </c>
@@ -11183,7 +11255,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="100" spans="1:9">
+    <row r="100" spans="1:9" hidden="1">
       <c r="A100" t="s">
         <v>182</v>
       </c>
@@ -11195,17 +11267,17 @@
         <v>0</v>
       </c>
       <c r="F100">
-        <v>3733</v>
+        <v>3974</v>
       </c>
       <c r="G100">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6007.6830106329262</v>
+        <v>6395.5350346250334</v>
       </c>
       <c r="I100" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="101" spans="1:9">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" hidden="1">
       <c r="A101" t="s">
         <v>183</v>
       </c>
@@ -11230,7 +11302,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="102" spans="1:9">
+    <row r="102" spans="1:9" hidden="1">
       <c r="A102" t="s">
         <v>183</v>
       </c>
@@ -11242,20 +11314,20 @@
         <v>0</v>
       </c>
       <c r="F102">
-        <v>4514</v>
+        <v>6177</v>
       </c>
       <c r="G102">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7264.5810634870159</v>
+        <v>9940.9209634823437</v>
       </c>
       <c r="H102" t="s">
         <v>213</v>
       </c>
       <c r="I102" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="103" spans="1:9">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" hidden="1">
       <c r="A103" t="s">
         <v>183</v>
       </c>
@@ -11280,7 +11352,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="104" spans="1:9">
+    <row r="104" spans="1:9" hidden="1">
       <c r="A104" t="s">
         <v>183</v>
       </c>
@@ -11305,7 +11377,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="105" spans="1:9">
+    <row r="105" spans="1:9" hidden="1">
       <c r="A105" t="s">
         <v>183</v>
       </c>
@@ -11330,7 +11402,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="106" spans="1:9">
+    <row r="106" spans="1:9" hidden="1">
       <c r="A106" t="s">
         <v>183</v>
       </c>
@@ -11355,7 +11427,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="107" spans="1:9">
+    <row r="107" spans="1:9" hidden="1">
       <c r="A107" t="s">
         <v>183</v>
       </c>
@@ -11380,7 +11452,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="108" spans="1:9">
+    <row r="108" spans="1:9" hidden="1">
       <c r="A108" t="s">
         <v>183</v>
       </c>
@@ -11405,7 +11477,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="109" spans="1:9">
+    <row r="109" spans="1:9" hidden="1">
       <c r="A109" t="s">
         <v>183</v>
       </c>
@@ -11430,7 +11502,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="110" spans="1:9">
+    <row r="110" spans="1:9" hidden="1">
       <c r="A110" t="s">
         <v>183</v>
       </c>
@@ -11455,7 +11527,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="111" spans="1:9">
+    <row r="111" spans="1:9" hidden="1">
       <c r="A111" t="s">
         <v>183</v>
       </c>
@@ -11480,7 +11552,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="112" spans="1:9">
+    <row r="112" spans="1:9" hidden="1">
       <c r="A112" t="s">
         <v>183</v>
       </c>
@@ -11505,7 +11577,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="113" spans="1:9">
+    <row r="113" spans="1:9" hidden="1">
       <c r="A113" t="s">
         <v>185</v>
       </c>
@@ -11527,7 +11599,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="114" spans="1:9">
+    <row r="114" spans="1:9" hidden="1">
       <c r="A114" t="s">
         <v>185</v>
       </c>
@@ -11539,17 +11611,17 @@
         <v>0</v>
       </c>
       <c r="F114">
-        <v>4027</v>
+        <v>3980</v>
       </c>
       <c r="G114">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6480.8302930133386</v>
+        <v>6405.1911016123886</v>
       </c>
       <c r="I114" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="115" spans="1:9">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" hidden="1">
       <c r="A115" t="s">
         <v>185</v>
       </c>
@@ -11571,7 +11643,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="116" spans="1:9">
+    <row r="116" spans="1:9" hidden="1">
       <c r="A116" t="s">
         <v>185</v>
       </c>
@@ -11583,17 +11655,17 @@
         <v>0</v>
       </c>
       <c r="F116">
-        <v>4206</v>
+        <v>4172</v>
       </c>
       <c r="G116">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6768.9029581361074</v>
+        <v>6714.1852452077601</v>
       </c>
       <c r="I116" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="117" spans="1:9">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" hidden="1">
       <c r="A117" t="s">
         <v>185</v>
       </c>
@@ -11615,7 +11687,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="118" spans="1:9">
+    <row r="118" spans="1:9" hidden="1">
       <c r="A118" t="s">
         <v>185</v>
       </c>
@@ -11637,7 +11709,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="119" spans="1:9">
+    <row r="119" spans="1:9" hidden="1">
       <c r="A119" t="s">
         <v>185</v>
       </c>
@@ -11659,7 +11731,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="120" spans="1:9">
+    <row r="120" spans="1:9" hidden="1">
       <c r="A120" t="s">
         <v>185</v>
       </c>
@@ -11681,7 +11753,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="121" spans="1:9">
+    <row r="121" spans="1:9" hidden="1">
       <c r="A121" t="s">
         <v>185</v>
       </c>
@@ -11703,7 +11775,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="122" spans="1:9">
+    <row r="122" spans="1:9" hidden="1">
       <c r="A122" t="s">
         <v>185</v>
       </c>
@@ -11725,7 +11797,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="123" spans="1:9">
+    <row r="123" spans="1:9" hidden="1">
       <c r="A123" t="s">
         <v>185</v>
       </c>
@@ -11737,17 +11809,17 @@
         <v>0</v>
       </c>
       <c r="F123">
-        <v>4978</v>
+        <v>5109</v>
       </c>
       <c r="G123">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8011.3169105091638</v>
+        <v>8222.1410397330892</v>
       </c>
       <c r="I123" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="124" spans="1:9">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" hidden="1">
       <c r="A124" t="s">
         <v>185</v>
       </c>
@@ -11759,17 +11831,17 @@
         <v>0</v>
       </c>
       <c r="F124">
-        <v>4162</v>
+        <v>4309</v>
       </c>
       <c r="G124">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6698.0918002288345</v>
+        <v>6934.6654414190407</v>
       </c>
       <c r="I124" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="125" spans="1:9">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" hidden="1">
       <c r="A125" t="s">
         <v>186</v>
       </c>
@@ -11794,7 +11866,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="126" spans="1:9">
+    <row r="126" spans="1:9" hidden="1">
       <c r="A126" t="s">
         <v>186</v>
       </c>
@@ -11819,7 +11891,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="127" spans="1:9">
+    <row r="127" spans="1:9" hidden="1">
       <c r="A127" t="s">
         <v>186</v>
       </c>
@@ -11844,7 +11916,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="128" spans="1:9">
+    <row r="128" spans="1:9" hidden="1">
       <c r="A128" t="s">
         <v>186</v>
       </c>
@@ -11869,7 +11941,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="129" spans="1:9">
+    <row r="129" spans="1:9" hidden="1">
       <c r="A129" t="s">
         <v>186</v>
       </c>
@@ -11894,7 +11966,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="130" spans="1:9">
+    <row r="130" spans="1:9" hidden="1">
       <c r="A130" t="s">
         <v>186</v>
       </c>
@@ -11919,7 +11991,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="131" spans="1:9">
+    <row r="131" spans="1:9" hidden="1">
       <c r="A131" t="s">
         <v>186</v>
       </c>
@@ -11944,7 +12016,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="132" spans="1:9">
+    <row r="132" spans="1:9" hidden="1">
       <c r="A132" t="s">
         <v>186</v>
       </c>
@@ -11969,7 +12041,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="133" spans="1:9">
+    <row r="133" spans="1:9" hidden="1">
       <c r="A133" t="s">
         <v>186</v>
       </c>
@@ -11994,7 +12066,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="134" spans="1:9">
+    <row r="134" spans="1:9" hidden="1">
       <c r="A134" t="s">
         <v>186</v>
       </c>
@@ -12019,7 +12091,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="135" spans="1:9">
+    <row r="135" spans="1:9" hidden="1">
       <c r="A135" t="s">
         <v>186</v>
       </c>
@@ -12044,7 +12116,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="136" spans="1:9">
+    <row r="136" spans="1:9" hidden="1">
       <c r="A136" t="s">
         <v>186</v>
       </c>
@@ -12069,7 +12141,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="137" spans="1:9">
+    <row r="137" spans="1:9" hidden="1">
       <c r="A137" t="s">
         <v>192</v>
       </c>
@@ -12091,7 +12163,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="138" spans="1:9">
+    <row r="138" spans="1:9" hidden="1">
       <c r="A138" t="s">
         <v>192</v>
       </c>
@@ -12103,17 +12175,17 @@
         <v>0</v>
       </c>
       <c r="F138">
-        <v>1512</v>
+        <v>1405</v>
       </c>
       <c r="G138">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>2433.3288808135508</v>
+        <v>2261.1290195390466</v>
       </c>
       <c r="I138" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="139" spans="1:9">
+    <row r="139" spans="1:9" hidden="1">
       <c r="A139" t="s">
         <v>192</v>
       </c>
@@ -12125,17 +12197,17 @@
         <v>0</v>
       </c>
       <c r="F139">
-        <v>599</v>
+        <v>518</v>
       </c>
       <c r="G139">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>963.99735423764344</v>
+        <v>833.64044990834611</v>
       </c>
       <c r="I139" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="140" spans="1:9">
+    <row r="140" spans="1:9" hidden="1">
       <c r="A140" t="s">
         <v>192</v>
       </c>
@@ -12147,17 +12219,17 @@
         <v>0</v>
       </c>
       <c r="F140">
-        <v>1383</v>
+        <v>1239</v>
       </c>
       <c r="G140">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>2225.7234405854106</v>
+        <v>1993.9778328888817</v>
       </c>
       <c r="I140" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="141" spans="1:9">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" hidden="1">
       <c r="A141" t="s">
         <v>192</v>
       </c>
@@ -12179,7 +12251,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="142" spans="1:9">
+    <row r="142" spans="1:9" hidden="1">
       <c r="A142" t="s">
         <v>192</v>
       </c>
@@ -12201,7 +12273,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="143" spans="1:9">
+    <row r="143" spans="1:9" hidden="1">
       <c r="A143" t="s">
         <v>192</v>
       </c>
@@ -12223,7 +12295,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="144" spans="1:9">
+    <row r="144" spans="1:9" hidden="1">
       <c r="A144" t="s">
         <v>192</v>
       </c>
@@ -12235,17 +12307,17 @@
         <v>0</v>
       </c>
       <c r="F144">
-        <v>3951</v>
+        <v>3836</v>
       </c>
       <c r="G144">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6358.5201111735041</v>
+        <v>6173.4454939158604</v>
       </c>
       <c r="I144" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="145" spans="1:9">
+    <row r="145" spans="1:9" hidden="1">
       <c r="A145" t="s">
         <v>192</v>
       </c>
@@ -12257,17 +12329,17 @@
         <v>0</v>
       </c>
       <c r="F145">
-        <v>2197</v>
+        <v>2082</v>
       </c>
       <c r="G145">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>3535.7298618699542</v>
+        <v>3350.6552446123096</v>
       </c>
       <c r="I145" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="146" spans="1:9">
+    <row r="146" spans="1:9" hidden="1">
       <c r="A146" t="s">
         <v>192</v>
       </c>
@@ -12279,17 +12351,17 @@
         <v>0</v>
       </c>
       <c r="F146">
-        <v>1588</v>
+        <v>1696</v>
       </c>
       <c r="G146">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>2555.6390626533853</v>
+        <v>2729.4482684257819</v>
       </c>
       <c r="I146" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="147" spans="1:9">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" hidden="1">
       <c r="A147" t="s">
         <v>192</v>
       </c>
@@ -12301,17 +12373,17 @@
         <v>0</v>
       </c>
       <c r="F147">
-        <v>598</v>
+        <v>722</v>
       </c>
       <c r="G147">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>962.38800973975083</v>
+        <v>1161.9467274784283</v>
       </c>
       <c r="I147" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="148" spans="1:9">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" hidden="1">
       <c r="A148" t="s">
         <v>192</v>
       </c>
@@ -12323,17 +12395,17 @@
         <v>0</v>
       </c>
       <c r="F148">
-        <v>3022</v>
+        <v>2907</v>
       </c>
       <c r="G148">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4863.4390726313159</v>
+        <v>4678.3644553736722</v>
       </c>
       <c r="I148" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="149" spans="1:9">
+    <row r="149" spans="1:9" hidden="1">
       <c r="A149" t="s">
         <v>195</v>
       </c>
@@ -12358,7 +12430,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="150" spans="1:9">
+    <row r="150" spans="1:9" hidden="1">
       <c r="A150" t="s">
         <v>195</v>
       </c>
@@ -12370,20 +12442,20 @@
         <v>0</v>
       </c>
       <c r="F150">
-        <v>7541</v>
+        <v>8897</v>
       </c>
       <c r="G150">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>12136.066858607795</v>
+        <v>14318.337997750106</v>
       </c>
       <c r="H150" t="s">
         <v>213</v>
       </c>
       <c r="I150" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="151" spans="1:9">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" hidden="1">
       <c r="A151" t="s">
         <v>195</v>
       </c>
@@ -12395,20 +12467,20 @@
         <v>0</v>
       </c>
       <c r="F151">
-        <v>6628</v>
+        <v>6737</v>
       </c>
       <c r="G151">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10666.735332031887</v>
+        <v>10842.153882302176</v>
       </c>
       <c r="H151" t="s">
         <v>213</v>
       </c>
       <c r="I151" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="152" spans="1:9">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" hidden="1">
       <c r="A152" t="s">
         <v>195</v>
       </c>
@@ -12433,7 +12505,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="153" spans="1:9">
+    <row r="153" spans="1:9" hidden="1">
       <c r="A153" t="s">
         <v>195</v>
       </c>
@@ -12458,7 +12530,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="154" spans="1:9">
+    <row r="154" spans="1:9" hidden="1">
       <c r="A154" t="s">
         <v>195</v>
       </c>
@@ -12483,7 +12555,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="155" spans="1:9">
+    <row r="155" spans="1:9" hidden="1">
       <c r="A155" t="s">
         <v>195</v>
       </c>
@@ -12508,7 +12580,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="156" spans="1:9">
+    <row r="156" spans="1:9" hidden="1">
       <c r="A156" t="s">
         <v>195</v>
       </c>
@@ -12533,7 +12605,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="157" spans="1:9">
+    <row r="157" spans="1:9" hidden="1">
       <c r="A157" t="s">
         <v>195</v>
       </c>
@@ -12558,7 +12630,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="158" spans="1:9">
+    <row r="158" spans="1:9" hidden="1">
       <c r="A158" t="s">
         <v>195</v>
       </c>
@@ -12583,7 +12655,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="159" spans="1:9">
+    <row r="159" spans="1:9" hidden="1">
       <c r="A159" t="s">
         <v>195</v>
       </c>
@@ -12608,7 +12680,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="160" spans="1:9">
+    <row r="160" spans="1:9" hidden="1">
       <c r="A160" t="s">
         <v>195</v>
       </c>
@@ -12633,7 +12705,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="161" spans="1:9">
+    <row r="161" spans="1:9" hidden="1">
       <c r="A161" t="s">
         <v>194</v>
       </c>
@@ -12655,7 +12727,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="162" spans="1:9">
+    <row r="162" spans="1:9" hidden="1">
       <c r="A162" t="s">
         <v>194</v>
       </c>
@@ -12667,17 +12739,17 @@
         <v>0</v>
       </c>
       <c r="F162">
-        <v>2873</v>
+        <v>3331</v>
       </c>
       <c r="G162">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4623.6467424453249</v>
+        <v>5360.7265224801176</v>
       </c>
       <c r="I162" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="163" spans="1:9">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9" hidden="1">
       <c r="A163" t="s">
         <v>194</v>
       </c>
@@ -12699,7 +12771,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="164" spans="1:9">
+    <row r="164" spans="1:9" hidden="1">
       <c r="A164" t="s">
         <v>194</v>
       </c>
@@ -12711,17 +12783,17 @@
         <v>0</v>
       </c>
       <c r="F164">
-        <v>4964</v>
+        <v>5759</v>
       </c>
       <c r="G164">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7988.7860875386677</v>
+        <v>9268.2149633632525</v>
       </c>
       <c r="I164" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="165" spans="1:9">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" hidden="1">
       <c r="A165" t="s">
         <v>194</v>
       </c>
@@ -12743,7 +12815,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="166" spans="1:9">
+    <row r="166" spans="1:9" hidden="1">
       <c r="A166" t="s">
         <v>194</v>
       </c>
@@ -12765,7 +12837,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="167" spans="1:9">
+    <row r="167" spans="1:9" hidden="1">
       <c r="A167" t="s">
         <v>194</v>
       </c>
@@ -12787,7 +12859,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="168" spans="1:9">
+    <row r="168" spans="1:9" hidden="1">
       <c r="A168" t="s">
         <v>194</v>
       </c>
@@ -12809,7 +12881,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="169" spans="1:9">
+    <row r="169" spans="1:9" hidden="1">
       <c r="A169" t="s">
         <v>194</v>
       </c>
@@ -12831,7 +12903,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="170" spans="1:9">
+    <row r="170" spans="1:9" hidden="1">
       <c r="A170" t="s">
         <v>194</v>
       </c>
@@ -12853,7 +12925,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="171" spans="1:9">
+    <row r="171" spans="1:9" hidden="1">
       <c r="A171" t="s">
         <v>194</v>
       </c>
@@ -12875,7 +12947,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="172" spans="1:9">
+    <row r="172" spans="1:9" hidden="1">
       <c r="A172" t="s">
         <v>194</v>
       </c>
@@ -12894,7 +12966,7 @@
         <v>4612.3813309600764</v>
       </c>
       <c r="I172" t="s">
-        <v>274</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update global LNG connections 2024
update the port to port information
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C918F4-F712-4020-8DA5-1C33F77A146A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA3E34E-253C-4D50-A14C-04E7B7A63E9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2652" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2660" uniqueCount="289">
   <si>
     <t>Belgium</t>
   </si>
@@ -791,42 +791,27 @@
     <t>Bangkok</t>
   </si>
   <si>
-    <t>Port Said</t>
-  </si>
-  <si>
     <t>Trinidad from Point Fortin</t>
   </si>
   <si>
     <t>ME from Das Island (UAE)</t>
   </si>
   <si>
-    <t>AF from Port Harcourt (Nigeria)</t>
-  </si>
-  <si>
     <t>Huelva</t>
   </si>
   <si>
-    <t>Mumbai</t>
-  </si>
-  <si>
     <t>AU from Darwin</t>
   </si>
   <si>
     <t>Quintero (Chile)</t>
   </si>
   <si>
-    <t>EG from Port Said to Europe, AF and from Suez to Asian Regions</t>
-  </si>
-  <si>
     <t xml:space="preserve">IM from Balikpapan (bestguess  in the middle) </t>
   </si>
   <si>
     <t>Dunkirk</t>
   </si>
   <si>
-    <t xml:space="preserve">RU from Sabetta (plus 1200 mi to west, minus 1200 mi to east as Murmansk is the closest port) except for JS, there it's from Vladivostok </t>
-  </si>
-  <si>
     <t>comment</t>
   </si>
   <si>
@@ -873,9 +858,6 @@
   </si>
   <si>
     <t>EL_LNG</t>
-  </si>
-  <si>
-    <t>Isle of ELain</t>
   </si>
   <si>
     <t>assumption for distance</t>
@@ -1804,13 +1786,7 @@
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I172" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
-  <autoFilter ref="A1:I172" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}">
-    <filterColumn colId="8">
-      <filters>
-        <filter val="Wadi Feiran"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:I172" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
     <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
@@ -2431,7 +2407,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C4">
         <v>7</v>
@@ -2459,7 +2435,7 @@
         <v>73.274999999999991</v>
       </c>
       <c r="K4" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="L4" t="s">
         <v>101</v>
@@ -3654,7 +3630,7 @@
         <v>32</v>
       </c>
       <c r="B13" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C13">
         <v>117.8</v>
@@ -4251,7 +4227,7 @@
     </row>
     <row r="43" spans="1:8">
       <c r="A43" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B43" t="s">
         <v>42</v>
@@ -4276,7 +4252,7 @@
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B44" t="s">
         <v>32</v>
@@ -5410,7 +5386,7 @@
         <v>47</v>
       </c>
       <c r="B101" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C101">
         <v>398.6</v>
@@ -6088,7 +6064,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B26" t="s">
         <v>42</v>
@@ -6110,7 +6086,7 @@
         <v>47</v>
       </c>
       <c r="B27" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C27">
         <v>395</v>
@@ -6514,7 +6490,7 @@
         <v>32</v>
       </c>
       <c r="B13" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C13">
         <v>120.36</v>
@@ -7127,7 +7103,7 @@
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B44" t="s">
         <v>42</v>
@@ -7149,7 +7125,7 @@
     </row>
     <row r="45" spans="1:8">
       <c r="A45" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B45" t="s">
         <v>32</v>
@@ -8369,7 +8345,7 @@
         <v>47</v>
       </c>
       <c r="B107" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C107">
         <v>398.6</v>
@@ -8580,7 +8556,7 @@
         <v>94</v>
       </c>
       <c r="C1" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="D1" t="s">
         <v>106</v>
@@ -8589,19 +8565,19 @@
         <v>107</v>
       </c>
       <c r="F1" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="G1" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="H1" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="I1" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="L1" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -8626,7 +8602,7 @@
         <v>5000</v>
       </c>
       <c r="I2" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -8652,7 +8628,7 @@
         <v>850</v>
       </c>
       <c r="I3" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -8678,7 +8654,7 @@
         <v>2400</v>
       </c>
       <c r="I4" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -8707,7 +8683,7 @@
         <v>4828.0334936776799</v>
       </c>
       <c r="I5" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -8736,7 +8712,7 @@
         <v>4828.0334936776799</v>
       </c>
       <c r="I6" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -8761,7 +8737,7 @@
         <v>7378</v>
       </c>
       <c r="I7" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -8787,7 +8763,7 @@
         <v>1000</v>
       </c>
       <c r="I8" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -8812,7 +8788,7 @@
         <v>1200</v>
       </c>
       <c r="I9" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -8838,7 +8814,7 @@
         <v>200</v>
       </c>
       <c r="I10" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -8867,7 +8843,7 @@
         <v>370.14923451528881</v>
       </c>
       <c r="I11" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -8896,7 +8872,7 @@
         <v>370.14923451528881</v>
       </c>
       <c r="I12" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -8921,7 +8897,7 @@
         <v>2520</v>
       </c>
       <c r="I13" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -8976,7 +8952,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="2" spans="1:13" hidden="1">
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
         <v>180</v>
       </c>
@@ -9001,7 +8977,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="3" spans="1:13" hidden="1">
+    <row r="3" spans="1:13">
       <c r="A3" t="s">
         <v>180</v>
       </c>
@@ -9026,7 +9002,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="4" spans="1:13" hidden="1">
+    <row r="4" spans="1:13">
       <c r="A4" t="s">
         <v>180</v>
       </c>
@@ -9048,13 +9024,13 @@
         <v>241</v>
       </c>
       <c r="I4" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="M4" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" hidden="1">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
         <v>180</v>
       </c>
@@ -9079,10 +9055,10 @@
         <v>243</v>
       </c>
       <c r="M5" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" hidden="1">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" t="s">
         <v>180</v>
       </c>
@@ -9107,10 +9083,10 @@
         <v>244</v>
       </c>
       <c r="M6" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" hidden="1">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" t="s">
         <v>180</v>
       </c>
@@ -9135,7 +9111,7 @@
         <v>245</v>
       </c>
       <c r="M7" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -9160,13 +9136,13 @@
         <v>213</v>
       </c>
       <c r="I8" t="s">
+        <v>278</v>
+      </c>
+      <c r="M8" t="s">
         <v>284</v>
       </c>
-      <c r="M8" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" hidden="1">
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" t="s">
         <v>182</v>
       </c>
@@ -9188,10 +9164,10 @@
         <v>239</v>
       </c>
       <c r="M9" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" hidden="1">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" t="s">
         <v>182</v>
       </c>
@@ -9213,10 +9189,10 @@
         <v>240</v>
       </c>
       <c r="M10" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" hidden="1">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
       <c r="A11" t="s">
         <v>182</v>
       </c>
@@ -9238,10 +9214,10 @@
         <v>241</v>
       </c>
       <c r="I11" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" hidden="1">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
       <c r="A12" t="s">
         <v>182</v>
       </c>
@@ -9266,7 +9242,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="13" spans="1:13" hidden="1">
+    <row r="13" spans="1:13">
       <c r="A13" t="s">
         <v>182</v>
       </c>
@@ -9291,7 +9267,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="14" spans="1:13" hidden="1">
+    <row r="14" spans="1:13">
       <c r="A14" t="s">
         <v>182</v>
       </c>
@@ -9338,10 +9314,10 @@
         <v>213</v>
       </c>
       <c r="I15" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" hidden="1">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
       <c r="A16" t="s">
         <v>183</v>
       </c>
@@ -9363,7 +9339,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="17" spans="1:9" hidden="1">
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>183</v>
       </c>
@@ -9385,7 +9361,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="18" spans="1:9" hidden="1">
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>183</v>
       </c>
@@ -9404,10 +9380,10 @@
         <v>8048.3318339606922</v>
       </c>
       <c r="I18" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" hidden="1">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>183</v>
       </c>
@@ -9429,7 +9405,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="20" spans="1:9" hidden="1">
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>183</v>
       </c>
@@ -9451,7 +9427,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="21" spans="1:9" hidden="1">
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>183</v>
       </c>
@@ -9473,7 +9449,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="22" spans="1:9" hidden="1">
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
         <v>183</v>
       </c>
@@ -9495,7 +9471,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="23" spans="1:9" hidden="1">
+    <row r="23" spans="1:9">
       <c r="A23" t="s">
         <v>184</v>
       </c>
@@ -9517,7 +9493,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="24" spans="1:9" hidden="1">
+    <row r="24" spans="1:9">
       <c r="A24" t="s">
         <v>184</v>
       </c>
@@ -9539,7 +9515,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="25" spans="1:9" hidden="1">
+    <row r="25" spans="1:9">
       <c r="A25" t="s">
         <v>184</v>
       </c>
@@ -9558,10 +9534,10 @@
         <v>9406.6185901820136</v>
       </c>
       <c r="I25" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" hidden="1">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
       <c r="A26" t="s">
         <v>184</v>
       </c>
@@ -9583,7 +9559,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="27" spans="1:9" hidden="1">
+    <row r="27" spans="1:9">
       <c r="A27" t="s">
         <v>184</v>
       </c>
@@ -9605,7 +9581,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="28" spans="1:9" hidden="1">
+    <row r="28" spans="1:9">
       <c r="A28" t="s">
         <v>184</v>
       </c>
@@ -9646,10 +9622,10 @@
         <v>4676.7551108757789</v>
       </c>
       <c r="I29" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" hidden="1">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" t="s">
         <v>185</v>
       </c>
@@ -9671,7 +9647,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="31" spans="1:9" hidden="1">
+    <row r="31" spans="1:9">
       <c r="A31" t="s">
         <v>185</v>
       </c>
@@ -9690,10 +9666,10 @@
         <v>14976.559897388162</v>
       </c>
       <c r="I31" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" hidden="1">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
       <c r="A32" t="s">
         <v>185</v>
       </c>
@@ -9715,7 +9691,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="33" spans="1:9" hidden="1">
+    <row r="33" spans="1:9">
       <c r="A33" t="s">
         <v>185</v>
       </c>
@@ -9737,7 +9713,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="34" spans="1:9" hidden="1">
+    <row r="34" spans="1:9">
       <c r="A34" t="s">
         <v>185</v>
       </c>
@@ -9781,10 +9757,10 @@
         <v>213</v>
       </c>
       <c r="I35" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" hidden="1">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
       <c r="A36" t="s">
         <v>186</v>
       </c>
@@ -9803,10 +9779,10 @@
         <v>13800.129069428702</v>
       </c>
       <c r="I36" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" hidden="1">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
       <c r="A37" t="s">
         <v>186</v>
       </c>
@@ -9828,7 +9804,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="38" spans="1:9" hidden="1">
+    <row r="38" spans="1:9">
       <c r="A38" t="s">
         <v>186</v>
       </c>
@@ -9847,10 +9823,10 @@
         <v>3786.7876035411937</v>
       </c>
       <c r="I38" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" hidden="1">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
       <c r="A39" t="s">
         <v>186</v>
       </c>
@@ -9872,7 +9848,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="40" spans="1:9" hidden="1">
+    <row r="40" spans="1:9">
       <c r="A40" t="s">
         <v>186</v>
       </c>
@@ -9894,7 +9870,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="41" spans="1:9" hidden="1">
+    <row r="41" spans="1:9">
       <c r="A41" t="s">
         <v>186</v>
       </c>
@@ -9935,10 +9911,10 @@
         <v>10587.877451635151</v>
       </c>
       <c r="I42" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" hidden="1">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
       <c r="A43" t="s">
         <v>194</v>
       </c>
@@ -9960,7 +9936,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="44" spans="1:9" hidden="1">
+    <row r="44" spans="1:9">
       <c r="A44" t="s">
         <v>194</v>
       </c>
@@ -9982,7 +9958,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="45" spans="1:9" hidden="1">
+    <row r="45" spans="1:9">
       <c r="A45" t="s">
         <v>194</v>
       </c>
@@ -10004,10 +9980,10 @@
         <v>213</v>
       </c>
       <c r="I45" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" hidden="1">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
       <c r="A46" t="s">
         <v>194</v>
       </c>
@@ -10029,7 +10005,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="47" spans="1:9" hidden="1">
+    <row r="47" spans="1:9">
       <c r="A47" t="s">
         <v>194</v>
       </c>
@@ -10054,7 +10030,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="48" spans="1:9" hidden="1">
+    <row r="48" spans="1:9">
       <c r="A48" t="s">
         <v>194</v>
       </c>
@@ -10101,10 +10077,10 @@
         <v>213</v>
       </c>
       <c r="I49" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" hidden="1">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
       <c r="A50" t="s">
         <v>192</v>
       </c>
@@ -10126,7 +10102,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="51" spans="1:9" hidden="1">
+    <row r="51" spans="1:9">
       <c r="A51" t="s">
         <v>192</v>
       </c>
@@ -10148,7 +10124,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="52" spans="1:9" hidden="1">
+    <row r="52" spans="1:9">
       <c r="A52" t="s">
         <v>192</v>
       </c>
@@ -10170,10 +10146,10 @@
         <v>213</v>
       </c>
       <c r="I52" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" hidden="1">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
       <c r="A53" t="s">
         <v>192</v>
       </c>
@@ -10198,7 +10174,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="54" spans="1:9" hidden="1">
+    <row r="54" spans="1:9">
       <c r="A54" t="s">
         <v>192</v>
       </c>
@@ -10223,7 +10199,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="55" spans="1:9" hidden="1">
+    <row r="55" spans="1:9">
       <c r="A55" t="s">
         <v>192</v>
       </c>
@@ -10248,7 +10224,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="56" spans="1:9" hidden="1">
+    <row r="56" spans="1:9">
       <c r="A56" t="s">
         <v>195</v>
       </c>
@@ -10270,7 +10246,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="57" spans="1:9" hidden="1">
+    <row r="57" spans="1:9">
       <c r="A57" t="s">
         <v>195</v>
       </c>
@@ -10292,7 +10268,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="58" spans="1:9" hidden="1">
+    <row r="58" spans="1:9">
       <c r="A58" t="s">
         <v>195</v>
       </c>
@@ -10311,10 +10287,10 @@
         <v>3518.0270723931362</v>
       </c>
       <c r="I58" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" hidden="1">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9">
       <c r="A59" t="s">
         <v>195</v>
       </c>
@@ -10336,7 +10312,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="60" spans="1:9" hidden="1">
+    <row r="60" spans="1:9">
       <c r="A60" t="s">
         <v>195</v>
       </c>
@@ -10358,7 +10334,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="61" spans="1:9" hidden="1">
+    <row r="61" spans="1:9">
       <c r="A61" t="s">
         <v>195</v>
       </c>
@@ -10399,10 +10375,10 @@
         <v>9440.4148246377572</v>
       </c>
       <c r="I62" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" hidden="1">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9">
       <c r="A63" t="s">
         <v>184</v>
       </c>
@@ -10427,7 +10403,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="64" spans="1:9" hidden="1">
+    <row r="64" spans="1:9">
       <c r="A64" t="s">
         <v>184</v>
       </c>
@@ -10452,12 +10428,12 @@
         <v>214</v>
       </c>
     </row>
-    <row r="65" spans="1:9" hidden="1">
+    <row r="65" spans="1:9">
       <c r="A65" t="s">
         <v>184</v>
       </c>
       <c r="B65" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E65">
         <f t="shared" si="7"/>
@@ -10477,7 +10453,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="66" spans="1:9" hidden="1">
+    <row r="66" spans="1:9">
       <c r="A66" t="s">
         <v>184</v>
       </c>
@@ -10499,10 +10475,10 @@
         <v>213</v>
       </c>
       <c r="I66" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" hidden="1">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9">
       <c r="A67" t="s">
         <v>184</v>
       </c>
@@ -10527,7 +10503,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="68" spans="1:9" hidden="1">
+    <row r="68" spans="1:9">
       <c r="A68" t="s">
         <v>184</v>
       </c>
@@ -10552,7 +10528,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="69" spans="1:9" hidden="1">
+    <row r="69" spans="1:9">
       <c r="A69" t="s">
         <v>184</v>
       </c>
@@ -10577,7 +10553,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="70" spans="1:9" hidden="1">
+    <row r="70" spans="1:9">
       <c r="A70" t="s">
         <v>184</v>
       </c>
@@ -10602,7 +10578,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="71" spans="1:9" hidden="1">
+    <row r="71" spans="1:9">
       <c r="A71" t="s">
         <v>184</v>
       </c>
@@ -10627,7 +10603,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="72" spans="1:9" hidden="1">
+    <row r="72" spans="1:9">
       <c r="A72" t="s">
         <v>184</v>
       </c>
@@ -10652,7 +10628,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="73" spans="1:9" hidden="1">
+    <row r="73" spans="1:9">
       <c r="A73" t="s">
         <v>184</v>
       </c>
@@ -10677,7 +10653,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="74" spans="1:9" hidden="1">
+    <row r="74" spans="1:9">
       <c r="A74" t="s">
         <v>184</v>
       </c>
@@ -10702,7 +10678,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="75" spans="1:9" hidden="1">
+    <row r="75" spans="1:9">
       <c r="A75" t="s">
         <v>184</v>
       </c>
@@ -10727,7 +10703,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="76" spans="1:9" hidden="1">
+    <row r="76" spans="1:9">
       <c r="A76" t="s">
         <v>180</v>
       </c>
@@ -10749,7 +10725,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="77" spans="1:9" hidden="1">
+    <row r="77" spans="1:9">
       <c r="A77" t="s">
         <v>180</v>
       </c>
@@ -10768,15 +10744,15 @@
         <v>7979.1300205513126</v>
       </c>
       <c r="I77" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9" hidden="1">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9">
       <c r="A78" t="s">
         <v>180</v>
       </c>
       <c r="B78" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E78">
         <f t="shared" si="9"/>
@@ -10793,7 +10769,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="79" spans="1:9" hidden="1">
+    <row r="79" spans="1:9">
       <c r="A79" t="s">
         <v>180</v>
       </c>
@@ -10812,10 +10788,10 @@
         <v>9062.2188676330043</v>
       </c>
       <c r="I79" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" hidden="1">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9">
       <c r="A80" t="s">
         <v>180</v>
       </c>
@@ -10837,7 +10813,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="81" spans="1:9" hidden="1">
+    <row r="81" spans="1:9">
       <c r="A81" t="s">
         <v>180</v>
       </c>
@@ -10859,7 +10835,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="82" spans="1:9" hidden="1">
+    <row r="82" spans="1:9">
       <c r="A82" t="s">
         <v>180</v>
       </c>
@@ -10881,7 +10857,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="83" spans="1:9" hidden="1">
+    <row r="83" spans="1:9">
       <c r="A83" t="s">
         <v>180</v>
       </c>
@@ -10903,7 +10879,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="84" spans="1:9" hidden="1">
+    <row r="84" spans="1:9">
       <c r="A84" t="s">
         <v>180</v>
       </c>
@@ -10925,7 +10901,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="85" spans="1:9" hidden="1">
+    <row r="85" spans="1:9">
       <c r="A85" t="s">
         <v>180</v>
       </c>
@@ -10944,10 +10920,10 @@
         <v>7559.0911066013541</v>
       </c>
       <c r="I85" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9" hidden="1">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9">
       <c r="A86" t="s">
         <v>180</v>
       </c>
@@ -10969,7 +10945,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="87" spans="1:9" hidden="1">
+    <row r="87" spans="1:9">
       <c r="A87" t="s">
         <v>180</v>
       </c>
@@ -10991,7 +10967,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="88" spans="1:9" hidden="1">
+    <row r="88" spans="1:9">
       <c r="A88" t="s">
         <v>180</v>
       </c>
@@ -11013,7 +10989,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="89" spans="1:9" hidden="1">
+    <row r="89" spans="1:9">
       <c r="A89" t="s">
         <v>182</v>
       </c>
@@ -11035,7 +11011,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="90" spans="1:9" hidden="1">
+    <row r="90" spans="1:9">
       <c r="A90" t="s">
         <v>182</v>
       </c>
@@ -11054,15 +11030,15 @@
         <v>6360.1294556713965</v>
       </c>
       <c r="I90" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9" hidden="1">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9">
       <c r="A91" t="s">
         <v>182</v>
       </c>
       <c r="B91" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E91">
         <f t="shared" si="10"/>
@@ -11079,7 +11055,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="92" spans="1:9" hidden="1">
+    <row r="92" spans="1:9">
       <c r="A92" t="s">
         <v>182</v>
       </c>
@@ -11098,10 +11074,10 @@
         <v>8167.4233268047419</v>
       </c>
       <c r="I92" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="93" spans="1:9" hidden="1">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9">
       <c r="A93" t="s">
         <v>182</v>
       </c>
@@ -11123,7 +11099,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="94" spans="1:9" hidden="1">
+    <row r="94" spans="1:9">
       <c r="A94" t="s">
         <v>182</v>
       </c>
@@ -11145,7 +11121,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="95" spans="1:9" hidden="1">
+    <row r="95" spans="1:9">
       <c r="A95" t="s">
         <v>182</v>
       </c>
@@ -11167,7 +11143,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="96" spans="1:9" hidden="1">
+    <row r="96" spans="1:9">
       <c r="A96" t="s">
         <v>182</v>
       </c>
@@ -11189,7 +11165,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="97" spans="1:9" hidden="1">
+    <row r="97" spans="1:9">
       <c r="A97" t="s">
         <v>182</v>
       </c>
@@ -11211,7 +11187,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="98" spans="1:9" hidden="1">
+    <row r="98" spans="1:9">
       <c r="A98" t="s">
         <v>182</v>
       </c>
@@ -11233,7 +11209,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="99" spans="1:9" hidden="1">
+    <row r="99" spans="1:9">
       <c r="A99" t="s">
         <v>182</v>
       </c>
@@ -11255,7 +11231,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="100" spans="1:9" hidden="1">
+    <row r="100" spans="1:9">
       <c r="A100" t="s">
         <v>182</v>
       </c>
@@ -11274,10 +11250,10 @@
         <v>6395.5350346250334</v>
       </c>
       <c r="I100" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="101" spans="1:9" hidden="1">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9">
       <c r="A101" t="s">
         <v>183</v>
       </c>
@@ -11302,7 +11278,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="102" spans="1:9" hidden="1">
+    <row r="102" spans="1:9">
       <c r="A102" t="s">
         <v>183</v>
       </c>
@@ -11324,15 +11300,15 @@
         <v>213</v>
       </c>
       <c r="I102" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="103" spans="1:9" hidden="1">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9">
       <c r="A103" t="s">
         <v>183</v>
       </c>
       <c r="B103" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E103">
         <f t="shared" si="11"/>
@@ -11352,7 +11328,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="104" spans="1:9" hidden="1">
+    <row r="104" spans="1:9">
       <c r="A104" t="s">
         <v>183</v>
       </c>
@@ -11377,7 +11353,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="105" spans="1:9" hidden="1">
+    <row r="105" spans="1:9">
       <c r="A105" t="s">
         <v>183</v>
       </c>
@@ -11402,7 +11378,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="106" spans="1:9" hidden="1">
+    <row r="106" spans="1:9">
       <c r="A106" t="s">
         <v>183</v>
       </c>
@@ -11427,7 +11403,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="107" spans="1:9" hidden="1">
+    <row r="107" spans="1:9">
       <c r="A107" t="s">
         <v>183</v>
       </c>
@@ -11452,7 +11428,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="108" spans="1:9" hidden="1">
+    <row r="108" spans="1:9">
       <c r="A108" t="s">
         <v>183</v>
       </c>
@@ -11477,7 +11453,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="109" spans="1:9" hidden="1">
+    <row r="109" spans="1:9">
       <c r="A109" t="s">
         <v>183</v>
       </c>
@@ -11502,7 +11478,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="110" spans="1:9" hidden="1">
+    <row r="110" spans="1:9">
       <c r="A110" t="s">
         <v>183</v>
       </c>
@@ -11527,7 +11503,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="111" spans="1:9" hidden="1">
+    <row r="111" spans="1:9">
       <c r="A111" t="s">
         <v>183</v>
       </c>
@@ -11552,7 +11528,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="112" spans="1:9" hidden="1">
+    <row r="112" spans="1:9">
       <c r="A112" t="s">
         <v>183</v>
       </c>
@@ -11577,7 +11553,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="113" spans="1:9" hidden="1">
+    <row r="113" spans="1:9">
       <c r="A113" t="s">
         <v>185</v>
       </c>
@@ -11599,7 +11575,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="114" spans="1:9" hidden="1">
+    <row r="114" spans="1:9">
       <c r="A114" t="s">
         <v>185</v>
       </c>
@@ -11618,15 +11594,15 @@
         <v>6405.1911016123886</v>
       </c>
       <c r="I114" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="115" spans="1:9" hidden="1">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9">
       <c r="A115" t="s">
         <v>185</v>
       </c>
       <c r="B115" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E115">
         <f t="shared" si="12"/>
@@ -11643,7 +11619,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="116" spans="1:9" hidden="1">
+    <row r="116" spans="1:9">
       <c r="A116" t="s">
         <v>185</v>
       </c>
@@ -11662,10 +11638,10 @@
         <v>6714.1852452077601</v>
       </c>
       <c r="I116" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="117" spans="1:9" hidden="1">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9">
       <c r="A117" t="s">
         <v>185</v>
       </c>
@@ -11687,7 +11663,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="118" spans="1:9" hidden="1">
+    <row r="118" spans="1:9">
       <c r="A118" t="s">
         <v>185</v>
       </c>
@@ -11709,7 +11685,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="119" spans="1:9" hidden="1">
+    <row r="119" spans="1:9">
       <c r="A119" t="s">
         <v>185</v>
       </c>
@@ -11731,7 +11707,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="120" spans="1:9" hidden="1">
+    <row r="120" spans="1:9">
       <c r="A120" t="s">
         <v>185</v>
       </c>
@@ -11753,7 +11729,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="121" spans="1:9" hidden="1">
+    <row r="121" spans="1:9">
       <c r="A121" t="s">
         <v>185</v>
       </c>
@@ -11775,7 +11751,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="122" spans="1:9" hidden="1">
+    <row r="122" spans="1:9">
       <c r="A122" t="s">
         <v>185</v>
       </c>
@@ -11794,10 +11770,10 @@
         <v>5405.7881684211088</v>
       </c>
       <c r="I122" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="123" spans="1:9" hidden="1">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9">
       <c r="A123" t="s">
         <v>185</v>
       </c>
@@ -11816,10 +11792,10 @@
         <v>8222.1410397330892</v>
       </c>
       <c r="I123" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="124" spans="1:9" hidden="1">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9">
       <c r="A124" t="s">
         <v>185</v>
       </c>
@@ -11838,10 +11814,10 @@
         <v>6934.6654414190407</v>
       </c>
       <c r="I124" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="125" spans="1:9" hidden="1">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9">
       <c r="A125" t="s">
         <v>186</v>
       </c>
@@ -11866,7 +11842,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="126" spans="1:9" hidden="1">
+    <row r="126" spans="1:9">
       <c r="A126" t="s">
         <v>186</v>
       </c>
@@ -11891,12 +11867,12 @@
         <v>214</v>
       </c>
     </row>
-    <row r="127" spans="1:9" hidden="1">
+    <row r="127" spans="1:9">
       <c r="A127" t="s">
         <v>186</v>
       </c>
       <c r="B127" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E127">
         <f t="shared" si="13"/>
@@ -11916,7 +11892,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="128" spans="1:9" hidden="1">
+    <row r="128" spans="1:9">
       <c r="A128" t="s">
         <v>186</v>
       </c>
@@ -11941,7 +11917,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="129" spans="1:9" hidden="1">
+    <row r="129" spans="1:9">
       <c r="A129" t="s">
         <v>186</v>
       </c>
@@ -11966,7 +11942,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="130" spans="1:9" hidden="1">
+    <row r="130" spans="1:9">
       <c r="A130" t="s">
         <v>186</v>
       </c>
@@ -11991,7 +11967,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="131" spans="1:9" hidden="1">
+    <row r="131" spans="1:9">
       <c r="A131" t="s">
         <v>186</v>
       </c>
@@ -12016,7 +11992,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="132" spans="1:9" hidden="1">
+    <row r="132" spans="1:9">
       <c r="A132" t="s">
         <v>186</v>
       </c>
@@ -12041,7 +12017,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="133" spans="1:9" hidden="1">
+    <row r="133" spans="1:9">
       <c r="A133" t="s">
         <v>186</v>
       </c>
@@ -12066,7 +12042,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="134" spans="1:9" hidden="1">
+    <row r="134" spans="1:9">
       <c r="A134" t="s">
         <v>186</v>
       </c>
@@ -12091,7 +12067,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="135" spans="1:9" hidden="1">
+    <row r="135" spans="1:9">
       <c r="A135" t="s">
         <v>186</v>
       </c>
@@ -12116,7 +12092,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="136" spans="1:9" hidden="1">
+    <row r="136" spans="1:9">
       <c r="A136" t="s">
         <v>186</v>
       </c>
@@ -12141,7 +12117,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="137" spans="1:9" hidden="1">
+    <row r="137" spans="1:9">
       <c r="A137" t="s">
         <v>192</v>
       </c>
@@ -12163,7 +12139,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="138" spans="1:9" hidden="1">
+    <row r="138" spans="1:9">
       <c r="A138" t="s">
         <v>192</v>
       </c>
@@ -12185,12 +12161,12 @@
         <v>214</v>
       </c>
     </row>
-    <row r="139" spans="1:9" hidden="1">
+    <row r="139" spans="1:9">
       <c r="A139" t="s">
         <v>192</v>
       </c>
       <c r="B139" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E139">
         <f t="shared" si="14"/>
@@ -12207,7 +12183,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="140" spans="1:9" hidden="1">
+    <row r="140" spans="1:9">
       <c r="A140" t="s">
         <v>192</v>
       </c>
@@ -12226,10 +12202,10 @@
         <v>1993.9778328888817</v>
       </c>
       <c r="I140" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="141" spans="1:9" hidden="1">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9">
       <c r="A141" t="s">
         <v>192</v>
       </c>
@@ -12251,7 +12227,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="142" spans="1:9" hidden="1">
+    <row r="142" spans="1:9">
       <c r="A142" t="s">
         <v>192</v>
       </c>
@@ -12273,7 +12249,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="143" spans="1:9" hidden="1">
+    <row r="143" spans="1:9">
       <c r="A143" t="s">
         <v>192</v>
       </c>
@@ -12295,7 +12271,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="144" spans="1:9" hidden="1">
+    <row r="144" spans="1:9">
       <c r="A144" t="s">
         <v>192</v>
       </c>
@@ -12317,7 +12293,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="145" spans="1:9" hidden="1">
+    <row r="145" spans="1:9">
       <c r="A145" t="s">
         <v>192</v>
       </c>
@@ -12339,7 +12315,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="146" spans="1:9" hidden="1">
+    <row r="146" spans="1:9">
       <c r="A146" t="s">
         <v>192</v>
       </c>
@@ -12358,10 +12334,10 @@
         <v>2729.4482684257819</v>
       </c>
       <c r="I146" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="147" spans="1:9" hidden="1">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9">
       <c r="A147" t="s">
         <v>192</v>
       </c>
@@ -12380,10 +12356,10 @@
         <v>1161.9467274784283</v>
       </c>
       <c r="I147" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="148" spans="1:9" hidden="1">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9">
       <c r="A148" t="s">
         <v>192</v>
       </c>
@@ -12405,7 +12381,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="149" spans="1:9" hidden="1">
+    <row r="149" spans="1:9">
       <c r="A149" t="s">
         <v>195</v>
       </c>
@@ -12430,7 +12406,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="150" spans="1:9" hidden="1">
+    <row r="150" spans="1:9">
       <c r="A150" t="s">
         <v>195</v>
       </c>
@@ -12452,15 +12428,15 @@
         <v>213</v>
       </c>
       <c r="I150" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="151" spans="1:9" hidden="1">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9">
       <c r="A151" t="s">
         <v>195</v>
       </c>
       <c r="B151" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E151">
         <f t="shared" si="15"/>
@@ -12477,10 +12453,10 @@
         <v>213</v>
       </c>
       <c r="I151" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="152" spans="1:9" hidden="1">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9">
       <c r="A152" t="s">
         <v>195</v>
       </c>
@@ -12505,7 +12481,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="153" spans="1:9" hidden="1">
+    <row r="153" spans="1:9">
       <c r="A153" t="s">
         <v>195</v>
       </c>
@@ -12530,7 +12506,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="154" spans="1:9" hidden="1">
+    <row r="154" spans="1:9">
       <c r="A154" t="s">
         <v>195</v>
       </c>
@@ -12555,7 +12531,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="155" spans="1:9" hidden="1">
+    <row r="155" spans="1:9">
       <c r="A155" t="s">
         <v>195</v>
       </c>
@@ -12580,7 +12556,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="156" spans="1:9" hidden="1">
+    <row r="156" spans="1:9">
       <c r="A156" t="s">
         <v>195</v>
       </c>
@@ -12605,7 +12581,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="157" spans="1:9" hidden="1">
+    <row r="157" spans="1:9">
       <c r="A157" t="s">
         <v>195</v>
       </c>
@@ -12630,7 +12606,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="158" spans="1:9" hidden="1">
+    <row r="158" spans="1:9">
       <c r="A158" t="s">
         <v>195</v>
       </c>
@@ -12655,7 +12631,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="159" spans="1:9" hidden="1">
+    <row r="159" spans="1:9">
       <c r="A159" t="s">
         <v>195</v>
       </c>
@@ -12680,7 +12656,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="160" spans="1:9" hidden="1">
+    <row r="160" spans="1:9">
       <c r="A160" t="s">
         <v>195</v>
       </c>
@@ -12705,7 +12681,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="161" spans="1:9" hidden="1">
+    <row r="161" spans="1:9">
       <c r="A161" t="s">
         <v>194</v>
       </c>
@@ -12727,7 +12703,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="162" spans="1:9" hidden="1">
+    <row r="162" spans="1:9">
       <c r="A162" t="s">
         <v>194</v>
       </c>
@@ -12746,15 +12722,15 @@
         <v>5360.7265224801176</v>
       </c>
       <c r="I162" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="163" spans="1:9" hidden="1">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9">
       <c r="A163" t="s">
         <v>194</v>
       </c>
       <c r="B163" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E163">
         <f t="shared" si="16"/>
@@ -12771,7 +12747,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="164" spans="1:9" hidden="1">
+    <row r="164" spans="1:9">
       <c r="A164" t="s">
         <v>194</v>
       </c>
@@ -12790,10 +12766,10 @@
         <v>9268.2149633632525</v>
       </c>
       <c r="I164" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="165" spans="1:9" hidden="1">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9">
       <c r="A165" t="s">
         <v>194</v>
       </c>
@@ -12815,7 +12791,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="166" spans="1:9" hidden="1">
+    <row r="166" spans="1:9">
       <c r="A166" t="s">
         <v>194</v>
       </c>
@@ -12837,7 +12813,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="167" spans="1:9" hidden="1">
+    <row r="167" spans="1:9">
       <c r="A167" t="s">
         <v>194</v>
       </c>
@@ -12859,7 +12835,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="168" spans="1:9" hidden="1">
+    <row r="168" spans="1:9">
       <c r="A168" t="s">
         <v>194</v>
       </c>
@@ -12881,7 +12857,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="169" spans="1:9" hidden="1">
+    <row r="169" spans="1:9">
       <c r="A169" t="s">
         <v>194</v>
       </c>
@@ -12903,7 +12879,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="170" spans="1:9" hidden="1">
+    <row r="170" spans="1:9">
       <c r="A170" t="s">
         <v>194</v>
       </c>
@@ -12925,7 +12901,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="171" spans="1:9" hidden="1">
+    <row r="171" spans="1:9">
       <c r="A171" t="s">
         <v>194</v>
       </c>
@@ -12947,7 +12923,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="172" spans="1:9" hidden="1">
+    <row r="172" spans="1:9">
       <c r="A172" t="s">
         <v>194</v>
       </c>
@@ -12966,7 +12942,7 @@
         <v>4612.3813309600764</v>
       </c>
       <c r="I172" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -13082,20 +13058,20 @@
         <v>0</v>
       </c>
       <c r="F4">
-        <v>10194</v>
+        <v>10339</v>
       </c>
       <c r="G4">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>16405.657811516758</v>
+        <v>16639.012763711176</v>
       </c>
       <c r="H4" t="s">
         <v>241</v>
       </c>
       <c r="I4" t="s">
-        <v>242</v>
+        <v>275</v>
       </c>
       <c r="M4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -13123,7 +13099,7 @@
         <v>243</v>
       </c>
       <c r="M5" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -13151,7 +13127,7 @@
         <v>244</v>
       </c>
       <c r="M6" t="s">
-        <v>249</v>
+        <v>282</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -13179,7 +13155,7 @@
         <v>245</v>
       </c>
       <c r="M7" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -13194,17 +13170,20 @@
         <v>0</v>
       </c>
       <c r="F8">
-        <v>6681</v>
+        <v>6850</v>
       </c>
       <c r="G8">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10752.030590420192</v>
+        <v>11024.009810564035</v>
+      </c>
+      <c r="H8" t="s">
+        <v>213</v>
       </c>
       <c r="I8" t="s">
-        <v>246</v>
+        <v>278</v>
       </c>
       <c r="M8" t="s">
-        <v>254</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -13229,7 +13208,7 @@
         <v>239</v>
       </c>
       <c r="M9" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -13254,7 +13233,7 @@
         <v>240</v>
       </c>
       <c r="M10" t="s">
-        <v>257</v>
+        <v>288</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -13269,17 +13248,17 @@
         <v>0</v>
       </c>
       <c r="F11">
-        <v>9806</v>
+        <v>9750</v>
       </c>
       <c r="G11">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>15781.232146334443</v>
+        <v>15691.108854452459</v>
       </c>
       <c r="H11" t="s">
         <v>241</v>
       </c>
       <c r="I11" t="s">
-        <v>242</v>
+        <v>285</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -13369,14 +13348,17 @@
         <v>0</v>
       </c>
       <c r="F15">
-        <v>5324</v>
+        <v>5493</v>
       </c>
       <c r="G15">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8568.1501067799891</v>
+        <v>8840.1293269238322</v>
+      </c>
+      <c r="H15" t="s">
+        <v>213</v>
       </c>
       <c r="I15" t="s">
-        <v>246</v>
+        <v>278</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -13435,11 +13417,11 @@
         <v>0</v>
       </c>
       <c r="F18">
-        <v>6160</v>
+        <v>5001</v>
       </c>
       <c r="G18">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9913.5621070181696</v>
+        <v>8048.3318339606922</v>
       </c>
       <c r="I18" t="s">
         <v>242</v>
@@ -13589,11 +13571,11 @@
         <v>0</v>
       </c>
       <c r="F25">
-        <v>6227</v>
+        <v>5845</v>
       </c>
       <c r="G25">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10021.38818837697</v>
+        <v>9406.6185901820136</v>
       </c>
       <c r="I25" t="s">
         <v>242</v>
@@ -13677,11 +13659,11 @@
         <v>0</v>
       </c>
       <c r="F29">
-        <v>2982</v>
+        <v>2906</v>
       </c>
       <c r="G29">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4799.0652927156134</v>
+        <v>4676.7551108757789</v>
       </c>
       <c r="I29" t="s">
         <v>213</v>
@@ -13699,11 +13681,11 @@
         <v>0</v>
       </c>
       <c r="F30">
-        <v>3420</v>
+        <v>3392</v>
       </c>
       <c r="G30">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5503.9581827925549</v>
+        <v>5458.8965368515637</v>
       </c>
       <c r="I30" t="s">
         <v>239</v>
@@ -13721,11 +13703,11 @@
         <v>0</v>
       </c>
       <c r="F31">
-        <v>10496</v>
+        <v>9306</v>
       </c>
       <c r="G31">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>16891.679849880311</v>
+        <v>14976.559897388162</v>
       </c>
       <c r="I31" t="s">
         <v>242</v>
@@ -13743,11 +13725,11 @@
         <v>0</v>
       </c>
       <c r="F32">
-        <v>10780</v>
+        <v>10752</v>
       </c>
       <c r="G32">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>17348.733687281798</v>
+        <v>17303.672041340804</v>
       </c>
       <c r="I32" t="s">
         <v>243</v>
@@ -13765,14 +13747,14 @@
         <v>0</v>
       </c>
       <c r="F33">
-        <v>7016</v>
+        <v>7030</v>
       </c>
       <c r="G33">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11291.160997214201</v>
+        <v>11313.691820184697</v>
       </c>
       <c r="I33" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -13787,11 +13769,11 @@
         <v>0</v>
       </c>
       <c r="F34">
-        <v>8836</v>
+        <v>8808</v>
       </c>
       <c r="G34">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>14220.16798337866</v>
+        <v>14175.106337437668</v>
       </c>
       <c r="I34" t="s">
         <v>245</v>
@@ -13809,14 +13791,17 @@
         <v>0</v>
       </c>
       <c r="F35">
-        <v>5250</v>
+        <v>5391</v>
       </c>
       <c r="G35">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8449.0586139359402</v>
+        <v>8675.9761881387913</v>
+      </c>
+      <c r="H35" t="s">
+        <v>213</v>
       </c>
       <c r="I35" t="s">
-        <v>246</v>
+        <v>278</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -13838,7 +13823,7 @@
         <v>13800.129069428702</v>
       </c>
       <c r="I36" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -13875,14 +13860,14 @@
         <v>0</v>
       </c>
       <c r="F38">
-        <v>3175</v>
+        <v>2353</v>
       </c>
       <c r="G38">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5109.6687808088782</v>
+        <v>3786.7876035411937</v>
       </c>
       <c r="I38" t="s">
-        <v>242</v>
+        <v>277</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -13919,14 +13904,14 @@
         <v>0</v>
       </c>
       <c r="F40">
-        <v>4180</v>
+        <v>4477</v>
       </c>
       <c r="G40">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6727.0600011909009</v>
+        <v>7205.0353170649905</v>
       </c>
       <c r="I40" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -13963,14 +13948,14 @@
         <v>0</v>
       </c>
       <c r="F42">
-        <v>6655</v>
+        <v>6579</v>
       </c>
       <c r="G42">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10710.187633474987</v>
+        <v>10587.877451635151</v>
       </c>
       <c r="I42" t="s">
-        <v>213</v>
+        <v>278</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -14029,17 +14014,17 @@
         <v>0</v>
       </c>
       <c r="F45">
-        <v>13641</v>
+        <v>13259</v>
       </c>
       <c r="G45">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>21953.068295752411</v>
+        <v>21338.298697557453</v>
       </c>
       <c r="H45" t="s">
         <v>213</v>
       </c>
       <c r="I45" t="s">
-        <v>242</v>
+        <v>285</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -14126,14 +14111,17 @@
         <v>0</v>
       </c>
       <c r="F49">
-        <v>6008</v>
+        <v>6177</v>
       </c>
       <c r="G49">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9668.9417433385006</v>
+        <v>9940.9209634823437</v>
+      </c>
+      <c r="H49" t="s">
+        <v>213</v>
       </c>
       <c r="I49" t="s">
-        <v>246</v>
+        <v>278</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -14148,11 +14136,11 @@
         <v>0</v>
       </c>
       <c r="F50">
-        <v>6103</v>
+        <v>5988</v>
       </c>
       <c r="G50">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9821.8294706382931</v>
+        <v>9636.7548533806494</v>
       </c>
       <c r="I50" t="s">
         <v>239</v>
@@ -14170,11 +14158,11 @@
         <v>0</v>
       </c>
       <c r="F51">
-        <v>5250</v>
+        <v>5135</v>
       </c>
       <c r="G51">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8449.0586139359402</v>
+        <v>8263.9839966782947</v>
       </c>
       <c r="I51" t="s">
         <v>240</v>
@@ -14192,14 +14180,17 @@
         <v>0</v>
       </c>
       <c r="F52">
-        <v>7546</v>
+        <v>7934</v>
       </c>
       <c r="G52">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>12144.113581097257</v>
+        <v>12768.53924627957</v>
+      </c>
+      <c r="H52" t="s">
+        <v>213</v>
       </c>
       <c r="I52" t="s">
-        <v>242</v>
+        <v>275</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -14214,11 +14205,14 @@
         <v>0</v>
       </c>
       <c r="F53">
-        <v>7831</v>
+        <v>8074</v>
       </c>
       <c r="G53">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>12602.776762996637</v>
+        <v>12993.847475984529</v>
+      </c>
+      <c r="H53" t="s">
+        <v>213</v>
       </c>
       <c r="I53" t="s">
         <v>243</v>
@@ -14236,11 +14230,14 @@
         <v>0</v>
       </c>
       <c r="F54">
-        <v>2800</v>
+        <v>3043</v>
       </c>
       <c r="G54">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4506.1645940991675</v>
+        <v>4897.2353070870604</v>
+      </c>
+      <c r="H54" t="s">
+        <v>213</v>
       </c>
       <c r="I54" t="s">
         <v>244</v>
@@ -14258,11 +14255,14 @@
         <v>0</v>
       </c>
       <c r="F55">
-        <v>5758</v>
+        <v>6001</v>
       </c>
       <c r="G55">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9266.6056188653602</v>
+        <v>9657.6763318532521</v>
+      </c>
+      <c r="H55" t="s">
+        <v>213</v>
       </c>
       <c r="I55" t="s">
         <v>245</v>
@@ -14324,14 +14324,14 @@
         <v>0</v>
       </c>
       <c r="F58">
-        <v>2583</v>
+        <v>2186</v>
       </c>
       <c r="G58">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4156.936838056482</v>
+        <v>3518.0270723931362</v>
       </c>
       <c r="I58" t="s">
-        <v>242</v>
+        <v>285</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -14368,14 +14368,14 @@
         <v>0</v>
       </c>
       <c r="F60">
-        <v>3463</v>
+        <v>3760</v>
       </c>
       <c r="G60">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5573.1599962019354</v>
+        <v>6051.135312076025</v>
       </c>
       <c r="I60" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -14412,14 +14412,14 @@
         <v>0</v>
       </c>
       <c r="F62">
-        <v>5942</v>
+        <v>5866</v>
       </c>
       <c r="G62">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9562.7250064775908</v>
+        <v>9440.4148246377572</v>
       </c>
       <c r="I62" t="s">
-        <v>213</v>
+        <v>278</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -14477,7 +14477,7 @@
         <v>184</v>
       </c>
       <c r="B65" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E65">
         <f t="shared" si="5"/>
@@ -14509,17 +14509,17 @@
         <v>0</v>
       </c>
       <c r="F66">
-        <v>4452</v>
+        <v>4380</v>
       </c>
       <c r="G66">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7164.8017046176765</v>
+        <v>7048.9289007694124</v>
       </c>
       <c r="H66" t="s">
         <v>213</v>
       </c>
       <c r="I66" t="s">
-        <v>216</v>
+        <v>287</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -14881,14 +14881,14 @@
         <v>0</v>
       </c>
       <c r="F81">
-        <v>4815</v>
+        <v>4958</v>
       </c>
       <c r="G81">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7748.9937573526759</v>
+        <v>7979.1300205513126</v>
       </c>
       <c r="I81" t="s">
-        <v>214</v>
+        <v>252</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -14896,7 +14896,7 @@
         <v>180</v>
       </c>
       <c r="B82" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E82">
         <f t="shared" si="6"/>
@@ -14925,14 +14925,14 @@
         <v>0</v>
       </c>
       <c r="F83">
-        <v>5637</v>
+        <v>5631</v>
       </c>
       <c r="G83">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9071.8749346203604</v>
+        <v>9062.2188676330043</v>
       </c>
       <c r="I83" t="s">
-        <v>216</v>
+        <v>276</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -15057,14 +15057,14 @@
         <v>0</v>
       </c>
       <c r="F89">
-        <v>4786</v>
+        <v>4697</v>
       </c>
       <c r="G89">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7702.3227669137923</v>
+        <v>7559.0911066013541</v>
       </c>
       <c r="I89" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -15255,14 +15255,14 @@
         <v>0</v>
       </c>
       <c r="F98">
-        <v>4101</v>
+        <v>3952</v>
       </c>
       <c r="G98">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6599.9217858573884</v>
+        <v>6360.1294556713965</v>
       </c>
       <c r="I98" t="s">
-        <v>214</v>
+        <v>252</v>
       </c>
     </row>
     <row r="99" spans="1:9">
@@ -15270,7 +15270,7 @@
         <v>182</v>
       </c>
       <c r="B99" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E99">
         <f t="shared" si="7"/>
@@ -15299,14 +15299,14 @@
         <v>0</v>
       </c>
       <c r="F100">
-        <v>4280</v>
+        <v>5075</v>
       </c>
       <c r="G100">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6887.9944509801562</v>
+        <v>8167.4233268047419</v>
       </c>
       <c r="I100" t="s">
-        <v>216</v>
+        <v>287</v>
       </c>
     </row>
     <row r="101" spans="1:9">
@@ -15431,14 +15431,14 @@
         <v>0</v>
       </c>
       <c r="F106">
-        <v>3366</v>
+        <v>3645</v>
       </c>
       <c r="G106">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5417.0535799063564</v>
+        <v>5866.0606948183813</v>
       </c>
       <c r="I106" t="s">
-        <v>250</v>
+        <v>237</v>
       </c>
     </row>
     <row r="107" spans="1:9">
@@ -15475,14 +15475,14 @@
         <v>0</v>
       </c>
       <c r="F108">
-        <v>3733</v>
+        <v>3974</v>
       </c>
       <c r="G108">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6007.6830106329262</v>
+        <v>6395.5350346250334</v>
       </c>
       <c r="I108" t="s">
-        <v>238</v>
+        <v>281</v>
       </c>
     </row>
     <row r="109" spans="1:9">
@@ -15632,17 +15632,17 @@
         <v>0</v>
       </c>
       <c r="F115">
-        <v>4514</v>
+        <v>6177</v>
       </c>
       <c r="G115">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7264.5810634870159</v>
+        <v>9940.9209634823437</v>
       </c>
       <c r="H115" t="s">
         <v>213</v>
       </c>
       <c r="I115" t="s">
-        <v>214</v>
+        <v>252</v>
       </c>
     </row>
     <row r="116" spans="1:9">
@@ -15650,7 +15650,7 @@
         <v>183</v>
       </c>
       <c r="B116" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E116">
         <f t="shared" si="8"/>
@@ -16054,14 +16054,14 @@
         <v>0</v>
       </c>
       <c r="F132">
-        <v>4027</v>
+        <v>3980</v>
       </c>
       <c r="G132">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6480.8302930133386</v>
+        <v>6405.1911016123886</v>
       </c>
       <c r="I132" t="s">
-        <v>214</v>
+        <v>279</v>
       </c>
     </row>
     <row r="133" spans="1:9">
@@ -16069,7 +16069,7 @@
         <v>185</v>
       </c>
       <c r="B133" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E133">
         <f t="shared" si="8"/>
@@ -16098,14 +16098,14 @@
         <v>0</v>
       </c>
       <c r="F134">
-        <v>4206</v>
+        <v>4172</v>
       </c>
       <c r="G134">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6768.9029581361074</v>
+        <v>6714.1852452077601</v>
       </c>
       <c r="I134" t="s">
-        <v>216</v>
+        <v>276</v>
       </c>
     </row>
     <row r="135" spans="1:9">
@@ -16237,7 +16237,7 @@
         <v>5405.7881684211088</v>
       </c>
       <c r="I140" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="141" spans="1:9">
@@ -16252,14 +16252,14 @@
         <v>0</v>
       </c>
       <c r="F141">
-        <v>4978</v>
+        <v>5109</v>
       </c>
       <c r="G141">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8011.3169105091638</v>
+        <v>8222.1410397330892</v>
       </c>
       <c r="I141" t="s">
-        <v>223</v>
+        <v>280</v>
       </c>
     </row>
     <row r="142" spans="1:9">
@@ -16274,14 +16274,14 @@
         <v>0</v>
       </c>
       <c r="F142">
-        <v>4162</v>
+        <v>4309</v>
       </c>
       <c r="G142">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6698.0918002288345</v>
+        <v>6934.6654414190407</v>
       </c>
       <c r="I142" t="s">
-        <v>238</v>
+        <v>281</v>
       </c>
     </row>
     <row r="143" spans="1:9">
@@ -16449,7 +16449,7 @@
         <v>186</v>
       </c>
       <c r="B150" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E150">
         <f t="shared" si="9"/>
@@ -16853,11 +16853,11 @@
         <v>0</v>
       </c>
       <c r="F166">
-        <v>1512</v>
+        <v>1405</v>
       </c>
       <c r="G166">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>2433.3288808135508</v>
+        <v>2261.1290195390466</v>
       </c>
       <c r="I166" t="s">
         <v>214</v>
@@ -16868,18 +16868,18 @@
         <v>192</v>
       </c>
       <c r="B167" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E167">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F167">
-        <v>599</v>
+        <v>518</v>
       </c>
       <c r="G167">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>963.99735423764344</v>
+        <v>833.64044990834611</v>
       </c>
       <c r="I167" t="s">
         <v>215</v>
@@ -16897,14 +16897,14 @@
         <v>0</v>
       </c>
       <c r="F168">
-        <v>1383</v>
+        <v>1239</v>
       </c>
       <c r="G168">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>2225.7234405854106</v>
+        <v>1993.9778328888817</v>
       </c>
       <c r="I168" t="s">
-        <v>216</v>
+        <v>276</v>
       </c>
     </row>
     <row r="169" spans="1:9">
@@ -16985,11 +16985,11 @@
         <v>0</v>
       </c>
       <c r="F172">
-        <v>3951</v>
+        <v>3836</v>
       </c>
       <c r="G172">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6358.5201111735041</v>
+        <v>6173.4454939158604</v>
       </c>
       <c r="I172" t="s">
         <v>220</v>
@@ -17007,11 +17007,11 @@
         <v>0</v>
       </c>
       <c r="F173">
-        <v>2197</v>
+        <v>2082</v>
       </c>
       <c r="G173">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>3535.7298618699542</v>
+        <v>3350.6552446123096</v>
       </c>
       <c r="I173" t="s">
         <v>221</v>
@@ -17029,14 +17029,14 @@
         <v>0</v>
       </c>
       <c r="F174">
-        <v>1588</v>
+        <v>1696</v>
       </c>
       <c r="G174">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>2555.6390626533853</v>
+        <v>2729.4482684257819</v>
       </c>
       <c r="I174" t="s">
-        <v>222</v>
+        <v>283</v>
       </c>
     </row>
     <row r="175" spans="1:9">
@@ -17051,14 +17051,14 @@
         <v>0</v>
       </c>
       <c r="F175">
-        <v>598</v>
+        <v>722</v>
       </c>
       <c r="G175">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>962.38800973975083</v>
+        <v>1161.9467274784283</v>
       </c>
       <c r="I175" t="s">
-        <v>223</v>
+        <v>280</v>
       </c>
     </row>
     <row r="176" spans="1:9">
@@ -17073,11 +17073,11 @@
         <v>0</v>
       </c>
       <c r="F176">
-        <v>3022</v>
+        <v>2907</v>
       </c>
       <c r="G176">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4863.4390726313159</v>
+        <v>4678.3644553736722</v>
       </c>
       <c r="I176" t="s">
         <v>238</v>
@@ -17230,17 +17230,17 @@
         <v>0</v>
       </c>
       <c r="F183">
-        <v>7541</v>
+        <v>8897</v>
       </c>
       <c r="G183">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>12136.066858607795</v>
+        <v>14318.337997750106</v>
       </c>
       <c r="H183" t="s">
         <v>213</v>
       </c>
       <c r="I183" t="s">
-        <v>214</v>
+        <v>279</v>
       </c>
     </row>
     <row r="184" spans="1:9">
@@ -17248,24 +17248,24 @@
         <v>195</v>
       </c>
       <c r="B184" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E184">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F184">
-        <v>6628</v>
+        <v>6737</v>
       </c>
       <c r="G184">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10666.735332031887</v>
+        <v>10842.153882302176</v>
       </c>
       <c r="H184" t="s">
         <v>213</v>
       </c>
       <c r="I184" t="s">
-        <v>215</v>
+        <v>286</v>
       </c>
     </row>
     <row r="185" spans="1:9">
@@ -17652,14 +17652,14 @@
         <v>0</v>
       </c>
       <c r="F200">
-        <v>2873</v>
+        <v>3331</v>
       </c>
       <c r="G200">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4623.6467424453249</v>
+        <v>5360.7265224801176</v>
       </c>
       <c r="I200" t="s">
-        <v>256</v>
+        <v>279</v>
       </c>
     </row>
     <row r="201" spans="1:9">
@@ -17667,7 +17667,7 @@
         <v>194</v>
       </c>
       <c r="B201" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E201">
         <f t="shared" si="12"/>
@@ -17696,14 +17696,14 @@
         <v>0</v>
       </c>
       <c r="F202">
-        <v>4964</v>
+        <v>5759</v>
       </c>
       <c r="G202">
         <f>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7988.7860875386677</v>
+        <v>9268.2149633632525</v>
       </c>
       <c r="I202" t="s">
-        <v>216</v>
+        <v>287</v>
       </c>
     </row>
     <row r="203" spans="1:9">
@@ -17879,7 +17879,7 @@
         <v>4612.3813309600764</v>
       </c>
       <c r="I210" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
     </row>
     <row r="211" spans="1:9">
@@ -18128,7 +18128,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C4">
         <v>7</v>
@@ -18152,7 +18152,7 @@
         <v>73.274999999999991</v>
       </c>
       <c r="J4" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="K4" t="s">
         <v>101</v>
@@ -18799,10 +18799,10 @@
         <v>122</v>
       </c>
       <c r="F1" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="G1" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="M1" t="s">
         <v>93</v>
@@ -19276,7 +19276,7 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B16" t="s">
         <v>3</v>
@@ -20242,10 +20242,10 @@
         <v>172</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -20631,10 +20631,10 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="B21" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -22269,10 +22269,10 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="B21" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -22316,7 +22316,7 @@
         <v>119</v>
       </c>
       <c r="G1" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -22629,7 +22629,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B14" t="s">
         <v>3</v>
@@ -23432,7 +23432,7 @@
         <v>172</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>105</v>
@@ -24253,7 +24253,7 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B14" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
update data prep and bug fix
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA3E34E-253C-4D50-A14C-04E7B7A63E9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50CA3225-8092-4FB6-88FE-855204EAD512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="13" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng_europe_2020" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
get first (preliminary) results
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50CA3225-8092-4FB6-88FE-855204EAD512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{747E3476-195E-4041-AE21-6096722456BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="13" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2660" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2653" uniqueCount="289">
   <si>
     <t>Belgium</t>
   </si>
@@ -1785,8 +1785,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I172" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
-  <autoFilter ref="A1:I172" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I170" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
+  <autoFilter ref="A1:I170" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
     <tableColumn id="2" xr3:uid="{36192F9A-102D-4019-9A43-508B12FDAFA2}" name="To"/>
@@ -8911,7 +8911,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M172"/>
+  <dimension ref="A1:M170"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="21.81640625" customWidth="1"/>
@@ -10680,27 +10680,24 @@
     </row>
     <row r="75" spans="1:9">
       <c r="A75" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B75" t="s">
-        <v>224</v>
+        <v>201</v>
       </c>
       <c r="E75">
-        <f t="shared" ref="E75" si="8">D75/1000</f>
+        <f>D75/1000</f>
         <v>0</v>
       </c>
       <c r="F75">
-        <v>7423</v>
+        <v>4986</v>
       </c>
       <c r="G75">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11946.164207856473</v>
-      </c>
-      <c r="H75" t="s">
-        <v>213</v>
+        <v>8024.1916664923037</v>
       </c>
       <c r="I75" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -10708,21 +10705,21 @@
         <v>180</v>
       </c>
       <c r="B76" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E76">
-        <f>D76/1000</f>
+        <f t="shared" ref="E76:E86" si="8">D76/1000</f>
         <v>0</v>
       </c>
       <c r="F76">
-        <v>4986</v>
+        <v>4958</v>
       </c>
       <c r="G76">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8024.1916664923037</v>
+        <v>7979.1300205513126</v>
       </c>
       <c r="I76" t="s">
-        <v>234</v>
+        <v>252</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -10730,21 +10727,21 @@
         <v>180</v>
       </c>
       <c r="B77" t="s">
-        <v>202</v>
+        <v>268</v>
       </c>
       <c r="E77">
-        <f t="shared" ref="E77:E88" si="9">D77/1000</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F77">
-        <v>4958</v>
+        <v>6255</v>
       </c>
       <c r="G77">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7979.1300205513126</v>
+        <v>10066.449834317962</v>
       </c>
       <c r="I77" t="s">
-        <v>252</v>
+        <v>215</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -10752,21 +10749,21 @@
         <v>180</v>
       </c>
       <c r="B78" t="s">
-        <v>268</v>
+        <v>203</v>
       </c>
       <c r="E78">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F78">
-        <v>6255</v>
+        <v>5631</v>
       </c>
       <c r="G78">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10066.449834317962</v>
+        <v>9062.2188676330043</v>
       </c>
       <c r="I78" t="s">
-        <v>215</v>
+        <v>276</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -10774,21 +10771,21 @@
         <v>180</v>
       </c>
       <c r="B79" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E79">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F79">
-        <v>5631</v>
+        <v>6380</v>
       </c>
       <c r="G79">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9062.2188676330043</v>
+        <v>10267.617896554533</v>
       </c>
       <c r="I79" t="s">
-        <v>276</v>
+        <v>217</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -10796,21 +10793,21 @@
         <v>180</v>
       </c>
       <c r="B80" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E80">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F80">
-        <v>6380</v>
+        <v>5634</v>
       </c>
       <c r="G80">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10267.617896554533</v>
+        <v>9067.0469011266832</v>
       </c>
       <c r="I80" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -10818,21 +10815,21 @@
         <v>180</v>
       </c>
       <c r="B81" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E81">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F81">
-        <v>5634</v>
+        <v>5052</v>
       </c>
       <c r="G81">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9067.0469011266832</v>
+        <v>8130.4084033532126</v>
       </c>
       <c r="I81" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -10840,21 +10837,21 @@
         <v>180</v>
       </c>
       <c r="B82" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E82">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F82">
-        <v>5052</v>
+        <v>5443</v>
       </c>
       <c r="G82">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8130.4084033532126</v>
+        <v>8759.6621020292041</v>
       </c>
       <c r="I82" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -10862,21 +10859,21 @@
         <v>180</v>
       </c>
       <c r="B83" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E83">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F83">
-        <v>5443</v>
+        <v>4565</v>
       </c>
       <c r="G83">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8759.6621020292041</v>
+        <v>7346.6576328795363</v>
       </c>
       <c r="I83" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -10884,21 +10881,21 @@
         <v>180</v>
       </c>
       <c r="B84" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E84">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F84">
-        <v>4565</v>
+        <v>4697</v>
       </c>
       <c r="G84">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7346.6576328795363</v>
+        <v>7559.0911066013541</v>
       </c>
       <c r="I84" t="s">
-        <v>221</v>
+        <v>248</v>
       </c>
     </row>
     <row r="85" spans="1:9">
@@ -10906,21 +10903,21 @@
         <v>180</v>
       </c>
       <c r="B85" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E85">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F85">
-        <v>4697</v>
+        <v>6409</v>
       </c>
       <c r="G85">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7559.0911066013541</v>
+        <v>10314.288886993416</v>
       </c>
       <c r="I85" t="s">
-        <v>248</v>
+        <v>223</v>
       </c>
     </row>
     <row r="86" spans="1:9">
@@ -10928,65 +10925,65 @@
         <v>180</v>
       </c>
       <c r="B86" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E86">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="F86">
-        <v>6409</v>
+        <v>4666</v>
       </c>
       <c r="G86">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10314.288886993416</v>
+        <v>7509.2014271666849</v>
       </c>
       <c r="I86" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
     </row>
     <row r="87" spans="1:9">
       <c r="A87" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B87" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="E87">
-        <f t="shared" si="9"/>
+        <f>D87/1000</f>
         <v>0</v>
       </c>
       <c r="F87">
-        <v>4666</v>
+        <v>3985</v>
       </c>
       <c r="G87">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7509.2014271666849</v>
+        <v>6413.2378241018514</v>
       </c>
       <c r="I87" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
     </row>
     <row r="88" spans="1:9">
       <c r="A88" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B88" t="s">
-        <v>224</v>
+        <v>202</v>
       </c>
       <c r="E88">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="E88:E98" si="9">D88/1000</f>
         <v>0</v>
       </c>
       <c r="F88">
-        <v>5846</v>
+        <v>3952</v>
       </c>
       <c r="G88">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9408.227934679906</v>
+        <v>6360.1294556713965</v>
       </c>
       <c r="I88" t="s">
-        <v>229</v>
+        <v>252</v>
       </c>
     </row>
     <row r="89" spans="1:9">
@@ -10994,21 +10991,21 @@
         <v>182</v>
       </c>
       <c r="B89" t="s">
-        <v>201</v>
+        <v>268</v>
       </c>
       <c r="E89">
-        <f>D89/1000</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F89">
-        <v>3985</v>
+        <v>4898</v>
       </c>
       <c r="G89">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6413.2378241018514</v>
+        <v>7882.5693506777588</v>
       </c>
       <c r="I89" t="s">
-        <v>234</v>
+        <v>215</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -11016,21 +11013,21 @@
         <v>182</v>
       </c>
       <c r="B90" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E90">
-        <f t="shared" ref="E90:E100" si="10">D90/1000</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F90">
-        <v>3952</v>
+        <v>5075</v>
       </c>
       <c r="G90">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6360.1294556713965</v>
+        <v>8167.4233268047419</v>
       </c>
       <c r="I90" t="s">
-        <v>252</v>
+        <v>287</v>
       </c>
     </row>
     <row r="91" spans="1:9">
@@ -11038,21 +11035,21 @@
         <v>182</v>
       </c>
       <c r="B91" t="s">
-        <v>268</v>
+        <v>204</v>
       </c>
       <c r="E91">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F91">
-        <v>4898</v>
+        <v>5023</v>
       </c>
       <c r="G91">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7882.5693506777588</v>
+        <v>8083.7374129143291</v>
       </c>
       <c r="I91" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="92" spans="1:9">
@@ -11060,21 +11057,21 @@
         <v>182</v>
       </c>
       <c r="B92" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E92">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F92">
-        <v>5075</v>
+        <v>4823</v>
       </c>
       <c r="G92">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8167.4233268047419</v>
+        <v>7761.8685133358167</v>
       </c>
       <c r="I92" t="s">
-        <v>287</v>
+        <v>218</v>
       </c>
     </row>
     <row r="93" spans="1:9">
@@ -11082,21 +11079,21 @@
         <v>182</v>
       </c>
       <c r="B93" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E93">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F93">
-        <v>5023</v>
+        <v>4051</v>
       </c>
       <c r="G93">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8083.7374129143291</v>
+        <v>6519.4545609627603</v>
       </c>
       <c r="I93" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="94" spans="1:9">
@@ -11104,21 +11101,21 @@
         <v>182</v>
       </c>
       <c r="B94" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E94">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F94">
-        <v>4823</v>
+        <v>4632</v>
       </c>
       <c r="G94">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7761.8685133358167</v>
+        <v>7454.4837142383376</v>
       </c>
       <c r="I94" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="95" spans="1:9">
@@ -11126,21 +11123,21 @@
         <v>182</v>
       </c>
       <c r="B95" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E95">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F95">
-        <v>4051</v>
+        <v>3299</v>
       </c>
       <c r="G95">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6519.4545609627603</v>
+        <v>5309.2274985475551</v>
       </c>
       <c r="I95" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="96" spans="1:9">
@@ -11148,21 +11145,21 @@
         <v>182</v>
       </c>
       <c r="B96" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E96">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F96">
-        <v>4632</v>
+        <v>3645</v>
       </c>
       <c r="G96">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7454.4837142383376</v>
+        <v>5866.0606948183813</v>
       </c>
       <c r="I96" t="s">
-        <v>220</v>
+        <v>237</v>
       </c>
     </row>
     <row r="97" spans="1:9">
@@ -11170,21 +11167,21 @@
         <v>182</v>
       </c>
       <c r="B97" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E97">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F97">
-        <v>3299</v>
+        <v>5052</v>
       </c>
       <c r="G97">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5309.2274985475551</v>
+        <v>8130.4084033532126</v>
       </c>
       <c r="I97" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="98" spans="1:9">
@@ -11192,65 +11189,71 @@
         <v>182</v>
       </c>
       <c r="B98" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E98">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="F98">
-        <v>3645</v>
+        <v>3974</v>
       </c>
       <c r="G98">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5866.0606948183813</v>
+        <v>6395.5350346250334</v>
       </c>
       <c r="I98" t="s">
-        <v>237</v>
+        <v>281</v>
       </c>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B99" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="E99">
-        <f t="shared" si="10"/>
+        <f>D99/1000</f>
         <v>0</v>
       </c>
       <c r="F99">
-        <v>5052</v>
+        <v>6210</v>
       </c>
       <c r="G99">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8130.4084033532126</v>
+        <v>9994.0293319127977</v>
+      </c>
+      <c r="H99" t="s">
+        <v>213</v>
       </c>
       <c r="I99" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
     </row>
     <row r="100" spans="1:9">
       <c r="A100" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B100" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="E100">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="E100:E110" si="10">D100/1000</f>
         <v>0</v>
       </c>
       <c r="F100">
-        <v>3974</v>
+        <v>6177</v>
       </c>
       <c r="G100">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6395.5350346250334</v>
+        <v>9940.9209634823437</v>
+      </c>
+      <c r="H100" t="s">
+        <v>213</v>
       </c>
       <c r="I100" t="s">
-        <v>281</v>
+        <v>252</v>
       </c>
     </row>
     <row r="101" spans="1:9">
@@ -11258,24 +11261,24 @@
         <v>183</v>
       </c>
       <c r="B101" t="s">
-        <v>201</v>
+        <v>268</v>
       </c>
       <c r="E101">
-        <f>D101/1000</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F101">
-        <v>6210</v>
+        <v>3601</v>
       </c>
       <c r="G101">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9994.0293319127977</v>
+        <v>5795.2495369111084</v>
       </c>
       <c r="H101" t="s">
         <v>213</v>
       </c>
       <c r="I101" t="s">
-        <v>234</v>
+        <v>215</v>
       </c>
     </row>
     <row r="102" spans="1:9">
@@ -11283,24 +11286,24 @@
         <v>183</v>
       </c>
       <c r="B102" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E102">
-        <f t="shared" ref="E102:E112" si="11">D102/1000</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F102">
-        <v>6177</v>
+        <v>4385</v>
       </c>
       <c r="G102">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9940.9209634823437</v>
+        <v>7056.9756232588752</v>
       </c>
       <c r="H102" t="s">
         <v>213</v>
       </c>
       <c r="I102" t="s">
-        <v>252</v>
+        <v>216</v>
       </c>
     </row>
     <row r="103" spans="1:9">
@@ -11308,24 +11311,24 @@
         <v>183</v>
       </c>
       <c r="B103" t="s">
-        <v>268</v>
+        <v>204</v>
       </c>
       <c r="E103">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F103">
-        <v>3601</v>
+        <v>4260</v>
       </c>
       <c r="G103">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5795.2495369111084</v>
+        <v>6855.807561022305</v>
       </c>
       <c r="H103" t="s">
         <v>213</v>
       </c>
       <c r="I103" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="104" spans="1:9">
@@ -11333,24 +11336,24 @@
         <v>183</v>
       </c>
       <c r="B104" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E104">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F104">
-        <v>4385</v>
+        <v>7144</v>
       </c>
       <c r="G104">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7056.9756232588752</v>
+        <v>11497.157092944448</v>
       </c>
       <c r="H104" t="s">
         <v>213</v>
       </c>
       <c r="I104" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="105" spans="1:9">
@@ -11358,24 +11361,24 @@
         <v>183</v>
       </c>
       <c r="B105" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E105">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F105">
-        <v>4260</v>
+        <v>6276</v>
       </c>
       <c r="G105">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6855.807561022305</v>
+        <v>10100.246068773706</v>
       </c>
       <c r="H105" t="s">
         <v>213</v>
       </c>
       <c r="I105" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="106" spans="1:9">
@@ -11383,24 +11386,24 @@
         <v>183</v>
       </c>
       <c r="B106" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E106">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F106">
-        <v>7144</v>
+        <v>6953</v>
       </c>
       <c r="G106">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11497.157092944448</v>
+        <v>11189.772293846969</v>
       </c>
       <c r="H106" t="s">
         <v>213</v>
       </c>
       <c r="I106" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="107" spans="1:9">
@@ -11408,24 +11411,24 @@
         <v>183</v>
       </c>
       <c r="B107" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E107">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F107">
-        <v>6276</v>
+        <v>5199</v>
       </c>
       <c r="G107">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10100.246068773706</v>
+        <v>8366.9820445434198</v>
       </c>
       <c r="H107" t="s">
         <v>213</v>
       </c>
       <c r="I107" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="108" spans="1:9">
@@ -11433,24 +11436,24 @@
         <v>183</v>
       </c>
       <c r="B108" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E108">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F108">
-        <v>6953</v>
+        <v>4590</v>
       </c>
       <c r="G108">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11189.772293846969</v>
+        <v>7386.8912453268504</v>
       </c>
       <c r="H108" t="s">
         <v>213</v>
       </c>
       <c r="I108" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="109" spans="1:9">
@@ -11458,24 +11461,24 @@
         <v>183</v>
       </c>
       <c r="B109" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E109">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F109">
-        <v>5199</v>
+        <v>3600</v>
       </c>
       <c r="G109">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8366.9820445434198</v>
+        <v>5793.640192413216</v>
       </c>
       <c r="H109" t="s">
         <v>213</v>
       </c>
       <c r="I109" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="110" spans="1:9">
@@ -11483,74 +11486,68 @@
         <v>183</v>
       </c>
       <c r="B110" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E110">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="F110">
-        <v>4590</v>
+        <v>6024</v>
       </c>
       <c r="G110">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7386.8912453268504</v>
+        <v>9694.6912553047805</v>
       </c>
       <c r="H110" t="s">
         <v>213</v>
       </c>
       <c r="I110" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
     </row>
     <row r="111" spans="1:9">
       <c r="A111" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B111" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="E111">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="E111:E122" si="11">D111/1000</f>
         <v>0</v>
       </c>
       <c r="F111">
-        <v>3600</v>
+        <v>4348</v>
       </c>
       <c r="G111">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5793.640192413216</v>
-      </c>
-      <c r="H111" t="s">
-        <v>213</v>
+        <v>6997.4298768368508</v>
       </c>
       <c r="I111" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
     </row>
     <row r="112" spans="1:9">
       <c r="A112" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B112" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="E112">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F112">
-        <v>6024</v>
+        <v>3980</v>
       </c>
       <c r="G112">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9694.6912553047805</v>
-      </c>
-      <c r="H112" t="s">
-        <v>213</v>
+        <v>6405.1911016123886</v>
       </c>
       <c r="I112" t="s">
-        <v>238</v>
+        <v>279</v>
       </c>
     </row>
     <row r="113" spans="1:9">
@@ -11558,21 +11555,21 @@
         <v>185</v>
       </c>
       <c r="B113" t="s">
-        <v>201</v>
+        <v>268</v>
       </c>
       <c r="E113">
-        <f t="shared" ref="E113:E124" si="12">D113/1000</f>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F113">
-        <v>4348</v>
+        <v>4824</v>
       </c>
       <c r="G113">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6997.4298768368508</v>
+        <v>7763.4778578337091</v>
       </c>
       <c r="I113" t="s">
-        <v>234</v>
+        <v>215</v>
       </c>
     </row>
     <row r="114" spans="1:9">
@@ -11580,21 +11577,21 @@
         <v>185</v>
       </c>
       <c r="B114" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E114">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F114">
-        <v>3980</v>
+        <v>4172</v>
       </c>
       <c r="G114">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6405.1911016123886</v>
+        <v>6714.1852452077601</v>
       </c>
       <c r="I114" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="115" spans="1:9">
@@ -11602,21 +11599,21 @@
         <v>185</v>
       </c>
       <c r="B115" t="s">
-        <v>268</v>
+        <v>204</v>
       </c>
       <c r="E115">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F115">
-        <v>4824</v>
+        <v>4949</v>
       </c>
       <c r="G115">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7763.4778578337091</v>
+        <v>7964.6459200702793</v>
       </c>
       <c r="I115" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="116" spans="1:9">
@@ -11624,21 +11621,21 @@
         <v>185</v>
       </c>
       <c r="B116" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E116">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F116">
-        <v>4172</v>
+        <v>5282</v>
       </c>
       <c r="G116">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6714.1852452077601</v>
+        <v>8500.5576378685018</v>
       </c>
       <c r="I116" t="s">
-        <v>276</v>
+        <v>218</v>
       </c>
     </row>
     <row r="117" spans="1:9">
@@ -11646,21 +11643,21 @@
         <v>185</v>
       </c>
       <c r="B117" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E117">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F117">
-        <v>4949</v>
+        <v>4414</v>
       </c>
       <c r="G117">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7964.6459200702793</v>
+        <v>7103.6466136977597</v>
       </c>
       <c r="I117" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="118" spans="1:9">
@@ -11668,21 +11665,21 @@
         <v>185</v>
       </c>
       <c r="B118" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E118">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F118">
-        <v>5282</v>
+        <v>5091</v>
       </c>
       <c r="G118">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8500.5576378685018</v>
+        <v>8193.1728387710227</v>
       </c>
       <c r="I118" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="119" spans="1:9">
@@ -11690,21 +11687,21 @@
         <v>185</v>
       </c>
       <c r="B119" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E119">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F119">
-        <v>4414</v>
+        <v>3389</v>
       </c>
       <c r="G119">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>7103.6466136977597</v>
+        <v>5454.0685033578857</v>
       </c>
       <c r="I119" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="120" spans="1:9">
@@ -11712,21 +11709,21 @@
         <v>185</v>
       </c>
       <c r="B120" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E120">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F120">
-        <v>5091</v>
+        <v>3359</v>
       </c>
       <c r="G120">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8193.1728387710227</v>
+        <v>5405.7881684211088</v>
       </c>
       <c r="I120" t="s">
-        <v>220</v>
+        <v>248</v>
       </c>
     </row>
     <row r="121" spans="1:9">
@@ -11734,21 +11731,21 @@
         <v>185</v>
       </c>
       <c r="B121" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E121">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F121">
-        <v>3389</v>
+        <v>5109</v>
       </c>
       <c r="G121">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5454.0685033578857</v>
+        <v>8222.1410397330892</v>
       </c>
       <c r="I121" t="s">
-        <v>221</v>
+        <v>280</v>
       </c>
     </row>
     <row r="122" spans="1:9">
@@ -11756,65 +11753,71 @@
         <v>185</v>
       </c>
       <c r="B122" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E122">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="F122">
-        <v>3359</v>
+        <v>4309</v>
       </c>
       <c r="G122">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5405.7881684211088</v>
+        <v>6934.6654414190407</v>
       </c>
       <c r="I122" t="s">
-        <v>248</v>
+        <v>281</v>
       </c>
     </row>
     <row r="123" spans="1:9">
       <c r="A123" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B123" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="E123">
-        <f t="shared" si="12"/>
+        <f>D123/1000</f>
         <v>0</v>
       </c>
       <c r="F123">
-        <v>5109</v>
+        <v>9950</v>
       </c>
       <c r="G123">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8222.1410397330892</v>
+        <v>16012.977754030971</v>
+      </c>
+      <c r="H123" t="s">
+        <v>213</v>
       </c>
       <c r="I123" t="s">
-        <v>280</v>
+        <v>234</v>
       </c>
     </row>
     <row r="124" spans="1:9">
       <c r="A124" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B124" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="E124">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="E124:E134" si="12">D124/1000</f>
         <v>0</v>
       </c>
       <c r="F124">
-        <v>4309</v>
+        <v>8254</v>
       </c>
       <c r="G124">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6934.6654414190407</v>
+        <v>13283.52948560519</v>
+      </c>
+      <c r="H124" t="s">
+        <v>213</v>
       </c>
       <c r="I124" t="s">
-        <v>281</v>
+        <v>214</v>
       </c>
     </row>
     <row r="125" spans="1:9">
@@ -11822,24 +11825,24 @@
         <v>186</v>
       </c>
       <c r="B125" t="s">
-        <v>201</v>
+        <v>268</v>
       </c>
       <c r="E125">
-        <f>D125/1000</f>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F125">
-        <v>9950</v>
+        <v>7341</v>
       </c>
       <c r="G125">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>16012.977754030971</v>
+        <v>11814.197959029283</v>
       </c>
       <c r="H125" t="s">
         <v>213</v>
       </c>
       <c r="I125" t="s">
-        <v>234</v>
+        <v>215</v>
       </c>
     </row>
     <row r="126" spans="1:9">
@@ -11847,24 +11850,24 @@
         <v>186</v>
       </c>
       <c r="B126" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E126">
-        <f t="shared" ref="E126:E136" si="13">D126/1000</f>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F126">
-        <v>8254</v>
+        <v>8125</v>
       </c>
       <c r="G126">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>13283.52948560519</v>
+        <v>13075.924045377049</v>
       </c>
       <c r="H126" t="s">
         <v>213</v>
       </c>
       <c r="I126" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="127" spans="1:9">
@@ -11872,24 +11875,24 @@
         <v>186</v>
       </c>
       <c r="B127" t="s">
-        <v>268</v>
+        <v>204</v>
       </c>
       <c r="E127">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F127">
-        <v>7341</v>
+        <v>8000</v>
       </c>
       <c r="G127">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11814.197959029283</v>
+        <v>12874.75598314048</v>
       </c>
       <c r="H127" t="s">
         <v>213</v>
       </c>
       <c r="I127" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="128" spans="1:9">
@@ -11897,24 +11900,24 @@
         <v>186</v>
       </c>
       <c r="B128" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E128">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F128">
-        <v>8125</v>
+        <v>10884</v>
       </c>
       <c r="G128">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>13075.924045377049</v>
+        <v>17516.105515062623</v>
       </c>
       <c r="H128" t="s">
         <v>213</v>
       </c>
       <c r="I128" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="129" spans="1:9">
@@ -11922,24 +11925,24 @@
         <v>186</v>
       </c>
       <c r="B129" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E129">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F129">
-        <v>8000</v>
+        <v>10016</v>
       </c>
       <c r="G129">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>12874.75598314048</v>
+        <v>16119.194490891881</v>
       </c>
       <c r="H129" t="s">
         <v>213</v>
       </c>
       <c r="I129" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="130" spans="1:9">
@@ -11947,24 +11950,24 @@
         <v>186</v>
       </c>
       <c r="B130" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E130">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F130">
-        <v>10884</v>
+        <v>10693</v>
       </c>
       <c r="G130">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>17516.105515062623</v>
+        <v>17208.720715965144</v>
       </c>
       <c r="H130" t="s">
         <v>213</v>
       </c>
       <c r="I130" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="131" spans="1:9">
@@ -11972,24 +11975,24 @@
         <v>186</v>
       </c>
       <c r="B131" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E131">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F131">
-        <v>10016</v>
+        <v>8939</v>
       </c>
       <c r="G131">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>16119.194490891881</v>
+        <v>14385.930466661594</v>
       </c>
       <c r="H131" t="s">
         <v>213</v>
       </c>
       <c r="I131" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="132" spans="1:9">
@@ -11997,24 +12000,24 @@
         <v>186</v>
       </c>
       <c r="B132" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E132">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F132">
-        <v>10693</v>
+        <v>8330</v>
       </c>
       <c r="G132">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>17208.720715965144</v>
+        <v>13405.839667445025</v>
       </c>
       <c r="H132" t="s">
         <v>213</v>
       </c>
       <c r="I132" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="133" spans="1:9">
@@ -12022,24 +12025,24 @@
         <v>186</v>
       </c>
       <c r="B133" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E133">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F133">
-        <v>8939</v>
+        <v>7340</v>
       </c>
       <c r="G133">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>14385.930466661594</v>
+        <v>11812.588614531391</v>
       </c>
       <c r="H133" t="s">
         <v>213</v>
       </c>
       <c r="I133" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="134" spans="1:9">
@@ -12047,74 +12050,68 @@
         <v>186</v>
       </c>
       <c r="B134" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E134">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="F134">
-        <v>8330</v>
+        <v>9764</v>
       </c>
       <c r="G134">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>13405.839667445025</v>
+        <v>15713.639677422956</v>
       </c>
       <c r="H134" t="s">
         <v>213</v>
       </c>
       <c r="I134" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
     </row>
     <row r="135" spans="1:9">
       <c r="A135" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="B135" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="E135">
-        <f t="shared" si="13"/>
+        <f>D135/1000</f>
         <v>0</v>
       </c>
       <c r="F135">
-        <v>7340</v>
+        <v>3208</v>
       </c>
       <c r="G135">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11812.588614531391</v>
-      </c>
-      <c r="H135" t="s">
-        <v>213</v>
+        <v>5162.7771492393322</v>
       </c>
       <c r="I135" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
     </row>
     <row r="136" spans="1:9">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="B136" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="E136">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="E136:E146" si="13">D136/1000</f>
         <v>0</v>
       </c>
       <c r="F136">
-        <v>9764</v>
+        <v>1405</v>
       </c>
       <c r="G136">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>15713.639677422956</v>
-      </c>
-      <c r="H136" t="s">
-        <v>213</v>
+        <v>2261.1290195390466</v>
       </c>
       <c r="I136" t="s">
-        <v>238</v>
+        <v>214</v>
       </c>
     </row>
     <row r="137" spans="1:9">
@@ -12122,21 +12119,21 @@
         <v>192</v>
       </c>
       <c r="B137" t="s">
-        <v>201</v>
+        <v>268</v>
       </c>
       <c r="E137">
-        <f>D137/1000</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="F137">
-        <v>3208</v>
+        <v>518</v>
       </c>
       <c r="G137">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5162.7771492393322</v>
+        <v>833.64044990834611</v>
       </c>
       <c r="I137" t="s">
-        <v>234</v>
+        <v>215</v>
       </c>
     </row>
     <row r="138" spans="1:9">
@@ -12144,21 +12141,21 @@
         <v>192</v>
       </c>
       <c r="B138" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E138">
-        <f t="shared" ref="E138:E148" si="14">D138/1000</f>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="F138">
-        <v>1405</v>
+        <v>1239</v>
       </c>
       <c r="G138">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>2261.1290195390466</v>
+        <v>1993.9778328888817</v>
       </c>
       <c r="I138" t="s">
-        <v>214</v>
+        <v>276</v>
       </c>
     </row>
     <row r="139" spans="1:9">
@@ -12166,21 +12163,21 @@
         <v>192</v>
       </c>
       <c r="B139" t="s">
-        <v>268</v>
+        <v>204</v>
       </c>
       <c r="E139">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="F139">
-        <v>518</v>
+        <v>1258</v>
       </c>
       <c r="G139">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>833.64044990834611</v>
+        <v>2024.5553783488403</v>
       </c>
       <c r="I139" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="140" spans="1:9">
@@ -12188,21 +12185,21 @@
         <v>192</v>
       </c>
       <c r="B140" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E140">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="F140">
-        <v>1239</v>
+        <v>4142</v>
       </c>
       <c r="G140">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>1993.9778328888817</v>
+        <v>6665.9049102709832</v>
       </c>
       <c r="I140" t="s">
-        <v>276</v>
+        <v>218</v>
       </c>
     </row>
     <row r="141" spans="1:9">
@@ -12210,21 +12207,21 @@
         <v>192</v>
       </c>
       <c r="B141" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E141">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="F141">
-        <v>1258</v>
+        <v>3274</v>
       </c>
       <c r="G141">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>2024.5553783488403</v>
+        <v>5268.9938861002411</v>
       </c>
       <c r="I141" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="142" spans="1:9">
@@ -12232,21 +12229,21 @@
         <v>192</v>
       </c>
       <c r="B142" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E142">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="F142">
-        <v>4142</v>
+        <v>3836</v>
       </c>
       <c r="G142">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6665.9049102709832</v>
+        <v>6173.4454939158604</v>
       </c>
       <c r="I142" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="143" spans="1:9">
@@ -12254,21 +12251,21 @@
         <v>192</v>
       </c>
       <c r="B143" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E143">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="F143">
-        <v>3274</v>
+        <v>2082</v>
       </c>
       <c r="G143">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5268.9938861002411</v>
+        <v>3350.6552446123096</v>
       </c>
       <c r="I143" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="144" spans="1:9">
@@ -12276,21 +12273,21 @@
         <v>192</v>
       </c>
       <c r="B144" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E144">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="F144">
-        <v>3836</v>
+        <v>1696</v>
       </c>
       <c r="G144">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6173.4454939158604</v>
+        <v>2729.4482684257819</v>
       </c>
       <c r="I144" t="s">
-        <v>220</v>
+        <v>283</v>
       </c>
     </row>
     <row r="145" spans="1:9">
@@ -12298,21 +12295,21 @@
         <v>192</v>
       </c>
       <c r="B145" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E145">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="F145">
-        <v>2082</v>
+        <v>722</v>
       </c>
       <c r="G145">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>3350.6552446123096</v>
+        <v>1161.9467274784283</v>
       </c>
       <c r="I145" t="s">
-        <v>221</v>
+        <v>280</v>
       </c>
     </row>
     <row r="146" spans="1:9">
@@ -12320,65 +12317,71 @@
         <v>192</v>
       </c>
       <c r="B146" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E146">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
       <c r="F146">
-        <v>1696</v>
+        <v>2907</v>
       </c>
       <c r="G146">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>2729.4482684257819</v>
+        <v>4678.3644553736722</v>
       </c>
       <c r="I146" t="s">
-        <v>283</v>
+        <v>238</v>
       </c>
     </row>
     <row r="147" spans="1:9">
       <c r="A147" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B147" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="E147">
-        <f t="shared" si="14"/>
+        <f>D147/1000</f>
         <v>0</v>
       </c>
       <c r="F147">
-        <v>722</v>
+        <v>9237</v>
       </c>
       <c r="G147">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>1161.9467274784283</v>
+        <v>14865.515127033575</v>
+      </c>
+      <c r="H147" t="s">
+        <v>213</v>
       </c>
       <c r="I147" t="s">
-        <v>280</v>
+        <v>234</v>
       </c>
     </row>
     <row r="148" spans="1:9">
       <c r="A148" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B148" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="E148">
-        <f t="shared" si="14"/>
+        <f t="shared" ref="E148:E158" si="14">D148/1000</f>
         <v>0</v>
       </c>
       <c r="F148">
-        <v>2907</v>
+        <v>8897</v>
       </c>
       <c r="G148">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4678.3644553736722</v>
+        <v>14318.337997750106</v>
+      </c>
+      <c r="H148" t="s">
+        <v>213</v>
       </c>
       <c r="I148" t="s">
-        <v>238</v>
+        <v>279</v>
       </c>
     </row>
     <row r="149" spans="1:9">
@@ -12386,24 +12389,24 @@
         <v>195</v>
       </c>
       <c r="B149" t="s">
-        <v>201</v>
+        <v>268</v>
       </c>
       <c r="E149">
-        <f>D149/1000</f>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F149">
-        <v>9237</v>
+        <v>6737</v>
       </c>
       <c r="G149">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>14865.515127033575</v>
+        <v>10842.153882302176</v>
       </c>
       <c r="H149" t="s">
         <v>213</v>
       </c>
       <c r="I149" t="s">
-        <v>234</v>
+        <v>286</v>
       </c>
     </row>
     <row r="150" spans="1:9">
@@ -12411,24 +12414,24 @@
         <v>195</v>
       </c>
       <c r="B150" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E150">
-        <f t="shared" ref="E150:E160" si="15">D150/1000</f>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F150">
-        <v>8897</v>
+        <v>7412</v>
       </c>
       <c r="G150">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>14318.337997750106</v>
+        <v>11928.461418379655</v>
       </c>
       <c r="H150" t="s">
         <v>213</v>
       </c>
       <c r="I150" t="s">
-        <v>279</v>
+        <v>216</v>
       </c>
     </row>
     <row r="151" spans="1:9">
@@ -12436,24 +12439,24 @@
         <v>195</v>
       </c>
       <c r="B151" t="s">
-        <v>268</v>
+        <v>204</v>
       </c>
       <c r="E151">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F151">
-        <v>6737</v>
+        <v>7287</v>
       </c>
       <c r="G151">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10842.153882302176</v>
+        <v>11727.293356143084</v>
       </c>
       <c r="H151" t="s">
         <v>213</v>
       </c>
       <c r="I151" t="s">
-        <v>286</v>
+        <v>217</v>
       </c>
     </row>
     <row r="152" spans="1:9">
@@ -12461,24 +12464,24 @@
         <v>195</v>
       </c>
       <c r="B152" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E152">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F152">
-        <v>7412</v>
+        <v>10171</v>
       </c>
       <c r="G152">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11928.461418379655</v>
+        <v>16368.642888065227</v>
       </c>
       <c r="H152" t="s">
         <v>213</v>
       </c>
       <c r="I152" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="153" spans="1:9">
@@ -12486,24 +12489,24 @@
         <v>195</v>
       </c>
       <c r="B153" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E153">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F153">
-        <v>7287</v>
+        <v>9303</v>
       </c>
       <c r="G153">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>11727.293356143084</v>
+        <v>14971.731863894485</v>
       </c>
       <c r="H153" t="s">
         <v>213</v>
       </c>
       <c r="I153" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="154" spans="1:9">
@@ -12511,24 +12514,24 @@
         <v>195</v>
       </c>
       <c r="B154" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E154">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F154">
-        <v>10171</v>
+        <v>9980</v>
       </c>
       <c r="G154">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>16368.642888065227</v>
+        <v>16061.258088967748</v>
       </c>
       <c r="H154" t="s">
         <v>213</v>
       </c>
       <c r="I154" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="155" spans="1:9">
@@ -12536,24 +12539,24 @@
         <v>195</v>
       </c>
       <c r="B155" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E155">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F155">
-        <v>9303</v>
+        <v>8226</v>
       </c>
       <c r="G155">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>14971.731863894485</v>
+        <v>13238.467839664198</v>
       </c>
       <c r="H155" t="s">
         <v>213</v>
       </c>
       <c r="I155" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="156" spans="1:9">
@@ -12561,24 +12564,24 @@
         <v>195</v>
       </c>
       <c r="B156" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E156">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F156">
-        <v>9980</v>
+        <v>7617</v>
       </c>
       <c r="G156">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>16061.258088967748</v>
+        <v>12258.377040447629</v>
       </c>
       <c r="H156" t="s">
         <v>213</v>
       </c>
       <c r="I156" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="157" spans="1:9">
@@ -12586,24 +12589,24 @@
         <v>195</v>
       </c>
       <c r="B157" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E157">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F157">
-        <v>8226</v>
+        <v>6627</v>
       </c>
       <c r="G157">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>13238.467839664198</v>
+        <v>10665.125987533995</v>
       </c>
       <c r="H157" t="s">
         <v>213</v>
       </c>
       <c r="I157" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="158" spans="1:9">
@@ -12611,74 +12614,68 @@
         <v>195</v>
       </c>
       <c r="B158" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E158">
-        <f t="shared" si="15"/>
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
       <c r="F158">
-        <v>7617</v>
+        <v>9051</v>
       </c>
       <c r="G158">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>12258.377040447629</v>
+        <v>14566.17705042556</v>
       </c>
       <c r="H158" t="s">
         <v>213</v>
       </c>
       <c r="I158" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
     </row>
     <row r="159" spans="1:9">
       <c r="A159" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B159" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="E159">
-        <f t="shared" si="15"/>
+        <f>D159/1000</f>
         <v>0</v>
       </c>
       <c r="F159">
-        <v>6627</v>
+        <v>2843</v>
       </c>
       <c r="G159">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>10665.125987533995</v>
-      </c>
-      <c r="H159" t="s">
-        <v>213</v>
+        <v>4575.366407508548</v>
       </c>
       <c r="I159" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
     </row>
     <row r="160" spans="1:9">
       <c r="A160" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B160" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="E160">
-        <f t="shared" si="15"/>
+        <f t="shared" ref="E160:E170" si="15">D160/1000</f>
         <v>0</v>
       </c>
       <c r="F160">
-        <v>9051</v>
+        <v>3331</v>
       </c>
       <c r="G160">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>14566.17705042556</v>
-      </c>
-      <c r="H160" t="s">
-        <v>213</v>
+        <v>5360.7265224801176</v>
       </c>
       <c r="I160" t="s">
-        <v>238</v>
+        <v>279</v>
       </c>
     </row>
     <row r="161" spans="1:9">
@@ -12686,21 +12683,21 @@
         <v>194</v>
       </c>
       <c r="B161" t="s">
-        <v>201</v>
+        <v>268</v>
       </c>
       <c r="E161">
-        <f>D161/1000</f>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F161">
-        <v>2843</v>
+        <v>5582</v>
       </c>
       <c r="G161">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4575.366407508548</v>
+        <v>8983.3609872362704</v>
       </c>
       <c r="I161" t="s">
-        <v>234</v>
+        <v>215</v>
       </c>
     </row>
     <row r="162" spans="1:9">
@@ -12708,21 +12705,21 @@
         <v>194</v>
       </c>
       <c r="B162" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E162">
-        <f t="shared" ref="E162:E172" si="16">D162/1000</f>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F162">
-        <v>3331</v>
+        <v>5759</v>
       </c>
       <c r="G162">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5360.7265224801176</v>
+        <v>9268.2149633632525</v>
       </c>
       <c r="I162" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
     </row>
     <row r="163" spans="1:9">
@@ -12730,21 +12727,21 @@
         <v>194</v>
       </c>
       <c r="B163" t="s">
-        <v>268</v>
+        <v>204</v>
       </c>
       <c r="E163">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F163">
-        <v>5582</v>
+        <v>5707</v>
       </c>
       <c r="G163">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8983.3609872362704</v>
+        <v>9184.5290494728397</v>
       </c>
       <c r="I163" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="164" spans="1:9">
@@ -12752,21 +12749,21 @@
         <v>194</v>
       </c>
       <c r="B164" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E164">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F164">
-        <v>5759</v>
+        <v>3047</v>
       </c>
       <c r="G164">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9268.2149633632525</v>
+        <v>4903.6726850786299</v>
       </c>
       <c r="I164" t="s">
-        <v>287</v>
+        <v>218</v>
       </c>
     </row>
     <row r="165" spans="1:9">
@@ -12774,21 +12771,21 @@
         <v>194</v>
       </c>
       <c r="B165" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E165">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F165">
-        <v>5707</v>
+        <v>2827</v>
       </c>
       <c r="G165">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9184.5290494728397</v>
+        <v>4549.6168955422672</v>
       </c>
       <c r="I165" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="166" spans="1:9">
@@ -12796,21 +12793,21 @@
         <v>194</v>
       </c>
       <c r="B166" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E166">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F166">
-        <v>3047</v>
+        <v>2856</v>
       </c>
       <c r="G166">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4903.6726850786299</v>
+        <v>4596.2878859811508</v>
       </c>
       <c r="I166" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="167" spans="1:9">
@@ -12818,21 +12815,21 @@
         <v>194</v>
       </c>
       <c r="B167" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E167">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F167">
-        <v>2827</v>
+        <v>3840</v>
       </c>
       <c r="G167">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4549.6168955422672</v>
+        <v>6179.8828719074299</v>
       </c>
       <c r="I167" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="168" spans="1:9">
@@ -12840,21 +12837,21 @@
         <v>194</v>
       </c>
       <c r="B168" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E168">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F168">
-        <v>2856</v>
+        <v>3499</v>
       </c>
       <c r="G168">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4596.2878859811508</v>
+        <v>5631.0963981260675</v>
       </c>
       <c r="I168" t="s">
-        <v>220</v>
+        <v>237</v>
       </c>
     </row>
     <row r="169" spans="1:9">
@@ -12862,21 +12859,21 @@
         <v>194</v>
       </c>
       <c r="B169" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E169">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F169">
-        <v>3840</v>
+        <v>5736</v>
       </c>
       <c r="G169">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>6179.8828719074299</v>
+        <v>9231.2000399117242</v>
       </c>
       <c r="I169" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="170" spans="1:9">
@@ -12884,64 +12881,20 @@
         <v>194</v>
       </c>
       <c r="B170" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E170">
-        <f t="shared" si="16"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F170">
-        <v>3499</v>
+        <v>2866</v>
       </c>
       <c r="G170">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>5631.0963981260675</v>
+        <v>4612.3813309600764</v>
       </c>
       <c r="I170" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="171" spans="1:9">
-      <c r="A171" t="s">
-        <v>194</v>
-      </c>
-      <c r="B171" t="s">
-        <v>210</v>
-      </c>
-      <c r="E171">
-        <f t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="F171">
-        <v>5736</v>
-      </c>
-      <c r="G171">
-        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>9231.2000399117242</v>
-      </c>
-      <c r="I171" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="172" spans="1:9">
-      <c r="A172" t="s">
-        <v>194</v>
-      </c>
-      <c r="B172" t="s">
-        <v>211</v>
-      </c>
-      <c r="E172">
-        <f t="shared" si="16"/>
-        <v>0</v>
-      </c>
-      <c r="F172">
-        <v>2866</v>
-      </c>
-      <c r="G172">
-        <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>4612.3813309600764</v>
-      </c>
-      <c r="I172" t="s">
         <v>281</v>
       </c>
     </row>

</xml_diff>

<commit_message>
bux fix in data prep inputs
add missing values
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A5F5D9-A0E0-45BE-8B55-C8BCC82604FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC67D363-7D5E-4AD7-A584-1663099FA2F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="8" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng_europe_2020" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2657" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2658" uniqueCount="289">
   <si>
     <t>Belgium</t>
   </si>
@@ -1242,7 +1242,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1258,7 +1258,6 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -1304,18 +1303,6 @@
     <cellStyle name="Percent 8" xfId="33" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
   <dxfs count="58">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1488,6 +1475,9 @@
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -1524,6 +1514,9 @@
           <bgColor theme="4"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1600,6 +1593,9 @@
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -1639,6 +1635,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
@@ -1761,7 +1760,7 @@
     <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="18">
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="14">
       <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
@@ -1780,10 +1779,10 @@
     <tableColumn id="1" xr3:uid="{8DC4F854-8C96-4C42-AF47-2C64D82D363F}" name="From"/>
     <tableColumn id="2" xr3:uid="{9178F7D7-E3CA-468B-8BE5-E203B9CC620E}" name="To"/>
     <tableColumn id="3" xr3:uid="{9BB01476-57DE-4D59-8170-98FAC18CF80C}" name="bcm/a  [capacity]"/>
-    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a" dataDxfId="17">
+    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a" dataDxfId="13">
       <calculatedColumnFormula>C2*9.77*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="16">
+    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="12">
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{19F26947-5FDD-4F06-A68D-DB6766B439A7}" name="distance [miles]"/>
@@ -1798,7 +1797,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I170" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13" totalsRowBorderDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I170" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
   <autoFilter ref="A1:I170" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
@@ -1811,10 +1810,10 @@
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{7E7B8CB5-D54F-4427-813D-93B66C13FCBB}" name="Distance [miles]"/>
-    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="11">
+    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="7">
       <calculatedColumnFormula>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="6"/>
     <tableColumn id="8" xr3:uid="{ECBB25E4-2145-4120-8981-E6E8E1591E5B}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1822,7 +1821,7 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{A41F31BC-0CA5-4B1A-808E-7A8A6507019C}" name="LNG_global14" displayName="LNG_global14" ref="A1:I215" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7" totalsRowBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{A41F31BC-0CA5-4B1A-808E-7A8A6507019C}" name="LNG_global14" displayName="LNG_global14" ref="A1:I215" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
   <autoFilter ref="A1:I215" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D01CBB17-E8FF-44A2-B87B-A0B5AC3337BA}" name="From"/>
@@ -1835,10 +1834,10 @@
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{B6C8563B-B70E-4D32-A7CA-353FAC6B7501}" name="Distance [miles]"/>
-    <tableColumn id="4" xr3:uid="{DB3ABB11-1F6C-4F58-B946-9343785CF33A}" name="Distance [km]" dataDxfId="5">
+    <tableColumn id="4" xr3:uid="{DB3ABB11-1F6C-4F58-B946-9343785CF33A}" name="Distance [km]" dataDxfId="1">
       <calculatedColumnFormula>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{601054B1-1B08-47CB-880D-0D80ED1BD0EA}" name="Suez or Panama" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{601054B1-1B08-47CB-880D-0D80ED1BD0EA}" name="Suez or Panama" dataDxfId="0"/>
     <tableColumn id="8" xr3:uid="{F8768BD8-8B11-4BD9-B074-AD5ADFFDF447}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1881,10 +1880,10 @@
     <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="44">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{7EF7045A-D72E-40AA-A523-1A389D57AAF5}" name="GWh [2020]" dataDxfId="3">
+    <tableColumn id="7" xr3:uid="{7EF7045A-D72E-40AA-A523-1A389D57AAF5}" name="GWh [2020]" dataDxfId="43">
       <calculatedColumnFormula>Table26[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="43">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="42">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1893,20 +1892,20 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A1:G17" totalsRowShown="0" headerRowDxfId="42" headerRowBorderDxfId="41" tableBorderDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A1:G17" totalsRowShown="0" headerRowDxfId="41" headerRowBorderDxfId="40" tableBorderDxfId="39">
   <autoFilter ref="A1:G17" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{02819FD0-F6B6-484E-B4DA-8262AECE7052}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{A15C284E-E91C-44C6-B3BB-CC2DD205DA84}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="39">
+    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="38">
       <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{A1AF1224-2FA6-47E0-9ECD-AB8B46DF628B}" name="GWh [2020]" dataDxfId="2">
+    <tableColumn id="7" xr3:uid="{A1AF1224-2FA6-47E0-9ECD-AB8B46DF628B}" name="GWh [2020]" dataDxfId="37">
       <calculatedColumnFormula>Table79[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="38">
+    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="36">
       <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1923,15 +1922,15 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="36">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="35"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="34">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="35">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="33">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{53C148C2-CAF7-47BC-9950-964805B82325}" name="GWh [2020]" dataDxfId="34">
+    <tableColumn id="7" xr3:uid="{53C148C2-CAF7-47BC-9950-964805B82325}" name="GWh [2020]" dataDxfId="32">
       <calculatedColumnFormula>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1940,20 +1939,20 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A1:G22" totalsRowShown="0" headerRowDxfId="33" headerRowBorderDxfId="32" tableBorderDxfId="31">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A1:G22" totalsRowShown="0" headerRowDxfId="31" headerRowBorderDxfId="30" tableBorderDxfId="29">
   <autoFilter ref="A1:G22" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{555371BF-8030-4257-9852-212E94829B9B}" name="Country"/>
     <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="30">
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="28">
       <calculatedColumnFormula>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{95C698CF-3EBE-40E8-840D-A6C3E41CFB2C}" name="GWh [2020]" dataDxfId="29">
+    <tableColumn id="7" xr3:uid="{95C698CF-3EBE-40E8-840D-A6C3E41CFB2C}" name="GWh [2020]" dataDxfId="27">
       <calculatedColumnFormula>Table7910[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="28">
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="26">
       <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1970,15 +1969,15 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="26">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="24">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="7" xr3:uid="{9AD7149D-CE4C-40DA-896B-BFCD92F06B1A}" name="GWh [2020]" dataDxfId="0">
+    <tableColumn id="7" xr3:uid="{9AD7149D-CE4C-40DA-896B-BFCD92F06B1A}" name="GWh [2020]" dataDxfId="23">
       <calculatedColumnFormula>MIN(Table15[[#This Row],[TWh '[2023']]],Table15[[#This Row],[TWh by share]])*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="25">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="22">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1987,20 +1986,20 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A1:G22" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A1:G22" totalsRowShown="0" headerRowDxfId="21" headerRowBorderDxfId="20" tableBorderDxfId="19">
   <autoFilter ref="A1:G22" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{779C3748-4ECD-495F-809A-B5DD28F5EC2F}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{94BC7314-C5A0-4AAD-895B-84E7A94D7CF7}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="21">
+    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="18">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{800E9158-5DB0-43C4-A644-BF3466322E9E}" name="GWh [2020]" dataDxfId="1">
+    <tableColumn id="7" xr3:uid="{800E9158-5DB0-43C4-A644-BF3466322E9E}" name="GWh [2020]" dataDxfId="17">
       <calculatedColumnFormula>Table791011[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="20">
+    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="16">
       <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2020,7 +2019,7 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="19">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="15">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
@@ -2983,7 +2982,7 @@
         <f>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F2" s="15">
+      <c r="F2" s="14">
         <f>Table791011[[#This Row],[TWh '[2020']]]*1000</f>
         <v>-8660784.6598998178</v>
       </c>
@@ -18069,10 +18068,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B0A4E44-EF0E-4B6E-954F-142396EAD0D0}">
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>12</v>
       </c>
@@ -18095,16 +18094,19 @@
         <v>103</v>
       </c>
       <c r="H1" t="s">
+        <v>106</v>
+      </c>
+      <c r="I1" t="s">
         <v>104</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>93</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -18129,25 +18131,29 @@
         <v>11.4</v>
       </c>
       <c r="H2">
+        <f>I2*1000</f>
+        <v>111378</v>
+      </c>
+      <c r="I2">
         <f>G2*9.77</f>
         <v>111.378</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>17</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>101</v>
       </c>
-      <c r="M2" t="str">
-        <f>_xlfn.CONCAT(J2,K2)</f>
+      <c r="N2" t="str">
+        <f>_xlfn.CONCAT(K2,L2)</f>
         <v>BE_LNG</v>
       </c>
-      <c r="N2" t="str">
-        <f>J2</f>
+      <c r="O2" t="str">
+        <f>K2</f>
         <v>BE</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:15">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -18172,25 +18178,29 @@
         <v>33</v>
       </c>
       <c r="H3">
-        <f t="shared" ref="H3:H19" si="1">G3*9.77</f>
+        <f t="shared" ref="H3:H19" si="1">I3*1000</f>
+        <v>322409.99999999994</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I19" si="2">G3*9.77</f>
         <v>322.40999999999997</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>25</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>101</v>
       </c>
-      <c r="M3" t="str">
-        <f t="shared" ref="M3:M19" si="2">_xlfn.CONCAT(J3,K3)</f>
+      <c r="N3" t="str">
+        <f t="shared" ref="N3:N19" si="3">_xlfn.CONCAT(K3,L3)</f>
         <v>FR_LNG</v>
       </c>
-      <c r="N3" t="str">
-        <f t="shared" ref="N3:N19" si="3">J3</f>
+      <c r="O3" t="str">
+        <f t="shared" ref="O3:O19" si="4">K3</f>
         <v>FR</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:15">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -18216,24 +18226,28 @@
       </c>
       <c r="H4">
         <f t="shared" si="1"/>
+        <v>73274.999999999985</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="2"/>
         <v>73.274999999999991</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>265</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>101</v>
-      </c>
-      <c r="M4" t="str">
-        <f t="shared" si="2"/>
-        <v>EL_LNG</v>
       </c>
       <c r="N4" t="str">
         <f t="shared" si="3"/>
+        <v>EL_LNG</v>
+      </c>
+      <c r="O4" t="str">
+        <f t="shared" si="4"/>
         <v>EL</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:15">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -18259,24 +18273,28 @@
       </c>
       <c r="H5">
         <f t="shared" si="1"/>
+        <v>155831.49999999997</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="2"/>
         <v>155.83149999999998</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>21</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>101</v>
-      </c>
-      <c r="M5" t="str">
-        <f t="shared" si="2"/>
-        <v>IT_LNG</v>
       </c>
       <c r="N5" t="str">
         <f t="shared" si="3"/>
+        <v>IT_LNG</v>
+      </c>
+      <c r="O5" t="str">
+        <f t="shared" si="4"/>
         <v>IT</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:15">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -18297,29 +18315,33 @@
         <v>2.6</v>
       </c>
       <c r="G6">
-        <f t="shared" ref="G6:G19" si="4">IF(C6&gt;F6,C6,F6)</f>
+        <f t="shared" ref="G6:G19" si="5">IF(C6&gt;F6,C6,F6)</f>
         <v>2.6</v>
       </c>
       <c r="H6">
         <f t="shared" si="1"/>
+        <v>25402</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="2"/>
         <v>25.402000000000001</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>24</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>101</v>
-      </c>
-      <c r="M6" t="str">
-        <f t="shared" si="2"/>
-        <v>HR_LNG</v>
       </c>
       <c r="N6" t="str">
         <f t="shared" si="3"/>
+        <v>HR_LNG</v>
+      </c>
+      <c r="O6" t="str">
+        <f t="shared" si="4"/>
         <v>HR</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:15">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -18340,29 +18362,33 @@
         <v>4</v>
       </c>
       <c r="G7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>4</v>
       </c>
       <c r="H7">
         <f t="shared" si="1"/>
+        <v>39080</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="2"/>
         <v>39.08</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>35</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>101</v>
-      </c>
-      <c r="M7" t="str">
-        <f t="shared" si="2"/>
-        <v>LT_LNG</v>
       </c>
       <c r="N7" t="str">
         <f t="shared" si="3"/>
+        <v>LT_LNG</v>
+      </c>
+      <c r="O7" t="str">
+        <f t="shared" si="4"/>
         <v>LT</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:15">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -18383,29 +18409,33 @@
         <v>12.5</v>
       </c>
       <c r="G8">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>12.5</v>
       </c>
       <c r="H8">
         <f t="shared" si="1"/>
+        <v>122125</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="2"/>
         <v>122.125</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>18</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>101</v>
-      </c>
-      <c r="M8" t="str">
-        <f t="shared" si="2"/>
-        <v>NL_LNG</v>
       </c>
       <c r="N8" t="str">
         <f t="shared" si="3"/>
+        <v>NL_LNG</v>
+      </c>
+      <c r="O8" t="str">
+        <f t="shared" si="4"/>
         <v>NL</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:15">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -18426,29 +18456,33 @@
         <v>5.8</v>
       </c>
       <c r="G9">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>6.2</v>
       </c>
       <c r="H9">
         <f t="shared" si="1"/>
+        <v>60574</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="2"/>
         <v>60.573999999999998</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>27</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>101</v>
-      </c>
-      <c r="M9" t="str">
-        <f t="shared" si="2"/>
-        <v>PL_LNG</v>
       </c>
       <c r="N9" t="str">
         <f t="shared" si="3"/>
+        <v>PL_LNG</v>
+      </c>
+      <c r="O9" t="str">
+        <f t="shared" si="4"/>
         <v>PL</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:15">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -18469,29 +18503,33 @@
         <v>7.3</v>
       </c>
       <c r="G10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>7.6</v>
       </c>
       <c r="H10">
         <f t="shared" si="1"/>
+        <v>74252</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="2"/>
         <v>74.251999999999995</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>38</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>101</v>
-      </c>
-      <c r="M10" t="str">
-        <f t="shared" si="2"/>
-        <v>PT_LNG</v>
       </c>
       <c r="N10" t="str">
         <f t="shared" si="3"/>
+        <v>PT_LNG</v>
+      </c>
+      <c r="O10" t="str">
+        <f t="shared" si="4"/>
         <v>PT</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:15">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -18512,29 +18550,33 @@
         <v>67.099999999999994</v>
       </c>
       <c r="G11">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>67.099999999999994</v>
       </c>
       <c r="H11">
         <f t="shared" si="1"/>
+        <v>655566.99999999988</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="2"/>
         <v>655.56699999999989</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>37</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>101</v>
-      </c>
-      <c r="M11" t="str">
-        <f t="shared" si="2"/>
-        <v>ES_LNG</v>
       </c>
       <c r="N11" t="str">
         <f t="shared" si="3"/>
+        <v>ES_LNG</v>
+      </c>
+      <c r="O11" t="str">
+        <f t="shared" si="4"/>
         <v>ES</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:15">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -18555,29 +18597,33 @@
         <v>14.8</v>
       </c>
       <c r="G12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>43.6</v>
       </c>
       <c r="H12">
         <f t="shared" si="1"/>
+        <v>425972</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="2"/>
         <v>425.97199999999998</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>47</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>101</v>
-      </c>
-      <c r="M12" t="str">
-        <f t="shared" si="2"/>
-        <v>TR_LNG</v>
       </c>
       <c r="N12" t="str">
         <f t="shared" si="3"/>
+        <v>TR_LNG</v>
+      </c>
+      <c r="O12" t="str">
+        <f t="shared" si="4"/>
         <v>TR</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:15">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -18598,29 +18644,33 @@
         <v>52.3</v>
       </c>
       <c r="G13">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>52.3</v>
       </c>
       <c r="H13">
         <f t="shared" si="1"/>
+        <v>510970.99999999994</v>
+      </c>
+      <c r="I13">
+        <f t="shared" si="2"/>
         <v>510.97099999999995</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>11</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>101</v>
-      </c>
-      <c r="M13" t="str">
-        <f t="shared" si="2"/>
-        <v>UK_LNG</v>
       </c>
       <c r="N13" t="str">
         <f t="shared" si="3"/>
+        <v>UK_LNG</v>
+      </c>
+      <c r="O13" t="str">
+        <f t="shared" si="4"/>
         <v>UK</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:15">
       <c r="A14" t="s">
         <v>92</v>
       </c>
@@ -18635,18 +18685,22 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.7</v>
       </c>
       <c r="H14">
         <f t="shared" si="1"/>
+        <v>6838.9999999999991</v>
+      </c>
+      <c r="I14">
+        <f t="shared" si="2"/>
         <v>6.8389999999999995</v>
       </c>
-      <c r="J14" t="s">
+      <c r="K14" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:15">
       <c r="A15" t="s">
         <v>129</v>
       </c>
@@ -18661,29 +18715,33 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2.5</v>
       </c>
       <c r="H15">
         <f t="shared" si="1"/>
+        <v>24424.999999999996</v>
+      </c>
+      <c r="I15">
+        <f t="shared" si="2"/>
         <v>24.424999999999997</v>
       </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>54</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
         <v>101</v>
-      </c>
-      <c r="M15" t="str">
-        <f t="shared" si="2"/>
-        <v>EE_LNG</v>
       </c>
       <c r="N15" t="str">
         <f t="shared" si="3"/>
+        <v>EE_LNG</v>
+      </c>
+      <c r="O15" t="str">
+        <f t="shared" si="4"/>
         <v>EE</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:15">
       <c r="A16" t="s">
         <v>128</v>
       </c>
@@ -18698,29 +18756,33 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>5</v>
       </c>
       <c r="H16">
         <f t="shared" si="1"/>
+        <v>48849.999999999993</v>
+      </c>
+      <c r="I16">
+        <f t="shared" si="2"/>
         <v>48.849999999999994</v>
       </c>
-      <c r="J16" t="s">
+      <c r="K16" t="s">
         <v>55</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>101</v>
-      </c>
-      <c r="M16" t="str">
-        <f t="shared" si="2"/>
-        <v>FI_LNG</v>
       </c>
       <c r="N16" t="str">
         <f t="shared" si="3"/>
+        <v>FI_LNG</v>
+      </c>
+      <c r="O16" t="str">
+        <f t="shared" si="4"/>
         <v>FI</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:15">
       <c r="A17" t="s">
         <v>130</v>
       </c>
@@ -18735,29 +18797,33 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>31.2</v>
       </c>
       <c r="H17">
         <f t="shared" si="1"/>
+        <v>304823.99999999994</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="2"/>
         <v>304.82399999999996</v>
       </c>
-      <c r="J17" t="s">
+      <c r="K17" t="s">
         <v>19</v>
       </c>
-      <c r="K17" t="s">
+      <c r="L17" t="s">
         <v>101</v>
-      </c>
-      <c r="M17" t="str">
-        <f t="shared" si="2"/>
-        <v>DE_LNG</v>
       </c>
       <c r="N17" t="str">
         <f t="shared" si="3"/>
+        <v>DE_LNG</v>
+      </c>
+      <c r="O17" t="str">
+        <f t="shared" si="4"/>
         <v>DE</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:15">
       <c r="A18" t="s">
         <v>131</v>
       </c>
@@ -18772,29 +18838,33 @@
         <v>0</v>
       </c>
       <c r="G18">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2.6</v>
       </c>
       <c r="H18">
         <f t="shared" si="1"/>
+        <v>25402</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="2"/>
         <v>25.402000000000001</v>
       </c>
-      <c r="J18" t="s">
+      <c r="K18" t="s">
         <v>44</v>
       </c>
-      <c r="K18" t="s">
+      <c r="L18" t="s">
         <v>101</v>
-      </c>
-      <c r="M18" t="str">
-        <f t="shared" si="2"/>
-        <v>IE_LNG</v>
       </c>
       <c r="N18" t="str">
         <f t="shared" si="3"/>
+        <v>IE_LNG</v>
+      </c>
+      <c r="O18" t="str">
+        <f t="shared" si="4"/>
         <v>IE</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:15">
       <c r="A19" t="s">
         <v>132</v>
       </c>
@@ -18809,25 +18879,29 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1.5</v>
       </c>
       <c r="H19">
         <f t="shared" si="1"/>
+        <v>14655</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="2"/>
         <v>14.654999999999999</v>
       </c>
-      <c r="J19" t="s">
+      <c r="K19" t="s">
         <v>36</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>101</v>
-      </c>
-      <c r="M19" t="str">
-        <f t="shared" si="2"/>
-        <v>LV_LNG</v>
       </c>
       <c r="N19" t="str">
         <f t="shared" si="3"/>
+        <v>LV_LNG</v>
+      </c>
+      <c r="O19" t="str">
+        <f t="shared" si="4"/>
         <v>LV</v>
       </c>
     </row>
@@ -22203,7 +22277,7 @@
         <f>Table79[[#This Row],[Mil m3 '[2020']]]/1000</f>
         <v>0</v>
       </c>
-      <c r="F2" s="15">
+      <c r="F2" s="14">
         <f>Table79[[#This Row],[TWh '[2020']]]*1000</f>
         <v>10114848.636708323</v>
       </c>

</xml_diff>

<commit_message>
testing and bug fixing
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B153FB65-8973-4BC8-A337-BCCC262D9E9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92C3F80D-412D-4C03-8043-0BF09EA5C975}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng_europe_2020" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2658" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2661" uniqueCount="289">
   <si>
     <t>Belgium</t>
   </si>
@@ -915,6 +915,9 @@
   </si>
   <si>
     <t xml:space="preserve">RU from Sabetta (Murmansk plus 1200 mi to west, minus 1200 mi to east as Murmansk is the closest port) except for JS, there it's from Vladivostok </t>
+  </si>
+  <si>
+    <t>same as DK to PL</t>
   </si>
 </sst>
 </file>
@@ -1239,7 +1242,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1255,6 +1258,7 @@
     <xf numFmtId="0" fontId="22" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -1746,10 +1750,10 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FC7F2F97-F859-4A2C-9657-17C35EEFE785}" name="Table37" displayName="Table37" ref="A1:H115" totalsRowShown="0">
-  <autoFilter ref="A1:H115" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H115">
-    <sortCondition ref="A1:A115"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{FC7F2F97-F859-4A2C-9657-17C35EEFE785}" name="Table37" displayName="Table37" ref="A1:H116" totalsRowShown="0">
+  <autoFilter ref="A1:H116" xr:uid="{E12C0BEF-3C88-4803-B1D2-BF2F4DD3F518}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H116">
+    <sortCondition ref="A1:A116"/>
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{F94559DC-2602-4FF1-9531-3B8A374512C0}" name="From"/>
@@ -2358,7 +2362,7 @@
         <v>111378</v>
       </c>
       <c r="I2">
-        <f t="shared" ref="I2:I14" si="0">G2*9.77</f>
+        <f>G2*9.77</f>
         <v>111.378</v>
       </c>
       <c r="K2" t="s">
@@ -2390,7 +2394,7 @@
         <v>19.600000000000001</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" ref="E3:E14" si="1">D3/C3</f>
+        <f t="shared" ref="E3:E14" si="0">D3/C3</f>
         <v>0.59393939393939399</v>
       </c>
       <c r="F3">
@@ -2401,11 +2405,11 @@
         <v>33</v>
       </c>
       <c r="H3">
-        <f t="shared" ref="H3:H14" si="2">I3*1000</f>
+        <f t="shared" ref="H3:H14" si="1">I3*1000</f>
         <v>322409.99999999994</v>
       </c>
       <c r="I3">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="I2:I14" si="2">G3*9.77</f>
         <v>322.40999999999997</v>
       </c>
       <c r="K3" t="s">
@@ -2437,7 +2441,7 @@
         <v>2.5</v>
       </c>
       <c r="E4" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.35714285714285715</v>
       </c>
       <c r="F4">
@@ -2448,11 +2452,11 @@
         <v>7.5</v>
       </c>
       <c r="H4">
+        <f t="shared" si="1"/>
+        <v>73274.999999999985</v>
+      </c>
+      <c r="I4">
         <f t="shared" si="2"/>
-        <v>73274.999999999985</v>
-      </c>
-      <c r="I4">
-        <f t="shared" si="0"/>
         <v>73.274999999999991</v>
       </c>
       <c r="K4" t="s">
@@ -2484,7 +2488,7 @@
         <v>12.1</v>
       </c>
       <c r="E5" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.75862068965517238</v>
       </c>
       <c r="F5">
@@ -2495,11 +2499,11 @@
         <v>15.95</v>
       </c>
       <c r="H5">
+        <f t="shared" si="1"/>
+        <v>155831.49999999997</v>
+      </c>
+      <c r="I5">
         <f t="shared" si="2"/>
-        <v>155831.49999999997</v>
-      </c>
-      <c r="I5">
-        <f t="shared" si="0"/>
         <v>155.83149999999998</v>
       </c>
       <c r="K5" t="s">
@@ -2531,7 +2535,7 @@
         <v>0.4</v>
       </c>
       <c r="E6" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.15384615384615385</v>
       </c>
       <c r="F6">
@@ -2542,11 +2546,11 @@
         <v>2.6</v>
       </c>
       <c r="H6">
+        <f t="shared" si="1"/>
+        <v>25402</v>
+      </c>
+      <c r="I6">
         <f t="shared" si="2"/>
-        <v>25402</v>
-      </c>
-      <c r="I6">
-        <f t="shared" si="0"/>
         <v>25.402000000000001</v>
       </c>
       <c r="K6" t="s">
@@ -2578,7 +2582,7 @@
         <v>1.6</v>
       </c>
       <c r="E7" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
       <c r="F7">
@@ -2589,11 +2593,11 @@
         <v>4</v>
       </c>
       <c r="H7">
+        <f t="shared" si="1"/>
+        <v>39080</v>
+      </c>
+      <c r="I7">
         <f t="shared" si="2"/>
-        <v>39080</v>
-      </c>
-      <c r="I7">
-        <f t="shared" si="0"/>
         <v>39.08</v>
       </c>
       <c r="K7" t="s">
@@ -2625,7 +2629,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="E8" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.68333333333333324</v>
       </c>
       <c r="F8">
@@ -2636,11 +2640,11 @@
         <v>12.5</v>
       </c>
       <c r="H8">
+        <f t="shared" si="1"/>
+        <v>122125</v>
+      </c>
+      <c r="I8">
         <f t="shared" si="2"/>
-        <v>122125</v>
-      </c>
-      <c r="I8">
-        <f t="shared" si="0"/>
         <v>122.125</v>
       </c>
       <c r="K8" t="s">
@@ -2672,7 +2676,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="E9" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.66129032258064513</v>
       </c>
       <c r="F9">
@@ -2683,11 +2687,11 @@
         <v>6.2</v>
       </c>
       <c r="H9">
+        <f t="shared" si="1"/>
+        <v>60574</v>
+      </c>
+      <c r="I9">
         <f t="shared" si="2"/>
-        <v>60574</v>
-      </c>
-      <c r="I9">
-        <f t="shared" si="0"/>
         <v>60.573999999999998</v>
       </c>
       <c r="K9" t="s">
@@ -2719,7 +2723,7 @@
         <v>6.1</v>
       </c>
       <c r="E10" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.80263157894736836</v>
       </c>
       <c r="F10">
@@ -2730,11 +2734,11 @@
         <v>7.6</v>
       </c>
       <c r="H10">
+        <f t="shared" si="1"/>
+        <v>74252</v>
+      </c>
+      <c r="I10">
         <f t="shared" si="2"/>
-        <v>74252</v>
-      </c>
-      <c r="I10">
-        <f t="shared" si="0"/>
         <v>74.251999999999995</v>
       </c>
       <c r="K10" t="s">
@@ -2766,7 +2770,7 @@
         <v>20.9</v>
       </c>
       <c r="E11" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.3477537437603993</v>
       </c>
       <c r="F11">
@@ -2777,11 +2781,11 @@
         <v>67.099999999999994</v>
       </c>
       <c r="H11">
+        <f t="shared" si="1"/>
+        <v>655566.99999999988</v>
+      </c>
+      <c r="I11">
         <f t="shared" si="2"/>
-        <v>655566.99999999988</v>
-      </c>
-      <c r="I11">
-        <f t="shared" si="0"/>
         <v>655.56699999999989</v>
       </c>
       <c r="K11" t="s">
@@ -2813,7 +2817,7 @@
         <v>14.8</v>
       </c>
       <c r="E12" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.33944954128440369</v>
       </c>
       <c r="F12">
@@ -2824,11 +2828,11 @@
         <v>43.6</v>
       </c>
       <c r="H12">
+        <f t="shared" si="1"/>
+        <v>425972</v>
+      </c>
+      <c r="I12">
         <f t="shared" si="2"/>
-        <v>425972</v>
-      </c>
-      <c r="I12">
-        <f t="shared" si="0"/>
         <v>425.97199999999998</v>
       </c>
       <c r="K12" t="s">
@@ -2860,7 +2864,7 @@
         <v>18.600000000000001</v>
       </c>
       <c r="E13" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.38669438669438672</v>
       </c>
       <c r="F13">
@@ -2871,11 +2875,11 @@
         <v>52.3</v>
       </c>
       <c r="H13">
+        <f t="shared" si="1"/>
+        <v>510970.99999999994</v>
+      </c>
+      <c r="I13">
         <f t="shared" si="2"/>
-        <v>510970.99999999994</v>
-      </c>
-      <c r="I13">
-        <f t="shared" si="0"/>
         <v>510.97099999999995</v>
       </c>
       <c r="K13" t="s">
@@ -2904,7 +2908,7 @@
         <v>0.7</v>
       </c>
       <c r="E14" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G14">
@@ -2912,11 +2916,11 @@
         <v>0.7</v>
       </c>
       <c r="H14">
+        <f t="shared" si="1"/>
+        <v>6838.9999999999991</v>
+      </c>
+      <c r="I14">
         <f t="shared" si="2"/>
-        <v>6838.9999999999991</v>
-      </c>
-      <c r="I14">
-        <f t="shared" si="0"/>
         <v>6.8389999999999995</v>
       </c>
       <c r="K14" t="s">
@@ -6344,7 +6348,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67CAB708-6819-43AD-B444-2B653F840206}">
-  <dimension ref="A1:H115"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="20.453125" customWidth="1"/>
@@ -7005,7 +7009,7 @@
         <v>8760</v>
       </c>
       <c r="G33">
-        <f t="shared" ref="G33:G64" si="1">F33/1000</f>
+        <f t="shared" ref="G33:G65" si="1">F33/1000</f>
         <v>8.76</v>
       </c>
     </row>
@@ -7087,46 +7091,46 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38" t="s">
+        <v>48</v>
+      </c>
+      <c r="B38" t="s">
         <v>26</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38">
+        <v>321.60000000000002</v>
+      </c>
+      <c r="F38" s="15">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>117384.00000000001</v>
+      </c>
+      <c r="G38">
+        <f>F38/1000</f>
+        <v>117.38400000000001</v>
+      </c>
+      <c r="H38" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" t="s">
+        <v>26</v>
+      </c>
+      <c r="B39" t="s">
         <v>82</v>
       </c>
-      <c r="E38">
+      <c r="E39">
         <v>30</v>
       </c>
-      <c r="F38">
+      <c r="F39">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>10950</v>
       </c>
-      <c r="G38">
+      <c r="G39">
         <f t="shared" si="1"/>
         <v>10.95</v>
       </c>
-      <c r="H38" t="s">
+      <c r="H39" t="s">
         <v>145</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8">
-      <c r="A39" t="s">
-        <v>49</v>
-      </c>
-      <c r="B39" t="s">
-        <v>36</v>
-      </c>
-      <c r="C39">
-        <v>337.12</v>
-      </c>
-      <c r="D39">
-        <v>337.1</v>
-      </c>
-      <c r="F39">
-        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>123041.50000000001</v>
-      </c>
-      <c r="G39">
-        <f t="shared" si="1"/>
-        <v>123.04150000000001</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -7134,21 +7138,21 @@
         <v>49</v>
       </c>
       <c r="B40" t="s">
-        <v>96</v>
+        <v>36</v>
+      </c>
+      <c r="C40">
+        <v>337.12</v>
       </c>
       <c r="D40">
-        <v>31.92</v>
+        <v>337.1</v>
       </c>
       <c r="F40">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>11650.800000000001</v>
+        <v>123041.50000000001</v>
       </c>
       <c r="G40">
         <f t="shared" si="1"/>
-        <v>11.6508</v>
-      </c>
-      <c r="H40" t="s">
-        <v>146</v>
+        <v>123.04150000000001</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -7156,40 +7160,43 @@
         <v>49</v>
       </c>
       <c r="B41" t="s">
-        <v>50</v>
-      </c>
-      <c r="C41">
-        <v>1154.47</v>
+        <v>96</v>
+      </c>
+      <c r="D41">
+        <v>31.92</v>
       </c>
       <c r="F41">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>421381.55</v>
+        <v>11650.800000000001</v>
       </c>
       <c r="G41">
         <f t="shared" si="1"/>
-        <v>421.38155</v>
+        <v>11.6508</v>
       </c>
       <c r="H41" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="42" spans="1:8">
       <c r="A42" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B42" t="s">
-        <v>54</v>
-      </c>
-      <c r="E42">
-        <v>61.341321000000001</v>
+        <v>50</v>
+      </c>
+      <c r="C42">
+        <v>1154.47</v>
       </c>
       <c r="F42">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>22389.582165</v>
+        <v>421381.55</v>
       </c>
       <c r="G42">
         <f t="shared" si="1"/>
-        <v>22.389582165</v>
+        <v>421.38155</v>
+      </c>
+      <c r="H42" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -7197,40 +7204,37 @@
         <v>53</v>
       </c>
       <c r="B43" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="E43">
-        <v>67.7</v>
+        <v>61.341321000000001</v>
       </c>
       <c r="F43">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>24710.5</v>
+        <v>22389.582165</v>
       </c>
       <c r="G43">
         <f t="shared" si="1"/>
-        <v>24.7105</v>
+        <v>22.389582165</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="A44" t="s">
-        <v>264</v>
+        <v>53</v>
       </c>
       <c r="B44" t="s">
-        <v>41</v>
-      </c>
-      <c r="C44">
-        <v>487.1</v>
+        <v>35</v>
+      </c>
+      <c r="E44">
+        <v>67.7</v>
       </c>
       <c r="F44">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>177791.5</v>
+        <v>24710.5</v>
       </c>
       <c r="G44">
         <f t="shared" si="1"/>
-        <v>177.79150000000001</v>
-      </c>
-      <c r="H44" t="s">
-        <v>143</v>
+        <v>24.7105</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -7238,37 +7242,40 @@
         <v>264</v>
       </c>
       <c r="B45" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C45">
-        <v>172.57</v>
+        <v>487.1</v>
       </c>
       <c r="F45">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>62988.049999999996</v>
+        <v>177791.5</v>
       </c>
       <c r="G45">
         <f t="shared" si="1"/>
-        <v>62.988049999999994</v>
+        <v>177.79150000000001</v>
+      </c>
+      <c r="H45" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="46" spans="1:8">
       <c r="A46" t="s">
-        <v>36</v>
+        <v>264</v>
       </c>
       <c r="B46" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C46">
-        <v>224.4</v>
+        <v>172.57</v>
       </c>
       <c r="F46">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>81906</v>
+        <v>62988.049999999996</v>
       </c>
       <c r="G46">
         <f t="shared" si="1"/>
-        <v>81.906000000000006</v>
+        <v>62.988049999999994</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -7276,388 +7283,388 @@
         <v>36</v>
       </c>
       <c r="B47" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="C47">
-        <v>144</v>
+        <v>224.4</v>
       </c>
       <c r="F47">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>52560</v>
+        <v>81906</v>
       </c>
       <c r="G47">
         <f t="shared" si="1"/>
-        <v>52.56</v>
+        <v>81.906000000000006</v>
       </c>
     </row>
     <row r="48" spans="1:8">
       <c r="A48" t="s">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="B48" t="s">
-        <v>53</v>
-      </c>
-      <c r="C48" s="5">
-        <v>78</v>
-      </c>
-      <c r="E48">
-        <v>32.802250000000008</v>
+        <v>37</v>
+      </c>
+      <c r="C48">
+        <v>144</v>
       </c>
       <c r="F48">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>11972.821250000003</v>
+        <v>52560</v>
       </c>
       <c r="G48">
         <f t="shared" si="1"/>
-        <v>11.972821250000003</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8">
+        <v>52.56</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
       <c r="A49" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="B49" t="s">
-        <v>17</v>
-      </c>
-      <c r="C49">
-        <v>270</v>
+        <v>53</v>
+      </c>
+      <c r="C49" s="5">
+        <v>78</v>
+      </c>
+      <c r="E49">
+        <v>32.802250000000008</v>
       </c>
       <c r="F49">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>98550</v>
+        <v>11972.821250000003</v>
       </c>
       <c r="G49">
         <f t="shared" si="1"/>
-        <v>98.55</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8">
+        <v>11.972821250000003</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
       <c r="A50" t="s">
         <v>25</v>
       </c>
       <c r="B50" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C50">
-        <v>259.02</v>
+        <v>270</v>
       </c>
       <c r="F50">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>94542.299999999988</v>
+        <v>98550</v>
       </c>
       <c r="G50">
         <f t="shared" si="1"/>
-        <v>94.542299999999983</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8">
+        <v>98.55</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
       <c r="A51" t="s">
         <v>25</v>
       </c>
       <c r="B51" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C51">
-        <v>100</v>
+        <v>259.02</v>
       </c>
       <c r="F51">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>36500</v>
+        <v>94542.299999999988</v>
       </c>
       <c r="G51">
         <f t="shared" si="1"/>
-        <v>36.5</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8">
+        <v>94.542299999999983</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
       <c r="A52" t="s">
         <v>25</v>
       </c>
       <c r="B52" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="C52">
-        <v>164.57</v>
+        <v>100</v>
       </c>
       <c r="F52">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>60068.049999999996</v>
+        <v>36500</v>
       </c>
       <c r="G52">
         <f t="shared" si="1"/>
-        <v>60.068049999999992</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8">
+        <v>36.5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
       <c r="A53" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B53" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C53">
-        <v>50.9</v>
+        <v>164.57</v>
       </c>
       <c r="F53">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>18578.5</v>
+        <v>60068.049999999996</v>
       </c>
       <c r="G53">
         <f t="shared" si="1"/>
-        <v>18.578499999999998</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8">
+        <v>60.068049999999992</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
       <c r="A54" t="s">
         <v>24</v>
       </c>
       <c r="B54" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C54">
-        <v>7.7</v>
+        <v>50.9</v>
       </c>
       <c r="F54">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>2810.5</v>
+        <v>18578.5</v>
       </c>
       <c r="G54">
         <f t="shared" si="1"/>
-        <v>2.8105000000000002</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8">
+        <v>18.578499999999998</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
       <c r="A55" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B55" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C55">
-        <v>77.2</v>
+        <v>7.7</v>
       </c>
       <c r="F55">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>28178</v>
+        <v>2810.5</v>
       </c>
       <c r="G55">
         <f t="shared" si="1"/>
-        <v>28.178000000000001</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8">
+        <v>2.8105000000000002</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
       <c r="A56" t="s">
         <v>30</v>
       </c>
       <c r="B56" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C56">
-        <v>77.459999999999994</v>
+        <v>77.2</v>
       </c>
       <c r="F56">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>28272.899999999998</v>
+        <v>28178</v>
       </c>
       <c r="G56">
         <f t="shared" si="1"/>
-        <v>28.272899999999996</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8">
+        <v>28.178000000000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
       <c r="A57" t="s">
         <v>30</v>
       </c>
       <c r="B57" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C57">
-        <v>141.97999999999999</v>
-      </c>
-      <c r="D57">
-        <v>245.8</v>
+        <v>77.459999999999994</v>
       </c>
       <c r="F57">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>51822.7</v>
+        <v>28272.899999999998</v>
       </c>
       <c r="G57">
         <f t="shared" si="1"/>
-        <v>51.822699999999998</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8">
+        <v>28.272899999999996</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
       <c r="A58" t="s">
         <v>30</v>
       </c>
       <c r="B58" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C58">
-        <v>50.88</v>
+        <v>141.97999999999999</v>
+      </c>
+      <c r="D58">
+        <v>245.8</v>
       </c>
       <c r="F58">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>18571.2</v>
+        <v>51822.7</v>
       </c>
       <c r="G58">
         <f t="shared" si="1"/>
-        <v>18.571200000000001</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8">
+        <v>51.822699999999998</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
       <c r="A59" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B59" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C59">
-        <v>194.05</v>
+        <v>50.88</v>
       </c>
       <c r="F59">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>70828.25</v>
+        <v>18571.2</v>
       </c>
       <c r="G59">
         <f t="shared" si="1"/>
-        <v>70.828249999999997</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8">
+        <v>18.571200000000001</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
       <c r="A60" t="s">
         <v>21</v>
       </c>
       <c r="B60" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C60">
-        <v>387.85</v>
+        <v>194.05</v>
       </c>
       <c r="F60">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>141565.25</v>
+        <v>70828.25</v>
       </c>
       <c r="G60">
         <f t="shared" si="1"/>
-        <v>141.56524999999999</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8">
+        <v>70.828249999999997</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
       <c r="A61" t="s">
         <v>21</v>
       </c>
       <c r="B61" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C61">
-        <v>38.99</v>
+        <v>387.85</v>
       </c>
       <c r="F61">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>14231.35</v>
+        <v>141565.25</v>
       </c>
       <c r="G61">
         <f t="shared" si="1"/>
-        <v>14.231350000000001</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8">
+        <v>141.56524999999999</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
       <c r="A62" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="B62" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="C62">
-        <v>90</v>
+        <v>38.99</v>
       </c>
       <c r="F62">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>32850</v>
+        <v>14231.35</v>
       </c>
       <c r="G62">
         <f t="shared" si="1"/>
-        <v>32.85</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8">
+        <v>14.231350000000001</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
       <c r="A63" t="s">
         <v>34</v>
       </c>
       <c r="B63" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C63">
-        <v>58.069200000000002</v>
+        <v>90</v>
       </c>
       <c r="F63">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>21195.258000000002</v>
+        <v>32850</v>
       </c>
       <c r="G63">
         <f t="shared" si="1"/>
-        <v>21.195258000000003</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8">
+        <v>32.85</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
       <c r="A64" t="s">
         <v>34</v>
       </c>
       <c r="B64" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="C64">
-        <v>0</v>
+        <v>58.069200000000002</v>
       </c>
       <c r="F64">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
+        <v>21195.258000000002</v>
       </c>
       <c r="G64">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H64" t="s">
-        <v>148</v>
+        <v>21.195258000000003</v>
       </c>
     </row>
     <row r="65" spans="1:8">
       <c r="A65" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="B65" t="s">
-        <v>17</v>
-      </c>
-      <c r="E65">
-        <v>41.973541999999995</v>
+        <v>40</v>
+      </c>
+      <c r="C65">
+        <v>0</v>
       </c>
       <c r="F65">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>15320.342829999998</v>
+        <v>0</v>
       </c>
       <c r="G65">
-        <f t="shared" ref="G65:G95" si="2">F65/1000</f>
-        <v>15.320342829999998</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="H65" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="66" spans="1:8">
       <c r="A66" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B66" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="E66">
-        <v>67.7</v>
+        <v>41.973541999999995</v>
       </c>
       <c r="F66">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>24710.5</v>
+        <v>15320.342829999998</v>
       </c>
       <c r="G66">
-        <f t="shared" si="2"/>
-        <v>24.7105</v>
+        <f t="shared" ref="G66:G96" si="2">F66/1000</f>
+        <v>15.320342829999998</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -7665,18 +7672,18 @@
         <v>35</v>
       </c>
       <c r="B67" t="s">
-        <v>34</v>
-      </c>
-      <c r="C67">
-        <v>82</v>
+        <v>53</v>
+      </c>
+      <c r="E67">
+        <v>67.7</v>
       </c>
       <c r="F67">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>29930</v>
+        <v>24710.5</v>
       </c>
       <c r="G67">
         <f t="shared" si="2"/>
-        <v>29.93</v>
+        <v>24.7105</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -7684,78 +7691,78 @@
         <v>35</v>
       </c>
       <c r="B68" t="s">
-        <v>40</v>
-      </c>
-      <c r="D68">
-        <v>0</v>
+        <v>34</v>
+      </c>
+      <c r="C68">
+        <v>82</v>
       </c>
       <c r="F68">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
+        <v>29930</v>
       </c>
       <c r="G68">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>29.93</v>
       </c>
     </row>
     <row r="69" spans="1:8">
       <c r="A69" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="B69" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="D69">
-        <v>493.7</v>
+        <v>0</v>
       </c>
       <c r="F69">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>180200.5</v>
+        <v>0</v>
       </c>
       <c r="G69">
         <f t="shared" si="2"/>
-        <v>180.20050000000001</v>
-      </c>
-      <c r="H69" t="s">
-        <v>148</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:8">
       <c r="A70" t="s">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="B70" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="D70">
-        <v>31.92</v>
+        <v>493.7</v>
       </c>
       <c r="F70">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>11650.800000000001</v>
+        <v>180200.5</v>
       </c>
       <c r="G70">
         <f t="shared" si="2"/>
-        <v>11.6508</v>
+        <v>180.20050000000001</v>
+      </c>
+      <c r="H70" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="71" spans="1:8">
       <c r="A71" t="s">
-        <v>39</v>
+        <v>96</v>
       </c>
       <c r="B71" t="s">
-        <v>33</v>
-      </c>
-      <c r="C71">
-        <v>2.2000000000000002</v>
+        <v>36</v>
+      </c>
+      <c r="D71">
+        <v>31.92</v>
       </c>
       <c r="F71">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>803.00000000000011</v>
+        <v>11650.800000000001</v>
       </c>
       <c r="G71">
         <f t="shared" si="2"/>
-        <v>0.80300000000000016</v>
+        <v>11.6508</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -7763,37 +7770,37 @@
         <v>39</v>
       </c>
       <c r="B72" t="s">
-        <v>38</v>
-      </c>
-      <c r="E72">
-        <v>80.846503979999994</v>
+        <v>33</v>
+      </c>
+      <c r="C72">
+        <v>2.2000000000000002</v>
       </c>
       <c r="F72">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>29508.973952699998</v>
+        <v>803.00000000000011</v>
       </c>
       <c r="G72">
         <f t="shared" si="2"/>
-        <v>29.5089739527</v>
+        <v>0.80300000000000016</v>
       </c>
     </row>
     <row r="73" spans="1:8">
       <c r="A73" t="s">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="B73" t="s">
-        <v>17</v>
-      </c>
-      <c r="C73">
-        <v>1387.5634559999999</v>
+        <v>38</v>
+      </c>
+      <c r="E73">
+        <v>80.846503979999994</v>
       </c>
       <c r="F73">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>506460.66143999994</v>
+        <v>29508.973952699998</v>
       </c>
       <c r="G73">
         <f t="shared" si="2"/>
-        <v>506.46066143999991</v>
+        <v>29.5089739527</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -7801,18 +7808,18 @@
         <v>18</v>
       </c>
       <c r="B74" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C74">
-        <v>1849.1500000000003</v>
+        <v>1387.5634559999999</v>
       </c>
       <c r="F74">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>674939.75000000012</v>
+        <v>506460.66143999994</v>
       </c>
       <c r="G74">
         <f t="shared" si="2"/>
-        <v>674.93975000000012</v>
+        <v>506.46066143999991</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -7820,40 +7827,37 @@
         <v>18</v>
       </c>
       <c r="B75" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C75">
-        <v>494.4</v>
+        <v>1849.1500000000003</v>
       </c>
       <c r="F75">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>180456</v>
+        <v>674939.75000000012</v>
       </c>
       <c r="G75">
         <f t="shared" si="2"/>
-        <v>180.45599999999999</v>
+        <v>674.93975000000012</v>
       </c>
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="B76" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C76">
-        <v>488.4</v>
-      </c>
-      <c r="D76">
-        <v>453.2</v>
+        <v>494.4</v>
       </c>
       <c r="F76">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>165418</v>
+        <v>180456</v>
       </c>
       <c r="G76">
         <f t="shared" si="2"/>
-        <v>165.41800000000001</v>
+        <v>180.45599999999999</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -7861,21 +7865,21 @@
         <v>48</v>
       </c>
       <c r="B77" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C77">
-        <v>2195.9271199999998</v>
+        <v>488.4</v>
       </c>
       <c r="D77">
-        <v>1226</v>
+        <v>453.2</v>
       </c>
       <c r="F77">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>447490</v>
+        <v>165418</v>
       </c>
       <c r="G77">
         <f t="shared" si="2"/>
-        <v>447.49</v>
+        <v>165.41800000000001</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -7883,21 +7887,21 @@
         <v>48</v>
       </c>
       <c r="B78" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C78">
-        <v>575</v>
+        <v>2195.9271199999998</v>
       </c>
       <c r="D78">
-        <v>568.5</v>
+        <v>1226</v>
       </c>
       <c r="F78">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>207502.5</v>
+        <v>447490</v>
       </c>
       <c r="G78">
         <f t="shared" si="2"/>
-        <v>207.5025</v>
+        <v>447.49</v>
       </c>
     </row>
     <row r="79" spans="1:8">
@@ -7905,18 +7909,21 @@
         <v>48</v>
       </c>
       <c r="B79" t="s">
-        <v>18</v>
+        <v>25</v>
+      </c>
+      <c r="C79">
+        <v>575</v>
       </c>
       <c r="D79">
-        <v>963.6</v>
+        <v>568.5</v>
       </c>
       <c r="F79">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>351714</v>
+        <v>207502.5</v>
       </c>
       <c r="G79">
         <f t="shared" si="2"/>
-        <v>351.714</v>
+        <v>207.5025</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -7924,279 +7931,279 @@
         <v>48</v>
       </c>
       <c r="B80" t="s">
-        <v>11</v>
-      </c>
-      <c r="C80">
-        <v>1499.1</v>
+        <v>18</v>
       </c>
       <c r="D80">
-        <v>1406</v>
+        <v>963.6</v>
       </c>
       <c r="F80">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>513190</v>
+        <v>351714</v>
       </c>
       <c r="G80">
         <f t="shared" si="2"/>
-        <v>513.19000000000005</v>
-      </c>
-    </row>
-    <row r="81" spans="1:8">
+        <v>351.714</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7">
       <c r="A81" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="B81" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C81">
-        <v>0.09</v>
+        <v>1499.1</v>
+      </c>
+      <c r="D81">
+        <v>1406</v>
       </c>
       <c r="F81">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>32.85</v>
+        <v>513190</v>
       </c>
       <c r="G81">
         <f t="shared" si="2"/>
-        <v>3.2850000000000004E-2</v>
-      </c>
-    </row>
-    <row r="82" spans="1:8">
+        <v>513.19000000000005</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7">
       <c r="A82" t="s">
         <v>27</v>
       </c>
       <c r="B82" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C82">
-        <v>91.2</v>
+        <v>0.09</v>
       </c>
       <c r="F82">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>33288</v>
+        <v>32.85</v>
       </c>
       <c r="G82">
         <f t="shared" si="2"/>
-        <v>33.287999999999997</v>
-      </c>
-    </row>
-    <row r="83" spans="1:8">
+        <v>3.2850000000000004E-2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7">
       <c r="A83" t="s">
         <v>27</v>
       </c>
       <c r="B83" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C83">
-        <v>173.94</v>
+        <v>91.2</v>
       </c>
       <c r="F83">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>63488.1</v>
+        <v>33288</v>
       </c>
       <c r="G83">
         <f t="shared" si="2"/>
-        <v>63.488099999999996</v>
-      </c>
-    </row>
-    <row r="84" spans="1:8">
+        <v>33.287999999999997</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7">
       <c r="A84" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="B84" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C84">
-        <v>80</v>
+        <v>173.94</v>
       </c>
       <c r="F84">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>29200</v>
+        <v>63488.1</v>
       </c>
       <c r="G84">
         <f t="shared" si="2"/>
-        <v>29.2</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8">
+        <v>63.488099999999996</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7">
       <c r="A85" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B85" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C85">
-        <v>231.417</v>
+        <v>80</v>
       </c>
       <c r="F85">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>84467.205000000002</v>
+        <v>29200</v>
       </c>
       <c r="G85">
         <f t="shared" si="2"/>
-        <v>84.467205000000007</v>
-      </c>
-    </row>
-    <row r="86" spans="1:8">
+        <v>29.2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7">
       <c r="A86" t="s">
         <v>33</v>
       </c>
       <c r="B86" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C86">
-        <v>73.37</v>
+        <v>231.417</v>
       </c>
       <c r="F86">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>26780.050000000003</v>
+        <v>84467.205000000002</v>
       </c>
       <c r="G86">
         <f t="shared" si="2"/>
-        <v>26.780050000000003</v>
-      </c>
-    </row>
-    <row r="87" spans="1:8">
+        <v>84.467205000000007</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7">
       <c r="A87" t="s">
         <v>33</v>
       </c>
       <c r="B87" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C87">
-        <v>55.7</v>
-      </c>
-      <c r="E87">
-        <v>55.7</v>
+        <v>73.37</v>
       </c>
       <c r="F87">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>20330.5</v>
+        <v>26780.050000000003</v>
       </c>
       <c r="G87">
         <f t="shared" si="2"/>
-        <v>20.330500000000001</v>
-      </c>
-    </row>
-    <row r="88" spans="1:8">
+        <v>26.780050000000003</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7">
       <c r="A88" t="s">
         <v>33</v>
       </c>
       <c r="B88" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C88">
-        <v>122.2</v>
+        <v>55.7</v>
+      </c>
+      <c r="E88">
+        <v>55.7</v>
       </c>
       <c r="F88">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>44603</v>
+        <v>20330.5</v>
       </c>
       <c r="G88">
         <f t="shared" si="2"/>
-        <v>44.603000000000002</v>
-      </c>
-    </row>
-    <row r="89" spans="1:8">
+        <v>20.330500000000001</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7">
       <c r="A89" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B89" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C89">
-        <v>14</v>
+        <v>122.2</v>
       </c>
       <c r="F89">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>5110</v>
+        <v>44603</v>
       </c>
       <c r="G89">
         <f t="shared" si="2"/>
-        <v>5.1100000000000003</v>
-      </c>
-    </row>
-    <row r="90" spans="1:8">
+        <v>44.603000000000002</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7">
       <c r="A90" t="s">
         <v>31</v>
       </c>
       <c r="B90" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="C90">
-        <v>350.11200000000002</v>
+        <v>14</v>
       </c>
       <c r="F90">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>127790.88</v>
+        <v>5110</v>
       </c>
       <c r="G90">
         <f t="shared" si="2"/>
-        <v>127.79088</v>
-      </c>
-    </row>
-    <row r="91" spans="1:8">
+        <v>5.1100000000000003</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7">
       <c r="A91" t="s">
         <v>31</v>
       </c>
       <c r="B91" t="s">
-        <v>30</v>
-      </c>
-      <c r="D91">
-        <v>245.8</v>
+        <v>32</v>
+      </c>
+      <c r="C91">
+        <v>350.11200000000002</v>
       </c>
       <c r="F91">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>89717</v>
+        <v>127790.88</v>
       </c>
       <c r="G91">
         <f t="shared" si="2"/>
-        <v>89.716999999999999</v>
-      </c>
-    </row>
-    <row r="92" spans="1:8">
+        <v>127.79088</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7">
       <c r="A92" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="B92" t="s">
-        <v>52</v>
-      </c>
-      <c r="C92">
-        <v>1203.4999999999998</v>
+        <v>30</v>
+      </c>
+      <c r="D92">
+        <v>245.8</v>
       </c>
       <c r="F92">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>439277.49999999994</v>
+        <v>89717</v>
       </c>
       <c r="G92">
         <f t="shared" si="2"/>
-        <v>439.27749999999992</v>
-      </c>
-    </row>
-    <row r="93" spans="1:8">
+        <v>89.716999999999999</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7">
       <c r="A93" t="s">
         <v>40</v>
       </c>
       <c r="B93" t="s">
-        <v>19</v>
-      </c>
-      <c r="D93">
-        <v>0</v>
+        <v>52</v>
+      </c>
+      <c r="C93">
+        <v>1203.4999999999998</v>
       </c>
       <c r="F93">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
+        <v>439277.49999999994</v>
       </c>
       <c r="G93">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" spans="1:8">
+        <v>439.27749999999992</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7">
       <c r="A94" t="s">
         <v>40</v>
       </c>
       <c r="B94" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
       <c r="D94">
         <v>0</v>
@@ -8210,12 +8217,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8">
+    <row r="95" spans="1:7">
       <c r="A95" t="s">
         <v>40</v>
       </c>
       <c r="B95" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="D95">
         <v>0</v>
@@ -8229,26 +8236,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8">
+    <row r="96" spans="1:7">
       <c r="A96" t="s">
         <v>40</v>
       </c>
       <c r="B96" t="s">
-        <v>46</v>
-      </c>
-      <c r="E96">
-        <v>958.9</v>
+        <v>35</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
       </c>
       <c r="F96">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>349998.5</v>
+        <v>0</v>
       </c>
       <c r="G96">
-        <f t="shared" ref="G96:G115" si="3">F96/1000</f>
-        <v>349.99849999999998</v>
-      </c>
-      <c r="H96" t="s">
-        <v>141</v>
+        <f t="shared" si="2"/>
+        <v>0</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -8256,37 +8260,40 @@
         <v>40</v>
       </c>
       <c r="B97" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="E97">
-        <v>5459.5088498999994</v>
+        <v>958.9</v>
       </c>
       <c r="F97">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>349998.5</v>
+      </c>
+      <c r="G97">
+        <f t="shared" ref="G97:G116" si="3">F97/1000</f>
+        <v>349.99849999999998</v>
+      </c>
+      <c r="H97" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8">
+      <c r="A98" t="s">
+        <v>40</v>
+      </c>
+      <c r="B98" t="s">
+        <v>38</v>
+      </c>
+      <c r="E98">
+        <v>5459.5088498999994</v>
+      </c>
+      <c r="F98">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>1992720.7302134999</v>
       </c>
-      <c r="G97">
+      <c r="G98">
         <f t="shared" si="3"/>
         <v>1992.7207302134998</v>
-      </c>
-    </row>
-    <row r="98" spans="1:8">
-      <c r="A98" t="s">
-        <v>23</v>
-      </c>
-      <c r="B98" t="s">
-        <v>24</v>
-      </c>
-      <c r="C98">
-        <v>53.7</v>
-      </c>
-      <c r="F98">
-        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>19600.5</v>
-      </c>
-      <c r="G98">
-        <f t="shared" si="3"/>
-        <v>19.6005</v>
       </c>
     </row>
     <row r="99" spans="1:8">
@@ -8294,37 +8301,37 @@
         <v>23</v>
       </c>
       <c r="B99" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C99">
-        <v>25.77</v>
+        <v>53.7</v>
       </c>
       <c r="F99">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>9406.0499999999993</v>
+        <v>19600.5</v>
       </c>
       <c r="G99">
         <f t="shared" si="3"/>
-        <v>9.4060499999999987</v>
+        <v>19.6005</v>
       </c>
     </row>
     <row r="100" spans="1:8">
       <c r="A100" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B100" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C100">
-        <v>1708.7</v>
+        <v>25.77</v>
       </c>
       <c r="F100">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>623675.5</v>
+        <v>9406.0499999999993</v>
       </c>
       <c r="G100">
         <f t="shared" si="3"/>
-        <v>623.67550000000006</v>
+        <v>9.4060499999999987</v>
       </c>
     </row>
     <row r="101" spans="1:8">
@@ -8332,18 +8339,18 @@
         <v>29</v>
       </c>
       <c r="B101" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C101">
-        <v>395.2</v>
+        <v>1708.7</v>
       </c>
       <c r="F101">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>144248</v>
+        <v>623675.5</v>
       </c>
       <c r="G101">
         <f t="shared" si="3"/>
-        <v>144.24799999999999</v>
+        <v>623.67550000000006</v>
       </c>
     </row>
     <row r="102" spans="1:8">
@@ -8351,18 +8358,18 @@
         <v>29</v>
       </c>
       <c r="B102" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C102">
-        <v>128.97</v>
+        <v>395.2</v>
       </c>
       <c r="F102">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>47074.05</v>
+        <v>144248</v>
       </c>
       <c r="G102">
         <f t="shared" si="3"/>
-        <v>47.07405</v>
+        <v>144.24799999999999</v>
       </c>
     </row>
     <row r="103" spans="1:8">
@@ -8370,18 +8377,18 @@
         <v>29</v>
       </c>
       <c r="B103" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C103">
-        <v>144.50399999999999</v>
+        <v>128.97</v>
       </c>
       <c r="F103">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>52743.96</v>
+        <v>47074.05</v>
       </c>
       <c r="G103">
         <f t="shared" si="3"/>
-        <v>52.743960000000001</v>
+        <v>47.07405</v>
       </c>
     </row>
     <row r="104" spans="1:8">
@@ -8389,65 +8396,65 @@
         <v>29</v>
       </c>
       <c r="B104" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C104">
-        <v>436.8</v>
-      </c>
-      <c r="D104">
-        <v>280.8</v>
+        <v>144.50399999999999</v>
       </c>
       <c r="F104">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>102492</v>
+        <v>52743.96</v>
       </c>
       <c r="G104">
         <f t="shared" si="3"/>
-        <v>102.492</v>
+        <v>52.743960000000001</v>
       </c>
     </row>
     <row r="105" spans="1:8">
       <c r="A105" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="B105" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="C105">
-        <v>1154.47</v>
+        <v>436.8</v>
       </c>
       <c r="D105">
-        <v>1154</v>
+        <v>280.8</v>
       </c>
       <c r="F105">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>421210</v>
+        <v>102492</v>
       </c>
       <c r="G105">
         <f t="shared" si="3"/>
-        <v>421.21</v>
-      </c>
-      <c r="H105" t="s">
-        <v>147</v>
+        <v>102.492</v>
       </c>
     </row>
     <row r="106" spans="1:8">
       <c r="A106" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B106" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="C106">
-        <v>576.03</v>
+        <v>1154.47</v>
+      </c>
+      <c r="D106">
+        <v>1154</v>
       </c>
       <c r="F106">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>210250.94999999998</v>
+        <v>421210</v>
       </c>
       <c r="G106">
         <f t="shared" si="3"/>
-        <v>210.25094999999999</v>
+        <v>421.21</v>
+      </c>
+      <c r="H106" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="107" spans="1:8">
@@ -8455,37 +8462,37 @@
         <v>46</v>
       </c>
       <c r="B107" t="s">
-        <v>264</v>
+        <v>32</v>
       </c>
       <c r="C107">
-        <v>398.6</v>
+        <v>576.03</v>
       </c>
       <c r="F107">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>145489</v>
+        <v>210250.94999999998</v>
       </c>
       <c r="G107">
         <f t="shared" si="3"/>
-        <v>145.489</v>
+        <v>210.25094999999999</v>
       </c>
     </row>
     <row r="108" spans="1:8">
       <c r="A108" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B108" t="s">
-        <v>30</v>
-      </c>
-      <c r="D108">
-        <v>84.77</v>
+        <v>264</v>
+      </c>
+      <c r="C108">
+        <v>398.6</v>
       </c>
       <c r="F108">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>30941.05</v>
+        <v>145489</v>
       </c>
       <c r="G108">
         <f t="shared" si="3"/>
-        <v>30.941050000000001</v>
+        <v>145.489</v>
       </c>
     </row>
     <row r="109" spans="1:8">
@@ -8493,18 +8500,18 @@
         <v>38</v>
       </c>
       <c r="B109" t="s">
-        <v>39</v>
-      </c>
-      <c r="E109">
-        <v>255.46047452000005</v>
+        <v>30</v>
+      </c>
+      <c r="D109">
+        <v>84.77</v>
       </c>
       <c r="F109">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>93243.073199800012</v>
+        <v>30941.05</v>
       </c>
       <c r="G109">
         <f t="shared" si="3"/>
-        <v>93.243073199800008</v>
+        <v>30.941050000000001</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -8512,21 +8519,18 @@
         <v>38</v>
       </c>
       <c r="B110" t="s">
-        <v>27</v>
-      </c>
-      <c r="D110">
-        <v>135.6</v>
+        <v>39</v>
+      </c>
+      <c r="E110">
+        <v>255.46047452000005</v>
       </c>
       <c r="F110">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>49494</v>
+        <v>93243.073199800012</v>
       </c>
       <c r="G110">
         <f t="shared" si="3"/>
-        <v>49.494</v>
-      </c>
-      <c r="H110" t="s">
-        <v>148</v>
+        <v>93.243073199800008</v>
       </c>
     </row>
     <row r="111" spans="1:8">
@@ -8534,21 +8538,18 @@
         <v>38</v>
       </c>
       <c r="B111" t="s">
-        <v>33</v>
-      </c>
-      <c r="C111">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="D111">
-        <v>0</v>
+        <v>135.6</v>
       </c>
       <c r="F111">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>0</v>
+        <v>49494</v>
       </c>
       <c r="G111">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>49.494</v>
       </c>
       <c r="H111" t="s">
         <v>148</v>
@@ -8559,43 +8560,46 @@
         <v>38</v>
       </c>
       <c r="B112" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C112">
-        <v>249.6</v>
+        <v>0</v>
       </c>
       <c r="D112">
-        <v>1799</v>
+        <v>0</v>
       </c>
       <c r="F112">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>91104</v>
+        <v>0</v>
       </c>
       <c r="G112">
         <f t="shared" si="3"/>
-        <v>91.103999999999999</v>
+        <v>0</v>
+      </c>
+      <c r="H112" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="113" spans="1:7">
       <c r="A113" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="B113" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C113">
-        <v>651.70000000000005</v>
+        <v>249.6</v>
       </c>
       <c r="D113">
-        <v>205.9</v>
+        <v>1799</v>
       </c>
       <c r="F113">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>75153.5</v>
+        <v>91104</v>
       </c>
       <c r="G113">
         <f t="shared" si="3"/>
-        <v>75.153499999999994</v>
+        <v>91.103999999999999</v>
       </c>
     </row>
     <row r="114" spans="1:7">
@@ -8603,21 +8607,21 @@
         <v>11</v>
       </c>
       <c r="B114" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="C114">
-        <v>386.58</v>
+        <v>651.70000000000005</v>
       </c>
       <c r="D114">
-        <v>385</v>
+        <v>205.9</v>
       </c>
       <c r="F114">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
-        <v>140525</v>
+        <v>75153.5</v>
       </c>
       <c r="G114">
         <f t="shared" si="3"/>
-        <v>140.52500000000001</v>
+        <v>75.153499999999994</v>
       </c>
     </row>
     <row r="115" spans="1:7">
@@ -8625,16 +8629,38 @@
         <v>11</v>
       </c>
       <c r="B115" t="s">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="C115">
-        <v>168</v>
+        <v>386.58</v>
+      </c>
+      <c r="D115">
+        <v>385</v>
       </c>
       <c r="F115">
         <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
+        <v>140525</v>
+      </c>
+      <c r="G115">
+        <f t="shared" si="3"/>
+        <v>140.52500000000001</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7">
+      <c r="A116" t="s">
+        <v>11</v>
+      </c>
+      <c r="B116" t="s">
+        <v>18</v>
+      </c>
+      <c r="C116">
+        <v>168</v>
+      </c>
+      <c r="F116">
+        <f>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</f>
         <v>61320</v>
       </c>
-      <c r="G115">
+      <c r="G116">
         <f t="shared" si="3"/>
         <v>61.32</v>
       </c>
@@ -18164,7 +18190,7 @@
         <v>19.600000000000001</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" ref="E3:E19" si="0">D3/C3</f>
+        <f t="shared" ref="E3:E18" si="0">D3/C3</f>
         <v>0.59393939393939399</v>
       </c>
       <c r="F3">
@@ -18175,11 +18201,11 @@
         <v>33</v>
       </c>
       <c r="H3">
-        <f t="shared" ref="H3:H19" si="1">I3*1000</f>
+        <f t="shared" ref="H3:H18" si="1">I3*1000</f>
         <v>322409.99999999994</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I19" si="2">G3*9.77</f>
+        <f t="shared" ref="I3:I18" si="2">G3*9.77</f>
         <v>322.40999999999997</v>
       </c>
       <c r="K3" t="s">
@@ -18189,11 +18215,11 @@
         <v>100</v>
       </c>
       <c r="N3" t="str">
-        <f t="shared" ref="N3:N19" si="3">_xlfn.CONCAT(K3,L3)</f>
+        <f t="shared" ref="N3:N18" si="3">_xlfn.CONCAT(K3,L3)</f>
         <v>FR_LNG</v>
       </c>
       <c r="O3" t="str">
-        <f t="shared" ref="O3:O19" si="4">K3</f>
+        <f t="shared" ref="O3:O18" si="4">K3</f>
         <v>FR</v>
       </c>
     </row>
@@ -18312,7 +18338,7 @@
         <v>2.6</v>
       </c>
       <c r="G6">
-        <f t="shared" ref="G6:G19" si="5">IF(C6&gt;F6,C6,F6)</f>
+        <f t="shared" ref="G6:G18" si="5">IF(C6&gt;F6,C6,F6)</f>
         <v>2.6</v>
       </c>
       <c r="H6">
@@ -18669,13 +18695,13 @@
     </row>
     <row r="14" spans="1:15">
       <c r="A14" t="s">
-        <v>91</v>
+        <v>128</v>
       </c>
       <c r="B14" t="s">
-        <v>99</v>
+        <v>53</v>
       </c>
       <c r="C14">
-        <v>0.7</v>
+        <v>2.5</v>
       </c>
       <c r="E14" s="1">
         <f t="shared" si="0"/>
@@ -18683,29 +18709,40 @@
       </c>
       <c r="G14">
         <f t="shared" si="5"/>
-        <v>0.7</v>
+        <v>2.5</v>
       </c>
       <c r="H14">
         <f t="shared" si="1"/>
-        <v>6838.9999999999991</v>
+        <v>24424.999999999996</v>
       </c>
       <c r="I14">
         <f t="shared" si="2"/>
-        <v>6.8389999999999995</v>
+        <v>24.424999999999997</v>
       </c>
       <c r="K14" t="s">
-        <v>99</v>
+        <v>53</v>
+      </c>
+      <c r="L14" t="s">
+        <v>100</v>
+      </c>
+      <c r="N14" t="str">
+        <f t="shared" si="3"/>
+        <v>EE_LNG</v>
+      </c>
+      <c r="O14" t="str">
+        <f t="shared" si="4"/>
+        <v>EE</v>
       </c>
     </row>
     <row r="15" spans="1:15">
       <c r="A15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C15">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="E15" s="1">
         <f t="shared" si="0"/>
@@ -18713,40 +18750,40 @@
       </c>
       <c r="G15">
         <f t="shared" si="5"/>
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="H15">
         <f t="shared" si="1"/>
-        <v>24424.999999999996</v>
+        <v>48849.999999999993</v>
       </c>
       <c r="I15">
         <f t="shared" si="2"/>
-        <v>24.424999999999997</v>
+        <v>48.849999999999994</v>
       </c>
       <c r="K15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L15" t="s">
         <v>100</v>
       </c>
       <c r="N15" t="str">
         <f t="shared" si="3"/>
-        <v>EE_LNG</v>
+        <v>FI_LNG</v>
       </c>
       <c r="O15" t="str">
         <f t="shared" si="4"/>
-        <v>EE</v>
+        <v>FI</v>
       </c>
     </row>
     <row r="16" spans="1:15">
       <c r="A16" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B16" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
       <c r="C16">
-        <v>5</v>
+        <v>31.2</v>
       </c>
       <c r="E16" s="1">
         <f t="shared" si="0"/>
@@ -18754,40 +18791,40 @@
       </c>
       <c r="G16">
         <f t="shared" si="5"/>
-        <v>5</v>
+        <v>31.2</v>
       </c>
       <c r="H16">
         <f t="shared" si="1"/>
-        <v>48849.999999999993</v>
+        <v>304823.99999999994</v>
       </c>
       <c r="I16">
         <f t="shared" si="2"/>
-        <v>48.849999999999994</v>
+        <v>304.82399999999996</v>
       </c>
       <c r="K16" t="s">
-        <v>54</v>
+        <v>19</v>
       </c>
       <c r="L16" t="s">
         <v>100</v>
       </c>
       <c r="N16" t="str">
         <f t="shared" si="3"/>
-        <v>FI_LNG</v>
+        <v>DE_LNG</v>
       </c>
       <c r="O16" t="str">
         <f t="shared" si="4"/>
-        <v>FI</v>
+        <v>DE</v>
       </c>
     </row>
     <row r="17" spans="1:15">
       <c r="A17" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B17" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="C17">
-        <v>31.2</v>
+        <v>2.6</v>
       </c>
       <c r="E17" s="1">
         <f t="shared" si="0"/>
@@ -18795,40 +18832,40 @@
       </c>
       <c r="G17">
         <f t="shared" si="5"/>
-        <v>31.2</v>
+        <v>2.6</v>
       </c>
       <c r="H17">
         <f t="shared" si="1"/>
-        <v>304823.99999999994</v>
+        <v>25402</v>
       </c>
       <c r="I17">
         <f t="shared" si="2"/>
-        <v>304.82399999999996</v>
+        <v>25.402000000000001</v>
       </c>
       <c r="K17" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="L17" t="s">
         <v>100</v>
       </c>
       <c r="N17" t="str">
         <f t="shared" si="3"/>
-        <v>DE_LNG</v>
+        <v>IE_LNG</v>
       </c>
       <c r="O17" t="str">
         <f t="shared" si="4"/>
-        <v>DE</v>
+        <v>IE</v>
       </c>
     </row>
     <row r="18" spans="1:15">
       <c r="A18" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="C18">
-        <v>2.6</v>
+        <v>1.5</v>
       </c>
       <c r="E18" s="1">
         <f t="shared" si="0"/>
@@ -18836,70 +18873,59 @@
       </c>
       <c r="G18">
         <f t="shared" si="5"/>
-        <v>2.6</v>
+        <v>1.5</v>
       </c>
       <c r="H18">
         <f t="shared" si="1"/>
-        <v>25402</v>
+        <v>14655</v>
       </c>
       <c r="I18">
         <f t="shared" si="2"/>
-        <v>25.402000000000001</v>
+        <v>14.654999999999999</v>
       </c>
       <c r="K18" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="L18" t="s">
         <v>100</v>
       </c>
       <c r="N18" t="str">
         <f t="shared" si="3"/>
-        <v>IE_LNG</v>
+        <v>LV_LNG</v>
       </c>
       <c r="O18" t="str">
         <f t="shared" si="4"/>
-        <v>IE</v>
+        <v>LV</v>
       </c>
     </row>
     <row r="19" spans="1:15">
       <c r="A19" t="s">
-        <v>131</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="C19">
-        <v>1.5</v>
+        <v>0.7</v>
       </c>
       <c r="E19" s="1">
-        <f t="shared" si="0"/>
+        <f>D19/C19</f>
         <v>0</v>
       </c>
       <c r="G19">
-        <f t="shared" si="5"/>
-        <v>1.5</v>
+        <f>IF(C19&gt;F19,C19,F19)</f>
+        <v>0.7</v>
       </c>
       <c r="H19">
-        <f t="shared" si="1"/>
-        <v>14655</v>
+        <f>I19*1000</f>
+        <v>6838.9999999999991</v>
       </c>
       <c r="I19">
-        <f t="shared" si="2"/>
-        <v>14.654999999999999</v>
+        <f>G19*9.77</f>
+        <v>6.8389999999999995</v>
       </c>
       <c r="K19" t="s">
-        <v>35</v>
-      </c>
-      <c r="L19" t="s">
-        <v>100</v>
-      </c>
-      <c r="N19" t="str">
-        <f t="shared" si="3"/>
-        <v>LV_LNG</v>
-      </c>
-      <c r="O19" t="str">
-        <f t="shared" si="4"/>
-        <v>LV</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix LNG data error for TR LNG import
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D1FD654-22F3-4AC3-81DE-9CBBA6A3F9C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06CE56BC-1B15-4FBF-BAC0-FC2181ABA5EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7390" yWindow="0" windowWidth="14400" windowHeight="10170" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng_europe_2020" sheetId="1" r:id="rId1"/>
@@ -926,9 +926,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -1207,7 +1207,7 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0">
       <alignment horizontal="right"/>
@@ -1228,13 +1228,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyFill="0" applyBorder="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyFill="0" applyBorder="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
@@ -1246,19 +1246,19 @@
   <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="41">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -1473,10 +1473,10 @@
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1526,16 +1526,16 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1585,16 +1585,16 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1638,25 +1638,25 @@
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -1700,16 +1700,16 @@
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
+      <numFmt numFmtId="165" formatCode="0.0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2296,7 +2296,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O14"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" t="s">
@@ -2821,19 +2821,19 @@
         <v>0.33944954128440369</v>
       </c>
       <c r="F12">
-        <v>14.8</v>
+        <v>43.6</v>
       </c>
       <c r="G12">
-        <f t="shared" si="1"/>
-        <v>14.8</v>
+        <f>IF(C12&gt;F12,F12,C12)</f>
+        <v>43.6</v>
       </c>
       <c r="H12">
         <f t="shared" si="2"/>
-        <v>144596</v>
+        <v>425972</v>
       </c>
       <c r="I12">
         <f t="shared" si="3"/>
-        <v>144.596</v>
+        <v>425.97199999999998</v>
       </c>
       <c r="K12" t="s">
         <v>46</v>
@@ -2938,13 +2938,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06AEBB83-8C6D-4234-B52F-BC23EBBF1927}">
   <dimension ref="A1:G53"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" customWidth="1"/>
-    <col min="2" max="2" width="20.36328125" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" customWidth="1"/>
+    <col min="5" max="5" width="22.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4050,14 +4050,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB74EFE2-1976-4863-9D34-7D94C847C875}">
   <dimension ref="A1:G25"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" customWidth="1"/>
-    <col min="2" max="2" width="20.36328125" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="6" width="22.26953125" customWidth="1"/>
-    <col min="7" max="7" width="12.81640625" customWidth="1"/>
+    <col min="5" max="6" width="22.21875" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4604,13 +4604,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD7211D-DC17-4DD6-B657-CA08F8FBC20F}">
   <dimension ref="A1:H109"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="3" width="20.453125" customWidth="1"/>
-    <col min="4" max="4" width="17.26953125" customWidth="1"/>
-    <col min="5" max="5" width="16.1796875" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" customWidth="1"/>
-    <col min="11" max="12" width="10.26953125" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="4" max="4" width="17.21875" customWidth="1"/>
+    <col min="5" max="5" width="16.21875" customWidth="1"/>
+    <col min="6" max="6" width="8.77734375" customWidth="1"/>
+    <col min="11" max="12" width="10.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -6815,7 +6815,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58F6DC53-AE01-4DBE-BF9B-43427CD51EF0}">
   <dimension ref="A1:F37"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -7464,13 +7464,13 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67CAB708-6819-43AD-B444-2B653F840206}">
   <dimension ref="A1:H116"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="3" width="20.453125" customWidth="1"/>
-    <col min="4" max="4" width="17.26953125" customWidth="1"/>
-    <col min="5" max="5" width="16.1796875" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" customWidth="1"/>
-    <col min="11" max="12" width="10.26953125" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
+    <col min="4" max="4" width="17.21875" customWidth="1"/>
+    <col min="5" max="5" width="16.21875" customWidth="1"/>
+    <col min="6" max="6" width="8.77734375" customWidth="1"/>
+    <col min="11" max="12" width="10.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -9791,12 +9791,12 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B77213A-E4EC-469C-967C-1084709D3A56}">
   <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="3" width="17.453125" customWidth="1"/>
-    <col min="4" max="4" width="8.81640625" customWidth="1"/>
-    <col min="6" max="6" width="16.08984375" customWidth="1"/>
-    <col min="7" max="7" width="14.36328125" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" customWidth="1"/>
+    <col min="4" max="4" width="8.77734375" customWidth="1"/>
+    <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -10163,12 +10163,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A362E1-49DF-4BF1-8271-A810EC1D90D2}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:M170"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="3" width="21.81640625" customWidth="1"/>
+    <col min="3" max="3" width="21.77734375" customWidth="1"/>
     <col min="4" max="4" width="9" customWidth="1"/>
-    <col min="6" max="6" width="16.453125" customWidth="1"/>
-    <col min="7" max="7" width="15.54296875" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" customWidth="1"/>
+    <col min="7" max="7" width="15.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -14160,12 +14160,12 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72793A9-6514-42B6-BB9D-65D406982860}">
   <dimension ref="A1:M215"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="3" width="21.81640625" customWidth="1"/>
+    <col min="3" max="3" width="21.77734375" customWidth="1"/>
     <col min="4" max="4" width="9" customWidth="1"/>
-    <col min="6" max="6" width="16.453125" customWidth="1"/>
-    <col min="7" max="7" width="15.54296875" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" customWidth="1"/>
+    <col min="7" max="7" width="15.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
@@ -19207,7 +19207,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B0A4E44-EF0E-4B6E-954F-142396EAD0D0}">
   <dimension ref="A1:O19"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" t="s">
@@ -20087,7 +20087,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21A4C99F-E9F5-40FD-9F17-3E8BE1B3E129}">
   <dimension ref="A1:O19"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" t="s">
@@ -20967,13 +20967,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77CF82F4-4954-4D06-9A30-AE8575CA18DE}">
   <dimension ref="A1:N49"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" customWidth="1"/>
-    <col min="2" max="2" width="19.26953125" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" customWidth="1"/>
+    <col min="2" max="2" width="19.21875" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="17.08984375" customWidth="1"/>
-    <col min="5" max="6" width="17.7265625" customWidth="1"/>
+    <col min="4" max="4" width="17.109375" customWidth="1"/>
+    <col min="5" max="6" width="17.77734375" customWidth="1"/>
     <col min="7" max="8" width="15" customWidth="1"/>
   </cols>
   <sheetData>
@@ -22410,13 +22410,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CB51A3E-1808-4462-B1E3-D6075EC1FD95}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" customWidth="1"/>
-    <col min="2" max="2" width="19.26953125" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" customWidth="1"/>
+    <col min="2" max="2" width="19.21875" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="17.08984375" customWidth="1"/>
-    <col min="5" max="6" width="17.7265625" customWidth="1"/>
+    <col min="4" max="4" width="17.109375" customWidth="1"/>
+    <col min="5" max="6" width="17.77734375" customWidth="1"/>
     <col min="7" max="8" width="15" customWidth="1"/>
   </cols>
   <sheetData>
@@ -22844,15 +22844,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{036BBBE1-80BC-4BBB-9141-C576056723F9}">
   <dimension ref="A1:N49"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
     <col min="3" max="8" width="15" customWidth="1"/>
-    <col min="12" max="12" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.453125" customWidth="1"/>
-    <col min="17" max="17" width="18.1796875" customWidth="1"/>
-    <col min="18" max="18" width="14.453125" customWidth="1"/>
+    <col min="12" max="12" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.44140625" customWidth="1"/>
+    <col min="17" max="17" width="18.21875" customWidth="1"/>
+    <col min="18" max="18" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -24282,15 +24282,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69DF3FF5-BC43-47FD-93E8-972E7148D64B}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
     <col min="3" max="8" width="15" customWidth="1"/>
-    <col min="12" max="12" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.453125" customWidth="1"/>
-    <col min="17" max="17" width="18.1796875" customWidth="1"/>
-    <col min="18" max="18" width="14.453125" customWidth="1"/>
+    <col min="12" max="12" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.44140625" customWidth="1"/>
+    <col min="17" max="17" width="18.21875" customWidth="1"/>
+    <col min="18" max="18" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -24717,14 +24717,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE55996C-4401-4161-B17D-CF2A8462856A}">
   <dimension ref="A1:G53"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" customWidth="1"/>
-    <col min="14" max="14" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.21875" customWidth="1"/>
+    <col min="14" max="14" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -25836,14 +25836,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FF12057-E499-4FE6-95AB-7A9B585F85EC}">
   <dimension ref="A1:I25"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.54296875" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="6" width="22.26953125" customWidth="1"/>
-    <col min="15" max="15" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="22.21875" customWidth="1"/>
+    <col min="15" max="15" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">

</xml_diff>

<commit_message>
add input files for future scenarios
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63F5A98-2299-478A-B607-EBDC24F31B25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E704C5A7-308B-4E93-8A68-E9D295DCCD93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-4590" yWindow="-21720" windowWidth="38640" windowHeight="21120" firstSheet="8" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng_europe_2020" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3091" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3091" uniqueCount="304">
   <si>
     <t>Belgium</t>
   </si>
@@ -958,9 +958,6 @@
     <t>Sum not EU</t>
   </si>
   <si>
-    <t>GWh [2035]</t>
-  </si>
-  <si>
     <t>Mrd m3 [2035] AP</t>
   </si>
   <si>
@@ -1358,33 +1355,6 @@
   </cellStyles>
   <dxfs count="81">
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
@@ -1550,6 +1520,9 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
@@ -1592,6 +1565,30 @@
           <bgColor theme="4"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -1909,17 +1906,17 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{CA354A90-14CD-497C-B488-7AEC84647A3E}" name="Country"/>
     <tableColumn id="2" xr3:uid="{8DE20B36-5C6F-46B2-80C9-98806D0DE7C8}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{F7413FD2-EBE6-4DD0-9ECA-4E33D07269BA}" name="GWh [2035] SP" dataDxfId="7">
+    <tableColumn id="3" xr3:uid="{F7413FD2-EBE6-4DD0-9ECA-4E33D07269BA}" name="GWh [2035] SP" dataDxfId="29">
       <calculatedColumnFormula>Table1515[[#This Row],[GWh '[2035'] SP]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{B0F52B8B-7854-4A88-A627-18C628B9FFAB}" name="TWh [2023]" dataDxfId="4">
+    <tableColumn id="4" xr3:uid="{B0F52B8B-7854-4A88-A627-18C628B9FFAB}" name="TWh [2023]" dataDxfId="28">
       <calculatedColumnFormula>Table1517[[#This Row],[GWh '[2035'] SP]]/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{F2B47B18-6912-445C-AA80-0884F2982CF7}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="7" xr3:uid="{479DE42A-4BF3-4462-BF4B-2B4124E58CD6}" name="GWh [2035]" dataDxfId="5">
+    <tableColumn id="7" xr3:uid="{479DE42A-4BF3-4462-BF4B-2B4124E58CD6}" name="GWh [2020]" dataDxfId="27">
       <calculatedColumnFormula>Table1517[[#This Row],[TWh '[2023']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{3EC6FD5C-175B-4AEC-9875-DCE8BEBC18DA}" name="TWh by share" dataDxfId="6">
+    <tableColumn id="6" xr3:uid="{3EC6FD5C-175B-4AEC-9875-DCE8BEBC18DA}" name="TWh by share" dataDxfId="26">
       <calculatedColumnFormula>IF(Table1517[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1936,17 +1933,17 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{525F5FD4-F46E-4308-AA80-F6754BF33842}" name="Country"/>
     <tableColumn id="2" xr3:uid="{EE4F2458-B9D9-4284-9A97-E1F2DBBADABD}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{4BCACEF1-2365-46F5-80EF-FF82C7864181}" name="GWh [2035] SP" dataDxfId="0">
+    <tableColumn id="3" xr3:uid="{4BCACEF1-2365-46F5-80EF-FF82C7864181}" name="GWh [2035] SP" dataDxfId="25">
       <calculatedColumnFormula>Table1515[[#This Row],[GWh '[2035'] AP]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{242F6F74-7D77-4BEA-9D4C-482848363307}" name="TWh [2023]" dataDxfId="3">
+    <tableColumn id="4" xr3:uid="{242F6F74-7D77-4BEA-9D4C-482848363307}" name="TWh [2023]" dataDxfId="24">
       <calculatedColumnFormula>Table151718[[#This Row],[GWh '[2035'] SP]]/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{351CAF98-30C7-4411-A6AE-C7305BC7E6B7}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="7" xr3:uid="{B08E4D2A-92D2-4C87-BFBE-D74D0C85B64C}" name="GWh [2035]" dataDxfId="2">
+    <tableColumn id="7" xr3:uid="{B08E4D2A-92D2-4C87-BFBE-D74D0C85B64C}" name="GWh [2020]" dataDxfId="23">
       <calculatedColumnFormula>Table151718[[#This Row],[TWh '[2023']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{F133F4B6-959B-4931-9BF3-538BD68B0E51}" name="TWh by share" dataDxfId="1">
+    <tableColumn id="6" xr3:uid="{F133F4B6-959B-4931-9BF3-538BD68B0E51}" name="TWh by share" dataDxfId="22">
       <calculatedColumnFormula>IF(Table151718[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1955,20 +1952,20 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{5979395A-60EB-4AFC-9198-70689EC3039D}" name="Table79101116" displayName="Table79101116" ref="A1:G22" totalsRowShown="0" headerRowDxfId="29" headerRowBorderDxfId="28" tableBorderDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{5979395A-60EB-4AFC-9198-70689EC3039D}" name="Table79101116" displayName="Table79101116" ref="A1:G22" totalsRowShown="0" headerRowDxfId="21" headerRowBorderDxfId="20" tableBorderDxfId="19">
   <autoFilter ref="A1:G22" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{D09F8E08-D996-4BEB-AB9C-D48B4A898D7C}" name="Country"/>
     <tableColumn id="2" xr3:uid="{202242D6-E4EB-4567-904C-69F3B6D0975C}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{81E76B95-7303-43E1-9C36-60BF9F571714}" name="Mrd m3 [2035]"/>
     <tableColumn id="4" xr3:uid="{056327DC-03D3-42F1-9E67-77A2986E3E1D}" name="values 2024"/>
-    <tableColumn id="5" xr3:uid="{045572F5-912C-4B6C-8BCA-CCE183AD4A4E}" name="Mrd m3 [2020]2" dataDxfId="26">
+    <tableColumn id="5" xr3:uid="{045572F5-912C-4B6C-8BCA-CCE183AD4A4E}" name="Mrd m3 [2020]2" dataDxfId="18">
       <calculatedColumnFormula>Table79101116[[#This Row],[values 2024]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{DA064D9E-1168-4CB6-B3AA-E50FAC653181}" name="GWh [2020]" dataDxfId="25">
+    <tableColumn id="7" xr3:uid="{DA064D9E-1168-4CB6-B3AA-E50FAC653181}" name="GWh [2020]" dataDxfId="17">
       <calculatedColumnFormula>Table79101116[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{EAF9FC8E-89CB-4295-BD8E-F84762361F50}" name="TWh [2020]" dataDxfId="8">
+    <tableColumn id="6" xr3:uid="{EAF9FC8E-89CB-4295-BD8E-F84762361F50}" name="TWh [2020]" dataDxfId="16">
       <calculatedColumnFormula>Table79101116[[#This Row],[Mrd m3 '[2035']]]*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1988,7 +1985,7 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="24">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="15">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
@@ -2012,7 +2009,7 @@
     <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="23">
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="14">
       <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
@@ -2031,10 +2028,10 @@
     <tableColumn id="1" xr3:uid="{8DC4F854-8C96-4C42-AF47-2C64D82D363F}" name="From"/>
     <tableColumn id="2" xr3:uid="{9178F7D7-E3CA-468B-8BE5-E203B9CC620E}" name="To"/>
     <tableColumn id="3" xr3:uid="{9BB01476-57DE-4D59-8170-98FAC18CF80C}" name="bcm/a  [capacity]"/>
-    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a" dataDxfId="22">
+    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a" dataDxfId="13">
       <calculatedColumnFormula>C2*9.77*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="21">
+    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="12">
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{19F26947-5FDD-4F06-A68D-DB6766B439A7}" name="distance [miles]"/>
@@ -2049,7 +2046,7 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I170" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18" totalsRowBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I170" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
   <autoFilter ref="A1:I170" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
@@ -2062,10 +2059,10 @@
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{7E7B8CB5-D54F-4427-813D-93B66C13FCBB}" name="Distance [miles]"/>
-    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="16">
+    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="7">
       <calculatedColumnFormula>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="6"/>
     <tableColumn id="8" xr3:uid="{ECBB25E4-2145-4120-8981-E6E8E1591E5B}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2073,7 +2070,7 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{A41F31BC-0CA5-4B1A-808E-7A8A6507019C}" name="LNG_global14" displayName="LNG_global14" ref="A1:I215" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="13" tableBorderDxfId="12" totalsRowBorderDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{A41F31BC-0CA5-4B1A-808E-7A8A6507019C}" name="LNG_global14" displayName="LNG_global14" ref="A1:I215" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
   <autoFilter ref="A1:I215" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D01CBB17-E8FF-44A2-B87B-A0B5AC3337BA}" name="From"/>
@@ -2086,10 +2083,10 @@
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{B6C8563B-B70E-4D32-A7CA-353FAC6B7501}" name="Distance [miles]"/>
-    <tableColumn id="4" xr3:uid="{DB3ABB11-1F6C-4F58-B946-9343785CF33A}" name="Distance [km]" dataDxfId="10">
+    <tableColumn id="4" xr3:uid="{DB3ABB11-1F6C-4F58-B946-9343785CF33A}" name="Distance [km]" dataDxfId="1">
       <calculatedColumnFormula>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{601054B1-1B08-47CB-880D-0D80ED1BD0EA}" name="Suez or Panama" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{601054B1-1B08-47CB-880D-0D80ED1BD0EA}" name="Suez or Panama" dataDxfId="0"/>
     <tableColumn id="8" xr3:uid="{F8768BD8-8B11-4BD9-B074-AD5ADFFDF447}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -4888,10 +4885,10 @@
         <v>55</v>
       </c>
       <c r="C1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E1" t="s">
         <v>134</v>
@@ -4906,10 +4903,10 @@
         <v>266</v>
       </c>
       <c r="I1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K1" t="s">
         <v>118</v>
@@ -6850,7 +6847,7 @@
         <v>55</v>
       </c>
       <c r="C1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D1" t="s">
         <v>133</v>
@@ -6859,7 +6856,7 @@
         <v>107</v>
       </c>
       <c r="F1" t="s">
-        <v>300</v>
+        <v>266</v>
       </c>
       <c r="G1" t="s">
         <v>118</v>
@@ -8022,7 +8019,7 @@
         <v>55</v>
       </c>
       <c r="C1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D1" t="s">
         <v>133</v>
@@ -8031,7 +8028,7 @@
         <v>107</v>
       </c>
       <c r="F1" t="s">
-        <v>300</v>
+        <v>266</v>
       </c>
       <c r="G1" t="s">
         <v>118</v>

</xml_diff>

<commit_message>
update with more 2019 data
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marianapessoa/Desktop/gas_infrastructure_model/01_data/01_input_data/02_processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FE361DB-5C15-7847-8575-AF0818D28CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC1B6802-6AAC-434F-8A4F-A3918366CFEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15100" yWindow="680" windowWidth="15140" windowHeight="18040" tabRatio="790" firstSheet="19" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="790" firstSheet="26" activeTab="31" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EDIT_nodes_lng_europe_2019" sheetId="32" r:id="rId1"/>
@@ -1066,7 +1066,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1217,6 +1217,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1395,7 +1402,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1418,6 +1425,7 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -1463,7 +1471,38 @@
     <cellStyle name="Percent 4" xfId="35" xr:uid="{FBC58B8C-7B58-4A54-9EE4-7950F3EA222E}"/>
     <cellStyle name="Percent 8" xfId="33" xr:uid="{304ED844-55A0-412B-ADC5-6D43390D8D63}"/>
   </cellStyles>
-  <dxfs count="132">
+  <dxfs count="134">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0" tint="-0.499984740745262"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0" tint="-0.499984740745262"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1753,9 +1792,6 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
@@ -1869,53 +1905,6 @@
       <border outline="0">
         <bottom style="thin">
           <color rgb="FF9BC2E6"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
         </bottom>
       </border>
     </dxf>
@@ -2293,6 +2282,53 @@
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2315,15 +2351,15 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{4EA90B67-C1EA-3F49-80BD-F698B4BB1753}" name="Country"/>
     <tableColumn id="2" xr3:uid="{DE488C4E-BA4D-1C47-919F-17B200DC8E8E}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{40424F55-FF29-C846-9670-45BDC1946AF7}" name="Mrd m3 [2019]" dataDxfId="131"/>
-    <tableColumn id="5" xr3:uid="{CE68E676-D995-F544-BEB7-55E7188768DB}" name="Mil m3 EU [2019]" dataDxfId="130"/>
-    <tableColumn id="6" xr3:uid="{9428BA11-0FA4-4E43-B422-05EB8A043647}" name="Mrd m3 EU [2019]2" dataDxfId="129">
+    <tableColumn id="3" xr3:uid="{40424F55-FF29-C846-9670-45BDC1946AF7}" name="Mrd m3 [2019]" dataDxfId="127"/>
+    <tableColumn id="5" xr3:uid="{CE68E676-D995-F544-BEB7-55E7188768DB}" name="Mil m3 EU [2019]" dataDxfId="126"/>
+    <tableColumn id="6" xr3:uid="{9428BA11-0FA4-4E43-B422-05EB8A043647}" name="Mrd m3 EU [2019]2" dataDxfId="125">
       <calculatedColumnFormula>Table224[[#This Row],[Mil m3 EU '[2019']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{444B9436-1239-F240-B4BF-1A913EC4CFF6}" name="GWh [2019]" dataDxfId="128">
+    <tableColumn id="7" xr3:uid="{444B9436-1239-F240-B4BF-1A913EC4CFF6}" name="GWh [2019]" dataDxfId="124">
       <calculatedColumnFormula>Table224[[#This Row],[TWh '[2019']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5EF9A97F-15E9-B540-80E9-F7A73E08637D}" name="TWh [2019]" dataDxfId="127">
+    <tableColumn id="4" xr3:uid="{5EF9A97F-15E9-B540-80E9-F7A73E08637D}" name="TWh [2019]" dataDxfId="123">
       <calculatedColumnFormula>IF(Table224[[#This Row],[Mil m3 EU '[2019']]]&gt;0,Table224[[#This Row],[Mrd m3 EU '[2019']2]],Table224[[#This Row],[Mrd m3 '[2019']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2340,15 +2376,15 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{4489F77B-7E3D-6B40-999F-0A5CFAAD43D0}" name="Country"/>
     <tableColumn id="2" xr3:uid="{ED6C7C95-39E5-C744-B5E7-2363DA50B5F7}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{480BAFC6-8BED-3B47-93A3-FFC4E41F5BDF}" name="Mrd m3 [2019]" dataDxfId="82"/>
-    <tableColumn id="4" xr3:uid="{5500BCB9-3E14-4C44-A98A-BF3DBD011C25}" name="TWh [2019]" dataDxfId="81">
+    <tableColumn id="3" xr3:uid="{480BAFC6-8BED-3B47-93A3-FFC4E41F5BDF}" name="Mrd m3 [2019]" dataDxfId="78"/>
+    <tableColumn id="4" xr3:uid="{5500BCB9-3E14-4C44-A98A-BF3DBD011C25}" name="TWh [2019]" dataDxfId="77">
       <calculatedColumnFormula>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{88D78A88-5D7E-CD41-AD80-CBB8F276CCA0}" name="Population 2019 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{895AA06E-8015-F44E-8A03-C29DA4E1A648}" name="TWh by share" dataDxfId="80">
+    <tableColumn id="6" xr3:uid="{895AA06E-8015-F44E-8A03-C29DA4E1A648}" name="TWh by share" dataDxfId="76">
       <calculatedColumnFormula>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{474AC10A-97FA-2941-AAF0-7C38AC898810}" name="GWh [2019]" dataDxfId="79">
+    <tableColumn id="7" xr3:uid="{474AC10A-97FA-2941-AAF0-7C38AC898810}" name="GWh [2019]" dataDxfId="75">
       <calculatedColumnFormula>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2365,15 +2401,15 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{2E667126-F0AE-4045-8045-2063C112853F}" name="Country"/>
     <tableColumn id="2" xr3:uid="{536DA57B-A186-41E1-8967-E3467594200F}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="78"/>
-    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="77">
+    <tableColumn id="3" xr3:uid="{DEF527B1-DA00-467C-9DB5-2DC94D9B506B}" name="Mrd m3 [2020]" dataDxfId="74"/>
+    <tableColumn id="4" xr3:uid="{1618AAC4-0782-47C3-91CE-2FEB95FBDD58}" name="TWh [2020]" dataDxfId="73">
       <calculatedColumnFormula>Table1[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{0221D38A-A241-4AD5-A477-B5DD5AC2F6CF}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="76">
+    <tableColumn id="6" xr3:uid="{3EB83E78-D0C6-4E28-AD34-69D840CBB511}" name="TWh by share" dataDxfId="72">
       <calculatedColumnFormula>IF(Table1[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{53C148C2-CAF7-47BC-9950-964805B82325}" name="GWh [2020]" dataDxfId="75">
+    <tableColumn id="7" xr3:uid="{53C148C2-CAF7-47BC-9950-964805B82325}" name="GWh [2020]" dataDxfId="71">
       <calculatedColumnFormula>MIN(Table1[[#This Row],[TWh '[2020']]],Table1[[#This Row],[TWh by share]])*1000</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2390,15 +2426,15 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{1826A6AD-7549-4A36-9CAD-F7CC4267BC89}" name="Country"/>
     <tableColumn id="2" xr3:uid="{14DF1FF8-80AC-4997-9DB3-672516878B5D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="74"/>
-    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="73">
+    <tableColumn id="3" xr3:uid="{889AC7A4-1DBA-4A7D-96F7-5301C2F9E594}" name="Mrd m3 [2023]" dataDxfId="70"/>
+    <tableColumn id="4" xr3:uid="{60E83C2D-D521-4D6A-800D-160C3176DFC7}" name="TWh [2023]" dataDxfId="69">
       <calculatedColumnFormula>Table15[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{1EC72689-3FEE-4998-85C2-E4533CF3E650}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="7" xr3:uid="{9AD7149D-CE4C-40DA-896B-BFCD92F06B1A}" name="GWh [2020]" dataDxfId="72">
+    <tableColumn id="7" xr3:uid="{9AD7149D-CE4C-40DA-896B-BFCD92F06B1A}" name="GWh [2020]" dataDxfId="68">
       <calculatedColumnFormula>MIN(Table15[[#This Row],[TWh '[2023']]],Table15[[#This Row],[TWh by share]])*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="71">
+    <tableColumn id="6" xr3:uid="{EA1A4D0E-E13A-491B-8024-93E1A98AD8DD}" name="TWh by share" dataDxfId="67">
       <calculatedColumnFormula>IF(Table15[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2415,30 +2451,30 @@
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{2B878B00-DE19-4457-BC2C-B8AE9F12C299}" name="Country"/>
     <tableColumn id="2" xr3:uid="{628D4239-33B0-4A80-B761-460829DFA970}" name="Long_name"/>
-    <tableColumn id="8" xr3:uid="{DFE1B0E7-A509-470D-83D5-78DA81BD7A41}" name="Mrd m3 [2035] SP" dataDxfId="70">
+    <tableColumn id="8" xr3:uid="{DFE1B0E7-A509-470D-83D5-78DA81BD7A41}" name="Mrd m3 [2035] SP" dataDxfId="66">
       <calculatedColumnFormula>IF(Table1515[[#This Row],[EU]]=1,$R$19*Table1515[[#This Row],[GWh '[2020']]]/$H$44,$R$18*Table1515[[#This Row],[GWh '[2020']]]/$H$45)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{254B24B5-02B5-4792-8B10-81658E257110}" name="Mrd m3 [2035] AP" dataDxfId="69">
+    <tableColumn id="11" xr3:uid="{254B24B5-02B5-4792-8B10-81658E257110}" name="Mrd m3 [2035] AP" dataDxfId="65">
       <calculatedColumnFormula>IF(Table1515[[#This Row],[EU]]=1,$T$19*Table1515[[#This Row],[GWh '[2020']]]/$H$44,$T$18*Table1515[[#This Row],[GWh '[2020']]]/$H$45)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{295B0DCE-300D-471F-B88E-BD00D3141C70}" name="Mrd m3 [2023]" dataDxfId="68"/>
-    <tableColumn id="4" xr3:uid="{CFF2A961-5340-417B-A68C-5AA0571EECB8}" name="TWh [2023]" dataDxfId="67">
+    <tableColumn id="3" xr3:uid="{295B0DCE-300D-471F-B88E-BD00D3141C70}" name="Mrd m3 [2023]" dataDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{CFF2A961-5340-417B-A68C-5AA0571EECB8}" name="TWh [2023]" dataDxfId="63">
       <calculatedColumnFormula>Table1515[[#This Row],[Mrd m3 '[2023']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{5B526716-F904-4504-B78C-90658BFD4732}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="7" xr3:uid="{F8E669A0-69F8-498E-A3E1-14221B73E054}" name="GWh [2020]" dataDxfId="66">
+    <tableColumn id="7" xr3:uid="{F8E669A0-69F8-498E-A3E1-14221B73E054}" name="GWh [2020]" dataDxfId="62">
       <calculatedColumnFormula>MIN(Table1515[[#This Row],[TWh '[2023']]],Table1515[[#This Row],[TWh by share]])*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{C231D16E-346D-4A6C-BDE3-02DCD7F98838}" name="GWh [2035] SP" dataDxfId="65">
+    <tableColumn id="10" xr3:uid="{C231D16E-346D-4A6C-BDE3-02DCD7F98838}" name="GWh [2035] SP" dataDxfId="61">
       <calculatedColumnFormula>Table1515[[#This Row],[Mrd m3 '[2035'] SP]]*9.77*-1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{B7100D75-BF53-4B84-BEA5-5B8213EA443B}" name="GWh [2035] AP" dataDxfId="64">
+    <tableColumn id="12" xr3:uid="{B7100D75-BF53-4B84-BEA5-5B8213EA443B}" name="GWh [2035] AP" dataDxfId="60">
       <calculatedColumnFormula>Table1515[[#This Row],[Mrd m3 '[2035'] AP]]*9.77*-1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{38428858-BB77-4254-A9E7-787AC7919612}" name="TWh by share" dataDxfId="63">
+    <tableColumn id="6" xr3:uid="{38428858-BB77-4254-A9E7-787AC7919612}" name="TWh by share" dataDxfId="59">
       <calculatedColumnFormula>IF(Table1515[[#This Row],[TWh '[2023']]]=0,$F$27*(G2/$G$27),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{062339C5-9866-4A10-AB51-65D785DCAE56}" name="EU" dataDxfId="62"/>
+    <tableColumn id="9" xr3:uid="{062339C5-9866-4A10-AB51-65D785DCAE56}" name="EU" dataDxfId="58"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2453,17 +2489,17 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{CA354A90-14CD-497C-B488-7AEC84647A3E}" name="Country"/>
     <tableColumn id="2" xr3:uid="{8DE20B36-5C6F-46B2-80C9-98806D0DE7C8}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{F7413FD2-EBE6-4DD0-9ECA-4E33D07269BA}" name="GWh [2035] SP" dataDxfId="61">
+    <tableColumn id="3" xr3:uid="{F7413FD2-EBE6-4DD0-9ECA-4E33D07269BA}" name="GWh [2035] SP" dataDxfId="57">
       <calculatedColumnFormula>Table1515[[#This Row],[GWh '[2035'] SP]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{B0F52B8B-7854-4A88-A627-18C628B9FFAB}" name="TWh [2023]" dataDxfId="60">
+    <tableColumn id="4" xr3:uid="{B0F52B8B-7854-4A88-A627-18C628B9FFAB}" name="TWh [2023]" dataDxfId="56">
       <calculatedColumnFormula>Table1517[[#This Row],[GWh '[2035'] SP]]/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{F2B47B18-6912-445C-AA80-0884F2982CF7}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="7" xr3:uid="{479DE42A-4BF3-4462-BF4B-2B4124E58CD6}" name="GWh [2020]" dataDxfId="59">
+    <tableColumn id="7" xr3:uid="{479DE42A-4BF3-4462-BF4B-2B4124E58CD6}" name="GWh [2020]" dataDxfId="55">
       <calculatedColumnFormula>Table1517[[#This Row],[TWh '[2023']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{3EC6FD5C-175B-4AEC-9875-DCE8BEBC18DA}" name="TWh by share" dataDxfId="58">
+    <tableColumn id="6" xr3:uid="{3EC6FD5C-175B-4AEC-9875-DCE8BEBC18DA}" name="TWh by share" dataDxfId="54">
       <calculatedColumnFormula>IF(Table1517[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2480,17 +2516,17 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{525F5FD4-F46E-4308-AA80-F6754BF33842}" name="Country"/>
     <tableColumn id="2" xr3:uid="{EE4F2458-B9D9-4284-9A97-E1F2DBBADABD}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{4BCACEF1-2365-46F5-80EF-FF82C7864181}" name="GWh [2035] SP" dataDxfId="57">
+    <tableColumn id="3" xr3:uid="{4BCACEF1-2365-46F5-80EF-FF82C7864181}" name="GWh [2035] SP" dataDxfId="53">
       <calculatedColumnFormula>Table1515[[#This Row],[GWh '[2035'] AP]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{242F6F74-7D77-4BEA-9D4C-482848363307}" name="TWh [2023]" dataDxfId="56">
+    <tableColumn id="4" xr3:uid="{242F6F74-7D77-4BEA-9D4C-482848363307}" name="TWh [2023]" dataDxfId="52">
       <calculatedColumnFormula>Table151718[[#This Row],[GWh '[2035'] SP]]/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{351CAF98-30C7-4411-A6AE-C7305BC7E6B7}" name="Population 2020 [Tsd]"/>
-    <tableColumn id="7" xr3:uid="{B08E4D2A-92D2-4C87-BFBE-D74D0C85B64C}" name="GWh [2020]" dataDxfId="55">
+    <tableColumn id="7" xr3:uid="{B08E4D2A-92D2-4C87-BFBE-D74D0C85B64C}" name="GWh [2020]" dataDxfId="51">
       <calculatedColumnFormula>Table151718[[#This Row],[TWh '[2023']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{F133F4B6-959B-4931-9BF3-538BD68B0E51}" name="TWh by share" dataDxfId="54">
+    <tableColumn id="6" xr3:uid="{F133F4B6-959B-4931-9BF3-538BD68B0E51}" name="TWh by share" dataDxfId="50">
       <calculatedColumnFormula>IF(Table151718[[#This Row],[TWh '[2023']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2499,20 +2535,20 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A1:G22" totalsRowShown="0" headerRowDxfId="53" headerRowBorderDxfId="52" tableBorderDxfId="51">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}" name="Table7910" displayName="Table7910" ref="A1:G22" totalsRowShown="0" headerRowDxfId="133" headerRowBorderDxfId="132" tableBorderDxfId="131">
   <autoFilter ref="A1:G22" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{555371BF-8030-4257-9852-212E94829B9B}" name="Country"/>
     <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2019]"/>
     <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2019]"/>
-    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2019]2" dataDxfId="50">
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2019]2" dataDxfId="130">
       <calculatedColumnFormula>Table7910[[#This Row],[Mil m3 '[2019']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{95C698CF-3EBE-40E8-840D-A6C3E41CFB2C}" name="GWh [2019]" dataDxfId="49">
+    <tableColumn id="7" xr3:uid="{95C698CF-3EBE-40E8-840D-A6C3E41CFB2C}" name="GWh [2019]" dataDxfId="129">
       <calculatedColumnFormula>Table7910[[#This Row],[TWh '[2019']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2019]" dataDxfId="48">
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2019]" dataDxfId="128">
       <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2019']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2019']2]],Table7910[[#This Row],[Mrd m3 '[2019']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2521,20 +2557,20 @@
 </file>
 
 <file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{FA734C83-A3FC-1B48-B23D-DCF1ABCAC446}" name="Table791028" displayName="Table791028" ref="A1:G22" totalsRowShown="0" headerRowDxfId="47" headerRowBorderDxfId="46" tableBorderDxfId="45">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{FA734C83-A3FC-1B48-B23D-DCF1ABCAC446}" name="Table791028" displayName="Table791028" ref="A1:G22" totalsRowShown="0" headerRowDxfId="49" headerRowBorderDxfId="48" tableBorderDxfId="47">
   <autoFilter ref="A1:G22" xr:uid="{2521D055-B007-41DB-BE6E-1CB7426AD04E}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{96F9D675-7256-9548-A428-311E909136A4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{124C11A7-4DFC-5948-A199-975ABC0AEF7A}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{0914DDA8-8934-4F4A-8B46-640C3B973A1D}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{EF70BB4A-CEE2-2449-AC67-0D0F88B3ED5D}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{7FA62D69-F373-DD4F-B89C-E6869397A85D}" name="Mrd m3 [2020]2" dataDxfId="44">
+    <tableColumn id="5" xr3:uid="{7FA62D69-F373-DD4F-B89C-E6869397A85D}" name="Mrd m3 [2020]2" dataDxfId="46">
       <calculatedColumnFormula>Table791028[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{12CA027F-55E7-0848-B901-45DB1F90674E}" name="GWh [2020]" dataDxfId="43">
+    <tableColumn id="7" xr3:uid="{12CA027F-55E7-0848-B901-45DB1F90674E}" name="GWh [2020]" dataDxfId="45">
       <calculatedColumnFormula>Table791028[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{AD4B7D3C-301E-CF4D-9ECD-2BA1C009652D}" name="TWh [2020]" dataDxfId="42">
+    <tableColumn id="6" xr3:uid="{AD4B7D3C-301E-CF4D-9ECD-2BA1C009652D}" name="TWh [2020]" dataDxfId="44">
       <calculatedColumnFormula>IF(Table791028[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791028[[#This Row],[Mrd m3 '[2020']2]],Table791028[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2543,20 +2579,20 @@
 </file>
 
 <file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A1:G22" totalsRowShown="0" headerRowDxfId="41" headerRowBorderDxfId="40" tableBorderDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}" name="Table791011" displayName="Table791011" ref="A1:G22" totalsRowShown="0" headerRowDxfId="43" headerRowBorderDxfId="42" tableBorderDxfId="41">
   <autoFilter ref="A1:G22" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C2F3768C-4A25-4EBA-988D-C95C814AC7F5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{644153F9-1004-4913-B5A7-2379099164C2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{779C3748-4ECD-495F-809A-B5DD28F5EC2F}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{94BC7314-C5A0-4AAD-895B-84E7A94D7CF7}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="38">
+    <tableColumn id="5" xr3:uid="{21C0A2F1-DDD6-47B5-AF7F-8D71E23D7D04}" name="Mrd m3 [2020]2" dataDxfId="40">
       <calculatedColumnFormula>Table791011[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{800E9158-5DB0-43C4-A644-BF3466322E9E}" name="GWh [2020]" dataDxfId="37">
+    <tableColumn id="7" xr3:uid="{800E9158-5DB0-43C4-A644-BF3466322E9E}" name="GWh [2020]" dataDxfId="39">
       <calculatedColumnFormula>Table791011[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="36">
+    <tableColumn id="6" xr3:uid="{28EBAF35-966D-44B9-8859-9AC70136DAAC}" name="TWh [2020]" dataDxfId="38">
       <calculatedColumnFormula>IF(Table791011[[#This Row],[Mil m3 '[2020']]]&gt;0,Table791011[[#This Row],[Mrd m3 '[2020']2]],Table791011[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2565,20 +2601,20 @@
 </file>
 
 <file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{5979395A-60EB-4AFC-9198-70689EC3039D}" name="Table79101116" displayName="Table79101116" ref="A1:G22" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{5979395A-60EB-4AFC-9198-70689EC3039D}" name="Table79101116" displayName="Table79101116" ref="A1:G22" totalsRowShown="0" headerRowDxfId="37" headerRowBorderDxfId="36" tableBorderDxfId="35">
   <autoFilter ref="A1:G22" xr:uid="{F8148266-610F-49B2-B97A-CC785A7B2E24}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{D09F8E08-D996-4BEB-AB9C-D48B4A898D7C}" name="Country"/>
     <tableColumn id="2" xr3:uid="{202242D6-E4EB-4567-904C-69F3B6D0975C}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{81E76B95-7303-43E1-9C36-60BF9F571714}" name="Mrd m3 [2035]"/>
     <tableColumn id="4" xr3:uid="{056327DC-03D3-42F1-9E67-77A2986E3E1D}" name="values 2024"/>
-    <tableColumn id="5" xr3:uid="{045572F5-912C-4B6C-8BCA-CCE183AD4A4E}" name="Mrd m3 [2020]2" dataDxfId="32">
+    <tableColumn id="5" xr3:uid="{045572F5-912C-4B6C-8BCA-CCE183AD4A4E}" name="Mrd m3 [2020]2" dataDxfId="34">
       <calculatedColumnFormula>Table79101116[[#This Row],[values 2024]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{DA064D9E-1168-4CB6-B3AA-E50FAC653181}" name="GWh [2020]" dataDxfId="31">
+    <tableColumn id="7" xr3:uid="{DA064D9E-1168-4CB6-B3AA-E50FAC653181}" name="GWh [2020]" dataDxfId="33">
       <calculatedColumnFormula>Table79101116[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{EAF9FC8E-89CB-4295-BD8E-F84762361F50}" name="TWh [2020]" dataDxfId="30">
+    <tableColumn id="6" xr3:uid="{EAF9FC8E-89CB-4295-BD8E-F84762361F50}" name="TWh [2020]" dataDxfId="32">
       <calculatedColumnFormula>Table79101116[[#This Row],[Mrd m3 '[2035']]]*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2587,20 +2623,20 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{D048BCD9-5248-F845-A865-B0D8AE3995E8}" name="Table725" displayName="Table725" ref="A1:G17" totalsRowShown="0" headerRowDxfId="126" headerRowBorderDxfId="125" tableBorderDxfId="124">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{D048BCD9-5248-F845-A865-B0D8AE3995E8}" name="Table725" displayName="Table725" ref="A1:G17" totalsRowShown="0" headerRowDxfId="122" headerRowBorderDxfId="121" tableBorderDxfId="120">
   <autoFilter ref="A1:G17" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{A255C403-77A0-0149-952F-A878846F39C1}" name="Country"/>
     <tableColumn id="2" xr3:uid="{923C0F82-BEBC-E940-A917-C4E2F7D4734E}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{FFD27A1A-A51B-1C48-8D57-2446CC1CEFBF}" name="Mrd m3 [2019]"/>
     <tableColumn id="4" xr3:uid="{78BA9F62-196E-484F-9DEC-52A98B938429}" name="Mil m3 [2019]"/>
-    <tableColumn id="5" xr3:uid="{1E9161F2-5CB8-5841-990F-B983C48048E4}" name="Mrd m3 [2019]2" dataDxfId="123">
+    <tableColumn id="5" xr3:uid="{1E9161F2-5CB8-5841-990F-B983C48048E4}" name="Mrd m3 [2019]2" dataDxfId="119">
       <calculatedColumnFormula>Table725[[#This Row],[Mil m3 '[2019']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{81E6D352-CF73-E24E-8012-656B58D4230F}" name="GWh [2019]" dataDxfId="122">
+    <tableColumn id="7" xr3:uid="{81E6D352-CF73-E24E-8012-656B58D4230F}" name="GWh [2019]" dataDxfId="118">
       <calculatedColumnFormula>Table725[[#This Row],[TWh '[2019']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{8E2D017E-D664-6848-A8DA-CC37D1BE073D}" name="TWh [2019]" dataDxfId="121">
+    <tableColumn id="6" xr3:uid="{8E2D017E-D664-6848-A8DA-CC37D1BE073D}" name="TWh [2019]" dataDxfId="117">
       <calculatedColumnFormula>IF(Table725[[#This Row],[Mil m3 '[2019']]]&gt;0,Table725[[#This Row],[Mrd m3 '[2019']2]],Table725[[#This Row],[Mrd m3 '[2019']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2618,9 +2654,9 @@
     <tableColumn id="1" xr3:uid="{29343813-41E4-A641-8070-D67ABD64BE0A}" name="From"/>
     <tableColumn id="2" xr3:uid="{ACE05D0C-4E30-D74A-92C2-F973C8BB52B6}" name="To"/>
     <tableColumn id="3" xr3:uid="{8ED81F2C-2D22-F744-B283-1E89EB88A242}" name="GWh/d [capacity map]"/>
-    <tableColumn id="6" xr3:uid="{5195E297-94C2-0645-B87C-EC1A27BB9F99}" name="GWh/d [gasdashboard]"/>
-    <tableColumn id="7" xr3:uid="{BA9104A7-0F21-764E-9BBD-AC74D83C7439}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{9FFECE37-B748-7342-A5CB-C4979434A80F}" name="GWh/a" dataDxfId="29">
+    <tableColumn id="6" xr3:uid="{5195E297-94C2-0645-B87C-EC1A27BB9F99}" name="GWh/d [gasdashboard]" dataDxfId="2"/>
+    <tableColumn id="7" xr3:uid="{BA9104A7-0F21-764E-9BBD-AC74D83C7439}" name="GWh/d [transparency map]" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{9FFECE37-B748-7342-A5CB-C4979434A80F}" name="GWh/a" dataDxfId="1">
       <calculatedColumnFormula>MIN(Table329[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{6E249BB4-5D70-7943-B2C0-4E614A3FBCDE}" name="TWh/a">
@@ -2644,7 +2680,7 @@
     <tableColumn id="3" xr3:uid="{E3A34820-3FE9-4103-AD3C-3049C2E0EF69}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{A0FB7BA7-3F41-4BBA-8A14-1E94492463BD}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{397AB07D-FFB8-4071-9AA1-95B47650C2EE}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="28">
+    <tableColumn id="4" xr3:uid="{3AEF69B4-7F8D-4A8D-9ECC-304CF79E8972}" name="GWh/a" dataDxfId="31">
       <calculatedColumnFormula>MIN(Table3[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C0891C32-33A4-460A-9650-5007708D8C42}" name="TWh/a">
@@ -2668,7 +2704,7 @@
     <tableColumn id="3" xr3:uid="{25844A02-A5B8-4E0F-A1F1-CADE8B45CB0B}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{F541A5EF-AB26-4856-A267-7C479F3C28D6}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{62596593-818F-4275-8D67-AF2318066747}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="27">
+    <tableColumn id="4" xr3:uid="{5C8FC5F5-71C8-46FA-A71A-C76F6BCDF27A}" name="GWh/a" dataDxfId="30">
       <calculatedColumnFormula>MIN(Table37[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{4A6D83FB-F45E-426C-993C-A96BB790CCE2}" name="TWh/a">
@@ -2692,7 +2728,7 @@
     <tableColumn id="3" xr3:uid="{3961CA94-120C-4D7F-838A-2782DE770307}" name="GWh/d [capacity map]"/>
     <tableColumn id="6" xr3:uid="{BC96C019-BAD0-42F2-A4E0-6FC2B5CF7E7E}" name="GWh/d [gasdashboard]"/>
     <tableColumn id="7" xr3:uid="{BA51C83F-53CF-4697-8BF0-04CFAA5A3ABA}" name="GWh/d [transparency map]"/>
-    <tableColumn id="4" xr3:uid="{0AF8716B-5260-42CA-B823-A9869A7B5780}" name="GWh/a" dataDxfId="26">
+    <tableColumn id="4" xr3:uid="{0AF8716B-5260-42CA-B823-A9869A7B5780}" name="GWh/a" dataDxfId="29">
       <calculatedColumnFormula>MIN(Table3722[[#This Row],[GWh/d '[capacity map']]:[GWh/d '[transparency map']]])*365</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{94A09920-447D-4D05-850B-5DCBDB5251A4}" name="TWh/a">
@@ -2711,10 +2747,10 @@
     <tableColumn id="1" xr3:uid="{8DC4F854-8C96-4C42-AF47-2C64D82D363F}" name="From"/>
     <tableColumn id="2" xr3:uid="{9178F7D7-E3CA-468B-8BE5-E203B9CC620E}" name="To"/>
     <tableColumn id="3" xr3:uid="{9BB01476-57DE-4D59-8170-98FAC18CF80C}" name="bcm/a  [capacity]"/>
-    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a" dataDxfId="25">
+    <tableColumn id="4" xr3:uid="{C2ACAF97-BD78-4A6B-9BC8-C18DDEE06FC3}" name="GWh/a" dataDxfId="28">
       <calculatedColumnFormula>C2*9.77*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="24">
+    <tableColumn id="5" xr3:uid="{01416B1F-02D4-4015-854F-1DF81E1DF7B6}" name="TWh/a" dataDxfId="27">
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{19F26947-5FDD-4F06-A68D-DB6766B439A7}" name="distance [miles]"/>
@@ -2729,7 +2765,7 @@
 </file>
 
 <file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{BB378895-57ED-AD4E-8811-E43BB6AA90EE}" name="LNG_global27" displayName="LNG_global27" ref="A1:I170" totalsRowShown="0" headerRowDxfId="23" headerRowBorderDxfId="22" tableBorderDxfId="21" totalsRowBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="26" xr:uid="{BB378895-57ED-AD4E-8811-E43BB6AA90EE}" name="LNG_global27" displayName="LNG_global27" ref="A1:I170" totalsRowShown="0" headerRowDxfId="26" headerRowBorderDxfId="25" tableBorderDxfId="24" totalsRowBorderDxfId="23">
   <autoFilter ref="A1:I170" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{EAD47311-2421-F946-A66E-74B2C1272520}" name="From"/>
@@ -2742,10 +2778,10 @@
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{B8560B18-F458-1D48-8E57-992A195CF954}" name="Distance [miles]"/>
-    <tableColumn id="4" xr3:uid="{67FC28D9-1637-1F44-A6D5-007D6902FAF9}" name="Distance [km]" dataDxfId="19">
+    <tableColumn id="4" xr3:uid="{67FC28D9-1637-1F44-A6D5-007D6902FAF9}" name="Distance [km]" dataDxfId="22">
       <calculatedColumnFormula>LNG_global27[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{15BD6826-0224-DB4A-BFC1-6F6D7F582F74}" name="Suez or Panama" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{15BD6826-0224-DB4A-BFC1-6F6D7F582F74}" name="Suez or Panama" dataDxfId="21"/>
     <tableColumn id="8" xr3:uid="{814F8409-DF49-C04A-A92B-5D72A857789A}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2753,7 +2789,7 @@
 </file>
 
 <file path=xl/tables/table26.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I170" totalsRowShown="0" headerRowDxfId="17" headerRowBorderDxfId="16" tableBorderDxfId="15" totalsRowBorderDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}" name="LNG_global" displayName="LNG_global" ref="A1:I170" totalsRowShown="0" headerRowDxfId="20" headerRowBorderDxfId="19" tableBorderDxfId="18" totalsRowBorderDxfId="17">
   <autoFilter ref="A1:I170" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D87F3249-C438-463D-BC6F-F254968A928D}" name="From"/>
@@ -2766,10 +2802,10 @@
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{7E7B8CB5-D54F-4427-813D-93B66C13FCBB}" name="Distance [miles]"/>
-    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="13">
+    <tableColumn id="4" xr3:uid="{471A6E47-FCB7-45E1-9F0A-DCC77964F44D}" name="Distance [km]" dataDxfId="16">
       <calculatedColumnFormula>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{DD9D70F1-D00A-43D9-9F09-037C2573E34A}" name="Suez or Panama" dataDxfId="15"/>
     <tableColumn id="8" xr3:uid="{ECBB25E4-2145-4120-8981-E6E8E1591E5B}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2777,7 +2813,7 @@
 </file>
 
 <file path=xl/tables/table27.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{A41F31BC-0CA5-4B1A-808E-7A8A6507019C}" name="LNG_global14" displayName="LNG_global14" ref="A1:I239" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{A41F31BC-0CA5-4B1A-808E-7A8A6507019C}" name="LNG_global14" displayName="LNG_global14" ref="A1:I239" totalsRowShown="0" headerRowDxfId="14" headerRowBorderDxfId="13" tableBorderDxfId="12" totalsRowBorderDxfId="11">
   <autoFilter ref="A1:I239" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{D01CBB17-E8FF-44A2-B87B-A0B5AC3337BA}" name="From"/>
@@ -2790,10 +2826,10 @@
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{B6C8563B-B70E-4D32-A7CA-353FAC6B7501}" name="Distance [miles]"/>
-    <tableColumn id="4" xr3:uid="{DB3ABB11-1F6C-4F58-B946-9343785CF33A}" name="Distance [km]" dataDxfId="7">
+    <tableColumn id="4" xr3:uid="{DB3ABB11-1F6C-4F58-B946-9343785CF33A}" name="Distance [km]" dataDxfId="10">
       <calculatedColumnFormula>LNG_global14[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{601054B1-1B08-47CB-880D-0D80ED1BD0EA}" name="Suez or Panama" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{601054B1-1B08-47CB-880D-0D80ED1BD0EA}" name="Suez or Panama" dataDxfId="9"/>
     <tableColumn id="8" xr3:uid="{F8768BD8-8B11-4BD9-B074-AD5ADFFDF447}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2801,7 +2837,7 @@
 </file>
 
 <file path=xl/tables/table28.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{FB6F6EBF-837E-4C6E-87B9-22B5E7C1A32C}" name="LNG_global1423" displayName="LNG_global1423" ref="A1:I215" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="22" xr:uid="{FB6F6EBF-837E-4C6E-87B9-22B5E7C1A32C}" name="LNG_global1423" displayName="LNG_global1423" ref="A1:I215" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7" tableBorderDxfId="6" totalsRowBorderDxfId="5">
   <autoFilter ref="A1:I215" xr:uid="{CA4061AA-5D26-4056-B170-4E1336D4AD38}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{EAA26E2C-1949-4C4F-8D8C-2606BC6C5C27}" name="From"/>
@@ -2814,10 +2850,10 @@
       <calculatedColumnFormula>D2/1000</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{2A3DF244-4FAE-4993-9DEA-495BB43BB92E}" name="Distance [miles]"/>
-    <tableColumn id="4" xr3:uid="{BC8012D2-BA58-4D3F-BAC0-AF085B2E1A4C}" name="Distance [km]" dataDxfId="1">
+    <tableColumn id="4" xr3:uid="{BC8012D2-BA58-4D3F-BAC0-AF085B2E1A4C}" name="Distance [km]" dataDxfId="4">
       <calculatedColumnFormula>LNG_global1423[[#This Row],[Distance '[miles']]]*1.60934449789256</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{01A3A191-9692-4C2C-A7B3-0D2196CA510D}" name="Suez or Panama" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{01A3A191-9692-4C2C-A7B3-0D2196CA510D}" name="Suez or Panama" dataDxfId="3"/>
     <tableColumn id="8" xr3:uid="{8F94EED9-C1D5-4756-ACF3-482717384D23}" name="Comment"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2833,15 +2869,15 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{D3465064-BCEE-4D04-A8E6-DEAE11BBDA92}" name="Country"/>
     <tableColumn id="2" xr3:uid="{D66D54B4-4DED-47C6-BE50-755A236428ED}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="120"/>
-    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="119"/>
-    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="118">
+    <tableColumn id="3" xr3:uid="{DB34E8EE-2DCE-45DC-955E-A0569FED64E5}" name="Mrd m3 [2020]" dataDxfId="116"/>
+    <tableColumn id="5" xr3:uid="{4278F9D8-E46F-44B9-A622-727B8E2C8EF1}" name="Mil m3 EU [2020]" dataDxfId="115"/>
+    <tableColumn id="6" xr3:uid="{F2BDB73C-713D-4BC7-B762-048AA072F297}" name="Mrd m3 EU [2020]" dataDxfId="114">
       <calculatedColumnFormula>Table2[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{337F5DC2-FD6B-445B-A2F7-5464B34B589E}" name="GWh [2020]" dataDxfId="117">
+    <tableColumn id="7" xr3:uid="{337F5DC2-FD6B-445B-A2F7-5464B34B589E}" name="GWh [2020]" dataDxfId="113">
       <calculatedColumnFormula>Table2[[#This Row],[TWh '[2020']2]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]2" dataDxfId="116">
+    <tableColumn id="4" xr3:uid="{5BB2DA97-8C23-44BC-9268-BDBE2BCDBBC8}" name="TWh [2020]2" dataDxfId="112">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table2[[#This Row],[Mrd m3 EU '[2020']]],Table2[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2850,20 +2886,20 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A1:G17" totalsRowShown="0" headerRowDxfId="115" headerRowBorderDxfId="114" tableBorderDxfId="113">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}" name="Table7" displayName="Table7" ref="A1:G17" totalsRowShown="0" headerRowDxfId="111" headerRowBorderDxfId="110" tableBorderDxfId="109">
   <autoFilter ref="A1:G17" xr:uid="{E6071428-9756-478B-B239-1474A97B9EF4}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{3F684FB4-9656-4C92-BAF4-456019B2B924}" name="Country"/>
     <tableColumn id="2" xr3:uid="{082B059D-405D-407D-8F97-297DCD23D3B2}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{388F462C-127F-4CB7-B46A-1DD19D06D0E8}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{ACDF4345-6201-4524-A8D7-A0CE31D137A6}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="112">
+    <tableColumn id="5" xr3:uid="{7B596C1D-5C84-4EE8-9BEB-2A91E37A640C}" name="Mrd m3 [2020]2" dataDxfId="108">
       <calculatedColumnFormula>Table7[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{4A1E0E2A-2ECC-45EB-9D63-EC01B197BAA8}" name="GWh [2020]" dataDxfId="111">
+    <tableColumn id="7" xr3:uid="{4A1E0E2A-2ECC-45EB-9D63-EC01B197BAA8}" name="GWh [2020]" dataDxfId="107">
       <calculatedColumnFormula>Table7[[#This Row],[TWh '[2020']2]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]2" dataDxfId="110">
+    <tableColumn id="6" xr3:uid="{ECFA587C-DE79-4510-9945-328AB8DBC35F}" name="TWh [2020]2" dataDxfId="106">
       <calculatedColumnFormula>IF(Table7[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7[[#This Row],[Mrd m3 '[2020']2]],Table7[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2880,15 +2916,15 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{0D4D6418-D624-47ED-891A-572FBFD244A5}" name="Country"/>
     <tableColumn id="2" xr3:uid="{41AC793D-EB9C-4A09-A496-420AADE8645A}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="109"/>
-    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="108"/>
-    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="107">
+    <tableColumn id="3" xr3:uid="{07045358-68F1-4DE8-BDB8-9DFBCD592DF5}" name="Mrd m3 [2020]" dataDxfId="105"/>
+    <tableColumn id="5" xr3:uid="{42F1A333-D727-4655-B618-A9AB5617745F}" name="Mil m3 EU [2020]" dataDxfId="104"/>
+    <tableColumn id="6" xr3:uid="{326B3A9A-70B2-4D34-8E01-54CBBD0565E6}" name="Mrd m3 EU [2020]" dataDxfId="103">
       <calculatedColumnFormula>Table26[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{7EF7045A-D72E-40AA-A523-1A389D57AAF5}" name="GWh [2020]" dataDxfId="106">
+    <tableColumn id="7" xr3:uid="{7EF7045A-D72E-40AA-A523-1A389D57AAF5}" name="GWh [2020]" dataDxfId="102">
       <calculatedColumnFormula>Table26[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="105">
+    <tableColumn id="4" xr3:uid="{DC1916A1-B3CC-4586-AE6D-12CF46A9C0F0}" name="TWh [2020]" dataDxfId="101">
       <calculatedColumnFormula>IF(Table26[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table26[[#This Row],[Mrd m3 EU '[2020']]],Table26[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2897,20 +2933,20 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A1:G17" totalsRowShown="0" headerRowDxfId="104" headerRowBorderDxfId="103" tableBorderDxfId="102">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}" name="Table79" displayName="Table79" ref="A1:G17" totalsRowShown="0" headerRowDxfId="100" headerRowBorderDxfId="99" tableBorderDxfId="98">
   <autoFilter ref="A1:G17" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{3A97CAD5-3E8B-4CBA-A265-7CE9E55AACD4}" name="Country"/>
     <tableColumn id="2" xr3:uid="{0BE0E24B-4D76-4AFC-B5E9-84E609FF4FC0}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{02819FD0-F6B6-484E-B4DA-8262AECE7052}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{A15C284E-E91C-44C6-B3BB-CC2DD205DA84}" name="Mil m3 [2020]"/>
-    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="101">
+    <tableColumn id="5" xr3:uid="{27836BC3-6815-42AC-A9E2-8AADB6115B0F}" name="Mrd m3 [2020]2" dataDxfId="97">
       <calculatedColumnFormula>Table79[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{A1AF1224-2FA6-47E0-9ECD-AB8B46DF628B}" name="GWh [2020]" dataDxfId="100">
+    <tableColumn id="7" xr3:uid="{A1AF1224-2FA6-47E0-9ECD-AB8B46DF628B}" name="GWh [2020]" dataDxfId="96">
       <calculatedColumnFormula>Table79[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="99">
+    <tableColumn id="6" xr3:uid="{0CF67BB6-4E02-4893-BB83-4858F32AB909}" name="TWh [2020]" dataDxfId="95">
       <calculatedColumnFormula>IF(Table79[[#This Row],[Mil m3 '[2020']]]&gt;0,Table79[[#This Row],[Mrd m3 '[2020']2]],Table79[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2927,13 +2963,13 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{372275E9-F8BA-48D2-ACA0-A4A1A54CB9AA}" name="Country"/>
     <tableColumn id="2" xr3:uid="{82057241-5F95-4876-AE25-27D76578972D}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{87A0EF48-52CD-4413-BE4C-7A6E497EBCAC}" name="Mrd m3 [2035] SP" dataDxfId="98"/>
-    <tableColumn id="5" xr3:uid="{6BE9D8BC-17DF-46B0-904B-E214536BC73C}" name="Mil m3 EU [2024]" dataDxfId="97"/>
-    <tableColumn id="6" xr3:uid="{88443DA7-833C-4668-ABC7-6640612488C4}" name="Mrd m3 EU [2020]" dataDxfId="96"/>
-    <tableColumn id="7" xr3:uid="{64FD0380-738D-4F61-AAEA-FA6952811E43}" name="GWh [2020]" dataDxfId="95">
+    <tableColumn id="3" xr3:uid="{87A0EF48-52CD-4413-BE4C-7A6E497EBCAC}" name="Mrd m3 [2035] SP" dataDxfId="94"/>
+    <tableColumn id="5" xr3:uid="{6BE9D8BC-17DF-46B0-904B-E214536BC73C}" name="Mil m3 EU [2024]" dataDxfId="93"/>
+    <tableColumn id="6" xr3:uid="{88443DA7-833C-4668-ABC7-6640612488C4}" name="Mrd m3 EU [2020]" dataDxfId="92"/>
+    <tableColumn id="7" xr3:uid="{64FD0380-738D-4F61-AAEA-FA6952811E43}" name="GWh [2020]" dataDxfId="91">
       <calculatedColumnFormula>Table2620[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{920F5378-329F-48CE-AB35-E8FBBE6E4295}" name="TWh [2020]" dataDxfId="94">
+    <tableColumn id="4" xr3:uid="{920F5378-329F-48CE-AB35-E8FBBE6E4295}" name="TWh [2020]" dataDxfId="90">
       <calculatedColumnFormula>(Table2620[[#This Row],[Mrd m3 '[2035'] SP]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2950,13 +2986,13 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{0483DC4F-74A0-4FD7-965D-2CF2BE907B9E}" name="Country"/>
     <tableColumn id="2" xr3:uid="{79BB7EB0-D282-4AEF-A564-63421732A219}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{FF87377E-E2DA-4047-84FC-189C87065CD1}" name="Mrd m3 [2035] SP" dataDxfId="93"/>
-    <tableColumn id="5" xr3:uid="{31D61434-4BE8-4DF8-919D-0B08C9C85FF9}" name="Mil m3 EU [2024]" dataDxfId="92"/>
-    <tableColumn id="6" xr3:uid="{791C1399-23F6-4DDC-8608-02DCF3203E4D}" name="Mrd m3 EU [2020]" dataDxfId="91"/>
-    <tableColumn id="7" xr3:uid="{C7B33927-885B-433C-9C92-1A5BB72E75AE}" name="GWh [2020]" dataDxfId="90">
+    <tableColumn id="3" xr3:uid="{FF87377E-E2DA-4047-84FC-189C87065CD1}" name="Mrd m3 [2035] SP" dataDxfId="89"/>
+    <tableColumn id="5" xr3:uid="{31D61434-4BE8-4DF8-919D-0B08C9C85FF9}" name="Mil m3 EU [2024]" dataDxfId="88"/>
+    <tableColumn id="6" xr3:uid="{791C1399-23F6-4DDC-8608-02DCF3203E4D}" name="Mrd m3 EU [2020]" dataDxfId="87"/>
+    <tableColumn id="7" xr3:uid="{C7B33927-885B-433C-9C92-1A5BB72E75AE}" name="GWh [2020]" dataDxfId="86">
       <calculatedColumnFormula>Table262021[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5CDEC814-A327-4D11-A6C7-3DEC6EA2D16D}" name="TWh [2020]" dataDxfId="89">
+    <tableColumn id="4" xr3:uid="{5CDEC814-A327-4D11-A6C7-3DEC6EA2D16D}" name="TWh [2020]" dataDxfId="85">
       <calculatedColumnFormula>(Table262021[[#This Row],[Mrd m3 '[2035'] SP]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2965,18 +3001,18 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{FB215816-2FDA-4829-AC16-2EE92DD94CC3}" name="Table7919" displayName="Table7919" ref="A1:G17" totalsRowShown="0" headerRowDxfId="88" headerRowBorderDxfId="87" tableBorderDxfId="86">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{FB215816-2FDA-4829-AC16-2EE92DD94CC3}" name="Table7919" displayName="Table7919" ref="A1:G17" totalsRowShown="0" headerRowDxfId="84" headerRowBorderDxfId="83" tableBorderDxfId="82">
   <autoFilter ref="A1:G17" xr:uid="{FA14358E-0A26-44DE-ADCA-3F13E2A3D0D9}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{B2335C45-F098-43ED-B93A-E5FB5EF8509D}" name="Country"/>
     <tableColumn id="2" xr3:uid="{154B3C8E-B922-470F-AE16-75ED247FB778}" name="Long_name"/>
     <tableColumn id="3" xr3:uid="{2680A50A-41AA-4265-9E71-910C95E8A40D}" name="Mrd m3 [2020]"/>
     <tableColumn id="4" xr3:uid="{6E87E63F-505E-420A-A1BB-88EED1DA4433}" name="Mil m3 [2024]"/>
-    <tableColumn id="5" xr3:uid="{A4F80785-5D31-4DEB-8C9A-B8678AC91976}" name="Mrd m3 [2020]2" dataDxfId="85"/>
-    <tableColumn id="7" xr3:uid="{5E4FB509-2E7C-4F35-ABA3-27B44D26F2A0}" name="GWh [2020]" dataDxfId="84">
+    <tableColumn id="5" xr3:uid="{A4F80785-5D31-4DEB-8C9A-B8678AC91976}" name="Mrd m3 [2020]2" dataDxfId="81"/>
+    <tableColumn id="7" xr3:uid="{5E4FB509-2E7C-4F35-ABA3-27B44D26F2A0}" name="GWh [2020]" dataDxfId="80">
       <calculatedColumnFormula>Table7919[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{404CEA6B-9B54-4634-86D8-4FC47FBC55CD}" name="TWh [2020]" dataDxfId="83">
+    <tableColumn id="6" xr3:uid="{404CEA6B-9B54-4634-86D8-4FC47FBC55CD}" name="TWh [2020]" dataDxfId="79">
       <calculatedColumnFormula>(Table7919[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -19048,8 +19084,8 @@
     <col min="1" max="1" width="7.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.5" style="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25" style="18" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="45" bestFit="1" customWidth="1"/>
   </cols>
@@ -19064,10 +19100,10 @@
       <c r="C1" t="s">
         <v>138</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="20" t="s">
         <v>139</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="20" t="s">
         <v>140</v>
       </c>
       <c r="F1" t="s">
@@ -19090,7 +19126,7 @@
       <c r="C2">
         <v>0</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="18">
         <v>549.9</v>
       </c>
       <c r="F2">
@@ -19245,7 +19281,7 @@
       <c r="C10">
         <v>0</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="18">
         <v>41.973541999999995</v>
       </c>
       <c r="F10">
@@ -19286,7 +19322,7 @@
       <c r="C12">
         <v>803.4</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="18">
         <v>261.10000000000002</v>
       </c>
       <c r="F12">
@@ -19327,7 +19363,7 @@
       <c r="C14">
         <v>20.38</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="18">
         <v>33.380000000000003</v>
       </c>
       <c r="F14">
@@ -19368,7 +19404,7 @@
       <c r="C16">
         <v>0</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="18">
         <v>467.5</v>
       </c>
       <c r="F16">
@@ -19390,7 +19426,7 @@
       <c r="C17">
         <v>477</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="18">
         <v>576</v>
       </c>
       <c r="F17">
@@ -19412,7 +19448,7 @@
       <c r="C18">
         <v>325.39999999999998</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="18">
         <v>325.39999999999998</v>
       </c>
       <c r="F18">
@@ -19434,7 +19470,7 @@
       <c r="C19">
         <v>1200.6999999999998</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="18">
         <v>1203.4999999999998</v>
       </c>
       <c r="F19">
@@ -19456,7 +19492,7 @@
       <c r="C20">
         <v>0</v>
       </c>
-      <c r="E20">
+      <c r="E20" s="18">
         <v>35.53171072</v>
       </c>
       <c r="F20">
@@ -19782,7 +19818,7 @@
       <c r="C37">
         <v>0</v>
       </c>
-      <c r="E37">
+      <c r="E37" s="18">
         <v>41</v>
       </c>
       <c r="F37">
@@ -19807,7 +19843,7 @@
       <c r="C38">
         <v>731.7</v>
       </c>
-      <c r="D38">
+      <c r="D38" s="18">
         <v>337.1</v>
       </c>
       <c r="F38">
@@ -19829,7 +19865,7 @@
       <c r="C39">
         <v>0</v>
       </c>
-      <c r="D39">
+      <c r="D39" s="18">
         <v>337.1</v>
       </c>
       <c r="F39">
@@ -19854,7 +19890,7 @@
       <c r="C40">
         <v>0</v>
       </c>
-      <c r="D40">
+      <c r="D40" s="18">
         <v>1154</v>
       </c>
       <c r="F40">
@@ -19879,7 +19915,7 @@
       <c r="C41">
         <v>0</v>
       </c>
-      <c r="E41">
+      <c r="E41" s="18">
         <v>61.341321000000001</v>
       </c>
       <c r="F41">
@@ -19901,7 +19937,7 @@
       <c r="C42">
         <v>178.5</v>
       </c>
-      <c r="E42">
+      <c r="E42" s="18">
         <v>67.7</v>
       </c>
       <c r="F42">
@@ -19923,7 +19959,7 @@
       <c r="C43">
         <v>0</v>
       </c>
-      <c r="D43">
+      <c r="D43" s="18">
         <v>549.9</v>
       </c>
       <c r="F43">
@@ -20005,7 +20041,7 @@
       <c r="C47">
         <v>0</v>
       </c>
-      <c r="E47">
+      <c r="E47" s="18">
         <v>32.802250000000008</v>
       </c>
       <c r="F47">
@@ -20160,7 +20196,7 @@
       <c r="C55">
         <v>142</v>
       </c>
-      <c r="D55">
+      <c r="D55" s="18">
         <v>142</v>
       </c>
       <c r="F55">
@@ -20296,7 +20332,7 @@
       <c r="C62">
         <v>0</v>
       </c>
-      <c r="E62">
+      <c r="E62" s="18">
         <v>41.973541999999995</v>
       </c>
       <c r="F62">
@@ -20318,7 +20354,7 @@
       <c r="C63">
         <v>168</v>
       </c>
-      <c r="E63">
+      <c r="E63" s="18">
         <v>67.7</v>
       </c>
       <c r="F63">
@@ -20359,7 +20395,7 @@
       <c r="C65">
         <v>0</v>
       </c>
-      <c r="D65">
+      <c r="D65" s="18">
         <v>118</v>
       </c>
       <c r="F65">
@@ -20381,7 +20417,7 @@
       <c r="C66">
         <v>499</v>
       </c>
-      <c r="D66">
+      <c r="D66" s="18">
         <v>493.7</v>
       </c>
       <c r="F66">
@@ -20403,7 +20439,7 @@
       <c r="C67">
         <v>0</v>
       </c>
-      <c r="D67">
+      <c r="D67" s="18">
         <v>442.8</v>
       </c>
       <c r="F67">
@@ -20444,7 +20480,7 @@
       <c r="C69">
         <v>0</v>
       </c>
-      <c r="E69">
+      <c r="E69" s="18">
         <v>80.846503979999994</v>
       </c>
       <c r="F69">
@@ -20523,7 +20559,7 @@
       <c r="C73">
         <v>488</v>
       </c>
-      <c r="D73">
+      <c r="D73" s="18">
         <v>459.6</v>
       </c>
       <c r="F73">
@@ -20545,7 +20581,7 @@
       <c r="C74">
         <v>1904.258</v>
       </c>
-      <c r="D74">
+      <c r="D74" s="18">
         <v>1247</v>
       </c>
       <c r="F74">
@@ -20567,7 +20603,7 @@
       <c r="C75">
         <v>570</v>
       </c>
-      <c r="D75">
+      <c r="D75" s="18">
         <v>568.5</v>
       </c>
       <c r="F75">
@@ -20589,7 +20625,7 @@
       <c r="C76">
         <v>0</v>
       </c>
-      <c r="D76">
+      <c r="D76" s="18">
         <v>963.6</v>
       </c>
       <c r="F76">
@@ -20611,7 +20647,7 @@
       <c r="C77">
         <v>1499.1</v>
       </c>
-      <c r="D77">
+      <c r="D77" s="18">
         <v>1406</v>
       </c>
       <c r="F77">
@@ -20709,7 +20745,7 @@
       <c r="C82">
         <v>1.3</v>
       </c>
-      <c r="E82">
+      <c r="E82" s="18">
         <v>55.7</v>
       </c>
       <c r="F82">
@@ -20788,7 +20824,7 @@
       <c r="C86">
         <v>0</v>
       </c>
-      <c r="D86">
+      <c r="D86" s="18">
         <v>245.8</v>
       </c>
       <c r="F86">
@@ -20829,7 +20865,7 @@
       <c r="C88">
         <v>1742</v>
       </c>
-      <c r="D88">
+      <c r="D88" s="18">
         <v>1406</v>
       </c>
       <c r="F88">
@@ -20851,7 +20887,7 @@
       <c r="C89">
         <v>220</v>
       </c>
-      <c r="D89">
+      <c r="D89" s="18">
         <v>220</v>
       </c>
       <c r="F89">
@@ -20873,7 +20909,7 @@
       <c r="C90">
         <v>0</v>
       </c>
-      <c r="D90">
+      <c r="D90" s="18">
         <v>168</v>
       </c>
       <c r="F90">
@@ -20895,7 +20931,7 @@
       <c r="C91">
         <v>0</v>
       </c>
-      <c r="E91">
+      <c r="E91" s="18">
         <v>958.9</v>
       </c>
       <c r="F91">
@@ -20920,10 +20956,10 @@
       <c r="C92">
         <v>0</v>
       </c>
-      <c r="D92">
+      <c r="D92" s="18">
         <v>1334</v>
       </c>
-      <c r="E92">
+      <c r="E92" s="18">
         <v>5459.5088498999994</v>
       </c>
       <c r="F92">
@@ -21040,7 +21076,7 @@
       <c r="C98">
         <v>416</v>
       </c>
-      <c r="D98">
+      <c r="D98" s="18">
         <v>280.8</v>
       </c>
       <c r="F98">
@@ -21062,7 +21098,7 @@
       <c r="C99">
         <v>0</v>
       </c>
-      <c r="D99">
+      <c r="D99" s="18">
         <v>1154</v>
       </c>
       <c r="F99">
@@ -21084,7 +21120,7 @@
       <c r="C100">
         <v>0</v>
       </c>
-      <c r="D100">
+      <c r="D100" s="18">
         <v>701.8</v>
       </c>
       <c r="F100">
@@ -21106,7 +21142,7 @@
       <c r="C101">
         <v>0</v>
       </c>
-      <c r="D101">
+      <c r="D101" s="18">
         <v>395</v>
       </c>
       <c r="F101">
@@ -21128,7 +21164,7 @@
       <c r="C102">
         <v>516.6</v>
       </c>
-      <c r="D102">
+      <c r="D102" s="18">
         <v>517.5</v>
       </c>
       <c r="F102">
@@ -21150,7 +21186,7 @@
       <c r="C103">
         <v>0</v>
       </c>
-      <c r="E103">
+      <c r="E103" s="18">
         <v>255.46047452000005</v>
       </c>
       <c r="F103">
@@ -21172,7 +21208,7 @@
       <c r="C104">
         <v>135.6</v>
       </c>
-      <c r="D104">
+      <c r="D104" s="18">
         <v>135.6</v>
       </c>
       <c r="F104">
@@ -21194,7 +21230,7 @@
       <c r="C105">
         <v>1114.0999999999999</v>
       </c>
-      <c r="D105">
+      <c r="D105" s="18">
         <v>201.6</v>
       </c>
       <c r="F105">
@@ -21216,7 +21252,7 @@
       <c r="C106">
         <v>2277.6</v>
       </c>
-      <c r="D106">
+      <c r="D106" s="18">
         <f>1799+436.8</f>
         <v>2235.8000000000002</v>
       </c>
@@ -21239,7 +21275,7 @@
       <c r="C107">
         <v>651.70000000000005</v>
       </c>
-      <c r="D107">
+      <c r="D107" s="18">
         <v>227.2</v>
       </c>
       <c r="F107">
@@ -21261,7 +21297,7 @@
       <c r="C108">
         <v>476.2</v>
       </c>
-      <c r="D108">
+      <c r="D108" s="18">
         <v>385</v>
       </c>
       <c r="F108">
@@ -21283,7 +21319,7 @@
       <c r="C109">
         <v>0</v>
       </c>
-      <c r="D109">
+      <c r="D109" s="18">
         <v>184.8</v>
       </c>
       <c r="F109">
@@ -33476,12 +33512,9 @@
         <f t="shared" ref="E2:E23" si="0">D2/1000</f>
         <v>0</v>
       </c>
-      <c r="F2">
-        <v>5323</v>
-      </c>
       <c r="G2">
         <f>LNG_global[[#This Row],[Distance '[miles']]]*1.60934449789256</f>
-        <v>8566.5407622820967</v>
+        <v>0</v>
       </c>
       <c r="I2" t="s">
         <v>238</v>

</xml_diff>

<commit_message>
create 2019 input data sheet for optimization
including additional sheets for updating 2019 values
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
+++ b/01_data/01_input_data/02_processed/Gas_Import_Russian_Invasion.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\gas_infrastructure_model\01_data\01_input_data\02_processed\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55324361-3220-40E6-B0BB-681FC226DA92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B452683D-708B-4E9C-B6BF-74529C00108D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="24" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="790" firstSheet="16" activeTab="19" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodes_lng_europe_2019" sheetId="32" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5572" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5572" uniqueCount="329">
   <si>
     <t>Belgium</t>
   </si>
@@ -1006,30 +1006,6 @@
     <t>NO from Hammerfest</t>
   </si>
   <si>
-    <t>LNG Capacity Mrd m3 [2019]</t>
-  </si>
-  <si>
-    <t>Imports [2019]</t>
-  </si>
-  <si>
-    <t>Share [2019]</t>
-  </si>
-  <si>
-    <t>Capacity after grid connection [2019]</t>
-  </si>
-  <si>
-    <t>Mrd m3 [2019]</t>
-  </si>
-  <si>
-    <t>Mil m3 EU [2019]</t>
-  </si>
-  <si>
-    <t>GWh [2019]</t>
-  </si>
-  <si>
-    <t>TWh [2019]</t>
-  </si>
-  <si>
     <t>https://www.iea.org/countries/Morocco/natural-gas</t>
   </si>
   <si>
@@ -1043,15 +1019,6 @@
   </si>
   <si>
     <t>Population 2019 [Tsd]</t>
-  </si>
-  <si>
-    <t>Mil m3 [2019]</t>
-  </si>
-  <si>
-    <t>Mrd m3 [2019]2</t>
-  </si>
-  <si>
-    <t>Mrd m3 EU [2019]2</t>
   </si>
   <si>
     <t>sum of values in "6.2 GAZ NATUREL - Consommation", used conversion factor of 1 mil tonnes of oil equivalent (TOE in english, TEP in french) equals 1 milliard cubic meters of naturgal gas (from Energy Insititute's Statistical Review of World Energy)</t>
@@ -1088,6 +1055,9 @@
   </si>
   <si>
     <t>based on GEM (Source)</t>
+  </si>
+  <si>
+    <t>Mrd m3 EU [2020]2</t>
   </si>
 </sst>
 </file>
@@ -1443,7 +1413,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1468,7 +1438,6 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="C01_Main head" xfId="22" xr:uid="{3FF1BF2F-769C-4CF6-BB03-FA58B69C5545}"/>
@@ -2394,16 +2363,16 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{4EA90B67-C1EA-3F49-80BD-F698B4BB1753}" name="Country"/>
     <tableColumn id="2" xr3:uid="{DE488C4E-BA4D-1C47-919F-17B200DC8E8E}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{40424F55-FF29-C846-9670-45BDC1946AF7}" name="Mrd m3 [2019]" dataDxfId="133"/>
-    <tableColumn id="5" xr3:uid="{CE68E676-D995-F544-BEB7-55E7188768DB}" name="Mil m3 EU [2019]" dataDxfId="132"/>
-    <tableColumn id="6" xr3:uid="{9428BA11-0FA4-4E43-B422-05EB8A043647}" name="Mrd m3 EU [2019]2" dataDxfId="131">
-      <calculatedColumnFormula>Table224[[#This Row],[Mil m3 EU '[2019']]]/1000</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{40424F55-FF29-C846-9670-45BDC1946AF7}" name="Mrd m3 [2020]" dataDxfId="133"/>
+    <tableColumn id="5" xr3:uid="{CE68E676-D995-F544-BEB7-55E7188768DB}" name="Mil m3 EU [2020]" dataDxfId="132"/>
+    <tableColumn id="6" xr3:uid="{9428BA11-0FA4-4E43-B422-05EB8A043647}" name="Mrd m3 EU [2020]2" dataDxfId="131">
+      <calculatedColumnFormula>Table224[[#This Row],[Mil m3 EU '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{444B9436-1239-F240-B4BF-1A913EC4CFF6}" name="GWh [2019]" dataDxfId="130">
-      <calculatedColumnFormula>Table224[[#This Row],[TWh '[2019']]]*1000</calculatedColumnFormula>
+    <tableColumn id="7" xr3:uid="{444B9436-1239-F240-B4BF-1A913EC4CFF6}" name="GWh [2020]" dataDxfId="130">
+      <calculatedColumnFormula>Table224[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5EF9A97F-15E9-B540-80E9-F7A73E08637D}" name="TWh [2019]" dataDxfId="129">
-      <calculatedColumnFormula>IF(Table224[[#This Row],[Mil m3 EU '[2019']]]&gt;0,Table224[[#This Row],[Mrd m3 EU '[2019']2]],Table224[[#This Row],[Mrd m3 '[2019']]])*9.77</calculatedColumnFormula>
+    <tableColumn id="4" xr3:uid="{5EF9A97F-15E9-B540-80E9-F7A73E08637D}" name="TWh [2020]" dataDxfId="129">
+      <calculatedColumnFormula>IF(Table224[[#This Row],[Mil m3 EU '[2020']]]&gt;0,Table224[[#This Row],[Mrd m3 EU '[2020']2]],Table224[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2419,16 +2388,16 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{4489F77B-7E3D-6B40-999F-0A5CFAAD43D0}" name="Country"/>
     <tableColumn id="2" xr3:uid="{ED6C7C95-39E5-C744-B5E7-2363DA50B5F7}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{480BAFC6-8BED-3B47-93A3-FFC4E41F5BDF}" name="Mrd m3 [2019]" dataDxfId="84"/>
-    <tableColumn id="4" xr3:uid="{5500BCB9-3E14-4C44-A98A-BF3DBD011C25}" name="TWh [2019]" dataDxfId="83">
-      <calculatedColumnFormula>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{480BAFC6-8BED-3B47-93A3-FFC4E41F5BDF}" name="Mrd m3 [2020]" dataDxfId="84"/>
+    <tableColumn id="4" xr3:uid="{5500BCB9-3E14-4C44-A98A-BF3DBD011C25}" name="TWh [2020]" dataDxfId="83">
+      <calculatedColumnFormula>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{88D78A88-5D7E-CD41-AD80-CBB8F276CCA0}" name="Population 2019 [Tsd]"/>
     <tableColumn id="6" xr3:uid="{895AA06E-8015-F44E-8A03-C29DA4E1A648}" name="TWh by share" dataDxfId="82">
-      <calculatedColumnFormula>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{474AC10A-97FA-2941-AAF0-7C38AC898810}" name="GWh [2019]" dataDxfId="81">
-      <calculatedColumnFormula>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</calculatedColumnFormula>
+    <tableColumn id="7" xr3:uid="{474AC10A-97FA-2941-AAF0-7C38AC898810}" name="GWh [2020]" dataDxfId="81">
+      <calculatedColumnFormula>MIN(Table126[[#This Row],[TWh '[2020']]],Table126[[#This Row],[TWh by share]])*1000</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2583,16 +2552,16 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{555371BF-8030-4257-9852-212E94829B9B}" name="Country"/>
     <tableColumn id="2" xr3:uid="{7A6B9E51-21D4-42B2-AFBA-7B60A87AD8C0}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2019]"/>
-    <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2019]"/>
-    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2019]2" dataDxfId="52">
-      <calculatedColumnFormula>Table7910[[#This Row],[Mil m3 '[2019']]]/1000</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{236E80DE-4D1E-44E6-BEEB-14AFF8D0DDB8}" name="Mrd m3 [2020]"/>
+    <tableColumn id="4" xr3:uid="{E205F142-327E-4DD1-B26C-F606AE947DFF}" name="Mil m3 [2020]"/>
+    <tableColumn id="5" xr3:uid="{75FBA110-8C6B-463E-9AAF-A26754EAB077}" name="Mrd m3 [2020]2" dataDxfId="52">
+      <calculatedColumnFormula>Table7910[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{95C698CF-3EBE-40E8-840D-A6C3E41CFB2C}" name="GWh [2019]" dataDxfId="51">
-      <calculatedColumnFormula>Table7910[[#This Row],[TWh '[2019']]]*1000</calculatedColumnFormula>
+    <tableColumn id="7" xr3:uid="{95C698CF-3EBE-40E8-840D-A6C3E41CFB2C}" name="GWh [2020]" dataDxfId="51">
+      <calculatedColumnFormula>Table7910[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2019]" dataDxfId="50">
-      <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2019']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2019']2]],Table7910[[#This Row],[Mrd m3 '[2019']]])*9.77*(-1)</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{44160680-3C35-4A7A-9677-B7F78304684A}" name="TWh [2020]" dataDxfId="50">
+      <calculatedColumnFormula>IF(Table7910[[#This Row],[Mil m3 '[2020']]]&gt;0,Table7910[[#This Row],[Mrd m3 '[2020']2]],Table7910[[#This Row],[Mrd m3 '[2020']]])*9.77*(-1)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2671,16 +2640,16 @@
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{A255C403-77A0-0149-952F-A878846F39C1}" name="Country"/>
     <tableColumn id="2" xr3:uid="{923C0F82-BEBC-E940-A917-C4E2F7D4734E}" name="Long_name"/>
-    <tableColumn id="3" xr3:uid="{FFD27A1A-A51B-1C48-8D57-2446CC1CEFBF}" name="Mrd m3 [2019]"/>
-    <tableColumn id="4" xr3:uid="{78BA9F62-196E-484F-9DEC-52A98B938429}" name="Mil m3 [2019]"/>
-    <tableColumn id="5" xr3:uid="{1E9161F2-5CB8-5841-990F-B983C48048E4}" name="Mrd m3 [2019]2" dataDxfId="125">
-      <calculatedColumnFormula>Table725[[#This Row],[Mil m3 '[2019']]]/1000</calculatedColumnFormula>
+    <tableColumn id="3" xr3:uid="{FFD27A1A-A51B-1C48-8D57-2446CC1CEFBF}" name="Mrd m3 [2020]"/>
+    <tableColumn id="4" xr3:uid="{78BA9F62-196E-484F-9DEC-52A98B938429}" name="Mil m3 [2020]"/>
+    <tableColumn id="5" xr3:uid="{1E9161F2-5CB8-5841-990F-B983C48048E4}" name="Mrd m3 [2020]2" dataDxfId="125">
+      <calculatedColumnFormula>Table725[[#This Row],[Mil m3 '[2020']]]/1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{81E6D352-CF73-E24E-8012-656B58D4230F}" name="GWh [2019]" dataDxfId="124">
-      <calculatedColumnFormula>Table725[[#This Row],[TWh '[2019']]]*1000</calculatedColumnFormula>
+    <tableColumn id="7" xr3:uid="{81E6D352-CF73-E24E-8012-656B58D4230F}" name="GWh [2020]" dataDxfId="124">
+      <calculatedColumnFormula>Table725[[#This Row],[TWh '[2020']]]*1000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{8E2D017E-D664-6848-A8DA-CC37D1BE073D}" name="TWh [2019]" dataDxfId="123">
-      <calculatedColumnFormula>IF(Table725[[#This Row],[Mil m3 '[2019']]]&gt;0,Table725[[#This Row],[Mrd m3 '[2019']2]],Table725[[#This Row],[Mrd m3 '[2019']]])*9.77</calculatedColumnFormula>
+    <tableColumn id="6" xr3:uid="{8E2D017E-D664-6848-A8DA-CC37D1BE073D}" name="TWh [2020]" dataDxfId="123">
+      <calculatedColumnFormula>IF(Table725[[#This Row],[Mil m3 '[2020']]]&gt;0,Table725[[#This Row],[Mrd m3 '[2020']2]],Table725[[#This Row],[Mrd m3 '[2020']]])*9.77</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3330,21 +3299,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F148C2B-1FF1-134F-9293-670021B40696}">
   <dimension ref="A1:O14"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="3.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="3.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="7.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="3.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="29.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="3.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="3.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -3355,16 +3324,16 @@
         <v>93</v>
       </c>
       <c r="C1" t="s">
-        <v>311</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>312</v>
+        <v>90</v>
       </c>
       <c r="E1" t="s">
-        <v>313</v>
+        <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>314</v>
+        <v>14</v>
       </c>
       <c r="G1" t="s">
         <v>102</v>
@@ -3988,15 +3957,15 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69DF3FF5-BC43-47FD-93E8-972E7148D64B}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.453125" customWidth="1"/>
-    <col min="2" max="2" width="12.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" customWidth="1"/>
     <col min="3" max="8" width="15" customWidth="1"/>
-    <col min="12" max="12" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.453125" customWidth="1"/>
-    <col min="17" max="17" width="18.1796875" customWidth="1"/>
-    <col min="18" max="18" width="14.453125" customWidth="1"/>
+    <col min="12" max="12" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.44140625" customWidth="1"/>
+    <col min="17" max="17" width="18.21875" customWidth="1"/>
+    <col min="18" max="18" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4423,16 +4392,16 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7B45B38-002A-48AE-A33D-051F4A624C81}">
   <dimension ref="A1:N49"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.453125" customWidth="1"/>
-    <col min="2" max="2" width="12.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" customWidth="1"/>
     <col min="3" max="8" width="15" customWidth="1"/>
-    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.453125" customWidth="1"/>
-    <col min="17" max="17" width="18.1796875" customWidth="1"/>
-    <col min="18" max="18" width="14.453125" customWidth="1"/>
+    <col min="11" max="11" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.44140625" customWidth="1"/>
+    <col min="17" max="17" width="18.21875" customWidth="1"/>
+    <col min="18" max="18" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -5908,16 +5877,16 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F7561FF-3CAF-499E-B5E7-936081CDB469}">
   <dimension ref="A1:N49"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.453125" customWidth="1"/>
-    <col min="2" max="2" width="12.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" customWidth="1"/>
     <col min="3" max="8" width="15" customWidth="1"/>
-    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.453125" customWidth="1"/>
-    <col min="17" max="17" width="18.1796875" customWidth="1"/>
-    <col min="18" max="18" width="14.453125" customWidth="1"/>
+    <col min="11" max="11" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.44140625" customWidth="1"/>
+    <col min="17" max="17" width="18.21875" customWidth="1"/>
+    <col min="18" max="18" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
@@ -7393,15 +7362,15 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{358ACD06-E0FC-4391-8CB7-FEB185F8EE0B}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.453125" customWidth="1"/>
-    <col min="2" max="2" width="12.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" customWidth="1"/>
     <col min="3" max="8" width="15" customWidth="1"/>
-    <col min="12" max="12" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.453125" customWidth="1"/>
-    <col min="17" max="17" width="18.1796875" customWidth="1"/>
-    <col min="18" max="18" width="14.453125" customWidth="1"/>
+    <col min="12" max="12" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.44140625" customWidth="1"/>
+    <col min="17" max="17" width="18.21875" customWidth="1"/>
+    <col min="18" max="18" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -7849,14 +7818,14 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4771FD01-41CB-F843-B0F0-6DF6DCAB7ADE}">
   <dimension ref="A1:G53"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.453125" customWidth="1"/>
-    <col min="2" max="2" width="12.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
-    <col min="5" max="5" width="22.1796875" customWidth="1"/>
-    <col min="14" max="14" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.21875" customWidth="1"/>
+    <col min="14" max="14" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -7867,19 +7836,19 @@
         <v>55</v>
       </c>
       <c r="C1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E1" t="s">
         <v>315</v>
-      </c>
-      <c r="D1" t="s">
-        <v>318</v>
-      </c>
-      <c r="E1" t="s">
-        <v>323</v>
       </c>
       <c r="F1" t="s">
         <v>118</v>
       </c>
       <c r="G1" t="s">
-        <v>317</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -7891,18 +7860,18 @@
       </c>
       <c r="C2" s="2"/>
       <c r="D2">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>0</v>
       </c>
       <c r="E2">
         <v>2862.4</v>
       </c>
       <c r="F2">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E2/$E$27),0)</f>
+        <f>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E2/$E$27),0)</f>
         <v>-7.7379100801224432</v>
       </c>
       <c r="G2">
-        <f>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</f>
+        <f>MIN(Table126[[#This Row],[TWh '[2020']]],Table126[[#This Row],[TWh by share]])*1000</f>
         <v>-7737.9100801224431</v>
       </c>
     </row>
@@ -7917,18 +7886,18 @@
         <v>8.9004410370900011</v>
       </c>
       <c r="D3">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>-86.957308932369301</v>
       </c>
       <c r="E3">
         <v>8858.7999999999993</v>
       </c>
       <c r="F3">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E3/$E$27),0)</f>
+        <f>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E3/$E$27),0)</f>
         <v>0</v>
       </c>
       <c r="G3">
-        <f>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</f>
+        <f>MIN(Table126[[#This Row],[TWh '[2020']]],Table126[[#This Row],[TWh by share]])*1000</f>
         <v>-86957.308932369298</v>
       </c>
     </row>
@@ -7943,18 +7912,18 @@
         <v>17.386897499999996</v>
       </c>
       <c r="D4">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>-169.86998857499995</v>
       </c>
       <c r="E4">
         <v>11455.5</v>
       </c>
       <c r="F4">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E4/$E$27),0)</f>
+        <f>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E4/$E$27),0)</f>
         <v>0</v>
       </c>
       <c r="G4">
-        <f>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</f>
+        <f>MIN(Table126[[#This Row],[TWh '[2020']]],Table126[[#This Row],[TWh by share]])*1000</f>
         <v>-169869.98857499994</v>
       </c>
     </row>
@@ -7967,14 +7936,14 @@
       </c>
       <c r="C5" s="2"/>
       <c r="D5">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>0</v>
       </c>
       <c r="E5">
         <v>3492</v>
       </c>
       <c r="F5">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E5/$E$27),0)</f>
+        <f>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E5/$E$27),0)</f>
         <v>-9.4399042760577032</v>
       </c>
       <c r="G5">
@@ -7992,18 +7961,18 @@
         <v>2.8308749999999998</v>
       </c>
       <c r="D6">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>-27.657648749999996</v>
       </c>
       <c r="E6">
         <v>7000</v>
       </c>
       <c r="F6">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E6/$E$27),0)</f>
+        <f>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E6/$E$27),0)</f>
         <v>0</v>
       </c>
       <c r="G6">
-        <f>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</f>
+        <f>MIN(Table126[[#This Row],[TWh '[2020']]],Table126[[#This Row],[TWh by share]])*1000</f>
         <v>-27657.648749999997</v>
       </c>
     </row>
@@ -8018,18 +7987,18 @@
         <v>2.7981422222222223</v>
       </c>
       <c r="D7">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>-27.337849511111109</v>
       </c>
       <c r="E7">
         <v>4076.2</v>
       </c>
       <c r="F7">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E7/$E$27),0)</f>
+        <f>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E7/$E$27),0)</f>
         <v>0</v>
       </c>
       <c r="G7">
-        <f>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</f>
+        <f>MIN(Table126[[#This Row],[TWh '[2020']]],Table126[[#This Row],[TWh by share]])*1000</f>
         <v>-27337.849511111108</v>
       </c>
     </row>
@@ -8044,18 +8013,18 @@
         <v>8.3249499999999976</v>
       </c>
       <c r="D8">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>-81.334761499999971</v>
       </c>
       <c r="E8">
         <v>10649.8</v>
       </c>
       <c r="F8">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E8/$E$27),0)</f>
+        <f>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E8/$E$27),0)</f>
         <v>0</v>
       </c>
       <c r="G8">
-        <f>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</f>
+        <f>MIN(Table126[[#This Row],[TWh '[2020']]],Table126[[#This Row],[TWh by share]])*1000</f>
         <v>-81334.761499999964</v>
       </c>
     </row>
@@ -8070,18 +8039,18 @@
         <v>2.8977778452312215</v>
       </c>
       <c r="D9">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>-28.311289547909034</v>
       </c>
       <c r="E9">
         <v>5806.1</v>
       </c>
       <c r="F9">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E9/$E$27),0)</f>
+        <f>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E9/$E$27),0)</f>
         <v>0</v>
       </c>
       <c r="G9">
-        <f>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</f>
+        <f>MIN(Table126[[#This Row],[TWh '[2020']]],Table126[[#This Row],[TWh by share]])*1000</f>
         <v>-28311.289547909033</v>
       </c>
     </row>
@@ -8096,18 +8065,18 @@
         <v>0.46605538888888887</v>
       </c>
       <c r="D10">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>-4.5533611494444441</v>
       </c>
       <c r="E10">
         <v>1324.8</v>
       </c>
       <c r="F10">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E10/$E$27),0)</f>
+        <f>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E10/$E$27),0)</f>
         <v>0</v>
       </c>
       <c r="G10">
-        <f>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</f>
+        <f>MIN(Table126[[#This Row],[TWh '[2020']]],Table126[[#This Row],[TWh by share]])*1000</f>
         <v>-4553.361149444444</v>
       </c>
     </row>
@@ -8122,18 +8091,18 @@
         <v>2.0338333333333334</v>
       </c>
       <c r="D11">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>-19.870551666666668</v>
       </c>
       <c r="E11">
         <v>5517.9</v>
       </c>
       <c r="F11">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E11/$E$27),0)</f>
+        <f>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E11/$E$27),0)</f>
         <v>0</v>
       </c>
       <c r="G11">
-        <f>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</f>
+        <f>MIN(Table126[[#This Row],[TWh '[2020']]],Table126[[#This Row],[TWh by share]])*1000</f>
         <v>-19870.551666666666</v>
       </c>
     </row>
@@ -8148,18 +8117,18 @@
         <v>43.662042325000002</v>
       </c>
       <c r="D12">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>-426.57815351524999</v>
       </c>
       <c r="E12">
         <v>67012.899999999994</v>
       </c>
       <c r="F12">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E12/$E$27),0)</f>
+        <f>IF(Table126[[#This Row],[TWh '[2020']]]=0,$D$27*(E12/$E$27),0)</f>
         <v>0</v>
       </c>
       <c r="G12">
-        <f>MIN(Table126[[#This Row],[TWh '[2019']]],Table126[[#This Row],[TWh by share]])*1000</f>
+        <f>MIN(Table126[[#This Row],[TWh '[2020']]],Table126[[#This Row],[TWh by share]])*1000</f>
         <v>-426578.15351525001</v>
       </c>
     </row>
@@ -8174,18 +8143,18 @@
         <v>89.283027777777761</v>
       </c>
       <c r="D13">
-        <f>Table126[[#This Row],[Mrd m3 '[2019']]]*9.77*-1</f>
+        <f>Table126[[#This Row],[Mrd m3 '[2020']]]*9.77*-1</f>
         <v>-872.29518138888864</v>
       </c>
       <c r="E13">
         <v>83019.199999999997</v>
       </c>
       <c r="F13">
-        <f>IF(Table126[[#This Row],[TWh '[2019']]]=0,$D$27*(E13/$E$27),0)</